<commit_message>
Update data pasar & berita - 2026-09-18 12:51 UTC
</commit_message>
<xml_diff>
--- a/data/market_news_latest.xlsx
+++ b/data/market_news_latest.xlsx
@@ -487,20 +487,20 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>6436.853</v>
+        <v>6441.1592</v>
       </c>
       <c r="F2" t="n">
-        <v>-24.2998</v>
+        <v>-21.272</v>
       </c>
       <c r="G2" t="n">
-        <v>-0.38</v>
+        <v>-0.33</v>
       </c>
       <c r="H2" t="n">
-        <v>222552300</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -534,7 +534,7 @@
         <v>1.14</v>
       </c>
       <c r="H3" t="n">
-        <v>2887250000</v>
+        <v>5058210000</v>
       </c>
     </row>
     <row r="4">
@@ -568,7 +568,7 @@
         <v>0.61</v>
       </c>
       <c r="H4" t="n">
-        <v>406102188</v>
+        <v>406100000</v>
       </c>
     </row>
     <row r="5">
@@ -593,16 +593,16 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>26418.2988</v>
+        <v>26418.3008</v>
       </c>
       <c r="F5" t="n">
-        <v>439.8691</v>
+        <v>439.8711</v>
       </c>
       <c r="G5" t="n">
         <v>1.69</v>
       </c>
       <c r="H5" t="n">
-        <v>9127066000</v>
+        <v>9884890000</v>
       </c>
     </row>
     <row r="6">
@@ -623,20 +623,20 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>63923</v>
+        <v>65018.9492</v>
       </c>
       <c r="F6" t="n">
-        <v>438.8984</v>
+        <v>882.6992</v>
       </c>
       <c r="G6" t="n">
-        <v>0.6899999999999999</v>
+        <v>1.38</v>
       </c>
       <c r="H6" t="n">
-        <v>124200000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -657,20 +657,20 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>24713.7793</v>
+        <v>24750.7793</v>
       </c>
       <c r="F7" t="n">
-        <v>46.5391</v>
+        <v>146.4902</v>
       </c>
       <c r="G7" t="n">
-        <v>0.19</v>
+        <v>0.6</v>
       </c>
       <c r="H7" t="n">
-        <v>2163400000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -691,14 +691,20 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>3911.8713</v>
+      </c>
+      <c r="F8" t="n">
+        <v>36.2673</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0.9399999999999999</v>
+      </c>
       <c r="H8" t="n">
-        <v>2338973440</v>
+        <v>1326610444</v>
       </c>
     </row>
     <row r="9">
@@ -719,20 +725,20 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>10688.5</v>
+        <v>10700.71</v>
       </c>
       <c r="F9" t="n">
-        <v>30.4004</v>
+        <v>-115.3896</v>
       </c>
       <c r="G9" t="n">
-        <v>0.29</v>
+        <v>-1.07</v>
       </c>
       <c r="H9" t="n">
-        <v>973251300</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -753,20 +759,20 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>25537.75</v>
+        <v>25425.4707</v>
       </c>
       <c r="F10" t="n">
-        <v>135.4707</v>
+        <v>-291.2402</v>
       </c>
       <c r="G10" t="n">
-        <v>0.53</v>
+        <v>-1.13</v>
       </c>
       <c r="H10" t="n">
-        <v>47164400</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -787,20 +793,20 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>5635.4102</v>
+        <v>5656.1099</v>
       </c>
       <c r="F11" t="n">
-        <v>-3.23</v>
+        <v>-4.4102</v>
       </c>
       <c r="G11" t="n">
-        <v>-0.06</v>
+        <v>-0.08</v>
       </c>
       <c r="H11" t="n">
-        <v>236209300</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -821,17 +827,17 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>17718</v>
+        <v>17735</v>
       </c>
       <c r="F12" t="n">
-        <v>53</v>
+        <v>17</v>
       </c>
       <c r="G12" t="n">
-        <v>0.3</v>
+        <v>0.1</v>
       </c>
       <c r="H12" t="n">
         <v>0</v>
@@ -855,17 +861,17 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>100.236</v>
+        <v>100.502</v>
       </c>
       <c r="F13" t="n">
-        <v>-0.074</v>
+        <v>0.282</v>
       </c>
       <c r="G13" t="n">
-        <v>-0.07000000000000001</v>
+        <v>0.28</v>
       </c>
       <c r="H13" t="n">
         <v>0</v>
@@ -893,13 +899,13 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>156.089</v>
+        <v>157.806</v>
       </c>
       <c r="F14" t="n">
-        <v>0.075</v>
+        <v>1.792</v>
       </c>
       <c r="G14" t="n">
-        <v>0.05</v>
+        <v>1.15</v>
       </c>
       <c r="H14" t="n">
         <v>0</v>
@@ -923,17 +929,17 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>0.4947</v>
+        <v>0.4971</v>
       </c>
       <c r="F15" t="n">
-        <v>-0.0059</v>
+        <v>0.0024</v>
       </c>
       <c r="G15" t="n">
-        <v>-1.18</v>
+        <v>0.49</v>
       </c>
       <c r="H15" t="n">
         <v>0</v>
@@ -957,17 +963,17 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>0.5296</v>
+        <v>0.5303</v>
       </c>
       <c r="F16" t="n">
-        <v>-0.0053</v>
+        <v>0.0007</v>
       </c>
       <c r="G16" t="n">
-        <v>-0.99</v>
+        <v>0.13</v>
       </c>
       <c r="H16" t="n">
         <v>0</v>
@@ -991,17 +997,17 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="E17" t="n">
         <v>0.3965</v>
       </c>
       <c r="F17" t="n">
-        <v>-0.0005</v>
+        <v>0</v>
       </c>
       <c r="G17" t="n">
-        <v>-0.13</v>
+        <v>0</v>
       </c>
       <c r="H17" t="n">
         <v>0</v>
@@ -1038,7 +1044,7 @@
         <v>1.11</v>
       </c>
       <c r="H18" t="n">
-        <v>41562692</v>
+        <v>41584300</v>
       </c>
     </row>
     <row r="19">
@@ -1072,7 +1078,7 @@
         <v>0.38</v>
       </c>
       <c r="H19" t="n">
-        <v>45333928</v>
+        <v>45334500</v>
       </c>
     </row>
     <row r="20">
@@ -1093,20 +1099,20 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>4383.2002</v>
+        <v>4408.2002</v>
       </c>
       <c r="F20" t="n">
-        <v>-4.2998</v>
+        <v>8.5</v>
       </c>
       <c r="G20" t="n">
-        <v>-0.1</v>
+        <v>0.19</v>
       </c>
       <c r="H20" t="n">
-        <v>6437</v>
+        <v>77095</v>
       </c>
     </row>
     <row r="21">
@@ -1127,20 +1133,20 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>101.1</v>
+        <v>96.8</v>
       </c>
       <c r="F21" t="n">
-        <v>-1.33</v>
+        <v>-5.11</v>
       </c>
       <c r="G21" t="n">
-        <v>-1.3</v>
+        <v>-5.01</v>
       </c>
       <c r="H21" t="n">
-        <v>601</v>
+        <v>111999</v>
       </c>
     </row>
     <row r="22">
@@ -1161,20 +1167,20 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="E22" t="n">
-        <v>104.07</v>
+        <v>98.91</v>
       </c>
       <c r="F22" t="n">
-        <v>-1.76</v>
+        <v>-5.91</v>
       </c>
       <c r="G22" t="n">
-        <v>-1.66</v>
+        <v>-5.64</v>
       </c>
       <c r="H22" t="n">
-        <v>61</v>
+        <v>17389</v>
       </c>
     </row>
     <row r="23">
@@ -1195,20 +1201,20 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="E23" t="n">
-        <v>6.6205</v>
+        <v>6.667</v>
       </c>
       <c r="F23" t="n">
-        <v>0.189</v>
+        <v>0.0805</v>
       </c>
       <c r="G23" t="n">
-        <v>2.94</v>
+        <v>1.22</v>
       </c>
       <c r="H23" t="n">
-        <v>405</v>
+        <v>15556</v>
       </c>
     </row>
     <row r="24">
@@ -1242,7 +1248,7 @@
         <v>1.81</v>
       </c>
       <c r="H24" t="n">
-        <v>18535030</v>
+        <v>18586500</v>
       </c>
     </row>
     <row r="25">
@@ -1263,17 +1269,17 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="E25" t="n">
-        <v>15.44</v>
+        <v>15.51</v>
       </c>
       <c r="F25" t="n">
-        <v>-2.27</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="G25" t="n">
-        <v>-12.82</v>
+        <v>0.45</v>
       </c>
       <c r="H25" t="n">
         <v>0</v>
@@ -1297,20 +1303,20 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="E26" t="n">
-        <v>76363.9375</v>
+        <v>78018.47659999999</v>
       </c>
       <c r="F26" t="n">
-        <v>213.6172</v>
+        <v>1614.7031</v>
       </c>
       <c r="G26" t="n">
-        <v>0.28</v>
+        <v>2.11</v>
       </c>
       <c r="H26" t="n">
-        <v>21708255232</v>
+        <v>26979530752</v>
       </c>
     </row>
     <row r="27">
@@ -1331,20 +1337,20 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="E27" t="n">
         <v>1610</v>
       </c>
       <c r="F27" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="G27" t="n">
-        <v>0.62</v>
+        <v>0</v>
       </c>
       <c r="H27" t="n">
-        <v>60726100</v>
+        <v>56733600</v>
       </c>
     </row>
     <row r="28">
@@ -1365,11 +1371,11 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="E28" t="n">
-        <v>1830</v>
+        <v>1835</v>
       </c>
       <c r="F28" t="n">
         <v>5</v>
@@ -1378,7 +1384,7 @@
         <v>0.27</v>
       </c>
       <c r="H28" t="n">
-        <v>80199800</v>
+        <v>88082300</v>
       </c>
     </row>
     <row r="29">
@@ -1399,20 +1405,20 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="E29" t="n">
-        <v>945</v>
+        <v>925</v>
       </c>
       <c r="F29" t="n">
-        <v>45</v>
+        <v>-20</v>
       </c>
       <c r="G29" t="n">
-        <v>5</v>
+        <v>-2.12</v>
       </c>
       <c r="H29" t="n">
-        <v>499691600</v>
+        <v>304158300</v>
       </c>
     </row>
     <row r="30">
@@ -1433,20 +1439,20 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="E30" t="n">
-        <v>3080</v>
+        <v>3180</v>
       </c>
       <c r="F30" t="n">
-        <v>-10</v>
+        <v>100</v>
       </c>
       <c r="G30" t="n">
-        <v>-0.32</v>
+        <v>3.25</v>
       </c>
       <c r="H30" t="n">
-        <v>6475500</v>
+        <v>17135700</v>
       </c>
     </row>
     <row r="31">
@@ -1467,20 +1473,20 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="E31" t="n">
         <v>5325</v>
       </c>
       <c r="F31" t="n">
-        <v>250</v>
+        <v>0</v>
       </c>
       <c r="G31" t="n">
-        <v>4.93</v>
+        <v>0</v>
       </c>
       <c r="H31" t="n">
-        <v>42409400</v>
+        <v>80621900</v>
       </c>
     </row>
     <row r="32">
@@ -1501,20 +1507,20 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="E32" t="n">
-        <v>650</v>
+        <v>645</v>
       </c>
       <c r="F32" t="n">
-        <v>5</v>
+        <v>-5</v>
       </c>
       <c r="G32" t="n">
-        <v>0.78</v>
+        <v>-0.77</v>
       </c>
       <c r="H32" t="n">
-        <v>40687300</v>
+        <v>28813000</v>
       </c>
     </row>
     <row r="33">
@@ -1535,20 +1541,20 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="E33" t="n">
-        <v>760</v>
+        <v>725</v>
       </c>
       <c r="F33" t="n">
-        <v>5</v>
+        <v>-35</v>
       </c>
       <c r="G33" t="n">
-        <v>0.66</v>
+        <v>-4.61</v>
       </c>
       <c r="H33" t="n">
-        <v>29722700</v>
+        <v>44267000</v>
       </c>
     </row>
     <row r="34">
@@ -1569,20 +1575,20 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="E34" t="n">
-        <v>4350</v>
+        <v>4210</v>
       </c>
       <c r="F34" t="n">
-        <v>30</v>
+        <v>-140</v>
       </c>
       <c r="G34" t="n">
-        <v>0.6899999999999999</v>
+        <v>-3.22</v>
       </c>
       <c r="H34" t="n">
-        <v>4854800</v>
+        <v>5643800</v>
       </c>
     </row>
     <row r="35">
@@ -1603,20 +1609,20 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="E35" t="n">
-        <v>685</v>
+        <v>665</v>
       </c>
       <c r="F35" t="n">
-        <v>-15</v>
+        <v>-20</v>
       </c>
       <c r="G35" t="n">
-        <v>-2.14</v>
+        <v>-2.92</v>
       </c>
       <c r="H35" t="n">
-        <v>93121400</v>
+        <v>49365100</v>
       </c>
     </row>
     <row r="36">
@@ -1637,20 +1643,20 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="E36" t="n">
-        <v>250</v>
+        <v>238</v>
       </c>
       <c r="F36" t="n">
-        <v>-10</v>
+        <v>-12</v>
       </c>
       <c r="G36" t="n">
-        <v>-3.85</v>
+        <v>-4.8</v>
       </c>
       <c r="H36" t="n">
-        <v>60362400</v>
+        <v>45839200</v>
       </c>
     </row>
     <row r="37">
@@ -1671,20 +1677,20 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="E37" t="n">
-        <v>16800</v>
+        <v>16900</v>
       </c>
       <c r="F37" t="n">
-        <v>2325</v>
+        <v>100</v>
       </c>
       <c r="G37" t="n">
-        <v>16.06</v>
+        <v>0.6</v>
       </c>
       <c r="H37" t="n">
-        <v>20753600</v>
+        <v>12231600</v>
       </c>
     </row>
   </sheetData>
@@ -1743,22 +1749,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Manajer Kopdes Merah Putih Mulai Ngantor 25 September</t>
+          <t>1 Juta Jaringan Gas Ditargetkan Rampung 2028</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Fri, 18 Sep 2026 06:25:00 +0700</t>
+          <t>Fri, 18 Sep 2026 19:43:52 +0700</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/04/18/penyerahan-truk-kdmp-di-temanggung-1776489684625_169.jpeg?w=360&amp;amp;q=90" /&gt; Manajer Koperasi Desa/Kelurahan Merah Putih (KDKMP) ditempatkan paling lambat 25 September 2026.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/05/21/kepala-kantor-staf-presiden-ksp-dudung-abdurachman-1779342097390_169.png?w=360&amp;amp;q=90" /&gt; Kepala Staf Kepresidenan (KSP) Dudung Abdurachman menargetkan pembangunan 1 juta jaringan gas (jargas) rumah tangga rampung pada 2028.</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8667677/manajer-kopdes-merah-putih-mulai-ngantor-25-september</t>
+          <t>https://finance.detik.com/energi/d-8669161/1-juta-jaringan-gas-ditargetkan-rampung-2028</t>
         </is>
       </c>
     </row>
@@ -1770,22 +1776,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Prabowo Ungkap Mesin Pertumbuhan Ekonomi, Bukan Cuma Kopdes &amp;amp; MBG</t>
+          <t>17.288 Koperasi Desa Merah Putih Siap Beroperasi, Ditargetkan Oktober 2026</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Fri, 18 Sep 2026 05:55:00 +0700</t>
+          <t>Fri, 18 Sep 2026 19:00:30 +0700</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/07/presiden-prabowo-subianto-1788766824465_169.png?w=360&amp;amp;q=90" /&gt; Presiden Prabowo Subianto menepis kabar pertumbuhan ekonomi hanya bergantung pada pengeluaran pemerintah saja.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/18/17288-koperasi-desa-merah-putih-siap-beroperasi-ditargetkan-oktober-2026-1789704925923_169.jpeg?w=360&amp;amp;q=90" /&gt; Sebanyak 17.288 KDKMP ditargetkan mulai beroperasi pada akhir September atau awal Oktober 2026 setelah pembangunan</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8667682/prabowo-ungkap-mesin-pertumbuhan-ekonomi-bukan-cuma-kopdes-mbg</t>
+          <t>https://finance.detik.com/foto-bisnis/d-8668326/17-288-koperasi-desa-merah-putih-siap-beroperasi-ditargetkan-oktober-2026</t>
         </is>
       </c>
     </row>
@@ -1797,22 +1803,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Bantu Finansial Masyarakat, Pegadaian Hadirkan Layanan Gadai-Bank Emas</t>
+          <t>Dirjen Pajak Pastikan Tak Ada Kenaikan Tarif PPN</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Thu, 17 Sep 2026 23:59:31 +0700</t>
+          <t>Fri, 18 Sep 2026 18:51:40 +0700</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/08/21/pegadaian-1787309668013_169.jpeg?w=360&amp;amp;q=90" /&gt; PT Pegadaian mencatat laba bersih tumbuh 84,4% hingga Juni 2026. Transformasi digital dan layanan Bank Emas jadi kunci kesuksesan dalam mendukung ekonomi.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/07/31/dirjen-pajak-bimo-wijayanto-1753973379712_169.jpeg?w=360&amp;amp;q=90" /&gt; Tarif PPN yang berlaku secara efektif saat ini sebesar 11% untuk barang/jasa non-mewah.</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8667709/bantu-finansial-masyarakat-pegadaian-hadirkan-layanan-gadai-bank-emas</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8669067/dirjen-pajak-pastikan-tak-ada-kenaikan-tarif-ppn</t>
         </is>
       </c>
     </row>
@@ -1824,22 +1830,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Pegadaian Dorong Penetrasi Inklusi Keuangan di Indonesia, Ini Caranya</t>
+          <t>RI &amp;amp; Malaysia Kerja Sama Garap Industri Halal</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Thu, 17 Sep 2026 23:30:27 +0700</t>
+          <t>Fri, 18 Sep 2026 18:36:24 +0700</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/10/09/pegadaian-luncurkan-super-apps-tring-1760013227685_169.jpeg?w=360&amp;amp;q=90" /&gt; PT Pegadaian mencatat laba bersih tumbuh 84,4% hingga Juni 2026. Transformasi digital dan layanan finansial inovatif mendukung inklusi keuangan di Ind</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/18/presiden-prabowo-subianto-menerima-kunjungan-wakil-perdana-menteri-malaysia-ahmad-zahid-hamidi-1789726788207_169.jpeg?w=360&amp;amp;q=90" /&gt; Presiden Prabowo Subianto menerima kunjungan Wakil PM Malaysia Ahmad Zahid Hamidi. Salah sat</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8667707/pegadaian-dorong-penetrasi-inklusi-keuangan-di-indonesia-ini-caranya</t>
+          <t>https://finance.detik.com/industri/d-8669041/ri-malaysia-kerja-sama-garap-industri-halal</t>
         </is>
       </c>
     </row>
@@ -1851,22 +1857,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Mau Lebih Jago Akuntansi? Yuk, Perdalam Materinya Lewat Kelas Ini</t>
+          <t>Harga BBM Malaysia Naik!</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Thu, 17 Sep 2026 23:22:46 +0700</t>
+          <t>Fri, 18 Sep 2026 18:06:51 +0700</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/17/detikevent-pede-akuntansi-1789662142983_169.jpeg?w=360&amp;amp;q=90" /&gt; Belajar akuntansi nggak berhenti di memahami debit, kredit, jurnal, dan laporan keuangan.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/02/26/ilustrasi-bbm-ron-90-dan-ron-92-1740541037771_169.jpeg?w=360&amp;amp;q=90" /&gt; Pemerintah Malaysia mengumumkan kenaikan harga Bahan Bakar Minyak (BBM) untuk bensin eceran nonsubsidi.</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8667777/mau-lebih-jago-akuntansi-yuk-perdalam-materinya-lewat-kelas-ini</t>
+          <t>https://finance.detik.com/energi/d-8668996/harga-bbm-malaysia-naik</t>
         </is>
       </c>
     </row>
@@ -1878,22 +1884,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Pakistan Berlakukan Subsidi BBM untuk Kendaraan Kecil</t>
+          <t>RSPI Group Beri Privilege Kesehatan bagi Nasabah BRI Private-BRI Prioritas</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Thu, 17 Sep 2026 23:00:54 +0700</t>
+          <t>Fri, 18 Sep 2026 17:25:11 +0700</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/17/pakistan-berlakukan-subsidi-bbm-untuk-kendaraan-kecil-1789627177235.jpeg?w=360&amp;amp;q=90" /&gt; Warga Karachi antre mengisi BBM setelah skema subsidi nasional mulai berlaku. Subsidi diberikan Rp100 per liter untuk kendaraan yang meme</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/18/bri-1789727091160.jpeg?w=360&amp;amp;q=90" /&gt; BRI Private dan BRI Prioritas menawarkan layanan kesehatan eksklusif melalui kolaborasi dengan RSPI Group, termasuk promo pemeriksaan kesehatan dan rawat inap.</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/foto-bisnis/d-8666828/pakistan-berlakukan-subsidi-bbm-untuk-kendaraan-kecil</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8668941/rspi-group-beri-privilege-kesehatan-bagi-nasabah-bri-private-bri-prioritas</t>
         </is>
       </c>
     </row>
@@ -1905,22 +1911,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Mengelola Bank Emas, Begini Peran Pegadaian Kelola Ekosistem Bisnis</t>
+          <t>Malaysia Mau Bantu RI Padamkan Karhutla</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Thu, 17 Sep 2026 23:00:27 +0700</t>
+          <t>Fri, 18 Sep 2026 17:20:10 +0700</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/08/14/pegadaian-kadin-indonesia-kolaborasi-mengemaskan-indonesia-1786682392293_169.jpeg?w=360&amp;amp;q=90" /&gt; PT Pegadaian berperan penting dalam pengembangan Bank Emas di Indonesia, mengelola 153 ton emas dan menawarkan berbagai layanan </t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/18/presiden-prabowo-subianto-dok-youtube-prabowo-subianto-1789716861096_169.jpeg?w=360&amp;amp;q=90" /&gt; Yang pertama, dari pihak Malaysia menawarkan bantuan, ingin ikut membantu kita untuk mengatasi kebakaran hutan di Kalimantan, kata P</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8667699/mengelola-bank-emas-begini-peran-pegadaian-kelola-ekosistem-bisnis</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8668930/malaysia-mau-bantu-ri-padamkan-karhutla</t>
         </is>
       </c>
     </row>
@@ -1932,22 +1938,22 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Produk Buatan Desa Langsung Tembus Pasar Dunia Tanpa Perantara</t>
+          <t>IHSG Berbalik Melemah ke 6.441 Jelang Akhir Pekan</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Thu, 17 Sep 2026 23:00:00 +0700</t>
+          <t>Fri, 18 Sep 2026 17:17:22 +0700</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/07/31/mendes-yandri-minta-masyarakat-waspadai-konten-yang-menyesatkan-1785458634777_43.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Desa dan Pembangunan Daerah Tertinggal Yandri Susanto mengatakan produk-produk lokal dari desa kini bisa langsung di</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/05/18/ihsg-anjlok-ke-zona-merah-bursa-saham-melemah-tajam-1779098741262_169.jpeg?w=360&amp;amp;q=90" /&gt; Indeks Harga Saham Gabungan (IHSG) berbalik melemah pada penutupan perdagangan Jumat (18/9).</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8667565/produk-buatan-desa-langsung-tembus-pasar-dunia-tanpa-perantara</t>
+          <t>https://finance.detik.com/bursa-dan-valas/d-8668924/ihsg-berbalik-melemah-ke-6-441-jelang-akhir-pekan</t>
         </is>
       </c>
     </row>
@@ -1959,22 +1965,22 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Produksi Sumur Minyak Tua Digenjot</t>
+          <t>Golongan Baru Cukai Rokok Masih Dibahas, Jadi Diterapkan?</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Thu, 17 Sep 2026 22:31:56 +0700</t>
+          <t>Fri, 18 Sep 2026 17:07:40 +0700</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2016/05/08/9081adef-1ebd-4014-833b-caf0b085830a_169.jpg?w=360&amp;amp;q=90" /&gt; Pemerintah akan menggenjot produksi minyak dalam negeri dengan cara meningkatkan kapasitas sumur-sumur tua dengan teknologi dan pemanfaatan 45.000 sumur rakyat.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/11/24/dirjen-bea-cukai-djaka-budhi-utama-1763987444131_169.jpeg?w=360&amp;amp;q=90" /&gt; Saat ini, rencana tersebut masih dalam tahap pembahasan internal dan pengkajian mendalam.</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8667747/produksi-sumur-minyak-tua-digenjot</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8668902/golongan-baru-cukai-rokok-masih-dibahas-jadi-diterapkan</t>
         </is>
       </c>
     </row>
@@ -1986,22 +1992,22 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Dari Gadai hingga Emas, Ini Bisnis Penopang Kinerja Pegadaian</t>
+          <t>Layanan Drive Thru Permudah Pengambilan Paspor di Imigrasi Dumai</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Thu, 17 Sep 2026 22:30:54 +0700</t>
+          <t>Fri, 18 Sep 2026 17:00:41 +0700</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/07/06/berkilau-di-bawah-danantara-pegadaian-akselerasi-ekosistem-bank-emas-1783337310220_169.jpeg?w=360&amp;amp;q=90" /&gt; Pegadaian bertransformasi menjadi pemain utama ekosistem emas nasional dengan aplikasi Tring! dan mencatat laba bersih</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/18/layanan-drive-thru-permudah-pengambilan-paspor-di-imigrasi-dumai-1789712173304.jpeg?w=360&amp;amp;q=90" /&gt; Imigrasi Dumai menghadirkan layanan drive thru untuk pengambilan paspor. Sepanjang 2026, sebanyak 12.849 paspor telah diterbit</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8667693/dari-gadai-hingga-emas-ini-bisnis-penopang-kinerja-pegadaian</t>
+          <t>https://finance.detik.com/foto-bisnis/d-8668409/layanan-drive-thru-permudah-pengambilan-paspor-di-imigrasi-dumai</t>
         </is>
       </c>
     </row>
@@ -2013,22 +2019,22 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Bitcoin Melesat Usai Pengumuman Suku Bunga AS</t>
+          <t>Thailand Bangun Jalur Darat Rp 533 Triliun, Saingi Selat Malaka</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Thu, 17 Sep 2026 22:00:39 +0700</t>
+          <t>Fri, 18 Sep 2026 16:59:09 +0700</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/12/02/asia-tenggara-waspadai-penambangan-kripto-1764646630714_169.jpeg?w=360&amp;amp;q=90" /&gt; Harga Bitcoin (BTC) bergerak naik dari kisaran US$ 75.400 atau sekitar Rp 1,33 miliar (asumsi kurs Rp 17.746) usai kenaikan suku bunga Federal Re</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/06/18/thailand-hidupkan-rencana-proyek-rp495-triliun-saingi-selat-malaka-1781781659138_169.jpeg?w=360&amp;amp;q=90" /&gt; Thailand rencanakan jalur alternatif di Selat Malaka untuk menghubungkan Samudra Hindia dan Pasifik. Proyek ini bertujua</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/fintech/d-8667716/bitcoin-melesat-usai-pengumuman-suku-bunga-as</t>
+          <t>https://finance.detik.com/energi/d-8668889/thailand-bangun-jalur-darat-rp-533-triliun-saingi-selat-malaka</t>
         </is>
       </c>
     </row>
@@ -2040,22 +2046,22 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Bukan Sekadar Naik, Ini Cerita di Balik Laba Pegadaian Rp 6,59 Triliun</t>
+          <t>Sekolah Bisa Tolak MBG, Bos BGN Beberkan Syaratnya</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Thu, 17 Sep 2026 22:00:11 +0700</t>
+          <t>Fri, 18 Sep 2026 16:41:58 +0700</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/05/21/pegadaian-1779358942933_169.jpeg?w=360&amp;amp;q=90" /&gt; Pegadaian mencatat laba bersih Rp 6,59 triliun pada Semester I 2026, meningkat 84,4%. Pertumbuhan didukung ekspansi bisnis dan kualitas pembiayaan yang terjaga.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/17/kepala-badan-gizi-nasional-bgn-sudaryono-1789642729998_169.jpeg?w=360&amp;amp;q=90" /&gt; Sekolah diperbolehkan menolak program Makan Bergizi Gratis (MBG)</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8667686/bukan-sekadar-naik-ini-cerita-di-balik-laba-pegadaian-rp-6-59-triliun</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8668865/sekolah-bisa-tolak-mbg-bos-bgn-beberkan-syaratnya</t>
         </is>
       </c>
     </row>
@@ -2067,22 +2073,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Laba Pegadaian Naik 84,6%, Ini Angka Penting di Balik Kinerjanya</t>
+          <t>Kemenkeu Belum Bayar Cicilan Rp 37 T Kopdes Merah Putih, Ini Sebabnya</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Thu, 17 Sep 2026 21:54:20 +0700</t>
+          <t>Fri, 18 Sep 2026 16:39:47 +0700</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/07/06/berkilau-di-bawah-danantara-pegadaian-akselerasi-ekosistem-bank-emas-1783337310220_169.jpeg?w=360&amp;amp;q=90" /&gt; Laba Pegadaian tumbuh 84,4% di Semester I 2026, didorong oleh pertumbuhan aset, pembiayaan, dan penguatan bisnis emas.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/18/17288-koperasi-desa-merah-putih-siap-beroperasi-ditargetkan-oktober-2026-1789704926087_169.jpeg?w=360&amp;amp;q=90" /&gt; Kementerian Keuangan (Kemenkeu) belum membayar cicilan dan bunga pembiayaan Koperasi Desa/Kelurahan Merah Putih (K</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/infografis/d-8667713/laba-pegadaian-naik-84-6-ini-angka-penting-di-balik-kinerjanya</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8668864/kemenkeu-belum-bayar-cicilan-rp-37-t-kopdes-merah-putih-ini-sebabnya</t>
         </is>
       </c>
     </row>
@@ -2094,22 +2100,22 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Surpres Prabowo soal RUU Migas Terbit, Bahlil Jadi Ketua Tim</t>
+          <t>Suahasil soal Permintaan Batalkan Keputusan Purbaya Rombak Pejabat: Lagi Dibicarakan</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Thu, 17 Sep 2026 21:43:25 +0700</t>
+          <t>Fri, 18 Sep 2026 15:58:47 +0700</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/07/22/bahlil-lahadalia-1753180928818_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri ESDM Bahlil Lahadalia menyatakan Presiden Prabowo Subianto telah mengirimkan Surpres atau Surat Presiden soal pembahasan RUU Migas, ke DPR.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/14/pesan-suahasil-nazara-usai-jadi-menkeu-lanjutkan-tugas-dan-jaga-kepercayaan-1789383969847_169.jpeg?w=360&amp;amp;q=90" /&gt; Suahasil mengatakan permintaan tersebut masih dalam tahap pembahasan.</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8667700/surpres-prabowo-soal-ruu-migas-terbit-bahlil-jadi-ketua-tim</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8668778/suahasil-soal-permintaan-batalkan-keputusan-purbaya-rombak-pejabat-lagi-dibicarakan</t>
         </is>
       </c>
     </row>
@@ -2121,22 +2127,22 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Laba Pegadaian Melonjak 84,6%, Apa yang Mendorong Kinerja Semester I 2026?</t>
+          <t>Pelita Air Sebar Tiket MotoGP Mandalika Gratis di Pesawat</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Thu, 17 Sep 2026 21:34:14 +0700</t>
+          <t>Fri, 18 Sep 2026 15:57:08 +0700</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/08/14/prabowo-sampaikan-rencana-apbn-2027-1786699285146_169.jpeg?w=360&amp;amp;q=90" /&gt; PT Pegadaian mencatat laba bersih Rp 6,59 triliun, tumbuh 84,4% di 2026. Fokus pada ekosistem emas dan layanan Bank Emas untuk dukung perekonomian.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/04/24/pelita-air-secara-resmi-menyambut-kedatangan-armada-terbarunya-airbus-a320-dengan-registrasi-pk-pwn-kamis-24-april-2025-1745484764494_169.jpeg?w=360&amp;amp;q=90" /&gt; Pelita Air menebar tiket MotoGP Mandalika gratis secara acak di set</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8667680/laba-pegadaian-melonjak-84-6-apa-yang-mendorong-kinerja-semester-i-2026</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8668774/pelita-air-sebar-tiket-motogp-mandalika-gratis-di-pesawat</t>
         </is>
       </c>
     </row>
@@ -2148,22 +2154,22 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>27 Ribu Hektare Terbakar, 50 Perusahaan Pembakar Hutan Disegel</t>
+          <t>Infografis: 10 Terowongan Kereta Terpanjang di Dunia</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Fri, 18 Sep 2026 06:32:19 +0700</t>
+          <t>Fri, 18 Sep 2026 19:00:51 +0700</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>KLH menyegel 50 badan usaha terkait kebakaran di lahan seluas 27.333 hektare serta mengingatkan warga imbas kualitas udara Kalsel dan Kalteng yang mencapai status berbahaya.</t>
+          <t>Terowongan raksasa yang dirancang dengan teknologi dan rekayasa sipil mutakhir.</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8294171/27-ribu-hektare-terbakar-50-perusahaan-pembakar-hutan-disegel</t>
+          <t>https://www.liputan6.com/news/read/8294727/infografis-10-terowongan-kereta-terpanjang-di-dunia</t>
         </is>
       </c>
     </row>
@@ -2175,22 +2181,22 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Nasib PPPK Damkar dan Satpol PP Masih Menggantung, Mendagri Buka Suara</t>
+          <t>Mengenal Perdagangan Karbon Sebagai Sumber Ekonomi Baru</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Fri, 18 Sep 2026 06:15:14 +0700</t>
+          <t>Fri, 18 Sep 2026 18:59:54 +0700</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Skema pengalihan status PPPK damkar dan Satpol PP menjadi pegawai penuh waktu atau PNS masih dalam tahap pendataan dan kajian teknis.</t>
+          <t>Perdagangan karbon tak hanya soal kredit emisi. Pemerintah melihatnya sebagai peluang ekonomi sekaligus upaya menjaga hutan.</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8294168/nasib-pppk-damkar-dan-satpol-pp-masih-menggantung-mendagri-buka-suara</t>
+          <t>https://www.liputan6.com/news/read/8289853/mengenal-perdagangan-karbon-sebagai-sumber-ekonomi-baru</t>
         </is>
       </c>
     </row>
@@ -2202,22 +2208,22 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Dana Bencana Flores Naik 2 Kali Lipat, Ini Rinciannya</t>
+          <t>Kriyanusa 2026, Dekranas Dorong Perajin Tembus Pasar Global</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Fri, 18 Sep 2026 06:00:17 +0700</t>
+          <t>Fri, 18 Sep 2026 18:14:17 +0700</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Prabowo menggandakan alokasi tambahan Belanja Tidak Terduga (BTT) bencana untuk delapan kabupaten di Flores dan Pemprov NTT hingga mencapai Rp200 miliar.</t>
+          <t>Dekranas mendorong sinergi 14 kementerian dan lembaga untuk memperluas pembinaan perajin hingga ke pelosok daerah.</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8294161/dana-bencana-flores-naik-2-kali-lipat-ini-rinciannya</t>
+          <t>https://www.liputan6.com/news/read/8294699/kriyanusa-2026-dekranas-dorong-perajin-tembus-pasar-global</t>
         </is>
       </c>
     </row>
@@ -2229,22 +2235,22 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Peringatan Keras Kepala BGN buat Kepala Dapur MBG</t>
+          <t>Sosok Pria Tendang Wanita di Mal Jakpus</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Fri, 18 Sep 2026 06:00:00 +0700</t>
+          <t>Fri, 18 Sep 2026 18:12:56 +0700</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Kepala dapur kini wajib hadir langsung saat proses memasak MBG.</t>
+          <t>Motif pelaku menendang wanita di sebuah food court mal masih diselidiki.</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8294145/peringatan-keras-kepala-bgn-buat-kepala-dapur-mbg</t>
+          <t>https://www.liputan6.com/news/read/8294696/sosok-pria-tendang-wanita-di-mal-jakpus</t>
         </is>
       </c>
     </row>
@@ -2256,22 +2262,22 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>BPOM Siapkan 41 Ribu Sampel MBG Meski Anggaran Pengawasan Dipangkas</t>
+          <t>Geledah Kantor Summarecon, KPK Bawa Sejumlah Barang</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Fri, 18 Sep 2026 05:37:46 +0700</t>
+          <t>Fri, 18 Sep 2026 18:03:40 +0700</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>BPOM berkomitmen mengawal keamanan pangan program Makan Bergizi Gratis melalui uji 41.150 sampel di 27.000 SPPG meski anggaran yang disetujui hanya Rp509 miliar.</t>
+          <t>KPK menyasar kantor Summarecon dalam perkara dugaan suap HGB Bogor.</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8294159/bpom-siapkan-41-ribu-sampel-mbg-meski-anggaran-pengawasan-dipangkas</t>
+          <t>https://www.liputan6.com/news/read/8294684/geledah-kantor-summarecon-kpk-bawa-sejumlah-barang</t>
         </is>
       </c>
     </row>
@@ -2283,22 +2289,22 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Mendagri Garansi Nasib 172 Ribu PPPK Guru Paruh Waktu</t>
+          <t>Jakarta Padamkan Lampu 60 Menit pada 19 September, Cek Lokasinya</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Fri, 18 Sep 2026 05:20:34 +0700</t>
+          <t>Fri, 18 Sep 2026 17:18:18 +0700</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Mendagri Tito Karnavian memastikan PPPK guru paruh waktu yang belum lulus tes menjadi penuh waktu tidak akan dipecat dan tetap menerima pembiayaan dari dana BOS.</t>
+          <t>Sejumlah lokasi di Jakarta akan gelap selama satu jam pada Sabtu malam.</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8294158/mendagri-garansi-nasib-172-ribu-pppk-guru-paruh-waktu</t>
+          <t>https://www.liputan6.com/news/read/8294651/jakarta-padamkan-lampu-60-menit-pada-19-september-cek-lokasinya</t>
         </is>
       </c>
     </row>
@@ -2310,22 +2316,22 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Pencarian Panjang 5 Jurnalis dan 3 Awak Kapal di Selat Sunda</t>
+          <t>Kronologi Penangkapan Pria Tendang Wanita di Mal Jakpus</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Thu, 17 Sep 2026 19:29:42 +0700</t>
+          <t>Fri, 18 Sep 2026 16:49:07 +0700</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Keberadaan mereka hingga kini belum diketahui.</t>
+          <t>Motif pelaku menendang korban masih misteri.</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8293989/pencarian-panjang-5-jurnalis-dan-3-awak-kapal-di-selat-sunda</t>
+          <t>https://www.liputan6.com/news/read/8294626/kronologi-penangkapan-pria-tendang-wanita-di-mal-jakpus</t>
         </is>
       </c>
     </row>
@@ -2337,22 +2343,22 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Sudaryono Sebut Gangguan Kesehatan MBG Banyak Dipicu Makanan Rusak</t>
+          <t>Ambang Batas Parlemen Pengaruhi Kalkulasi Politik Pemilu 2029</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Fri, 18 Sep 2026 01:30:07 +0700</t>
+          <t>Fri, 18 Sep 2026 16:53:26 +0700</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Makanan rusak tersebut terutama ditemukan pada lauk dan sayur MBG.</t>
+          <t>Namun, angka ambang batas parlemen tersebut belum menemukan titik temu di antara partai politik.</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8294150/sudaryono-sebut-gangguan-kesehatan-mbg-banyak-dipicu-makanan-rusak</t>
+          <t>https://www.liputan6.com/news/read/8294632/ambang-batas-parlemen-pengaruhi-kalkulasi-politik-pemilu-2029</t>
         </is>
       </c>
     </row>
@@ -2364,22 +2370,22 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Polri Tangani 219 Kasus Kebakaran Hutan, Tetapkan 162 Tersangka</t>
+          <t>Klaim Kubu Febrie soal Asal Usul Tanah Disita Kejagung</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Thu, 17 Sep 2026 23:13:19 +0700</t>
+          <t>Fri, 18 Sep 2026 16:37:17 +0700</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Polri menempuh langkah hukum terhadap pihak-pihak yang diduga terlibat dalam peristiwa tersebut.</t>
+          <t>Total 38 tanah senilai Rp 800-an miliar berlokasi di Bandung disita Kejagung.</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8294132/polri-tangani-219-kasus-kebakaran-hutan-tetapkan-162-tersangka</t>
+          <t>https://www.liputan6.com/news/read/8294617/klaim-kubu-febrie-soal-asal-usul-tanah-disita-kejagung</t>
         </is>
       </c>
     </row>
@@ -2391,22 +2397,22 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Delapan Mawar dan Sejuta Doa untuk Jurnalis Arupadhatu 1</t>
+          <t>Peta Sikap Partai soal Wacana Kenaikan Ambang Batas Parlemen</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Thu, 17 Sep 2026 23:39:18 +0700</t>
+          <t>Fri, 18 Sep 2026 16:16:14 +0700</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Rekan-rekan jurnalis dan warga mengikuti doa bersama untuk lima jurnalis dan tiga kru kapal Arupadhatu 1 di pinggir dermaga Carita, Pandeglang, Banten, Kamis (17/9/2026). Delapan mawar putih dan sejumlah pesan harapan turut diletakkan di samping flyer berisi foto para penumpang kapal yang hilang kon</t>
+          <t>Angka 5 persen menjadi salah satu opsi yang dibicarakan sejumlah partai politik, meski belum ada keputusan mengenai besaran PT.</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/photo/read/8294137/delapan-mawar-dan-sejuta-doa-untuk-jurnalis-arupadhatu-1</t>
+          <t>https://www.liputan6.com/news/read/8294598/peta-sikap-partai-soal-wacana-kenaikan-ambang-batas-parlemen</t>
         </is>
       </c>
     </row>
@@ -2418,22 +2424,22 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>BGN Ultimatum 1.200 Dapur MBG Tanpa SLHS: Perbaiki atau Ditutup</t>
+          <t>Kapal Induk Italia Giuseppe Garibaldi Tiba di Tanjung Priok</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Thu, 17 Sep 2026 23:30:00 +0700</t>
+          <t>Fri, 18 Sep 2026 15:56:17 +0700</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Sekitar 1.200 dapur yang belum mengantongi Sertifikat Laik Higiene Sanitasi atau SLHS.</t>
+          <t xml:space="preserve">Kapal induk ITS Giuseppe Garibaldi-551 tiba di Dermaga 107 Pelabuhan Tanjung Priok, Jakarta, Jumat (18/9/2026). Kedatangan kapal milik Angkatan Laut Italia tersebut menjadi bagian dari kerja sama dan kegiatan di bidang kemaritiman. Kapal induk ITS Giuseppe Garibaldi-551 akan digunakan dalam Operasi </t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8294129/bgn-ultimatum-1200-dapur-mbg-tanpa-slhs-perbaiki-atau-ditutup</t>
+          <t>https://www.liputan6.com/photo/read/8294582/kapal-induk-italia-giuseppe-garibaldi-tiba-di-tanjung-priok</t>
         </is>
       </c>
     </row>
@@ -2445,22 +2451,22 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Seskab Teddy Ungkap 6 Langkah Prabowo Menuju Kemandirian Energi</t>
+          <t>Saksi Kasus Bea Cukai Ngamuk ke Hakim: Rumah Bapak akan Didatangi Rakyat</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Thu, 17 Sep 2026 23:00:00 +0700</t>
+          <t>Fri, 18 Sep 2026 15:39:52 +0700</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Prabowo mendorong percepatan swasembada energi dengan mengoptimalkan sumber daya yang tersedia di dalam negeri.</t>
+          <t>Emosi Faizal Assegaf memuncak saat dirinya memprotes penyitaan peralatan studio rekaman digital (podcast).</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8294122/seskab-teddy-ungkap-6-langkah-prabowo-menuju-kemandirian-energi</t>
+          <t>https://www.liputan6.com/news/read/8294564/saksi-kasus-bea-cukai-ngamuk-ke-hakim-rumah-bapak-akan-didatangi-rakyat</t>
         </is>
       </c>
     </row>
@@ -2472,22 +2478,22 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Menjajal Langsung LRT Manggarai-Kelapa Gading, dari Penasaran hingga Jadi Alternatif</t>
+          <t>Polisi Geledah 9 Lokasi Dugaan Korupsi Proyek Alat Konstruksi</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Thu, 17 Sep 2026 22:30:00 +0700</t>
+          <t>Fri, 18 Sep 2026 14:06:22 +0700</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Perjalanan belum benar-benar dimulai ketika akses menuju LRT justru harus dicari terlebih dahulu.</t>
+          <t>Kasus dugaan korupsi proyek alat konstruksi ini menyeret enam tersangka dengan kerugian negara Rp 37,35 miliar.</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8294120/menjajal-langsung-lrt-manggarai-kelapa-gading-dari-penasaran-hingga-jadi-alternatif</t>
+          <t>https://www.liputan6.com/news/read/8294447/polisi-geledah-9-lokasi-dugaan-korupsi-proyek-alat-konstruksi</t>
         </is>
       </c>
     </row>
@@ -2499,22 +2505,22 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Anggaran MBG Terserap Rp 139,77 Triliun hingga September 2026</t>
+          <t>Pramono Terbang ke AS, Bertemu Wali Kota New York Zohran Mamdani</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Thu, 17 Sep 2026 22:00:00 +0700</t>
+          <t>Fri, 18 Sep 2026 13:58:57 +0700</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Angka tersebut setara dengan 63,89 persen dari total pagu anggaran MBG sebesar Rp 218,77 triliun.</t>
+          <t>Wali Kota New York mengajak Pramono membahas solusi atas berbagai persoalan perkotaan.</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8294110/anggaran-mbg-terserap-rp-13977-triliun-hingga-september-2026</t>
+          <t>https://www.liputan6.com/news/read/8294439/pramono-terbang-ke-as-bertemu-wali-kota-new-york-zohran-mamdani</t>
         </is>
       </c>
     </row>
@@ -2526,22 +2532,22 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Mawar Putih dan Doa Kembali Selamat untuk 5 Jurnalis Hilang di Selat Sunda</t>
+          <t>Nusron Wahid Respons Kasus Suap di Kementerian ATR/BPN</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Thu, 17 Sep 2026 21:47:46 +0700</t>
+          <t>Fri, 18 Sep 2026 13:42:29 +0700</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Wartawan bersama tim SAR gabungan dan Gubernur Banten Andra Soni menggelar doa bersama untuk keselamatan jurnalis hilang kontak.</t>
+          <t>KPK menetapkan delapan orang sebagai tersangka dalam kasus dugaan suap di lingkungan Kementerian ATR/BPN.</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8294113/mawar-putih-dan-doa-kembali-selamat-untuk-5-jurnalis-hilang-di-selat-sunda</t>
+          <t>https://www.liputan6.com/news/read/8294425/nusron-wahid-respons-kasus-suap-di-kementerian-atrbpn</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data pasar & berita - 2026-09-22 00:19 UTC
</commit_message>
<xml_diff>
--- a/data/market_news_latest.xlsx
+++ b/data/market_news_latest.xlsx
@@ -487,20 +487,20 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>6384.7261</v>
+        <v>6441.1592</v>
       </c>
       <c r="F2" t="n">
-        <v>-56.4331</v>
+        <v>-21.272</v>
       </c>
       <c r="G2" t="n">
-        <v>-0.88</v>
+        <v>-0.33</v>
       </c>
       <c r="H2" t="n">
-        <v>0</v>
+        <v>283004400</v>
       </c>
     </row>
     <row r="3">
@@ -525,16 +525,16 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>7722.73</v>
+        <v>7764.7002</v>
       </c>
       <c r="F3" t="n">
-        <v>72.23</v>
+        <v>114.2002</v>
       </c>
       <c r="G3" t="n">
-        <v>0.9399999999999999</v>
+        <v>1.49</v>
       </c>
       <c r="H3" t="n">
-        <v>841056999</v>
+        <v>3278075000</v>
       </c>
     </row>
     <row r="4">
@@ -559,16 +559,16 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>51872.4414</v>
+        <v>52048.8281</v>
       </c>
       <c r="F4" t="n">
-        <v>189.8008</v>
+        <v>366.1875</v>
       </c>
       <c r="G4" t="n">
-        <v>0.37</v>
+        <v>0.71</v>
       </c>
       <c r="H4" t="n">
-        <v>112646949</v>
+        <v>444358134</v>
       </c>
     </row>
     <row r="5">
@@ -593,16 +593,16 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>26930.5586</v>
+        <v>27122.0938</v>
       </c>
       <c r="F5" t="n">
-        <v>408.0195</v>
+        <v>599.5547</v>
       </c>
       <c r="G5" t="n">
-        <v>1.54</v>
+        <v>2.26</v>
       </c>
       <c r="H5" t="n">
-        <v>2952693000</v>
+        <v>7862256000</v>
       </c>
     </row>
     <row r="6">
@@ -657,20 +657,20 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>25042.7109</v>
+        <v>24750.7793</v>
       </c>
       <c r="F7" t="n">
-        <v>291.9316</v>
+        <v>146.4902</v>
       </c>
       <c r="G7" t="n">
-        <v>1.18</v>
+        <v>0.6</v>
       </c>
       <c r="H7" t="n">
-        <v>0</v>
+        <v>3420800000</v>
       </c>
     </row>
     <row r="8">
@@ -694,15 +694,9 @@
           <t>2026-09-21</t>
         </is>
       </c>
-      <c r="E8" t="n">
-        <v>3949.9067</v>
-      </c>
-      <c r="F8" t="n">
-        <v>38.0356</v>
-      </c>
-      <c r="G8" t="n">
-        <v>0.97</v>
-      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
       <c r="H8" t="n">
         <v>2990847444</v>
       </c>
@@ -725,20 +719,20 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>10735.6699</v>
+        <v>10659.0996</v>
       </c>
       <c r="F9" t="n">
-        <v>76.5703</v>
+        <v>-157</v>
       </c>
       <c r="G9" t="n">
-        <v>0.72</v>
+        <v>-1.45</v>
       </c>
       <c r="H9" t="n">
-        <v>0</v>
+        <v>1825121500</v>
       </c>
     </row>
     <row r="10">
@@ -759,20 +753,20 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>25564.4297</v>
+        <v>25304.0605</v>
       </c>
       <c r="F10" t="n">
-        <v>260.3691</v>
+        <v>-412.6504</v>
       </c>
       <c r="G10" t="n">
-        <v>1.03</v>
+        <v>-1.6</v>
       </c>
       <c r="H10" t="n">
-        <v>0</v>
+        <v>165009400</v>
       </c>
     </row>
     <row r="11">
@@ -793,20 +787,20 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>5675.23</v>
+        <v>5656.1099</v>
       </c>
       <c r="F11" t="n">
-        <v>19.1201</v>
+        <v>-4.4102</v>
       </c>
       <c r="G11" t="n">
-        <v>0.34</v>
+        <v>-0.08</v>
       </c>
       <c r="H11" t="n">
-        <v>0</v>
+        <v>448210400</v>
       </c>
     </row>
     <row r="12">
@@ -827,17 +821,17 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="E12" t="n">
         <v>17808</v>
       </c>
       <c r="F12" t="n">
-        <v>51</v>
+        <v>2</v>
       </c>
       <c r="G12" t="n">
-        <v>0.29</v>
+        <v>0.01</v>
       </c>
       <c r="H12" t="n">
         <v>0</v>
@@ -865,13 +859,13 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>100.377</v>
+        <v>100.391</v>
       </c>
       <c r="F13" t="n">
-        <v>0.157</v>
+        <v>0.171</v>
       </c>
       <c r="G13" t="n">
-        <v>0.16</v>
+        <v>0.17</v>
       </c>
       <c r="H13" t="n">
         <v>0</v>
@@ -895,17 +889,17 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>157.454</v>
+        <v>157.38</v>
       </c>
       <c r="F14" t="n">
-        <v>1.325</v>
+        <v>0.334</v>
       </c>
       <c r="G14" t="n">
-        <v>0.85</v>
+        <v>0.21</v>
       </c>
       <c r="H14" t="n">
         <v>0</v>
@@ -933,13 +927,13 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>0.4959</v>
+        <v>0.4963</v>
       </c>
       <c r="F15" t="n">
-        <v>-0.0039</v>
+        <v>-0.0035</v>
       </c>
       <c r="G15" t="n">
-        <v>-0.78</v>
+        <v>-0.7</v>
       </c>
       <c r="H15" t="n">
         <v>0</v>
@@ -1001,13 +995,13 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>0.3987</v>
+        <v>0.3982</v>
       </c>
       <c r="F17" t="n">
-        <v>0.0009</v>
+        <v>0.0004</v>
       </c>
       <c r="G17" t="n">
-        <v>0.23</v>
+        <v>0.1</v>
       </c>
       <c r="H17" t="n">
         <v>0</v>
@@ -1034,17 +1028,11 @@
           <t>2026-09-21</t>
         </is>
       </c>
-      <c r="E18" t="n">
-        <v>81.66</v>
-      </c>
-      <c r="F18" t="n">
-        <v>0.41</v>
-      </c>
-      <c r="G18" t="n">
-        <v>0.5</v>
-      </c>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
       <c r="H18" t="n">
-        <v>11098463</v>
+        <v>26948257</v>
       </c>
     </row>
     <row r="19">
@@ -1068,17 +1056,11 @@
           <t>2026-09-21</t>
         </is>
       </c>
-      <c r="E19" t="n">
-        <v>78.70999999999999</v>
-      </c>
-      <c r="F19" t="n">
-        <v>0.18</v>
-      </c>
-      <c r="G19" t="n">
-        <v>0.23</v>
-      </c>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr"/>
       <c r="H19" t="n">
-        <v>11942405</v>
+        <v>43472166</v>
       </c>
     </row>
     <row r="20">
@@ -1103,16 +1085,16 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>4374</v>
+        <v>4410.2002</v>
       </c>
       <c r="F20" t="n">
-        <v>-50.8999</v>
+        <v>-14.6997</v>
       </c>
       <c r="G20" t="n">
-        <v>-1.15</v>
+        <v>-0.33</v>
       </c>
       <c r="H20" t="n">
-        <v>96207</v>
+        <v>10895</v>
       </c>
     </row>
     <row r="21">
@@ -1137,16 +1119,16 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>91.87</v>
+        <v>92.20999999999999</v>
       </c>
       <c r="F21" t="n">
-        <v>-8.43</v>
+        <v>-8.09</v>
       </c>
       <c r="G21" t="n">
-        <v>-8.4</v>
+        <v>-8.07</v>
       </c>
       <c r="H21" t="n">
-        <v>189652</v>
+        <v>3106</v>
       </c>
     </row>
     <row r="22">
@@ -1171,16 +1153,16 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>99.84</v>
+        <v>96.18000000000001</v>
       </c>
       <c r="F22" t="n">
-        <v>-4.03</v>
+        <v>-7.69</v>
       </c>
       <c r="G22" t="n">
-        <v>-3.88</v>
+        <v>-7.4</v>
       </c>
       <c r="H22" t="n">
-        <v>24291</v>
+        <v>204</v>
       </c>
     </row>
     <row r="23">
@@ -1205,16 +1187,16 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>6.7735</v>
+        <v>6.8065</v>
       </c>
       <c r="F23" t="n">
-        <v>0.1585</v>
+        <v>0.1915</v>
       </c>
       <c r="G23" t="n">
-        <v>2.4</v>
+        <v>2.89</v>
       </c>
       <c r="H23" t="n">
-        <v>26056</v>
+        <v>855</v>
       </c>
     </row>
     <row r="24">
@@ -1238,17 +1220,11 @@
           <t>2026-09-21</t>
         </is>
       </c>
-      <c r="E24" t="n">
-        <v>68.36499999999999</v>
-      </c>
-      <c r="F24" t="n">
-        <v>1.335</v>
-      </c>
-      <c r="G24" t="n">
-        <v>1.99</v>
-      </c>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr"/>
       <c r="H24" t="n">
-        <v>4648283</v>
+        <v>21965463</v>
       </c>
     </row>
     <row r="25">
@@ -1273,13 +1249,13 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>14.7</v>
+        <v>14.87</v>
       </c>
       <c r="F25" t="n">
-        <v>-0.11</v>
+        <v>0.06</v>
       </c>
       <c r="G25" t="n">
-        <v>-0.74</v>
+        <v>0.41</v>
       </c>
       <c r="H25" t="n">
         <v>0</v>
@@ -1303,20 +1279,20 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="E26" t="n">
-        <v>85814.3906</v>
+        <v>86425.2969</v>
       </c>
       <c r="F26" t="n">
-        <v>4671.7812</v>
+        <v>5282.6875</v>
       </c>
       <c r="G26" t="n">
-        <v>5.76</v>
+        <v>6.51</v>
       </c>
       <c r="H26" t="n">
-        <v>47774760960</v>
+        <v>57600937984</v>
       </c>
     </row>
     <row r="27">
@@ -1749,22 +1725,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>OJK Buka Suara soal Isu Gaji ASN Dipindah dari BPD ke Bank BUMN</t>
+          <t>Mau Usaha Makin Cuan dan Berkembang? Ini Hal yang Perlu Diperhatikan</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Mon, 21 Sep 2026 21:25:46 +0700</t>
+          <t>Tue, 22 Sep 2026 07:10:48 +0700</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/01/09/ilustrasi-gaji-1767955120071_169.jpeg?w=360&amp;amp;q=90" /&gt; OJK buka suara soal kabar pemindahan payroll atau pembayaran gaji Aparatur Sipil Negara (ASN) daerah dari Bank Pembangunan Daerah (BPD) ke Bank BUMN.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/21/ilustrasi-bisnis-umkm-1789974254174.png?w=360&amp;amp;q=90" /&gt; Pelajari cara mengelola usaha dengan efektif, dari memahami pelanggan hingga memanfaatkan DANA Bisnis untuk transaksi praktis. Tingkatkan bisnis Anda sekarang!</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/moneter/d-8673130/ojk-buka-suara-soal-isu-gaji-asn-dipindah-dari-bpd-ke-bank-bumn</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8672312/mau-usaha-makin-cuan-dan-berkembang-ini-hal-yang-perlu-diperhatikan</t>
         </is>
       </c>
     </row>
@@ -1776,22 +1752,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Dukung Ziswaf Digital, BYOND by BSI Hadirkan Fitur Otomatis Infaq Rutin</t>
+          <t>Beras di Toko Ritel Modern Kosong, Mentan: Beli di Pasar, Murah Kan?</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Mon, 21 Sep 2026 21:22:47 +0700</t>
+          <t>Tue, 22 Sep 2026 06:55:00 +0700</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/21/bsi-1790000547525_169.jpeg?w=360&amp;amp;q=90" /&gt; Hasil survei menunjukkan masyarakat Muslim Indonesia mengeluarkan Rp343,08 triliun untuk Ziswaf. BSI luncurkan fitur Infaq Rutin untuk memudahkan berbagi.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/07/28/wawancara-khusus-menteri-pertanian-ri-andi-amran-sulaiman-1753687994199_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Pertanian Andi Amran Sulaiman menepis kekosongan beras. Ia menyebut stok beras masih banyak di pasar tradisional.</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/moneter/d-8673128/dukung-ziswaf-digital-byond-by-bsi-hadirkan-fitur-otomatis-infaq-rutin</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8673023/beras-di-toko-ritel-modern-kosong-mentan-beli-di-pasar-murah-kan</t>
         </is>
       </c>
     </row>
@@ -1803,22 +1779,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Mentan Amran Siapkan Skema BUMN-Swasta untuk Industri Bioetanol</t>
+          <t>Pembeli Pasar Pondok Labu Tinggal Hitungan Jari, Pedagang Terlilit Utang</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Mon, 21 Sep 2026 20:55:09 +0700</t>
+          <t>Tue, 22 Sep 2026 06:45:16 +0700</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/21/kementan-1789998877923_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Pertanian Andi Amran Sulaiman mengungkapkan skema pengembangan bioetanol melibatkan BUMN dan swasta, untuk kemandirian energi dan ekonomi rakyat.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/21/pasar-pondok-labu-1789969187504_169.jpeg?w=360&amp;amp;q=90" /&gt; Pasar Pondok Labu sepi pembeli, banyak kios tutup. Pedagang mengalami penurunan omzet hingga 80%, terpaksa utang untuk modal usaha.</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8673098/mentan-amran-siapkan-skema-bumn-swasta-untuk-industri-bioetanol</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8673095/pembeli-pasar-pondok-labu-tinggal-hitungan-jari-pedagang-terlilit-utang</t>
         </is>
       </c>
     </row>
@@ -1830,22 +1806,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Penjualan Motor Listrik Merosot Tajam, Pengusaha Ungkap Biang Keroknya</t>
+          <t>Suahasil ke Pegawai Pajak &amp;amp; Bea Cukai: Pengawasan Semakin Tajam!</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Mon, 21 Sep 2026 20:41:39 +0700</t>
+          <t>Tue, 22 Sep 2026 06:25:00 +0700</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2024/10/09/nasib-insentif-kendaraan-listrik-di-tangan-prabowo-2_169.jpeg?w=360&amp;amp;q=90" /&gt; Ketua Asosiasi Industri Sepeda Motor Listrik Indonesia (Aismoli) Budi Setiyadi melaporkan penjualan sepeda motor listrik di Indonesia merosot tajam.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/21/menteri-keuangan-suahasil-nazara-melantik-14-pejabat-1789959240542_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Keuangan Suahasil Nazara meminta jajaran Direktorat Jenderal Pajak (DJP) dan Direktorat Jenderal Bea dan Cukai (DJBC) meningka</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/industri/d-8673078/penjualan-motor-listrik-merosot-tajam-pengusaha-ungkap-biang-keroknya</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8673012/suahasil-ke-pegawai-pajak-bea-cukai-pengawasan-semakin-tajam</t>
         </is>
       </c>
     </row>
@@ -1857,22 +1833,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Pengeboran Sumur Kedua Pengembangan PLTP 55 Megawatt Dimulai</t>
+          <t>Wanti-wanti Pengusaha ke Buruh yang Minta UMP Naik 9%</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Mon, 21 Sep 2026 19:47:06 +0700</t>
+          <t>Tue, 22 Sep 2026 05:55:00 +0700</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/21/pengeboran-sumur-untuk-pltp-lumut-balai-dimulai-1789994770073_169.jpeg?w=360&amp;amp;q=90" /&gt; PT Pertamina Geothermal Energy Tbk (PGE) Area Lumut Balai resmi memulai pengeboran sumur kedua, LMB-19.4,</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2022/04/21/thr_169.jpeg?w=360&amp;amp;q=90" /&gt; Usulan kenaikan Upah Minimum Provinsi (UMP) 2027 sebesar 9% direspons kalangan pengusaha.</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8673001/pengeboran-sumur-kedua-pengembangan-pltp-55-megawatt-dimulai</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8673008/wanti-wanti-pengusaha-ke-buruh-yang-minta-ump-naik-9</t>
         </is>
       </c>
     </row>
@@ -1884,22 +1860,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>748 Orang Direkrut Jadi Petugas Jaga Lintasan Kereta</t>
+          <t>Pembiayaan Pergadaian Tembus Rp 160 Triliun, Gadai Barang Mewah Diminati</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Mon, 21 Sep 2026 19:30:38 +0700</t>
+          <t>Mon, 21 Sep 2026 22:54:00 +0700</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/21/748-orang-direkrut-jadi-petugas-jaga-lintasan-kereta-1789985421130_169.jpeg?w=360&amp;amp;q=90" /&gt; Sebanyak 748 calon Petugas Jaga Lintasan mengikuti pembekalan dan sertifikasi. Tahapan ini disiapkan guna memperkuat keselamatan perli</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/04/22/sultan-merapat-ada-tempat-gadai-barang-mewah-1776830585380_169.jpeg?w=360&amp;amp;q=90" /&gt; Otoritas Jasa Keuangan (OJK) mencatat penyaluran pembiayaan industri pergadaian hingga Juli 2026 tumbuh tinggi.</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/foto-bisnis/d-8672742/748-orang-direkrut-jadi-petugas-jaga-lintasan-kereta</t>
+          <t>https://finance.detik.com/moneter/d-8673196/pembiayaan-pergadaian-tembus-rp-160-triliun-gadai-barang-mewah-diminati</t>
         </is>
       </c>
     </row>
@@ -1911,22 +1887,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Promo Rp8, Warga Ramai Jajal Rute Baru LRT ke Manggarai</t>
+          <t>Usaha Jasa Ramai Tapi Laporan Keuangan Berantakan? Ini Jalannya</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Mon, 21 Sep 2026 19:07:25 +0700</t>
+          <t>Mon, 21 Sep 2026 22:38:25 +0700</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/21/promo-rp8-warga-ramai-jajal-rute-baru-lrt-ke-manggarai-1789970710411.jpeg?w=360&amp;amp;q=90" /&gt; Sejumlah warga menggunakan transportasi umum LRT Jakarta dari Stasiun LRT Velodrome - Stasiun LRT Manggarai.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/08/detikevent-accurate-service-company-1788883745552_169.jpeg?w=360&amp;amp;q=90" /&gt; ACCURATE for Service Company Batch 4 diselenggarakan Piranha Smart Center melalui Education Visionary Lab (EVL) bersama detikEvent.</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/foto-bisnis/d-8672226/promo-rp8-warga-ramai-jajal-rute-baru-lrt-ke-manggarai</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8673184/usaha-jasa-ramai-tapi-laporan-keuangan-berantakan-ini-jalannya</t>
         </is>
       </c>
     </row>
@@ -1938,22 +1914,22 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Mentan Yakin dalam Seminggu Harga Beras Turun!</t>
+          <t>Pesan Suahasil ke 14 Pejabat Baru: Yang Kita Kelola Bukan Sekadar Angka</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Mon, 21 Sep 2026 18:41:40 +0700</t>
+          <t>Mon, 21 Sep 2026 22:33:22 +0700</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/03/30/menteri-pertanian-mentan-andi-amran-sulaiman-1774846718356_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Pertanian Andi Amran Sulaiman optimistis harga beras akan turun dalam sepekan. Amran juga tidak menampik saat ini harga beras saat ini</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/14/pesan-suahasil-nazara-usai-jadi-menkeu-lanjutkan-tugas-dan-jaga-kepercayaan-1789383969386_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Keuangan Suahasil Nazara melantik 14 Pejabat Pimpinan Tinggi Pratama dan Pejabat pada Sekretariat Komit</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8672930/mentan-yakin-dalam-seminggu-harga-beras-turun</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8673180/pesan-suahasil-ke-14-pejabat-baru-yang-kita-kelola-bukan-sekadar-angka</t>
         </is>
       </c>
     </row>
@@ -1965,22 +1941,22 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Mudahkan Investasi, Pegadaian Gaet BCA Digital Hadirkan bluInvest Emas</t>
+          <t>Terungkap Alasan Bensin di RI Bakal Dicampur Etanol 50%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Mon, 21 Sep 2026 17:38:47 +0700</t>
+          <t>Mon, 21 Sep 2026 22:04:12 +0700</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/21/pegadaian-gaet-bca-digital-hadirkan-bluinvest-emas-modal-awal-rp-10000-1789986947811_169.jpeg?w=360&amp;amp;q=90" /&gt; PT Bank Digital BCA dan Pegadaian luncurkan bluInvest Emas, memudahkan investasi emas digital mulai dari Rp10.000. A</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/08/04/bahlil-lahadalia-1785840108228_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri ESDM Bahlil Lahadalia menyampaikan pemerintah menyiapkan pengembangan bensin dengan campuran etanol hingga 50% atau E50.</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8672815/mudahkan-investasi-pegadaian-gaet-bca-digital-hadirkan-bluinvest-emas</t>
+          <t>https://finance.detik.com/energi/d-8673160/terungkap-alasan-bensin-di-ri-bakal-dicampur-etanol-50</t>
         </is>
       </c>
     </row>
@@ -1992,22 +1968,22 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Saham Rp 1 Mulai Berlaku</t>
+          <t>OJK Buka Suara soal Isu Gaji ASN Dipindah dari BPD ke Bank BUMN</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Mon, 21 Sep 2026 17:30:35 +0700</t>
+          <t>Mon, 21 Sep 2026 21:25:46 +0700</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/06/04/ihsg-terpuruk-kekhawatiran-pasar-meningkat-1780558039733_169.jpeg?w=360&amp;amp;q=90" /&gt; PT Bursa Efek Indonesia menurunkan batas harga saham minimum dari Rp 50 menjadi Rp 1. Perubahan ini bertujuan meningkatkan likuiditas dan fleksi</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/01/09/ilustrasi-gaji-1767955120071_169.jpeg?w=360&amp;amp;q=90" /&gt; OJK buka suara soal kabar pemindahan payroll atau pembayaran gaji Aparatur Sipil Negara (ASN) daerah dari Bank Pembangunan Daerah (BPD) ke Bank BUMN.</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/bursa-dan-valas/d-8672776/saham-rp-1-mulai-berlaku</t>
+          <t>https://finance.detik.com/moneter/d-8673130/ojk-buka-suara-soal-isu-gaji-asn-dipindah-dari-bpd-ke-bank-bumn</t>
         </is>
       </c>
     </row>
@@ -2019,22 +1995,22 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Perusahaan Singapura Gandeng APCO Group, Investasi Awal Rp 10 M di Bogor</t>
+          <t>Dukung Ziswaf Digital, BYOND by BSI Hadirkan Fitur Otomatis Infaq Rutin</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Mon, 21 Sep 2026 17:15:37 +0700</t>
+          <t>Mon, 21 Sep 2026 21:22:47 +0700</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/21/apco-group-1789985627691_169.jpeg?w=360&amp;amp;q=90" /&gt; APCO Group dan Entech Global Solution bentuk joint venture PT Entech APCO Environmental dengan investasi Rp 10 miliar.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/21/bsi-1790000547525_169.jpeg?w=360&amp;amp;q=90" /&gt; Hasil survei menunjukkan masyarakat Muslim Indonesia mengeluarkan Rp343,08 triliun untuk Ziswaf. BSI luncurkan fitur Infaq Rutin untuk memudahkan berbagi.</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8672752/perusahaan-singapura-gandeng-apco-group-investasi-awal-rp-10-m-di-bogor</t>
+          <t>https://finance.detik.com/moneter/d-8673128/dukung-ziswaf-digital-byond-by-bsi-hadirkan-fitur-otomatis-infaq-rutin</t>
         </is>
       </c>
     </row>
@@ -2046,22 +2022,22 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Beras di Ritel Modern Kosong Imbas Fortifikasi Disetop, Mentan Buka Suara</t>
+          <t>Mentan Amran Siapkan Skema BUMN-Swasta untuk Industri Bioetanol</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Mon, 21 Sep 2026 17:07:51 +0700</t>
+          <t>Mon, 21 Sep 2026 20:55:09 +0700</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/15/25-merek-beras-fortifikasi-dinyatakan-tak-sesuai-standar-1789447060266_169.jpeg?w=360&amp;amp;q=90" /&gt; Stok beras premium masih kosong di toko ritel modern. Kekosongan ini terjadi karena kasus beras fortifikasi yang sedang bergulir s</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/21/kementan-1789998877923_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Pertanian Andi Amran Sulaiman mengungkapkan skema pengembangan bioetanol melibatkan BUMN dan swasta, untuk kemandirian energi dan ekonomi rakyat.</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8672732/beras-di-ritel-modern-kosong-imbas-fortifikasi-disetop-mentan-buka-suara</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8673098/mentan-amran-siapkan-skema-bumn-swasta-untuk-industri-bioetanol</t>
         </is>
       </c>
     </row>
@@ -2073,22 +2049,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Dolar AS Tembus Rp 17.800, BI Ungkap Biang Keroknya</t>
+          <t>Penjualan Motor Listrik Merosot Tajam, Pengusaha Ungkap Biang Keroknya</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Mon, 21 Sep 2026 16:53:00 +0700</t>
+          <t>Mon, 21 Sep 2026 20:41:39 +0700</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2021/10/29/ilustrasi-bank-indonesia-6_169.jpeg?w=360&amp;amp;q=90" /&gt; Nilai tukar dolar Amerika Serikat (AS) terhadap rupiah berada di level Rp 17.847 terhadap rupiah. Bank Indonesia (BI) buka suara soal hal ini.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2024/10/09/nasib-insentif-kendaraan-listrik-di-tangan-prabowo-2_169.jpeg?w=360&amp;amp;q=90" /&gt; Ketua Asosiasi Industri Sepeda Motor Listrik Indonesia (Aismoli) Budi Setiyadi melaporkan penjualan sepeda motor listrik di Indonesia merosot tajam.</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/bursa-dan-valas/d-8672704/dolar-as-tembus-rp-17-800-bi-ungkap-biang-keroknya</t>
+          <t>https://finance.detik.com/industri/d-8673078/penjualan-motor-listrik-merosot-tajam-pengusaha-ungkap-biang-keroknya</t>
         </is>
       </c>
     </row>
@@ -2100,22 +2076,22 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>IHSG Ditutup Melemah ke Level 6.384</t>
+          <t>Pengeboran Sumur Kedua Pengembangan PLTP 55 Megawatt Dimulai</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Mon, 21 Sep 2026 16:45:31 +0700</t>
+          <t>Mon, 21 Sep 2026 19:47:06 +0700</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/06/04/ihsg-terpuruk-kekhawatiran-pasar-meningkat-1780558039793_169.jpeg?w=360&amp;amp;q=90" /&gt; IHSG ditutup melemah di level 6.384, turun 0,88%. Tercatat 280 saham menguat, 354 melemah, dan 156 stagnan.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/21/pengeboran-sumur-untuk-pltp-lumut-balai-dimulai-1789994770073_169.jpeg?w=360&amp;amp;q=90" /&gt; PT Pertamina Geothermal Energy Tbk (PGE) Area Lumut Balai resmi memulai pengeboran sumur kedua, LMB-19.4,</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/bursa-dan-valas/d-8672678/ihsg-ditutup-melemah-ke-level-6-384</t>
+          <t>https://finance.detik.com/energi/d-8673001/pengeboran-sumur-kedua-pengembangan-pltp-55-megawatt-dimulai</t>
         </is>
       </c>
     </row>
@@ -2127,22 +2103,22 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Beras di Toko Ritel Modern Kosong, Bulog Diminta Guyur 300.000 Ton</t>
+          <t>748 Orang Direkrut Jadi Petugas Jaga Lintasan Kereta</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Mon, 21 Sep 2026 16:42:24 +0700</t>
+          <t>Mon, 21 Sep 2026 19:30:38 +0700</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2024/02/13/penampakan-rak-beras-kosong-di-toko-ritel-ada-yang-diganti-kardus-mie-instan-3_169.jpeg?w=360&amp;amp;q=90" /&gt; Beras premium langka, bahkan di toko-toko ritel modern kosong. Bulog diminta guyur 300.000 ton.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/21/748-orang-direkrut-jadi-petugas-jaga-lintasan-kereta-1789985421130_169.jpeg?w=360&amp;amp;q=90" /&gt; Sebanyak 748 calon Petugas Jaga Lintasan mengikuti pembekalan dan sertifikasi. Tahapan ini disiapkan guna memperkuat keselamatan perli</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8672666/beras-di-toko-ritel-modern-kosong-bulog-diminta-guyur-300-000-ton</t>
+          <t>https://finance.detik.com/foto-bisnis/d-8672742/748-orang-direkrut-jadi-petugas-jaga-lintasan-kereta</t>
         </is>
       </c>
     </row>
@@ -2154,22 +2130,22 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Wamendagri Bima Arya Bicara Kunci Atasi Konflik Kebebasan Beragama</t>
+          <t>Gempa M 5,2 Guncang Tahuna Kepulauan Sangihe Sulut</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Mon, 21 Sep 2026 21:51:39 +0700</t>
+          <t>Tue, 22 Sep 2026 07:02:52 +0700</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Wamendagri Bima Arya mengatakan, kebebasan beragama membutuhkan kolaborasi di antara semua stakeholders dalam unsur masyarakat.</t>
+          <t>Gempa bumi Magnitudo 5,2 terjadi di Kepulauan Sangihe, Sulut. Gempa tidak berpotensi tsunami.</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8296469/wamendagri-bima-arya-bicara-kunci-atasi-konflik-kebebasan-beragama</t>
+          <t>https://www.liputan6.com/news/read/8296553/gempa-m-52-guncang-tahuna-kepulauan-sangihe-sulut</t>
         </is>
       </c>
     </row>
@@ -2181,22 +2157,22 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Pemerintah Ungkap Alasan Penempatan Manajer Kopdes Tak Bisa Asal Cepat</t>
+          <t>Jawaban Nusron Wahid Ditanya Soal Dugaan Korupsi di ATR/BPN</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Mon, 21 Sep 2026 21:27:12 +0700</t>
+          <t>Tue, 22 Sep 2026 06:08:54 +0700</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Pemerintah memastikan sumber daya manusia menggerakkan koperasi dan kampung nelayan tersebut dapat bekerja dengan sistem jelas dan memiliki kepastian.</t>
+          <t>Nusron Wahid enggan banyak bicara soal dugaan korupsi di lingkungan ATR/BPN.</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8296460/pemerintah-ungkap-alasan-penempatan-manajer-kopdes-tak-bisa-asal-cepat</t>
+          <t>https://www.liputan6.com/news/read/8296541/jawaban-nusron-wahid-ditanya-soal-dugaan-korupsi-di-atrbpn</t>
         </is>
       </c>
     </row>
@@ -2208,22 +2184,22 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Di Balik Pencarian 5 Jurnalis Hilang di Selat Sunda</t>
+          <t>1.487 Sekolah NTT Direvitalisasi Usai Gempa, Anggaran Rp 1,2 T Disiapkan</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Mon, 21 Sep 2026 21:12:34 +0700</t>
+          <t>Tue, 22 Sep 2026 01:36:43 +0700</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Rasa lelah tidak menyurutkan rekan kerja hingga keluarga menanti kepulangan rombongan jurnalis hilang di Selat Sunda.</t>
+          <t>Revitalisasi tersebut merupakan bentuk komitmen pemerintah untuk memastikan proses pemulihan pendidikan di daerah terdampak bencana dapat berjalan dengan baik.</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8296456/di-balik-pencarian-5-jurnalis-hilang-di-selat-sunda</t>
+          <t>https://www.liputan6.com/news/read/8296533/1487-sekolah-ntt-direvitalisasi-usai-gempa-anggaran-rp-12-t-disiapkan</t>
         </is>
       </c>
     </row>
@@ -2235,22 +2211,22 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>OTT Bupati Bolmut Diduga Terkait Korupsi Proyek Jalan</t>
+          <t>Keluarga Ungkap Momen Terakhir Seniman Den Baguse Ngarso Sebelum Wafat</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Mon, 21 Sep 2026 20:52:53 +0700</t>
+          <t>Tue, 22 Sep 2026 01:30:25 +0700</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Dalam OTT tersebut, KPK mengamankan 14 orang, termasuk Bupati Bolmut.</t>
+          <t>Seniman Yogyakarta Den Baguse Ngarso meninggal Senin (21/9) pukul 17.30 WIB di usia 67. Dimakamkan Selasa (22/9) pukul 16.00 WIB di TPU Krapyak.</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8296446/ott-bupati-bolmut-diduga-terkait-korupsi-proyek-jalan</t>
+          <t>https://www.liputan6.com/news/read/8296532/keluarga-ungkap-momen-terakhir-seniman-den-baguse-ngarso-sebelum-wafat</t>
         </is>
       </c>
     </row>
@@ -2262,22 +2238,22 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Uang Ratusan Juta Disita Saat OTT Bupati Bolmut</t>
+          <t>Mengintip Potensi Ekonomi Nelayan di Balik PLTS Pulau Sembur</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Mon, 21 Sep 2026 20:37:01 +0700</t>
+          <t>Mon, 21 Sep 2026 23:36:28 +0700</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Sebanyak 14 orang ditangkap di tiga wilayah terkait dugaan suap proyek infrastruktur.</t>
+          <t>PLTS Pulau Sembur telah selesai dibangun dan kini memasuki tahap pemanfaatan produktif.</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8296439/uang-ratusan-juta-disita-saat-ott-bupati-bolmut</t>
+          <t>https://www.liputan6.com/news/read/8296522/mengintip-potensi-ekonomi-nelayan-di-balik-plts-pulau-sembur</t>
         </is>
       </c>
     </row>
@@ -2289,22 +2265,22 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Ditangkap di Jakarta, Bupati Bolmut Diduga Terlibat Suap Proyek</t>
+          <t>Wamendagri Ribka Haluk Dorong NTT Berinovasi, Sektor Ini Jadi Sorotan</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Mon, 21 Sep 2026 20:18:46 +0700</t>
+          <t>Mon, 21 Sep 2026 21:57:17 +0700</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Sebanyak 14 orang diamankan dari tiga lokasi terkait dugaan suap proyek di lingkungan Pemkab Bolaang Mongondow Utara.</t>
+          <t>Wamendagri Ribka Haluk mengatakan, NTT memiliki potensi yang besar, baik dari sisi budaya maupun alam.</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8296434/ditangkap-di-jakarta-bupati-bolmut-diduga-terlibat-suap-proyek</t>
+          <t>https://www.liputan6.com/news/read/8296473/wamendagri-ribka-haluk-dorong-ntt-berinovasi-sektor-ini-jadi-sorotan</t>
         </is>
       </c>
     </row>
@@ -2316,22 +2292,22 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Seniman Den Baguse Ngarso Berpulang</t>
+          <t>Wamendagri Bima Arya Bicara Kunci Atasi Konflik Kebebasan Beragama</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Mon, 21 Sep 2026 20:06:53 +0700</t>
+          <t>Mon, 21 Sep 2026 21:51:39 +0700</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Kabar berpulangnya Den Baguse Ngarso dikonfirmasi oleh sejumlah rekan seniman. Salah satunya R.M. Bambang Ekoloyo Butet Kartaredjasa.</t>
+          <t>Wamendagri Bima Arya mengatakan, kebebasan beragama membutuhkan kolaborasi di antara semua stakeholders dalam unsur masyarakat.</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8296425/seniman-den-baguse-ngarso-berpulang</t>
+          <t>https://www.liputan6.com/news/read/8296469/wamendagri-bima-arya-bicara-kunci-atasi-konflik-kebebasan-beragama</t>
         </is>
       </c>
     </row>
@@ -2343,22 +2319,22 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Sosok Den Baguse Ngarso, Seniman Jogja dan Pendiri Teater Gandrik</t>
+          <t>Pemerintah Ungkap Alasan Penempatan Manajer Kopdes Tak Bisa Asal Cepat</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Mon, 21 Sep 2026 20:01:10 +0700</t>
+          <t>Mon, 21 Sep 2026 21:27:12 +0700</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Dalam perjalanan berkesenian, Den Baguse Ngarso tidak hanya bermain teater. Ia juga terlibat dalam seni dagelan, ketoprak, dan sinetron.</t>
+          <t>Pemerintah memastikan sumber daya manusia menggerakkan koperasi dan kampung nelayan tersebut dapat bekerja dengan sistem jelas dan memiliki kepastian.</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8296427/sosok-den-baguse-ngarso-seniman-jogja-dan-pendiri-teater-gandrik</t>
+          <t>https://www.liputan6.com/news/read/8296460/pemerintah-ungkap-alasan-penempatan-manajer-kopdes-tak-bisa-asal-cepat</t>
         </is>
       </c>
     </row>
@@ -2370,22 +2346,22 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Warga Cilandak Timur Antre Air Bersih di Tengah Kekeringan</t>
+          <t>Di Balik Pencarian 5 Jurnalis Hilang di Selat Sunda</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Mon, 21 Sep 2026 19:15:43 +0700</t>
+          <t>Mon, 21 Sep 2026 21:12:34 +0700</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Warga mengantre untuk mendapatkan bantuan air bersih di Gang H Soleh, Cilandak Timur, Jakarta Selatan, Senin (21/9/2026). Kekeringan yang melanda sejumlah wilayah di Kelurahan Cilandak Timur selama dua pekan terakhir membuat warga kesulitan memperoleh air untuk kebutuhan sehari-hari. Badan Penanggul</t>
+          <t>Rasa lelah tidak menyurutkan rekan kerja hingga keluarga menanti kepulangan rombongan jurnalis hilang di Selat Sunda.</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/photo/read/8296398/warga-cilandak-timur-antre-air-bersih-di-tengah-kekeringan</t>
+          <t>https://www.liputan6.com/news/read/8296456/di-balik-pencarian-5-jurnalis-hilang-di-selat-sunda</t>
         </is>
       </c>
     </row>
@@ -2397,22 +2373,22 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>KPK OTT Bupati Bolaang Mongondow Utara Sirajudin Lasena</t>
+          <t>OTT Bupati Bolmut Diduga Terkait Korupsi Proyek Jalan</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Mon, 21 Sep 2026 19:52:23 +0700</t>
+          <t>Mon, 21 Sep 2026 20:52:53 +0700</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>KPK gelar OTT di Kabupaten Bolaang Mongondow Utara (Bolmut). Dalam operasi tersebut, Bupati Bolmut Sirajudin Lasena ikut diamankan beserta penyegelan sejumlah ruang kerja kepala dinas.</t>
+          <t>Dalam OTT tersebut, KPK mengamankan 14 orang, termasuk Bupati Bolmut.</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8296400/kpk-ott-bupati-bolaang-mongondow-utara-sirajudin-lasena</t>
+          <t>https://www.liputan6.com/news/read/8296446/ott-bupati-bolmut-diduga-terkait-korupsi-proyek-jalan</t>
         </is>
       </c>
     </row>
@@ -2424,22 +2400,22 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Kronologi Bus Tabrak Truk hingga Terguling di Tol Cipali KM 176</t>
+          <t>Uang Ratusan Juta Disita Saat OTT Bupati Bolmut</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Mon, 21 Sep 2026 19:08:53 +0700</t>
+          <t>Mon, 21 Sep 2026 20:37:01 +0700</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Tidak ada korban jiwa maupun luka atas insiden tersebut.</t>
+          <t>Sebanyak 14 orang ditangkap di tiga wilayah terkait dugaan suap proyek infrastruktur.</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8296391/kronologi-bus-tabrak-truk-hingga-terguling-di-tol-cipali-km-176</t>
+          <t>https://www.liputan6.com/news/read/8296439/uang-ratusan-juta-disita-saat-ott-bupati-bolmut</t>
         </is>
       </c>
     </row>
@@ -2451,22 +2427,22 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>KPK Periksa Perdana Fahd Arafiq dan Eks Bupati Kebumen</t>
+          <t>Ditangkap di Jakarta, Bupati Bolmut Diduga Terlibat Suap Proyek</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Mon, 21 Sep 2026 19:00:56 +0700</t>
+          <t>Mon, 21 Sep 2026 20:18:46 +0700</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Fahd Arafiq dan mantan Bupati Kebumen Arif Sugiyanto menjalani pemeriksaan perdana sebagai tersangka kasus suap pembukaan blokir HGB Summarecon di KPK.</t>
+          <t>Sebanyak 14 orang diamankan dari tiga lokasi terkait dugaan suap proyek di lingkungan Pemkab Bolaang Mongondow Utara.</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8296382/kpk-periksa-perdana-fahd-arafiq-dan-eks-bupati-kebumen</t>
+          <t>https://www.liputan6.com/news/read/8296434/ditangkap-di-jakarta-bupati-bolmut-diduga-terlibat-suap-proyek</t>
         </is>
       </c>
     </row>
@@ -2478,22 +2454,22 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Kecelakaan Bus Tabrak Truk di Tol Cipali KM 176 Arah Jakarta</t>
+          <t>Seniman Den Baguse Ngarso Berpulang</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Mon, 21 Sep 2026 19:00:52 +0700</t>
+          <t>Tue, 22 Sep 2026 01:17:19 +0700</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Pengemudi bus diduga kurang mengantisipasi kendaraan di depannya sehingga tidak dapat menjaga jarak aman.</t>
+          <t>Kabar berpulangnya Den Baguse Ngarso dikonfirmasi oleh sejumlah rekan seniman. Salah satunya R.M. Bambang Ekoloyo Butet Kartaredjasa.</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8296387/kecelakaan-bus-tabrak-truk-di-tol-cipali-km-176-arah-jakarta</t>
+          <t>https://www.liputan6.com/news/read/8296425/seniman-den-baguse-ngarso-berpulang</t>
         </is>
       </c>
     </row>
@@ -2505,22 +2481,22 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>PDIP: Ambang Batas Parlemen Ideal di Kisaran 4 sampai 7 Persen</t>
+          <t>Sosok Den Baguse Ngarso, Seniman Jogja dan Pendiri Teater Gandrik</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Mon, 21 Sep 2026 19:01:22 +0700</t>
+          <t>Mon, 21 Sep 2026 20:01:10 +0700</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>PDIP masih menunggu hasil dialog dengan berbagai pihak sebelum menentukan besaran parliamentary threshold.</t>
+          <t>Dalam perjalanan berkesenian, Den Baguse Ngarso tidak hanya bermain teater. Ia juga terlibat dalam seni dagelan, ketoprak, dan sinetron.</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8296350/pdip-ambang-batas-parlemen-ideal-di-kisaran-4-sampai-7-persen</t>
+          <t>https://www.liputan6.com/news/read/8296427/sosok-den-baguse-ngarso-seniman-jogja-dan-pendiri-teater-gandrik</t>
         </is>
       </c>
     </row>
@@ -2532,22 +2508,22 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Lembaga Reforma Agraria Tetap Dibentuk, Nama Tunggu Presiden</t>
+          <t>Warga Cilandak Timur Antre Air Bersih di Tengah Kekeringan</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Mon, 21 Sep 2026 17:53:46 +0700</t>
+          <t>Mon, 21 Sep 2026 19:15:43 +0700</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Pasal 11 RUU Reforma Agraria mengatur pembentukan lembaga di bawah Presiden untuk mengelola reforma agraria.</t>
+          <t>Warga mengantre untuk mendapatkan bantuan air bersih di Gang H Soleh, Cilandak Timur, Jakarta Selatan, Senin (21/9/2026). Kekeringan yang melanda sejumlah wilayah di Kelurahan Cilandak Timur selama dua pekan terakhir membuat warga kesulitan memperoleh air untuk kebutuhan sehari-hari. Badan Penanggul</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8296340/lembaga-reforma-agraria-tetap-dibentuk-nama-tunggu-presiden</t>
+          <t>https://www.liputan6.com/photo/read/8296398/warga-cilandak-timur-antre-air-bersih-di-tengah-kekeringan</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data pasar & berita - 2026-09-22 23:53 UTC
</commit_message>
<xml_diff>
--- a/data/market_news_latest.xlsx
+++ b/data/market_news_latest.xlsx
@@ -487,20 +487,20 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>6277.0439</v>
+        <v>6384.7261</v>
       </c>
       <c r="F2" t="n">
-        <v>-107.6821</v>
+        <v>-56.4331</v>
       </c>
       <c r="G2" t="n">
-        <v>-1.69</v>
+        <v>-0.88</v>
       </c>
       <c r="H2" t="n">
-        <v>0</v>
+        <v>232135300</v>
       </c>
     </row>
     <row r="3">
@@ -521,20 +521,20 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>7764.7002</v>
+        <v>7764.6401</v>
       </c>
       <c r="F3" t="n">
-        <v>114.2002</v>
+        <v>-0.0601</v>
       </c>
       <c r="G3" t="n">
-        <v>1.49</v>
+        <v>-0</v>
       </c>
       <c r="H3" t="n">
-        <v>4828050000</v>
+        <v>3164537000</v>
       </c>
     </row>
     <row r="4">
@@ -555,20 +555,20 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>52048.8281</v>
+        <v>51863.6914</v>
       </c>
       <c r="F4" t="n">
-        <v>366.1875</v>
+        <v>-185.1367</v>
       </c>
       <c r="G4" t="n">
-        <v>0.71</v>
+        <v>-0.36</v>
       </c>
       <c r="H4" t="n">
-        <v>444350000</v>
+        <v>444772813</v>
       </c>
     </row>
     <row r="5">
@@ -589,20 +589,20 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>27122.0898</v>
+        <v>27244.2773</v>
       </c>
       <c r="F5" t="n">
-        <v>599.5508</v>
+        <v>122.1875</v>
       </c>
       <c r="G5" t="n">
-        <v>2.26</v>
+        <v>0.45</v>
       </c>
       <c r="H5" t="n">
-        <v>8813260000</v>
+        <v>8014146000</v>
       </c>
     </row>
     <row r="6">
@@ -657,20 +657,20 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>25087.75</v>
+        <v>25042.7109</v>
       </c>
       <c r="F7" t="n">
-        <v>45.0391</v>
+        <v>291.9316</v>
       </c>
       <c r="G7" t="n">
-        <v>0.18</v>
+        <v>1.18</v>
       </c>
       <c r="H7" t="n">
-        <v>0</v>
+        <v>2541100000</v>
       </c>
     </row>
     <row r="8">
@@ -694,15 +694,9 @@
           <t>2026-09-22</t>
         </is>
       </c>
-      <c r="E8" t="n">
-        <v>3952.1279</v>
-      </c>
-      <c r="F8" t="n">
-        <v>2.2209</v>
-      </c>
-      <c r="G8" t="n">
-        <v>0.06</v>
-      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
       <c r="H8" t="n">
         <v>3370196644</v>
       </c>
@@ -725,20 +719,20 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>10751.5</v>
+        <v>10739</v>
       </c>
       <c r="F9" t="n">
-        <v>12.5</v>
+        <v>79.9004</v>
       </c>
       <c r="G9" t="n">
-        <v>0.12</v>
+        <v>0.75</v>
       </c>
       <c r="H9" t="n">
-        <v>0</v>
+        <v>733429900</v>
       </c>
     </row>
     <row r="10">
@@ -759,20 +753,20 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>25743.5801</v>
+        <v>25575.0098</v>
       </c>
       <c r="F10" t="n">
-        <v>168.5703</v>
+        <v>270.9492</v>
       </c>
       <c r="G10" t="n">
-        <v>0.66</v>
+        <v>1.07</v>
       </c>
       <c r="H10" t="n">
-        <v>0</v>
+        <v>50641100</v>
       </c>
     </row>
     <row r="11">
@@ -793,20 +787,20 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>5723.7598</v>
+        <v>5675.23</v>
       </c>
       <c r="F11" t="n">
-        <v>48.5298</v>
+        <v>19.1201</v>
       </c>
       <c r="G11" t="n">
-        <v>0.86</v>
+        <v>0.34</v>
       </c>
       <c r="H11" t="n">
-        <v>0</v>
+        <v>241063200</v>
       </c>
     </row>
     <row r="12">
@@ -831,13 +825,13 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>17865</v>
+        <v>17846</v>
       </c>
       <c r="F12" t="n">
-        <v>59</v>
+        <v>40</v>
       </c>
       <c r="G12" t="n">
-        <v>0.33</v>
+        <v>0.22</v>
       </c>
       <c r="H12" t="n">
         <v>0</v>
@@ -865,13 +859,13 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>100.451</v>
+        <v>100.56</v>
       </c>
       <c r="F13" t="n">
-        <v>0.021</v>
+        <v>0.13</v>
       </c>
       <c r="G13" t="n">
-        <v>0.02</v>
+        <v>0.13</v>
       </c>
       <c r="H13" t="n">
         <v>0</v>
@@ -895,17 +889,17 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>157.262</v>
+        <v>157.452</v>
       </c>
       <c r="F14" t="n">
-        <v>0.216</v>
+        <v>0.083</v>
       </c>
       <c r="G14" t="n">
-        <v>0.14</v>
+        <v>0.05</v>
       </c>
       <c r="H14" t="n">
         <v>0</v>
@@ -933,13 +927,13 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>0.4943</v>
+        <v>0.4968</v>
       </c>
       <c r="F15" t="n">
-        <v>-0.002</v>
+        <v>0.0005</v>
       </c>
       <c r="G15" t="n">
-        <v>-0.4</v>
+        <v>0.1</v>
       </c>
       <c r="H15" t="n">
         <v>0</v>
@@ -967,13 +961,13 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>0.5275</v>
+        <v>0.5303</v>
       </c>
       <c r="F16" t="n">
-        <v>-0.0021</v>
+        <v>0.0007</v>
       </c>
       <c r="G16" t="n">
-        <v>-0.4</v>
+        <v>0.13</v>
       </c>
       <c r="H16" t="n">
         <v>0</v>
@@ -1031,20 +1025,20 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>81.8</v>
+        <v>81.75</v>
       </c>
       <c r="F18" t="n">
-        <v>0.55</v>
+        <v>-0.05</v>
       </c>
       <c r="G18" t="n">
-        <v>0.68</v>
+        <v>-0.06</v>
       </c>
       <c r="H18" t="n">
-        <v>26972500</v>
+        <v>22666158</v>
       </c>
     </row>
     <row r="19">
@@ -1065,20 +1059,20 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>78.68000000000001</v>
+        <v>78.67</v>
       </c>
       <c r="F19" t="n">
-        <v>0.15</v>
+        <v>-0.01</v>
       </c>
       <c r="G19" t="n">
-        <v>0.19</v>
+        <v>-0.01</v>
       </c>
       <c r="H19" t="n">
-        <v>44420000</v>
+        <v>29519116</v>
       </c>
     </row>
     <row r="20">
@@ -1103,16 +1097,16 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>4370.6001</v>
+        <v>4403.2002</v>
       </c>
       <c r="F20" t="n">
-        <v>-13.2998</v>
+        <v>19.3003</v>
       </c>
       <c r="G20" t="n">
-        <v>-0.3</v>
+        <v>0.44</v>
       </c>
       <c r="H20" t="n">
-        <v>104430</v>
+        <v>3177</v>
       </c>
     </row>
     <row r="21">
@@ -1137,16 +1131,16 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>90.06999999999999</v>
+        <v>89.63</v>
       </c>
       <c r="F21" t="n">
-        <v>-5.71</v>
+        <v>-6.15</v>
       </c>
       <c r="G21" t="n">
-        <v>-5.96</v>
+        <v>-6.42</v>
       </c>
       <c r="H21" t="n">
-        <v>162441</v>
+        <v>1700</v>
       </c>
     </row>
     <row r="22">
@@ -1171,16 +1165,16 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>98.63</v>
+        <v>98.52</v>
       </c>
       <c r="F22" t="n">
-        <v>-1.71</v>
+        <v>-1.82</v>
       </c>
       <c r="G22" t="n">
-        <v>-1.7</v>
+        <v>-1.81</v>
       </c>
       <c r="H22" t="n">
-        <v>22010</v>
+        <v>52</v>
       </c>
     </row>
     <row r="23">
@@ -1205,16 +1199,16 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>6.846</v>
+        <v>6.91</v>
       </c>
       <c r="F23" t="n">
-        <v>0.1595</v>
+        <v>0.2235</v>
       </c>
       <c r="G23" t="n">
-        <v>2.39</v>
+        <v>3.34</v>
       </c>
       <c r="H23" t="n">
-        <v>20449</v>
+        <v>428</v>
       </c>
     </row>
     <row r="24">
@@ -1235,20 +1229,20 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="E24" t="n">
-        <v>68.83</v>
+        <v>69.09999999999999</v>
       </c>
       <c r="F24" t="n">
-        <v>1.8</v>
+        <v>0.27</v>
       </c>
       <c r="G24" t="n">
-        <v>2.69</v>
+        <v>0.39</v>
       </c>
       <c r="H24" t="n">
-        <v>21966000</v>
+        <v>20103328</v>
       </c>
     </row>
     <row r="25">
@@ -1273,13 +1267,13 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>14.64</v>
+        <v>14.21</v>
       </c>
       <c r="F25" t="n">
-        <v>-0.23</v>
+        <v>-0.66</v>
       </c>
       <c r="G25" t="n">
-        <v>-1.55</v>
+        <v>-4.44</v>
       </c>
       <c r="H25" t="n">
         <v>0</v>
@@ -1307,16 +1301,16 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>85999.89840000001</v>
+        <v>86155.7812</v>
       </c>
       <c r="F26" t="n">
-        <v>-603.0155999999999</v>
+        <v>-447.1328</v>
       </c>
       <c r="G26" t="n">
-        <v>-0.7</v>
+        <v>-0.52</v>
       </c>
       <c r="H26" t="n">
-        <v>46771695616</v>
+        <v>40770478080</v>
       </c>
     </row>
     <row r="27">
@@ -1749,22 +1743,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Prabowo Minta Perjanjian Dagang dengan Eropa Dikebut</t>
+          <t>UU Reforma Agraria Disahkan, Aturan Batas Maksimal Pemilikan Tanah Disiapkan</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Tue, 22 Sep 2026 20:00:54 +0700</t>
+          <t>Wed, 23 Sep 2026 06:25:00 +0700</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/08/20/jaga-pertumbuhan-ekonomi-nasional-pemerintah-perkuat-sektor-strategis-1787215028622_169.jpeg?w=360&amp;amp;q=90" /&gt; Saat ini dokumen IEU-CEPA sedang dalam tahap finalisasi kelengkapan bahan berbahasa Inggris sebelum diserahkan ke Par</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/08/03/menteri-atrbpn-nusron-wahid-1785735730541_169.jpeg?w=360&amp;amp;q=90" /&gt; DPR mengesahkan Rancangan Undang-Undang (RUU) tentang Pengaturan Reforma Agraria menjadi Undang-Undang dalam rapat paripurna.</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8674608/prabowo-minta-perjanjian-dagang-dengan-eropa-dikebut</t>
+          <t>https://finance.detik.com/infrastruktur/d-8674670/uu-reforma-agraria-disahkan-aturan-batas-maksimal-pemilikan-tanah-disiapkan</t>
         </is>
       </c>
     </row>
@@ -1776,22 +1770,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Daftar Lengkap Perusahaan Dicabut Izinnya Usai Kebakaran Hutan</t>
+          <t>Uang Rupiah Bertanda Tangan Purbaya Diburu Warga</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Tue, 22 Sep 2026 19:38:26 +0700</t>
+          <t>Wed, 23 Sep 2026 05:55:00 +0700</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/08/31/menembus-asap-petugas-berjibaku-padamkan-karhutla-kalimantan-1788157037741_169.jpeg?w=360&amp;amp;q=90" /&gt; Pemerintah resmi mencabut izin lima perusahaan di Kalimantan Barat, Kalimantan Selatan, dan Kalimantan Tengah.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/22/ilustrasi-rupiah-1790057101049_169.jpeg?w=360&amp;amp;q=90" /&gt; Uang kertas rupiah yang memuat tanda tangan Purbaya Yudhi Sadewa mendadak viral dan disebut-sebut menjadi buruan bagi sebagian masyarakat.</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8674625/daftar-lengkap-perusahaan-dicabut-izinnya-usai-kebakaran-hutan</t>
+          <t>https://finance.detik.com/moneter/d-8674635/uang-rupiah-bertanda-tangan-purbaya-diburu-warga</t>
         </is>
       </c>
     </row>
@@ -1803,22 +1797,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Sempat Terputus Banjir Bandang, Ruas Jalan Padang-Solok Sudah Dapat Dilalui</t>
+          <t>Mau Terjun ke Dunia Pasar Modal? Yuk, Siapkan Diri Lewat Pelatihan WPPE</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Tue, 22 Sep 2026 19:34:37 +0700</t>
+          <t>Tue, 22 Sep 2026 23:32:52 +0700</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/22/jalan-solok-padang-1790080458278_169.jpeg?w=360&amp;amp;q=90" /&gt; Kementerian PU memastikan ruas jalan Padang-Solok pascabanjir bandang dapat dilalui. Pemulihan akses dilakukan bersama Forkopimda dan BUMN Infrastruktur.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/22/bnsp-wakil-perantaran-perdagangan-efek-1790094740378_169.jpeg?w=360&amp;amp;q=90" /&gt; Tertarik membangun karier di dunia pasar modal, tapi masih bingung harus mulai belajar dari mana?</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/infrastruktur/d-8674619/sempat-terputus-banjir-bandang-ruas-jalan-padang-solok-sudah-dapat-dilalui</t>
+          <t>https://finance.detik.com/bursa-dan-valas/d-8674845/mau-terjun-ke-dunia-pasar-modal-yuk-siapkan-diri-lewat-pelatihan-wppe</t>
         </is>
       </c>
     </row>
@@ -1830,22 +1824,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Diminta Prabowo Bantu Perpanjang LRT Jakarta, Danantara Buka Suara</t>
+          <t>Permintaan Tabung Oksigen Naik di Tengah Kabut Asap Palangka Raya</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Tue, 22 Sep 2026 19:01:16 +0700</t>
+          <t>Tue, 22 Sep 2026 23:00:51 +0700</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/04/coo-danantara-dony-oskaria-dan-direksi-ihc-1788531353185_169.jpeg?w=360&amp;amp;q=90" /&gt; Dony menyebut pihaknya tengah mengkaji rencana tersebut agar moda transportasi umum di ibu kota dapat terintegrasi secara utuh.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/22/permintaan-tabung-oksigen-di-palangka-raya-meningkat-1790061890912.jpeg?w=360&amp;amp;q=90" /&gt; Kabut asap akibat kebakaran hutan dan lahan melanda Palangka Raya.Permintaan tabung oksigen pun meningkat hingga tiga kali lipat.</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/infrastruktur/d-8674583/diminta-prabowo-bantu-perpanjang-lrt-jakarta-danantara-buka-suara</t>
+          <t>https://finance.detik.com/foto-bisnis/d-8674008/permintaan-tabung-oksigen-naik-di-tengah-kabut-asap-palangka-raya</t>
         </is>
       </c>
     </row>
@@ -1857,22 +1851,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>BUMN Tekstil Tak Kunjung Jadi, Bos Danantara: Kita Bikin Perusahaan Baru</t>
+          <t>Bitcoin Tembus US$ 87.000, Ini Sederet Pemicunya</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Tue, 22 Sep 2026 18:35:00 +0700</t>
+          <t>Tue, 22 Sep 2026 22:35:26 +0700</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/11/20/menteri-investasi-dan-hilirisasikepala-bkpm-rosan-roeslani-1763634019135_169.jpeg?w=360&amp;amp;q=90" /&gt; Sejak awal tahun rencana pembentukan BUMN tekstil tak kunjung terlaksana.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/07/20/mulai-investasi-di-exchange-crypto-2026-simak-tipsnya-untuk-pemula-1784542058111_169.png?w=360&amp;amp;q=90" /&gt; Harga Bitcoin (BTC) sempat menembus level tertinggi di US$ 87.000 pada perdagangan awal pekan.</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8674535/bumn-tekstil-tak-kunjung-jadi-bos-danantara-kita-bikin-perusahaan-baru</t>
+          <t>https://finance.detik.com/fintech/d-8674812/bitcoin-tembus-us-87-000-ini-sederet-pemicunya</t>
         </is>
       </c>
     </row>
@@ -1884,22 +1878,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Mendag Ancam Cabut Izin Pedagang yang Jual Minyakita di Atas HET</t>
+          <t>Efek El Nino, Kapasitas PLTA di Sulawesi Berkurang hingga 650 MW</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Tue, 22 Sep 2026 18:30:52 +0700</t>
+          <t>Tue, 22 Sep 2026 22:30:00 +0700</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/22/menteri-perdagangan-mendag-budi-santoso-1790064694064_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Perdagangan (Mendag) Budi Santoso memastikan terus mengawasi distribusi Minyakita.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2023/07/30/plta-balambano-di-luwu-timur_169.mpo?w=360&amp;amp;q=90" /&gt; Menteri ESDM Bahlil mengungkapkan dampak El Nino pada PLTA, mengurangi produksi listrik. PLN menambah kapasitas dengan pembangkit tenaga surya dan BESS.</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8674492/mendag-ancam-cabut-izin-pedagang-yang-jual-minyakita-di-atas-het</t>
+          <t>https://finance.detik.com/energi/d-8674607/efek-el-nino-kapasitas-plta-di-sulawesi-berkurang-hingga-650-mw</t>
         </is>
       </c>
     </row>
@@ -1911,22 +1905,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Melihat Kebun Kopi di Tengah Hutan Kota Jakarta</t>
+          <t>Situasi Global Memanas, Pertamina Perkuat Pasokan BBM-LPG</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Tue, 22 Sep 2026 18:03:20 +0700</t>
+          <t>Tue, 22 Sep 2026 22:14:14 +0700</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/22/melihat-kebun-kopi-di-tengah-hutan-kota-jakarta-1790060682921.jpeg?w=360&amp;amp;q=90" /&gt; Ribuan pohon kopi tumbuh di Hutan Kota Pesanggrahan Sangga Buana, Lebak Bulus, menjadi bagian dari upaya konservasi sekaligus edukasi.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2021/07/16/gedung-pertamina-pusat_169.jpeg?w=360&amp;amp;q=90" /&gt; Pertamina Patra Niaga memastikan terus memperkuat langkah pengamanan pasokan BBM dan LPG di tengah dinamika geopolitik global.</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/foto-bisnis/d-8673926/melihat-kebun-kopi-di-tengah-hutan-kota-jakarta</t>
+          <t>https://finance.detik.com/energi/d-8674786/situasi-global-memanas-pertamina-perkuat-pasokan-bbm-lpg</t>
         </is>
       </c>
     </row>
@@ -1938,22 +1932,22 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Tugas Khusus dari Prabowo ke Dirjen Bea Cukai: Perketat Perbatasan!</t>
+          <t>Pertamina Buka Suara soal Isu Orang Luar Intervensi Pengadaan BBM-LPG</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Tue, 22 Sep 2026 17:54:16 +0700</t>
+          <t>Tue, 22 Sep 2026 21:59:36 +0700</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/22/direktur-jenderal-bea-dan-cukai-kementerian-keuangan-djaka-budhi-utama-1790067626026_169.jpeg?w=360&amp;amp;q=90" /&gt; Dirjen Bea dan Cukai Kementerian Keuangan Djaka Budhi Utama buka-bukaan soal tugas dari Presiden Prabowo Subianto us</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/05/05/gedung-pertamina-1777965806138_169.jpeg?w=360&amp;amp;q=90" /&gt; Corporate Secretary Pertamina Patra Niaga, Roberth MV Dumatubun mengatakan Pertamina mengambil langkah strategis untuk eliminir intervensi.</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8674486/tugas-khusus-dari-prabowo-ke-dirjen-bea-cukai-perketat-perbatasan</t>
+          <t>https://finance.detik.com/energi/d-8674772/pertamina-buka-suara-soal-isu-orang-luar-intervensi-pengadaan-bbm-lpg</t>
         </is>
       </c>
     </row>
@@ -1965,22 +1959,22 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Pembatasan Pertalite Pakai Desil 9-10 Lanjut? Begini Jawaban Bahlil</t>
+          <t>Industri Tekstil Bakal Dapat Tax Holiday</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Tue, 22 Sep 2026 17:50:20 +0700</t>
+          <t>Tue, 22 Sep 2026 21:48:32 +0700</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/22/menteri-esdm-bahlil-lahadalia-1790052927263_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri ESDM Bahlil Lahadalia menegaskan pembatasan Pertalite untuk desil 9-10 masih dalam kajian. Data akurat diperlukan agar subsidi tepat sasaran.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/04/15/melihat-pameran-mesin-produksi-tekstil-di-jiexpo-kemayoran-1776240166100_169.jpeg?w=360&amp;amp;q=90" /&gt; CEO Danantara Rosan Roeslani menyampaikan pemerintah membuka peluang pemberian insentif fiskal berupa tax holiday untuk industri</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8674473/pembatasan-pertalite-pakai-desil-9-10-lanjut-begini-jawaban-bahlil</t>
+          <t>https://finance.detik.com/industri/d-8674761/industri-tekstil-bakal-dapat-tax-holiday</t>
         </is>
       </c>
     </row>
@@ -1992,22 +1986,22 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Bahlil Rayu Investor Bangun Data Center di RI: Pulau Kami Masih Terlalu Banyak</t>
+          <t>Balai Pengelolaan Dana Pengembangan Jalan Tol Dibentuk, Ini Fungsinya</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Tue, 22 Sep 2026 16:50:01 +0700</t>
+          <t>Tue, 22 Sep 2026 21:37:41 +0700</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/03/05/menteri-esdm-bahlil-lahadalia-1772707662547_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri ESDM Bahlil mengajak investor bangun data center di Indonesia, memanfaatkan luas wilayah dan sumber energi beragam.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2020/11/08/siap-siap-tol-cimanggis-cibitung-bakal-segera-dibuka-2_169.jpeg?w=360&amp;amp;q=90" /&gt; Kementerian Pekerjaan Umum (PU) membentuk Balai Pengelolaan Dana Pengembangan Jalan Tol sebagai Unit Pelaksana Teknis di bawah Direktorat Jenderal</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8674339/bahlil-rayu-investor-bangun-data-center-di-ri-pulau-kami-masih-terlalu-banyak</t>
+          <t>https://finance.detik.com/infrastruktur/d-8674749/balai-pengelolaan-dana-pengembangan-jalan-tol-dibentuk-ini-fungsinya</t>
         </is>
       </c>
     </row>
@@ -2019,22 +2013,22 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Pemerintah Siapkan Rp 3,29 T buat Tuntaskan 3 Proyek Tol</t>
+          <t>Pemerintah Sebut Tekstil Bukan Sunset Industry, Minta Bank BUMN Dukung Modal</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Tue, 22 Sep 2026 16:42:15 +0700</t>
+          <t>Tue, 22 Sep 2026 21:11:04 +0700</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2019/06/18/050ff4f1-b046-42ec-9c7d-f7cc933db6f2_169.jpeg?w=360&amp;amp;q=90" /&gt; Pemerintah mengalokasikan dukungan konstruksi untuk pembangunan tol sebesar Rp 3,29 triliun untuk tahun anggaran 2027.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/08/20/jaga-pertumbuhan-ekonomi-nasional-pemerintah-perkuat-sektor-strategis-1787215028622_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Koordinator Perekonomian Airlangga Hartarto menyampaikan Presiden Prabowo Subianto menegaskan industri teksti</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/infrastruktur/d-8674314/pemerintah-siapkan-rp-3-29-t-buat-tuntaskan-3-proyek-tol</t>
+          <t>https://finance.detik.com/industri/d-8674724/pemerintah-sebut-tekstil-bukan-sunset-industry-minta-bank-bumn-dukung-modal</t>
         </is>
       </c>
     </row>
@@ -2046,22 +2040,22 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Potret Warga Berburu Lowongan Kerja dari Puluhan Perusahaan di Cengkareng</t>
+          <t>Prabowo Mau Genjot Industri Tekstil, Begini Caranya</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Tue, 22 Sep 2026 16:30:00 +0700</t>
+          <t>Tue, 22 Sep 2026 20:30:00 +0700</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/22/potret-warga-berburu-lowongan-kerja-dari-puluhan-perusahaan-di-cengkareng-1790066353857_169.jpeg?w=360&amp;amp;q=90" /&gt; Job fair digelar di Gelanggang Remaja Cengkareng, Jakarta Barat. Sebanyak 37 perusahaan dan tiga instansi pemerin</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/04/15/melihat-pameran-mesin-produksi-tekstil-di-jiexpo-kemayoran-1776240166364_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Koordinator Perekonomian Airlangga Hartarto mengatakan industri TPT yang mencakup sektor hulu, antara, hingga hilir memi</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/foto-bisnis/d-8674153/potret-warga-berburu-lowongan-kerja-dari-puluhan-perusahaan-di-cengkareng</t>
+          <t>https://finance.detik.com/industri/d-8674657/prabowo-mau-genjot-industri-tekstil-begini-caranya</t>
         </is>
       </c>
     </row>
@@ -2073,22 +2067,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>IFG Life Sudah Bayar Klaim Rp 9,4 Triliun</t>
+          <t>PNM Dampingi Karyawan dan Nasabah Pascagempa NTT Lewat Trauma Healing</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Tue, 22 Sep 2026 16:28:15 +0700</t>
+          <t>Tue, 22 Sep 2026 20:26:04 +0700</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2024/12/31/ilustrasi-asuransi_169.jpeg?w=360&amp;amp;q=90" /&gt; IFG Life sudah bayar klaim Rp 9,4 triliun.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/22/pnm-1790083550132_169.jpeg?w=360&amp;amp;q=90" /&gt; PT Permodalan Nasional Madani (PNM) melalui program PNM Peduli memberikan dukungan trauma healing bagi karyawan dan nasabah terdampak gempa di NTT.</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/moneter/d-8674364/ifg-life-sudah-bayar-klaim-rp-9-4-triliun</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8674676/pnm-dampingi-karyawan-dan-nasabah-pascagempa-ntt-lewat-trauma-healing</t>
         </is>
       </c>
     </row>
@@ -2100,22 +2094,22 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>IHSG Ditutup Melemah ke Level 6.277, Turun 1,69%</t>
+          <t>Prabowo Minta Perjanjian Dagang dengan Eropa Dikebut</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Tue, 22 Sep 2026 16:23:00 +0700</t>
+          <t>Tue, 22 Sep 2026 20:00:54 +0700</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/05/22/ihsg-anjlok-ke-level-5000-sentuh-titik-terburuk-sejak-era-covid-19-1779437111616_169.jpeg?w=360&amp;amp;q=90" /&gt; Indeks Harga Saham Gabungan (IHSG) ditutup melemah pada perdagangan hari ini.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/08/20/jaga-pertumbuhan-ekonomi-nasional-pemerintah-perkuat-sektor-strategis-1787215028622_169.jpeg?w=360&amp;amp;q=90" /&gt; Saat ini dokumen IEU-CEPA sedang dalam tahap finalisasi kelengkapan bahan berbahasa Inggris sebelum diserahkan ke Par</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/bursa-dan-valas/d-8674270/ihsg-ditutup-melemah-ke-level-6-277-turun-1-69</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8674608/prabowo-minta-perjanjian-dagang-dengan-eropa-dikebut</t>
         </is>
       </c>
     </row>
@@ -2127,22 +2121,22 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Harga Minyak Mendidih, Mendag Waswas Neraca Dagang Tekor</t>
+          <t>Daftar Lengkap Perusahaan Dicabut Izinnya Usai Kebakaran Hutan</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Tue, 22 Sep 2026 16:14:30 +0700</t>
+          <t>Tue, 22 Sep 2026 19:38:26 +0700</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/22/menteri-perdagangan-mendag-budi-santoso-1790064694064_169.jpeg?w=360&amp;amp;q=90" /&gt; Harga minyak dunia sempat menembus level US$ 104 per barel pada perdagangan Senin (21/9) kemarin.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/08/31/menembus-asap-petugas-berjibaku-padamkan-karhutla-kalimantan-1788157037741_169.jpeg?w=360&amp;amp;q=90" /&gt; Pemerintah resmi mencabut izin lima perusahaan di Kalimantan Barat, Kalimantan Selatan, dan Kalimantan Tengah.</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8674256/harga-minyak-mendidih-mendag-waswas-neraca-dagang-tekor</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8674625/daftar-lengkap-perusahaan-dicabut-izinnya-usai-kebakaran-hutan</t>
         </is>
       </c>
     </row>
@@ -2154,22 +2148,22 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Hot Spot Kebakaran Hutan Turun, Kemenhut Ingatkan Waspada</t>
+          <t>Kisah 1 Jam Bersama Arbas, 'Jangan Pernah Sombong'</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Tue, 22 Sep 2026 19:46:24 +0700</t>
+          <t>Wed, 23 Sep 2026 06:30:43 +0700</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Jumlah hot spot karhutla nasional turun pada 21 September 2026 setelah sehari sebelumnya mencapai 1.988 titik.</t>
+          <t>Meski memenangkan banyak perlombaan, Arbas tak sungkan melihat karya fotografer lainnya.</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8297314/hot-spot-kebakaran-hutan-turun-kemenhut-ingatkan-waspada</t>
+          <t>https://www.liputan6.com/news/read/8297308/kisah-1-jam-bersama-arbas-jangan-pernah-sombong</t>
         </is>
       </c>
     </row>
@@ -2181,22 +2175,22 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Mobil Ugal-ugalan Sampai Naik Trotoar Lalu Tabrak 2 Pemotor</t>
+          <t>Gempa Magnitudo 4,6 Guncang Sumur Banten, Berpusat di Laut</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Tue, 22 Sep 2026 19:56:15 +0700</t>
+          <t>Wed, 23 Sep 2026 06:26:39 +0700</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Setelah menabrak sepeda motor Yamaha, Toyota Avanza tersebut kembali menabrak sepeda motor Honda</t>
+          <t>Pusat gempa berada di laut, sekitar 38 kilometer (km) sebelah selatan Sumur.</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8297316/mobil-ugal-ugalan-sampai-naik-trotoar-lalu-tabrak-2-pemotor</t>
+          <t>https://www.liputan6.com/news/read/8297481/gempa-magnitudo-46-guncang-sumur-banten-berpusat-di-laut</t>
         </is>
       </c>
     </row>
@@ -2208,22 +2202,22 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Bentuk Ditjen Pesantren, Menag Soroti Anggaran 42 Ribu Ponpes Belum Sepadan</t>
+          <t>OTT Bupati Bolmut, KPK Tegaskan Tak Pilih-Pilih Kasus</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Tue, 22 Sep 2026 19:43:47 +0700</t>
+          <t>Wed, 23 Sep 2026 06:12:16 +0700</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Menag mengatakan pembentukan Ditjen Pesantren menjadi langkah baru pemerintah untuk memperkuat keberadaan pesantren.</t>
+          <t>OTT Bupati Bolmut menjadi peringatan agar tidak beranggapan KPK hanya melakukan penindakan di kota-kota besar.</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8297311/bentuk-ditjen-pesantren-menag-soroti-anggaran-42-ribu-ponpes-belum-sepadan</t>
+          <t>https://www.liputan6.com/news/read/8297478/ott-bupati-bolmut-kpk-tegaskan-tak-pilih-pilih-kasus</t>
         </is>
       </c>
     </row>
@@ -2235,22 +2229,22 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Pertolongan Pertama Ketika Anda Tersedak</t>
+          <t>PKB Minta Jabatan Rektor UIN Surabaya Ditangguhkan</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Tue, 22 Sep 2026 19:08:44 +0700</t>
+          <t>Wed, 23 Sep 2026 06:16:04 +0700</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Tersedak bisa fatal. Pahami perbedaan pertolongan pertama untuk bayi, anak, dewasa, dan ibu hamil.</t>
+          <t>Maman menilai polemik pengangkatan rektor tidak cukup dijawab dengan prosedur formal.</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8297270/pertolongan-pertama-ketika-anda-tersedak</t>
+          <t>https://www.liputan6.com/news/read/8297477/pkb-minta-jabatan-rektor-uin-surabaya-ditangguhkan</t>
         </is>
       </c>
     </row>
@@ -2262,22 +2256,22 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Bupati Gowa Diperiksa Polisi, Kantor dan Rumah Jabatan Digeledah</t>
+          <t>Kepala Daerah dan Rasa Haus Pundi-Pundi Kekayaan</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Tue, 22 Sep 2026 19:04:47 +0700</t>
+          <t>Wed, 23 Sep 2026 05:00:05 +0700</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Bupati Gowa Sitti Husniah Talenrang telah diperiksa sebagai saksi setelah Polri menggeledah kantor dan rumah jabatannya.</t>
+          <t>Akar masalah korupsi disebut bukan hanya celah sistem, tetapi juga faktor personal dan kewenangan jabatan.</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8297275/bupati-gowa-diperiksa-polisi-kantor-dan-rumah-jabatan-digeledah</t>
+          <t>https://www.liputan6.com/news/read/8297205/kepala-daerah-dan-rasa-haus-pundi-pundi-kekayaan</t>
         </is>
       </c>
     </row>
@@ -2289,22 +2283,22 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Alasan KPK Baru Tetapkan 1 Tersangka dalam Korupsi Bupati Bolmut</t>
+          <t>Industri Pertambangan Diminta Perkuat Dekarbonisasi</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Tue, 22 Sep 2026 19:12:20 +0700</t>
+          <t>Tue, 22 Sep 2026 23:58:16 +0700</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Tersangka dalam perkara tersebut adalah Bupati Bolmut Sirajudin Lasena.</t>
+          <t>Industri pertambangan didorong melaporkan pengurangan emisi melalui SIGN-SMART untuk mendukung pemantauan pemerintah.</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8297286/alasan-kpk-baru-tetapkan-1-tersangka-dalam-korupsi-bupati-bolmut</t>
+          <t>https://www.liputan6.com/news/read/8297454/industri-pertambangan-diminta-perkuat-dekarbonisasi</t>
         </is>
       </c>
     </row>
@@ -2316,22 +2310,22 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Polemik Rektor UIN Sunan Ampel Ganggu Perkuliahan, Ini Respons Menag</t>
+          <t>Hari Santri 2026, Kemenag Buka Sayembara Surat untuk Presiden</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Tue, 22 Sep 2026 18:35:19 +0700</t>
+          <t>Tue, 22 Sep 2026 23:46:42 +0700</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Polemik Rektor Ganggu Kuliah Mahasiswa UIN Surabaya, Menag Siapkan Solusi</t>
+          <t>Santri berkesempatan menyampaikan mimpi, gagasan, dan harapan tentang masa depan bangsa melalui surat kepada Presiden.</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8297236/polemik-rektor-uin-sunan-ampel-ganggu-perkuliahan-ini-respons-menag</t>
+          <t>https://www.liputan6.com/news/read/8297448/hari-santri-2026-kemenag-buka-sayembara-surat-untuk-presiden</t>
         </is>
       </c>
     </row>
@@ -2343,22 +2337,22 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Cegah Penyelundupan, Prabowo Minta Bea Cukai Perketat Perbatasan dan Pesisir</t>
+          <t>Penyelam Tembus KM Virgo, Banyak Korban Terjebak di Kamar</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Tue, 22 Sep 2026 18:25:44 +0700</t>
+          <t>Tue, 22 Sep 2026 23:28:02 +0700</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Bea Cukai akan menambah peralatan serta memperketat satuan tugas (satgas) di lapangan.</t>
+          <t>Pencarian kini difokuskan pada badan KM Virgo, terutama kamar penumpang.</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8297231/cegah-penyelundupan-prabowo-minta-bea-cukai-perketat-perbatasan-dan-pesisir</t>
+          <t>https://www.liputan6.com/news/read/8297436/penyelam-tembus-km-virgo-banyak-korban-terjebak-di-kamar</t>
         </is>
       </c>
     </row>
@@ -2370,22 +2364,22 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Pejabat Bea Cukai Mangkir dari Panggilan KPK</t>
+          <t>BNPB Ungkap Kendala Pemadaman Kebakaran Hutan dari Udara</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Tue, 22 Sep 2026 18:14:48 +0700</t>
+          <t>Tue, 22 Sep 2026 23:04:57 +0700</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>KPK kembali memanggil Ahmad Dedi terkait dugaan korupsi DJBC. Namun, ia tidak hadir karena dikonfirmasi sedang sakit.</t>
+          <t>BNPB mengungkap kendala penanganan karhutla di Kalbar, mulai jarak pandang rendah hingga minimnya bibit awan.</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8297222/pejabat-bea-cukai-mangkir-dari-panggilan-kpk</t>
+          <t>https://www.liputan6.com/news/read/8297428/bnpb-ungkap-kendala-pemadaman-kebakaran-hutan-dari-udara</t>
         </is>
       </c>
     </row>
@@ -2397,22 +2391,22 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>DPRD DKI Soroti Desil Bansos, Biaya Hidup Jakarta Jadi Pertimbangan</t>
+          <t>Kronologi Kebakaran di Kebayoran Lama, Api Muncul dari Warteg</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Tue, 22 Sep 2026 18:15:05 +0700</t>
+          <t>Tue, 22 Sep 2026 23:04:07 +0700</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>DPRD DKI meminta parameter desil penerima bansos disesuaikan dengan karakteristik serta kondisi sosial ekonomi warga Jakarta.</t>
+          <t>Api pertama kali terlihat dari area warteg dan kemudian menjalar ke bangunan di belakangnya.</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8297223/dprd-dki-soroti-desil-bansos-biaya-hidup-jakarta-jadi-pertimbangan</t>
+          <t>https://www.liputan6.com/news/read/8297427/kronologi-kebakaran-di-kebayoran-lama-api-muncul-dari-warteg</t>
         </is>
       </c>
     </row>
@@ -2424,22 +2418,22 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Separuh Jalan di Bolmut Rusak Parah saat Bupati Sirajudin Memperkaya Diri</t>
+          <t>Kasus HGB Summarecon, KPK Usut Dugaan Aliran Dana Rp 106,3 M ke Nusron Wahid</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Tue, 22 Sep 2026 18:02:36 +0700</t>
+          <t>Tue, 22 Sep 2026 22:33:52 +0700</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Dalam kasus ini, Sirajudin diduga menerima gratifikasi total Rp 11,14 miliar dalam kurun waktu tahun 2023-2026.</t>
+          <t>Selain menelusuri aliran dana, KPK juga memetakan sumber penerimaan uang yang berkaitan dengan perkara tersebut.</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8297209/separuh-jalan-di-bolmut-rusak-parah-saat-bupati-sirajudin-memperkaya-diri</t>
+          <t>https://www.liputan6.com/news/read/8297413/kasus-hgb-summarecon-kpk-usut-dugaan-aliran-dana-rp-1063-m-ke-nusron-wahid</t>
         </is>
       </c>
     </row>
@@ -2451,22 +2445,22 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>100 Satwa Liar Diselamatkan dari Kebakaran Hutan, Orangutan Mendominasi</t>
+          <t>Infografis: Tahapan Pertolongan Saat Tersedak</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Tue, 22 Sep 2026 17:52:03 +0700</t>
+          <t>Tue, 22 Sep 2026 21:56:59 +0700</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Dari 100 satwa liar yang diselamatkan, 53 di antaranya orangutan yang berada di sejumlah wilayah Kalimantan.</t>
+          <t>Tersedak bisa berubah menjadi kondisi darurat dalam hitungan menit. Lantas, apa yang harus dilakukan saat korban tak bisa bernapas?</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8297202/100-satwa-liar-diselamatkan-dari-kebakaran-hutan-orangutan-mendominasi</t>
+          <t>https://www.liputan6.com/news/read/8297393/infografis-tahapan-pertolongan-saat-tersedak</t>
         </is>
       </c>
     </row>
@@ -2478,22 +2472,22 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Divonis 7 Tahun, Pelaku Kekerasan Seksual Santriwati Sudah Dibebaskan</t>
+          <t>Kebakaran Rumah di Kebayoran Lama, 128 Personel Dikerahkan</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Tue, 22 Sep 2026 17:32:42 +0700</t>
+          <t>Tue, 22 Sep 2026 21:42:17 +0700</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Investigasi BBC mengungkapkan Bechi hanya menjalani 3 tahun dari hukuman 7 tahun penjara.</t>
+          <t>Status kebakaran tercatat dalam kategori merah atau masih dalam proses pemadaman.</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8297026/divonis-7-tahun-pelaku-kekerasan-seksual-santriwati-sudah-dibebaskan</t>
+          <t>https://www.liputan6.com/news/read/8297385/kebakaran-rumah-di-kebayoran-lama-128-personel-dikerahkan</t>
         </is>
       </c>
     </row>
@@ -2505,22 +2499,22 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Banjir Bandang Terjang Solok, Puan Soroti Mitigasi Bencana</t>
+          <t>Banjir Bandang Solok, 2 Orang Hilang dan Jembatan Sempat Terputus</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Tue, 22 Sep 2026 17:29:59 +0700</t>
+          <t>Tue, 22 Sep 2026 21:23:41 +0700</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Puan menyoroti ancaman bencana saat musim hujan dan meminta pemerintah memastikan kebutuhan warga terdampak terpenuhi.</t>
+          <t>Banjir bandang di Solok menyebabkan dua orang belum ditemukan, tiga warga luka ringan, dan sekitar 50 orang mengungsi.</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8297187/banjir-bandang-terjang-solok-puan-soroti-mitigasi-bencana</t>
+          <t>https://www.liputan6.com/news/read/8297374/banjir-bandang-solok-2-orang-hilang-dan-jembatan-sempat-terputus</t>
         </is>
       </c>
     </row>
@@ -2532,22 +2526,22 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Konstruksi Kasus Korupsi Bupati Bolmut Sirajudin Lasena</t>
+          <t>Penjelasan Pemerintah soal Isu Manajer Kopdes Langsung Jadi Pegawai BUMN</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Tue, 22 Sep 2026 17:02:32 +0700</t>
+          <t>Tue, 22 Sep 2026 21:06:03 +0700</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Bupati Bolmut Sirajudin Lasena diduga mematok fee proyek sebesar 10 persen.</t>
+          <t>Menurut Dony, para manajer Kopdes Merah Putih akan dibina dan ditugaskan selama dua tahun di koperasi.</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8297157/konstruksi-kasus-korupsi-bupati-bolmut-sirajudin-lasena</t>
+          <t>https://www.liputan6.com/news/read/8297366/penjelasan-pemerintah-soal-isu-manajer-kopdes-langsung-jadi-pegawai-bumn</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data pasar & berita - 2026-10-08 01:22 UTC
</commit_message>
<xml_diff>
--- a/data/market_news_latest.xlsx
+++ b/data/market_news_latest.xlsx
@@ -487,20 +487,20 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>6146.7241</v>
+        <v>6192.9268</v>
       </c>
       <c r="F2" t="n">
-        <v>-46.2026</v>
+        <v>74.0669</v>
       </c>
       <c r="G2" t="n">
-        <v>-0.75</v>
+        <v>1.21</v>
       </c>
       <c r="H2" t="n">
-        <v>0</v>
+        <v>464436200</v>
       </c>
     </row>
     <row r="3">
@@ -525,16 +525,16 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>7774.8799</v>
+        <v>7801.77</v>
       </c>
       <c r="F3" t="n">
-        <v>-44.0503</v>
+        <v>-17.1602</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.5600000000000001</v>
+        <v>-0.22</v>
       </c>
       <c r="H3" t="n">
-        <v>761743993</v>
+        <v>2648837000</v>
       </c>
     </row>
     <row r="4">
@@ -559,16 +559,16 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>50980.5312</v>
+        <v>51179.8711</v>
       </c>
       <c r="F4" t="n">
-        <v>-540.75</v>
+        <v>-341.4102</v>
       </c>
       <c r="G4" t="n">
-        <v>-1.05</v>
+        <v>-0.66</v>
       </c>
       <c r="H4" t="n">
-        <v>117680252</v>
+        <v>364125864</v>
       </c>
     </row>
     <row r="5">
@@ -593,16 +593,16 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>27417.9648</v>
+        <v>27538.6914</v>
       </c>
       <c r="F5" t="n">
-        <v>-181.8242</v>
+        <v>-61.0977</v>
       </c>
       <c r="G5" t="n">
-        <v>-0.66</v>
+        <v>-0.22</v>
       </c>
       <c r="H5" t="n">
-        <v>2603745000</v>
+        <v>6457816000</v>
       </c>
     </row>
     <row r="6">
@@ -623,20 +623,20 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>70683.97659999999</v>
+        <v>69289.0938</v>
       </c>
       <c r="F6" t="n">
-        <v>737.1172</v>
+        <v>-1394.8828</v>
       </c>
       <c r="G6" t="n">
-        <v>1.05</v>
+        <v>-1.97</v>
       </c>
       <c r="H6" t="n">
-        <v>149100000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -657,20 +657,20 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>24130.5</v>
+        <v>24280.5605</v>
       </c>
       <c r="F7" t="n">
-        <v>-150.0605</v>
+        <v>240.2207</v>
       </c>
       <c r="G7" t="n">
-        <v>-0.62</v>
+        <v>1</v>
       </c>
       <c r="H7" t="n">
-        <v>0</v>
+        <v>1292200000</v>
       </c>
     </row>
     <row r="8">
@@ -725,20 +725,20 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>10457.7998</v>
+        <v>10541.7002</v>
       </c>
       <c r="F9" t="n">
-        <v>-83.9004</v>
+        <v>43.7998</v>
       </c>
       <c r="G9" t="n">
-        <v>-0.8</v>
+        <v>0.42</v>
       </c>
       <c r="H9" t="n">
-        <v>0</v>
+        <v>717797000</v>
       </c>
     </row>
     <row r="10">
@@ -759,20 +759,20 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>25070.6094</v>
+        <v>25449.1895</v>
       </c>
       <c r="F10" t="n">
-        <v>-378.5801</v>
+        <v>194.9785</v>
       </c>
       <c r="G10" t="n">
-        <v>-1.49</v>
+        <v>0.77</v>
       </c>
       <c r="H10" t="n">
-        <v>0</v>
+        <v>42539000</v>
       </c>
     </row>
     <row r="11">
@@ -793,17 +793,17 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>5608.4399</v>
+        <v>5524.4502</v>
       </c>
       <c r="F11" t="n">
-        <v>-93.1001</v>
+        <v>-177.0898</v>
       </c>
       <c r="G11" t="n">
-        <v>-1.63</v>
+        <v>-3.11</v>
       </c>
       <c r="H11" t="n">
         <v>0</v>
@@ -827,17 +827,17 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>17878</v>
+        <v>17875</v>
       </c>
       <c r="F12" t="n">
-        <v>-9.900399999999999</v>
+        <v>46</v>
       </c>
       <c r="G12" t="n">
-        <v>-0.06</v>
+        <v>0.26</v>
       </c>
       <c r="H12" t="n">
         <v>0</v>
@@ -865,13 +865,13 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>102.259</v>
+        <v>102.247</v>
       </c>
       <c r="F13" t="n">
-        <v>0.429</v>
+        <v>0.417</v>
       </c>
       <c r="G13" t="n">
-        <v>0.42</v>
+        <v>0.41</v>
       </c>
       <c r="H13" t="n">
         <v>0</v>
@@ -895,17 +895,17 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>158.159</v>
+        <v>157.833</v>
       </c>
       <c r="F14" t="n">
-        <v>0.196</v>
+        <v>-0.463</v>
       </c>
       <c r="G14" t="n">
-        <v>0.12</v>
+        <v>-0.29</v>
       </c>
       <c r="H14" t="n">
         <v>0</v>
@@ -933,13 +933,13 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>0.5305</v>
+        <v>0.5276999999999999</v>
       </c>
       <c r="F15" t="n">
-        <v>0.0036</v>
+        <v>0.0008</v>
       </c>
       <c r="G15" t="n">
-        <v>0.68</v>
+        <v>0.15</v>
       </c>
       <c r="H15" t="n">
         <v>0</v>
@@ -967,13 +967,13 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>0.5681</v>
+        <v>0.5661</v>
       </c>
       <c r="F16" t="n">
-        <v>0.004</v>
+        <v>0.002</v>
       </c>
       <c r="G16" t="n">
-        <v>0.71</v>
+        <v>0.35</v>
       </c>
       <c r="H16" t="n">
         <v>0</v>
@@ -1001,13 +1001,13 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>0.4043</v>
+        <v>0.4037</v>
       </c>
       <c r="F17" t="n">
-        <v>0.0005999999999999999</v>
+        <v>-0</v>
       </c>
       <c r="G17" t="n">
-        <v>0.15</v>
+        <v>-0</v>
       </c>
       <c r="H17" t="n">
         <v>0</v>
@@ -1034,17 +1034,11 @@
           <t>2026-10-07</t>
         </is>
       </c>
-      <c r="E18" t="n">
-        <v>76.855</v>
-      </c>
-      <c r="F18" t="n">
-        <v>-0.425</v>
-      </c>
-      <c r="G18" t="n">
-        <v>-0.55</v>
-      </c>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
       <c r="H18" t="n">
-        <v>16635141</v>
+        <v>39684163</v>
       </c>
     </row>
     <row r="19">
@@ -1068,17 +1062,11 @@
           <t>2026-10-07</t>
         </is>
       </c>
-      <c r="E19" t="n">
-        <v>77.035</v>
-      </c>
-      <c r="F19" t="n">
-        <v>-0.235</v>
-      </c>
-      <c r="G19" t="n">
-        <v>-0.3</v>
-      </c>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr"/>
       <c r="H19" t="n">
-        <v>28482219</v>
+        <v>59233080</v>
       </c>
     </row>
     <row r="20">
@@ -1103,16 +1091,16 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>4131</v>
+        <v>4149.7998</v>
       </c>
       <c r="F20" t="n">
-        <v>-56.1001</v>
+        <v>-37.3003</v>
       </c>
       <c r="G20" t="n">
-        <v>-1.34</v>
+        <v>-0.89</v>
       </c>
       <c r="H20" t="n">
-        <v>119281</v>
+        <v>13359</v>
       </c>
     </row>
     <row r="21">
@@ -1137,16 +1125,16 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>89.79000000000001</v>
+        <v>89.40000000000001</v>
       </c>
       <c r="F21" t="n">
-        <v>0.35</v>
+        <v>-0.04</v>
       </c>
       <c r="G21" t="n">
-        <v>0.39</v>
+        <v>-0.04</v>
       </c>
       <c r="H21" t="n">
-        <v>129689</v>
+        <v>5991</v>
       </c>
     </row>
     <row r="22">
@@ -1171,16 +1159,16 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>101.84</v>
+        <v>101.54</v>
       </c>
       <c r="F22" t="n">
-        <v>1.26</v>
+        <v>0.96</v>
       </c>
       <c r="G22" t="n">
-        <v>1.25</v>
+        <v>0.95</v>
       </c>
       <c r="H22" t="n">
-        <v>27340</v>
+        <v>1164</v>
       </c>
     </row>
     <row r="23">
@@ -1205,16 +1193,16 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>6.653</v>
+        <v>6.713</v>
       </c>
       <c r="F23" t="n">
-        <v>0.0585</v>
+        <v>0.1185</v>
       </c>
       <c r="G23" t="n">
-        <v>0.89</v>
+        <v>1.8</v>
       </c>
       <c r="H23" t="n">
-        <v>25778</v>
+        <v>2956</v>
       </c>
     </row>
     <row r="24">
@@ -1238,17 +1226,11 @@
           <t>2026-10-07</t>
         </is>
       </c>
-      <c r="E24" t="n">
-        <v>67.265</v>
-      </c>
-      <c r="F24" t="n">
-        <v>-1.005</v>
-      </c>
-      <c r="G24" t="n">
-        <v>-1.47</v>
-      </c>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr"/>
       <c r="H24" t="n">
-        <v>5730572</v>
+        <v>17155771</v>
       </c>
     </row>
     <row r="25">
@@ -1273,13 +1255,13 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>15.68</v>
+        <v>15.08</v>
       </c>
       <c r="F25" t="n">
-        <v>0.67</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="G25" t="n">
-        <v>4.46</v>
+        <v>0.47</v>
       </c>
       <c r="H25" t="n">
         <v>0</v>
@@ -1303,20 +1285,20 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="E26" t="n">
-        <v>82989.2812</v>
+        <v>83136.25780000001</v>
       </c>
       <c r="F26" t="n">
-        <v>-2568.2812</v>
+        <v>-2421.3047</v>
       </c>
       <c r="G26" t="n">
-        <v>-3</v>
+        <v>-2.83</v>
       </c>
       <c r="H26" t="n">
-        <v>38036103168</v>
+        <v>39172456448</v>
       </c>
     </row>
     <row r="27">
@@ -1749,22 +1731,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>OJK Cabut Izin Usaha BTPN Syariah Ventura, Likuidasi Sedang Berjalan</t>
+          <t>Harga Minyak Masih Betah di US$ 100 per Barel</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Wed, 07 Oct 2026 21:32:17 +0700</t>
+          <t>Thu, 08 Oct 2026 07:40:44 +0700</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2016/12/30/ed5ec33a-5357-40f8-8f66-6713c06687ea_169.jpg?w=360&amp;amp;q=90" /&gt; Otoritas Jasa Keuangan (OJK) telah mencabut izin usaha perusahaan modal ventura Syariah PT BTPN Syariah Ventura. Saat ini, proses likuidasi sedang berjalan.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2023/08/16/ilustrasi-pengeboran-migas_169.jpeg?w=360&amp;amp;q=90" /&gt; Badan Energi Internasional (International Energy Agency/IEA) sepakat untuk mempercepat pelepasan stok minyak ke pasar.</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/moneter/d-8697158/ojk-cabut-izin-usaha-btpn-syariah-ventura-likuidasi-sedang-berjalan</t>
+          <t>https://finance.detik.com/energi/d-8697313/harga-minyak-masih-betah-di-us-100-per-barel</t>
         </is>
       </c>
     </row>
@@ -1776,22 +1758,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Mengenalkan Maritim-Literasi ke Generasi Muda Lewat Cara Fun</t>
+          <t>Hitungan Buruh Minta Upah Minimum 2027 Naik 9,5%</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Wed, 07 Oct 2026 21:00:19 +0700</t>
+          <t>Thu, 08 Oct 2026 07:00:54 +0700</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/07/mengenalkan-maritim-literasi-ke-generasi-muda-lewat-cara-fun-1791379146358.jpeg?w=360&amp;amp;q=90" /&gt; Pertamina International Shipping menggelar Bahtera LiteraSEA di TIM. Kegiatan ini mengajak pelajar mengenal dunia maritim secara i</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/04/16/demo-buruh-di-surabaya-1776329957688_169.jpeg?w=360&amp;amp;q=90" /&gt; Kalangan buruh mulai menyodorkan usulan angka kenaikan upah minimum untuk tahun 2027.</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/foto-bisnis/d-8697076/mengenalkan-maritim-literasi-ke-generasi-muda-lewat-cara-fun</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8697152/hitungan-buruh-minta-upah-minimum-2027-naik-9-5</t>
         </is>
       </c>
     </row>
@@ -1803,22 +1785,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Pemerintah Kejar Pertumbuhan Ekonomi 6%, Pakai Jurus Ini</t>
+          <t>OJK &amp;amp; LPS Angkat Bicara soal Rencana Gaji PNS Lewat Koperasi</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Wed, 07 Oct 2026 20:37:04 +0700</t>
+          <t>Thu, 08 Oct 2026 06:30:41 +0700</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2021/05/27/bangkit-dari-pandemi-ekonomi-ri-kuartal-ii-2021-diramal-tembus-7-1_169.jpeg?w=360&amp;amp;q=90" /&gt; Wakil Menteri Koordinator (Wamenko) Perekonomian Dradjad Hari Wibowo membeberkan strategi mengejar pertumbuhan ekonomi 6% tahun depan.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2023/02/23/ilustrasi-pns_169.jpeg?w=360&amp;amp;q=90" /&gt; Pemerintah berencana memperluas peran koperasi sebagai penyalur gaji pegawai negeri sipil (PNS) dan pembayaran pensiun.</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8697096/pemerintah-kejar-pertumbuhan-ekonomi-6-pakai-jurus-ini</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8697140/ojk-lps-angkat-bicara-soal-rencana-gaji-pns-lewat-koperasi</t>
         </is>
       </c>
     </row>
@@ -1830,22 +1812,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Penjelasan Pengusaha soal Usulan Waktu Kerja 45 Jam/ Minggu</t>
+          <t>Bahlil Bicara Rangkap Jabatan Menteri, Gajinya Dobel?</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Wed, 07 Oct 2026 20:00:23 +0700</t>
+          <t>Thu, 08 Oct 2026 05:55:39 +0700</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/08/21/ketua-umum-asosiasi-pengusaha-indonesia-apindo-shinta-kamdani-1787293865409_169.jpeg?w=360&amp;amp;q=90" /&gt; Shinta mengatakan usulan ini menjadi sorotan karena dinilai adanya kesalahpahaman penafsiran.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/08/04/bahlil-lahadalia-1785840108228_169.jpeg?w=360&amp;amp;q=90" /&gt; Bahlil Lahadalia menjelaskan perannya sebagai Menko Hilirisasi dan ESDM. Ia menegaskan hanya menerima satu gaji untuk menghindari pemborosan anggaran.</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8697011/penjelasan-pengusaha-soal-usulan-waktu-kerja-45-jam-minggu</t>
+          <t>https://finance.detik.com/energi/d-8697131/bahlil-bicara-rangkap-jabatan-menteri-gajinya-dobel</t>
         </is>
       </c>
     </row>
@@ -1857,22 +1839,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Luhut Minta Investor Tak Ragu: Indonesia Tidak Akan Kolaps!</t>
+          <t>Masih Catat Transaksi Manual? Saatnya Kenalan dengan Accurate Biar Laporan Rapi</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Wed, 07 Oct 2026 19:30:27 +0700</t>
+          <t>Wed, 07 Oct 2026 23:32:17 +0700</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/08/20/ketua-den-luhut-binsar-pandjaitan-dan-kepala-bgn-sudaryono-1787233734124_169.jpeg?w=360&amp;amp;q=90" /&gt; Ketua Dewan Ekonomi Nasional (DEN) Luhut Binsar Pandjaitan meminta agar para investor untuk jangan ragu menanamkan modalnya ke I</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/07/accurate-online-b14-1791381301555_169.png?w=360&amp;amp;q=90" /&gt; Pengelolaan keuangan yang presisi dan minim risiko error jadi kebutuhan, dan software akuntansi seperti Accurate membantu mewujudkannya.</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8696992/luhut-minta-investor-tak-ragu-indonesia-tidak-akan-kolaps</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8697221/masih-catat-transaksi-manual-saatnya-kenalan-dengan-accurate-biar-laporan-rapi</t>
         </is>
       </c>
     </row>
@@ -1884,22 +1866,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Hashim Sebut Indonesia Makin Terang Jika Harga Minyak Dunia Turun</t>
+          <t>Masih Hitung Manual? 7 Skill Excel Ini Bikin Laporan Keuangan Lebih Cepat</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Wed, 07 Oct 2026 19:00:21 +0700</t>
+          <t>Wed, 07 Oct 2026 23:28:01 +0700</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/06/utusan-khusus-presiden-bidang-iklim-dan-energi-hashim-djojohadikusumo-1791262508691_169.jpeg?w=360&amp;amp;q=90" /&gt; Utusan Khusus Presiden Hashim Djojohadikusumo menegaskan Indonesia dalam kondisi terang, meski harga minyak dunia ber</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/08/15/excel-accounting-1786812755686_169.png?w=360&amp;amp;q=90" /&gt; Di dunia kerja yang makin berbasis data, kemampuan Excel sudah dianggap standar, bukan lagi nilai tambah.</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8696903/hashim-sebut-indonesia-makin-terang-jika-harga-minyak-dunia-turun</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8697220/masih-hitung-manual-7-skill-excel-ini-bikin-laporan-keuangan-lebih-cepat</t>
         </is>
       </c>
     </row>
@@ -1911,22 +1893,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Shopee Hadirkan 2 Inovasi Baru Bantu UMKM Atur Harga hingga Jualan Live</t>
+          <t>Utang di Bawah Rp 1 Juta Tak Masuk SLIK, OJK Beri Penjelasan</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Wed, 07 Oct 2026 18:31:19 +0700</t>
+          <t>Wed, 07 Oct 2026 22:27:21 +0700</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/07/shopee-1791372512087_169.jpeg?w=360&amp;amp;q=90" /&gt; Shopee dorong UMKM dengan inovasi Kalkulator Biaya dan Shopee Live Studio. Fokus pada produk lokal, transparansi biaya, dan perluasan pasar.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/05/07/ilustrasi-cicilan-rumah-1778123144660_169.jpeg?w=360&amp;amp;q=90" /&gt; Otoritas Jasa Keuangan (OJK) telah memutuskan utang dengan nominal di bawah Rp 1 juta tidak ditampilkan dalam laporan Sistem Layanan Informasi Keuangan (SLIK).</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8696923/shopee-hadirkan-2-inovasi-baru-bantu-umkm-atur-harga-hingga-jualan-live</t>
+          <t>https://finance.detik.com/moneter/d-8697194/utang-di-bawah-rp-1-juta-tak-masuk-slik-ojk-beri-penjelasan</t>
         </is>
       </c>
     </row>
@@ -1938,22 +1920,22 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Luhut soal Subsidi Barang Diganti Cash: Bertahap</t>
+          <t>OJK Cabut Izin Usaha BTPN Syariah Ventura, Likuidasi Sedang Berjalan</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Wed, 07 Oct 2026 18:30:42 +0700</t>
+          <t>Wed, 07 Oct 2026 21:32:17 +0700</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/10/ketua-komite-percepatan-transformasi-digital-pemerintah-luhut-binsar-pandjaitan-1789019836285_169.jpeg?w=360&amp;amp;q=90" /&gt; Penyaluran subsidi yang biasanya diberikan dalam bentuk barang akan diubah menjadi bantuan langsung tunai (</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2016/12/30/ed5ec33a-5357-40f8-8f66-6713c06687ea_169.jpg?w=360&amp;amp;q=90" /&gt; Otoritas Jasa Keuangan (OJK) telah mencabut izin usaha perusahaan modal ventura Syariah PT BTPN Syariah Ventura. Saat ini, proses likuidasi sedang berjalan.</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8696894/luhut-soal-subsidi-barang-diganti-cash-bertahap</t>
+          <t>https://finance.detik.com/moneter/d-8697158/ojk-cabut-izin-usaha-btpn-syariah-ventura-likuidasi-sedang-berjalan</t>
         </is>
       </c>
     </row>
@@ -1965,22 +1947,22 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Samator Tingkatkan Keandalan Specialty Gas untuk Industri-Laboratorium</t>
+          <t>Mengenalkan Maritim-Literasi ke Generasi Muda Lewat Cara Fun</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Wed, 07 Oct 2026 18:22:40 +0700</t>
+          <t>Wed, 07 Oct 2026 21:00:19 +0700</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/07/ilustrasi-gas-produksi-samator-1791372135858.jpeg?w=360&amp;amp;q=90" /&gt; PT Samator Indo Gas Tbk perkuat kapabilitas dengan akreditasi ISO/IEC 17025:2017. Ini mendukung kualitas produk specialty gas untuk industri.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/07/mengenalkan-maritim-literasi-ke-generasi-muda-lewat-cara-fun-1791379146358.jpeg?w=360&amp;amp;q=90" /&gt; Pertamina International Shipping menggelar Bahtera LiteraSEA di TIM. Kegiatan ini mengajak pelajar mengenal dunia maritim secara i</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8696909/samator-tingkatkan-keandalan-specialty-gas-untuk-industri-laboratorium</t>
+          <t>https://finance.detik.com/foto-bisnis/d-8697076/mengenalkan-maritim-literasi-ke-generasi-muda-lewat-cara-fun</t>
         </is>
       </c>
     </row>
@@ -1992,22 +1974,22 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>KAI Mau Impor Kereta Bekas Jepang,  Begini Respons AHY</t>
+          <t>Pemerintah Kejar Pertumbuhan Ekonomi 6%, Pakai Jurus Ini</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Wed, 07 Oct 2026 18:09:05 +0700</t>
+          <t>Wed, 07 Oct 2026 20:37:04 +0700</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/14/menteri-koordinator-bidang-infrastruktur-dan-pembangunan-kewilayahan-agus-harimurti-yudhoyono-ahy-1789371416249_169.jpeg?w=360&amp;amp;q=90" /&gt; AHY mengaku belum bisa memberikan komentar terlalu jauh terkait rencana tersebut.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2021/05/27/bangkit-dari-pandemi-ekonomi-ri-kuartal-ii-2021-diramal-tembus-7-1_169.jpeg?w=360&amp;amp;q=90" /&gt; Wakil Menteri Koordinator (Wamenko) Perekonomian Dradjad Hari Wibowo membeberkan strategi mengejar pertumbuhan ekonomi 6% tahun depan.</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/infrastruktur/d-8696889/kai-mau-impor-kereta-bekas-jepang-begini-respons-ahy</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8697096/pemerintah-kejar-pertumbuhan-ekonomi-6-pakai-jurus-ini</t>
         </is>
       </c>
     </row>
@@ -2019,22 +2001,22 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>KemenUMKM Puji Kalkulator Biaya Shopee, Seller Kini Bisa Simulasi Margin</t>
+          <t>Penjelasan Pengusaha soal Usulan Waktu Kerja 45 Jam/ Minggu</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Wed, 07 Oct 2026 18:05:15 +0700</t>
+          <t>Wed, 07 Oct 2026 20:00:23 +0700</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/07/sea-group-1791371093464_169.png?w=360&amp;amp;q=90" /&gt; Shopee luncurkan fitur Kalkulator Biaya untuk seller, memudahkan perhitungan harga jual dan margin. Kementerian UMKM apresiasi dukungan untuk pengusaha lokal.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/08/21/ketua-umum-asosiasi-pengusaha-indonesia-apindo-shinta-kamdani-1787293865409_169.jpeg?w=360&amp;amp;q=90" /&gt; Shinta mengatakan usulan ini menjadi sorotan karena dinilai adanya kesalahpahaman penafsiran.</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8696866/kemenumkm-puji-kalkulator-biaya-shopee-seller-kini-bisa-simulasi-margin</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8697011/penjelasan-pengusaha-soal-usulan-waktu-kerja-45-jam-minggu</t>
         </is>
       </c>
     </row>
@@ -2046,22 +2028,22 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>bank bjb Perkuat Dukungan bagi Komunitas PERSIB Lewat Kartu ATM Edisi PERSIB</t>
+          <t>Luhut Minta Investor Tak Ragu: Indonesia Tidak Akan Kolaps!</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Wed, 07 Oct 2026 17:53:34 +0700</t>
+          <t>Wed, 07 Oct 2026 19:30:27 +0700</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/07/bank-bjb-1791370394240_169.jpeg?w=360&amp;amp;q=90" /&gt; Bank bjb rilis Kartu ATM Edisi PERSIB untuk mendekatkan layanan perbankan dengan komunitas. Nikmati kemudahan transaksi dan semangat PERSIB dalam sehari-hari.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/08/20/ketua-den-luhut-binsar-pandjaitan-dan-kepala-bgn-sudaryono-1787233734124_169.jpeg?w=360&amp;amp;q=90" /&gt; Ketua Dewan Ekonomi Nasional (DEN) Luhut Binsar Pandjaitan meminta agar para investor untuk jangan ragu menanamkan modalnya ke I</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/moneter/d-8696838/bank-bjb-perkuat-dukungan-bagi-komunitas-persib-lewat-kartu-atm-edisi-persib</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8696992/luhut-minta-investor-tak-ragu-indonesia-tidak-akan-kolaps</t>
         </is>
       </c>
     </row>
@@ -2073,22 +2055,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Dukung Program Pemerintah, bank bjb Perluas Akses Kredit Perumahan Warga-UMKM</t>
+          <t>Hashim Sebut Indonesia Makin Terang Jika Harga Minyak Dunia Turun</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Wed, 07 Oct 2026 17:05:51 +0700</t>
+          <t>Wed, 07 Oct 2026 19:00:21 +0700</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/07/bank-bjb-1791367537990_169.png?w=360&amp;amp;q=90" /&gt; Bank bjb memperkuat komitmen dukung program perumahan pemerintah dengan sosialisasi kredit perumahan dan subsidi.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/06/utusan-khusus-presiden-bidang-iklim-dan-energi-hashim-djojohadikusumo-1791262508691_169.jpeg?w=360&amp;amp;q=90" /&gt; Utusan Khusus Presiden Hashim Djojohadikusumo menegaskan Indonesia dalam kondisi terang, meski harga minyak dunia ber</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8696751/dukung-program-pemerintah-bank-bjb-perluas-akses-kredit-perumahan-warga-umkm</t>
+          <t>https://finance.detik.com/energi/d-8696903/hashim-sebut-indonesia-makin-terang-jika-harga-minyak-dunia-turun</t>
         </is>
       </c>
     </row>
@@ -2100,22 +2082,22 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Proyek Giant Sea Wall Bakal Groundbreaking di Demak, Diawali Tanam Mangrove</t>
+          <t>Shopee Hadirkan 2 Inovasi Baru Bantu UMKM Atur Harga hingga Jualan Live</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Wed, 07 Oct 2026 16:57:46 +0700</t>
+          <t>Wed, 07 Oct 2026 18:31:19 +0700</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/04/22/ahy-dorong-percepatan-pengembangan-kereta-api-di-sumatera-sulawesi-1776841867228_169.jpeg?w=360&amp;amp;q=90" /&gt; Untuk kawasan pesisir Demak, pemerintah memilih untuk mengawali dengan program berbasis alam, yakni penanaman mangrove.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/07/shopee-1791372512087_169.jpeg?w=360&amp;amp;q=90" /&gt; Shopee dorong UMKM dengan inovasi Kalkulator Biaya dan Shopee Live Studio. Fokus pada produk lokal, transparansi biaya, dan perluasan pasar.</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/infrastruktur/d-8696736/proyek-giant-sea-wall-bakal-groundbreaking-di-demak-diawali-tanam-mangrove</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8696923/shopee-hadirkan-2-inovasi-baru-bantu-umkm-atur-harga-hingga-jualan-live</t>
         </is>
       </c>
     </row>
@@ -2127,22 +2109,22 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Setelah 42 Tahun, Akhirnya RI Ekspor Beras 500 Ribu Ton ke Malaysia</t>
+          <t>Luhut soal Subsidi Barang Diganti Cash: Bertahap</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Wed, 07 Oct 2026 16:53:12 +0700</t>
+          <t>Wed, 07 Oct 2026 18:30:42 +0700</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2023/06/26/ilustrasi-kontainer-ekspor_169.jpeg?w=360&amp;amp;q=90" /&gt; Setelah 42 tahun, Indonesia kembali ekspor 500 ribu ton beras ke Malaysia. Hashim Djojohadikusumo menyatakan langkah ini menguntungkan dan efisien.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/10/ketua-komite-percepatan-transformasi-digital-pemerintah-luhut-binsar-pandjaitan-1789019836285_169.jpeg?w=360&amp;amp;q=90" /&gt; Penyaluran subsidi yang biasanya diberikan dalam bentuk barang akan diubah menjadi bantuan langsung tunai (</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8696727/setelah-42-tahun-akhirnya-ri-ekspor-beras-500-ribu-ton-ke-malaysia</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8696894/luhut-soal-subsidi-barang-diganti-cash-bertahap</t>
         </is>
       </c>
     </row>
@@ -2154,22 +2136,22 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Infografis: Struktur Biaya Haji 2027</t>
+          <t>Ledakan Tabung Oksigen di Kelapa Gading, 1 Orang Tewas</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Wed, 07 Oct 2026 22:11:35 +0700</t>
+          <t>Thu, 08 Oct 2026 08:13:05 +0700</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Total biaya haji mencapai Rp 98,47 juta, dengan sebagian ditanggung jemaah dan sebagian berasal dari nilai manfaat.</t>
+          <t>Ledakan terjadi saat proses pengisian tabung oksigen berukuran sekitar 48 hingga 50 kilogram.</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8308336/infografis-struktur-biaya-haji-2027</t>
+          <t>https://www.liputan6.com/news/read/8308438/ledakan-tabung-oksigen-di-kelapa-gading-1-orang-tewas</t>
         </is>
       </c>
     </row>
@@ -2181,22 +2163,22 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Rita Widyasari Diperiksa KPK 6 Jam, Jadi Saksi Kasus TPPU Khairudin</t>
+          <t>Khalid Basalamah Absen di Sidang Kuota Haji</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Wed, 07 Oct 2026 21:33:39 +0700</t>
+          <t>Thu, 08 Oct 2026 07:54:57 +0700</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Rita Widyasari diperiksa sekitar enam jam sebagai saksi dalam kasus dugaan TPPU Khairudin.</t>
+          <t>KPK menyebut Khalid Basalamah tidak hadir sesuai jadwal sebagai saksi kasus kuota haji dan meyakini dia akan memenuhi panggilan berikutnya.</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8308290/rita-widyasari-diperiksa-kpk-6-jam-jadi-saksi-kasus-tppu-khairudin</t>
+          <t>https://www.liputan6.com/news/read/8308430/khalid-basalamah-absen-di-sidang-kuota-haji</t>
         </is>
       </c>
     </row>
@@ -2208,22 +2190,22 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Peternak Telur Merugi, Titiek Soeharto Minta Pemerintah Serap Produksi</t>
+          <t>Dugaan Politik Uang Muktamar NU Dilaporkan ke KPK</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Wed, 07 Oct 2026 21:29:34 +0700</t>
+          <t>Thu, 08 Oct 2026 07:34:26 +0700</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Peternak mengeluhkan harga telur yang turun saat biaya pakan meningkat hingga memicu kerugian.</t>
+          <t>Aduan PCNU tersebut terkait dugaan politik uang dalam pengondisian dukungan Rais Aam pada Muktamar Ke-35 NU.</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8308317/peternak-telur-merugi-titiek-soeharto-minta-pemerintah-serap-produksi</t>
+          <t>https://www.liputan6.com/news/read/8308425/dugaan-politik-uang-muktamar-nu-dilaporkan-ke-kpk</t>
         </is>
       </c>
     </row>
@@ -2235,22 +2217,22 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Sudah Daftar Haji, Berapa Lama Harus Menunggu?</t>
+          <t>Nilai Manfaat Rp 8,83 Triliun Digunakan untuk Biaya Haji 2027</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Wed, 07 Oct 2026 21:09:24 +0700</t>
+          <t>Thu, 08 Oct 2026 07:24:07 +0700</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Validasi data pemerintah mengungkap masa tunggu faktual jemaah haji Indonesia kini rata-rata 14 tahun.</t>
+          <t>Sementara, sekitar Rp 2,6 triliun dari sisa nilai manfaat dialokasikan ke rekening virtual jemaah haji dalam daftar tunggu.</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8308274/sudah-daftar-haji-berapa-lama-harus-menunggu</t>
+          <t>https://www.liputan6.com/news/read/8308423/nilai-manfaat-rp-883-triliun-digunakan-untuk-biaya-haji-2027</t>
         </is>
       </c>
     </row>
@@ -2262,22 +2244,22 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Menteri LH Ungkap Tantangan Terbesar Aksi Iklim Dunia</t>
+          <t>BMKG Prakirakan Suhu Jakarta Capai 34 Derajat Celsius</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Wed, 07 Oct 2026 20:54:16 +0700</t>
+          <t>Thu, 08 Oct 2026 06:33:59 +0700</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Hal itu disampaikan Menteri LH Moh Jumhur Hidayat dalam Leader’s Plenary pada Pre-COP Leader’s Event.</t>
+          <t>Suhu Jakarta diprakirakan mencapai 34 derajat Celsius pada Kamis (8/10/2026), dengan cuaca didominasi berawan tebal.</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8308306/menteri-lh-ungkap-tantangan-terbesar-aksi-iklim-dunia</t>
+          <t>https://www.liputan6.com/news/read/8308405/bmkg-prakirakan-suhu-jakarta-capai-34-derajat-celsius</t>
         </is>
       </c>
     </row>
@@ -2289,22 +2271,22 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Didakwa Cuci Uang, Febrie Adriansyah Siapkan Nota Perlawanan</t>
+          <t>'Kue' Tak Biasa untuk Sang Jaksa</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Wed, 07 Oct 2026 20:07:48 +0700</t>
+          <t>Thu, 08 Oct 2026 06:08:28 +0700</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Didakwa Cuci Uang Rp 346,7 Miliar, Febrie Adriansyah Bakal Siapkan Nota Perlawanan</t>
+          <t>Jaksa mengungkap kode “kue” dalam penyerahan uang Rp20 miliar kepada Febrie Adriansyah serta penerimaan THR Rp600 juta.</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8308254/didakwa-cuci-uang-febrie-adriansyah-siapkan-nota-perlawanan</t>
+          <t>https://www.liputan6.com/news/read/8308386/kue-tak-biasa-untuk-sang-jaksa</t>
         </is>
       </c>
     </row>
@@ -2316,22 +2298,22 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Haji 2027 Lebih Murah Rp 3,2 Juta, Ini Hitungannya</t>
+          <t>Golkar: Putusan MK soal Gibran Jadi Bahan Evaluasi Sistem Pemilu</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Wed, 07 Oct 2026 21:34:49 +0700</t>
+          <t>Thu, 08 Oct 2026 05:46:31 +0700</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Pelunasan Bipih 2027 turun menjadi Rp23,2 juta setelah pemerintah memberikan subsidi Rp3 juta.</t>
+          <t>Doli juga menilai putusan MK perlu menjadi bahan introspeksi bagi penyelenggara pemilu.</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8308240/haji-2027-lebih-murah-rp-32-juta-ini-hitungannya</t>
+          <t>https://www.liputan6.com/news/read/8308393/golkar-putusan-mk-soal-gibran-jadi-bahan-evaluasi-sistem-pemilu</t>
         </is>
       </c>
     </row>
@@ -2343,22 +2325,22 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Nusron Wahid Tak Hadiri Pemeriksaan KPK</t>
+          <t>Prabowo Minta TNI-Polri Hilangkan Ego Sektoral dan Perkuat Kesiapsiagaan</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Wed, 07 Oct 2026 18:59:55 +0700</t>
+          <t>Thu, 08 Oct 2026 05:34:59 +0700</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Nusron sedianya diperiksa terkait kasus dugaan korupsi di lingkungan Kementerian ATR/BPN.</t>
+          <t>Presiden Prabowo Subianto mengingatkan TNI-Polri untuk menjaga kepercayaan rakyat dan memperbaiki pelayanan kepada masyarakat.</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8308234/nusron-wahid-tak-hadiri-pemeriksaan-kpk</t>
+          <t>https://www.liputan6.com/news/read/8308391/prabowo-minta-tni-polri-hilangkan-ego-sektoral-dan-perkuat-kesiapsiagaan</t>
         </is>
       </c>
     </row>
@@ -2370,22 +2352,22 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Kuasa Hukum Korban Minta Status Bebas Bersyarat Indra Kenz Segera Dicabut</t>
+          <t>Kubu Febrie Adriansyah Soroti Asal-usul Emas 74 Kg dalam Dakwaan Jaksa</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Wed, 07 Oct 2026 18:49:28 +0700</t>
+          <t>Thu, 08 Oct 2026 05:34:28 +0700</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Irsan Gusfrianto, kuasa hukum korban investasi bodong Indra Kenz meminta status pembebasan bersyarat terdakwa penipuan itu segera dicabut.</t>
+          <t>Emas seberat 74 kilogram menjadi salah satu barang bukti penting dalam perkara Febrie Adriansyah.</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8308231/kuasa-hukum-korban-minta-status-bebas-bersyarat-indra-kenz-segera-dicabut</t>
+          <t>https://www.liputan6.com/news/read/8308390/kubu-febrie-adriansyah-soroti-asal-usul-emas-74-kg-dalam-dakwaan-jaksa</t>
         </is>
       </c>
     </row>
@@ -2397,22 +2379,22 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Pelunasan Haji 2027 Turun Rp 3,2 Juta, Jadi Rp 23,2 Juta</t>
+          <t>Kejagung Periksa Saksi Kasus Dugaan Korupsi Pemanfaatan Hutan Lampung</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Wed, 07 Oct 2026 18:58:50 +0700</t>
+          <t>Thu, 08 Oct 2026 05:21:29 +0700</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Biaya pelunasan haji 2027 turun Rp 3,2 juta. Apa yang membuat jemaah cukup membayar Rp 23,2 juta?</t>
+          <t>Kejagung memeriksa dua saksi untuk memperkuat pembuktian kasus dugaan korupsi pemanfaatan kawasan hutan PT PSMI di Lampung.</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8308235/pelunasan-haji-2027-turun-rp-32-juta-jadi-rp-232-juta</t>
+          <t>https://www.liputan6.com/news/read/8308389/kejagung-periksa-saksi-kasus-dugaan-korupsi-pemanfaatan-hutan-lampung</t>
         </is>
       </c>
     </row>
@@ -2424,22 +2406,22 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Prabowo Ingin Rekrutmen TNI-Polisi Diubah: Boleh Pakai Kacamata Asal Pintar</t>
+          <t>Pramono Larang Pungutan PMI kepada ASN dan Warga DKI</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Wed, 07 Oct 2026 18:31:55 +0700</t>
+          <t>Thu, 08 Oct 2026 05:12:28 +0700</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Prabowo ingin rekrutmen prajurit TNI dan polisi tak lagi mengedepankan fisik saja, namun juga mengutamakan intelektual.</t>
+          <t>Gubernur DKI Jakarta Pramono Anung menegaskan tidak boleh ada pungutan PMI, termasuk yang berdalih bersifat sukarela.</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8308219/prabowo-ingin-rekrutmen-tni-polisi-diubah-boleh-pakai-kacamata-asal-pintar</t>
+          <t>https://www.liputan6.com/news/read/8308387/pramono-larang-pungutan-pmi-kepada-asn-dan-warga-dki</t>
         </is>
       </c>
     </row>
@@ -2451,22 +2433,22 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Turun Rp 3,2 Juta, Pelunasan Biaya Haji 2027 Jadi Rp 23,2 Juta</t>
+          <t>Geramnya Pramono Tanggapi Dugaan Pelecehan Guru terhadap Murid</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Wed, 07 Oct 2026 18:25:48 +0700</t>
+          <t>Thu, 08 Oct 2026 00:55:00 +0700</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Pemerintah memberikan subsidi sekitar Rp 3 juta untuk komponen biaya haji di dalam negeri.</t>
+          <t>Pramono meminta pelaku tidak lagi menjadi pendidik dan diproses hukum.</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8308210/turun-rp-32-juta-pelunasan-biaya-haji-2027-jadi-rp-232-juta</t>
+          <t>https://www.liputan6.com/news/read/8308382/geramnya-pramono-tanggapi-dugaan-pelecehan-guru-terhadap-murid</t>
         </is>
       </c>
     </row>
@@ -2478,22 +2460,22 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Dana Cadangan Jakarta Capai Rp 5,6 Triliun, Ini Peruntukannya</t>
+          <t>Asa Pramono Perluas Transjakarta Perluas Kelola Laut Masih Terganjal</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Wed, 07 Oct 2026 17:40:00 +0700</t>
+          <t>Thu, 08 Oct 2026 00:38:00 +0700</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Pembiayaan kreatif seperti obligasi daerah akan digunakan.</t>
+          <t>Pramono Anung berupaya memperluas Transjakarta ke Kepulauan Seribu demi akses publik merata dan ekonomi warga.</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8308172/dana-cadangan-jakarta-capai-rp-56-triliun-ini-peruntukannya</t>
+          <t>https://www.liputan6.com/news/read/8308377/asa-pramono-perluas-transjakarta-perluas-kelola-laut-masih-terganjal</t>
         </is>
       </c>
     </row>
@@ -2505,22 +2487,23 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Dakwaan Febrie Adriansyah, Terungkap Kode 'Kue' Rp 20 Miliar</t>
+          <t>Jaksa Bongkar Isi 3 Brankas Kasus Cuci Uang Febrie Adriansyah</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Wed, 07 Oct 2026 17:32:41 +0700</t>
+          <t>Wed, 07 Oct 2026 23:43:17 +0700</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Kode "Kue" dalam dakwaan Febrie Adriansyah itu salah satunya terkait dengan setoran dari Tria Bellitonito Aturbumi.</t>
+          <t>Jaksa mengungkap isi tiga brankas yang dikaitkan dengan perkara TPPU Febrie Adriansyah, termasuk 74 kilogram emas dan uang berbagai mata uang.
+Hasil rewrite</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8308156/dakwaan-febrie-adriansyah-terungkap-kode-kue-rp-20-miliar</t>
+          <t>https://www.liputan6.com/news/read/8308353/jaksa-bongkar-isi-3-brankas-kasus-cuci-uang-febrie-adriansyah</t>
         </is>
       </c>
     </row>
@@ -2532,22 +2515,22 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Letjen Tri Budi Utomo Jabat Wakil KSAD Gantikan Saleh Mustafa</t>
+          <t>Infografis: Struktur Biaya Haji 2027</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Wed, 07 Oct 2026 17:10:35 +0700</t>
+          <t>Wed, 07 Oct 2026 22:11:35 +0700</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Serah terima jabatan dilakukan pekan depan.</t>
+          <t>Total biaya haji mencapai Rp 98,47 juta, dengan sebagian ditanggung jemaah dan sebagian berasal dari nilai manfaat.</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8308135/letjen-tri-budi-utomo-jabat-wakil-ksad-gantikan-saleh-mustafa</t>
+          <t>https://www.liputan6.com/news/read/8308336/infografis-struktur-biaya-haji-2027</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data pasar & berita - 2026-10-12 00:46 UTC
</commit_message>
<xml_diff>
--- a/data/market_news_latest.xlsx
+++ b/data/market_news_latest.xlsx
@@ -500,7 +500,7 @@
         <v>1.04</v>
       </c>
       <c r="H2" t="n">
-        <v>0</v>
+        <v>350813700</v>
       </c>
     </row>
     <row r="3">
@@ -525,16 +525,16 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>7793.3398</v>
+        <v>7811.54</v>
       </c>
       <c r="F3" t="n">
-        <v>27.98</v>
+        <v>46.1802</v>
       </c>
       <c r="G3" t="n">
-        <v>0.36</v>
+        <v>0.59</v>
       </c>
       <c r="H3" t="n">
-        <v>763832962</v>
+        <v>4782640000</v>
       </c>
     </row>
     <row r="4">
@@ -559,16 +559,16 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>51442.4688</v>
+        <v>51654.9492</v>
       </c>
       <c r="F4" t="n">
-        <v>210.8281</v>
+        <v>423.3086</v>
       </c>
       <c r="G4" t="n">
-        <v>0.41</v>
+        <v>0.83</v>
       </c>
       <c r="H4" t="n">
-        <v>108188898</v>
+        <v>339470000</v>
       </c>
     </row>
     <row r="5">
@@ -593,16 +593,16 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>27294.6387</v>
+        <v>27366.1699</v>
       </c>
       <c r="F5" t="n">
-        <v>101.2988</v>
+        <v>172.8301</v>
       </c>
       <c r="G5" t="n">
-        <v>0.37</v>
+        <v>0.64</v>
       </c>
       <c r="H5" t="n">
-        <v>2297308000</v>
+        <v>6845310000</v>
       </c>
     </row>
     <row r="6">
@@ -623,20 +623,20 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>69042.1094</v>
+        <v>69030.9219</v>
       </c>
       <c r="F6" t="n">
-        <v>-993.6016</v>
+        <v>-11.1875</v>
       </c>
       <c r="G6" t="n">
-        <v>-1.42</v>
+        <v>-0.02</v>
       </c>
       <c r="H6" t="n">
-        <v>162200000</v>
+        <v>162000000</v>
       </c>
     </row>
     <row r="7">
@@ -670,7 +670,7 @@
         <v>1.79</v>
       </c>
       <c r="H7" t="n">
-        <v>0</v>
+        <v>2905300000</v>
       </c>
     </row>
     <row r="8">
@@ -695,16 +695,16 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>3813.7913</v>
+        <v>3813.791</v>
       </c>
       <c r="F8" t="n">
-        <v>1.8872</v>
+        <v>1.887</v>
       </c>
       <c r="G8" t="n">
         <v>0.05</v>
       </c>
       <c r="H8" t="n">
-        <v>1975384548</v>
+        <v>535100</v>
       </c>
     </row>
     <row r="9">
@@ -729,16 +729,16 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>10548.71</v>
+        <v>10552.0996</v>
       </c>
       <c r="F9" t="n">
-        <v>107.1104</v>
+        <v>110.5</v>
       </c>
       <c r="G9" t="n">
-        <v>1.03</v>
+        <v>1.06</v>
       </c>
       <c r="H9" t="n">
-        <v>0</v>
+        <v>787988200</v>
       </c>
     </row>
     <row r="10">
@@ -763,16 +763,16 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>25095.2695</v>
+        <v>25087.2695</v>
       </c>
       <c r="F10" t="n">
-        <v>288.2988</v>
+        <v>280.2988</v>
       </c>
       <c r="G10" t="n">
-        <v>1.16</v>
+        <v>1.13</v>
       </c>
       <c r="H10" t="n">
-        <v>0</v>
+        <v>59039100</v>
       </c>
     </row>
     <row r="11">
@@ -806,7 +806,7 @@
         <v>-0.2</v>
       </c>
       <c r="H11" t="n">
-        <v>0</v>
+        <v>341999600</v>
       </c>
     </row>
     <row r="12">
@@ -827,17 +827,17 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="E12" t="n">
         <v>17879</v>
       </c>
       <c r="F12" t="n">
-        <v>1.5</v>
+        <v>71.5</v>
       </c>
       <c r="G12" t="n">
-        <v>0.01</v>
+        <v>0.4</v>
       </c>
       <c r="H12" t="n">
         <v>0</v>
@@ -861,17 +861,17 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>102.301</v>
+        <v>102.133</v>
       </c>
       <c r="F13" t="n">
-        <v>0.161</v>
+        <v>-0.077</v>
       </c>
       <c r="G13" t="n">
-        <v>0.16</v>
+        <v>-0.08</v>
       </c>
       <c r="H13" t="n">
         <v>0</v>
@@ -895,17 +895,17 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>158.384</v>
+        <v>158.129</v>
       </c>
       <c r="F14" t="n">
-        <v>0.324</v>
+        <v>0.066</v>
       </c>
       <c r="G14" t="n">
-        <v>0.2</v>
+        <v>0.04</v>
       </c>
       <c r="H14" t="n">
         <v>0</v>
@@ -933,13 +933,13 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>0.5274</v>
+        <v>0.5244</v>
       </c>
       <c r="F15" t="n">
-        <v>0.0043</v>
+        <v>0.0013</v>
       </c>
       <c r="G15" t="n">
-        <v>0.82</v>
+        <v>0.25</v>
       </c>
       <c r="H15" t="n">
         <v>0</v>
@@ -967,13 +967,13 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>0.5633</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="F16" t="n">
-        <v>0.0027</v>
+        <v>-0.0005999999999999999</v>
       </c>
       <c r="G16" t="n">
-        <v>0.48</v>
+        <v>-0.11</v>
       </c>
       <c r="H16" t="n">
         <v>0</v>
@@ -1035,16 +1035,16 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>77.565</v>
+        <v>77.98</v>
       </c>
       <c r="F18" t="n">
-        <v>-0.305</v>
+        <v>0.11</v>
       </c>
       <c r="G18" t="n">
-        <v>-0.39</v>
+        <v>0.14</v>
       </c>
       <c r="H18" t="n">
-        <v>8074934</v>
+        <v>27247700</v>
       </c>
     </row>
     <row r="19">
@@ -1069,16 +1069,16 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>77.13500000000001</v>
+        <v>77.23</v>
       </c>
       <c r="F19" t="n">
-        <v>-0.005</v>
+        <v>0.09</v>
       </c>
       <c r="G19" t="n">
-        <v>-0.01</v>
+        <v>0.12</v>
       </c>
       <c r="H19" t="n">
-        <v>8602330</v>
+        <v>36922300</v>
       </c>
     </row>
     <row r="20">
@@ -1099,20 +1099,20 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>4208.7002</v>
+        <v>4230.3999</v>
       </c>
       <c r="F20" t="n">
-        <v>51.7002</v>
+        <v>14.1001</v>
       </c>
       <c r="G20" t="n">
-        <v>1.24</v>
+        <v>0.33</v>
       </c>
       <c r="H20" t="n">
-        <v>96934</v>
+        <v>8668</v>
       </c>
     </row>
     <row r="21">
@@ -1133,20 +1133,20 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>91.84999999999999</v>
+        <v>90.58</v>
       </c>
       <c r="F21" t="n">
-        <v>0.36</v>
+        <v>-1.27</v>
       </c>
       <c r="G21" t="n">
-        <v>0.39</v>
+        <v>-1.38</v>
       </c>
       <c r="H21" t="n">
-        <v>107007</v>
+        <v>11066</v>
       </c>
     </row>
     <row r="22">
@@ -1167,20 +1167,20 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="E22" t="n">
-        <v>104.66</v>
+        <v>103.38</v>
       </c>
       <c r="F22" t="n">
-        <v>0.38</v>
+        <v>-1.34</v>
       </c>
       <c r="G22" t="n">
-        <v>0.36</v>
+        <v>-1.28</v>
       </c>
       <c r="H22" t="n">
-        <v>15996</v>
+        <v>2422</v>
       </c>
     </row>
     <row r="23">
@@ -1201,20 +1201,20 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="E23" t="n">
-        <v>6.6955</v>
+        <v>6.7195</v>
       </c>
       <c r="F23" t="n">
-        <v>0.1765</v>
+        <v>0.077</v>
       </c>
       <c r="G23" t="n">
-        <v>2.71</v>
+        <v>1.16</v>
       </c>
       <c r="H23" t="n">
-        <v>29640</v>
+        <v>1207</v>
       </c>
     </row>
     <row r="24">
@@ -1239,16 +1239,16 @@
         </is>
       </c>
       <c r="E24" t="n">
-        <v>66.63</v>
+        <v>66.8</v>
       </c>
       <c r="F24" t="n">
-        <v>0.53</v>
+        <v>0.7</v>
       </c>
       <c r="G24" t="n">
-        <v>0.8</v>
+        <v>1.06</v>
       </c>
       <c r="H24" t="n">
-        <v>4871559</v>
+        <v>14966000</v>
       </c>
     </row>
     <row r="25">
@@ -1273,13 +1273,13 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>14.98</v>
+        <v>14.84</v>
       </c>
       <c r="F25" t="n">
-        <v>-0.43</v>
+        <v>-0.57</v>
       </c>
       <c r="G25" t="n">
-        <v>-2.79</v>
+        <v>-3.7</v>
       </c>
       <c r="H25" t="n">
         <v>0</v>
@@ -1303,20 +1303,20 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="E26" t="n">
-        <v>82793.0469</v>
+        <v>83765.10159999999</v>
       </c>
       <c r="F26" t="n">
-        <v>1116.7109</v>
+        <v>852.875</v>
       </c>
       <c r="G26" t="n">
-        <v>1.37</v>
+        <v>1.03</v>
       </c>
       <c r="H26" t="n">
-        <v>39730278400</v>
+        <v>12825135104</v>
       </c>
     </row>
     <row r="27">
@@ -1749,22 +1749,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Menteri PU Dorong Proyek KSPEAN Wanam Sejahterakan Warga Sekitar</t>
+          <t>Terkuak Modus Penipuan Tawarkan Urus Dapur MBG Kilat</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Fri, 09 Oct 2026 21:47:10 +0700</t>
+          <t>Mon, 12 Oct 2026 07:30:14 +0700</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/09/menteri-pu-dody-hanggodo-di-wanam-merauke-papua-1791557028439_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri PU Dody Hanggodo mendorong pembangunan Kawasan Swasembada Pangan, Energi, dan Air Nasional di Wanam, Merauke, memberikan kesejahter</t>
+          <t xml:space="preserve">&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/10/10/bandung-hadirkan-sppg-baru-2400-paket-makan-bergizi-siap-untuk-anak-sekolah-1760085494045_169.jpeg?w=360&amp;amp;q=90" /&gt; Badan Gizi Nasional (BGN) membongkar modus penipuan yang menawarkan pembukaan dapur Makan Bergizi Gratis (MBG) </t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/infrastruktur/d-8700296/menteri-pu-dorong-proyek-kspean-wanam-sejahterakan-warga-sekitar</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8702504/terkuak-modus-penipuan-tawarkan-urus-dapur-mbg-kilat</t>
         </is>
       </c>
     </row>
@@ -1776,22 +1776,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Belajar Kenali Risiko Bisnis dengan Data Science, Tak Harus Background Anak IT!</t>
+          <t>Waspada, El Nino Berpotensi Picu Kenaikan Harga Cabai dan Daging Ayam</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Fri, 09 Oct 2026 21:34:36 +0700</t>
+          <t>Mon, 12 Oct 2026 07:00:19 +0700</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/25/detikevent-data-science-dan-python-1790346113822_169.jpeg?w=360&amp;amp;q=90" /&gt; detikcourse membuka kelas Kenali Risiko Bisnis Lewat Data Science dan Python yang tidak mensyaratkan pengalaman sebagai programmer.</t>
+          <t xml:space="preserve">&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/11/waspada-el-nino-berpotensi-picu-kenaikan-harga-cabai-dan-daging-ayam-1791706439905_169.jpeg?w=360&amp;amp;q=90" /&gt; Pemerintah mewaspadai dampak El Nino terhadap harga pangan. Cabai rawit, cabai merah, dan daging ayam berpotensi naik </t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8700286/belajar-kenali-risiko-bisnis-dengan-data-science-tak-harus-background-anak-it</t>
+          <t>https://finance.detik.com/foto-bisnis/d-8702088/waspada-el-nino-berpotensi-picu-kenaikan-harga-cabai-dan-daging-ayam</t>
         </is>
       </c>
     </row>
@@ -1803,22 +1803,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Pasokan BBM ke Lombok Digenjot Jelang MotoGP Mandalika</t>
+          <t>Rencana Pemerintah Tambal Defisit di Akhir Tahun</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Fri, 09 Oct 2026 21:23:57 +0700</t>
+          <t>Mon, 12 Oct 2026 06:30:20 +0700</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/09/pt-pertamina-patra-niaga-menyiapkan-pasokan-bbm-1791555777873_169.jpeg?w=360&amp;amp;q=90" /&gt; PT Pertamina Patra Niaga menyiapkan pasokan Bahan Bakar Minyak (BBM) tambahan di kawasan Lombok, Nusa Tenggara Barat (NTB).</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2016/07/28/752567fe-0498-4b0f-9fd8-cde307b5d122_169.jpg?w=360&amp;amp;q=90" /&gt; Kemenkeu memperkirakan defisit Anggaran Pendapatan Belanja Negara (APBN) hingga akhir tahun mencapai 2,85% terhadap Produk Domestik Bruto (PDB).</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8700271/pasokan-bbm-ke-lombok-digenjot-jelang-motogp-mandalika</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8702496/rencana-pemerintah-tambal-defisit-di-akhir-tahun</t>
         </is>
       </c>
     </row>
@@ -1830,22 +1830,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Uang Pensiun PNS hingga Bansos Bakal Ditransfer Langsung ke Rekening</t>
+          <t>Gelaran Pertamina Grand Prix of Indonesia 2026 Perkuat Ekonomi Lokal</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Fri, 09 Oct 2026 21:04:00 +0700</t>
+          <t>Mon, 12 Oct 2026 06:08:28 +0700</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2018/03/07/04a334e0-fe12-4634-af17-4ff473c511fd_169.jpeg?w=360&amp;amp;q=90" /&gt; Uang pensiun bakal ditransfer langsung dari Rekening Kas Umum Negara (RKUN) ke rekening bank masing-masing pensiunan.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/12/gelaran-pertamina-grand-prix-of-indonesia-2026-perkuat-ekonomi-lokal-1791760079211.jpeg?w=360&amp;amp;q=90" /&gt; Pertamina Grand Prix of Indonesia 2026 sukses digelar di Mandalika, menarik perhatian global dan mendukung ekonomi lokal m</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8700246/uang-pensiun-pns-hingga-bansos-bakal-ditransfer-langsung-ke-rekening</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8702653/gelaran-pertamina-grand-prix-of-indonesia-2026-perkuat-ekonomi-lokal</t>
         </is>
       </c>
     </row>
@@ -1857,22 +1857,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Korea Bidik Proyek Irigasi 750.000 Hektare Lahan Pertanian di Merauke</t>
+          <t>63.789 Orang Jadi Korban PHK, Paling Banyak dari Provinsi Ini</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Fri, 09 Oct 2026 20:49:46 +0700</t>
+          <t>Mon, 12 Oct 2026 05:55:13 +0700</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/09/sentra-pangan-di-wanam-merauke-papua-selatan-1791553519140_169.jpeg?w=360&amp;amp;q=90" /&gt; Pemerintah menyiapkan Merauke, Papua Selatan, sebagai sentra pangan Indonesia Timur.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2019/07/30/559b04c3-168f-4c87-b3d4-cfad79eb8e5a_169.jpeg?w=360&amp;amp;q=90" /&gt; Data pemutusan hubungan kerja (PHK) terbaru kembali dirilis Kementerian Ketenagakerjaan.</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/infrastruktur/d-8700234/korea-bidik-proyek-irigasi-750-000-hektare-lahan-pertanian-di-merauke</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8702493/63-789-orang-jadi-korban-phk-paling-banyak-dari-provinsi-ini</t>
         </is>
       </c>
     </row>
@@ -1884,22 +1884,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>BULOG Cetak Pengadaan 4 Juta Ton, Gelar Tasyakuran Bersama Komisi IV</t>
+          <t>Bawa 30 UMKM ke Sirkuit Mandalika, Pertamina Dorong Ekonomi Lokal Berdaya</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Fri, 09 Oct 2026 20:15:43 +0700</t>
+          <t>Sun, 11 Oct 2026 22:21:12 +0700</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/09/bulog-cetak-pengadaan-4-juta-ton-gelar-tasyakuran-bersama-komisi-iv-1791551702801_169.jpeg?w=360&amp;amp;q=90" /&gt; Perum BULOG mencatatkan sejarah baru dengan pengadaan beras melampaui 4 juta ton. Capaian ini disyukuri dalam tasyakura</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/11/pertamina-1791731991936.jpeg?w=360&amp;amp;q=90" /&gt; PT Pertamina membawa 30 UMKM ke Pertamina Grand Prix of Indonesia 2026. Mereka berpartisipasi di bazar untuk memperluas pasar dan meningkatkan pendapatan.</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8700205/bulog-cetak-pengadaan-4-juta-ton-gelar-tasyakuran-bersama-komisi-iv</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8702573/bawa-30-umkm-ke-sirkuit-mandalika-pertamina-dorong-ekonomi-lokal-berdaya</t>
         </is>
       </c>
     </row>
@@ -1911,22 +1911,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Sekolah Gratis Jadi Tahun Depan? Suahasil Buka Suara soal Anggaran</t>
+          <t>Kementerian ATR &amp;amp; BRAN Mulai Bagi-bagi Tugas</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Fri, 09 Oct 2026 20:04:29 +0700</t>
+          <t>Sun, 11 Oct 2026 22:00:52 +0700</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/09/apbn-defisit-rp319-triliun-menkeu-sebut-masih-sesuai-target-1791525967190_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Keuangan Suahasil Nazara buka suara soal program sekolah gratis.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/08/14/ilustrasi-kementerian-atrbpn-1755140401786_169.jpeg?w=360&amp;amp;q=90" /&gt; Kelembagaan Badan Reforma Agraria Nasional (BRAN) terus dimatangkan sebagai tindak lanjut dari Undang-Undang Pengaturan Reforma Agraria.</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8700195/sekolah-gratis-jadi-tahun-depan-suahasil-buka-suara-soal-anggaran</t>
+          <t>https://finance.detik.com/infrastruktur/d-8701869/kementerian-atr-bran-mulai-bagi-bagi-tugas</t>
         </is>
       </c>
     </row>
@@ -1938,22 +1938,22 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Wanam Merauke 'Disulap' Jadi Sentra Produksi Pangan Indonesia Timur</t>
+          <t>BSI Ajak Masyarakat Bantu Pulihkan Desa Wisata Sade di Lombok</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Fri, 09 Oct 2026 19:55:44 +0700</t>
+          <t>Sun, 11 Oct 2026 21:36:43 +0700</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/09/menteri-pu-cek-pusat-produksi-pangan-di-wanam-merauke-1791550351807_169.jpeg?w=360&amp;amp;q=90" /&gt; Pemerintah menggenjot pembangunan pusat produksi pangan baru di berbagai daerah. Salah satunya di Wanam, Merauke, Papua Selatan.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/11/bsi-1791729263003_169.jpeg?w=360&amp;amp;q=90" /&gt; PT Bank Syariah Indonesia meluncurkan program 'Satu Benang untuk Sade' di Lombok untuk pemulihan ekonomi lokal pascabencana.</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/infrastruktur/d-8700188/wanam-merauke-disulap-jadi-sentra-produksi-pangan-indonesia-timur</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8702550/bsi-ajak-masyarakat-bantu-pulihkan-desa-wisata-sade-di-lombok</t>
         </is>
       </c>
     </row>
@@ -1965,22 +1965,22 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Bocoran Pertemuan Dua Menteri Prabowo di Kementerian ESDM</t>
+          <t>Pertamina EP Rantau Bor 5 Sumur Baru di Aceh Tamiang</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Fri, 09 Oct 2026 19:34:58 +0700</t>
+          <t>Sun, 11 Oct 2026 21:00:37 +0700</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/09/17/gedung-esdm-1758100960605_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Koordinator Hilirisasi dan Transisi Energi Bahlil Lahadalia menerima kunjungan Menteri Perumahan dan Kawasan Permukiman (PKP) Maruarar Sirait.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/11/pt-pertamina-ep-field-rantau-1791708867596_169.jpeg?w=360&amp;amp;q=90" /&gt; Pertamina EP Rantau Field melakukan pengeboran sumur baru di tengah pemulihan pascabencana banjir Aceh Tamiang.</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8700164/bocoran-pertemuan-dua-menteri-prabowo-di-kementerian-esdm</t>
+          <t>https://finance.detik.com/energi/d-8702140/pertamina-ep-rantau-bor-5-sumur-baru-di-aceh-tamiang</t>
         </is>
       </c>
     </row>
@@ -1992,22 +1992,22 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>TKD Rp 599 Triliun, buat Gaji 5,3 Juta ASN Daerah hingga Tunjangan Guru</t>
+          <t>Waspada! Ada Modus Penipuan Janjikan Urus Dapur MBG Kilat</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Fri, 09 Oct 2026 19:06:53 +0700</t>
+          <t>Sun, 11 Oct 2026 20:00:22 +0700</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2016/06/18/e7060b9d-8fd4-4ee9-9fb7-b015210b946b_169.jpg?w=360&amp;amp;q=90" /&gt; Pemerintah telah menyalurkan dana Transfer ke Daerah (TKD) sebesar Rp 599,2 triliun hingga September 2026.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/01/27/32-ribu-pegawai-inti-mbg-bakal-diangkat-jadi-asn-pppk-1769488598657_169.jpeg?w=360&amp;amp;q=90" /&gt; Juru Bicara BGN Tysa Novenny, mengatakan masyarakat perlu berhati-hati dalam menyikapi setiap tindakan yang mengatasnamakan BGN.</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8700127/tkd-rp-599-triliun-buat-gaji-5-3-juta-asn-daerah-hingga-tunjangan-guru</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8702086/waspada-ada-modus-penipuan-janjikan-urus-dapur-mbg-kilat</t>
         </is>
       </c>
     </row>
@@ -2019,22 +2019,22 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Manufaktur Jadi Motor Industri RI, Jangan Layu Sebelum Capai Puncak!</t>
+          <t>Produk UMKM Ikut Mejeng di Gelaran MotoGP Mandalika</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Fri, 09 Oct 2026 18:17:16 +0700</t>
+          <t>Sun, 11 Oct 2026 19:30:18 +0700</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/08/06/ekonomi-indonesia-kembali-ngebut-industri-dan-konsumsi-jadi-penopang-1786012269666_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Perindustrian (Menperin) Muhammad Sarmuji menegaskan industri manufaktur harus kembali menjadi motor utama per</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/11/produk-umkm-di-ajang-motogp-1791714381524_169.jpeg?w=360&amp;amp;q=90" /&gt; Pertamina melalui PT Pertamina Patra Niaga menghadirkan produk kerajinan unggulan Lombok sebagai official merchandise.</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/industri/d-8700068/manufaktur-jadi-motor-industri-ri-jangan-layu-sebelum-capai-puncak</t>
+          <t>https://finance.detik.com/energi/d-8702299/produk-umkm-ikut-mejeng-di-gelaran-motogp-mandalika</t>
         </is>
       </c>
     </row>
@@ -2046,22 +2046,22 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Serapan Beras Bulog Lampaui Target, Stok Tembus Rekor 4,5 Juta Ton</t>
+          <t>Tambal Defisit, Pemerintah Mau Lelang 12 Surat Utang-Tarik Pinjaman US$ 1,8 M</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Fri, 09 Oct 2026 18:00:51 +0700</t>
+          <t>Sun, 11 Oct 2026 19:00:43 +0700</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/09/serapan-beras-bulog-lampaui-target-stok-tembus-rekor-45-juta-ton-1791526902178_169.jpeg?w=360&amp;amp;q=90" /&gt; Bulog menyerap 4,11 juta ton beras hasil panen dalam negeri hingga 9 Oktober 2026. Stok beras mencapai 4,5 juta ton, terti</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2016/07/28/11b938f2-8964-482f-986f-f70f6458d154_169.jpg?w=360&amp;amp;q=90" /&gt; Direktur Jenderal Pengelolaan Pembiayaan dan Risiko (DJPPR) Kemenkeu Suminto mengatakan pemerintah masih mempunyai kesempatan untuk melelang 12 surat utang.</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/foto-bisnis/d-8699418/serapan-beras-bulog-lampaui-target-stok-tembus-rekor-4-5-juta-ton</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8702060/tambal-defisit-pemerintah-mau-lelang-12-surat-utang-tarik-pinjaman-us-1-8-m</t>
         </is>
       </c>
     </row>
@@ -2073,22 +2073,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>DJP Kembalikan Kelebihan Pajak Rp 198 T</t>
+          <t>Investasi Jakarta Tembus Rp173,6 Triliun, Tertinggi di Indonesia</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Fri, 09 Oct 2026 17:43:16 +0700</t>
+          <t>Sun, 11 Oct 2026 18:00:25 +0700</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2014/10/01/aba994a2-34ed-467e-b236-0838b109f70c_169.jpg?w=360&amp;amp;q=90" /&gt; Direktorat Jenderal Pajak (DJP) Kementerian Keuangan mencatat realisasi pengembalian kelebihan pembayaran pajak atau restitusi mencapai Rp 198,71 triliun.</t>
+          <t xml:space="preserve">&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/10/investasi-jakarta-tembus-rp1736-triliun-hingga-semester-i2026-1791636661420.jpeg?w=360&amp;amp;q=90" /&gt; Realisasi investasi di Jakarta mencapai Rp173,6 triliun hingga semester I 2026, tertinggi di Indonesia, menurut Gubernur Pramono </t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8700022/djp-kembalikan-kelebihan-pajak-rp-198-t</t>
+          <t>https://finance.detik.com/foto-bisnis/d-8701303/investasi-jakarta-tembus-rp173-6-triliun-tertinggi-di-indonesia</t>
         </is>
       </c>
     </row>
@@ -2100,22 +2100,22 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>MotoGP Mandalika Buka Peluang UMKM Lokal Tembus Pasar Global</t>
+          <t>Rosan Buka-bukaan soal Rencana Kerja Sama RI &amp;amp; Mesir</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Fri, 09 Oct 2026 17:40:30 +0700</t>
+          <t>Sun, 11 Oct 2026 17:16:45 +0700</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/09/pertamina-1791542407319_169.jpeg?w=360&amp;amp;q=90" /&gt; Pertamina Grand Prix of Indonesia di Mandalika beri peluang bagi UMKM lokal untuk memperluas pasar. Produk unik dan inovatif siap menarik perhatian wisatawan.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/06/18/menteri-hilirisasi-dan-investasi-rosan-roeslani-kamis-1862026-1781790660049_169.jpeg?w=360&amp;amp;q=90" /&gt; CEO Danantara Rosan Roeslani mengatakan pihaknya akan membentuk dana kelolaan investasi dengan pihak Mesir.</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8700018/motogp-mandalika-buka-peluang-umkm-lokal-tembus-pasar-global</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8702287/rosan-buka-bukaan-soal-rencana-kerja-sama-ri-mesir</t>
         </is>
       </c>
     </row>
@@ -2127,22 +2127,22 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Warga RI Tak Cuma Mau Wariskan Harta, Pendidikan Juga Jadi Prioritas</t>
+          <t>Harga Emas Mulai Bangkit, Naik Segini dalam Sepekan</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Fri, 09 Oct 2026 17:36:23 +0700</t>
+          <t>Sun, 11 Oct 2026 16:00:43 +0700</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/07/01/ilustrasi-biaya-pendidikan-1751353002946_169.jpeg?w=360&amp;amp;q=90" /&gt; Masyarakat Indonesia menempatkan kesempatan pendidikan setara dengan kepemilikan kekayaan sebagai prioritas utama.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/10/15/harga-emas-antam-tembus-rekor-tertinggi-sentuh-rp238-juta-per-gram-1760532607071_169.jpeg?w=360&amp;amp;q=90" /&gt; Harga emas mengalami kenaikan Rp 12 ribu per gram selama sepekan ini.</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8700012/warga-ri-tak-cuma-mau-wariskan-harta-pendidikan-juga-jadi-prioritas</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8701980/harga-emas-mulai-bangkit-naik-segini-dalam-sepekan</t>
         </is>
       </c>
     </row>
@@ -2154,22 +2154,22 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Akses Ditutup Ormas, Karyawan Club de Arjuna Demo Balai Kota</t>
+          <t>Dua Hari Berturut-turut Kebakaran di Wilayah Jakarta Utara</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Fri, 09 Oct 2026 22:01:15 +0700</t>
+          <t>Mon, 12 Oct 2026 07:38:34 +0700</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Ratusan karyawan Club de Arjuna meminta Pemprov DKI membongkar tembok yang menutup akses tempat usaha agar mereka bisa kembali bekerja.</t>
+          <t>Belum dijelaskan kerugian akibat kebakaran dua lokasi tersebut.</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8309989/akses-ditutup-ormas-karyawan-club-de-arjuna-demo-balai-kota</t>
+          <t>https://www.liputan6.com/news/read/8310953/dua-hari-berturut-turut-kebakaran-di-wilayah-jakarta-utara</t>
         </is>
       </c>
     </row>
@@ -2181,22 +2181,22 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Komnas HAM Terima 42 Aduan Dugaan Pelanggaran HAM di Lapas</t>
+          <t>Strategi Ada Gula Ada Semut Ala Mentrans di Festival Transmigrasi 2026</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Fri, 09 Oct 2026 22:00:00 +0700</t>
+          <t>Mon, 12 Oct 2026 06:59:05 +0700</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Aduan tersebut meliputi dugaan kekerasan, pungli, hingga warga binaan yang meninggal dunia akibat dikeroyok.</t>
+          <t>Festival Transmigrasi menjadi salah satu upaya untuk memperkenalkan potensi kawasan hingga pertukaran gagasan.</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8309931/komnas-ham-terima-42-aduan-dugaan-pelanggaran-ham-di-lapas</t>
+          <t>https://www.liputan6.com/news/read/8310941/strategi-ada-gula-ada-semut-ala-mentrans-di-festival-transmigrasi-2026</t>
         </is>
       </c>
     </row>
@@ -2208,22 +2208,22 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>PDIP Minta Kader di Malang Rutin Sentuh Akar Rumput</t>
+          <t>Nestapa 46 Orangutan Terjebak di Sisa Hutan Terbakar</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Fri, 09 Oct 2026 21:02:07 +0700</t>
+          <t>Mon, 12 Oct 2026 06:33:51 +0700</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Arahan itu disampaikan Ketua PDIP Jatim Said Abdullah saat menghadiri konsolidasi di DPC PDIP Kabupaten Malang, Jumat (/10/2026). (Istimewa).</t>
+          <t>46 Individu Orangutan terjebak kebakaran hutan</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8309950/pdip-minta-kader-di-malang-rutin-sentuh-akar-rumput</t>
+          <t>https://www.liputan6.com/news/read/8310938/nestapa-46-orangutan-terjebak-di-sisa-hutan-terbakar</t>
         </is>
       </c>
     </row>
@@ -2235,22 +2235,22 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Yusril Targetkan Revisi UU Narkotika Rampung Akhir 2026</t>
+          <t>Gempa Magnitudo 5,7 Guncang Pohuwato Gorontalo</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Fri, 09 Oct 2026 21:01:00 +0700</t>
+          <t>Mon, 12 Oct 2026 05:20:05 +0700</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Saat ini pemerintah tengah menyusun daftar inventarisasi masalah untuk RUU Narkotika.</t>
+          <t>Gempa tidak berpotensi tsunami.</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8309928/yusril-targetkan-revisi-uu-narkotika-rampung-akhir-2026</t>
+          <t>https://www.liputan6.com/news/read/8310918/gempa-magnitudo-57-guncang-pohuwato-gorontalo</t>
         </is>
       </c>
     </row>
@@ -2262,22 +2262,22 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Kemenkes Batasi Biaya Cek Kesehatan Haji, Maksimal Rp1,3 Juta</t>
+          <t>Cerita Bahlil, dari Jualan Kue Cucur hingga Alami Busung Lapar</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Fri, 09 Oct 2026 20:46:39 +0700</t>
+          <t>Sun, 11 Oct 2026 23:59:40 +0700</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Kemenkes menetapkan kisaran biaya pemeriksaan kesehatan dasar jemaah haji Rp800 ribu hingga Rp1,3 juta untuk menyeragamkan tarif di fasilitas kesehatan.</t>
+          <t>Bahlil Lahadalia mengenang perjuangan semasa kecilnya, mulai dari berjualan kue cucur hingga mengalami busung lapar.</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8309936/kemenkes-batasi-biaya-cek-kesehatan-haji-maksimal-rp13-juta</t>
+          <t>https://www.liputan6.com/news/read/8310900/cerita-bahlil-dari-jualan-kue-cucur-hingga-alami-busung-lapar</t>
         </is>
       </c>
     </row>
@@ -2289,22 +2289,22 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Ribuan Kadet Unhan Diberangkatkan ke 181 Sekolah Rakyat, Perkuat Karakter Siswa</t>
+          <t>Lapak Barang Bekas di Kalideres Kebakaran</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Fri, 09 Oct 2026 20:38:42 +0700</t>
+          <t>Sun, 11 Oct 2026 23:46:18 +0700</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Sebanyak 1.509 kadet dan personel Unhan RI bertugas di 181 Sekolah Rakyat pada 9–27 Oktober 2026 untuk mendukung pembentukan karakter dan kedisiplinan siswa.</t>
+          <t>Petugas pemadam kebakaran menerima informasi kejadian dari warga pada pukul 23.13 WIB.</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8309941/ribuan-kadet-unhan-diberangkatkan-ke-181-sekolah-rakyat-perkuat-karakter-siswa</t>
+          <t>https://www.liputan6.com/news/read/8310896/lapak-barang-bekas-di-kalideres-kebakaran</t>
         </is>
       </c>
     </row>
@@ -2316,22 +2316,22 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Puan Dorong IPU Perkuat Peran Perdamaian dan Tatanan Global Lebih Adil</t>
+          <t>Bahlil Bocorkan Kementerian yang Bakal Berada di Bawah Menko Hilirisasi</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Fri, 09 Oct 2026 20:16:56 +0700</t>
+          <t>Sun, 11 Oct 2026 22:30:07 +0700</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Puan berharap pemimpin terpilih IPU, Milton Dick dapat membawa peran forum parlemen dunia itu semakin kuat.</t>
+          <t>Bahlil memberikan bocoran mengenai sejumlah kementerian yang akan berada di bawah koordinasi Kementerian Koordinator Bidang Hilirisasi dan Transisi</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8309933/puan-dorong-ipu-perkuat-peran-perdamaian-dan-tatanan-global-lebih-adil</t>
+          <t>https://www.liputan6.com/news/read/8310871/bahlil-bocorkan-kementerian-yang-bakal-berada-di-bawah-menko-hilirisasi</t>
         </is>
       </c>
     </row>
@@ -2343,22 +2343,22 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Yusril Ungkap Lapas Penuh Sesak, 25 Orang Berbagi Satu Sel</t>
+          <t>Tawuran Pemuda di Jaktim Digagalkan Patroli Polisi, 9 Celurit Disita</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Fri, 09 Oct 2026 20:12:08 +0700</t>
+          <t>Sun, 11 Oct 2026 21:59:42 +0700</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Yusril menyebut lapas dan rutan di Indonesia dihuni hampir dua kali kapasitas ideal. Perubahan kebijakan pemidanaan menjadi salah satu upaya untuk mengurangi kepadatan.</t>
+          <t>Penindakan dilakukan setelah polisi menerima aduan masyarakat.</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8309919/yusril-ungkap-lapas-penuh-sesak-25-orang-berbagi-satu-sel</t>
+          <t>https://www.liputan6.com/news/read/8310864/tawuran-pemuda-di-jaktim-digagalkan-patroli-polisi-9-celurit-disita</t>
         </is>
       </c>
     </row>
@@ -2370,22 +2370,22 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Sikap Yusril Tekait Putusan MK soal Gibran</t>
+          <t>Peringati 100 Tahun Frans Seda, IMDE Gelar Lomba Film Vertikal</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Fri, 09 Oct 2026 19:42:11 +0700</t>
+          <t>Sun, 11 Oct 2026 20:22:02 +0700</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Posisinya sebagai anggota kabinet membuatnya perlu menjaga sikap terhadap persoalan yang menyangkut Wakil Presiden.</t>
+          <t>IMDE dan Frans Seda Foundation menggelar lomba film vertikal untuk pelajar SMA/SMK. Kompetisi ini mengangkat keberagaman, toleransi, dan kebersamaan.</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8309906/sikap-yusril-tekait-putusan-mk-soal-gibran</t>
+          <t>https://www.liputan6.com/news/read/8310823/peringati-100-tahun-frans-seda-imde-gelar-lomba-film-vertikal</t>
         </is>
       </c>
     </row>
@@ -2397,22 +2397,22 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>85 Orang Mengaku Jadi Korban Investasi Emas, Kerugian Rp 25 Miliar</t>
+          <t>Momen Prabowo Lepas Kepulangan Presiden Mesir El-Sisi di Halim</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Fri, 09 Oct 2026 19:30:55 +0700</t>
+          <t>Sun, 11 Oct 2026 19:35:02 +0700</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Kasus dugaan penipuan jual beli emas dan perak ini menyeret PT Divine Gold Jewelry.</t>
+          <t>Prabowo mengantar Presiden Mesir Abdel Fattah el-Sisi hingga ke tangga pesawat sebelum bertolak kembali ke negaranya.</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8309901/85-orang-mengaku-jadi-korban-investasi-emas-kerugian-rp-25-miliar</t>
+          <t>https://www.liputan6.com/news/read/8310808/momen-prabowo-lepas-kepulangan-presiden-mesir-el-sisi-di-halim</t>
         </is>
       </c>
     </row>
@@ -2424,22 +2424,22 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>3 Anggota OPM Tewas Usai Kontak Tembak dengan TNI di Maybrat</t>
+          <t>Sekolah Anak Pesisir di NTB Padukan Edukasi Lingkungan dan Ekonomi Lokal</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Fri, 09 Oct 2026 19:24:11 +0700</t>
+          <t>Sun, 11 Oct 2026 19:43:41 +0700</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Kontak tembak terjadi di kawasan hutan sebelah utara Kampung Kamat, Distrik Aifat Timur.</t>
+          <t>Melalui pembelajaran berbasis alam, anak-anak di Desa Cendi Manik belajar merawat mangrove, memahami lingkungan, dan mengenal potensi ekonomi lokal.</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8309896/3-anggota-opm-tewas-usai-kontak-tembak-dengan-tni-di-maybrat</t>
+          <t>https://www.liputan6.com/news/read/8310807/sekolah-anak-pesisir-di-ntb-padukan-edukasi-lingkungan-dan-ekonomi-lokal</t>
         </is>
       </c>
     </row>
@@ -2451,22 +2451,22 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Kapolri Pimpin Sertijab Irwasum dan 4 Kapolda, Ini Daftarnya</t>
+          <t>Teka-Teki Kematian Pemuda di Kos Jakbar, Empat Saksi Diperiksa</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Fri, 09 Oct 2026 18:17:47 +0700</t>
+          <t>Sun, 11 Oct 2026 18:46:09 +0700</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Mutasi dan rotasi jabatan merupakan bagian dari dinamika organisasi.</t>
+          <t>Polisi belum mengungkap penyebab kematian Fajri yang ditemukan terbungkus di kos Jakbar.</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8309849/kapolri-pimpin-sertijab-irwasum-dan-4-kapolda-ini-daftarnya</t>
+          <t>https://www.liputan6.com/news/read/8310795/teka-teki-kematian-pemuda-di-kos-jakbar-empat-saksi-diperiksa</t>
         </is>
       </c>
     </row>
@@ -2478,22 +2478,22 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Jelang Pemilihan Presiden IPU, Puan Dorong Perempuan di Politik</t>
+          <t>Cairan Pemadam Brasil Diuji di Kebakaran Gambut Sumsel</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Fri, 09 Oct 2026 18:20:41 +0700</t>
+          <t>Sun, 11 Oct 2026 18:36:07 +0700</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Puan Maharani bertemu Ketua Parlemen Azerbaijan Sahiba Gafarova di sela Sidang Umum IPU ke-153 dan membahas penguatan kepemimpinan serta partisipasi perempuan dalam politik.</t>
+          <t>Pemerintah menguji bahan pemadam kebakaran asal Brasil di Banyuasin, Sumatera Selatan, untuk membantu menghambat penyebaran karhutla, termasuk di lahan gambut.</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8309854/jelang-pemilihan-presiden-ipu-puan-dorong-perempuan-di-politik</t>
+          <t>https://www.liputan6.com/news/read/8310792/cairan-pemadam-brasil-diuji-di-kebakaran-gambut-sumsel</t>
         </is>
       </c>
     </row>
@@ -2505,22 +2505,22 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Fakta di Balik Mahasiswa Tertabrak KRL di Ciputat</t>
+          <t>Hasil Olah TKP Kematian Pemuda Terbungkus Sleeping Bag di Kos Jakbar</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Fri, 09 Oct 2026 18:01:42 +0700</t>
+          <t>Sun, 11 Oct 2026 18:22:59 +0700</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Insiden ini sempat menyebabkan keterlambatan perjalanan KRL.</t>
+          <t>Polisi mendalami kematian pemuda yang ditemukan terbungkus sleeping bag di kamar kos Kebon Jeruk, Jakarta Barat.</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8309831/fakta-di-balik-mahasiswa-tertabrak-krl-di-ciputat</t>
+          <t>https://www.liputan6.com/news/read/8310788/hasil-olah-tkp-kematian-pemuda-terbungkus-sleeping-bag-di-kos-jakbar</t>
         </is>
       </c>
     </row>
@@ -2532,22 +2532,22 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Perempuan Terikat Ditemukan Tewas di Pinang Ranti, 2 Tersangka Ditangkap</t>
+          <t>Prabowo dan El-Sisi Dorong Deeskalasi Konflik Timur Tengah Lewat Diplomasi</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Fri, 09 Oct 2026 17:44:23 +0700</t>
+          <t>Sun, 11 Oct 2026 17:37:26 +0700</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Pengungkapan kasus tersebut dilakukan melalui serangkaian penyelidikan,</t>
+          <t>Prabowo dan El-Sisi menekankan pentingnya koordinasi internasional dan penyelesaian konflik melalui dialog tanpa mencampuri urusan dalam negeri negara lain.</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8309817/perempuan-terikat-ditemukan-tewas-di-pinang-ranti-2-tersangka-ditangkap</t>
+          <t>https://www.liputan6.com/news/read/8310769/prabowo-dan-el-sisi-dorong-deeskalasi-konflik-timur-tengah-lewat-diplomasi</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data pasar & berita - 2026-10-12 17:39 UTC
</commit_message>
<xml_diff>
--- a/data/market_news_latest.xlsx
+++ b/data/market_news_latest.xlsx
@@ -422,7 +422,7 @@
     <col width="26" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
   </cols>
@@ -521,20 +521,20 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>7811.54</v>
+        <v>7803.1602</v>
       </c>
       <c r="F3" t="n">
-        <v>46.1802</v>
+        <v>-8.379899999999999</v>
       </c>
       <c r="G3" t="n">
-        <v>0.59</v>
+        <v>-0.11</v>
       </c>
       <c r="H3" t="n">
-        <v>4782640000</v>
+        <v>1099785000</v>
       </c>
     </row>
     <row r="4">
@@ -555,20 +555,20 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>51654.9492</v>
+        <v>51862.4688</v>
       </c>
       <c r="F4" t="n">
-        <v>423.3086</v>
+        <v>207.5195</v>
       </c>
       <c r="G4" t="n">
-        <v>0.83</v>
+        <v>0.4</v>
       </c>
       <c r="H4" t="n">
-        <v>339470000</v>
+        <v>159170043</v>
       </c>
     </row>
     <row r="5">
@@ -589,20 +589,20 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>27366.1699</v>
+        <v>27242.8789</v>
       </c>
       <c r="F5" t="n">
-        <v>172.8301</v>
+        <v>-123.291</v>
       </c>
       <c r="G5" t="n">
-        <v>0.64</v>
+        <v>-0.45</v>
       </c>
       <c r="H5" t="n">
-        <v>6845310000</v>
+        <v>3413307000</v>
       </c>
     </row>
     <row r="6">
@@ -691,20 +691,14 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="E8" t="n">
-        <v>3813.791</v>
-      </c>
-      <c r="F8" t="n">
-        <v>1.887</v>
-      </c>
-      <c r="G8" t="n">
-        <v>0.05</v>
-      </c>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
       <c r="H8" t="n">
-        <v>535100</v>
+        <v>3195225140</v>
       </c>
     </row>
     <row r="9">
@@ -725,20 +719,20 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>10552.0996</v>
+        <v>10656.2803</v>
       </c>
       <c r="F9" t="n">
-        <v>110.5</v>
+        <v>104.1807</v>
       </c>
       <c r="G9" t="n">
-        <v>1.06</v>
+        <v>0.99</v>
       </c>
       <c r="H9" t="n">
-        <v>787988200</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -759,20 +753,20 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>25087.2695</v>
+        <v>25277.6797</v>
       </c>
       <c r="F10" t="n">
-        <v>280.2988</v>
+        <v>190.4102</v>
       </c>
       <c r="G10" t="n">
-        <v>1.13</v>
+        <v>0.76</v>
       </c>
       <c r="H10" t="n">
-        <v>59039100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -827,17 +821,17 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>17879</v>
+        <v>17894</v>
       </c>
       <c r="F12" t="n">
-        <v>71.5</v>
+        <v>86.5</v>
       </c>
       <c r="G12" t="n">
-        <v>0.4</v>
+        <v>0.49</v>
       </c>
       <c r="H12" t="n">
         <v>0</v>
@@ -861,17 +855,17 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>102.133</v>
+        <v>102.567</v>
       </c>
       <c r="F13" t="n">
-        <v>-0.077</v>
+        <v>0.357</v>
       </c>
       <c r="G13" t="n">
-        <v>-0.08</v>
+        <v>0.35</v>
       </c>
       <c r="H13" t="n">
         <v>0</v>
@@ -899,13 +893,13 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>158.129</v>
+        <v>158.628</v>
       </c>
       <c r="F14" t="n">
-        <v>0.066</v>
+        <v>0.5649999999999999</v>
       </c>
       <c r="G14" t="n">
-        <v>0.04</v>
+        <v>0.36</v>
       </c>
       <c r="H14" t="n">
         <v>0</v>
@@ -929,17 +923,17 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>0.5244</v>
+        <v>0.524</v>
       </c>
       <c r="F15" t="n">
-        <v>0.0013</v>
+        <v>-0.0004</v>
       </c>
       <c r="G15" t="n">
-        <v>0.25</v>
+        <v>-0.08</v>
       </c>
       <c r="H15" t="n">
         <v>0</v>
@@ -963,17 +957,17 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.5598</v>
       </c>
       <c r="F16" t="n">
-        <v>-0.0005999999999999999</v>
+        <v>-0.0002</v>
       </c>
       <c r="G16" t="n">
-        <v>-0.11</v>
+        <v>-0.04</v>
       </c>
       <c r="H16" t="n">
         <v>0</v>
@@ -997,17 +991,17 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>0.4057</v>
+        <v>0.405</v>
       </c>
       <c r="F17" t="n">
-        <v>0.0014</v>
+        <v>-0.0007</v>
       </c>
       <c r="G17" t="n">
-        <v>0.35</v>
+        <v>-0.17</v>
       </c>
       <c r="H17" t="n">
         <v>0</v>
@@ -1031,20 +1025,20 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="E18" t="n">
         <v>77.98</v>
       </c>
       <c r="F18" t="n">
-        <v>0.11</v>
+        <v>0</v>
       </c>
       <c r="G18" t="n">
-        <v>0.14</v>
+        <v>0</v>
       </c>
       <c r="H18" t="n">
-        <v>27247700</v>
+        <v>9233293</v>
       </c>
     </row>
     <row r="19">
@@ -1065,20 +1059,20 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>77.23</v>
+        <v>77.39</v>
       </c>
       <c r="F19" t="n">
-        <v>0.09</v>
+        <v>0.16</v>
       </c>
       <c r="G19" t="n">
-        <v>0.12</v>
+        <v>0.21</v>
       </c>
       <c r="H19" t="n">
-        <v>36922300</v>
+        <v>9546926</v>
       </c>
     </row>
     <row r="20">
@@ -1099,20 +1093,20 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>4230.3999</v>
+        <v>4191.3999</v>
       </c>
       <c r="F20" t="n">
-        <v>14.1001</v>
+        <v>-24.8999</v>
       </c>
       <c r="G20" t="n">
-        <v>0.33</v>
+        <v>-0.59</v>
       </c>
       <c r="H20" t="n">
-        <v>8668</v>
+        <v>91365</v>
       </c>
     </row>
     <row r="21">
@@ -1133,20 +1127,20 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>90.58</v>
+        <v>93.78</v>
       </c>
       <c r="F21" t="n">
-        <v>-1.27</v>
+        <v>1.93</v>
       </c>
       <c r="G21" t="n">
-        <v>-1.38</v>
+        <v>2.1</v>
       </c>
       <c r="H21" t="n">
-        <v>11066</v>
+        <v>155677</v>
       </c>
     </row>
     <row r="22">
@@ -1167,20 +1161,20 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="E22" t="n">
-        <v>103.38</v>
+        <v>106.71</v>
       </c>
       <c r="F22" t="n">
-        <v>-1.34</v>
+        <v>1.99</v>
       </c>
       <c r="G22" t="n">
-        <v>-1.28</v>
+        <v>1.9</v>
       </c>
       <c r="H22" t="n">
-        <v>2422</v>
+        <v>28104</v>
       </c>
     </row>
     <row r="23">
@@ -1201,20 +1195,20 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="E23" t="n">
-        <v>6.7195</v>
+        <v>6.748</v>
       </c>
       <c r="F23" t="n">
-        <v>0.077</v>
+        <v>0.1055</v>
       </c>
       <c r="G23" t="n">
-        <v>1.16</v>
+        <v>1.59</v>
       </c>
       <c r="H23" t="n">
-        <v>1207</v>
+        <v>26599</v>
       </c>
     </row>
     <row r="24">
@@ -1235,20 +1229,20 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="E24" t="n">
-        <v>66.8</v>
+        <v>66.16500000000001</v>
       </c>
       <c r="F24" t="n">
-        <v>0.7</v>
+        <v>-0.635</v>
       </c>
       <c r="G24" t="n">
-        <v>1.06</v>
+        <v>-0.95</v>
       </c>
       <c r="H24" t="n">
-        <v>14966000</v>
+        <v>5358901</v>
       </c>
     </row>
     <row r="25">
@@ -1269,17 +1263,17 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="E25" t="n">
-        <v>14.84</v>
+        <v>15.22</v>
       </c>
       <c r="F25" t="n">
-        <v>-0.57</v>
+        <v>0.38</v>
       </c>
       <c r="G25" t="n">
-        <v>-3.7</v>
+        <v>2.56</v>
       </c>
       <c r="H25" t="n">
         <v>0</v>
@@ -1307,16 +1301,16 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>83765.10159999999</v>
+        <v>82362.1562</v>
       </c>
       <c r="F26" t="n">
-        <v>852.875</v>
+        <v>-1317.3125</v>
       </c>
       <c r="G26" t="n">
-        <v>1.03</v>
+        <v>-1.57</v>
       </c>
       <c r="H26" t="n">
-        <v>12825135104</v>
+        <v>22718736384</v>
       </c>
     </row>
     <row r="27">
@@ -1337,20 +1331,14 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="E27" t="n">
-        <v>1405</v>
-      </c>
-      <c r="F27" t="n">
-        <v>15</v>
-      </c>
-      <c r="G27" t="n">
-        <v>1.08</v>
-      </c>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr"/>
       <c r="H27" t="n">
-        <v>29789700</v>
+        <v>74254500</v>
       </c>
     </row>
     <row r="28">
@@ -1371,20 +1359,14 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="E28" t="n">
-        <v>1675</v>
-      </c>
-      <c r="F28" t="n">
-        <v>5</v>
-      </c>
-      <c r="G28" t="n">
-        <v>0.3</v>
-      </c>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr"/>
       <c r="H28" t="n">
-        <v>53663900</v>
+        <v>268524800</v>
       </c>
     </row>
     <row r="29">
@@ -1405,20 +1387,14 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="E29" t="n">
-        <v>770</v>
-      </c>
-      <c r="F29" t="n">
-        <v>5</v>
-      </c>
-      <c r="G29" t="n">
-        <v>0.65</v>
-      </c>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr"/>
+      <c r="F29" t="inlineStr"/>
+      <c r="G29" t="inlineStr"/>
       <c r="H29" t="n">
-        <v>274141700</v>
+        <v>726868700</v>
       </c>
     </row>
     <row r="30">
@@ -1439,20 +1415,14 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="E30" t="n">
-        <v>2700</v>
-      </c>
-      <c r="F30" t="n">
-        <v>40</v>
-      </c>
-      <c r="G30" t="n">
-        <v>1.5</v>
-      </c>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr"/>
+      <c r="F30" t="inlineStr"/>
+      <c r="G30" t="inlineStr"/>
       <c r="H30" t="n">
-        <v>4298000</v>
+        <v>28644700</v>
       </c>
     </row>
     <row r="31">
@@ -1473,20 +1443,14 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="E31" t="n">
-        <v>4750</v>
-      </c>
-      <c r="F31" t="n">
-        <v>0</v>
-      </c>
-      <c r="G31" t="n">
-        <v>0</v>
-      </c>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr"/>
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="inlineStr"/>
       <c r="H31" t="n">
-        <v>43558600</v>
+        <v>89943800</v>
       </c>
     </row>
     <row r="32">
@@ -1507,20 +1471,14 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="E32" t="n">
-        <v>555</v>
-      </c>
-      <c r="F32" t="n">
-        <v>5</v>
-      </c>
-      <c r="G32" t="n">
-        <v>0.91</v>
-      </c>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr"/>
+      <c r="F32" t="inlineStr"/>
+      <c r="G32" t="inlineStr"/>
       <c r="H32" t="n">
-        <v>16507700</v>
+        <v>48885500</v>
       </c>
     </row>
     <row r="33">
@@ -1541,20 +1499,14 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="E33" t="n">
-        <v>665</v>
-      </c>
-      <c r="F33" t="n">
-        <v>0</v>
-      </c>
-      <c r="G33" t="n">
-        <v>0</v>
-      </c>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr"/>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr"/>
       <c r="H33" t="n">
-        <v>51395100</v>
+        <v>67193800</v>
       </c>
     </row>
     <row r="34">
@@ -1575,20 +1527,14 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="E34" t="n">
-        <v>4040</v>
-      </c>
-      <c r="F34" t="n">
-        <v>10</v>
-      </c>
-      <c r="G34" t="n">
-        <v>0.25</v>
-      </c>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr"/>
+      <c r="F34" t="inlineStr"/>
+      <c r="G34" t="inlineStr"/>
       <c r="H34" t="n">
-        <v>2328400</v>
+        <v>9716100</v>
       </c>
     </row>
     <row r="35">
@@ -1609,20 +1555,14 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="E35" t="n">
-        <v>665</v>
-      </c>
-      <c r="F35" t="n">
-        <v>20</v>
-      </c>
-      <c r="G35" t="n">
-        <v>3.1</v>
-      </c>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr"/>
+      <c r="F35" t="inlineStr"/>
+      <c r="G35" t="inlineStr"/>
       <c r="H35" t="n">
-        <v>64139600</v>
+        <v>163564500</v>
       </c>
     </row>
     <row r="36">
@@ -1643,20 +1583,14 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="E36" t="n">
-        <v>210</v>
-      </c>
-      <c r="F36" t="n">
-        <v>6</v>
-      </c>
-      <c r="G36" t="n">
-        <v>2.94</v>
-      </c>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr"/>
+      <c r="F36" t="inlineStr"/>
+      <c r="G36" t="inlineStr"/>
       <c r="H36" t="n">
-        <v>16999100</v>
+        <v>45688900</v>
       </c>
     </row>
     <row r="37">
@@ -1677,20 +1611,14 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="E37" t="n">
-        <v>15800</v>
-      </c>
-      <c r="F37" t="n">
-        <v>800</v>
-      </c>
-      <c r="G37" t="n">
-        <v>5.33</v>
-      </c>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr"/>
+      <c r="F37" t="inlineStr"/>
+      <c r="G37" t="inlineStr"/>
       <c r="H37" t="n">
-        <v>13766800</v>
+        <v>20278800</v>
       </c>
     </row>
   </sheetData>
@@ -1749,22 +1677,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Terkuak Modus Penipuan Tawarkan Urus Dapur MBG Kilat</t>
+          <t>RI Genjot Koperasi Pertanian Bareng Negara Tetangga</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Mon, 12 Oct 2026 07:30:14 +0700</t>
+          <t>Mon, 12 Oct 2026 22:30:09 +0700</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/10/10/bandung-hadirkan-sppg-baru-2400-paket-makan-bergizi-siap-untuk-anak-sekolah-1760085494045_169.jpeg?w=360&amp;amp;q=90" /&gt; Badan Gizi Nasional (BGN) membongkar modus penipuan yang menawarkan pembukaan dapur Makan Bergizi Gratis (MBG) </t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/07/wakil-menteri-koperasi-wamenkop-farida-farichah-usai-menghadiri-pelantikan-dpd-knpi-lamongan-1791355884634_169.jpeg?w=360&amp;amp;q=90" /&gt; Indonesia menjalin kerja sama pengembangan koperasi pertanian bersama negara-negara ASEAN.</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8702504/terkuak-modus-penipuan-tawarkan-urus-dapur-mbg-kilat</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8704136/ri-genjot-koperasi-pertanian-bareng-negara-tetangga</t>
         </is>
       </c>
     </row>
@@ -1776,22 +1704,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Waspada, El Nino Berpotensi Picu Kenaikan Harga Cabai dan Daging Ayam</t>
+          <t>Konsumsi Pertalite Melonjak hingga Antre Panjang di SPBU, Pertamina Buka Suara</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Mon, 12 Oct 2026 07:00:19 +0700</t>
+          <t>Mon, 12 Oct 2026 21:40:33 +0700</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/11/waspada-el-nino-berpotensi-picu-kenaikan-harga-cabai-dan-daging-ayam-1791706439905_169.jpeg?w=360&amp;amp;q=90" /&gt; Pemerintah mewaspadai dampak El Nino terhadap harga pangan. Cabai rawit, cabai merah, dan daging ayam berpotensi naik </t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/08/20/pemerintah-perketat-penyaluran-pertalite-mulai-2027-1787210254331_169.jpeg?w=360&amp;amp;q=90" /&gt; PT Pertamina Patra Niaga turun tangan memasok bahan bakar minyak (BBM) Kabupaten Bondowoso, Jawa Timur, seiring peningkatan kebutuhan m</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/foto-bisnis/d-8702088/waspada-el-nino-berpotensi-picu-kenaikan-harga-cabai-dan-daging-ayam</t>
+          <t>https://finance.detik.com/energi/d-8704079/konsumsi-pertalite-melonjak-hingga-antre-panjang-di-spbu-pertamina-buka-suara</t>
         </is>
       </c>
     </row>
@@ -1803,22 +1731,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Rencana Pemerintah Tambal Defisit di Akhir Tahun</t>
+          <t>RI Bidik Peluang Investasi Lewat Penguatan Pasar Karbon di COP31</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Mon, 12 Oct 2026 06:30:20 +0700</t>
+          <t>Mon, 12 Oct 2026 21:13:52 +0700</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2016/07/28/752567fe-0498-4b0f-9fd8-cde307b5d122_169.jpg?w=360&amp;amp;q=90" /&gt; Kemenkeu memperkirakan defisit Anggaran Pendapatan Belanja Negara (APBN) hingga akhir tahun mencapai 2,85% terhadap Produk Domestik Bruto (PDB).</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/12/ri-bidik-peluang-investasi-lewat-penguatan-pasar-karbon-di-cop31-1791814371200.jpeg?w=360&amp;amp;q=90" /&gt; Pemerintah dorong pasar karbon untuk investasi hijau di Indonesia. Menjelang COP31, Zulkifli Hasan tekankan pentingnya pembiay</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8702496/rencana-pemerintah-tambal-defisit-di-akhir-tahun</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8704059/ri-bidik-peluang-investasi-lewat-penguatan-pasar-karbon-di-cop31</t>
         </is>
       </c>
     </row>
@@ -1830,22 +1758,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Gelaran Pertamina Grand Prix of Indonesia 2026 Perkuat Ekonomi Lokal</t>
+          <t>Harga Minyak Mentah Indonesia Naik, Tembus US$ 112,81/ Barel</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Mon, 12 Oct 2026 06:08:28 +0700</t>
+          <t>Mon, 12 Oct 2026 21:04:03 +0700</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/12/gelaran-pertamina-grand-prix-of-indonesia-2026-perkuat-ekonomi-lokal-1791760079211.jpeg?w=360&amp;amp;q=90" /&gt; Pertamina Grand Prix of Indonesia 2026 sukses digelar di Mandalika, menarik perhatian global dan mendukung ekonomi lokal m</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/08/09/kilang-pertamina-1786240625862_169.jpeg?w=360&amp;amp;q=90" /&gt; Pemerintah menetapkan rata-rata Harga Minyak Mentah Indonesia atau Indonesian Crude Price (ICP) September 2026 sebesar US$112,81 per barel</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8702653/gelaran-pertamina-grand-prix-of-indonesia-2026-perkuat-ekonomi-lokal</t>
+          <t>https://finance.detik.com/energi/d-8704053/harga-minyak-mentah-indonesia-naik-tembus-us-112-81-barel</t>
         </is>
       </c>
     </row>
@@ -1857,22 +1785,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>63.789 Orang Jadi Korban PHK, Paling Banyak dari Provinsi Ini</t>
+          <t>Harga Sapi Hidup Tinggi, RI Impor Kerbau Australia</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Mon, 12 Oct 2026 05:55:13 +0700</t>
+          <t>Mon, 12 Oct 2026 20:48:31 +0700</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2019/07/30/559b04c3-168f-4c87-b3d4-cfad79eb8e5a_169.jpeg?w=360&amp;amp;q=90" /&gt; Data pemutusan hubungan kerja (PHK) terbaru kembali dirilis Kementerian Ketenagakerjaan.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2021/05/20/indonesia-hentikan-sementara-impor-daging-kerbau-dari-india-terkait-pandemi-covid-19_169.jpeg?w=360&amp;amp;q=90" /&gt; PT Berdikari (Persero) resmi menerima kedatangan perdana kerbau hidup (Water Buffalo) asal Australia pada Minggu sor</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8702493/63-789-orang-jadi-korban-phk-paling-banyak-dari-provinsi-ini</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8704035/harga-sapi-hidup-tinggi-ri-impor-kerbau-australia</t>
         </is>
       </c>
     </row>
@@ -1884,22 +1812,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Bawa 30 UMKM ke Sirkuit Mandalika, Pertamina Dorong Ekonomi Lokal Berdaya</t>
+          <t>PAM Jaya Jajaki IPO, Direksi Sowan ke OJK</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Sun, 11 Oct 2026 22:21:12 +0700</t>
+          <t>Mon, 12 Oct 2026 20:22:50 +0700</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/11/pertamina-1791731991936.jpeg?w=360&amp;amp;q=90" /&gt; PT Pertamina membawa 30 UMKM ke Pertamina Grand Prix of Indonesia 2026. Mereka berpartisipasi di bazar untuk memperluas pasar dan meningkatkan pendapatan.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/09/30/ilustrasi-distribusi-air-bersih-pam-jaya-1759220832502_169.jpeg?w=360&amp;amp;q=90" /&gt; PT Air Minum Jaya (Perseroda) atau PAM Jaya disebut mulai menjajaki penawaran umum perdana saham atau initial public offering (IPO).</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8702573/bawa-30-umkm-ke-sirkuit-mandalika-pertamina-dorong-ekonomi-lokal-berdaya</t>
+          <t>https://finance.detik.com/bursa-dan-valas/d-8704019/pam-jaya-jajaki-ipo-direksi-sowan-ke-ojk</t>
         </is>
       </c>
     </row>
@@ -1911,22 +1839,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Kementerian ATR &amp;amp; BRAN Mulai Bagi-bagi Tugas</t>
+          <t>Kementan Tambah Anggaran Rp 600 Miliar untuk Peternakan-Bibit Ayam Jatim</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Sun, 11 Oct 2026 22:00:52 +0700</t>
+          <t>Mon, 12 Oct 2026 20:07:26 +0700</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/08/14/ilustrasi-kementerian-atrbpn-1755140401786_169.jpeg?w=360&amp;amp;q=90" /&gt; Kelembagaan Badan Reforma Agraria Nasional (BRAN) terus dimatangkan sebagai tindak lanjut dari Undang-Undang Pengaturan Reforma Agraria.</t>
+          <t xml:space="preserve">&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/12/kementan-tambah-anggaran-rp-600-miliar-untuk-peternakan-bibit-ayam-jatim-1791810366385_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Pertanian mengumumkan dukungan Rp3 triliun untuk Jawa Timur 2025-2026, termasuk Rp600 miliar untuk sektor </t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/infrastruktur/d-8701869/kementerian-atr-bran-mulai-bagi-bagi-tugas</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8704007/kementan-tambah-anggaran-rp-600-miliar-untuk-peternakan-bibit-ayam-jatim</t>
         </is>
       </c>
     </row>
@@ -1938,22 +1866,22 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>BSI Ajak Masyarakat Bantu Pulihkan Desa Wisata Sade di Lombok</t>
+          <t>Begini Jawaban Bos Bursa Efek soal IHSG Anjlok 2,59%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Sun, 11 Oct 2026 21:36:43 +0700</t>
+          <t>Mon, 12 Oct 2026 20:03:39 +0700</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/11/bsi-1791729263003_169.jpeg?w=360&amp;amp;q=90" /&gt; PT Bank Syariah Indonesia meluncurkan program 'Satu Benang untuk Sade' di Lombok untuk pemulihan ekonomi lokal pascabencana.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/07/13/direktur-utama-bei-jeffrey-hendrik-1783928734693_169.jpeg?w=360&amp;amp;q=90" /&gt; Indeks Harga Saham Gabungan (IHSG) anjlok 2,59% ke level 5.936,14 pada penutupan perdagangan Senin (12/10/2026).</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8702550/bsi-ajak-masyarakat-bantu-pulihkan-desa-wisata-sade-di-lombok</t>
+          <t>https://finance.detik.com/bursa-dan-valas/d-8704003/begini-jawaban-bos-bursa-efek-soal-ihsg-anjlok-2-59</t>
         </is>
       </c>
     </row>
@@ -1965,22 +1893,22 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Pertamina EP Rantau Bor 5 Sumur Baru di Aceh Tamiang</t>
+          <t>Dua Jembatan di Kalteng Diperbaiki, Telan Rp 3,16 Miliar</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Sun, 11 Oct 2026 21:00:37 +0700</t>
+          <t>Mon, 12 Oct 2026 19:50:35 +0700</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/11/pt-pertamina-ep-field-rantau-1791708867596_169.jpeg?w=360&amp;amp;q=90" /&gt; Pertamina EP Rantau Field melakukan pengeboran sumur baru di tengah pemulihan pascabencana banjir Aceh Tamiang.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/12/dua-jembatan-di-kalteng-diperbaiki-1791809412541_169.jpeg?w=360&amp;amp;q=90" /&gt; Kementerian Pekerjaan Umum (PU) memperbaiki Jembatan Pulau Telo dan Jembatan Pulau Petak yang membentang di sungai Kapuas, Kalimantan Tengah.</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8702140/pertamina-ep-rantau-bor-5-sumur-baru-di-aceh-tamiang</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8703981/dua-jembatan-di-kalteng-diperbaiki-telan-rp-3-16-miliar</t>
         </is>
       </c>
     </row>
@@ -1992,22 +1920,22 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Waspada! Ada Modus Penipuan Janjikan Urus Dapur MBG Kilat</t>
+          <t>IHSG Jatuh 2,5%, Balik ke Level 5.900an</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Sun, 11 Oct 2026 20:00:22 +0700</t>
+          <t>Mon, 12 Oct 2026 18:13:44 +0700</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/01/27/32-ribu-pegawai-inti-mbg-bakal-diangkat-jadi-asn-pppk-1769488598657_169.jpeg?w=360&amp;amp;q=90" /&gt; Juru Bicara BGN Tysa Novenny, mengatakan masyarakat perlu berhati-hati dalam menyikapi setiap tindakan yang mengatasnamakan BGN.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/06/04/ihsg-terpuruk-kekhawatiran-pasar-meningkat-1780558039793_169.jpeg?w=360&amp;amp;q=90" /&gt; IHSG hari ini jatuh 2,5% ke level 5.900an, dipicu aksi wait and see investor terhadap dinamika global dan konflik Houthi. Data inflasi AS jadi p</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8702086/waspada-ada-modus-penipuan-janjikan-urus-dapur-mbg-kilat</t>
+          <t>https://finance.detik.com/bursa-dan-valas/d-8703879/ihsg-jatuh-2-5-balik-ke-level-5-900an</t>
         </is>
       </c>
     </row>
@@ -2019,22 +1947,22 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Produk UMKM Ikut Mejeng di Gelaran MotoGP Mandalika</t>
+          <t>BULOG Cetak Rekor Pengadaan 4,13 Juta Ton Beras, Jatim Sumbang 23,7%</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Sun, 11 Oct 2026 19:30:18 +0700</t>
+          <t>Mon, 12 Oct 2026 16:58:19 +0700</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/11/produk-umkm-di-ajang-motogp-1791714381524_169.jpeg?w=360&amp;amp;q=90" /&gt; Pertamina melalui PT Pertamina Patra Niaga menghadirkan produk kerajinan unggulan Lombok sebagai official merchandise.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/12/bulog-cetak-rekor-pengadaan-413-juta-ton-beras-jatim-sumbang-237-1791798957038_169.jpeg?w=360&amp;amp;q=90" /&gt; Perum BULOG mencetak rekor pengadaan beras dengan serapan 4,13 juta ton, melampaui target nasional. Tasyakuran di Jatim me</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8702299/produk-umkm-ikut-mejeng-di-gelaran-motogp-mandalika</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8703713/bulog-cetak-rekor-pengadaan-4-13-juta-ton-beras-jatim-sumbang-23-7</t>
         </is>
       </c>
     </row>
@@ -2046,22 +1974,22 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Tambal Defisit, Pemerintah Mau Lelang 12 Surat Utang-Tarik Pinjaman US$ 1,8 M</t>
+          <t>PHE Akuisisi Saham Eni di 3 Blok Migas Strategis di Kalimantan Timur</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Sun, 11 Oct 2026 19:00:43 +0700</t>
+          <t>Mon, 12 Oct 2026 16:55:28 +0700</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2016/07/28/11b938f2-8964-482f-986f-f70f6458d154_169.jpg?w=360&amp;amp;q=90" /&gt; Direktur Jenderal Pengelolaan Pembiayaan dan Risiko (DJPPR) Kemenkeu Suminto mengatakan pemerintah masih mempunyai kesempatan untuk melelang 12 surat utang.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/23/pertamina-ep-1790145752344_169.jpeg?w=360&amp;amp;q=90" /&gt; PT Pertamina Hulu Energi akuisisi saham Eni di tiga blok migas strategis di Kalimantan Timur.</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8702060/tambal-defisit-pemerintah-mau-lelang-12-surat-utang-tarik-pinjaman-us-1-8-m</t>
+          <t>https://finance.detik.com/energi/d-8703708/phe-akuisisi-saham-eni-di-3-blok-migas-strategis-di-kalimantan-timur</t>
         </is>
       </c>
     </row>
@@ -2073,22 +2001,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Investasi Jakarta Tembus Rp173,6 Triliun, Tertinggi di Indonesia</t>
+          <t>Bayar Utang Pajak Kini Dahulukan Pokok Sebelum Denda, Ini Rinciannya</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Sun, 11 Oct 2026 18:00:25 +0700</t>
+          <t>Mon, 12 Oct 2026 16:50:42 +0700</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/10/investasi-jakarta-tembus-rp1736-triliun-hingga-semester-i2026-1791636661420.jpeg?w=360&amp;amp;q=90" /&gt; Realisasi investasi di Jakarta mencapai Rp173,6 triliun hingga semester I 2026, tertinggi di Indonesia, menurut Gubernur Pramono </t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2014/10/01/aba994a2-34ed-467e-b236-0838b109f70c_169.jpg?w=360&amp;amp;q=90" /&gt; Melalui ketentuan baru ini pembayaran akan diperhitungkan terlebih dahulu untuk melunasi pokok utang pajak.</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/foto-bisnis/d-8701303/investasi-jakarta-tembus-rp173-6-triliun-tertinggi-di-indonesia</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8703697/bayar-utang-pajak-kini-dahulukan-pokok-sebelum-denda-ini-rinciannya</t>
         </is>
       </c>
     </row>
@@ -2100,22 +2028,22 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Rosan Buka-bukaan soal Rencana Kerja Sama RI &amp;amp; Mesir</t>
+          <t>Di Depan Pengusaha Pribumi, Bahlil Klaim Keluarkan 4 Kebijakan Pro UMKM</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Sun, 11 Oct 2026 17:16:45 +0700</t>
+          <t>Mon, 12 Oct 2026 16:14:44 +0700</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/06/18/menteri-hilirisasi-dan-investasi-rosan-roeslani-kamis-1862026-1781790660049_169.jpeg?w=360&amp;amp;q=90" /&gt; CEO Danantara Rosan Roeslani mengatakan pihaknya akan membentuk dana kelolaan investasi dengan pihak Mesir.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/12/bahlil-lahadalia-1791784854378_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Bahlil mengumumkan 4 kebijakan pro-UMKM dalam pengelolaan sumber daya alam, termasuk legalisasi sumur minyak rakyat dan prioritas IUP untuk koperasi.</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8702287/rosan-buka-bukaan-soal-rencana-kerja-sama-ri-mesir</t>
+          <t>https://finance.detik.com/energi/d-8703599/di-depan-pengusaha-pribumi-bahlil-klaim-keluarkan-4-kebijakan-pro-umkm</t>
         </is>
       </c>
     </row>
@@ -2127,22 +2055,22 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Harga Emas Mulai Bangkit, Naik Segini dalam Sepekan</t>
+          <t>Budi Daya Lobster di RI Masih Belum Maksimal, Ini Alasannya</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Sun, 11 Oct 2026 16:00:43 +0700</t>
+          <t>Mon, 12 Oct 2026 15:59:32 +0700</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/10/15/harga-emas-antam-tembus-rekor-tertinggi-sentuh-rp238-juta-per-gram-1760532607071_169.jpeg?w=360&amp;amp;q=90" /&gt; Harga emas mengalami kenaikan Rp 12 ribu per gram selama sepekan ini.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/12/satgas-pemberantasan-benur-lobster-ilegal-dibentuk-tak-cuma-tangkap-kurir-1791785768415_169.jpeg?w=360&amp;amp;q=90" /&gt; Salah satu penyebabnya, nelayan lokal tergiur menjual BBL ke negara tetangga karena perbedaan harga yang sangat t</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8701980/harga-emas-mulai-bangkit-naik-segini-dalam-sepekan</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8703555/budi-daya-lobster-di-ri-masih-belum-maksimal-ini-alasannya</t>
         </is>
       </c>
     </row>
@@ -2154,22 +2082,22 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Dua Hari Berturut-turut Kebakaran di Wilayah Jakarta Utara</t>
+          <t>Menag Nasaruddin Ajak Tobat Ekologis, Ingatkan Bahaya Eksploitasi Alam</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Mon, 12 Oct 2026 07:38:34 +0700</t>
+          <t>Tue, 13 Oct 2026 00:06:28 +0700</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Belum dijelaskan kerugian akibat kebakaran dua lokasi tersebut.</t>
+          <t>Menag Nasaruddin Umar mengingatkan dampak kerusakan alam dan mengajak penerapan konsep ekoteologi dalam kehidupan sehari-hari.</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8310953/dua-hari-berturut-turut-kebakaran-di-wilayah-jakarta-utara</t>
+          <t>https://www.liputan6.com/news/read/8311654/menag-nasaruddin-ajak-tobat-ekologis-ingatkan-bahaya-eksploitasi-alam</t>
         </is>
       </c>
     </row>
@@ -2181,22 +2109,22 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Strategi Ada Gula Ada Semut Ala Mentrans di Festival Transmigrasi 2026</t>
+          <t>Tabligh Akbar di Monas, Habib Nabiel Ajak Umat Islam Jaga Persatuan</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Mon, 12 Oct 2026 06:59:05 +0700</t>
+          <t>Mon, 12 Oct 2026 23:58:20 +0700</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Festival Transmigrasi menjadi salah satu upaya untuk memperkenalkan potensi kawasan hingga pertukaran gagasan.</t>
+          <t>Dalam Tabligh Akbar di Monas, Habib Nabiel menyoroti perpecahan, korupsi, hingga kebiasaan memfitnah.</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8310941/strategi-ada-gula-ada-semut-ala-mentrans-di-festival-transmigrasi-2026</t>
+          <t>https://www.liputan6.com/news/read/8311651/tabligh-akbar-di-monas-habib-nabiel-ajak-umat-islam-jaga-persatuan</t>
         </is>
       </c>
     </row>
@@ -2208,22 +2136,22 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Nestapa 46 Orangutan Terjebak di Sisa Hutan Terbakar</t>
+          <t>Infografis: 5 Miliarder Asia dengan Penurunan Kekayaan Terbesar</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Mon, 12 Oct 2026 06:33:51 +0700</t>
+          <t>Mon, 12 Oct 2026 22:52:51 +0700</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>46 Individu Orangutan terjebak kebakaran hutan</t>
+          <t>Miliarder  dari China, Indonesia, dan Korea Selatan mengalami penurunan kekayaan dengan nilai fantastis.</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8310938/nestapa-46-orangutan-terjebak-di-sisa-hutan-terbakar</t>
+          <t>https://www.liputan6.com/news/read/8311630/infografis-5-miliarder-asia-dengan-penurunan-kekayaan-terbesar</t>
         </is>
       </c>
     </row>
@@ -2235,22 +2163,22 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Gempa Magnitudo 5,7 Guncang Pohuwato Gorontalo</t>
+          <t>Prabowo Kerahkan Seluruh Sumber Daya untuk Tangani Kabakaran Hutan</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Mon, 12 Oct 2026 05:20:05 +0700</t>
+          <t>Tue, 13 Oct 2026 00:12:43 +0700</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Gempa tidak berpotensi tsunami.</t>
+          <t>Sebanyak 60.177 personel gabungan dikerahkan untuk menangani kebakaran hutan dan lahan.</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8310918/gempa-magnitudo-57-guncang-pohuwato-gorontalo</t>
+          <t>https://www.liputan6.com/news/read/8311629/prabowo-kerahkan-seluruh-sumber-daya-untuk-tangani-kabakaran-hutan</t>
         </is>
       </c>
     </row>
@@ -2262,22 +2190,22 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Cerita Bahlil, dari Jualan Kue Cucur hingga Alami Busung Lapar</t>
+          <t>Jemaah Umrah Indonesia Dikabarkan Aman, Kemenhaj Minta Tetap Waspada</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Sun, 11 Oct 2026 23:59:40 +0700</t>
+          <t>Mon, 12 Oct 2026 22:31:58 +0700</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Bahlil Lahadalia mengenang perjuangan semasa kecilnya, mulai dari berjualan kue cucur hingga mengalami busung lapar.</t>
+          <t>Jemaah umrah Indonesiadi Arab Saudi diminta tetap waspada dan mengutamakan keselamatan.</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8310900/cerita-bahlil-dari-jualan-kue-cucur-hingga-alami-busung-lapar</t>
+          <t>https://www.liputan6.com/news/read/8311624/jemaah-umrah-indonesia-dikabarkan-aman-kemenhaj-minta-tetap-waspada</t>
         </is>
       </c>
     </row>
@@ -2289,22 +2217,22 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Lapak Barang Bekas di Kalideres Kebakaran</t>
+          <t>BRAN Percepat Penataan Kelembagaan dan Regulasi Reforma Agraria</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Sun, 11 Oct 2026 23:46:18 +0700</t>
+          <t>Mon, 12 Oct 2026 21:50:39 +0700</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Petugas pemadam kebakaran menerima informasi kejadian dari warga pada pukul 23.13 WIB.</t>
+          <t>BRAN menggandeng Kementerian Hukum dan berencana melibatkan akademisi untuk mengkaji regulasi yang menjadi landasan pelaksanaan reforma agraria.</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8310896/lapak-barang-bekas-di-kalideres-kebakaran</t>
+          <t>https://www.liputan6.com/news/read/8311607/bran-percepat-penataan-kelembagaan-dan-regulasi-reforma-agraria</t>
         </is>
       </c>
     </row>
@@ -2316,22 +2244,22 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Bahlil Bocorkan Kementerian yang Bakal Berada di Bawah Menko Hilirisasi</t>
+          <t>Mendagri Instruksikan Kepala Daerah Cegah Pembakaran Lahan</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Sun, 11 Oct 2026 22:30:07 +0700</t>
+          <t>Mon, 12 Oct 2026 20:27:46 +0700</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Bahlil memberikan bocoran mengenai sejumlah kementerian yang akan berada di bawah koordinasi Kementerian Koordinator Bidang Hilirisasi dan Transisi</t>
+          <t>Di tengah kondisi darurat karhutla dan lahan yang mengering akibat kemarau, pemerintah meminta tidak ada pembakaran lahan baru.</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8310871/bahlil-bocorkan-kementerian-yang-bakal-berada-di-bawah-menko-hilirisasi</t>
+          <t>https://www.liputan6.com/news/read/8311558/mendagri-instruksikan-kepala-daerah-cegah-pembakaran-lahan</t>
         </is>
       </c>
     </row>
@@ -2343,22 +2271,22 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Tawuran Pemuda di Jaktim Digagalkan Patroli Polisi, 9 Celurit Disita</t>
+          <t>Instruksi Prabowo Terkait Kebakaran Hutan di 6 Provinsi</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Sun, 11 Oct 2026 21:59:42 +0700</t>
+          <t>Mon, 12 Oct 2026 20:17:52 +0700</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Penindakan dilakukan setelah polisi menerima aduan masyarakat.</t>
+          <t>Prabowo ingin pencegahan dilakukan sebelum api menyala.</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8310864/tawuran-pemuda-di-jaktim-digagalkan-patroli-polisi-9-celurit-disita</t>
+          <t>https://www.liputan6.com/news/read/8311555/instruksi-prabowo-terkait-kebakaran-hutan-di-6-provinsi</t>
         </is>
       </c>
     </row>
@@ -2370,22 +2298,22 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Peringati 100 Tahun Frans Seda, IMDE Gelar Lomba Film Vertikal</t>
+          <t>Prabowo Tunjuk Satyawan Pudyatmoko Jadi Kepala Badan Pengelolaan Gambut dan Mangrove</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Sun, 11 Oct 2026 20:22:02 +0700</t>
+          <t>Mon, 12 Oct 2026 20:07:29 +0700</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>IMDE dan Frans Seda Foundation menggelar lomba film vertikal untuk pelajar SMA/SMK. Kompetisi ini mengangkat keberagaman, toleransi, dan kebersamaan.</t>
+          <t>Satyawan merupakan ahli di bidang pengelolaan gambut dan mangrove sehingga cocok memimpin badan tersebut.</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8310823/peringati-100-tahun-frans-seda-imde-gelar-lomba-film-vertikal</t>
+          <t>https://www.liputan6.com/news/read/8311541/prabowo-tunjuk-satyawan-pudyatmoko-jadi-kepala-badan-pengelolaan-gambut-dan-mangrove</t>
         </is>
       </c>
     </row>
@@ -2397,22 +2325,22 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Momen Prabowo Lepas Kepulangan Presiden Mesir El-Sisi di Halim</t>
+          <t>Separuh Anggaran Iklan BJB Jadi Dana Non-Budgeter, Siapa Penerimanya?</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Sun, 11 Oct 2026 19:35:02 +0700</t>
+          <t>Mon, 12 Oct 2026 19:33:50 +0700</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Prabowo mengantar Presiden Mesir Abdel Fattah el-Sisi hingga ke tangga pesawat sebelum bertolak kembali ke negaranya.</t>
+          <t>KPK mendalami dugaan penyisihan Rp 200 miliar dari pengadaan iklan Bank BJB. Penyidik menelusuri aliran dan peruntukan dana tersebut.</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8310808/momen-prabowo-lepas-kepulangan-presiden-mesir-el-sisi-di-halim</t>
+          <t>https://www.liputan6.com/news/read/8311524/separuh-anggaran-iklan-bjb-jadi-dana-non-budgeter-siapa-penerimanya</t>
         </is>
       </c>
     </row>
@@ -2424,22 +2352,22 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Sekolah Anak Pesisir di NTB Padukan Edukasi Lingkungan dan Ekonomi Lokal</t>
+          <t>Kebakaran Hutan Belum Berstatus Bencana Nasional, Dudung Ungkap Alasannya</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Sun, 11 Oct 2026 19:43:41 +0700</t>
+          <t>Mon, 12 Oct 2026 19:30:59 +0700</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Melalui pembelajaran berbasis alam, anak-anak di Desa Cendi Manik belajar merawat mangrove, memahami lingkungan, dan mengenal potensi ekonomi lokal.</t>
+          <t>Menko Polkam Dudung Abdurachman mengatakan pemerintah masih mampu menangani karhutla. Saat ini, penanganan difokuskan pada enam provinsi.</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8310807/sekolah-anak-pesisir-di-ntb-padukan-edukasi-lingkungan-dan-ekonomi-lokal</t>
+          <t>https://www.liputan6.com/news/read/8311537/kebakaran-hutan-belum-berstatus-bencana-nasional-dudung-ungkap-alasannya</t>
         </is>
       </c>
     </row>
@@ -2451,22 +2379,22 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Teka-Teki Kematian Pemuda di Kos Jakbar, Empat Saksi Diperiksa</t>
+          <t>Satpol PP dan Pekerja Proyek Bentrok, Begini Reaksi Pramono</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Sun, 11 Oct 2026 18:46:09 +0700</t>
+          <t>Mon, 12 Oct 2026 19:18:59 +0700</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Polisi belum mengungkap penyebab kematian Fajri yang ditemukan terbungkus di kos Jakbar.</t>
+          <t>Bentrokan antara petugas Satpol PP dan pekerja proyek di Bulungan viral di media sosial. Pramono Anung meminta hukum tetap ditegakkan.</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8310795/teka-teki-kematian-pemuda-di-kos-jakbar-empat-saksi-diperiksa</t>
+          <t>https://www.liputan6.com/news/read/8311529/satpol-pp-dan-pekerja-proyek-bentrok-begini-reaksi-pramono</t>
         </is>
       </c>
     </row>
@@ -2478,22 +2406,22 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Cairan Pemadam Brasil Diuji di Kebakaran Gambut Sumsel</t>
+          <t>Kapolri Lantik Kakorlantas dan Tiga Kapolda Baru</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Sun, 11 Oct 2026 18:36:07 +0700</t>
+          <t>Mon, 12 Oct 2026 20:07:12 +0700</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Pemerintah menguji bahan pemadam kebakaran asal Brasil di Banyuasin, Sumatera Selatan, untuk membantu menghambat penyebaran karhutla, termasuk di lahan gambut.</t>
+          <t>Kapolri memimpin pergantian Kakorlantas dan tiga Kapolda. Berikut daftar pejabat yang mengisi posisi baru.</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8310792/cairan-pemadam-brasil-diuji-di-kebakaran-gambut-sumsel</t>
+          <t>https://www.liputan6.com/news/read/8311495/kapolri-lantik-kakorlantas-dan-tiga-kapolda-baru</t>
         </is>
       </c>
     </row>
@@ -2505,22 +2433,22 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Hasil Olah TKP Kematian Pemuda Terbungkus Sleeping Bag di Kos Jakbar</t>
+          <t>Data Center AI Butuh Banyak Air, Menko AHY Beri Peringatan</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Sun, 11 Oct 2026 18:22:59 +0700</t>
+          <t>Mon, 12 Oct 2026 18:31:38 +0700</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Polisi mendalami kematian pemuda yang ditemukan terbungkus sleeping bag di kamar kos Kebon Jeruk, Jakarta Barat.</t>
+          <t>Kebutuhan air untuk pusat data AI menjadi sorotan AHY. Dia mengingatkan pentingnya menjaga pasokan air bersih bagi masyarakat.</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8310788/hasil-olah-tkp-kematian-pemuda-terbungkus-sleeping-bag-di-kos-jakbar</t>
+          <t>https://www.liputan6.com/news/read/8311477/data-center-ai-butuh-banyak-air-menko-ahy-beri-peringatan</t>
         </is>
       </c>
     </row>
@@ -2532,22 +2460,22 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Prabowo dan El-Sisi Dorong Deeskalasi Konflik Timur Tengah Lewat Diplomasi</t>
+          <t>KPK Geledah 3 Lokasi Terkait Kasus Bupati Pemalang, Ini Hasilnya</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Sun, 11 Oct 2026 17:37:26 +0700</t>
+          <t>Mon, 12 Oct 2026 18:29:51 +0700</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Prabowo dan El-Sisi menekankan pentingnya koordinasi internasional dan penyelesaian konflik melalui dialog tanpa mencampuri urusan dalam negeri negara lain.</t>
+          <t>KPK menyita dokumen dan barang bukti elektronik dari penggeledahan tiga lokasi terkait kasus Bupati Pemalang nonaktif.</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8310769/prabowo-dan-el-sisi-dorong-deeskalasi-konflik-timur-tengah-lewat-diplomasi</t>
+          <t>https://www.liputan6.com/news/read/8311494/kpk-geledah-3-lokasi-terkait-kasus-bupati-pemalang-ini-hasilnya</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data pasar & berita - 2026-10-13 02:44 UTC
</commit_message>
<xml_diff>
--- a/data/market_news_latest.xlsx
+++ b/data/market_news_latest.xlsx
@@ -422,7 +422,7 @@
     <col width="26" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
   </cols>
@@ -487,20 +487,20 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>6093.7588</v>
+        <v>5860.0571</v>
       </c>
       <c r="F2" t="n">
-        <v>62.4746</v>
+        <v>-76.0898</v>
       </c>
       <c r="G2" t="n">
-        <v>1.04</v>
+        <v>-1.28</v>
       </c>
       <c r="H2" t="n">
-        <v>350813700</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -525,16 +525,16 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>7803.1602</v>
+        <v>7807.2402</v>
       </c>
       <c r="F3" t="n">
-        <v>-8.379899999999999</v>
+        <v>-4.2998</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.11</v>
+        <v>-0.06</v>
       </c>
       <c r="H3" t="n">
-        <v>1099785000</v>
+        <v>2291949000</v>
       </c>
     </row>
     <row r="4">
@@ -559,16 +559,16 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>51862.4688</v>
+        <v>51850.5508</v>
       </c>
       <c r="F4" t="n">
-        <v>207.5195</v>
+        <v>195.6016</v>
       </c>
       <c r="G4" t="n">
-        <v>0.4</v>
+        <v>0.38</v>
       </c>
       <c r="H4" t="n">
-        <v>159170043</v>
+        <v>307464899</v>
       </c>
     </row>
     <row r="5">
@@ -593,16 +593,16 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>27242.8789</v>
+        <v>27245.9023</v>
       </c>
       <c r="F5" t="n">
-        <v>-123.291</v>
+        <v>-120.2676</v>
       </c>
       <c r="G5" t="n">
-        <v>-0.45</v>
+        <v>-0.44</v>
       </c>
       <c r="H5" t="n">
-        <v>3413307000</v>
+        <v>5794275000</v>
       </c>
     </row>
     <row r="6">
@@ -623,20 +623,20 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>69030.9219</v>
+        <v>67287.9219</v>
       </c>
       <c r="F6" t="n">
-        <v>-11.1875</v>
+        <v>-1743</v>
       </c>
       <c r="G6" t="n">
-        <v>-0.02</v>
+        <v>-2.52</v>
       </c>
       <c r="H6" t="n">
-        <v>162000000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -657,20 +657,20 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>24211.3496</v>
+        <v>24000.7598</v>
       </c>
       <c r="F7" t="n">
-        <v>425.5605</v>
+        <v>-270.4395</v>
       </c>
       <c r="G7" t="n">
-        <v>1.79</v>
+        <v>-1.11</v>
       </c>
       <c r="H7" t="n">
-        <v>2905300000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -691,14 +691,20 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>3756.5547</v>
+      </c>
+      <c r="F8" t="n">
+        <v>-40.6873</v>
+      </c>
+      <c r="G8" t="n">
+        <v>-1.07</v>
+      </c>
       <c r="H8" t="n">
-        <v>3195225140</v>
+        <v>893787720</v>
       </c>
     </row>
     <row r="9">
@@ -723,16 +729,16 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>10656.2803</v>
+        <v>10656.2998</v>
       </c>
       <c r="F9" t="n">
-        <v>104.1807</v>
+        <v>104.2002</v>
       </c>
       <c r="G9" t="n">
         <v>0.99</v>
       </c>
       <c r="H9" t="n">
-        <v>0</v>
+        <v>575809000</v>
       </c>
     </row>
     <row r="10">
@@ -766,7 +772,7 @@
         <v>0.76</v>
       </c>
       <c r="H10" t="n">
-        <v>0</v>
+        <v>39349200</v>
       </c>
     </row>
     <row r="11">
@@ -787,20 +793,20 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>5401.8901</v>
+        <v>5415.8901</v>
       </c>
       <c r="F11" t="n">
-        <v>-11.0698</v>
+        <v>0.4102</v>
       </c>
       <c r="G11" t="n">
-        <v>-0.2</v>
+        <v>0.01</v>
       </c>
       <c r="H11" t="n">
-        <v>341999600</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -821,7 +827,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="E12" t="n">
@@ -859,13 +865,13 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>102.567</v>
+        <v>102.417</v>
       </c>
       <c r="F13" t="n">
-        <v>0.357</v>
+        <v>0.207</v>
       </c>
       <c r="G13" t="n">
-        <v>0.35</v>
+        <v>0.2</v>
       </c>
       <c r="H13" t="n">
         <v>0</v>
@@ -889,17 +895,17 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>158.628</v>
+        <v>158.248</v>
       </c>
       <c r="F14" t="n">
-        <v>0.5649999999999999</v>
+        <v>0.185</v>
       </c>
       <c r="G14" t="n">
-        <v>0.36</v>
+        <v>0.12</v>
       </c>
       <c r="H14" t="n">
         <v>0</v>
@@ -1029,16 +1035,16 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>77.98</v>
+        <v>78.05</v>
       </c>
       <c r="F18" t="n">
-        <v>0</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="G18" t="n">
-        <v>0</v>
+        <v>0.09</v>
       </c>
       <c r="H18" t="n">
-        <v>9233293</v>
+        <v>15346700</v>
       </c>
     </row>
     <row r="19">
@@ -1063,16 +1069,16 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>77.39</v>
+        <v>77.29000000000001</v>
       </c>
       <c r="F19" t="n">
-        <v>0.16</v>
+        <v>0.06</v>
       </c>
       <c r="G19" t="n">
-        <v>0.21</v>
+        <v>0.08</v>
       </c>
       <c r="H19" t="n">
-        <v>9546926</v>
+        <v>21847900</v>
       </c>
     </row>
     <row r="20">
@@ -1097,16 +1103,16 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>4191.3999</v>
+        <v>4191.2998</v>
       </c>
       <c r="F20" t="n">
-        <v>-24.8999</v>
+        <v>-25</v>
       </c>
       <c r="G20" t="n">
         <v>-0.59</v>
       </c>
       <c r="H20" t="n">
-        <v>91365</v>
+        <v>18547</v>
       </c>
     </row>
     <row r="21">
@@ -1131,16 +1137,16 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>93.78</v>
+        <v>92.59999999999999</v>
       </c>
       <c r="F21" t="n">
-        <v>1.93</v>
+        <v>0.75</v>
       </c>
       <c r="G21" t="n">
-        <v>2.1</v>
+        <v>0.82</v>
       </c>
       <c r="H21" t="n">
-        <v>155677</v>
+        <v>9667</v>
       </c>
     </row>
     <row r="22">
@@ -1165,16 +1171,16 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>106.71</v>
+        <v>105.46</v>
       </c>
       <c r="F22" t="n">
-        <v>1.99</v>
+        <v>0.74</v>
       </c>
       <c r="G22" t="n">
-        <v>1.9</v>
+        <v>0.71</v>
       </c>
       <c r="H22" t="n">
-        <v>28104</v>
+        <v>1163</v>
       </c>
     </row>
     <row r="23">
@@ -1199,16 +1205,16 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>6.748</v>
+        <v>6.7085</v>
       </c>
       <c r="F23" t="n">
-        <v>0.1055</v>
+        <v>0.066</v>
       </c>
       <c r="G23" t="n">
-        <v>1.59</v>
+        <v>0.99</v>
       </c>
       <c r="H23" t="n">
-        <v>26599</v>
+        <v>2754</v>
       </c>
     </row>
     <row r="24">
@@ -1233,16 +1239,16 @@
         </is>
       </c>
       <c r="E24" t="n">
-        <v>66.16500000000001</v>
+        <v>66.15000000000001</v>
       </c>
       <c r="F24" t="n">
-        <v>-0.635</v>
+        <v>-0.65</v>
       </c>
       <c r="G24" t="n">
-        <v>-0.95</v>
+        <v>-0.97</v>
       </c>
       <c r="H24" t="n">
-        <v>5358901</v>
+        <v>10344700</v>
       </c>
     </row>
     <row r="25">
@@ -1267,13 +1273,13 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>15.22</v>
+        <v>15.21</v>
       </c>
       <c r="F25" t="n">
-        <v>0.38</v>
+        <v>0.37</v>
       </c>
       <c r="G25" t="n">
-        <v>2.56</v>
+        <v>2.49</v>
       </c>
       <c r="H25" t="n">
         <v>0</v>
@@ -1297,20 +1303,20 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="E26" t="n">
-        <v>82362.1562</v>
+        <v>82773.00780000001</v>
       </c>
       <c r="F26" t="n">
-        <v>-1317.3125</v>
+        <v>-906.4609</v>
       </c>
       <c r="G26" t="n">
-        <v>-1.57</v>
+        <v>-1.08</v>
       </c>
       <c r="H26" t="n">
-        <v>22718736384</v>
+        <v>29273978880</v>
       </c>
     </row>
     <row r="27">
@@ -1331,14 +1337,20 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr"/>
-      <c r="F27" t="inlineStr"/>
-      <c r="G27" t="inlineStr"/>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>1325</v>
+      </c>
+      <c r="F27" t="n">
+        <v>-80</v>
+      </c>
+      <c r="G27" t="n">
+        <v>-5.69</v>
+      </c>
       <c r="H27" t="n">
-        <v>74254500</v>
+        <v>21639800</v>
       </c>
     </row>
     <row r="28">
@@ -1359,14 +1371,20 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr"/>
-      <c r="F28" t="inlineStr"/>
-      <c r="G28" t="inlineStr"/>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>1470</v>
+      </c>
+      <c r="F28" t="n">
+        <v>-205</v>
+      </c>
+      <c r="G28" t="n">
+        <v>-12.24</v>
+      </c>
       <c r="H28" t="n">
-        <v>268524800</v>
+        <v>55172500</v>
       </c>
     </row>
     <row r="29">
@@ -1387,14 +1405,20 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr"/>
-      <c r="F29" t="inlineStr"/>
-      <c r="G29" t="inlineStr"/>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>670</v>
+      </c>
+      <c r="F29" t="n">
+        <v>-100</v>
+      </c>
+      <c r="G29" t="n">
+        <v>-12.99</v>
+      </c>
       <c r="H29" t="n">
-        <v>726868700</v>
+        <v>209845100</v>
       </c>
     </row>
     <row r="30">
@@ -1415,14 +1439,20 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr"/>
-      <c r="F30" t="inlineStr"/>
-      <c r="G30" t="inlineStr"/>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>2330</v>
+      </c>
+      <c r="F30" t="n">
+        <v>-370</v>
+      </c>
+      <c r="G30" t="n">
+        <v>-13.7</v>
+      </c>
       <c r="H30" t="n">
-        <v>28644700</v>
+        <v>5086800</v>
       </c>
     </row>
     <row r="31">
@@ -1443,14 +1473,20 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr"/>
-      <c r="F31" t="inlineStr"/>
-      <c r="G31" t="inlineStr"/>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>4140</v>
+      </c>
+      <c r="F31" t="n">
+        <v>-610</v>
+      </c>
+      <c r="G31" t="n">
+        <v>-12.84</v>
+      </c>
       <c r="H31" t="n">
-        <v>89943800</v>
+        <v>18795200</v>
       </c>
     </row>
     <row r="32">
@@ -1471,14 +1507,20 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr"/>
-      <c r="F32" t="inlineStr"/>
-      <c r="G32" t="inlineStr"/>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>494</v>
+      </c>
+      <c r="F32" t="n">
+        <v>-61</v>
+      </c>
+      <c r="G32" t="n">
+        <v>-10.99</v>
+      </c>
       <c r="H32" t="n">
-        <v>48885500</v>
+        <v>22162500</v>
       </c>
     </row>
     <row r="33">
@@ -1499,14 +1541,20 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr"/>
-      <c r="F33" t="inlineStr"/>
-      <c r="G33" t="inlineStr"/>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>585</v>
+      </c>
+      <c r="F33" t="n">
+        <v>-80</v>
+      </c>
+      <c r="G33" t="n">
+        <v>-12.03</v>
+      </c>
       <c r="H33" t="n">
-        <v>67193800</v>
+        <v>14884400</v>
       </c>
     </row>
     <row r="34">
@@ -1527,14 +1575,20 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr"/>
-      <c r="F34" t="inlineStr"/>
-      <c r="G34" t="inlineStr"/>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
+        <v>3610</v>
+      </c>
+      <c r="F34" t="n">
+        <v>-430</v>
+      </c>
+      <c r="G34" t="n">
+        <v>-10.64</v>
+      </c>
       <c r="H34" t="n">
-        <v>9716100</v>
+        <v>1723700</v>
       </c>
     </row>
     <row r="35">
@@ -1555,14 +1609,20 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr"/>
-      <c r="F35" t="inlineStr"/>
-      <c r="G35" t="inlineStr"/>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="E35" t="n">
+        <v>575</v>
+      </c>
+      <c r="F35" t="n">
+        <v>-90</v>
+      </c>
+      <c r="G35" t="n">
+        <v>-13.53</v>
+      </c>
       <c r="H35" t="n">
-        <v>163564500</v>
+        <v>21545100</v>
       </c>
     </row>
     <row r="36">
@@ -1583,14 +1643,20 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr"/>
-      <c r="F36" t="inlineStr"/>
-      <c r="G36" t="inlineStr"/>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>194</v>
+      </c>
+      <c r="F36" t="n">
+        <v>-16</v>
+      </c>
+      <c r="G36" t="n">
+        <v>-7.62</v>
+      </c>
       <c r="H36" t="n">
-        <v>45688900</v>
+        <v>4534500</v>
       </c>
     </row>
     <row r="37">
@@ -1611,14 +1677,20 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr"/>
-      <c r="F37" t="inlineStr"/>
-      <c r="G37" t="inlineStr"/>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
+        <v>14250</v>
+      </c>
+      <c r="F37" t="n">
+        <v>-1550</v>
+      </c>
+      <c r="G37" t="n">
+        <v>-9.81</v>
+      </c>
       <c r="H37" t="n">
-        <v>20278800</v>
+        <v>4277800</v>
       </c>
     </row>
   </sheetData>
@@ -1677,22 +1749,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>RI Genjot Koperasi Pertanian Bareng Negara Tetangga</t>
+          <t>Dolar AS Menguat ke Level Rp 17.948 Pagi Ini</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Mon, 12 Oct 2026 22:30:09 +0700</t>
+          <t>Tue, 13 Oct 2026 09:28:59 +0700</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/07/wakil-menteri-koperasi-wamenkop-farida-farichah-usai-menghadiri-pelantikan-dpd-knpi-lamongan-1791355884634_169.jpeg?w=360&amp;amp;q=90" /&gt; Indonesia menjalin kerja sama pengembangan koperasi pertanian bersama negara-negara ASEAN.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/07/20/dolar-as-tekuk-rupiah-ke-rp-17978-1784523338136_169.jpeg?w=360&amp;amp;q=90" /&gt; Nilai tukar dolar Amerika Serikat (AS) terpantau menguat terhadap rupiah.</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8704136/ri-genjot-koperasi-pertanian-bareng-negara-tetangga</t>
+          <t>https://finance.detik.com/bursa-dan-valas/d-8704398/dolar-as-menguat-ke-level-rp-17-948-pagi-ini</t>
         </is>
       </c>
     </row>
@@ -1704,22 +1776,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Konsumsi Pertalite Melonjak hingga Antre Panjang di SPBU, Pertamina Buka Suara</t>
+          <t>IHSG Melemah, Makin Jauh dari Level 6.000</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Mon, 12 Oct 2026 21:40:33 +0700</t>
+          <t>Tue, 13 Oct 2026 09:22:06 +0700</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/08/20/pemerintah-perketat-penyaluran-pertalite-mulai-2027-1787210254331_169.jpeg?w=360&amp;amp;q=90" /&gt; PT Pertamina Patra Niaga turun tangan memasok bahan bakar minyak (BBM) Kabupaten Bondowoso, Jawa Timur, seiring peningkatan kebutuhan m</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/05/22/ihsg-anjlok-ke-level-5000-sentuh-titik-terburuk-sejak-era-covid-19-1779437111616_169.jpeg?w=360&amp;amp;q=90" /&gt; Indeks Harga Saham Gabungan (IHSG) pagi ini dibuka jeblok ke zona merah.</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8704079/konsumsi-pertalite-melonjak-hingga-antre-panjang-di-spbu-pertamina-buka-suara</t>
+          <t>https://finance.detik.com/bursa-dan-valas/d-8704387/ihsg-melemah-makin-jauh-dari-level-6-000</t>
         </is>
       </c>
     </row>
@@ -1731,22 +1803,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>RI Bidik Peluang Investasi Lewat Penguatan Pasar Karbon di COP31</t>
+          <t>ASII Borong Saham AUTO, PGEO Rampungkan 5 Sumur Panas Bumi</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Mon, 12 Oct 2026 21:13:52 +0700</t>
+          <t>Tue, 13 Oct 2026 08:50:49 +0700</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/12/ri-bidik-peluang-investasi-lewat-penguatan-pasar-karbon-di-cop31-1791814371200.jpeg?w=360&amp;amp;q=90" /&gt; Pemerintah dorong pasar karbon untuk investasi hijau di Indonesia. Menjelang COP31, Zulkifli Hasan tekankan pentingnya pembiay</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/13/bursa-dan-valas-1791853978-1791853979228.jpeg?w=360&amp;amp;q=90" /&gt; IHSG turun 2,59%, ASII siapkan VTO AUTO Rp858 miliar, PGEO rampungkan 5 sumur panas bumi, dan VIVA konversi utang Rp1,72 triliun.</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8704059/ri-bidik-peluang-investasi-lewat-penguatan-pasar-karbon-di-cop31</t>
+          <t>https://finance.detik.com/bursa-dan-valas/d-8704335/asii-borong-saham-auto-pgeo-rampungkan-5-sumur-panas-bumi</t>
         </is>
       </c>
     </row>
@@ -1758,22 +1830,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Harga Minyak Mentah Indonesia Naik, Tembus US$ 112,81/ Barel</t>
+          <t>Bank Dunia &amp;amp; IMF Wanti-wanti Dampak AI ke Lapangan Kerja</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Mon, 12 Oct 2026 21:04:03 +0700</t>
+          <t>Tue, 13 Oct 2026 08:45:38 +0700</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/08/09/kilang-pertamina-1786240625862_169.jpeg?w=360&amp;amp;q=90" /&gt; Pemerintah menetapkan rata-rata Harga Minyak Mentah Indonesia atau Indonesian Crude Price (ICP) September 2026 sebesar US$112,81 per barel</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/05/19/pelamar-serbu-job-fair-jakarta-utara-berebut-asa-di-tengah-sulitnya-cari-kerja-1779173793394_169.jpeg?w=360&amp;amp;q=90" /&gt; Pemangku kepentingan dunia mulai memberikan peringatan keras tentang gangguan yang disebabkan oleh perkemban</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8704053/harga-minyak-mentah-indonesia-naik-tembus-us-112-81-barel</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8704324/bank-dunia-imf-wanti-wanti-dampak-ai-ke-lapangan-kerja</t>
         </is>
       </c>
     </row>
@@ -1785,22 +1857,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Harga Sapi Hidup Tinggi, RI Impor Kerbau Australia</t>
+          <t>Ojol Bakal Masuk Kategori Transportasi, Ini 3 Catatan Menhub</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Mon, 12 Oct 2026 20:48:31 +0700</t>
+          <t>Tue, 13 Oct 2026 08:30:40 +0700</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2021/05/20/indonesia-hentikan-sementara-impor-daging-kerbau-dari-india-terkait-pandemi-covid-19_169.jpeg?w=360&amp;amp;q=90" /&gt; PT Berdikari (Persero) resmi menerima kedatangan perdana kerbau hidup (Water Buffalo) asal Australia pada Minggu sor</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/25/menteri-perhubungan-menhub-dudy-purwagandhi-dokistimewa-1790318031224_169.jpeg?w=360&amp;amp;q=90" /&gt; Sejauh ini Kementerian Perhubungan sedang melakukan pembahasan revisi UU LLAJ dengan DPR.</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8704035/harga-sapi-hidup-tinggi-ri-impor-kerbau-australia</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8704123/ojol-bakal-masuk-kategori-transportasi-ini-3-catatan-menhub</t>
         </is>
       </c>
     </row>
@@ -1812,22 +1884,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>PAM Jaya Jajaki IPO, Direksi Sowan ke OJK</t>
+          <t>Menjaga Roda Ekonomi Pesisir Lewat Usaha Kerang Hijau di Jakarta Utara</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Mon, 12 Oct 2026 20:22:50 +0700</t>
+          <t>Tue, 13 Oct 2026 08:00:17 +0700</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/09/30/ilustrasi-distribusi-air-bersih-pam-jaya-1759220832502_169.jpeg?w=360&amp;amp;q=90" /&gt; PT Air Minum Jaya (Perseroda) atau PAM Jaya disebut mulai menjajaki penawaran umum perdana saham atau initial public offering (IPO).</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/12/menjaga-roda-ekonomi-pesisir-lewat-usaha-kerang-hijau-di-jakarta-utara-1791802797709_169.jpeg?w=360&amp;amp;q=90" /&gt; Pekerja merebus kerang hijau di Cilincing, Jakarta Utara, untuk memenuhi kebutuhan pasar. Usaha pengolahan ini menja</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/bursa-dan-valas/d-8704019/pam-jaya-jajaki-ipo-direksi-sowan-ke-ojk</t>
+          <t>https://finance.detik.com/foto-bisnis/d-8703856/menjaga-roda-ekonomi-pesisir-lewat-usaha-kerang-hijau-di-jakarta-utara</t>
         </is>
       </c>
     </row>
@@ -1839,22 +1911,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Kementan Tambah Anggaran Rp 600 Miliar untuk Peternakan-Bibit Ayam Jatim</t>
+          <t>Bandara Riyadh Ditutup, Penerbangan Langsung RI-Arab Saudi Masih Beroperasi</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Mon, 12 Oct 2026 20:07:26 +0700</t>
+          <t>Tue, 13 Oct 2026 07:54:50 +0700</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/12/kementan-tambah-anggaran-rp-600-miliar-untuk-peternakan-bibit-ayam-jatim-1791810366385_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Pertanian mengumumkan dukungan Rp3 triliun untuk Jawa Timur 2025-2026, termasuk Rp600 miliar untuk sektor </t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/12/potret-bandara-king-khalid-arab-saudi-diserang-houthi-yaman-1791779683573_169.jpeg?w=360&amp;amp;q=90" /&gt; Sejumlah penerbangan internasional mengalami pembatalan dampak insiden keamanan di Riyadh, Arab Saudi.</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8704007/kementan-tambah-anggaran-rp-600-miliar-untuk-peternakan-bibit-ayam-jatim</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8704285/bandara-riyadh-ditutup-penerbangan-langsung-ri-arab-saudi-masih-beroperasi</t>
         </is>
       </c>
     </row>
@@ -1866,22 +1938,22 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Begini Jawaban Bos Bursa Efek soal IHSG Anjlok 2,59%</t>
+          <t>Mentan Tunjuk Hidung Mafia Imbas Harga Ayam &amp;amp; Telur Naik</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Mon, 12 Oct 2026 20:03:39 +0700</t>
+          <t>Tue, 13 Oct 2026 07:30:17 +0700</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/07/13/direktur-utama-bei-jeffrey-hendrik-1783928734693_169.jpeg?w=360&amp;amp;q=90" /&gt; Indeks Harga Saham Gabungan (IHSG) anjlok 2,59% ke level 5.936,14 pada penutupan perdagangan Senin (12/10/2026).</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/07/28/wawancara-khusus-menteri-pertanian-ri-andi-amran-sulaiman-1753687994666_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Pertanian (Mentan) Andi Amran Sulaiman menuding mafia pangan berada di balik tingginya harga ayam dan telur di pasaran.</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/bursa-dan-valas/d-8704003/begini-jawaban-bos-bursa-efek-soal-ihsg-anjlok-2-59</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8704116/mentan-tunjuk-hidung-mafia-imbas-harga-ayam-telur-naik</t>
         </is>
       </c>
     </row>
@@ -1893,22 +1965,22 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Dua Jembatan di Kalteng Diperbaiki, Telan Rp 3,16 Miliar</t>
+          <t>Penjelasan Emiten Haji Isam soal Gadai Saham</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Mon, 12 Oct 2026 19:50:35 +0700</t>
+          <t>Tue, 13 Oct 2026 07:00:09 +0700</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/12/dua-jembatan-di-kalteng-diperbaiki-1791809412541_169.jpeg?w=360&amp;amp;q=90" /&gt; Kementerian Pekerjaan Umum (PU) memperbaiki Jembatan Pulau Telo dan Jembatan Pulau Petak yang membentang di sungai Kapuas, Kalimantan Tengah.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/05/18/ihsg-anjlok-ke-zona-merah-bursa-saham-melemah-tajam-1779098741437_169.jpeg?w=360&amp;amp;q=90" /&gt; Emiten milik konglomerat Andi Syamsuddin Arsyad alias Haji Isam, PT Pradiksi Gunatama Tbk (PGUN), mengaku tidak terlibat langsung denga</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8703981/dua-jembatan-di-kalteng-diperbaiki-telan-rp-3-16-miliar</t>
+          <t>https://finance.detik.com/bursa-dan-valas/d-8704113/penjelasan-emiten-haji-isam-soal-gadai-saham</t>
         </is>
       </c>
     </row>
@@ -1920,22 +1992,22 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>IHSG Jatuh 2,5%, Balik ke Level 5.900an</t>
+          <t>Ekspor Benih Lobster Ditutup Permanen</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Mon, 12 Oct 2026 18:13:44 +0700</t>
+          <t>Tue, 13 Oct 2026 06:30:14 +0700</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/06/04/ihsg-terpuruk-kekhawatiran-pasar-meningkat-1780558039793_169.jpeg?w=360&amp;amp;q=90" /&gt; IHSG hari ini jatuh 2,5% ke level 5.900an, dipicu aksi wait and see investor terhadap dinamika global dan konflik Houthi. Data inflasi AS jadi p</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/12/pemerintah-bentuk-satgas-p2bbl-berantas-penyelundupan-benih-bening-lobster-1791797202884_169.jpeg?w=360&amp;amp;q=90" /&gt; Pemerintah resmi menutup keran ekspor benih bening lobster (BBL) secara permanen</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/bursa-dan-valas/d-8703879/ihsg-jatuh-2-5-balik-ke-level-5-900an</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8704109/ekspor-benih-lobster-ditutup-permanen</t>
         </is>
       </c>
     </row>
@@ -1947,22 +2019,22 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>BULOG Cetak Rekor Pengadaan 4,13 Juta Ton Beras, Jatim Sumbang 23,7%</t>
+          <t>Revisi UU LLAJ Bakal Atur Ojol Penumpang hingga Pengiriman Barang</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Mon, 12 Oct 2026 16:58:19 +0700</t>
+          <t>Tue, 13 Oct 2026 06:00:09 +0700</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/12/bulog-cetak-rekor-pengadaan-413-juta-ton-beras-jatim-sumbang-237-1791798957038_169.jpeg?w=360&amp;amp;q=90" /&gt; Perum BULOG mencetak rekor pengadaan beras dengan serapan 4,13 juta ton, melampaui target nasional. Tasyakuran di Jatim me</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/12/revisi-uu-llaj-bakal-atur-ojol-penumpang-hingga-pengiriman-barang-1791821935791_169.jpeg?w=360&amp;amp;q=90" /&gt; Pemerintah menyiapkan aturan ojek online melalui revisi UU LLAJ untuk memperkuat kepastian hukum dan keselamatan. Regulas</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8703713/bulog-cetak-rekor-pengadaan-4-13-juta-ton-beras-jatim-sumbang-23-7</t>
+          <t>https://finance.detik.com/foto-bisnis/d-8704186/revisi-uu-llaj-bakal-atur-ojol-penumpang-hingga-pengiriman-barang</t>
         </is>
       </c>
     </row>
@@ -1974,22 +2046,22 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>PHE Akuisisi Saham Eni di 3 Blok Migas Strategis di Kalimantan Timur</t>
+          <t>Bahlil Sindir Bakrie di Depan Muka: Kawan Ini Tidak Paham-paham Juga</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Mon, 12 Oct 2026 16:55:28 +0700</t>
+          <t>Tue, 13 Oct 2026 05:55:05 +0700</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/23/pertamina-ep-1790145752344_169.jpeg?w=360&amp;amp;q=90" /&gt; PT Pertamina Hulu Energi akuisisi saham Eni di tiga blok migas strategis di Kalimantan Timur.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/07/16/menteri-esdm-bahlil-lahadalia-1784186781817_169.jpeg?w=360&amp;amp;q=90" /&gt; Indonesia menutup impor solar berkat program B50, namun beberapa perusahaan tambang masih ajukan izin. Bahlil dorong penggunaan etanol E50 untuk BBM.</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8703708/phe-akuisisi-saham-eni-di-3-blok-migas-strategis-di-kalimantan-timur</t>
+          <t>https://finance.detik.com/energi/d-8704070/bahlil-sindir-bakrie-di-depan-muka-kawan-ini-tidak-paham-paham-juga</t>
         </is>
       </c>
     </row>
@@ -2001,22 +2073,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Bayar Utang Pajak Kini Dahulukan Pokok Sebelum Denda, Ini Rinciannya</t>
+          <t>RI Genjot Koperasi Pertanian Bareng Negara Tetangga</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Mon, 12 Oct 2026 16:50:42 +0700</t>
+          <t>Mon, 12 Oct 2026 22:30:09 +0700</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2014/10/01/aba994a2-34ed-467e-b236-0838b109f70c_169.jpg?w=360&amp;amp;q=90" /&gt; Melalui ketentuan baru ini pembayaran akan diperhitungkan terlebih dahulu untuk melunasi pokok utang pajak.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/07/wakil-menteri-koperasi-wamenkop-farida-farichah-usai-menghadiri-pelantikan-dpd-knpi-lamongan-1791355884634_169.jpeg?w=360&amp;amp;q=90" /&gt; Indonesia menjalin kerja sama pengembangan koperasi pertanian bersama negara-negara ASEAN.</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8703697/bayar-utang-pajak-kini-dahulukan-pokok-sebelum-denda-ini-rinciannya</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8704136/ri-genjot-koperasi-pertanian-bareng-negara-tetangga</t>
         </is>
       </c>
     </row>
@@ -2028,22 +2100,22 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Di Depan Pengusaha Pribumi, Bahlil Klaim Keluarkan 4 Kebijakan Pro UMKM</t>
+          <t>Konsumsi Pertalite Melonjak hingga Antre Panjang di SPBU, Pertamina Buka Suara</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Mon, 12 Oct 2026 16:14:44 +0700</t>
+          <t>Mon, 12 Oct 2026 21:40:33 +0700</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/12/bahlil-lahadalia-1791784854378_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Bahlil mengumumkan 4 kebijakan pro-UMKM dalam pengelolaan sumber daya alam, termasuk legalisasi sumur minyak rakyat dan prioritas IUP untuk koperasi.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/08/20/pemerintah-perketat-penyaluran-pertalite-mulai-2027-1787210254331_169.jpeg?w=360&amp;amp;q=90" /&gt; PT Pertamina Patra Niaga turun tangan memasok bahan bakar minyak (BBM) Kabupaten Bondowoso, Jawa Timur, seiring peningkatan kebutuhan m</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8703599/di-depan-pengusaha-pribumi-bahlil-klaim-keluarkan-4-kebijakan-pro-umkm</t>
+          <t>https://finance.detik.com/energi/d-8704079/konsumsi-pertalite-melonjak-hingga-antre-panjang-di-spbu-pertamina-buka-suara</t>
         </is>
       </c>
     </row>
@@ -2055,22 +2127,22 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Budi Daya Lobster di RI Masih Belum Maksimal, Ini Alasannya</t>
+          <t>RI Bidik Peluang Investasi Lewat Penguatan Pasar Karbon di COP31</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Mon, 12 Oct 2026 15:59:32 +0700</t>
+          <t>Mon, 12 Oct 2026 21:13:52 +0700</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/12/satgas-pemberantasan-benur-lobster-ilegal-dibentuk-tak-cuma-tangkap-kurir-1791785768415_169.jpeg?w=360&amp;amp;q=90" /&gt; Salah satu penyebabnya, nelayan lokal tergiur menjual BBL ke negara tetangga karena perbedaan harga yang sangat t</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/12/ri-bidik-peluang-investasi-lewat-penguatan-pasar-karbon-di-cop31-1791814371200.jpeg?w=360&amp;amp;q=90" /&gt; Pemerintah dorong pasar karbon untuk investasi hijau di Indonesia. Menjelang COP31, Zulkifli Hasan tekankan pentingnya pembiay</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8703555/budi-daya-lobster-di-ri-masih-belum-maksimal-ini-alasannya</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8704059/ri-bidik-peluang-investasi-lewat-penguatan-pasar-karbon-di-cop31</t>
         </is>
       </c>
     </row>
@@ -2082,22 +2154,22 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Menag Nasaruddin Ajak Tobat Ekologis, Ingatkan Bahaya Eksploitasi Alam</t>
+          <t>Update Sebaran Titik Api Pemicu Kebakaran Hutan di Sumatra dan Kalimantan</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Tue, 13 Oct 2026 00:06:28 +0700</t>
+          <t>Tue, 13 Oct 2026 09:13:34 +0700</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Menag Nasaruddin Umar mengingatkan dampak kerusakan alam dan mengajak penerapan konsep ekoteologi dalam kehidupan sehari-hari.</t>
+          <t>Operasi modifikasi cuaca terus dimaksimalkan.</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8311654/menag-nasaruddin-ajak-tobat-ekologis-ingatkan-bahaya-eksploitasi-alam</t>
+          <t>https://www.liputan6.com/news/read/8311731/update-sebaran-titik-api-pemicu-kebakaran-hutan-di-sumatra-dan-kalimantan</t>
         </is>
       </c>
     </row>
@@ -2109,22 +2181,22 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Tabligh Akbar di Monas, Habib Nabiel Ajak Umat Islam Jaga Persatuan</t>
+          <t>Strategi Prabowo Atasi Kebakaran Hutan Tanjung Puting</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Mon, 12 Oct 2026 23:58:20 +0700</t>
+          <t>Tue, 13 Oct 2026 08:17:38 +0700</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Dalam Tabligh Akbar di Monas, Habib Nabiel menyoroti perpecahan, korupsi, hingga kebiasaan memfitnah.</t>
+          <t>Prabowo juga menekankan pentingnya memperkuat keberadaan polisi hutan untuk menjaga kawasan hutan.</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8311651/tabligh-akbar-di-monas-habib-nabiel-ajak-umat-islam-jaga-persatuan</t>
+          <t>https://www.liputan6.com/news/read/8311715/strategi-prabowo-atasi-kebakaran-hutan-tanjung-puting</t>
         </is>
       </c>
     </row>
@@ -2136,22 +2208,22 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Infografis: 5 Miliarder Asia dengan Penurunan Kekayaan Terbesar</t>
+          <t>Serangan Brutal KKB ke Warga Sipil di Yahukimo, 1 PNS Tewas</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Mon, 12 Oct 2026 22:52:51 +0700</t>
+          <t>Tue, 13 Oct 2026 06:49:33 +0700</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Miliarder  dari China, Indonesia, dan Korea Selatan mengalami penurunan kekayaan dengan nilai fantastis.</t>
+          <t>1 Lainnya dirawat intensif.</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8311630/infografis-5-miliarder-asia-dengan-penurunan-kekayaan-terbesar</t>
+          <t>https://www.liputan6.com/news/read/8311690/serangan-brutal-kkb-ke-warga-sipil-di-yahukimo-1-pns-tewas</t>
         </is>
       </c>
     </row>
@@ -2163,22 +2235,22 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Prabowo Kerahkan Seluruh Sumber Daya untuk Tangani Kabakaran Hutan</t>
+          <t>Saat Asap Mengepung Berbulan-bulan, Bencana Nasional Tak Ditetapkan</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Tue, 13 Oct 2026 00:12:43 +0700</t>
+          <t>Tue, 13 Oct 2026 07:18:11 +0700</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Sebanyak 60.177 personel gabungan dikerahkan untuk menangani kebakaran hutan dan lahan.</t>
+          <t>Bahkan beberapa negara tetangga juga ikut terpapar.</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8311629/prabowo-kerahkan-seluruh-sumber-daya-untuk-tangani-kabakaran-hutan</t>
+          <t>https://www.liputan6.com/news/read/8311631/saat-asap-mengepung-berbulan-bulan-bencana-nasional-tak-ditetapkan</t>
         </is>
       </c>
     </row>
@@ -2190,22 +2262,22 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Jemaah Umrah Indonesia Dikabarkan Aman, Kemenhaj Minta Tetap Waspada</t>
+          <t>Balita Tewas Terbakar di Kamar Tidur Saat Ditinggal Ayah Beli Token</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Mon, 12 Oct 2026 22:31:58 +0700</t>
+          <t>Tue, 13 Oct 2026 07:11:20 +0700</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Jemaah umrah Indonesiadi Arab Saudi diminta tetap waspada dan mengutamakan keselamatan.</t>
+          <t>Ditemukan obat nyamuk yang terpasang di kamar.</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8311624/jemaah-umrah-indonesia-dikabarkan-aman-kemenhaj-minta-tetap-waspada</t>
+          <t>https://www.liputan6.com/news/read/8311685/balita-tewas-terbakar-di-kamar-tidur-saat-ditinggal-ayah-beli-token</t>
         </is>
       </c>
     </row>
@@ -2217,22 +2289,22 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>BRAN Percepat Penataan Kelembagaan dan Regulasi Reforma Agraria</t>
+          <t>Petaka Telur Mentah Berujung Bayi Alena Meregang Nyawa</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Mon, 12 Oct 2026 21:50:39 +0700</t>
+          <t>Tue, 13 Oct 2026 05:00:45 +0700</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>BRAN menggandeng Kementerian Hukum dan berencana melibatkan akademisi untuk mengkaji regulasi yang menjadi landasan pelaksanaan reforma agraria.</t>
+          <t>Bayi Alena meninggal di usia 28 hari setelah sempat dirawat di rumah sakit. Begini keterangan pihak RSUD Dr. Soetomo.</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8311607/bran-percepat-penataan-kelembagaan-dan-regulasi-reforma-agraria</t>
+          <t>https://www.liputan6.com/news/read/8311665/petaka-telur-mentah-berujung-bayi-alena-meregang-nyawa</t>
         </is>
       </c>
     </row>
@@ -2244,22 +2316,22 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Mendagri Instruksikan Kepala Daerah Cegah Pembakaran Lahan</t>
+          <t>Menag Nasaruddin Ajak Tobat Ekologis, Ingatkan Bahaya Eksploitasi Alam</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Mon, 12 Oct 2026 20:27:46 +0700</t>
+          <t>Tue, 13 Oct 2026 00:06:28 +0700</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Di tengah kondisi darurat karhutla dan lahan yang mengering akibat kemarau, pemerintah meminta tidak ada pembakaran lahan baru.</t>
+          <t>Menag Nasaruddin Umar mengingatkan dampak kerusakan alam dan mengajak penerapan konsep ekoteologi dalam kehidupan sehari-hari.</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8311558/mendagri-instruksikan-kepala-daerah-cegah-pembakaran-lahan</t>
+          <t>https://www.liputan6.com/news/read/8311654/menag-nasaruddin-ajak-tobat-ekologis-ingatkan-bahaya-eksploitasi-alam</t>
         </is>
       </c>
     </row>
@@ -2271,22 +2343,22 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Instruksi Prabowo Terkait Kebakaran Hutan di 6 Provinsi</t>
+          <t>Tabligh Akbar di Monas, Habib Nabiel Ajak Umat Islam Jaga Persatuan</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Mon, 12 Oct 2026 20:17:52 +0700</t>
+          <t>Mon, 12 Oct 2026 23:58:20 +0700</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Prabowo ingin pencegahan dilakukan sebelum api menyala.</t>
+          <t>Dalam Tabligh Akbar di Monas, Habib Nabiel menyoroti perpecahan, korupsi, hingga kebiasaan memfitnah.</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8311555/instruksi-prabowo-terkait-kebakaran-hutan-di-6-provinsi</t>
+          <t>https://www.liputan6.com/news/read/8311651/tabligh-akbar-di-monas-habib-nabiel-ajak-umat-islam-jaga-persatuan</t>
         </is>
       </c>
     </row>
@@ -2298,22 +2370,22 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Prabowo Tunjuk Satyawan Pudyatmoko Jadi Kepala Badan Pengelolaan Gambut dan Mangrove</t>
+          <t>Infografis: 5 Miliarder Asia dengan Penurunan Kekayaan Terbesar</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Mon, 12 Oct 2026 20:07:29 +0700</t>
+          <t>Mon, 12 Oct 2026 22:52:51 +0700</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Satyawan merupakan ahli di bidang pengelolaan gambut dan mangrove sehingga cocok memimpin badan tersebut.</t>
+          <t>Miliarder  dari China, Indonesia, dan Korea Selatan mengalami penurunan kekayaan dengan nilai fantastis.</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8311541/prabowo-tunjuk-satyawan-pudyatmoko-jadi-kepala-badan-pengelolaan-gambut-dan-mangrove</t>
+          <t>https://www.liputan6.com/news/read/8311630/infografis-5-miliarder-asia-dengan-penurunan-kekayaan-terbesar</t>
         </is>
       </c>
     </row>
@@ -2325,22 +2397,22 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Separuh Anggaran Iklan BJB Jadi Dana Non-Budgeter, Siapa Penerimanya?</t>
+          <t>Prabowo Kerahkan Seluruh Sumber Daya untuk Tangani Kabakaran Hutan</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Mon, 12 Oct 2026 19:33:50 +0700</t>
+          <t>Tue, 13 Oct 2026 00:12:43 +0700</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>KPK mendalami dugaan penyisihan Rp 200 miliar dari pengadaan iklan Bank BJB. Penyidik menelusuri aliran dan peruntukan dana tersebut.</t>
+          <t>Sebanyak 60.177 personel gabungan dikerahkan untuk menangani kebakaran hutan dan lahan.</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8311524/separuh-anggaran-iklan-bjb-jadi-dana-non-budgeter-siapa-penerimanya</t>
+          <t>https://www.liputan6.com/news/read/8311629/prabowo-kerahkan-seluruh-sumber-daya-untuk-tangani-kabakaran-hutan</t>
         </is>
       </c>
     </row>
@@ -2352,22 +2424,22 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Kebakaran Hutan Belum Berstatus Bencana Nasional, Dudung Ungkap Alasannya</t>
+          <t>Jemaah Umrah Indonesia Dikabarkan Aman, Kemenhaj Minta Tetap Waspada</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Mon, 12 Oct 2026 19:30:59 +0700</t>
+          <t>Mon, 12 Oct 2026 22:31:58 +0700</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Menko Polkam Dudung Abdurachman mengatakan pemerintah masih mampu menangani karhutla. Saat ini, penanganan difokuskan pada enam provinsi.</t>
+          <t>Jemaah umrah Indonesiadi Arab Saudi diminta tetap waspada dan mengutamakan keselamatan.</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8311537/kebakaran-hutan-belum-berstatus-bencana-nasional-dudung-ungkap-alasannya</t>
+          <t>https://www.liputan6.com/news/read/8311624/jemaah-umrah-indonesia-dikabarkan-aman-kemenhaj-minta-tetap-waspada</t>
         </is>
       </c>
     </row>
@@ -2379,22 +2451,22 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Satpol PP dan Pekerja Proyek Bentrok, Begini Reaksi Pramono</t>
+          <t>BRAN Percepat Penataan Kelembagaan dan Regulasi Reforma Agraria</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Mon, 12 Oct 2026 19:18:59 +0700</t>
+          <t>Mon, 12 Oct 2026 21:50:39 +0700</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Bentrokan antara petugas Satpol PP dan pekerja proyek di Bulungan viral di media sosial. Pramono Anung meminta hukum tetap ditegakkan.</t>
+          <t>BRAN menggandeng Kementerian Hukum dan berencana melibatkan akademisi untuk mengkaji regulasi yang menjadi landasan pelaksanaan reforma agraria.</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8311529/satpol-pp-dan-pekerja-proyek-bentrok-begini-reaksi-pramono</t>
+          <t>https://www.liputan6.com/news/read/8311607/bran-percepat-penataan-kelembagaan-dan-regulasi-reforma-agraria</t>
         </is>
       </c>
     </row>
@@ -2406,22 +2478,22 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Kapolri Lantik Kakorlantas dan Tiga Kapolda Baru</t>
+          <t>Mendagri Instruksikan Kepala Daerah Cegah Pembakaran Lahan</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Mon, 12 Oct 2026 20:07:12 +0700</t>
+          <t>Mon, 12 Oct 2026 20:27:46 +0700</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Kapolri memimpin pergantian Kakorlantas dan tiga Kapolda. Berikut daftar pejabat yang mengisi posisi baru.</t>
+          <t>Di tengah kondisi darurat karhutla dan lahan yang mengering akibat kemarau, pemerintah meminta tidak ada pembakaran lahan baru.</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8311495/kapolri-lantik-kakorlantas-dan-tiga-kapolda-baru</t>
+          <t>https://www.liputan6.com/news/read/8311558/mendagri-instruksikan-kepala-daerah-cegah-pembakaran-lahan</t>
         </is>
       </c>
     </row>
@@ -2433,22 +2505,22 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Data Center AI Butuh Banyak Air, Menko AHY Beri Peringatan</t>
+          <t>Instruksi Prabowo Terkait Kebakaran Hutan di 6 Provinsi</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Mon, 12 Oct 2026 18:31:38 +0700</t>
+          <t>Mon, 12 Oct 2026 20:17:52 +0700</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Kebutuhan air untuk pusat data AI menjadi sorotan AHY. Dia mengingatkan pentingnya menjaga pasokan air bersih bagi masyarakat.</t>
+          <t>Prabowo ingin pencegahan dilakukan sebelum api menyala.</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8311477/data-center-ai-butuh-banyak-air-menko-ahy-beri-peringatan</t>
+          <t>https://www.liputan6.com/news/read/8311555/instruksi-prabowo-terkait-kebakaran-hutan-di-6-provinsi</t>
         </is>
       </c>
     </row>
@@ -2460,22 +2532,22 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>KPK Geledah 3 Lokasi Terkait Kasus Bupati Pemalang, Ini Hasilnya</t>
+          <t>Prabowo Tunjuk Satyawan Pudyatmoko Jadi Kepala Badan Pengelolaan Gambut dan Mangrove</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Mon, 12 Oct 2026 18:29:51 +0700</t>
+          <t>Mon, 12 Oct 2026 20:07:29 +0700</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>KPK menyita dokumen dan barang bukti elektronik dari penggeledahan tiga lokasi terkait kasus Bupati Pemalang nonaktif.</t>
+          <t>Satyawan merupakan ahli di bidang pengelolaan gambut dan mangrove sehingga cocok memimpin badan tersebut.</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8311494/kpk-geledah-3-lokasi-terkait-kasus-bupati-pemalang-ini-hasilnya</t>
+          <t>https://www.liputan6.com/news/read/8311541/prabowo-tunjuk-satyawan-pudyatmoko-jadi-kepala-badan-pengelolaan-gambut-dan-mangrove</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data pasar & berita - 2026-10-13 15:47 UTC
</commit_message>
<xml_diff>
--- a/data/market_news_latest.xlsx
+++ b/data/market_news_latest.xlsx
@@ -491,13 +491,13 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>5860.0571</v>
+        <v>5925.9761</v>
       </c>
       <c r="F2" t="n">
-        <v>-76.0898</v>
+        <v>-10.1709</v>
       </c>
       <c r="G2" t="n">
-        <v>-1.28</v>
+        <v>-0.17</v>
       </c>
       <c r="H2" t="n">
         <v>0</v>
@@ -521,20 +521,20 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>7807.2402</v>
+        <v>7787.8799</v>
       </c>
       <c r="F3" t="n">
-        <v>-4.2998</v>
+        <v>-19.3604</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.06</v>
+        <v>-0.25</v>
       </c>
       <c r="H3" t="n">
-        <v>2291949000</v>
+        <v>869506500</v>
       </c>
     </row>
     <row r="4">
@@ -555,20 +555,20 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>51850.5508</v>
+        <v>51678.6289</v>
       </c>
       <c r="F4" t="n">
-        <v>195.6016</v>
+        <v>-171.9219</v>
       </c>
       <c r="G4" t="n">
-        <v>0.38</v>
+        <v>-0.33</v>
       </c>
       <c r="H4" t="n">
-        <v>307464899</v>
+        <v>153969361</v>
       </c>
     </row>
     <row r="5">
@@ -589,20 +589,20 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>27245.9023</v>
+        <v>27149.7734</v>
       </c>
       <c r="F5" t="n">
-        <v>-120.2676</v>
+        <v>-96.127</v>
       </c>
       <c r="G5" t="n">
-        <v>-0.44</v>
+        <v>-0.35</v>
       </c>
       <c r="H5" t="n">
-        <v>5794275000</v>
+        <v>2719719000</v>
       </c>
     </row>
     <row r="6">
@@ -623,20 +623,20 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>67287.9219</v>
+        <v>69030.9219</v>
       </c>
       <c r="F6" t="n">
-        <v>-1743</v>
+        <v>-11.1875</v>
       </c>
       <c r="G6" t="n">
-        <v>-2.52</v>
+        <v>-0.02</v>
       </c>
       <c r="H6" t="n">
-        <v>0</v>
+        <v>162000000</v>
       </c>
     </row>
     <row r="7">
@@ -661,13 +661,13 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>24000.7598</v>
+        <v>24345.2207</v>
       </c>
       <c r="F7" t="n">
-        <v>-270.4395</v>
+        <v>74.0215</v>
       </c>
       <c r="G7" t="n">
-        <v>-1.11</v>
+        <v>0.3</v>
       </c>
       <c r="H7" t="n">
         <v>0</v>
@@ -695,16 +695,16 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>3756.5547</v>
+        <v>3800.8645</v>
       </c>
       <c r="F8" t="n">
-        <v>-40.6873</v>
+        <v>3.6226</v>
       </c>
       <c r="G8" t="n">
-        <v>-1.07</v>
+        <v>0.1</v>
       </c>
       <c r="H8" t="n">
-        <v>893787720</v>
+        <v>1085950644</v>
       </c>
     </row>
     <row r="9">
@@ -725,20 +725,20 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>10656.2998</v>
+        <v>10649.1201</v>
       </c>
       <c r="F9" t="n">
-        <v>104.2002</v>
+        <v>-7.1797</v>
       </c>
       <c r="G9" t="n">
-        <v>0.99</v>
+        <v>-0.07000000000000001</v>
       </c>
       <c r="H9" t="n">
-        <v>575809000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -759,20 +759,20 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>25277.6797</v>
+        <v>25251.1504</v>
       </c>
       <c r="F10" t="n">
-        <v>190.4102</v>
+        <v>-26.5293</v>
       </c>
       <c r="G10" t="n">
-        <v>0.76</v>
+        <v>-0.1</v>
       </c>
       <c r="H10" t="n">
-        <v>39349200</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -797,13 +797,13 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>5415.8901</v>
+        <v>5430.5</v>
       </c>
       <c r="F11" t="n">
-        <v>0.4102</v>
+        <v>15.02</v>
       </c>
       <c r="G11" t="n">
-        <v>0.01</v>
+        <v>0.28</v>
       </c>
       <c r="H11" t="n">
         <v>0</v>
@@ -831,13 +831,13 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>17894</v>
+        <v>17925</v>
       </c>
       <c r="F12" t="n">
-        <v>86.5</v>
+        <v>117.5</v>
       </c>
       <c r="G12" t="n">
-        <v>0.49</v>
+        <v>0.66</v>
       </c>
       <c r="H12" t="n">
         <v>0</v>
@@ -861,17 +861,17 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>102.417</v>
+        <v>102.283</v>
       </c>
       <c r="F13" t="n">
-        <v>0.207</v>
+        <v>-0.297</v>
       </c>
       <c r="G13" t="n">
-        <v>0.2</v>
+        <v>-0.29</v>
       </c>
       <c r="H13" t="n">
         <v>0</v>
@@ -899,13 +899,13 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>158.248</v>
+        <v>158.397</v>
       </c>
       <c r="F14" t="n">
-        <v>0.185</v>
+        <v>0.334</v>
       </c>
       <c r="G14" t="n">
-        <v>0.12</v>
+        <v>0.21</v>
       </c>
       <c r="H14" t="n">
         <v>0</v>
@@ -929,17 +929,17 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>0.524</v>
+        <v>0.5217000000000001</v>
       </c>
       <c r="F15" t="n">
-        <v>-0.0004</v>
+        <v>-0.0023</v>
       </c>
       <c r="G15" t="n">
-        <v>-0.08</v>
+        <v>-0.44</v>
       </c>
       <c r="H15" t="n">
         <v>0</v>
@@ -963,17 +963,17 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>0.5598</v>
+        <v>0.5565</v>
       </c>
       <c r="F16" t="n">
-        <v>-0.0002</v>
+        <v>-0.0033</v>
       </c>
       <c r="G16" t="n">
-        <v>-0.04</v>
+        <v>-0.59</v>
       </c>
       <c r="H16" t="n">
         <v>0</v>
@@ -997,17 +997,17 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>0.405</v>
+        <v>0.4063</v>
       </c>
       <c r="F17" t="n">
-        <v>-0.0007</v>
+        <v>0.0013</v>
       </c>
       <c r="G17" t="n">
-        <v>-0.17</v>
+        <v>0.32</v>
       </c>
       <c r="H17" t="n">
         <v>0</v>
@@ -1031,20 +1031,20 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>78.05</v>
+        <v>78.265</v>
       </c>
       <c r="F18" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.215</v>
       </c>
       <c r="G18" t="n">
-        <v>0.09</v>
+        <v>0.28</v>
       </c>
       <c r="H18" t="n">
-        <v>15346700</v>
+        <v>12544097</v>
       </c>
     </row>
     <row r="19">
@@ -1065,20 +1065,20 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>77.29000000000001</v>
+        <v>77.0001</v>
       </c>
       <c r="F19" t="n">
-        <v>0.06</v>
+        <v>-0.2899</v>
       </c>
       <c r="G19" t="n">
-        <v>0.08</v>
+        <v>-0.38</v>
       </c>
       <c r="H19" t="n">
-        <v>21847900</v>
+        <v>27766515</v>
       </c>
     </row>
     <row r="20">
@@ -1099,20 +1099,20 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>4191.2998</v>
+        <v>4184.6001</v>
       </c>
       <c r="F20" t="n">
-        <v>-25</v>
+        <v>-6</v>
       </c>
       <c r="G20" t="n">
-        <v>-0.59</v>
+        <v>-0.14</v>
       </c>
       <c r="H20" t="n">
-        <v>18547</v>
+        <v>90400</v>
       </c>
     </row>
     <row r="21">
@@ -1133,20 +1133,20 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>92.59999999999999</v>
+        <v>94.2</v>
       </c>
       <c r="F21" t="n">
-        <v>0.75</v>
+        <v>0.46</v>
       </c>
       <c r="G21" t="n">
-        <v>0.82</v>
+        <v>0.49</v>
       </c>
       <c r="H21" t="n">
-        <v>9667</v>
+        <v>135225</v>
       </c>
     </row>
     <row r="22">
@@ -1167,20 +1167,20 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="E22" t="n">
-        <v>105.46</v>
+        <v>106.07</v>
       </c>
       <c r="F22" t="n">
-        <v>0.74</v>
+        <v>-0.58</v>
       </c>
       <c r="G22" t="n">
-        <v>0.71</v>
+        <v>-0.54</v>
       </c>
       <c r="H22" t="n">
-        <v>1163</v>
+        <v>22916</v>
       </c>
     </row>
     <row r="23">
@@ -1201,20 +1201,20 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="E23" t="n">
-        <v>6.7085</v>
+        <v>6.733</v>
       </c>
       <c r="F23" t="n">
-        <v>0.066</v>
+        <v>0.0345</v>
       </c>
       <c r="G23" t="n">
-        <v>0.99</v>
+        <v>0.52</v>
       </c>
       <c r="H23" t="n">
-        <v>2754</v>
+        <v>21438</v>
       </c>
     </row>
     <row r="24">
@@ -1235,20 +1235,20 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="E24" t="n">
-        <v>66.15000000000001</v>
+        <v>65.45</v>
       </c>
       <c r="F24" t="n">
-        <v>-0.65</v>
+        <v>-0.7</v>
       </c>
       <c r="G24" t="n">
-        <v>-0.97</v>
+        <v>-1.06</v>
       </c>
       <c r="H24" t="n">
-        <v>10344700</v>
+        <v>7502005</v>
       </c>
     </row>
     <row r="25">
@@ -1269,17 +1269,17 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="E25" t="n">
-        <v>15.21</v>
+        <v>15.41</v>
       </c>
       <c r="F25" t="n">
-        <v>0.37</v>
+        <v>0.2</v>
       </c>
       <c r="G25" t="n">
-        <v>2.49</v>
+        <v>1.31</v>
       </c>
       <c r="H25" t="n">
         <v>0</v>
@@ -1307,16 +1307,16 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>82773.00780000001</v>
+        <v>83174.7188</v>
       </c>
       <c r="F26" t="n">
-        <v>-906.4609</v>
+        <v>1412.1562</v>
       </c>
       <c r="G26" t="n">
-        <v>-1.08</v>
+        <v>1.73</v>
       </c>
       <c r="H26" t="n">
-        <v>29273978880</v>
+        <v>31508934656</v>
       </c>
     </row>
     <row r="27">
@@ -1341,16 +1341,16 @@
         </is>
       </c>
       <c r="E27" t="n">
-        <v>1325</v>
+        <v>1310</v>
       </c>
       <c r="F27" t="n">
-        <v>-80</v>
+        <v>-95</v>
       </c>
       <c r="G27" t="n">
-        <v>-5.69</v>
+        <v>-6.76</v>
       </c>
       <c r="H27" t="n">
-        <v>21639800</v>
+        <v>80411200</v>
       </c>
     </row>
     <row r="28">
@@ -1375,16 +1375,16 @@
         </is>
       </c>
       <c r="E28" t="n">
-        <v>1470</v>
+        <v>1520</v>
       </c>
       <c r="F28" t="n">
-        <v>-205</v>
+        <v>-155</v>
       </c>
       <c r="G28" t="n">
-        <v>-12.24</v>
+        <v>-9.25</v>
       </c>
       <c r="H28" t="n">
-        <v>55172500</v>
+        <v>127296000</v>
       </c>
     </row>
     <row r="29">
@@ -1409,16 +1409,16 @@
         </is>
       </c>
       <c r="E29" t="n">
-        <v>670</v>
+        <v>665</v>
       </c>
       <c r="F29" t="n">
-        <v>-100</v>
+        <v>-105</v>
       </c>
       <c r="G29" t="n">
-        <v>-12.99</v>
+        <v>-13.64</v>
       </c>
       <c r="H29" t="n">
-        <v>209845100</v>
+        <v>434856000</v>
       </c>
     </row>
     <row r="30">
@@ -1443,16 +1443,16 @@
         </is>
       </c>
       <c r="E30" t="n">
-        <v>2330</v>
+        <v>2430</v>
       </c>
       <c r="F30" t="n">
-        <v>-370</v>
+        <v>-270</v>
       </c>
       <c r="G30" t="n">
-        <v>-13.7</v>
+        <v>-10</v>
       </c>
       <c r="H30" t="n">
-        <v>5086800</v>
+        <v>13220900</v>
       </c>
     </row>
     <row r="31">
@@ -1477,16 +1477,16 @@
         </is>
       </c>
       <c r="E31" t="n">
-        <v>4140</v>
+        <v>4180</v>
       </c>
       <c r="F31" t="n">
-        <v>-610</v>
+        <v>-570</v>
       </c>
       <c r="G31" t="n">
-        <v>-12.84</v>
+        <v>-12</v>
       </c>
       <c r="H31" t="n">
-        <v>18795200</v>
+        <v>47740700</v>
       </c>
     </row>
     <row r="32">
@@ -1511,16 +1511,16 @@
         </is>
       </c>
       <c r="E32" t="n">
-        <v>494</v>
+        <v>500</v>
       </c>
       <c r="F32" t="n">
-        <v>-61</v>
+        <v>-55</v>
       </c>
       <c r="G32" t="n">
-        <v>-10.99</v>
+        <v>-9.91</v>
       </c>
       <c r="H32" t="n">
-        <v>22162500</v>
+        <v>51400500</v>
       </c>
     </row>
     <row r="33">
@@ -1545,16 +1545,16 @@
         </is>
       </c>
       <c r="E33" t="n">
-        <v>585</v>
+        <v>605</v>
       </c>
       <c r="F33" t="n">
-        <v>-80</v>
+        <v>-60</v>
       </c>
       <c r="G33" t="n">
-        <v>-12.03</v>
+        <v>-9.02</v>
       </c>
       <c r="H33" t="n">
-        <v>14884400</v>
+        <v>50719300</v>
       </c>
     </row>
     <row r="34">
@@ -1579,16 +1579,16 @@
         </is>
       </c>
       <c r="E34" t="n">
-        <v>3610</v>
+        <v>3710</v>
       </c>
       <c r="F34" t="n">
-        <v>-430</v>
+        <v>-330</v>
       </c>
       <c r="G34" t="n">
-        <v>-10.64</v>
+        <v>-8.17</v>
       </c>
       <c r="H34" t="n">
-        <v>1723700</v>
+        <v>3833300</v>
       </c>
     </row>
     <row r="35">
@@ -1613,16 +1613,16 @@
         </is>
       </c>
       <c r="E35" t="n">
-        <v>575</v>
+        <v>590</v>
       </c>
       <c r="F35" t="n">
-        <v>-90</v>
+        <v>-75</v>
       </c>
       <c r="G35" t="n">
-        <v>-13.53</v>
+        <v>-11.28</v>
       </c>
       <c r="H35" t="n">
-        <v>21545100</v>
+        <v>67977500</v>
       </c>
     </row>
     <row r="36">
@@ -1647,16 +1647,16 @@
         </is>
       </c>
       <c r="E36" t="n">
-        <v>194</v>
+        <v>199</v>
       </c>
       <c r="F36" t="n">
-        <v>-16</v>
+        <v>-11</v>
       </c>
       <c r="G36" t="n">
-        <v>-7.62</v>
+        <v>-5.24</v>
       </c>
       <c r="H36" t="n">
-        <v>4534500</v>
+        <v>18782500</v>
       </c>
     </row>
     <row r="37">
@@ -1690,7 +1690,7 @@
         <v>-9.81</v>
       </c>
       <c r="H37" t="n">
-        <v>4277800</v>
+        <v>11233300</v>
       </c>
     </row>
   </sheetData>
@@ -1749,22 +1749,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Dolar AS Menguat ke Level Rp 17.948 Pagi Ini</t>
+          <t>BTPN Syariah (BTPS) Bakal Buyback Saham hingga Rp 1 Triliun</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Tue, 13 Oct 2026 09:28:59 +0700</t>
+          <t>Tue, 13 Oct 2026 22:35:02 +0700</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/07/20/dolar-as-tekuk-rupiah-ke-rp-17978-1784523338136_169.jpeg?w=360&amp;amp;q=90" /&gt; Nilai tukar dolar Amerika Serikat (AS) terpantau menguat terhadap rupiah.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/13/rupslb-btpn-syariah-1791905594130_169.jpeg?w=360&amp;amp;q=90" /&gt; PT Bank BTPN Syariah Tbk mengajukan rencana aksi korporasi pembelian kembali saham (buyback) dengan nilai maksimal hingga Rp1 triliun</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/bursa-dan-valas/d-8704398/dolar-as-menguat-ke-level-rp-17-948-pagi-ini</t>
+          <t>https://finance.detik.com/bursa-dan-valas/d-8705745/btpn-syariah-btps-bakal-buyback-saham-hingga-rp-1-triliun</t>
         </is>
       </c>
     </row>
@@ -1776,22 +1776,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>IHSG Melemah, Makin Jauh dari Level 6.000</t>
+          <t>Zero ODOL Bisa Gagal Jika Cuma Tertibkan Truk, Ini Saran buat Pemerintah</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Tue, 13 Oct 2026 09:22:06 +0700</t>
+          <t>Tue, 13 Oct 2026 22:30:00 +0700</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/05/22/ihsg-anjlok-ke-level-5000-sentuh-titik-terburuk-sejak-era-covid-19-1779437111616_169.jpeg?w=360&amp;amp;q=90" /&gt; Indeks Harga Saham Gabungan (IHSG) pagi ini dibuka jeblok ke zona merah.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/06/19/kepadatan-lalu-lintas-di-jalan-raya-wonokromo-surabaya-imbas-demo-sopir-truk-toal-aturan-odol-1750328242861_169.jpeg?w=360&amp;amp;q=90" /&gt; Pemerintah akan menerapkan Zero Over Dimension Overloading (ODOL) pada 2027.</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/bursa-dan-valas/d-8704387/ihsg-melemah-makin-jauh-dari-level-6-000</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8705733/zero-odol-bisa-gagal-jika-cuma-tertibkan-truk-ini-saran-buat-pemerintah</t>
         </is>
       </c>
     </row>
@@ -1803,22 +1803,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>ASII Borong Saham AUTO, PGEO Rampungkan 5 Sumur Panas Bumi</t>
+          <t>Panen Melimpah, Harga Garam Petani Takalar Turun Tajam</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Tue, 13 Oct 2026 08:50:49 +0700</t>
+          <t>Tue, 13 Oct 2026 22:00:16 +0700</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/13/bursa-dan-valas-1791853978-1791853979228.jpeg?w=360&amp;amp;q=90" /&gt; IHSG turun 2,59%, ASII siapkan VTO AUTO Rp858 miliar, PGEO rampungkan 5 sumur panas bumi, dan VIVA konversi utang Rp1,72 triliun.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/13/harga-garam-turun-di-kabupaten-takalar-1791872493195_169.jpeg?w=360&amp;amp;q=90" /&gt; Harga garam di Takalar anjlok dari Rp150 ribu menjadi Rp45 ribu per karung akibat panen melimpah saat kemarau. Petani berharap bantuan gudang.</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/bursa-dan-valas/d-8704335/asii-borong-saham-auto-pgeo-rampungkan-5-sumur-panas-bumi</t>
+          <t>https://finance.detik.com/foto-bisnis/d-8704804/panen-melimpah-harga-garam-petani-takalar-turun-tajam</t>
         </is>
       </c>
     </row>
@@ -1830,22 +1830,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Bank Dunia &amp;amp; IMF Wanti-wanti Dampak AI ke Lapangan Kerja</t>
+          <t>Mau Jago Hitung Pajak, Tapi Bingung Mulai dari Mana? Coba Kursus di Sini!</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Tue, 13 Oct 2026 08:45:38 +0700</t>
+          <t>Tue, 13 Oct 2026 21:40:18 +0700</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/05/19/pelamar-serbu-job-fair-jakarta-utara-berebut-asa-di-tengah-sulitnya-cari-kerja-1779173793394_169.jpeg?w=360&amp;amp;q=90" /&gt; Pemangku kepentingan dunia mulai memberikan peringatan keras tentang gangguan yang disebabkan oleh perkemban</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/07/28/smart-class-brevet-pajak-a-b-1785248368520_169.png?w=360&amp;amp;q=90" /&gt; i fokus Pelatihan Brevet Pajak AB + Sertifikasi CTT dan CCP dari Piranha Smart Center (PSC) bersama Education Visionary Lab (EVL).</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8704324/bank-dunia-imf-wanti-wanti-dampak-ai-ke-lapangan-kerja</t>
+          <t>https://finance.detik.com/energi/d-8705693/mau-jago-hitung-pajak-tapi-bingung-mulai-dari-mana-coba-kursus-di-sini</t>
         </is>
       </c>
     </row>
@@ -1857,22 +1857,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Ojol Bakal Masuk Kategori Transportasi, Ini 3 Catatan Menhub</t>
+          <t>Beli Token &amp;amp; Bayar Tagihan Listrik Bisa di Kopdes Merah Putih</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Tue, 13 Oct 2026 08:30:40 +0700</t>
+          <t>Tue, 13 Oct 2026 21:23:38 +0700</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/25/menteri-perhubungan-menhub-dudy-purwagandhi-dokistimewa-1790318031224_169.jpeg?w=360&amp;amp;q=90" /&gt; Sejauh ini Kementerian Perhubungan sedang melakukan pembahasan revisi UU LLAJ dengan DPR.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/21/kopdes-merah-putih-bersiap-operasional-23-ribu-bangunan-telah-rampung-1789986171319_169.jpeg?w=360&amp;amp;q=90" /&gt; PLN mendukung program Koperasi Desa/Kelurahan Merah Putih atau Kopdes Merah Putih melalui kemitraan layanan pembayara</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8704123/ojol-bakal-masuk-kategori-transportasi-ini-3-catatan-menhub</t>
+          <t>https://finance.detik.com/energi/d-8705683/beli-token-bayar-tagihan-listrik-bisa-di-kopdes-merah-putih</t>
         </is>
       </c>
     </row>
@@ -1884,22 +1884,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Menjaga Roda Ekonomi Pesisir Lewat Usaha Kerang Hijau di Jakarta Utara</t>
+          <t>1.813 Penerbangan Terdampak Karhutla, Mayoritas Gagal Terbang</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Tue, 13 Oct 2026 08:00:17 +0700</t>
+          <t>Tue, 13 Oct 2026 20:46:22 +0700</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/12/menjaga-roda-ekonomi-pesisir-lewat-usaha-kerang-hijau-di-jakarta-utara-1791802797709_169.jpeg?w=360&amp;amp;q=90" /&gt; Pekerja merebus kerang hijau di Cilincing, Jakarta Utara, untuk memenuhi kebutuhan pasar. Usaha pengolahan ini menja</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/17/kabut-asap-karhutla-ganggu-penerbangan-di-bandara-palembang-1789622375071_169.jpeg?w=360&amp;amp;q=90" /&gt; Kementerian Perhubungan (Kemenhub) mencatat total 1.813 penerbangan terdampak kebakaran hutan dan lahan (karhutla) sejak 11 Agu</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/foto-bisnis/d-8703856/menjaga-roda-ekonomi-pesisir-lewat-usaha-kerang-hijau-di-jakarta-utara</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8705647/1-813-penerbangan-terdampak-karhutla-mayoritas-gagal-terbang</t>
         </is>
       </c>
     </row>
@@ -1911,22 +1911,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Bandara Riyadh Ditutup, Penerbangan Langsung RI-Arab Saudi Masih Beroperasi</t>
+          <t>Menteri LH Ingatkan Pengusaha, Biaya Urus Lingkungan Hidup Bukan Beban!</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Tue, 13 Oct 2026 07:54:50 +0700</t>
+          <t>Tue, 13 Oct 2026 20:11:54 +0700</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/12/potret-bandara-king-khalid-arab-saudi-diserang-houthi-yaman-1791779683573_169.jpeg?w=360&amp;amp;q=90" /&gt; Sejumlah penerbangan internasional mengalami pembatalan dampak insiden keamanan di Riyadh, Arab Saudi.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/29/menteri-lh-mohammad-jumhur-hidayat-saat-kunjungi-objek-wisata-di-cisarua-1790687703176_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Lingkungan Hidup Mohammad Jumhur Hidayat menegaskan biaya yang dikeluarkan perusahaan dalam pengelolaan li</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8704285/bandara-riyadh-ditutup-penerbangan-langsung-ri-arab-saudi-masih-beroperasi</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8705607/menteri-lh-ingatkan-pengusaha-biaya-urus-lingkungan-hidup-bukan-beban</t>
         </is>
       </c>
     </row>
@@ -1938,22 +1938,22 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Mentan Tunjuk Hidung Mafia Imbas Harga Ayam &amp;amp; Telur Naik</t>
+          <t>Aturan Tarif Ojol Antar Barang &amp;amp; Makanan Lagi Digarap, Ini Bocorannya</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Tue, 13 Oct 2026 07:30:17 +0700</t>
+          <t>Tue, 13 Oct 2026 19:23:38 +0700</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/07/28/wawancara-khusus-menteri-pertanian-ri-andi-amran-sulaiman-1753687994666_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Pertanian (Mentan) Andi Amran Sulaiman menuding mafia pangan berada di balik tingginya harga ayam dan telur di pasaran.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2021/09/15/driver-ojol-saat-antar-makanan-2_169.jpeg?w=360&amp;amp;q=90" /&gt; Kementerian Komunikasi dan Digital (Komdigi) menyelesaikan aturan turunan dari Peraturan Presiden (Perpres) No. 27 tahun 2026 tentang layanan ojek online.</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8704116/mentan-tunjuk-hidung-mafia-imbas-harga-ayam-telur-naik</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8705522/aturan-tarif-ojol-antar-barang-makanan-lagi-digarap-ini-bocorannya</t>
         </is>
       </c>
     </row>
@@ -1965,22 +1965,22 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Penjelasan Emiten Haji Isam soal Gadai Saham</t>
+          <t>Dirut Pertamina Puji Kolaborasi Semua Pihak di Balik Suksesnya GP Mandalika</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Tue, 13 Oct 2026 07:00:09 +0700</t>
+          <t>Tue, 13 Oct 2026 19:16:44 +0700</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/05/18/ihsg-anjlok-ke-zona-merah-bursa-saham-melemah-tajam-1779098741437_169.jpeg?w=360&amp;amp;q=90" /&gt; Emiten milik konglomerat Andi Syamsuddin Arsyad alias Haji Isam, PT Pradiksi Gunatama Tbk (PGUN), mengaku tidak terlibat langsung denga</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/13/pertamina-1791893786349_169.jpeg?w=360&amp;amp;q=90" /&gt; Pertamina Grand Prix of Indonesia 2026 sukses berkat kolaborasi berbagai pihak. Acara ini mendukung pariwisata dan pelaku usaha di Lombok.</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/bursa-dan-valas/d-8704113/penjelasan-emiten-haji-isam-soal-gadai-saham</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8705512/dirut-pertamina-puji-kolaborasi-semua-pihak-di-balik-suksesnya-gp-mandalika</t>
         </is>
       </c>
     </row>
@@ -1992,22 +1992,22 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Ekspor Benih Lobster Ditutup Permanen</t>
+          <t>Wamenperin Gelisah Hilirisasi Kelapa Sawit RI Mandek</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Tue, 13 Oct 2026 06:30:14 +0700</t>
+          <t>Tue, 13 Oct 2026 19:00:59 +0700</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/12/pemerintah-bentuk-satgas-p2bbl-berantas-penyelundupan-benih-bening-lobster-1791797202884_169.jpeg?w=360&amp;amp;q=90" /&gt; Pemerintah resmi menutup keran ekspor benih bening lobster (BBL) secara permanen</t>
+          <t xml:space="preserve">&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/10/16/wakil-menteri-perindustrian-wamenperin-faisol-riza-1760607570152_169.jpeg?w=360&amp;amp;q=90" /&gt; Wamenperin Faisol Riza gelisah karena hilirisasi kelapa sawit di Indonesia mandek. Ia bandingkan produktivitas sawit RI dengan Malaysia </t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8704109/ekspor-benih-lobster-ditutup-permanen</t>
+          <t>https://finance.detik.com/industri/d-8705474/wamenperin-gelisah-hilirisasi-kelapa-sawit-ri-mandek</t>
         </is>
       </c>
     </row>
@@ -2019,22 +2019,22 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Revisi UU LLAJ Bakal Atur Ojol Penumpang hingga Pengiriman Barang</t>
+          <t>IHSG Ditutup Melemah ke Level 5.925</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Tue, 13 Oct 2026 06:00:09 +0700</t>
+          <t>Tue, 13 Oct 2026 18:56:08 +0700</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/12/revisi-uu-llaj-bakal-atur-ojol-penumpang-hingga-pengiriman-barang-1791821935791_169.jpeg?w=360&amp;amp;q=90" /&gt; Pemerintah menyiapkan aturan ojek online melalui revisi UU LLAJ untuk memperkuat kepastian hukum dan keselamatan. Regulas</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/06/04/ihsg-terpuruk-kekhawatiran-pasar-meningkat-1780558039733_169.jpeg?w=360&amp;amp;q=90" /&gt; IHSG ditutup melemah di level 5.925, turun 0,17%. Volume transaksi mencapai 36.511 miliar saham. IHSG juga melemah 4,31% secara mingguan.</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/foto-bisnis/d-8704186/revisi-uu-llaj-bakal-atur-ojol-penumpang-hingga-pengiriman-barang</t>
+          <t>https://finance.detik.com/bursa-dan-valas/d-8705487/ihsg-ditutup-melemah-ke-level-5-925</t>
         </is>
       </c>
     </row>
@@ -2046,22 +2046,22 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Bahlil Sindir Bakrie di Depan Muka: Kawan Ini Tidak Paham-paham Juga</t>
+          <t>Penulis Why Nations Fail Ungkap Kunci Ekonomi RI Bisa Tumbuh 8%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Tue, 13 Oct 2026 05:55:05 +0700</t>
+          <t>Tue, 13 Oct 2026 18:00:10 +0700</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/07/16/menteri-esdm-bahlil-lahadalia-1784186781817_169.jpeg?w=360&amp;amp;q=90" /&gt; Indonesia menutup impor solar berkat program B50, namun beberapa perusahaan tambang masih ajukan izin. Bahlil dorong penggunaan etanol E50 untuk BBM.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/13/peraih-nobel-ekonomi-2024-sekaligus-penulis-buku-why-nations-fail-james-a-robinson-1791889160368_169.jpeg?w=360&amp;amp;q=90" /&gt; Peraih Nobel Ekonomi 2024 sekaligus penulis buku Why Nations Fail, James A. Robinson, membeberkan sejuml</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8704070/bahlil-sindir-bakrie-di-depan-muka-kawan-ini-tidak-paham-paham-juga</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8705395/penulis-why-nations-fail-ungkap-kunci-ekonomi-ri-bisa-tumbuh-8</t>
         </is>
       </c>
     </row>
@@ -2073,22 +2073,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>RI Genjot Koperasi Pertanian Bareng Negara Tetangga</t>
+          <t>Tak Kembalikan Duit Negara Rp 18 M, 91 Dapur MBG Kena Suspend!</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Mon, 12 Oct 2026 22:30:09 +0700</t>
+          <t>Tue, 13 Oct 2026 17:32:32 +0700</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/07/wakil-menteri-koperasi-wamenkop-farida-farichah-usai-menghadiri-pelantikan-dpd-knpi-lamongan-1791355884634_169.jpeg?w=360&amp;amp;q=90" /&gt; Indonesia menjalin kerja sama pengembangan koperasi pertanian bersama negara-negara ASEAN.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/02/ketut-sumedana-dok-istimewa-1788336147357_169.jpeg?w=360&amp;amp;q=90" /&gt; Sebanyak 91 SPPG yang dikenai suspend khusus tersebut tersebar di tiga wilayah, dengan total nilai temuan mencapai Rp 18,19 miliar.</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8704136/ri-genjot-koperasi-pertanian-bareng-negara-tetangga</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8705348/tak-kembalikan-duit-negara-rp-18-m-91-dapur-mbg-kena-suspend</t>
         </is>
       </c>
     </row>
@@ -2100,22 +2100,22 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Konsumsi Pertalite Melonjak hingga Antre Panjang di SPBU, Pertamina Buka Suara</t>
+          <t>Harga Minyak Melonjak, Wamenkeu Pastikan BBM Subsidi Tak Naik</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Mon, 12 Oct 2026 21:40:33 +0700</t>
+          <t>Tue, 13 Oct 2026 17:28:43 +0700</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/08/20/pemerintah-perketat-penyaluran-pertalite-mulai-2027-1787210254331_169.jpeg?w=360&amp;amp;q=90" /&gt; PT Pertamina Patra Niaga turun tangan memasok bahan bakar minyak (BBM) Kabupaten Bondowoso, Jawa Timur, seiring peningkatan kebutuhan m</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/02/05/juda-agung-tiba-di-kemenkeu-usai-dilantik-jadi-wakil-menteri-keuangan-1770289077443_169.jpeg?w=360&amp;amp;q=90" /&gt; Wakil Menteri Keuangan (Wamenkeu) Juda Agung memastikan pemerintah tidak berencana menaikkan harga bahan bakar minyak</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8704079/konsumsi-pertalite-melonjak-hingga-antre-panjang-di-spbu-pertamina-buka-suara</t>
+          <t>https://finance.detik.com/energi/d-8705338/harga-minyak-melonjak-wamenkeu-pastikan-bbm-subsidi-tak-naik</t>
         </is>
       </c>
     </row>
@@ -2127,22 +2127,22 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>RI Bidik Peluang Investasi Lewat Penguatan Pasar Karbon di COP31</t>
+          <t>Wamenperin soal Proyek Data Center Jatiluhur Disetop KDM: Itu Investasi Besar!</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Mon, 12 Oct 2026 21:13:52 +0700</t>
+          <t>Tue, 13 Oct 2026 17:17:31 +0700</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/12/ri-bidik-peluang-investasi-lewat-penguatan-pasar-karbon-di-cop31-1791814371200.jpeg?w=360&amp;amp;q=90" /&gt; Pemerintah dorong pasar karbon untuk investasi hijau di Indonesia. Menjelang COP31, Zulkifli Hasan tekankan pentingnya pembiay</t>
+          <t xml:space="preserve">&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/11/10/wakil-menteri-perindustrian-wamenperin-faisol-riza-1762753557434_169.jpeg?w=360&amp;amp;q=90" /&gt; Wamenperin Faisol Riza menyoroti penghentian proyek data center Jatiluhur oleh Gubernur Jabar. Ia menekankan pentingnya investasi untuk </t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8704059/ri-bidik-peluang-investasi-lewat-penguatan-pasar-karbon-di-cop31</t>
+          <t>https://finance.detik.com/industri/d-8705308/wamenperin-soal-proyek-data-center-jatiluhur-disetop-kdm-itu-investasi-besar</t>
         </is>
       </c>
     </row>
@@ -2154,22 +2154,22 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Update Sebaran Titik Api Pemicu Kebakaran Hutan di Sumatra dan Kalimantan</t>
+          <t>KPK Amankan 14 Orang dari OTT BNPB, Sestama Ikut Diciduk</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Tue, 13 Oct 2026 09:13:34 +0700</t>
+          <t>Tue, 13 Oct 2026 22:42:03 +0700</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Operasi modifikasi cuaca terus dimaksimalkan.</t>
+          <t>Salah satu pihak yang diamankan dalam OTT adalah Sekretaris Utama (Sestama) BNPB, Dr. apt. Rustian.</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8311731/update-sebaran-titik-api-pemicu-kebakaran-hutan-di-sumatra-dan-kalimantan</t>
+          <t>https://www.liputan6.com/news/read/8312529/kpk-amankan-14-orang-dari-ott-bnpb-sestama-ikut-diciduk</t>
         </is>
       </c>
     </row>
@@ -2181,22 +2181,22 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Strategi Prabowo Atasi Kebakaran Hutan Tanjung Puting</t>
+          <t>KPK Sita Rp 1,4 M dan Emas dalam OTT di BNPB</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Tue, 13 Oct 2026 08:17:38 +0700</t>
+          <t>Tue, 13 Oct 2026 22:37:59 +0700</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Prabowo juga menekankan pentingnya memperkuat keberadaan polisi hutan untuk menjaga kawasan hutan.</t>
+          <t>Sebanyak 14 orang, termasuk Sestama BNPB dan sejumlah pihak swasta, diamankan dalam OTT KPK</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8311715/strategi-prabowo-atasi-kebakaran-hutan-tanjung-puting</t>
+          <t>https://www.liputan6.com/news/read/8312525/kpk-sita-rp-14-m-dan-emas-dalam-ott-di-bnpb</t>
         </is>
       </c>
     </row>
@@ -2208,22 +2208,22 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Serangan Brutal KKB ke Warga Sipil di Yahukimo, 1 PNS Tewas</t>
+          <t>Lapak di Kampung Ambon Dibongkar, Polisi Buru Pemiliknya</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Tue, 13 Oct 2026 06:49:33 +0700</t>
+          <t>Tue, 13 Oct 2026 22:02:13 +0700</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>1 Lainnya dirawat intensif.</t>
+          <t>Pembongkaran lapak di Kampung Ambon mengungkap temuan alat isap sabu dan sisa narkoba.</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8311690/serangan-brutal-kkb-ke-warga-sipil-di-yahukimo-1-pns-tewas</t>
+          <t>https://www.liputan6.com/news/read/8312514/lapak-di-kampung-ambon-dibongkar-polisi-buru-pemiliknya</t>
         </is>
       </c>
     </row>
@@ -2235,22 +2235,22 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Saat Asap Mengepung Berbulan-bulan, Bencana Nasional Tak Ditetapkan</t>
+          <t>Guru Besar UGM Ungkap Masalah Pancasila dalam Praktik Bernegara</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Tue, 13 Oct 2026 07:18:11 +0700</t>
+          <t>Tue, 13 Oct 2026 22:00:37 +0700</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Bahkan beberapa negara tetangga juga ikut terpapar.</t>
+          <t>Guru Besar UGM Zainal Arifin Muchtar menilai Pancasila semestinya menjadi alat kontrol kekuasaan, bukan sekadar pembenar kebijakan penguasa.</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8311631/saat-asap-mengepung-berbulan-bulan-bencana-nasional-tak-ditetapkan</t>
+          <t>https://www.liputan6.com/news/read/8312422/guru-besar-ugm-ungkap-masalah-pancasila-dalam-praktik-bernegara</t>
         </is>
       </c>
     </row>
@@ -2262,22 +2262,22 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Balita Tewas Terbakar di Kamar Tidur Saat Ditinggal Ayah Beli Token</t>
+          <t>Pramono Pilih Dialog dalam Kasus Bentrokan Satpol PP di Bulungan</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Tue, 13 Oct 2026 07:11:20 +0700</t>
+          <t>Tue, 13 Oct 2026 21:47:02 +0700</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Ditemukan obat nyamuk yang terpasang di kamar.</t>
+          <t>Gubernur DKI Jakarta Pramono Anung memilih penyelesaian melalui dialog dan musyawarah dalam kasus bentrokan anggota Satpol PP</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8311685/balita-tewas-terbakar-di-kamar-tidur-saat-ditinggal-ayah-beli-token</t>
+          <t>https://www.liputan6.com/news/read/8312506/pramono-pilih-dialog-dalam-kasus-bentrokan-satpol-pp-di-bulungan</t>
         </is>
       </c>
     </row>
@@ -2289,22 +2289,22 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Petaka Telur Mentah Berujung Bayi Alena Meregang Nyawa</t>
+          <t>Gudang Paralon di Tangerang Kebakaran</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Tue, 13 Oct 2026 05:00:45 +0700</t>
+          <t>Tue, 13 Oct 2026 20:55:59 +0700</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Bayi Alena meninggal di usia 28 hari setelah sempat dirawat di rumah sakit. Begini keterangan pihak RSUD Dr. Soetomo.</t>
+          <t>Proses pemadaman sempat terkendala akibat sulitnya mendapatkan sumber air dan kemacetan parah di sekitar lokasi.</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8311665/petaka-telur-mentah-berujung-bayi-alena-meregang-nyawa</t>
+          <t>https://www.liputan6.com/news/read/8312474/gudang-paralon-di-tangerang-kebakaran</t>
         </is>
       </c>
     </row>
@@ -2316,22 +2316,22 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Menag Nasaruddin Ajak Tobat Ekologis, Ingatkan Bahaya Eksploitasi Alam</t>
+          <t>Kabar OTT KPK di Kantor BNPB, Begini Tanggapan Pegawai</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Tue, 13 Oct 2026 00:06:28 +0700</t>
+          <t>Tue, 13 Oct 2026 20:47:05 +0700</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Menag Nasaruddin Umar mengingatkan dampak kerusakan alam dan mengajak penerapan konsep ekoteologi dalam kehidupan sehari-hari.</t>
+          <t>BNPB Sebut Tak Ada OTT KPK di Kantor</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8311654/menag-nasaruddin-ajak-tobat-ekologis-ingatkan-bahaya-eksploitasi-alam</t>
+          <t>https://www.liputan6.com/news/read/8312467/kabar-ott-kpk-di-kantor-bnpb-begini-tanggapan-pegawai</t>
         </is>
       </c>
     </row>
@@ -2343,22 +2343,22 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Tabligh Akbar di Monas, Habib Nabiel Ajak Umat Islam Jaga Persatuan</t>
+          <t>Denny Indrayana Bakal Laporkan Dugaan Pasal Selundupan ke DKPP</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Mon, 12 Oct 2026 23:58:20 +0700</t>
+          <t>Tue, 13 Oct 2026 20:46:40 +0700</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Dalam Tabligh Akbar di Monas, Habib Nabiel menyoroti perpecahan, korupsi, hingga kebiasaan memfitnah.</t>
+          <t>Denny Indrayana menduga ada persoalan etik dalam penyusunan aturan syarat pendidikan capres-cawapres yang dikaitkan dengan pencalonan Gibran.</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8311651/tabligh-akbar-di-monas-habib-nabiel-ajak-umat-islam-jaga-persatuan</t>
+          <t>https://www.liputan6.com/news/read/8312458/denny-indrayana-bakal-laporkan-dugaan-pasal-selundupan-ke-dkpp</t>
         </is>
       </c>
     </row>
@@ -2370,22 +2370,22 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Infografis: 5 Miliarder Asia dengan Penurunan Kekayaan Terbesar</t>
+          <t>Gandeng Polda Metro Jaya, Pramono Siap Tertibkan Kampung Ambon</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Mon, 12 Oct 2026 22:52:51 +0700</t>
+          <t>Tue, 13 Oct 2026 20:08:32 +0700</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Miliarder  dari China, Indonesia, dan Korea Selatan mengalami penurunan kekayaan dengan nilai fantastis.</t>
+          <t>Pemprov DKI akan bersinergi dengan Polda Metro Jaya untuk menertibkan sejumlah kawasan yang menjadi sarang peredaran narkoba.</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8311630/infografis-5-miliarder-asia-dengan-penurunan-kekayaan-terbesar</t>
+          <t>https://www.liputan6.com/news/read/8312451/gandeng-polda-metro-jaya-pramono-siap-tertibkan-kampung-ambon</t>
         </is>
       </c>
     </row>
@@ -2397,22 +2397,22 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Prabowo Kerahkan Seluruh Sumber Daya untuk Tangani Kabakaran Hutan</t>
+          <t>Polisi Ungkap Dugaan Peredaran Catridge Mengandung Etomidate</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Tue, 13 Oct 2026 00:12:43 +0700</t>
+          <t>Tue, 13 Oct 2026 20:02:06 +0700</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Sebanyak 60.177 personel gabungan dikerahkan untuk menangani kebakaran hutan dan lahan.</t>
+          <t>Polisi mengembangkan penyelidikan ke rumah tersangka, menemukan 30 catridge yang diduga mengandung etomidate.</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8311629/prabowo-kerahkan-seluruh-sumber-daya-untuk-tangani-kabakaran-hutan</t>
+          <t>https://www.liputan6.com/news/read/8312444/polisi-ungkap-dugaan-peredaran-catridge-mengandung-etomidate</t>
         </is>
       </c>
     </row>
@@ -2424,22 +2424,22 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Jemaah Umrah Indonesia Dikabarkan Aman, Kemenhaj Minta Tetap Waspada</t>
+          <t>Tiga Embung dan Waduk Ini Disiapkan untuk Tekan Banjir Jakarta</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Mon, 12 Oct 2026 22:31:58 +0700</t>
+          <t>Tue, 13 Oct 2026 19:45:00 +0700</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Jemaah umrah Indonesiadi Arab Saudi diminta tetap waspada dan mengutamakan keselamatan.</t>
+          <t>Pembangunan ini disebutkan untuk mengurangi dampak banjir di Jakarta Selatan dan Timur.</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8311624/jemaah-umrah-indonesia-dikabarkan-aman-kemenhaj-minta-tetap-waspada</t>
+          <t>https://www.liputan6.com/news/read/8312439/tiga-embung-dan-waduk-ini-disiapkan-untuk-tekan-banjir-jakarta</t>
         </is>
       </c>
     </row>
@@ -2451,22 +2451,22 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>BRAN Percepat Penataan Kelembagaan dan Regulasi Reforma Agraria</t>
+          <t>YPP Emtek Salurkan Bantuan dan Layanan Kesehatan untuk Penyintas Gempa Flores</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Mon, 12 Oct 2026 21:50:39 +0700</t>
+          <t>Tue, 13 Oct 2026 19:38:25 +0700</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>BRAN menggandeng Kementerian Hukum dan berencana melibatkan akademisi untuk mengkaji regulasi yang menjadi landasan pelaksanaan reforma agraria.</t>
+          <t>YPP Emtek Media menyalurkan bantuan kebutuhan pokok, layanan kesehatan gratis, dan pendampingan psikososial.</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8311607/bran-percepat-penataan-kelembagaan-dan-regulasi-reforma-agraria</t>
+          <t>https://www.liputan6.com/news/read/8312437/ypp-emtek-salurkan-bantuan-dan-layanan-kesehatan-untuk-penyintas-gempa-flores</t>
         </is>
       </c>
     </row>
@@ -2478,22 +2478,22 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Mendagri Instruksikan Kepala Daerah Cegah Pembakaran Lahan</t>
+          <t>KPK OTT di BNPB</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Mon, 12 Oct 2026 20:27:46 +0700</t>
+          <t>Tue, 13 Oct 2026 19:18:48 +0700</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Di tengah kondisi darurat karhutla dan lahan yang mengering akibat kemarau, pemerintah meminta tidak ada pembakaran lahan baru.</t>
+          <t>Ketua KPK mengonfirmasi OTT di BNPB.</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8311558/mendagri-instruksikan-kepala-daerah-cegah-pembakaran-lahan</t>
+          <t>https://www.liputan6.com/news/read/8312425/kpk-ott-di-bnpb</t>
         </is>
       </c>
     </row>
@@ -2505,22 +2505,22 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Instruksi Prabowo Terkait Kebakaran Hutan di 6 Provinsi</t>
+          <t>Kasus Penyerangan Koorbid BEM UI Naik ke Penyidikan, 26 Titik CCTV Ditelusuri</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Mon, 12 Oct 2026 20:17:52 +0700</t>
+          <t>Tue, 13 Oct 2026 19:22:51 +0700</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Prabowo ingin pencegahan dilakukan sebelum api menyala.</t>
+          <t>Penyidik SPolda Metro Jaya menelusuri sekitar 26 titik CCTV dan mengamankan sejumlah barang bukti.</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8311555/instruksi-prabowo-terkait-kebakaran-hutan-di-6-provinsi</t>
+          <t>https://www.liputan6.com/news/read/8312420/kasus-penyerangan-koorbid-bem-ui-naik-ke-penyidikan-26-titik-cctv-ditelusuri</t>
         </is>
       </c>
     </row>
@@ -2532,22 +2532,22 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Prabowo Tunjuk Satyawan Pudyatmoko Jadi Kepala Badan Pengelolaan Gambut dan Mangrove</t>
+          <t>KPK Sita Land Cruiser Orang Dekat Nusron Wahid di Kasus HGB Summarecon</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Mon, 12 Oct 2026 20:07:29 +0700</t>
+          <t>Tue, 13 Oct 2026 18:59:33 +0700</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Satyawan merupakan ahli di bidang pengelolaan gambut dan mangrove sehingga cocok memimpin badan tersebut.</t>
+          <t>KPK menyita Toyota Land Cruiser milik tersangka kasus suap HGB Summarecon yang diduga digunakan untuk aktivitas pengumpulan uang.</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8311541/prabowo-tunjuk-satyawan-pudyatmoko-jadi-kepala-badan-pengelolaan-gambut-dan-mangrove</t>
+          <t>https://www.liputan6.com/news/read/8312406/kpk-sita-land-cruiser-orang-dekat-nusron-wahid-di-kasus-hgb-summarecon</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data pasar & berita - 2026-10-14 00:40 UTC
</commit_message>
<xml_diff>
--- a/data/market_news_latest.xlsx
+++ b/data/market_news_latest.xlsx
@@ -422,7 +422,7 @@
     <col width="26" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
   </cols>
@@ -487,20 +487,20 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>5925.9761</v>
+        <v>5936.147</v>
       </c>
       <c r="F2" t="n">
-        <v>-10.1709</v>
+        <v>-157.6118</v>
       </c>
       <c r="G2" t="n">
-        <v>-0.17</v>
+        <v>-2.59</v>
       </c>
       <c r="H2" t="n">
-        <v>0</v>
+        <v>559257300</v>
       </c>
     </row>
     <row r="3">
@@ -525,16 +525,16 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>7787.8799</v>
+        <v>7805.4502</v>
       </c>
       <c r="F3" t="n">
-        <v>-19.3604</v>
+        <v>-1.79</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.25</v>
+        <v>-0.02</v>
       </c>
       <c r="H3" t="n">
-        <v>869506500</v>
+        <v>2640232000</v>
       </c>
     </row>
     <row r="4">
@@ -559,16 +559,16 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>51678.6289</v>
+        <v>51670.1016</v>
       </c>
       <c r="F4" t="n">
-        <v>-171.9219</v>
+        <v>-180.4492</v>
       </c>
       <c r="G4" t="n">
-        <v>-0.33</v>
+        <v>-0.35</v>
       </c>
       <c r="H4" t="n">
-        <v>153969361</v>
+        <v>395694761</v>
       </c>
     </row>
     <row r="5">
@@ -593,16 +593,16 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>27149.7734</v>
+        <v>27204.3809</v>
       </c>
       <c r="F5" t="n">
-        <v>-96.127</v>
+        <v>-41.5195</v>
       </c>
       <c r="G5" t="n">
-        <v>-0.35</v>
+        <v>-0.15</v>
       </c>
       <c r="H5" t="n">
-        <v>2719719000</v>
+        <v>6273913000</v>
       </c>
     </row>
     <row r="6">
@@ -623,20 +623,20 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>69030.9219</v>
+        <v>67943.1094</v>
       </c>
       <c r="F6" t="n">
-        <v>-11.1875</v>
+        <v>-1087.8125</v>
       </c>
       <c r="G6" t="n">
-        <v>-0.02</v>
+        <v>-1.58</v>
       </c>
       <c r="H6" t="n">
-        <v>162000000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -657,20 +657,20 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>24345.2207</v>
+        <v>24271.1992</v>
       </c>
       <c r="F7" t="n">
-        <v>74.0215</v>
+        <v>59.8496</v>
       </c>
       <c r="G7" t="n">
-        <v>0.3</v>
+        <v>0.25</v>
       </c>
       <c r="H7" t="n">
-        <v>0</v>
+        <v>2229800000</v>
       </c>
     </row>
     <row r="8">
@@ -694,15 +694,9 @@
           <t>2026-10-13</t>
         </is>
       </c>
-      <c r="E8" t="n">
-        <v>3800.8645</v>
-      </c>
-      <c r="F8" t="n">
-        <v>3.6226</v>
-      </c>
-      <c r="G8" t="n">
-        <v>0.1</v>
-      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
       <c r="H8" t="n">
         <v>1085950644</v>
       </c>
@@ -725,20 +719,20 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>10649.1201</v>
+        <v>10656.2998</v>
       </c>
       <c r="F9" t="n">
-        <v>-7.1797</v>
+        <v>104.2002</v>
       </c>
       <c r="G9" t="n">
-        <v>-0.07000000000000001</v>
+        <v>0.99</v>
       </c>
       <c r="H9" t="n">
-        <v>0</v>
+        <v>575809000</v>
       </c>
     </row>
     <row r="10">
@@ -759,20 +753,20 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>25251.1504</v>
+        <v>25277.6797</v>
       </c>
       <c r="F10" t="n">
-        <v>-26.5293</v>
+        <v>190.4102</v>
       </c>
       <c r="G10" t="n">
-        <v>-0.1</v>
+        <v>0.76</v>
       </c>
       <c r="H10" t="n">
-        <v>0</v>
+        <v>39349200</v>
       </c>
     </row>
     <row r="11">
@@ -793,20 +787,20 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>5430.5</v>
+        <v>5415.48</v>
       </c>
       <c r="F11" t="n">
-        <v>15.02</v>
+        <v>13.5898</v>
       </c>
       <c r="G11" t="n">
-        <v>0.28</v>
+        <v>0.25</v>
       </c>
       <c r="H11" t="n">
-        <v>0</v>
+        <v>243072800</v>
       </c>
     </row>
     <row r="12">
@@ -831,13 +825,13 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>17925</v>
+        <v>17913</v>
       </c>
       <c r="F12" t="n">
-        <v>117.5</v>
+        <v>3</v>
       </c>
       <c r="G12" t="n">
-        <v>0.66</v>
+        <v>0.02</v>
       </c>
       <c r="H12" t="n">
         <v>0</v>
@@ -865,13 +859,13 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>102.283</v>
+        <v>102.173</v>
       </c>
       <c r="F13" t="n">
-        <v>-0.297</v>
+        <v>-0.407</v>
       </c>
       <c r="G13" t="n">
-        <v>-0.29</v>
+        <v>-0.4</v>
       </c>
       <c r="H13" t="n">
         <v>0</v>
@@ -895,17 +889,17 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>158.397</v>
+        <v>158.378</v>
       </c>
       <c r="F14" t="n">
-        <v>0.334</v>
+        <v>-0.142</v>
       </c>
       <c r="G14" t="n">
-        <v>0.21</v>
+        <v>-0.09</v>
       </c>
       <c r="H14" t="n">
         <v>0</v>
@@ -967,13 +961,13 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>0.5565</v>
+        <v>0.5563</v>
       </c>
       <c r="F16" t="n">
-        <v>-0.0033</v>
+        <v>-0.0035</v>
       </c>
       <c r="G16" t="n">
-        <v>-0.59</v>
+        <v>-0.63</v>
       </c>
       <c r="H16" t="n">
         <v>0</v>
@@ -1001,13 +995,13 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>0.4063</v>
+        <v>0.4057</v>
       </c>
       <c r="F17" t="n">
-        <v>0.0013</v>
+        <v>0.0007</v>
       </c>
       <c r="G17" t="n">
-        <v>0.32</v>
+        <v>0.17</v>
       </c>
       <c r="H17" t="n">
         <v>0</v>
@@ -1034,17 +1028,11 @@
           <t>2026-10-13</t>
         </is>
       </c>
-      <c r="E18" t="n">
-        <v>78.265</v>
-      </c>
-      <c r="F18" t="n">
-        <v>0.215</v>
-      </c>
-      <c r="G18" t="n">
-        <v>0.28</v>
-      </c>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
       <c r="H18" t="n">
-        <v>12544097</v>
+        <v>29149160</v>
       </c>
     </row>
     <row r="19">
@@ -1068,17 +1056,11 @@
           <t>2026-10-13</t>
         </is>
       </c>
-      <c r="E19" t="n">
-        <v>77.0001</v>
-      </c>
-      <c r="F19" t="n">
-        <v>-0.2899</v>
-      </c>
-      <c r="G19" t="n">
-        <v>-0.38</v>
-      </c>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr"/>
       <c r="H19" t="n">
-        <v>27766515</v>
+        <v>60522261</v>
       </c>
     </row>
     <row r="20">
@@ -1103,16 +1085,16 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>4184.6001</v>
+        <v>4183.8999</v>
       </c>
       <c r="F20" t="n">
-        <v>-6</v>
+        <v>-6.7002</v>
       </c>
       <c r="G20" t="n">
-        <v>-0.14</v>
+        <v>-0.16</v>
       </c>
       <c r="H20" t="n">
-        <v>90400</v>
+        <v>4912</v>
       </c>
     </row>
     <row r="21">
@@ -1137,16 +1119,16 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>94.2</v>
+        <v>94.98</v>
       </c>
       <c r="F21" t="n">
-        <v>0.46</v>
+        <v>1.24</v>
       </c>
       <c r="G21" t="n">
-        <v>0.49</v>
+        <v>1.32</v>
       </c>
       <c r="H21" t="n">
-        <v>135225</v>
+        <v>3997</v>
       </c>
     </row>
     <row r="22">
@@ -1171,16 +1153,16 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>106.07</v>
+        <v>106.58</v>
       </c>
       <c r="F22" t="n">
-        <v>-0.58</v>
+        <v>-0.07000000000000001</v>
       </c>
       <c r="G22" t="n">
-        <v>-0.54</v>
+        <v>-0.07000000000000001</v>
       </c>
       <c r="H22" t="n">
-        <v>22916</v>
+        <v>404</v>
       </c>
     </row>
     <row r="23">
@@ -1205,16 +1187,16 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>6.733</v>
+        <v>6.7195</v>
       </c>
       <c r="F23" t="n">
-        <v>0.0345</v>
+        <v>0.021</v>
       </c>
       <c r="G23" t="n">
-        <v>0.52</v>
+        <v>0.31</v>
       </c>
       <c r="H23" t="n">
-        <v>21438</v>
+        <v>759</v>
       </c>
     </row>
     <row r="24">
@@ -1238,17 +1220,11 @@
           <t>2026-10-13</t>
         </is>
       </c>
-      <c r="E24" t="n">
-        <v>65.45</v>
-      </c>
-      <c r="F24" t="n">
-        <v>-0.7</v>
-      </c>
-      <c r="G24" t="n">
-        <v>-1.06</v>
-      </c>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr"/>
       <c r="H24" t="n">
-        <v>7502005</v>
+        <v>21414742</v>
       </c>
     </row>
     <row r="25">
@@ -1273,13 +1249,13 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>15.41</v>
+        <v>15.27</v>
       </c>
       <c r="F25" t="n">
-        <v>0.2</v>
+        <v>0.06</v>
       </c>
       <c r="G25" t="n">
-        <v>1.31</v>
+        <v>0.39</v>
       </c>
       <c r="H25" t="n">
         <v>0</v>
@@ -1303,20 +1279,20 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="E26" t="n">
-        <v>83174.7188</v>
+        <v>83618.5938</v>
       </c>
       <c r="F26" t="n">
-        <v>1412.1562</v>
+        <v>1856.0312</v>
       </c>
       <c r="G26" t="n">
-        <v>1.73</v>
+        <v>2.27</v>
       </c>
       <c r="H26" t="n">
-        <v>31508934656</v>
+        <v>29613316096</v>
       </c>
     </row>
     <row r="27">
@@ -1344,10 +1320,10 @@
         <v>1310</v>
       </c>
       <c r="F27" t="n">
-        <v>-95</v>
+        <v>-35</v>
       </c>
       <c r="G27" t="n">
-        <v>-6.76</v>
+        <v>-2.6</v>
       </c>
       <c r="H27" t="n">
         <v>80411200</v>
@@ -1378,10 +1354,10 @@
         <v>1520</v>
       </c>
       <c r="F28" t="n">
-        <v>-155</v>
+        <v>15</v>
       </c>
       <c r="G28" t="n">
-        <v>-9.25</v>
+        <v>1</v>
       </c>
       <c r="H28" t="n">
         <v>127296000</v>
@@ -1412,10 +1388,10 @@
         <v>665</v>
       </c>
       <c r="F29" t="n">
-        <v>-105</v>
+        <v>10</v>
       </c>
       <c r="G29" t="n">
-        <v>-13.64</v>
+        <v>1.53</v>
       </c>
       <c r="H29" t="n">
         <v>434856000</v>
@@ -1446,10 +1422,10 @@
         <v>2430</v>
       </c>
       <c r="F30" t="n">
-        <v>-270</v>
+        <v>40</v>
       </c>
       <c r="G30" t="n">
-        <v>-10</v>
+        <v>1.67</v>
       </c>
       <c r="H30" t="n">
         <v>13220900</v>
@@ -1480,10 +1456,10 @@
         <v>4180</v>
       </c>
       <c r="F31" t="n">
-        <v>-570</v>
+        <v>140</v>
       </c>
       <c r="G31" t="n">
-        <v>-12</v>
+        <v>3.47</v>
       </c>
       <c r="H31" t="n">
         <v>47740700</v>
@@ -1514,10 +1490,10 @@
         <v>500</v>
       </c>
       <c r="F32" t="n">
-        <v>-55</v>
+        <v>0</v>
       </c>
       <c r="G32" t="n">
-        <v>-9.91</v>
+        <v>0</v>
       </c>
       <c r="H32" t="n">
         <v>51400500</v>
@@ -1548,10 +1524,10 @@
         <v>605</v>
       </c>
       <c r="F33" t="n">
-        <v>-60</v>
+        <v>20</v>
       </c>
       <c r="G33" t="n">
-        <v>-9.02</v>
+        <v>3.42</v>
       </c>
       <c r="H33" t="n">
         <v>50719300</v>
@@ -1582,10 +1558,10 @@
         <v>3710</v>
       </c>
       <c r="F34" t="n">
-        <v>-330</v>
+        <v>130</v>
       </c>
       <c r="G34" t="n">
-        <v>-8.17</v>
+        <v>3.63</v>
       </c>
       <c r="H34" t="n">
         <v>3833300</v>
@@ -1613,16 +1589,16 @@
         </is>
       </c>
       <c r="E35" t="n">
-        <v>590</v>
+        <v>522</v>
       </c>
       <c r="F35" t="n">
-        <v>-75</v>
+        <v>-53</v>
       </c>
       <c r="G35" t="n">
-        <v>-11.28</v>
+        <v>-9.220000000000001</v>
       </c>
       <c r="H35" t="n">
-        <v>67977500</v>
+        <v>76832806</v>
       </c>
     </row>
     <row r="36">
@@ -1650,10 +1626,10 @@
         <v>199</v>
       </c>
       <c r="F36" t="n">
-        <v>-11</v>
+        <v>4</v>
       </c>
       <c r="G36" t="n">
-        <v>-5.24</v>
+        <v>2.05</v>
       </c>
       <c r="H36" t="n">
         <v>18782500</v>
@@ -1684,10 +1660,10 @@
         <v>14250</v>
       </c>
       <c r="F37" t="n">
-        <v>-1550</v>
+        <v>550</v>
       </c>
       <c r="G37" t="n">
-        <v>-9.81</v>
+        <v>4.01</v>
       </c>
       <c r="H37" t="n">
         <v>11233300</v>
@@ -1749,22 +1725,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>BTPN Syariah (BTPS) Bakal Buyback Saham hingga Rp 1 Triliun</t>
+          <t>Bukan UMP Naik, Bos Buruh Ungkap Biang Kerok Pabrik Tutup</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Tue, 13 Oct 2026 22:35:02 +0700</t>
+          <t>Wed, 14 Oct 2026 07:00:03 +0700</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/13/rupslb-btpn-syariah-1791905594130_169.jpeg?w=360&amp;amp;q=90" /&gt; PT Bank BTPN Syariah Tbk mengajukan rencana aksi korporasi pembelian kembali saham (buyback) dengan nilai maksimal hingga Rp1 triliun</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2021/02/23/ilustrasi-uang_169.jpeg?w=360&amp;amp;q=90" /&gt; Kenaikan upah minimum provinsi (UMP) dinilai bukan biang kerok beberapa pabrik di Indonesia tutup, menurut Presiden KSPI Said Iqbal.</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/bursa-dan-valas/d-8705745/btpn-syariah-btps-bakal-buyback-saham-hingga-rp-1-triliun</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8705738/bukan-ump-naik-bos-buruh-ungkap-biang-kerok-pabrik-tutup</t>
         </is>
       </c>
     </row>
@@ -1776,22 +1752,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Zero ODOL Bisa Gagal Jika Cuma Tertibkan Truk, Ini Saran buat Pemerintah</t>
+          <t>Bank Dunia &amp;amp; IMF Wanti-wanti Dampak Buruk AI</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Tue, 13 Oct 2026 22:30:00 +0700</t>
+          <t>Wed, 14 Oct 2026 06:30:15 +0700</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/06/19/kepadatan-lalu-lintas-di-jalan-raya-wonokromo-surabaya-imbas-demo-sopir-truk-toal-aturan-odol-1750328242861_169.jpeg?w=360&amp;amp;q=90" /&gt; Pemerintah akan menerapkan Zero Over Dimension Overloading (ODOL) pada 2027.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/30/ai-openai-1790740749134_169.jpeg?w=360&amp;amp;q=90" /&gt; IMF dan Bank Dunia memperingatkan dampak buruk artificial intelligence alias AI terhadap lapangan pekerjaan.</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8705733/zero-odol-bisa-gagal-jika-cuma-tertibkan-truk-ini-saran-buat-pemerintah</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8705734/bank-dunia-imf-wanti-wanti-dampak-buruk-ai</t>
         </is>
       </c>
     </row>
@@ -1803,22 +1779,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Panen Melimpah, Harga Garam Petani Takalar Turun Tajam</t>
+          <t>Heboh Rumor Emiten Bakrie Caplok Tambang Kideco Rp 17,9 Triliun</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Tue, 13 Oct 2026 22:00:16 +0700</t>
+          <t>Wed, 14 Oct 2026 05:55:45 +0700</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/13/harga-garam-turun-di-kabupaten-takalar-1791872493195_169.jpeg?w=360&amp;amp;q=90" /&gt; Harga garam di Takalar anjlok dari Rp150 ribu menjadi Rp45 ribu per karung akibat panen melimpah saat kemarau. Petani berharap bantuan gudang.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/12/menembus-perut-bumi-mahasiswa-belajar-di-tambang-tua-sawahlunto-1791790427682_169.jpeg?w=360&amp;amp;q=90" /&gt; PT Bumi Resources Tbk (BUMI) disebut akan mengakuisisi tambang batu bara termal milik PT Indika Energy Tbk (INDY), Kideco J</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/foto-bisnis/d-8704804/panen-melimpah-harga-garam-petani-takalar-turun-tajam</t>
+          <t>https://finance.detik.com/bursa-dan-valas/d-8705731/heboh-rumor-emiten-bakrie-caplok-tambang-kideco-rp-17-9-triliun</t>
         </is>
       </c>
     </row>
@@ -1830,22 +1806,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Mau Jago Hitung Pajak, Tapi Bingung Mulai dari Mana? Coba Kursus di Sini!</t>
+          <t>Perpres Ojol Terbit, Pengemudi Masih Keluhkan Potongan dan Tarif Jarak</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Tue, 13 Oct 2026 21:40:18 +0700</t>
+          <t>Wed, 14 Oct 2026 05:50:03 +0700</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/07/28/smart-class-brevet-pajak-a-b-1785248368520_169.png?w=360&amp;amp;q=90" /&gt; i fokus Pelatihan Brevet Pajak AB + Sertifikasi CTT dan CCP dari Piranha Smart Center (PSC) bersama Education Visionary Lab (EVL).</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/13/perpres-ojol-terbit-pengemudi-masih-keluhkan-potongan-dan-tarif-jarak-1791896085197.jpeg?w=360&amp;amp;q=90" /&gt; Pemerintah membatasi potongan biaya platform ojol maksimal 8% lewat Perpres 27/2026. Namun, pengemudi masih mengeluhkan p</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8705693/mau-jago-hitung-pajak-tapi-bingung-mulai-dari-mana-coba-kursus-di-sini</t>
+          <t>https://finance.detik.com/foto-bisnis/d-8705570/perpres-ojol-terbit-pengemudi-masih-keluhkan-potongan-dan-tarif-jarak</t>
         </is>
       </c>
     </row>
@@ -1857,22 +1833,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Beli Token &amp;amp; Bayar Tagihan Listrik Bisa di Kopdes Merah Putih</t>
+          <t>Transformasi PERURI, Jaga Warisan &amp;amp; Bangun Masa Depan Digital</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Tue, 13 Oct 2026 21:23:38 +0700</t>
+          <t>Wed, 14 Oct 2026 00:00:00 +0700</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/21/kopdes-merah-putih-bersiap-operasional-23-ribu-bangunan-telah-rampung-1789986171319_169.jpeg?w=360&amp;amp;q=90" /&gt; PLN mendukung program Koperasi Desa/Kelurahan Merah Putih atau Kopdes Merah Putih melalui kemitraan layanan pembayara</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/13/adv-peruri-1791887140082.png?w=360&amp;amp;q=90" /&gt; Selama puluhan tahun, PERURI memiliki peran dalam kehidupan masyarakat mulai dari bertransaksi menggunakan uang rupiah, menggunakan paspor saat bepergian</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8705683/beli-token-bayar-tagihan-listrik-bisa-di-kopdes-merah-putih</t>
+          <t>https://finance.detik.com/advertorial-news-block/d-8705335/transformasi-peruri-jaga-warisan-bangun-masa-depan-digital</t>
         </is>
       </c>
     </row>
@@ -1884,22 +1860,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>1.813 Penerbangan Terdampak Karhutla, Mayoritas Gagal Terbang</t>
+          <t>Mau Kelola Pajak dengan Lebih Terarah? Yuk, Pelajari Dasarnya!</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Tue, 13 Oct 2026 20:46:22 +0700</t>
+          <t>Tue, 13 Oct 2026 23:30:30 +0700</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/17/kabut-asap-karhutla-ganggu-penerbangan-di-bandara-palembang-1789622375071_169.jpeg?w=360&amp;amp;q=90" /&gt; Kementerian Perhubungan (Kemenhub) mencatat total 1.813 penerbangan terdampak kebakaran hutan dan lahan (karhutla) sejak 11 Agu</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/07/28/smart-class-brevet-pajak-a-b-1785248368520_169.png?w=360&amp;amp;q=90" /&gt; Piranha Smart Center (PSC) bersama Education Visionary Lab (EVL) menghadirkan Professional Smart Class: Pelatihan Brevet Pajak AB + Sertifikasi CTT dan CCP.</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8705647/1-813-penerbangan-terdampak-karhutla-mayoritas-gagal-terbang</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8705696/mau-kelola-pajak-dengan-lebih-terarah-yuk-pelajari-dasarnya</t>
         </is>
       </c>
     </row>
@@ -1911,22 +1887,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Menteri LH Ingatkan Pengusaha, Biaya Urus Lingkungan Hidup Bukan Beban!</t>
+          <t>Ingin Lebih Siap Jadi Auditor? Kenali Proses Audit Digital Lewat Pelatihan Ini</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Tue, 13 Oct 2026 20:11:54 +0700</t>
+          <t>Tue, 13 Oct 2026 22:45:52 +0700</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/29/menteri-lh-mohammad-jumhur-hidayat-saat-kunjungi-objek-wisata-di-cisarua-1790687703176_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Lingkungan Hidup Mohammad Jumhur Hidayat menegaskan biaya yang dikeluarkan perusahaan dalam pengelolaan li</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/13/detikevent-authen-1791906268082_169.jpeg?w=360&amp;amp;q=90" /&gt; Peserta akan mengikuti demonstrasi penggunaan platform AUTHEN, praktik berbasis studi kasus, diskusi interaktif, serta pendampingan mentor.</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8705607/menteri-lh-ingatkan-pengusaha-biaya-urus-lingkungan-hidup-bukan-beban</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8705759/ingin-lebih-siap-jadi-auditor-kenali-proses-audit-digital-lewat-pelatihan-ini</t>
         </is>
       </c>
     </row>
@@ -1938,22 +1914,22 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Aturan Tarif Ojol Antar Barang &amp;amp; Makanan Lagi Digarap, Ini Bocorannya</t>
+          <t>BTPN Syariah (BTPS) Bakal Buyback Saham hingga Rp 1 Triliun</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Tue, 13 Oct 2026 19:23:38 +0700</t>
+          <t>Tue, 13 Oct 2026 22:35:02 +0700</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2021/09/15/driver-ojol-saat-antar-makanan-2_169.jpeg?w=360&amp;amp;q=90" /&gt; Kementerian Komunikasi dan Digital (Komdigi) menyelesaikan aturan turunan dari Peraturan Presiden (Perpres) No. 27 tahun 2026 tentang layanan ojek online.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/13/rupslb-btpn-syariah-1791905594130_169.jpeg?w=360&amp;amp;q=90" /&gt; PT Bank BTPN Syariah Tbk mengajukan rencana aksi korporasi pembelian kembali saham (buyback) dengan nilai maksimal hingga Rp1 triliun</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8705522/aturan-tarif-ojol-antar-barang-makanan-lagi-digarap-ini-bocorannya</t>
+          <t>https://finance.detik.com/bursa-dan-valas/d-8705745/btpn-syariah-btps-bakal-buyback-saham-hingga-rp-1-triliun</t>
         </is>
       </c>
     </row>
@@ -1965,22 +1941,22 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Dirut Pertamina Puji Kolaborasi Semua Pihak di Balik Suksesnya GP Mandalika</t>
+          <t>Zero ODOL Bisa Gagal Jika Cuma Tertibkan Truk, Ini Saran buat Pemerintah</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Tue, 13 Oct 2026 19:16:44 +0700</t>
+          <t>Tue, 13 Oct 2026 22:30:00 +0700</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/13/pertamina-1791893786349_169.jpeg?w=360&amp;amp;q=90" /&gt; Pertamina Grand Prix of Indonesia 2026 sukses berkat kolaborasi berbagai pihak. Acara ini mendukung pariwisata dan pelaku usaha di Lombok.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/06/19/kepadatan-lalu-lintas-di-jalan-raya-wonokromo-surabaya-imbas-demo-sopir-truk-toal-aturan-odol-1750328242861_169.jpeg?w=360&amp;amp;q=90" /&gt; Pemerintah akan menerapkan Zero Over Dimension Overloading (ODOL) pada 2027.</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8705512/dirut-pertamina-puji-kolaborasi-semua-pihak-di-balik-suksesnya-gp-mandalika</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8705733/zero-odol-bisa-gagal-jika-cuma-tertibkan-truk-ini-saran-buat-pemerintah</t>
         </is>
       </c>
     </row>
@@ -1992,22 +1968,22 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Wamenperin Gelisah Hilirisasi Kelapa Sawit RI Mandek</t>
+          <t>Panen Melimpah, Harga Garam Petani Takalar Turun Tajam</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Tue, 13 Oct 2026 19:00:59 +0700</t>
+          <t>Tue, 13 Oct 2026 22:00:16 +0700</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/10/16/wakil-menteri-perindustrian-wamenperin-faisol-riza-1760607570152_169.jpeg?w=360&amp;amp;q=90" /&gt; Wamenperin Faisol Riza gelisah karena hilirisasi kelapa sawit di Indonesia mandek. Ia bandingkan produktivitas sawit RI dengan Malaysia </t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/13/harga-garam-turun-di-kabupaten-takalar-1791872493195_169.jpeg?w=360&amp;amp;q=90" /&gt; Harga garam di Takalar anjlok dari Rp150 ribu menjadi Rp45 ribu per karung akibat panen melimpah saat kemarau. Petani berharap bantuan gudang.</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/industri/d-8705474/wamenperin-gelisah-hilirisasi-kelapa-sawit-ri-mandek</t>
+          <t>https://finance.detik.com/foto-bisnis/d-8704804/panen-melimpah-harga-garam-petani-takalar-turun-tajam</t>
         </is>
       </c>
     </row>
@@ -2019,22 +1995,22 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>IHSG Ditutup Melemah ke Level 5.925</t>
+          <t>Mau Jago Hitung Pajak, Tapi Bingung Mulai dari Mana? Coba Kursus di Sini!</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Tue, 13 Oct 2026 18:56:08 +0700</t>
+          <t>Tue, 13 Oct 2026 21:40:18 +0700</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/06/04/ihsg-terpuruk-kekhawatiran-pasar-meningkat-1780558039733_169.jpeg?w=360&amp;amp;q=90" /&gt; IHSG ditutup melemah di level 5.925, turun 0,17%. Volume transaksi mencapai 36.511 miliar saham. IHSG juga melemah 4,31% secara mingguan.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/07/28/smart-class-brevet-pajak-a-b-1785248368520_169.png?w=360&amp;amp;q=90" /&gt; i fokus Pelatihan Brevet Pajak AB + Sertifikasi CTT dan CCP dari Piranha Smart Center (PSC) bersama Education Visionary Lab (EVL).</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/bursa-dan-valas/d-8705487/ihsg-ditutup-melemah-ke-level-5-925</t>
+          <t>https://finance.detik.com/energi/d-8705693/mau-jago-hitung-pajak-tapi-bingung-mulai-dari-mana-coba-kursus-di-sini</t>
         </is>
       </c>
     </row>
@@ -2046,22 +2022,22 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Penulis Why Nations Fail Ungkap Kunci Ekonomi RI Bisa Tumbuh 8%</t>
+          <t>Beli Token &amp;amp; Bayar Tagihan Listrik Bisa di Kopdes Merah Putih</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Tue, 13 Oct 2026 18:00:10 +0700</t>
+          <t>Tue, 13 Oct 2026 21:23:38 +0700</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/13/peraih-nobel-ekonomi-2024-sekaligus-penulis-buku-why-nations-fail-james-a-robinson-1791889160368_169.jpeg?w=360&amp;amp;q=90" /&gt; Peraih Nobel Ekonomi 2024 sekaligus penulis buku Why Nations Fail, James A. Robinson, membeberkan sejuml</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/21/kopdes-merah-putih-bersiap-operasional-23-ribu-bangunan-telah-rampung-1789986171319_169.jpeg?w=360&amp;amp;q=90" /&gt; PLN mendukung program Koperasi Desa/Kelurahan Merah Putih atau Kopdes Merah Putih melalui kemitraan layanan pembayara</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8705395/penulis-why-nations-fail-ungkap-kunci-ekonomi-ri-bisa-tumbuh-8</t>
+          <t>https://finance.detik.com/energi/d-8705683/beli-token-bayar-tagihan-listrik-bisa-di-kopdes-merah-putih</t>
         </is>
       </c>
     </row>
@@ -2073,22 +2049,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Tak Kembalikan Duit Negara Rp 18 M, 91 Dapur MBG Kena Suspend!</t>
+          <t>1.813 Penerbangan Terdampak Karhutla, Mayoritas Gagal Terbang</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Tue, 13 Oct 2026 17:32:32 +0700</t>
+          <t>Tue, 13 Oct 2026 20:46:22 +0700</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/02/ketut-sumedana-dok-istimewa-1788336147357_169.jpeg?w=360&amp;amp;q=90" /&gt; Sebanyak 91 SPPG yang dikenai suspend khusus tersebut tersebar di tiga wilayah, dengan total nilai temuan mencapai Rp 18,19 miliar.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/17/kabut-asap-karhutla-ganggu-penerbangan-di-bandara-palembang-1789622375071_169.jpeg?w=360&amp;amp;q=90" /&gt; Kementerian Perhubungan (Kemenhub) mencatat total 1.813 penerbangan terdampak kebakaran hutan dan lahan (karhutla) sejak 11 Agu</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8705348/tak-kembalikan-duit-negara-rp-18-m-91-dapur-mbg-kena-suspend</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8705647/1-813-penerbangan-terdampak-karhutla-mayoritas-gagal-terbang</t>
         </is>
       </c>
     </row>
@@ -2100,22 +2076,22 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Harga Minyak Melonjak, Wamenkeu Pastikan BBM Subsidi Tak Naik</t>
+          <t>Menteri LH Ingatkan Pengusaha, Biaya Urus Lingkungan Hidup Bukan Beban!</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Tue, 13 Oct 2026 17:28:43 +0700</t>
+          <t>Tue, 13 Oct 2026 20:11:54 +0700</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/02/05/juda-agung-tiba-di-kemenkeu-usai-dilantik-jadi-wakil-menteri-keuangan-1770289077443_169.jpeg?w=360&amp;amp;q=90" /&gt; Wakil Menteri Keuangan (Wamenkeu) Juda Agung memastikan pemerintah tidak berencana menaikkan harga bahan bakar minyak</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/29/menteri-lh-mohammad-jumhur-hidayat-saat-kunjungi-objek-wisata-di-cisarua-1790687703176_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Lingkungan Hidup Mohammad Jumhur Hidayat menegaskan biaya yang dikeluarkan perusahaan dalam pengelolaan li</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8705338/harga-minyak-melonjak-wamenkeu-pastikan-bbm-subsidi-tak-naik</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8705607/menteri-lh-ingatkan-pengusaha-biaya-urus-lingkungan-hidup-bukan-beban</t>
         </is>
       </c>
     </row>
@@ -2127,22 +2103,22 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Wamenperin soal Proyek Data Center Jatiluhur Disetop KDM: Itu Investasi Besar!</t>
+          <t>Aturan Tarif Ojol Antar Barang &amp;amp; Makanan Lagi Digarap, Ini Bocorannya</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Tue, 13 Oct 2026 17:17:31 +0700</t>
+          <t>Tue, 13 Oct 2026 19:23:38 +0700</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/11/10/wakil-menteri-perindustrian-wamenperin-faisol-riza-1762753557434_169.jpeg?w=360&amp;amp;q=90" /&gt; Wamenperin Faisol Riza menyoroti penghentian proyek data center Jatiluhur oleh Gubernur Jabar. Ia menekankan pentingnya investasi untuk </t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2021/09/15/driver-ojol-saat-antar-makanan-2_169.jpeg?w=360&amp;amp;q=90" /&gt; Kementerian Komunikasi dan Digital (Komdigi) menyelesaikan aturan turunan dari Peraturan Presiden (Perpres) No. 27 tahun 2026 tentang layanan ojek online.</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/industri/d-8705308/wamenperin-soal-proyek-data-center-jatiluhur-disetop-kdm-itu-investasi-besar</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8705522/aturan-tarif-ojol-antar-barang-makanan-lagi-digarap-ini-bocorannya</t>
         </is>
       </c>
     </row>
@@ -2154,22 +2130,22 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>KPK Amankan 14 Orang dari OTT BNPB, Sestama Ikut Diciduk</t>
+          <t>Kasus Penganiayaan Aktivis BEM UI, Polisi Periksa 7 Saksi dan 26 CCTV</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Tue, 13 Oct 2026 22:42:03 +0700</t>
+          <t>Wed, 14 Oct 2026 06:19:55 +0700</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Salah satu pihak yang diamankan dalam OTT adalah Sekretaris Utama (Sestama) BNPB, Dr. apt. Rustian.</t>
+          <t>Penanganan perkara tersebut telah ditingkatkan dari tahap penyelidikan ke tahap penyidikan.</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8312529/kpk-amankan-14-orang-dari-ott-bnpb-sestama-ikut-diciduk</t>
+          <t>https://www.liputan6.com/news/read/8312591/kasus-penganiayaan-aktivis-bem-ui-polisi-periksa-7-saksi-dan-26-cctv</t>
         </is>
       </c>
     </row>
@@ -2181,22 +2157,22 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>KPK Sita Rp 1,4 M dan Emas dalam OTT di BNPB</t>
+          <t>Eks Pejabat Polres Jakarta Pusat Diputus Langgar Etik Gara-Gara Hal Ini</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Tue, 13 Oct 2026 22:37:59 +0700</t>
+          <t>Wed, 14 Oct 2026 06:09:05 +0700</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Sebanyak 14 orang, termasuk Sestama BNPB dan sejumlah pihak swasta, diamankan dalam OTT KPK</t>
+          <t>Pamen tersebut kini dalam penempatan pada tempat khusus.</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8312525/kpk-sita-rp-14-m-dan-emas-dalam-ott-di-bnpb</t>
+          <t>https://www.liputan6.com/news/read/8312590/eks-pejabat-polres-jakarta-pusat-diputus-langgar-etik-gara-gara-hal-ini</t>
         </is>
       </c>
     </row>
@@ -2208,22 +2184,22 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Lapak di Kampung Ambon Dibongkar, Polisi Buru Pemiliknya</t>
+          <t>Geger OTT Pejabat BNPB saat Indonesia Terkepung Kebakaran Hutan</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Tue, 13 Oct 2026 22:02:13 +0700</t>
+          <t>Wed, 14 Oct 2026 06:00:47 +0700</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Pembongkaran lapak di Kampung Ambon mengungkap temuan alat isap sabu dan sisa narkoba.</t>
+          <t>Penyelidikan sementara mengarah pada dugaan korupsi pengadaan barang dan jasa, termasuk menggunakan dana siap pakai untuk penanganan bencana.</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8312514/lapak-di-kampung-ambon-dibongkar-polisi-buru-pemiliknya</t>
+          <t>https://www.liputan6.com/news/read/8312561/geger-ott-pejabat-bnpb-saat-indonesia-terkepung-kebakaran-hutan</t>
         </is>
       </c>
     </row>
@@ -2235,22 +2211,22 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Guru Besar UGM Ungkap Masalah Pancasila dalam Praktik Bernegara</t>
+          <t>Cerita Miris di Tengah Kabut Asap Kebakaran Hutan</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Tue, 13 Oct 2026 22:00:37 +0700</t>
+          <t>Wed, 14 Oct 2026 05:05:05 +0700</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Guru Besar UGM Zainal Arifin Muchtar menilai Pancasila semestinya menjadi alat kontrol kekuasaan, bukan sekadar pembenar kebijakan penguasa.</t>
+          <t>Dampak kebakaran hutan meluas dari gangguan kesehatan hingga satwa liar yang kehilangan habitatnya.</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8312422/guru-besar-ugm-ungkap-masalah-pancasila-dalam-praktik-bernegara</t>
+          <t>https://www.liputan6.com/news/read/8312576/cerita-miris-di-tengah-kabut-asap-kebakaran-hutan</t>
         </is>
       </c>
     </row>
@@ -2262,22 +2238,22 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Pramono Pilih Dialog dalam Kasus Bentrokan Satpol PP di Bulungan</t>
+          <t>Jejak Karier Rustian, Pejabat BNPB yang Diamankan dalam OTT KPK</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Tue, 13 Oct 2026 21:47:02 +0700</t>
+          <t>Tue, 13 Oct 2026 23:55:22 +0700</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Gubernur DKI Jakarta Pramono Anung memilih penyelesaian melalui dialog dan musyawarah dalam kasus bentrokan anggota Satpol PP</t>
+          <t>Sebelum diamankan KPK, Rustian pernah menduduki sejumlah jabatan strategis di BNPB, termasuk di bidang penanganan sumber daya darurat.</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8312506/pramono-pilih-dialog-dalam-kasus-bentrokan-satpol-pp-di-bulungan</t>
+          <t>https://www.liputan6.com/news/read/8312546/jejak-karier-rustian-pejabat-bnpb-yang-diamankan-dalam-ott-kpk</t>
         </is>
       </c>
     </row>
@@ -2289,22 +2265,22 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Gudang Paralon di Tangerang Kebakaran</t>
+          <t>OTT Pejabat BNPB Terkait Dana Siap Pakai untuk Kebencanaan</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Tue, 13 Oct 2026 20:55:59 +0700</t>
+          <t>Tue, 13 Oct 2026 23:11:42 +0700</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Proses pemadaman sempat terkendala akibat sulitnya mendapatkan sumber air dan kemacetan parah di sekitar lokasi.</t>
+          <t>Sebanyak 14 orang diamankan Komisi Pemberantasan Korupsi (KPK) dalam operasi tangkap tangan (OTT) di lingkungan Badan Nasional Penanggulangan Bencana (BNPB).</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8312474/gudang-paralon-di-tangerang-kebakaran</t>
+          <t>https://www.liputan6.com/news/read/8312543/ott-pejabat-bnpb-terkait-dana-siap-pakai-untuk-kebencanaan</t>
         </is>
       </c>
     </row>
@@ -2316,22 +2292,22 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Kabar OTT KPK di Kantor BNPB, Begini Tanggapan Pegawai</t>
+          <t>Kapolri Kembali Rombak Jabatan Pati dan Pamen</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Tue, 13 Oct 2026 20:47:05 +0700</t>
+          <t>Tue, 13 Oct 2026 22:55:21 +0700</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>BNPB Sebut Tak Ada OTT KPK di Kantor</t>
+          <t>Mutasi Polri berdasarkan surat telegram tertanggal 12 Oktober 2026 mencakup sejumlah posisi strategis.</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8312467/kabar-ott-kpk-di-kantor-bnpb-begini-tanggapan-pegawai</t>
+          <t>https://www.liputan6.com/news/read/8312531/kapolri-kembali-rombak-jabatan-pati-dan-pamen</t>
         </is>
       </c>
     </row>
@@ -2343,22 +2319,22 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Denny Indrayana Bakal Laporkan Dugaan Pasal Selundupan ke DKPP</t>
+          <t>KPK Amankan 14 Orang dari OTT BNPB, Sestama Ikut Diciduk</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Tue, 13 Oct 2026 20:46:40 +0700</t>
+          <t>Tue, 13 Oct 2026 23:11:49 +0700</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Denny Indrayana menduga ada persoalan etik dalam penyusunan aturan syarat pendidikan capres-cawapres yang dikaitkan dengan pencalonan Gibran.</t>
+          <t>Salah satu pihak yang diamankan dalam OTT adalah Sekretaris Utama (Sestama) BNPB, Dr. apt. Rustian.</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8312458/denny-indrayana-bakal-laporkan-dugaan-pasal-selundupan-ke-dkpp</t>
+          <t>https://www.liputan6.com/news/read/8312529/kpk-amankan-14-orang-dari-ott-bnpb-sestama-ikut-diciduk</t>
         </is>
       </c>
     </row>
@@ -2370,22 +2346,22 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Gandeng Polda Metro Jaya, Pramono Siap Tertibkan Kampung Ambon</t>
+          <t>KPK Sita Rp 1,4 M dan Emas dalam OTT di BNPB</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Tue, 13 Oct 2026 20:08:32 +0700</t>
+          <t>Tue, 13 Oct 2026 23:11:57 +0700</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Pemprov DKI akan bersinergi dengan Polda Metro Jaya untuk menertibkan sejumlah kawasan yang menjadi sarang peredaran narkoba.</t>
+          <t>Sebanyak 14 orang, termasuk Sestama BNPB dan sejumlah pihak swasta, diamankan dalam OTT KPK</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8312451/gandeng-polda-metro-jaya-pramono-siap-tertibkan-kampung-ambon</t>
+          <t>https://www.liputan6.com/news/read/8312525/kpk-sita-rp-14-m-dan-emas-dalam-ott-di-bnpb</t>
         </is>
       </c>
     </row>
@@ -2397,22 +2373,22 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Polisi Ungkap Dugaan Peredaran Catridge Mengandung Etomidate</t>
+          <t>Lapak di Kampung Ambon Dibongkar, Polisi Buru Pemiliknya</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Tue, 13 Oct 2026 20:02:06 +0700</t>
+          <t>Tue, 13 Oct 2026 22:02:13 +0700</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Polisi mengembangkan penyelidikan ke rumah tersangka, menemukan 30 catridge yang diduga mengandung etomidate.</t>
+          <t>Pembongkaran lapak di Kampung Ambon mengungkap temuan alat isap sabu dan sisa narkoba.</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8312444/polisi-ungkap-dugaan-peredaran-catridge-mengandung-etomidate</t>
+          <t>https://www.liputan6.com/news/read/8312514/lapak-di-kampung-ambon-dibongkar-polisi-buru-pemiliknya</t>
         </is>
       </c>
     </row>
@@ -2424,22 +2400,22 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Tiga Embung dan Waduk Ini Disiapkan untuk Tekan Banjir Jakarta</t>
+          <t>Guru Besar UGM Ungkap Masalah Pancasila dalam Praktik Bernegara</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Tue, 13 Oct 2026 19:45:00 +0700</t>
+          <t>Tue, 13 Oct 2026 22:00:37 +0700</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Pembangunan ini disebutkan untuk mengurangi dampak banjir di Jakarta Selatan dan Timur.</t>
+          <t>Guru Besar UGM Zainal Arifin Muchtar menilai Pancasila semestinya menjadi alat kontrol kekuasaan, bukan sekadar pembenar kebijakan penguasa.</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8312439/tiga-embung-dan-waduk-ini-disiapkan-untuk-tekan-banjir-jakarta</t>
+          <t>https://www.liputan6.com/news/read/8312422/guru-besar-ugm-ungkap-masalah-pancasila-dalam-praktik-bernegara</t>
         </is>
       </c>
     </row>
@@ -2451,22 +2427,22 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>YPP Emtek Salurkan Bantuan dan Layanan Kesehatan untuk Penyintas Gempa Flores</t>
+          <t>Pramono Pilih Dialog dalam Kasus Bentrokan Satpol PP di Bulungan</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Tue, 13 Oct 2026 19:38:25 +0700</t>
+          <t>Tue, 13 Oct 2026 21:47:02 +0700</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>YPP Emtek Media menyalurkan bantuan kebutuhan pokok, layanan kesehatan gratis, dan pendampingan psikososial.</t>
+          <t>Gubernur DKI Jakarta Pramono Anung memilih penyelesaian melalui dialog dan musyawarah dalam kasus bentrokan anggota Satpol PP</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8312437/ypp-emtek-salurkan-bantuan-dan-layanan-kesehatan-untuk-penyintas-gempa-flores</t>
+          <t>https://www.liputan6.com/news/read/8312506/pramono-pilih-dialog-dalam-kasus-bentrokan-satpol-pp-di-bulungan</t>
         </is>
       </c>
     </row>
@@ -2478,22 +2454,22 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>KPK OTT di BNPB</t>
+          <t>Gudang Paralon di Tangerang Kebakaran</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Tue, 13 Oct 2026 19:18:48 +0700</t>
+          <t>Tue, 13 Oct 2026 20:55:59 +0700</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Ketua KPK mengonfirmasi OTT di BNPB.</t>
+          <t>Proses pemadaman sempat terkendala akibat sulitnya mendapatkan sumber air dan kemacetan parah di sekitar lokasi.</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8312425/kpk-ott-di-bnpb</t>
+          <t>https://www.liputan6.com/news/read/8312474/gudang-paralon-di-tangerang-kebakaran</t>
         </is>
       </c>
     </row>
@@ -2505,22 +2481,22 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Kasus Penyerangan Koorbid BEM UI Naik ke Penyidikan, 26 Titik CCTV Ditelusuri</t>
+          <t>Kabar OTT KPK di Kantor BNPB, Begini Tanggapan Pegawai</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Tue, 13 Oct 2026 19:22:51 +0700</t>
+          <t>Tue, 13 Oct 2026 23:13:28 +0700</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Penyidik SPolda Metro Jaya menelusuri sekitar 26 titik CCTV dan mengamankan sejumlah barang bukti.</t>
+          <t>Ketua KPK Setyo Budiyanto membenarkan adanya kegiatan yang dilakukan pegawai KPK di lapangan.</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8312420/kasus-penyerangan-koorbid-bem-ui-naik-ke-penyidikan-26-titik-cctv-ditelusuri</t>
+          <t>https://www.liputan6.com/news/read/8312467/kabar-ott-kpk-di-kantor-bnpb-begini-tanggapan-pegawai</t>
         </is>
       </c>
     </row>
@@ -2532,22 +2508,22 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>KPK Sita Land Cruiser Orang Dekat Nusron Wahid di Kasus HGB Summarecon</t>
+          <t>Denny Indrayana Bakal Laporkan Dugaan Pasal Selundupan ke DKPP</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Tue, 13 Oct 2026 18:59:33 +0700</t>
+          <t>Tue, 13 Oct 2026 20:46:40 +0700</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>KPK menyita Toyota Land Cruiser milik tersangka kasus suap HGB Summarecon yang diduga digunakan untuk aktivitas pengumpulan uang.</t>
+          <t>Denny Indrayana menduga ada persoalan etik dalam penyusunan aturan syarat pendidikan capres-cawapres yang dikaitkan dengan pencalonan Gibran.</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8312406/kpk-sita-land-cruiser-orang-dekat-nusron-wahid-di-kasus-hgb-summarecon</t>
+          <t>https://www.liputan6.com/news/read/8312458/denny-indrayana-bakal-laporkan-dugaan-pasal-selundupan-ke-dkpp</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data pasar & berita - 2026-10-14 13:31 UTC
</commit_message>
<xml_diff>
--- a/data/market_news_latest.xlsx
+++ b/data/market_news_latest.xlsx
@@ -422,7 +422,7 @@
     <col width="26" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
   </cols>
@@ -487,20 +487,20 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>5936.147</v>
+        <v>5943.0239</v>
       </c>
       <c r="F2" t="n">
-        <v>-157.6118</v>
+        <v>17.0479</v>
       </c>
       <c r="G2" t="n">
-        <v>-2.59</v>
+        <v>0.29</v>
       </c>
       <c r="H2" t="n">
-        <v>559257300</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -521,20 +521,20 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>7805.4502</v>
+        <v>7771.8501</v>
       </c>
       <c r="F3" t="n">
-        <v>-1.79</v>
+        <v>-33.6001</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.02</v>
+        <v>-0.43</v>
       </c>
       <c r="H3" t="n">
-        <v>2640232000</v>
+        <v>87658820</v>
       </c>
     </row>
     <row r="4">
@@ -555,20 +555,20 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>51670.1016</v>
+        <v>51614.9688</v>
       </c>
       <c r="F4" t="n">
-        <v>-180.4492</v>
+        <v>-55.1328</v>
       </c>
       <c r="G4" t="n">
-        <v>-0.35</v>
+        <v>-0.11</v>
       </c>
       <c r="H4" t="n">
-        <v>395694761</v>
+        <v>15483932</v>
       </c>
     </row>
     <row r="5">
@@ -589,20 +589,20 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>27204.3809</v>
+        <v>27038.3027</v>
       </c>
       <c r="F5" t="n">
-        <v>-41.5195</v>
+        <v>-166.0781</v>
       </c>
       <c r="G5" t="n">
-        <v>-0.15</v>
+        <v>-0.61</v>
       </c>
       <c r="H5" t="n">
-        <v>6273913000</v>
+        <v>788159250</v>
       </c>
     </row>
     <row r="6">
@@ -627,13 +627,13 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>67943.1094</v>
+        <v>67744.28909999999</v>
       </c>
       <c r="F6" t="n">
-        <v>-1087.8125</v>
+        <v>-33.2344</v>
       </c>
       <c r="G6" t="n">
-        <v>-1.58</v>
+        <v>-0.05</v>
       </c>
       <c r="H6" t="n">
         <v>0</v>
@@ -657,20 +657,20 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>24271.1992</v>
+        <v>24314.1699</v>
       </c>
       <c r="F7" t="n">
-        <v>59.8496</v>
+        <v>-31.0508</v>
       </c>
       <c r="G7" t="n">
-        <v>0.25</v>
+        <v>-0.13</v>
       </c>
       <c r="H7" t="n">
-        <v>2229800000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -691,14 +691,20 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>3767.2271</v>
+      </c>
+      <c r="F8" t="n">
+        <v>-33.6379</v>
+      </c>
+      <c r="G8" t="n">
+        <v>-0.89</v>
+      </c>
       <c r="H8" t="n">
-        <v>1085950644</v>
+        <v>1646582440</v>
       </c>
     </row>
     <row r="9">
@@ -719,20 +725,20 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>10656.2998</v>
+        <v>10672.0703</v>
       </c>
       <c r="F9" t="n">
-        <v>104.2002</v>
+        <v>21.7705</v>
       </c>
       <c r="G9" t="n">
-        <v>0.99</v>
+        <v>0.2</v>
       </c>
       <c r="H9" t="n">
-        <v>575809000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -753,20 +759,20 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>25277.6797</v>
+        <v>25378.4199</v>
       </c>
       <c r="F10" t="n">
-        <v>190.4102</v>
+        <v>118.5195</v>
       </c>
       <c r="G10" t="n">
-        <v>0.76</v>
+        <v>0.47</v>
       </c>
       <c r="H10" t="n">
-        <v>39349200</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -787,20 +793,20 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>5415.48</v>
+        <v>5423.3301</v>
       </c>
       <c r="F11" t="n">
-        <v>13.5898</v>
+        <v>-7.1699</v>
       </c>
       <c r="G11" t="n">
-        <v>0.25</v>
+        <v>-0.13</v>
       </c>
       <c r="H11" t="n">
-        <v>243072800</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -821,17 +827,17 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>17913</v>
+        <v>17893</v>
       </c>
       <c r="F12" t="n">
-        <v>3</v>
+        <v>-20</v>
       </c>
       <c r="G12" t="n">
-        <v>0.02</v>
+        <v>-0.11</v>
       </c>
       <c r="H12" t="n">
         <v>0</v>
@@ -855,17 +861,17 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>102.173</v>
+        <v>102.873</v>
       </c>
       <c r="F13" t="n">
-        <v>-0.407</v>
+        <v>0.6929999999999999</v>
       </c>
       <c r="G13" t="n">
-        <v>-0.4</v>
+        <v>0.68</v>
       </c>
       <c r="H13" t="n">
         <v>0</v>
@@ -893,13 +899,13 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>158.378</v>
+        <v>158.878</v>
       </c>
       <c r="F14" t="n">
-        <v>-0.142</v>
+        <v>0.358</v>
       </c>
       <c r="G14" t="n">
-        <v>-0.09</v>
+        <v>0.23</v>
       </c>
       <c r="H14" t="n">
         <v>0</v>
@@ -923,17 +929,17 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>0.5217000000000001</v>
+        <v>0.5314</v>
       </c>
       <c r="F15" t="n">
-        <v>-0.0023</v>
+        <v>0.0097</v>
       </c>
       <c r="G15" t="n">
-        <v>-0.44</v>
+        <v>1.86</v>
       </c>
       <c r="H15" t="n">
         <v>0</v>
@@ -957,17 +963,17 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>0.5563</v>
+        <v>0.5621</v>
       </c>
       <c r="F16" t="n">
-        <v>-0.0035</v>
+        <v>0.0058</v>
       </c>
       <c r="G16" t="n">
-        <v>-0.63</v>
+        <v>1.04</v>
       </c>
       <c r="H16" t="n">
         <v>0</v>
@@ -991,17 +997,17 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>0.4057</v>
+        <v>0.4143</v>
       </c>
       <c r="F17" t="n">
-        <v>0.0007</v>
+        <v>0.0086</v>
       </c>
       <c r="G17" t="n">
-        <v>0.17</v>
+        <v>2.12</v>
       </c>
       <c r="H17" t="n">
         <v>0</v>
@@ -1025,14 +1031,20 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>77.785</v>
+      </c>
+      <c r="F18" t="n">
+        <v>-0.585</v>
+      </c>
+      <c r="G18" t="n">
+        <v>-0.75</v>
+      </c>
       <c r="H18" t="n">
-        <v>29149160</v>
+        <v>5088237</v>
       </c>
     </row>
     <row r="19">
@@ -1053,14 +1065,20 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>76.815</v>
+      </c>
+      <c r="F19" t="n">
+        <v>-0.275</v>
+      </c>
+      <c r="G19" t="n">
+        <v>-0.36</v>
+      </c>
       <c r="H19" t="n">
-        <v>60522261</v>
+        <v>1449804</v>
       </c>
     </row>
     <row r="20">
@@ -1081,20 +1099,20 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>4183.8999</v>
+        <v>4105.1001</v>
       </c>
       <c r="F20" t="n">
-        <v>-6.7002</v>
+        <v>-72.19970000000001</v>
       </c>
       <c r="G20" t="n">
-        <v>-0.16</v>
+        <v>-1.73</v>
       </c>
       <c r="H20" t="n">
-        <v>4912</v>
+        <v>109186</v>
       </c>
     </row>
     <row r="21">
@@ -1115,20 +1133,20 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>94.98</v>
+        <v>95.44</v>
       </c>
       <c r="F21" t="n">
-        <v>1.24</v>
+        <v>1.3</v>
       </c>
       <c r="G21" t="n">
-        <v>1.32</v>
+        <v>1.38</v>
       </c>
       <c r="H21" t="n">
-        <v>3997</v>
+        <v>88055</v>
       </c>
     </row>
     <row r="22">
@@ -1149,20 +1167,20 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="E22" t="n">
-        <v>106.58</v>
+        <v>105.65</v>
       </c>
       <c r="F22" t="n">
-        <v>-0.07000000000000001</v>
+        <v>-0.04</v>
       </c>
       <c r="G22" t="n">
-        <v>-0.07000000000000001</v>
+        <v>-0.04</v>
       </c>
       <c r="H22" t="n">
-        <v>404</v>
+        <v>17816</v>
       </c>
     </row>
     <row r="23">
@@ -1183,20 +1201,20 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="E23" t="n">
-        <v>6.7195</v>
+        <v>6.69</v>
       </c>
       <c r="F23" t="n">
-        <v>0.021</v>
+        <v>0.012</v>
       </c>
       <c r="G23" t="n">
-        <v>0.31</v>
+        <v>0.18</v>
       </c>
       <c r="H23" t="n">
-        <v>759</v>
+        <v>22094</v>
       </c>
     </row>
     <row r="24">
@@ -1217,14 +1235,20 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr"/>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr"/>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>64.84999999999999</v>
+      </c>
+      <c r="F24" t="n">
+        <v>-0.89</v>
+      </c>
+      <c r="G24" t="n">
+        <v>-1.35</v>
+      </c>
       <c r="H24" t="n">
-        <v>21414742</v>
+        <v>409003</v>
       </c>
     </row>
     <row r="25">
@@ -1245,17 +1269,17 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="E25" t="n">
-        <v>15.27</v>
+        <v>15.73</v>
       </c>
       <c r="F25" t="n">
-        <v>0.06</v>
+        <v>0.46</v>
       </c>
       <c r="G25" t="n">
-        <v>0.39</v>
+        <v>3.01</v>
       </c>
       <c r="H25" t="n">
         <v>0</v>
@@ -1283,16 +1307,16 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>83618.5938</v>
+        <v>82792.10159999999</v>
       </c>
       <c r="F26" t="n">
-        <v>1856.0312</v>
+        <v>-303.0234</v>
       </c>
       <c r="G26" t="n">
-        <v>2.27</v>
+        <v>-0.36</v>
       </c>
       <c r="H26" t="n">
-        <v>29613316096</v>
+        <v>28195371008</v>
       </c>
     </row>
     <row r="27">
@@ -1313,20 +1337,20 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="E27" t="n">
-        <v>1310</v>
+        <v>1430</v>
       </c>
       <c r="F27" t="n">
-        <v>-35</v>
+        <v>120</v>
       </c>
       <c r="G27" t="n">
-        <v>-2.6</v>
+        <v>9.16</v>
       </c>
       <c r="H27" t="n">
-        <v>80411200</v>
+        <v>182930700</v>
       </c>
     </row>
     <row r="28">
@@ -1347,20 +1371,20 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="E28" t="n">
-        <v>1520</v>
+        <v>1500</v>
       </c>
       <c r="F28" t="n">
-        <v>15</v>
+        <v>-20</v>
       </c>
       <c r="G28" t="n">
-        <v>1</v>
+        <v>-1.32</v>
       </c>
       <c r="H28" t="n">
-        <v>127296000</v>
+        <v>135916800</v>
       </c>
     </row>
     <row r="29">
@@ -1381,20 +1405,20 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="E29" t="n">
         <v>665</v>
       </c>
       <c r="F29" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="G29" t="n">
-        <v>1.53</v>
+        <v>0</v>
       </c>
       <c r="H29" t="n">
-        <v>434856000</v>
+        <v>380902600</v>
       </c>
     </row>
     <row r="30">
@@ -1415,20 +1439,20 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="E30" t="n">
-        <v>2430</v>
+        <v>2320</v>
       </c>
       <c r="F30" t="n">
-        <v>40</v>
+        <v>-110</v>
       </c>
       <c r="G30" t="n">
-        <v>1.67</v>
+        <v>-4.53</v>
       </c>
       <c r="H30" t="n">
-        <v>13220900</v>
+        <v>25909400</v>
       </c>
     </row>
     <row r="31">
@@ -1449,20 +1473,20 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="E31" t="n">
-        <v>4180</v>
+        <v>4120</v>
       </c>
       <c r="F31" t="n">
-        <v>140</v>
+        <v>-60</v>
       </c>
       <c r="G31" t="n">
-        <v>3.47</v>
+        <v>-1.44</v>
       </c>
       <c r="H31" t="n">
-        <v>47740700</v>
+        <v>44581400</v>
       </c>
     </row>
     <row r="32">
@@ -1483,7 +1507,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="E32" t="n">
@@ -1496,7 +1520,7 @@
         <v>0</v>
       </c>
       <c r="H32" t="n">
-        <v>51400500</v>
+        <v>35585800</v>
       </c>
     </row>
     <row r="33">
@@ -1517,20 +1541,20 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="E33" t="n">
-        <v>605</v>
+        <v>595</v>
       </c>
       <c r="F33" t="n">
-        <v>20</v>
+        <v>-10</v>
       </c>
       <c r="G33" t="n">
-        <v>3.42</v>
+        <v>-1.65</v>
       </c>
       <c r="H33" t="n">
-        <v>50719300</v>
+        <v>41452100</v>
       </c>
     </row>
     <row r="34">
@@ -1551,20 +1575,20 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="E34" t="n">
-        <v>3710</v>
+        <v>3620</v>
       </c>
       <c r="F34" t="n">
-        <v>130</v>
+        <v>-90</v>
       </c>
       <c r="G34" t="n">
-        <v>3.63</v>
+        <v>-2.43</v>
       </c>
       <c r="H34" t="n">
-        <v>3833300</v>
+        <v>1895800</v>
       </c>
     </row>
     <row r="35">
@@ -1585,20 +1609,20 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="E35" t="n">
-        <v>522</v>
+        <v>520</v>
       </c>
       <c r="F35" t="n">
-        <v>-53</v>
+        <v>-2</v>
       </c>
       <c r="G35" t="n">
-        <v>-9.220000000000001</v>
+        <v>-0.38</v>
       </c>
       <c r="H35" t="n">
-        <v>76832806</v>
+        <v>119209400</v>
       </c>
     </row>
     <row r="36">
@@ -1619,20 +1643,20 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="E36" t="n">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="F36" t="n">
-        <v>4</v>
+        <v>-4</v>
       </c>
       <c r="G36" t="n">
-        <v>2.05</v>
+        <v>-2.01</v>
       </c>
       <c r="H36" t="n">
-        <v>18782500</v>
+        <v>14683300</v>
       </c>
     </row>
     <row r="37">
@@ -1653,20 +1677,20 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="E37" t="n">
-        <v>14250</v>
+        <v>14550</v>
       </c>
       <c r="F37" t="n">
-        <v>550</v>
+        <v>300</v>
       </c>
       <c r="G37" t="n">
-        <v>4.01</v>
+        <v>2.11</v>
       </c>
       <c r="H37" t="n">
-        <v>11233300</v>
+        <v>10912400</v>
       </c>
     </row>
   </sheetData>
@@ -1725,22 +1749,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Bukan UMP Naik, Bos Buruh Ungkap Biang Kerok Pabrik Tutup</t>
+          <t>Danantara Indonesia Tegaskan Komitmen Peningkatan Layanan PLN</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Wed, 14 Oct 2026 07:00:03 +0700</t>
+          <t>Wed, 14 Oct 2026 20:24:45 +0700</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2021/02/23/ilustrasi-uang_169.jpeg?w=360&amp;amp;q=90" /&gt; Kenaikan upah minimum provinsi (UMP) dinilai bukan biang kerok beberapa pabrik di Indonesia tutup, menurut Presiden KSPI Said Iqbal.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/06/26/dony-oskaria-1782464979898.jpeg?w=360&amp;amp;q=90" /&gt; Danantara Indonesia berkomitmen meningkatkan layanan PLN, khususnya di Batam, untuk keandalan pasokan listrik dan respons terhadap kebutuhan pelanggan.</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8705738/bukan-ump-naik-bos-buruh-ungkap-biang-kerok-pabrik-tutup</t>
+          <t>https://finance.detik.com/energi/d-8707372/danantara-indonesia-tegaskan-komitmen-peningkatan-layanan-pln</t>
         </is>
       </c>
     </row>
@@ -1752,22 +1776,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Bank Dunia &amp;amp; IMF Wanti-wanti Dampak Buruk AI</t>
+          <t>Darmawan Prasodjo Dicopot dari Dirut PLN, Ini Penggantinya</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Wed, 14 Oct 2026 06:30:15 +0700</t>
+          <t>Wed, 14 Oct 2026 20:00:30 +0700</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/30/ai-openai-1790740749134_169.jpeg?w=360&amp;amp;q=90" /&gt; IMF dan Bank Dunia memperingatkan dampak buruk artificial intelligence alias AI terhadap lapangan pekerjaan.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2022/07/22/kantor-pln-1_169.jpeg?w=360&amp;amp;q=90" /&gt; Darmawan Prasodjo dicopot dari posisi Direktur Utama PT PLN (Persero).</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8705734/bank-dunia-imf-wanti-wanti-dampak-buruk-ai</t>
+          <t>https://finance.detik.com/energi/d-8707339/darmawan-prasodjo-dicopot-dari-dirut-pln-ini-penggantinya</t>
         </is>
       </c>
     </row>
@@ -1779,22 +1803,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Heboh Rumor Emiten Bakrie Caplok Tambang Kideco Rp 17,9 Triliun</t>
+          <t>BBM di Bali Langka Picu Antrean Panjang, Bahlil: Dirut Pertamina Sudah di Sana</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Wed, 14 Oct 2026 05:55:45 +0700</t>
+          <t>Wed, 14 Oct 2026 19:47:02 +0700</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/12/menembus-perut-bumi-mahasiswa-belajar-di-tambang-tua-sawahlunto-1791790427682_169.jpeg?w=360&amp;amp;q=90" /&gt; PT Bumi Resources Tbk (BUMI) disebut akan mengakuisisi tambang batu bara termal milik PT Indika Energy Tbk (INDY), Kideco J</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/11/18/antrean-kendaraan-di-salah-satu-spbu-di-kuta-selatan-badung-bali-selasa-18112025-foto-fabiola-dianiradetikbali-1763454407219_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Koordinator Hilirisasi dan Transisi Energi sekaligus Menteri ESDM Ba</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/bursa-dan-valas/d-8705731/heboh-rumor-emiten-bakrie-caplok-tambang-kideco-rp-17-9-triliun</t>
+          <t>https://finance.detik.com/energi/d-8707324/bbm-di-bali-langka-picu-antrean-panjang-bahlil-dirut-pertamina-sudah-di-sana</t>
         </is>
       </c>
     </row>
@@ -1806,22 +1830,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Perpres Ojol Terbit, Pengemudi Masih Keluhkan Potongan dan Tarif Jarak</t>
+          <t>Mendag Pede Harga Pangan Turun di Akhir Tahun, Ini Alasannya</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Wed, 14 Oct 2026 05:50:03 +0700</t>
+          <t>Wed, 14 Oct 2026 19:30:01 +0700</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/13/perpres-ojol-terbit-pengemudi-masih-keluhkan-potongan-dan-tarif-jarak-1791896085197.jpeg?w=360&amp;amp;q=90" /&gt; Pemerintah membatasi potongan biaya platform ojol maksimal 8% lewat Perpres 27/2026. Namun, pengemudi masih mengeluhkan p</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/14/menteri-perdagangan-mendag-budi-santoso-1791961572700_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Perdagangan (Mendag) Budi Santoso optimistis harga pangan berangsur turun menjelang akhir tahun.</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/foto-bisnis/d-8705570/perpres-ojol-terbit-pengemudi-masih-keluhkan-potongan-dan-tarif-jarak</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8707220/mendag-pede-harga-pangan-turun-di-akhir-tahun-ini-alasannya</t>
         </is>
       </c>
     </row>
@@ -1833,22 +1857,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Transformasi PERURI, Jaga Warisan &amp;amp; Bangun Masa Depan Digital</t>
+          <t>Bahlil Ungkap Biang Kerok Listrik Padam di Batam: Petir hingga Kelelawar</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Wed, 14 Oct 2026 00:00:00 +0700</t>
+          <t>Wed, 14 Oct 2026 19:16:02 +0700</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/13/adv-peruri-1791887140082.png?w=360&amp;amp;q=90" /&gt; Selama puluhan tahun, PERURI memiliki peran dalam kehidupan masyarakat mulai dari bertransaksi menggunakan uang rupiah, menggunakan paspor saat bepergian</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/04/28/menteri-esdm-bahlil-lahadalia-1777385212721_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Koordinator Bidang Hilirisasi dan Transisi Energi sekaligus Menteri ESDM Bahlil Lahadalia buka suara soal listrik padam di Batam</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/advertorial-news-block/d-8705335/transformasi-peruri-jaga-warisan-bangun-masa-depan-digital</t>
+          <t>https://finance.detik.com/energi/d-8707278/bahlil-ungkap-biang-kerok-listrik-padam-di-batam-petir-hingga-kelelawar</t>
         </is>
       </c>
     </row>
@@ -1860,22 +1884,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Mau Kelola Pajak dengan Lebih Terarah? Yuk, Pelajari Dasarnya!</t>
+          <t>Mendag Harap Tak Ada Impor KRL Bekas Jepang, Minta Pakai Produk RI</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Tue, 13 Oct 2026 23:30:30 +0700</t>
+          <t>Wed, 14 Oct 2026 19:00:14 +0700</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/07/28/smart-class-brevet-pajak-a-b-1785248368520_169.png?w=360&amp;amp;q=90" /&gt; Piranha Smart Center (PSC) bersama Education Visionary Lab (EVL) menghadirkan Professional Smart Class: Pelatihan Brevet Pajak AB + Sertifikasi CTT dan CCP.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/14/menteri-perdagangan-mendag-budi-santoso-1791961572700_169.jpeg?w=360&amp;amp;q=90" /&gt; Kalau kami sih berharapnya ya produksi dalam negeri kan sudah ada. Jadi, saya berharap tidak ada impor bekas ya, kata Budi.</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8705696/mau-kelola-pajak-dengan-lebih-terarah-yuk-pelajari-dasarnya</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8707212/mendag-harap-tak-ada-impor-krl-bekas-jepang-minta-pakai-produk-ri</t>
         </is>
       </c>
     </row>
@@ -1887,22 +1911,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Ingin Lebih Siap Jadi Auditor? Kenali Proses Audit Digital Lewat Pelatihan Ini</t>
+          <t>Beredar Kabar Prabowo Cari Menteri ESDM Baru, Bahlil Buka Suara</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Tue, 13 Oct 2026 22:45:52 +0700</t>
+          <t>Wed, 14 Oct 2026 18:32:39 +0700</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/13/detikevent-authen-1791906268082_169.jpeg?w=360&amp;amp;q=90" /&gt; Peserta akan mengikuti demonstrasi penggunaan platform AUTHEN, praktik berbasis studi kasus, diskusi interaktif, serta pendampingan mentor.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/16/menteri-esdm-bahlil-lahadalia-1789550049461_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Koordinator (Menko) Hilirisasi dan Transisi Energi Bahlil Lahadalia buka suara soal kabar bakal ada penggantinya sebagai Menteri ESDM.</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8705759/ingin-lebih-siap-jadi-auditor-kenali-proses-audit-digital-lewat-pelatihan-ini</t>
+          <t>https://finance.detik.com/energi/d-8707174/beredar-kabar-prabowo-cari-menteri-esdm-baru-bahlil-buka-suara</t>
         </is>
       </c>
     </row>
@@ -1914,22 +1938,22 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>BTPN Syariah (BTPS) Bakal Buyback Saham hingga Rp 1 Triliun</t>
+          <t>Usai Listrik Padam di Batam, Prabowo Minta Danantara Evaluasi PLN</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Tue, 13 Oct 2026 22:35:02 +0700</t>
+          <t>Wed, 14 Oct 2026 18:14:42 +0700</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/13/rupslb-btpn-syariah-1791905594130_169.jpeg?w=360&amp;amp;q=90" /&gt; PT Bank BTPN Syariah Tbk mengajukan rencana aksi korporasi pembelian kembali saham (buyback) dengan nilai maksimal hingga Rp1 triliun</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/13/presiden-prabowo-subianto-1791858890986_169.jpeg?w=360&amp;amp;q=90" /&gt; Presiden Prabowo perintahkan Danantara untuk percepat transformasi PLN. Fokus pada efisiensi dan penggunaan 100 GW pembangkit tenaga surya.</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/bursa-dan-valas/d-8705745/btpn-syariah-btps-bakal-buyback-saham-hingga-rp-1-triliun</t>
+          <t>https://finance.detik.com/energi/d-8707137/usai-listrik-padam-di-batam-prabowo-minta-danantara-evaluasi-pln</t>
         </is>
       </c>
     </row>
@@ -1941,22 +1965,22 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Zero ODOL Bisa Gagal Jika Cuma Tertibkan Truk, Ini Saran buat Pemerintah</t>
+          <t>Bahlil Targetkan Ekspor Nikel Naik Jadi Rp 805,5 T</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Tue, 13 Oct 2026 22:30:00 +0700</t>
+          <t>Wed, 14 Oct 2026 17:31:37 +0700</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/06/19/kepadatan-lalu-lintas-di-jalan-raya-wonokromo-surabaya-imbas-demo-sopir-truk-toal-aturan-odol-1750328242861_169.jpeg?w=360&amp;amp;q=90" /&gt; Pemerintah akan menerapkan Zero Over Dimension Overloading (ODOL) pada 2027.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/04/28/menteri-esdm-bahlil-lahadalia-1777385212721_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Koordinator Bidang Hilirisasi dan Transisi Energi sekaligus Menteri ESDM Bahlil Lahadalia menargetkan ekspor nikel US$ 45 miliar atau Rp 805,5 triliu</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8705733/zero-odol-bisa-gagal-jika-cuma-tertibkan-truk-ini-saran-buat-pemerintah</t>
+          <t>https://finance.detik.com/energi/d-8707056/bahlil-targetkan-ekspor-nikel-naik-jadi-rp-805-5-t</t>
         </is>
       </c>
     </row>
@@ -1968,22 +1992,22 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Panen Melimpah, Harga Garam Petani Takalar Turun Tajam</t>
+          <t>UMKM Lokal Mulai Bidik Pasar Dunia, Ini Bekal yang Disiapkan</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Tue, 13 Oct 2026 22:00:16 +0700</t>
+          <t>Wed, 14 Oct 2026 17:17:59 +0700</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/13/harga-garam-turun-di-kabupaten-takalar-1791872493195_169.jpeg?w=360&amp;amp;q=90" /&gt; Harga garam di Takalar anjlok dari Rp150 ribu menjadi Rp45 ribu per karung akibat panen melimpah saat kemarau. Petani berharap bantuan gudang.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/14/umkm-1791976666028_169.jpeg?w=360&amp;amp;q=90" /&gt; UMKM binaan Pertamina bersiap menembus pasar internasional melalui Trade Expo Indonesia 2026. Pelatihan ekspor dan promosi digelar untuk mempersiapkan mereka.</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/foto-bisnis/d-8704804/panen-melimpah-harga-garam-petani-takalar-turun-tajam</t>
+          <t>https://finance.detik.com/solusiukm/d-8707144/umkm-lokal-mulai-bidik-pasar-dunia-ini-bekal-yang-disiapkan</t>
         </is>
       </c>
     </row>
@@ -1995,22 +2019,22 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Mau Jago Hitung Pajak, Tapi Bingung Mulai dari Mana? Coba Kursus di Sini!</t>
+          <t>Pemerintah Mau Transfer Langsung Duit Pensiun PNS, Taspen Ingatkan Ini</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Tue, 13 Oct 2026 21:40:18 +0700</t>
+          <t>Wed, 14 Oct 2026 16:54:01 +0700</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/07/28/smart-class-brevet-pajak-a-b-1785248368520_169.png?w=360&amp;amp;q=90" /&gt; i fokus Pelatihan Brevet Pajak AB + Sertifikasi CTT dan CCP dari Piranha Smart Center (PSC) bersama Education Visionary Lab (EVL).</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/02/12/taspen_169.png?w=360&amp;amp;q=90" /&gt; Kementerian Keuangan (Kemenkeu) berencana mengubah mekanisme pembayaran uang pensiun aparatur sipil negara (ASN) dan TNI/Polri pada 2027.</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8705693/mau-jago-hitung-pajak-tapi-bingung-mulai-dari-mana-coba-kursus-di-sini</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8706938/pemerintah-mau-transfer-langsung-duit-pensiun-pns-taspen-ingatkan-ini</t>
         </is>
       </c>
     </row>
@@ -2022,22 +2046,22 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Beli Token &amp;amp; Bayar Tagihan Listrik Bisa di Kopdes Merah Putih</t>
+          <t>IHSG Ditutup Menguat ke 5.943</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Tue, 13 Oct 2026 21:23:38 +0700</t>
+          <t>Wed, 14 Oct 2026 16:19:07 +0700</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/21/kopdes-merah-putih-bersiap-operasional-23-ribu-bangunan-telah-rampung-1789986171319_169.jpeg?w=360&amp;amp;q=90" /&gt; PLN mendukung program Koperasi Desa/Kelurahan Merah Putih atau Kopdes Merah Putih melalui kemitraan layanan pembayara</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2021/11/19/ihsg-ditutup-menguat-3_169.jpeg?w=360&amp;amp;q=90" /&gt; Indeks Harga Saham Gabungan (IHSG) hari ini ditutup di zona hijau. IHSG bergerak dua arah hingga akhirnya ditutup di level 5.900.</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8705683/beli-token-bayar-tagihan-listrik-bisa-di-kopdes-merah-putih</t>
+          <t>https://finance.detik.com/bursa-dan-valas/d-8706823/ihsg-ditutup-menguat-ke-5-943</t>
         </is>
       </c>
     </row>
@@ -2049,22 +2073,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>1.813 Penerbangan Terdampak Karhutla, Mayoritas Gagal Terbang</t>
+          <t>Blibli Raup Pendapatan Neto Rp 14,8 T di Semester I-2026, Tumbuh 55%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Tue, 13 Oct 2026 20:46:22 +0700</t>
+          <t>Wed, 14 Oct 2026 16:09:29 +0700</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/17/kabut-asap-karhutla-ganggu-penerbangan-di-bandara-palembang-1789622375071_169.jpeg?w=360&amp;amp;q=90" /&gt; Kementerian Perhubungan (Kemenhub) mencatat total 1.813 penerbangan terdampak kebakaran hutan dan lahan (karhutla) sejak 11 Agu</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/14/blibli-raup-pendapatan-neto-rp-148-t-di-semester-i-2026-tumbuh-55-1791968919767.png?w=360&amp;amp;q=90" /&gt; Blibli mencatatkan pendapatan neto Rp 14,8 triliun, tumbuh 55% YoY pada semester I 2026, didorong oleh segmen lifestyle dan co</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8705647/1-813-penerbangan-terdampak-karhutla-mayoritas-gagal-terbang</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8706811/blibli-raup-pendapatan-neto-rp-14-8-t-di-semester-i-2026-tumbuh-55</t>
         </is>
       </c>
     </row>
@@ -2076,22 +2100,22 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Menteri LH Ingatkan Pengusaha, Biaya Urus Lingkungan Hidup Bukan Beban!</t>
+          <t>PHE Bor Sumur Eksplorasi di Kaltara, Bidik Cadangan Migas Baru</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Tue, 13 Oct 2026 20:11:54 +0700</t>
+          <t>Wed, 14 Oct 2026 16:09:19 +0700</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/29/menteri-lh-mohammad-jumhur-hidayat-saat-kunjungi-objek-wisata-di-cisarua-1790687703176_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Lingkungan Hidup Mohammad Jumhur Hidayat menegaskan biaya yang dikeluarkan perusahaan dalam pengelolaan li</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/23/pertamina-ep-1790145752075_169.jpeg?w=360&amp;amp;q=90" /&gt; PT Pertamina Hulu Energi memulai pengeboran sumur eksplorasi Tingkilan-001 di Kalimantan Utara untuk uji potensi hidrokarbon.</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8705607/menteri-lh-ingatkan-pengusaha-biaya-urus-lingkungan-hidup-bukan-beban</t>
+          <t>https://finance.detik.com/energi/d-8706800/phe-bor-sumur-eksplorasi-di-kaltara-bidik-cadangan-migas-baru</t>
         </is>
       </c>
     </row>
@@ -2103,22 +2127,22 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Aturan Tarif Ojol Antar Barang &amp;amp; Makanan Lagi Digarap, Ini Bocorannya</t>
+          <t>Bahlil Merapat ke Istana Lapor soal BBM Langka di Bali</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Tue, 13 Oct 2026 19:23:38 +0700</t>
+          <t>Wed, 14 Oct 2026 16:05:25 +0700</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2021/09/15/driver-ojol-saat-antar-makanan-2_169.jpeg?w=360&amp;amp;q=90" /&gt; Kementerian Komunikasi dan Digital (Komdigi) menyelesaikan aturan turunan dari Peraturan Presiden (Perpres) No. 27 tahun 2026 tentang layanan ojek online.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/14/menko-hilirisasi-dan-transisi-energi-bahlil-lahadalia-1791968692833_169.jpeg?w=360&amp;amp;q=90" /&gt; Menko Hilirisasi dan Transisi Energi Bahlil Lahadalia hari ini merapat ke Istana Kepresidenan, Jakarta Pusat.</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8705522/aturan-tarif-ojol-antar-barang-makanan-lagi-digarap-ini-bocorannya</t>
+          <t>https://finance.detik.com/energi/d-8706803/bahlil-merapat-ke-istana-lapor-soal-bbm-langka-di-bali</t>
         </is>
       </c>
     </row>
@@ -2130,22 +2154,22 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Kasus Penganiayaan Aktivis BEM UI, Polisi Periksa 7 Saksi dan 26 CCTV</t>
+          <t>KPK Tahan 5 Tersangka Korupsi BNPB</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Wed, 14 Oct 2026 06:19:55 +0700</t>
+          <t>Wed, 14 Oct 2026 20:21:23 +0700</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Penanganan perkara tersebut telah ditingkatkan dari tahap penyelidikan ke tahap penyidikan.</t>
+          <t>Penahanan dilakukan KPK setelah memeriksa lima tersangka di Gedung Merah Putih sejak Selasa (13/10/2026).</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8312591/kasus-penganiayaan-aktivis-bem-ui-polisi-periksa-7-saksi-dan-26-cctv</t>
+          <t>https://www.liputan6.com/news/read/8313324/kpk-tahan-5-tersangka-korupsi-bnpb</t>
         </is>
       </c>
     </row>
@@ -2157,22 +2181,22 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Eks Pejabat Polres Jakarta Pusat Diputus Langgar Etik Gara-Gara Hal Ini</t>
+          <t>Satgas PRR dan BRIN Pastikan Kesiapan Lokasi Arsinum di Aceh Utara</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Wed, 14 Oct 2026 06:09:05 +0700</t>
+          <t>Wed, 14 Oct 2026 20:16:15 +0700</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Pamen tersebut kini dalam penempatan pada tempat khusus.</t>
+          <t>Instalasi Arsinum yang direncanakan di Aceh Utara memiliki kapasitas pengolahan hingga 10.000 liter per hari.</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8312590/eks-pejabat-polres-jakarta-pusat-diputus-langgar-etik-gara-gara-hal-ini</t>
+          <t>https://www.liputan6.com/news/read/8313322/satgas-prr-dan-brin-pastikan-kesiapan-lokasi-arsinum-di-aceh-utara</t>
         </is>
       </c>
     </row>
@@ -2184,22 +2208,22 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Geger OTT Pejabat BNPB saat Indonesia Terkepung Kebakaran Hutan</t>
+          <t>Blak-blakan Terdakwa Nurman Herin Mengaku Ditekan Jaksa Kasus Febrie</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Wed, 14 Oct 2026 06:00:47 +0700</t>
+          <t>Wed, 14 Oct 2026 19:41:13 +0700</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Penyelidikan sementara mengarah pada dugaan korupsi pengadaan barang dan jasa, termasuk menggunakan dana siap pakai untuk penanganan bencana.</t>
+          <t>Pengakuan itu disampaikan Nurman saat membacakan eksepsi di pengadilan Tipikor Jakarta, Rabu (14/10/2026).</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8312561/geger-ott-pejabat-bnpb-saat-indonesia-terkepung-kebakaran-hutan</t>
+          <t>https://www.liputan6.com/news/read/8313304/blak-blakan-terdakwa-nurman-herin-mengaku-ditekan-jaksa-kasus-febrie</t>
         </is>
       </c>
     </row>
@@ -2211,22 +2235,22 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Cerita Miris di Tengah Kabut Asap Kebakaran Hutan</t>
+          <t>KPK Dalami Peran Adik Kepala BNPB Usai Ditetapkan sebagai Tersangka</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Wed, 14 Oct 2026 05:05:05 +0700</t>
+          <t>Wed, 14 Oct 2026 19:41:04 +0700</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Dampak kebakaran hutan meluas dari gangguan kesehatan hingga satwa liar yang kehilangan habitatnya.</t>
+          <t>KPK menetapkan Bima Setyawan, adik Kepala BNPB Suharyanto, sebagai salah satu dari lima tersangka OTT terkait dugaan penyalahgunaan dana kebencanaan.</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8312576/cerita-miris-di-tengah-kabut-asap-kebakaran-hutan</t>
+          <t>https://www.liputan6.com/news/read/8313300/kpk-dalami-peran-adik-kepala-bnpb-usai-ditetapkan-sebagai-tersangka</t>
         </is>
       </c>
     </row>
@@ -2238,22 +2262,22 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Jejak Karier Rustian, Pejabat BNPB yang Diamankan dalam OTT KPK</t>
+          <t>Berompi Oranye, Begini Penampakan Lima Tersangka Korupsi BNPB</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Tue, 13 Oct 2026 23:55:22 +0700</t>
+          <t>Wed, 14 Oct 2026 19:13:53 +0700</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Sebelum diamankan KPK, Rustian pernah menduduki sejumlah jabatan strategis di BNPB, termasuk di bidang penanganan sumber daya darurat.</t>
+          <t>Salah satu tersangka yang turut dibawa keluar adalah Bima Setyawan, yang disebut merupakan adik Kepala BNPB.</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8312546/jejak-karier-rustian-pejabat-bnpb-yang-diamankan-dalam-ott-kpk</t>
+          <t>https://www.liputan6.com/news/read/8313283/berompi-oranye-begini-penampakan-lima-tersangka-korupsi-bnpb</t>
         </is>
       </c>
     </row>
@@ -2265,22 +2289,22 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>OTT Pejabat BNPB Terkait Dana Siap Pakai untuk Kebencanaan</t>
+          <t>Daftar 12 Wilayah Masuk Zona Berbahaya Imbas Kebakaran Hutan</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Tue, 13 Oct 2026 23:11:42 +0700</t>
+          <t>Wed, 14 Oct 2026 19:08:42 +0700</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Sebanyak 14 orang diamankan Komisi Pemberantasan Korupsi (KPK) dalam operasi tangkap tangan (OTT) di lingkungan Badan Nasional Penanggulangan Bencana (BNPB).</t>
+          <t>Enam dari 12 wilayah tersebut didominasi daerah Kalimantan Tengah.</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8312543/ott-pejabat-bnpb-terkait-dana-siap-pakai-untuk-kebencanaan</t>
+          <t>https://www.liputan6.com/news/read/8313278/daftar-12-wilayah-masuk-zona-berbahaya-imbas-kebakaran-hutan</t>
         </is>
       </c>
     </row>
@@ -2292,22 +2316,22 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Kapolri Kembali Rombak Jabatan Pati dan Pamen</t>
+          <t>BRIN Sebut Pemadaman Saja Tak Cukup Atasi Kebakaran Hutan</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Tue, 13 Oct 2026 22:55:21 +0700</t>
+          <t>Wed, 14 Oct 2026 19:08:54 +0700</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Mutasi Polri berdasarkan surat telegram tertanggal 12 Oktober 2026 mencakup sejumlah posisi strategis.</t>
+          <t>BRIN menyoroti faktor manusia di balik kebakaran yang berulang.</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8312531/kapolri-kembali-rombak-jabatan-pati-dan-pamen</t>
+          <t>https://www.liputan6.com/news/read/8313277/brin-sebut-pemadaman-saja-tak-cukup-atasi-kebakaran-hutan</t>
         </is>
       </c>
     </row>
@@ -2319,22 +2343,22 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>KPK Amankan 14 Orang dari OTT BNPB, Sestama Ikut Diciduk</t>
+          <t>Adik Kepala BNPB Jadi Tersangka Dugaan Korupsi Dana Bencana</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Tue, 13 Oct 2026 23:11:49 +0700</t>
+          <t>Wed, 14 Oct 2026 19:03:13 +0700</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Salah satu pihak yang diamankan dalam OTT adalah Sekretaris Utama (Sestama) BNPB, Dr. apt. Rustian.</t>
+          <t>Lima tersangka OTT KPK di lingkungan BNPB ditahan terkait dugaan penyalahgunaan dana siap pakai kebencanaan. Salah satunya disebut merupakan adik Kepala BNPB Letjen Suharyanto.</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8312529/kpk-amankan-14-orang-dari-ott-bnpb-sestama-ikut-diciduk</t>
+          <t>https://www.liputan6.com/news/read/8313264/adik-kepala-bnpb-jadi-tersangka-dugaan-korupsi-dana-bencana</t>
         </is>
       </c>
     </row>
@@ -2346,22 +2370,22 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>KPK Sita Rp 1,4 M dan Emas dalam OTT di BNPB</t>
+          <t>Gibran: Kritik Pemerintah Harus Dijawab dengan Kerja Lebih Baik</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Tue, 13 Oct 2026 23:11:57 +0700</t>
+          <t>Wed, 14 Oct 2026 18:00:39 +0700</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Sebanyak 14 orang, termasuk Sestama BNPB dan sejumlah pihak swasta, diamankan dalam OTT KPK</t>
+          <t>Gibran Respon Survei Evaluasi 2 Tahun Kinerja Pemerintah: Kritik Dijawab dengan Kerja Nyata</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8312525/kpk-sita-rp-14-m-dan-emas-dalam-ott-di-bnpb</t>
+          <t>https://www.liputan6.com/news/read/8313214/gibran-kritik-pemerintah-harus-dijawab-dengan-kerja-lebih-baik</t>
         </is>
       </c>
     </row>
@@ -2373,22 +2397,22 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Lapak di Kampung Ambon Dibongkar, Polisi Buru Pemiliknya</t>
+          <t>BMKG Prediksi El Nino Bertahan hingga Awal 2027, Musim Hujan Mundur</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Tue, 13 Oct 2026 22:02:13 +0700</t>
+          <t>Wed, 14 Oct 2026 18:31:30 +0700</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Pembongkaran lapak di Kampung Ambon mengungkap temuan alat isap sabu dan sisa narkoba.</t>
+          <t>BMKG mengingatkan potensi banjir, banjir bandang, dan longsor ketika musim hujan tiba di tengah kondisi iklim yang dipengaruhi El Nino.</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8312514/lapak-di-kampung-ambon-dibongkar-polisi-buru-pemiliknya</t>
+          <t>https://www.liputan6.com/news/read/8313215/bmkg-prediksi-el-nino-bertahan-hingga-awal-2027-musim-hujan-mundur</t>
         </is>
       </c>
     </row>
@@ -2400,22 +2424,22 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Guru Besar UGM Ungkap Masalah Pancasila dalam Praktik Bernegara</t>
+          <t>Jakarta Raih Peringkat 117 Kota Pelajar Dunia, Pramono Apresiasi Guru</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Tue, 13 Oct 2026 22:00:37 +0700</t>
+          <t>Wed, 14 Oct 2026 17:23:58 +0700</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Guru Besar UGM Zainal Arifin Muchtar menilai Pancasila semestinya menjadi alat kontrol kekuasaan, bukan sekadar pembenar kebijakan penguasa.</t>
+          <t>Jakarta berada di peringkat ke-117 dunia dalam QS Best Student Cities 2027, satu tingkat di atas Yogyakarta.</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8312422/guru-besar-ugm-ungkap-masalah-pancasila-dalam-praktik-bernegara</t>
+          <t>https://www.liputan6.com/news/read/8313209/jakarta-raih-peringkat-117-kota-pelajar-dunia-pramono-apresiasi-guru</t>
         </is>
       </c>
     </row>
@@ -2427,22 +2451,22 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Pramono Pilih Dialog dalam Kasus Bentrokan Satpol PP di Bulungan</t>
+          <t>Mobil Listrik Terbakar di Tebet, Asap Hitam Membumbung</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Tue, 13 Oct 2026 21:47:02 +0700</t>
+          <t>Wed, 14 Oct 2026 17:00:43 +0700</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Gubernur DKI Jakarta Pramono Anung memilih penyelesaian melalui dialog dan musyawarah dalam kasus bentrokan anggota Satpol PP</t>
+          <t>Mobil listrik terbakar di Tebet, Jakarta Selatan, asap hitam membumbung dari lokasi kejadian.</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8312506/pramono-pilih-dialog-dalam-kasus-bentrokan-satpol-pp-di-bulungan</t>
+          <t>https://www.liputan6.com/news/read/8313179/mobil-listrik-terbakar-di-tebet-asap-hitam-membumbung</t>
         </is>
       </c>
     </row>
@@ -2454,22 +2478,22 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Gudang Paralon di Tangerang Kebakaran</t>
+          <t>513 Hektare Hutan Tanjung Puting Hangus, Api Belum Juga Padam</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Tue, 13 Oct 2026 20:55:59 +0700</t>
+          <t>Wed, 14 Oct 2026 16:40:33 +0700</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Proses pemadaman sempat terkendala akibat sulitnya mendapatkan sumber air dan kemacetan parah di sekitar lokasi.</t>
+          <t>Karhutla di Taman Nasional Tanjung Puting telah membakar sekitar 513 hektare lahan. Ratusan personel tambahan dikerahkan untuk menangani kebakaran.</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8312474/gudang-paralon-di-tangerang-kebakaran</t>
+          <t>https://www.liputan6.com/news/read/8313137/513-hektare-hutan-tanjung-puting-hangus-api-belum-juga-padam</t>
         </is>
       </c>
     </row>
@@ -2481,22 +2505,22 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Kabar OTT KPK di Kantor BNPB, Begini Tanggapan Pegawai</t>
+          <t>KPK Tetapkan Tersangka di Kasus OTT BNPB</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Tue, 13 Oct 2026 23:13:28 +0700</t>
+          <t>Wed, 14 Oct 2026 16:32:20 +0700</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Ketua KPK Setyo Budiyanto membenarkan adanya kegiatan yang dilakukan pegawai KPK di lapangan.</t>
+          <t>Pihak yang telah ditetapkan sebagai tersangka selanjutnya akan menjalani penahanan.</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8312467/kabar-ott-kpk-di-kantor-bnpb-begini-tanggapan-pegawai</t>
+          <t>https://www.liputan6.com/news/read/8313127/kpk-tetapkan-tersangka-di-kasus-ott-bnpb</t>
         </is>
       </c>
     </row>
@@ -2508,22 +2532,22 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Denny Indrayana Bakal Laporkan Dugaan Pasal Selundupan ke DKPP</t>
+          <t>Kubu Febrie Bongkar Peran Ferry Hongkiriwang dalam Kasus Pemerasan</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Tue, 13 Oct 2026 20:46:40 +0700</t>
+          <t>Wed, 14 Oct 2026 16:17:16 +0700</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Denny Indrayana menduga ada persoalan etik dalam penyusunan aturan syarat pendidikan capres-cawapres yang dikaitkan dengan pencalonan Gibran.</t>
+          <t>Kubu Febrie Adriansyah mengungkapkan dalam dakwaan Febrie tidak terdapat perintah kepada Ferry untuk memaksa Tan Kian menyerahkan sejumlah uang.</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8312458/denny-indrayana-bakal-laporkan-dugaan-pasal-selundupan-ke-dkpp</t>
+          <t>https://www.liputan6.com/news/read/8313114/kubu-febrie-bongkar-peran-ferry-hongkiriwang-dalam-kasus-pemerasan</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data pasar & berita - 2026-10-15 00:09 UTC
</commit_message>
<xml_diff>
--- a/data/market_news_latest.xlsx
+++ b/data/market_news_latest.xlsx
@@ -422,7 +422,7 @@
     <col width="26" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
   </cols>
@@ -487,20 +487,20 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>5943.0239</v>
+        <v>5925.9761</v>
       </c>
       <c r="F2" t="n">
-        <v>17.0479</v>
+        <v>-10.1709</v>
       </c>
       <c r="G2" t="n">
-        <v>0.29</v>
+        <v>-0.17</v>
       </c>
       <c r="H2" t="n">
-        <v>0</v>
+        <v>314688200</v>
       </c>
     </row>
     <row r="3">
@@ -525,16 +525,16 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>7771.8501</v>
+        <v>7718.9399</v>
       </c>
       <c r="F3" t="n">
-        <v>-33.6001</v>
+        <v>-86.5103</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.43</v>
+        <v>-1.11</v>
       </c>
       <c r="H3" t="n">
-        <v>87658820</v>
+        <v>3388032000</v>
       </c>
     </row>
     <row r="4">
@@ -559,16 +559,16 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>51614.9688</v>
+        <v>51621.4805</v>
       </c>
       <c r="F4" t="n">
-        <v>-55.1328</v>
+        <v>-48.6211</v>
       </c>
       <c r="G4" t="n">
-        <v>-0.11</v>
+        <v>-0.09</v>
       </c>
       <c r="H4" t="n">
-        <v>15483932</v>
+        <v>442523838</v>
       </c>
     </row>
     <row r="5">
@@ -593,16 +593,16 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>27038.3027</v>
+        <v>26692.8691</v>
       </c>
       <c r="F5" t="n">
-        <v>-166.0781</v>
+        <v>-511.5117</v>
       </c>
       <c r="G5" t="n">
-        <v>-0.61</v>
+        <v>-1.88</v>
       </c>
       <c r="H5" t="n">
-        <v>788159250</v>
+        <v>7640476000</v>
       </c>
     </row>
     <row r="6">
@@ -623,20 +623,20 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>67744.28909999999</v>
+        <v>67777.52340000001</v>
       </c>
       <c r="F6" t="n">
-        <v>-33.2344</v>
+        <v>-1253.3984</v>
       </c>
       <c r="G6" t="n">
-        <v>-0.05</v>
+        <v>-1.82</v>
       </c>
       <c r="H6" t="n">
-        <v>0</v>
+        <v>168000000</v>
       </c>
     </row>
     <row r="7">
@@ -657,20 +657,20 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>24314.1699</v>
+        <v>24345.2207</v>
       </c>
       <c r="F7" t="n">
-        <v>-31.0508</v>
+        <v>74.0215</v>
       </c>
       <c r="G7" t="n">
-        <v>-0.13</v>
+        <v>0.3</v>
       </c>
       <c r="H7" t="n">
-        <v>0</v>
+        <v>2546200000</v>
       </c>
     </row>
     <row r="8">
@@ -694,15 +694,9 @@
           <t>2026-10-14</t>
         </is>
       </c>
-      <c r="E8" t="n">
-        <v>3767.2271</v>
-      </c>
-      <c r="F8" t="n">
-        <v>-33.6379</v>
-      </c>
-      <c r="G8" t="n">
-        <v>-0.89</v>
-      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
       <c r="H8" t="n">
         <v>1646582440</v>
       </c>
@@ -725,20 +719,20 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>10672.0703</v>
+        <v>10650.2998</v>
       </c>
       <c r="F9" t="n">
-        <v>21.7705</v>
+        <v>-6</v>
       </c>
       <c r="G9" t="n">
-        <v>0.2</v>
+        <v>-0.06</v>
       </c>
       <c r="H9" t="n">
-        <v>0</v>
+        <v>670857300</v>
       </c>
     </row>
     <row r="10">
@@ -759,20 +753,20 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>25378.4199</v>
+        <v>25259.9004</v>
       </c>
       <c r="F10" t="n">
-        <v>118.5195</v>
+        <v>-17.7793</v>
       </c>
       <c r="G10" t="n">
-        <v>0.47</v>
+        <v>-0.07000000000000001</v>
       </c>
       <c r="H10" t="n">
-        <v>0</v>
+        <v>48379600</v>
       </c>
     </row>
     <row r="11">
@@ -793,20 +787,20 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>5423.3301</v>
+        <v>5430.5</v>
       </c>
       <c r="F11" t="n">
-        <v>-7.1699</v>
+        <v>15.02</v>
       </c>
       <c r="G11" t="n">
-        <v>-0.13</v>
+        <v>0.28</v>
       </c>
       <c r="H11" t="n">
-        <v>0</v>
+        <v>266038800</v>
       </c>
     </row>
     <row r="12">
@@ -831,13 +825,13 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>17893</v>
+        <v>17866.5</v>
       </c>
       <c r="F12" t="n">
-        <v>-20</v>
+        <v>-46.5</v>
       </c>
       <c r="G12" t="n">
-        <v>-0.11</v>
+        <v>-0.26</v>
       </c>
       <c r="H12" t="n">
         <v>0</v>
@@ -865,13 +859,13 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>102.873</v>
+        <v>102.207</v>
       </c>
       <c r="F13" t="n">
-        <v>0.6929999999999999</v>
+        <v>0.027</v>
       </c>
       <c r="G13" t="n">
-        <v>0.68</v>
+        <v>0.03</v>
       </c>
       <c r="H13" t="n">
         <v>0</v>
@@ -895,17 +889,17 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>158.878</v>
+        <v>157.933</v>
       </c>
       <c r="F14" t="n">
-        <v>0.358</v>
+        <v>-0.389</v>
       </c>
       <c r="G14" t="n">
-        <v>0.23</v>
+        <v>-0.25</v>
       </c>
       <c r="H14" t="n">
         <v>0</v>
@@ -933,13 +927,13 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>0.5314</v>
+        <v>0.519</v>
       </c>
       <c r="F15" t="n">
-        <v>0.0097</v>
+        <v>-0.0027</v>
       </c>
       <c r="G15" t="n">
-        <v>1.86</v>
+        <v>-0.52</v>
       </c>
       <c r="H15" t="n">
         <v>0</v>
@@ -967,13 +961,13 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>0.5621</v>
+        <v>0.5525</v>
       </c>
       <c r="F16" t="n">
-        <v>0.0058</v>
+        <v>-0.0038</v>
       </c>
       <c r="G16" t="n">
-        <v>1.04</v>
+        <v>-0.68</v>
       </c>
       <c r="H16" t="n">
         <v>0</v>
@@ -1001,13 +995,13 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>0.4143</v>
+        <v>0.4085</v>
       </c>
       <c r="F17" t="n">
-        <v>0.0086</v>
+        <v>0.0028</v>
       </c>
       <c r="G17" t="n">
-        <v>2.12</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="H17" t="n">
         <v>0</v>
@@ -1034,17 +1028,11 @@
           <t>2026-10-14</t>
         </is>
       </c>
-      <c r="E18" t="n">
-        <v>77.785</v>
-      </c>
-      <c r="F18" t="n">
-        <v>-0.585</v>
-      </c>
-      <c r="G18" t="n">
-        <v>-0.75</v>
-      </c>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
       <c r="H18" t="n">
-        <v>5088237</v>
+        <v>50953748</v>
       </c>
     </row>
     <row r="19">
@@ -1068,17 +1056,11 @@
           <t>2026-10-14</t>
         </is>
       </c>
-      <c r="E19" t="n">
-        <v>76.815</v>
-      </c>
-      <c r="F19" t="n">
-        <v>-0.275</v>
-      </c>
-      <c r="G19" t="n">
-        <v>-0.36</v>
-      </c>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr"/>
       <c r="H19" t="n">
-        <v>1449804</v>
+        <v>63579674</v>
       </c>
     </row>
     <row r="20">
@@ -1103,16 +1085,16 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>4105.1001</v>
+        <v>4133.1001</v>
       </c>
       <c r="F20" t="n">
-        <v>-72.19970000000001</v>
+        <v>-44.1997</v>
       </c>
       <c r="G20" t="n">
-        <v>-1.73</v>
+        <v>-1.06</v>
       </c>
       <c r="H20" t="n">
-        <v>109186</v>
+        <v>6554</v>
       </c>
     </row>
     <row r="21">
@@ -1137,16 +1119,16 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>95.44</v>
+        <v>94.77</v>
       </c>
       <c r="F21" t="n">
-        <v>1.3</v>
+        <v>0.63</v>
       </c>
       <c r="G21" t="n">
-        <v>1.38</v>
+        <v>0.67</v>
       </c>
       <c r="H21" t="n">
-        <v>88055</v>
+        <v>2481</v>
       </c>
     </row>
     <row r="22">
@@ -1171,16 +1153,16 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>105.65</v>
+        <v>105.63</v>
       </c>
       <c r="F22" t="n">
-        <v>-0.04</v>
+        <v>-0.06</v>
       </c>
       <c r="G22" t="n">
-        <v>-0.04</v>
+        <v>-0.06</v>
       </c>
       <c r="H22" t="n">
-        <v>17816</v>
+        <v>164</v>
       </c>
     </row>
     <row r="23">
@@ -1205,16 +1187,16 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>6.69</v>
+        <v>6.61</v>
       </c>
       <c r="F23" t="n">
-        <v>0.012</v>
+        <v>-0.068</v>
       </c>
       <c r="G23" t="n">
-        <v>0.18</v>
+        <v>-1.02</v>
       </c>
       <c r="H23" t="n">
-        <v>22094</v>
+        <v>754</v>
       </c>
     </row>
     <row r="24">
@@ -1238,17 +1220,11 @@
           <t>2026-10-14</t>
         </is>
       </c>
-      <c r="E24" t="n">
-        <v>64.84999999999999</v>
-      </c>
-      <c r="F24" t="n">
-        <v>-0.89</v>
-      </c>
-      <c r="G24" t="n">
-        <v>-1.35</v>
-      </c>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr"/>
       <c r="H24" t="n">
-        <v>409003</v>
+        <v>21163577</v>
       </c>
     </row>
     <row r="25">
@@ -1273,13 +1249,13 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>15.73</v>
+        <v>16.87</v>
       </c>
       <c r="F25" t="n">
-        <v>0.46</v>
+        <v>1.6</v>
       </c>
       <c r="G25" t="n">
-        <v>3.01</v>
+        <v>10.48</v>
       </c>
       <c r="H25" t="n">
         <v>0</v>
@@ -1303,20 +1279,20 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="E26" t="n">
-        <v>82792.10159999999</v>
+        <v>81650.47659999999</v>
       </c>
       <c r="F26" t="n">
-        <v>-303.0234</v>
+        <v>-1444.6484</v>
       </c>
       <c r="G26" t="n">
-        <v>-0.36</v>
+        <v>-1.74</v>
       </c>
       <c r="H26" t="n">
-        <v>28195371008</v>
+        <v>33361143808</v>
       </c>
     </row>
     <row r="27">
@@ -1749,22 +1725,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Danantara Indonesia Tegaskan Komitmen Peningkatan Layanan PLN</t>
+          <t>Pengganti LPG 3 Kg Mulai Dijual 2027, Tabungnya dari China</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Wed, 14 Oct 2026 20:24:45 +0700</t>
+          <t>Thu, 15 Oct 2026 06:55:00 +0700</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/06/26/dony-oskaria-1782464979898.jpeg?w=360&amp;amp;q=90" /&gt; Danantara Indonesia berkomitmen meningkatkan layanan PLN, khususnya di Batam, untuk keandalan pasokan listrik dan respons terhadap kebutuhan pelanggan.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2021/12/14/cng-gaslink-1_169.jpeg?w=360&amp;amp;q=90" /&gt; Program CNG 3 kg sebagai pengganti LPG akan diluncurkan pada 2027. Uji coba telah dilakukan, dengan 100 ribu tabung dari China siap didistribusikan.</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8707372/danantara-indonesia-tegaskan-komitmen-peningkatan-layanan-pln</t>
+          <t>https://finance.detik.com/energi/d-8707229/pengganti-lpg-3-kg-mulai-dijual-2027-tabungnya-dari-china</t>
         </is>
       </c>
     </row>
@@ -1776,22 +1752,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Darmawan Prasodjo Dicopot dari Dirut PLN, Ini Penggantinya</t>
+          <t>Bos Agrinas soal Ratusan Manajer Kopdes Mundur: Tidak Ada yang Rugi!</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Wed, 14 Oct 2026 20:00:30 +0700</t>
+          <t>Thu, 15 Oct 2026 06:25:00 +0700</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2022/07/22/kantor-pln-1_169.jpeg?w=360&amp;amp;q=90" /&gt; Darmawan Prasodjo dicopot dari posisi Direktur Utama PT PLN (Persero).</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/03/31/direktur-utama-pt-agrinas-pangan-nusantara-joao-angelo-de-sousa-mota-1774938653280_169.jpeg?w=360&amp;amp;q=90" /&gt; Itu kan anak bangsa, tidak ada yang rugi. Kalau saya dibina boleh lah, tegas dia.</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8707339/darmawan-prasodjo-dicopot-dari-dirut-pln-ini-penggantinya</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8706911/bos-agrinas-soal-ratusan-manajer-kopdes-mundur-tidak-ada-yang-rugi</t>
         </is>
       </c>
     </row>
@@ -1803,22 +1779,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>BBM di Bali Langka Picu Antrean Panjang, Bahlil: Dirut Pertamina Sudah di Sana</t>
+          <t>Dirut PLN Diganti di Tengah Masalah Listrik Batam Padam</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Wed, 14 Oct 2026 19:47:02 +0700</t>
+          <t>Thu, 15 Oct 2026 05:55:00 +0700</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/11/18/antrean-kendaraan-di-salah-satu-spbu-di-kuta-selatan-badung-bali-selasa-18112025-foto-fabiola-dianiradetikbali-1763454407219_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Koordinator Hilirisasi dan Transisi Energi sekaligus Menteri ESDM Ba</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2022/07/22/kantor-pln_169.jpeg?w=360&amp;amp;q=90" /&gt; Suroso Isnandar diangkat sebagai Direktur Utama (Dirut) baru PLN. Suroso menggantikan Darmawan Prasodjo.</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8707324/bbm-di-bali-langka-picu-antrean-panjang-bahlil-dirut-pertamina-sudah-di-sana</t>
+          <t>https://finance.detik.com/energi/d-8707520/dirut-pln-diganti-di-tengah-masalah-listrik-batam-padam</t>
         </is>
       </c>
     </row>
@@ -1830,22 +1806,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Mendag Pede Harga Pangan Turun di Akhir Tahun, Ini Alasannya</t>
+          <t>IKN Dapat Investasi Proyek Rusun hingga Restoran, Ini Rinciannya</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Wed, 14 Oct 2026 19:30:01 +0700</t>
+          <t>Wed, 14 Oct 2026 22:54:21 +0700</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/14/menteri-perdagangan-mendag-budi-santoso-1791961572700_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Perdagangan (Mendag) Budi Santoso optimistis harga pangan berangsur turun menjelang akhir tahun.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/14/otorita-ikn-teken-kerja-sama-dengan-badan-usaha-swasta-1791992731112_169.jpeg?w=360&amp;amp;q=90" /&gt; Otorita IKN menandatangani Perjanjian Kerja Sama proyek dengan Badan Usaha sektor perumahan dan investasi langsung swasta murni di G</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8707220/mendag-pede-harga-pangan-turun-di-akhir-tahun-ini-alasannya</t>
+          <t>https://finance.detik.com/infrastruktur/d-8707509/ikn-dapat-investasi-proyek-rusun-hingga-restoran-ini-rinciannya</t>
         </is>
       </c>
     </row>
@@ -1857,22 +1833,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Bahlil Ungkap Biang Kerok Listrik Padam di Batam: Petir hingga Kelelawar</t>
+          <t>Kontraktor Swasta Diprioritaskan Garap Proyek Rp 50-100 Miliar</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Wed, 14 Oct 2026 19:16:02 +0700</t>
+          <t>Wed, 14 Oct 2026 22:29:36 +0700</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/04/28/menteri-esdm-bahlil-lahadalia-1777385212721_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Koordinator Bidang Hilirisasi dan Transisi Energi sekaligus Menteri ESDM Bahlil Lahadalia buka suara soal listrik padam di Batam</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/09/07/bi-prediksi-ekonomi-ri-2026-tumbuh-53-1757231809204_169.jpeg?w=360&amp;amp;q=90" /&gt; Pengusaha konstruksi dapat angin segara dengan Peraturan Menteri Pekerjaan Umum nomor 6 tahun 2025.</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8707278/bahlil-ungkap-biang-kerok-listrik-padam-di-batam-petir-hingga-kelelawar</t>
+          <t>https://finance.detik.com/infrastruktur/d-8707496/kontraktor-swasta-diprioritaskan-garap-proyek-rp-50-100-miliar</t>
         </is>
       </c>
     </row>
@@ -1884,22 +1860,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Mendag Harap Tak Ada Impor KRL Bekas Jepang, Minta Pakai Produk RI</t>
+          <t>Pertamina Genjot Pasokan BBM ke Bali hingga 57,9 Juta Liter</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Wed, 14 Oct 2026 19:00:14 +0700</t>
+          <t>Wed, 14 Oct 2026 22:07:00 +0700</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/14/menteri-perdagangan-mendag-budi-santoso-1791961572700_169.jpeg?w=360&amp;amp;q=90" /&gt; Kalau kami sih berharapnya ya produksi dalam negeri kan sudah ada. Jadi, saya berharap tidak ada impor bekas ya, kata Budi.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/14/pertamina-genjot-pasokan-bbm-ke-bali-1791990343415_169.jpeg?w=360&amp;amp;q=90" /&gt; Pertamina Patra Niaga mengerahkan berbagai upaya untuk mempercepat pemulihan layanan Bahan Bakar Minyak (BBM) di Bali.</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8707212/mendag-harap-tak-ada-impor-krl-bekas-jepang-minta-pakai-produk-ri</t>
+          <t>https://finance.detik.com/energi/d-8707483/pertamina-genjot-pasokan-bbm-ke-bali-hingga-57-9-juta-liter</t>
         </is>
       </c>
     </row>
@@ -1911,22 +1887,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Beredar Kabar Prabowo Cari Menteri ESDM Baru, Bahlil Buka Suara</t>
+          <t>Profil Suroso Isnandar Dirut Baru PLN Pengganti Darmawan Prasodjo</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Wed, 14 Oct 2026 18:32:39 +0700</t>
+          <t>Wed, 14 Oct 2026 21:16:32 +0700</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/16/menteri-esdm-bahlil-lahadalia-1789550049461_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Koordinator (Menko) Hilirisasi dan Transisi Energi Bahlil Lahadalia buka suara soal kabar bakal ada penggantinya sebagai Menteri ESDM.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/14/dirut-baru-pln-suroso-isnandar-1791987368272_43.jpeg?w=360&amp;amp;q=90" /&gt; Suroso Isnandar ditunjuk menjadi Direktur Utama PT PLN (Persero) menggantikan Darmawan Prasodjo.</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8707174/beredar-kabar-prabowo-cari-menteri-esdm-baru-bahlil-buka-suara</t>
+          <t>https://finance.detik.com/energi/d-8707441/profil-suroso-isnandar-dirut-baru-pln-pengganti-darmawan-prasodjo</t>
         </is>
       </c>
     </row>
@@ -1938,22 +1914,22 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Usai Listrik Padam di Batam, Prabowo Minta Danantara Evaluasi PLN</t>
+          <t>Menkop Sudah Ajukan ke Kemenkeu Gaji PNS Dibayar Lewat Kopdes</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Wed, 14 Oct 2026 18:14:42 +0700</t>
+          <t>Wed, 14 Oct 2026 21:01:16 +0700</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/13/presiden-prabowo-subianto-1791858890986_169.jpeg?w=360&amp;amp;q=90" /&gt; Presiden Prabowo perintahkan Danantara untuk percepat transformasi PLN. Fokus pada efisiensi dan penggunaan 100 GW pembangkit tenaga surya.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/03/10/menteri-koperasi-menkop-ferry-juliantono-1773142898217_169.jpeg?w=360&amp;amp;q=90" /&gt; Pemerintah menyiapkan skema pembayaran gaji pegawai negeri sipil (PNS) melalui Koperasi Desa/Kelurahan Merah Putih (Kopdes Merah Putih).</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8707137/usai-listrik-padam-di-batam-prabowo-minta-danantara-evaluasi-pln</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8707426/menkop-sudah-ajukan-ke-kemenkeu-gaji-pns-dibayar-lewat-kopdes</t>
         </is>
       </c>
     </row>
@@ -1965,22 +1941,22 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Bahlil Targetkan Ekspor Nikel Naik Jadi Rp 805,5 T</t>
+          <t>Perluas Pasar Ekspor, APP Group Teken 5 Kesepakatan Dagang di TEI</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Wed, 14 Oct 2026 17:31:37 +0700</t>
+          <t>Wed, 14 Oct 2026 20:55:33 +0700</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/04/28/menteri-esdm-bahlil-lahadalia-1777385212721_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Koordinator Bidang Hilirisasi dan Transisi Energi sekaligus Menteri ESDM Bahlil Lahadalia menargetkan ekspor nikel US$ 45 miliar atau Rp 805,5 triliu</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/14/dukung-penguatan-ekspor-nasional-app-group-perluas-kerja-sama-perdagangan-di-tei-2026-1791985685053.jpeg?w=360&amp;amp;q=90" /&gt; APP Group memperkuat kontribusi ekspor nasional di TEI 2026 dengan kesepakatan perdagangan internasional.</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8707056/bahlil-targetkan-ekspor-nikel-naik-jadi-rp-805-5-t</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8707400/perluas-pasar-ekspor-app-group-teken-5-kesepakatan-dagang-di-tei</t>
         </is>
       </c>
     </row>
@@ -1992,22 +1968,22 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>UMKM Lokal Mulai Bidik Pasar Dunia, Ini Bekal yang Disiapkan</t>
+          <t>Danantara Indonesia Tegaskan Komitmen Peningkatan Layanan PLN</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Wed, 14 Oct 2026 17:17:59 +0700</t>
+          <t>Wed, 14 Oct 2026 20:24:45 +0700</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/14/umkm-1791976666028_169.jpeg?w=360&amp;amp;q=90" /&gt; UMKM binaan Pertamina bersiap menembus pasar internasional melalui Trade Expo Indonesia 2026. Pelatihan ekspor dan promosi digelar untuk mempersiapkan mereka.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/06/26/dony-oskaria-1782464979898.jpeg?w=360&amp;amp;q=90" /&gt; Danantara Indonesia berkomitmen meningkatkan layanan PLN, khususnya di Batam, untuk keandalan pasokan listrik dan respons terhadap kebutuhan pelanggan.</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/solusiukm/d-8707144/umkm-lokal-mulai-bidik-pasar-dunia-ini-bekal-yang-disiapkan</t>
+          <t>https://finance.detik.com/energi/d-8707372/danantara-indonesia-tegaskan-komitmen-peningkatan-layanan-pln</t>
         </is>
       </c>
     </row>
@@ -2019,22 +1995,22 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Pemerintah Mau Transfer Langsung Duit Pensiun PNS, Taspen Ingatkan Ini</t>
+          <t>Darmawan Prasodjo Diganti, Ini Dia Dirut Baru PLN</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Wed, 14 Oct 2026 16:54:01 +0700</t>
+          <t>Wed, 14 Oct 2026 20:00:30 +0700</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/02/12/taspen_169.png?w=360&amp;amp;q=90" /&gt; Kementerian Keuangan (Kemenkeu) berencana mengubah mekanisme pembayaran uang pensiun aparatur sipil negara (ASN) dan TNI/Polri pada 2027.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2022/07/22/kantor-pln-1_169.jpeg?w=360&amp;amp;q=90" /&gt; Darmawan Prasodjo dicopot dari posisi Direktur Utama PT PLN (Persero).</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8706938/pemerintah-mau-transfer-langsung-duit-pensiun-pns-taspen-ingatkan-ini</t>
+          <t>https://finance.detik.com/energi/d-8707339/darmawan-prasodjo-diganti-ini-dia-dirut-baru-pln</t>
         </is>
       </c>
     </row>
@@ -2046,22 +2022,22 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>IHSG Ditutup Menguat ke 5.943</t>
+          <t>BBM di Bali Langka Picu Antrean Panjang, Bahlil: Dirut Pertamina Sudah di Sana</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Wed, 14 Oct 2026 16:19:07 +0700</t>
+          <t>Wed, 14 Oct 2026 19:47:02 +0700</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2021/11/19/ihsg-ditutup-menguat-3_169.jpeg?w=360&amp;amp;q=90" /&gt; Indeks Harga Saham Gabungan (IHSG) hari ini ditutup di zona hijau. IHSG bergerak dua arah hingga akhirnya ditutup di level 5.900.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/11/18/antrean-kendaraan-di-salah-satu-spbu-di-kuta-selatan-badung-bali-selasa-18112025-foto-fabiola-dianiradetikbali-1763454407219_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Koordinator Hilirisasi dan Transisi Energi sekaligus Menteri ESDM Ba</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/bursa-dan-valas/d-8706823/ihsg-ditutup-menguat-ke-5-943</t>
+          <t>https://finance.detik.com/energi/d-8707324/bbm-di-bali-langka-picu-antrean-panjang-bahlil-dirut-pertamina-sudah-di-sana</t>
         </is>
       </c>
     </row>
@@ -2073,22 +2049,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Blibli Raup Pendapatan Neto Rp 14,8 T di Semester I-2026, Tumbuh 55%</t>
+          <t>Mendag Pede Harga Pangan Turun di Akhir Tahun, Ini Alasannya</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Wed, 14 Oct 2026 16:09:29 +0700</t>
+          <t>Wed, 14 Oct 2026 19:30:01 +0700</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/14/blibli-raup-pendapatan-neto-rp-148-t-di-semester-i-2026-tumbuh-55-1791968919767.png?w=360&amp;amp;q=90" /&gt; Blibli mencatatkan pendapatan neto Rp 14,8 triliun, tumbuh 55% YoY pada semester I 2026, didorong oleh segmen lifestyle dan co</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/14/menteri-perdagangan-mendag-budi-santoso-1791961572700_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Perdagangan (Mendag) Budi Santoso optimistis harga pangan berangsur turun menjelang akhir tahun.</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8706811/blibli-raup-pendapatan-neto-rp-14-8-t-di-semester-i-2026-tumbuh-55</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8707220/mendag-pede-harga-pangan-turun-di-akhir-tahun-ini-alasannya</t>
         </is>
       </c>
     </row>
@@ -2100,22 +2076,22 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>PHE Bor Sumur Eksplorasi di Kaltara, Bidik Cadangan Migas Baru</t>
+          <t>Bahlil Ungkap Biang Kerok Listrik Padam di Batam: Petir hingga Kelelawar</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Wed, 14 Oct 2026 16:09:19 +0700</t>
+          <t>Wed, 14 Oct 2026 19:16:02 +0700</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/23/pertamina-ep-1790145752075_169.jpeg?w=360&amp;amp;q=90" /&gt; PT Pertamina Hulu Energi memulai pengeboran sumur eksplorasi Tingkilan-001 di Kalimantan Utara untuk uji potensi hidrokarbon.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/04/28/menteri-esdm-bahlil-lahadalia-1777385212721_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Koordinator Bidang Hilirisasi dan Transisi Energi sekaligus Menteri ESDM Bahlil Lahadalia buka suara soal listrik padam di Batam</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8706800/phe-bor-sumur-eksplorasi-di-kaltara-bidik-cadangan-migas-baru</t>
+          <t>https://finance.detik.com/energi/d-8707278/bahlil-ungkap-biang-kerok-listrik-padam-di-batam-petir-hingga-kelelawar</t>
         </is>
       </c>
     </row>
@@ -2127,22 +2103,22 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Bahlil Merapat ke Istana Lapor soal BBM Langka di Bali</t>
+          <t>Mendag Harap Tak Ada Impor KRL Bekas Jepang, Minta Pakai Produk RI</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Wed, 14 Oct 2026 16:05:25 +0700</t>
+          <t>Wed, 14 Oct 2026 19:00:14 +0700</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/14/menko-hilirisasi-dan-transisi-energi-bahlil-lahadalia-1791968692833_169.jpeg?w=360&amp;amp;q=90" /&gt; Menko Hilirisasi dan Transisi Energi Bahlil Lahadalia hari ini merapat ke Istana Kepresidenan, Jakarta Pusat.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/14/menteri-perdagangan-mendag-budi-santoso-1791961572700_169.jpeg?w=360&amp;amp;q=90" /&gt; Kalau kami sih berharapnya ya produksi dalam negeri kan sudah ada. Jadi, saya berharap tidak ada impor bekas ya, kata Budi.</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8706803/bahlil-merapat-ke-istana-lapor-soal-bbm-langka-di-bali</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8707212/mendag-harap-tak-ada-impor-krl-bekas-jepang-minta-pakai-produk-ri</t>
         </is>
       </c>
     </row>
@@ -2154,22 +2130,22 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>KPK Tahan 5 Tersangka Korupsi BNPB</t>
+          <t>Husniah Talenrang Dipecat sebagai Bupati Gowa</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Wed, 14 Oct 2026 20:21:23 +0700</t>
+          <t>Thu, 15 Oct 2026 06:52:20 +0700</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Penahanan dilakukan KPK setelah memeriksa lima tersangka di Gedung Merah Putih sejak Selasa (13/10/2026).</t>
+          <t>Wakil Bupati Gowa, Darmawangsyah Muin ditunjuk sebagai Plt.</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8313324/kpk-tahan-5-tersangka-korupsi-bnpb</t>
+          <t>https://www.liputan6.com/news/read/8313504/husniah-talenrang-dipecat-sebagai-bupati-gowa</t>
         </is>
       </c>
     </row>
@@ -2181,22 +2157,22 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Satgas PRR dan BRIN Pastikan Kesiapan Lokasi Arsinum di Aceh Utara</t>
+          <t>Pemerintah Tambah 70.000 Polisi Hutan, Bantu Cegah Karhutla dan Lindungi Satwa</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Wed, 14 Oct 2026 20:16:15 +0700</t>
+          <t>Thu, 15 Oct 2026 06:35:27 +0700</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Instalasi Arsinum yang direncanakan di Aceh Utara memiliki kapasitas pengolahan hingga 10.000 liter per hari.</t>
+          <t>Polhut ke depan diharapkan tak hanya menindak, tetapi melakukan upaya pencegahan karhutla dan perlindungan satwa liar.</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8313322/satgas-prr-dan-brin-pastikan-kesiapan-lokasi-arsinum-di-aceh-utara</t>
+          <t>https://www.liputan6.com/news/read/8313497/pemerintah-tambah-70000-polisi-hutan-bantu-cegah-karhutla-dan-lindungi-satwa</t>
         </is>
       </c>
     </row>
@@ -2208,22 +2184,22 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Blak-blakan Terdakwa Nurman Herin Mengaku Ditekan Jaksa Kasus Febrie</t>
+          <t>PKS Ingin Gabungkan Wacana Dapil Nasional dan Sistem Proporsional Terbuka</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Wed, 14 Oct 2026 19:41:13 +0700</t>
+          <t>Thu, 15 Oct 2026 06:34:41 +0700</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Pengakuan itu disampaikan Nurman saat membacakan eksepsi di pengadilan Tipikor Jakarta, Rabu (14/10/2026).</t>
+          <t>Konsep dari dapil nasional ini adalah untuk mengakomodasi suara pemilih yang tidak terkonversi menjadi kursi DPR RI.</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8313304/blak-blakan-terdakwa-nurman-herin-mengaku-ditekan-jaksa-kasus-febrie</t>
+          <t>https://www.liputan6.com/news/read/8313496/pks-ingin-gabungkan-wacana-dapil-nasional-dan-sistem-proporsional-terbuka</t>
         </is>
       </c>
     </row>
@@ -2235,22 +2211,22 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>KPK Dalami Peran Adik Kepala BNPB Usai Ditetapkan sebagai Tersangka</t>
+          <t>Febrie Adriansyah yang Bersikukuh Tak Pernah Salah</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Wed, 14 Oct 2026 19:41:04 +0700</t>
+          <t>Wed, 14 Oct 2026 22:41:49 +0700</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>KPK menetapkan Bima Setyawan, adik Kepala BNPB Suharyanto, sebagai salah satu dari lima tersangka OTT terkait dugaan penyalahgunaan dana kebencanaan.</t>
+          <t>Febrie ingin majelis hakim mengembalikan berkas perkara dan barang bukti kepada jaksa penuntut umum (JPU), serta membebaskannya dari tahanan.</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8313300/kpk-dalami-peran-adik-kepala-bnpb-usai-ditetapkan-sebagai-tersangka</t>
+          <t>https://www.liputan6.com/news/read/8313411/febrie-adriansyah-yang-bersikukuh-tak-pernah-salah</t>
         </is>
       </c>
     </row>
@@ -2262,22 +2238,22 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Berompi Oranye, Begini Penampakan Lima Tersangka Korupsi BNPB</t>
+          <t>Ledakan di Pasar Cimanggis Tewaskan 2 Orang, Dipastikan Bukan Bom</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Wed, 14 Oct 2026 19:13:53 +0700</t>
+          <t>Thu, 15 Oct 2026 05:53:42 +0700</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Salah satu tersangka yang turut dibawa keluar adalah Bima Setyawan, yang disebut merupakan adik Kepala BNPB.</t>
+          <t>Belasan orang juga mengalai luka-luka.</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8313283/berompi-oranye-begini-penampakan-lima-tersangka-korupsi-bnpb</t>
+          <t>https://www.liputan6.com/news/read/8313491/ledakan-di-pasar-cimanggis-tewaskan-2-orang-dipastikan-bukan-bom</t>
         </is>
       </c>
     </row>
@@ -2289,22 +2265,22 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Daftar 12 Wilayah Masuk Zona Berbahaya Imbas Kebakaran Hutan</t>
+          <t>Mengurai Benang Kusut Kebakaran Hutan dan Lahan yang Terus Berulang</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Wed, 14 Oct 2026 19:08:42 +0700</t>
+          <t>Thu, 15 Oct 2026 05:00:42 +0700</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Enam dari 12 wilayah tersebut didominasi daerah Kalimantan Tengah.</t>
+          <t>Mengatasi kebakaran hutan dan lahan yang berulang membutuhkan lebih dari sekadar pemadaman api.</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8313278/daftar-12-wilayah-masuk-zona-berbahaya-imbas-kebakaran-hutan</t>
+          <t>https://www.liputan6.com/news/read/8313474/mengurai-benang-kusut-kebakaran-hutan-dan-lahan-yang-terus-berulang</t>
         </is>
       </c>
     </row>
@@ -2316,22 +2292,22 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>BRIN Sebut Pemadaman Saja Tak Cukup Atasi Kebakaran Hutan</t>
+          <t>Klarifikasi Pemerintah Soal Bantuan Kebakaran Hutan Malaysia dan Jepang</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Wed, 14 Oct 2026 19:08:54 +0700</t>
+          <t>Thu, 15 Oct 2026 01:28:51 +0700</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>BRIN menyoroti faktor manusia di balik kebakaran yang berulang.</t>
+          <t>Kemenko Polkam membantah Indonesia menolak tawaran bantuan Malaysia untuk mengatasi karhutla.</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8313277/brin-sebut-pemadaman-saja-tak-cukup-atasi-kebakaran-hutan</t>
+          <t>https://www.liputan6.com/news/read/8313473/klarifikasi-pemerintah-soal-bantuan-kebakaran-hutan-malaysia-dan-jepang</t>
         </is>
       </c>
     </row>
@@ -2343,22 +2319,22 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Adik Kepala BNPB Jadi Tersangka Dugaan Korupsi Dana Bencana</t>
+          <t>Cairan Pemadam Brasil Diuji di Kebakaran Hutan, Ini Hasil Awalnya</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Wed, 14 Oct 2026 19:03:13 +0700</t>
+          <t>Thu, 15 Oct 2026 01:19:35 +0700</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Lima tersangka OTT KPK di lingkungan BNPB ditahan terkait dugaan penyalahgunaan dana siap pakai kebencanaan. Salah satunya disebut merupakan adik Kepala BNPB Letjen Suharyanto.</t>
+          <t>Cairan pemadam Brasil diharapkan membantu memadamkan api dan mengurangi asap karhutla.</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8313264/adik-kepala-bnpb-jadi-tersangka-dugaan-korupsi-dana-bencana</t>
+          <t>https://www.liputan6.com/news/read/8313466/cairan-pemadam-brasil-diuji-di-kebakaran-hutan-ini-hasil-awalnya</t>
         </is>
       </c>
     </row>
@@ -2370,22 +2346,22 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Gibran: Kritik Pemerintah Harus Dijawab dengan Kerja Lebih Baik</t>
+          <t>Transformasi Digital PERURI, dari Mencetak Rupiah hingga Mengamankan Data Masyarakat</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Wed, 14 Oct 2026 18:00:39 +0700</t>
+          <t>Wed, 14 Oct 2026 19:20:09 +0700</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Gibran Respon Survei Evaluasi 2 Tahun Kinerja Pemerintah: Kritik Dijawab dengan Kerja Nyata</t>
+          <t>Kenali transformasi digital PERURI melalui e-Meterai, Peruri Sign, dan dukungan GovTech untuk menjaga kedaulatan serta kepercayaan masyarakat.</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8313214/gibran-kritik-pemerintah-harus-dijawab-dengan-kerja-lebih-baik</t>
+          <t>https://www.liputan6.com/news/read/8312930/transformasi-digital-peruri-dari-mencetak-rupiah-hingga-mengamankan-data-masyarakat</t>
         </is>
       </c>
     </row>
@@ -2397,22 +2373,22 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>BMKG Prediksi El Nino Bertahan hingga Awal 2027, Musim Hujan Mundur</t>
+          <t>Kejagung Buka Lelang Batu Bara Sitaan Kasus Samin Tan</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Wed, 14 Oct 2026 18:31:30 +0700</t>
+          <t>Wed, 14 Oct 2026 23:52:04 +0700</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>BMKG mengingatkan potensi banjir, banjir bandang, dan longsor ketika musim hujan tiba di tengah kondisi iklim yang dipengaruhi El Nino.</t>
+          <t>Lelang batu bara sitaan kasus PT Asmin Koalindo Tuhup digelar secara daring melalui mekanisme open bidding.</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8313215/bmkg-prediksi-el-nino-bertahan-hingga-awal-2027-musim-hujan-mundur</t>
+          <t>https://www.liputan6.com/news/read/8313447/kejagung-buka-lelang-batu-bara-sitaan-kasus-samin-tan</t>
         </is>
       </c>
     </row>
@@ -2424,22 +2400,22 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Jakarta Raih Peringkat 117 Kota Pelajar Dunia, Pramono Apresiasi Guru</t>
+          <t>Infografis: Rekam Jejak Kebakaran Hutan dan Lahan dalam 6 Tahun</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Wed, 14 Oct 2026 17:23:58 +0700</t>
+          <t>Wed, 14 Oct 2026 23:03:20 +0700</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Jakarta berada di peringkat ke-117 dunia dalam QS Best Student Cities 2027, satu tingkat di atas Yogyakarta.</t>
+          <t>Kalbar, Kalteng, Kalsel, Kaltim, Sumsel, Riau, dan Jambi menjadi wilayah prioritas penanganan karhutla.</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8313209/jakarta-raih-peringkat-117-kota-pelajar-dunia-pramono-apresiasi-guru</t>
+          <t>https://www.liputan6.com/news/read/8313425/infografis-rekam-jejak-kebakaran-hutan-dan-lahan-dalam-6-tahun</t>
         </is>
       </c>
     </row>
@@ -2451,22 +2427,22 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Mobil Listrik Terbakar di Tebet, Asap Hitam Membumbung</t>
+          <t>Diduga Terkait LPG, Polisi Selidiki Ledakan di Pasar Cimanggis</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Wed, 14 Oct 2026 17:00:43 +0700</t>
+          <t>Wed, 14 Oct 2026 22:53:09 +0700</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Mobil listrik terbakar di Tebet, Jakarta Selatan, asap hitam membumbung dari lokasi kejadian.</t>
+          <t>Polisi masih mendalami penyebab ledakan di sebuah pertokoan di Pasar Cimanggis, Ciputat, Tangerang Selatan.</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8313179/mobil-listrik-terbakar-di-tebet-asap-hitam-membumbung</t>
+          <t>https://www.liputan6.com/news/read/8313420/diduga-terkait-lpg-polisi-selidiki-ledakan-di-pasar-cimanggis</t>
         </is>
       </c>
     </row>
@@ -2478,22 +2454,22 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>513 Hektare Hutan Tanjung Puting Hangus, Api Belum Juga Padam</t>
+          <t>Gegana Tangani Ledakan di Pasar Cimanggis</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Wed, 14 Oct 2026 16:40:33 +0700</t>
+          <t>Wed, 14 Oct 2026 22:45:14 +0700</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Karhutla di Taman Nasional Tanjung Puting telah membakar sekitar 513 hektare lahan. Ratusan personel tambahan dikerahkan untuk menangani kebakaran.</t>
+          <t>Polisi masih melakukan evakuasi, sterilisasi, dan olah TKP setelah ledakan terjadi di kawasan Pasar Cimanggis, Tangsel.</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8313137/513-hektare-hutan-tanjung-puting-hangus-api-belum-juga-padam</t>
+          <t>https://www.liputan6.com/news/read/8313410/gegana-tangani-ledakan-di-pasar-cimanggis</t>
         </is>
       </c>
     </row>
@@ -2505,22 +2481,22 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>KPK Tetapkan Tersangka di Kasus OTT BNPB</t>
+          <t>Hotspot Sumsel Naik 92 Persen, Begini Aksi Kemenhut</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Wed, 14 Oct 2026 16:32:20 +0700</t>
+          <t>Wed, 14 Oct 2026 22:13:45 +0700</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Pihak yang telah ditetapkan sebagai tersangka selanjutnya akan menjalani penahanan.</t>
+          <t>Kemenhut menerapkan pemindahan personel untuk memperkuat penanganan karhutla</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8313127/kpk-tetapkan-tersangka-di-kasus-ott-bnpb</t>
+          <t>https://www.liputan6.com/news/read/8313400/hotspot-sumsel-naik-92-persen-begini-aksi-kemenhut</t>
         </is>
       </c>
     </row>
@@ -2532,22 +2508,22 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Kubu Febrie Bongkar Peran Ferry Hongkiriwang dalam Kasus Pemerasan</t>
+          <t>Ledakan di Pasar Cimanggis Ciputat, 8 Orang Dilarikan ke RS</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Wed, 14 Oct 2026 16:17:16 +0700</t>
+          <t>Wed, 14 Oct 2026 22:03:16 +0700</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Kubu Febrie Adriansyah mengungkapkan dalam dakwaan Febrie tidak terdapat perintah kepada Ferry untuk memaksa Tan Kian menyerahkan sejumlah uang.</t>
+          <t>Saat ini fokus utama yaitu menyelamatkan korban akibat ledakan tersebut.</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8313114/kubu-febrie-bongkar-peran-ferry-hongkiriwang-dalam-kasus-pemerasan</t>
+          <t>https://www.liputan6.com/news/read/8313396/ledakan-di-pasar-cimanggis-ciputat-8-orang-dilarikan-ke-rs</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data pasar & berita - 2026-10-15 13:14 UTC
</commit_message>
<xml_diff>
--- a/data/market_news_latest.xlsx
+++ b/data/market_news_latest.xlsx
@@ -487,20 +487,20 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>5925.9761</v>
+        <v>5863.7798</v>
       </c>
       <c r="F2" t="n">
-        <v>-10.1709</v>
+        <v>-79.2441</v>
       </c>
       <c r="G2" t="n">
-        <v>-0.17</v>
+        <v>-1.33</v>
       </c>
       <c r="H2" t="n">
-        <v>314688200</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -534,7 +534,7 @@
         <v>-1.11</v>
       </c>
       <c r="H3" t="n">
-        <v>3388032000</v>
+        <v>5955580000</v>
       </c>
     </row>
     <row r="4">
@@ -568,7 +568,7 @@
         <v>-0.09</v>
       </c>
       <c r="H4" t="n">
-        <v>442523838</v>
+        <v>442520000</v>
       </c>
     </row>
     <row r="5">
@@ -602,7 +602,7 @@
         <v>-1.88</v>
       </c>
       <c r="H5" t="n">
-        <v>7640476000</v>
+        <v>8568280000</v>
       </c>
     </row>
     <row r="6">
@@ -623,20 +623,20 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>67777.52340000001</v>
+        <v>64425.9492</v>
       </c>
       <c r="F6" t="n">
-        <v>-1253.3984</v>
+        <v>-3318.3398</v>
       </c>
       <c r="G6" t="n">
-        <v>-1.82</v>
+        <v>-4.9</v>
       </c>
       <c r="H6" t="n">
-        <v>168000000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -657,20 +657,20 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>24345.2207</v>
+        <v>24062.7207</v>
       </c>
       <c r="F7" t="n">
-        <v>74.0215</v>
+        <v>-251.4492</v>
       </c>
       <c r="G7" t="n">
-        <v>0.3</v>
+        <v>-1.03</v>
       </c>
       <c r="H7" t="n">
-        <v>2546200000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -691,14 +691,20 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>3707.4761</v>
+      </c>
+      <c r="F8" t="n">
+        <v>-59.751</v>
+      </c>
+      <c r="G8" t="n">
+        <v>-1.59</v>
+      </c>
       <c r="H8" t="n">
-        <v>1646582440</v>
+        <v>3771678644</v>
       </c>
     </row>
     <row r="9">
@@ -719,20 +725,20 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>10650.2998</v>
+        <v>10832.4697</v>
       </c>
       <c r="F9" t="n">
-        <v>-6</v>
+        <v>107.5693</v>
       </c>
       <c r="G9" t="n">
-        <v>-0.06</v>
+        <v>1</v>
       </c>
       <c r="H9" t="n">
-        <v>670857300</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -753,20 +759,20 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>25259.9004</v>
+        <v>25261.1094</v>
       </c>
       <c r="F10" t="n">
-        <v>-17.7793</v>
+        <v>-37.5</v>
       </c>
       <c r="G10" t="n">
-        <v>-0.07000000000000001</v>
+        <v>-0.15</v>
       </c>
       <c r="H10" t="n">
-        <v>48379600</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -787,20 +793,20 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>5430.5</v>
+        <v>5403.5</v>
       </c>
       <c r="F11" t="n">
-        <v>15.02</v>
+        <v>-19.8301</v>
       </c>
       <c r="G11" t="n">
-        <v>0.28</v>
+        <v>-0.37</v>
       </c>
       <c r="H11" t="n">
-        <v>266038800</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -821,17 +827,17 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>17866.5</v>
+        <v>17943</v>
       </c>
       <c r="F12" t="n">
-        <v>-46.5</v>
+        <v>76.5</v>
       </c>
       <c r="G12" t="n">
-        <v>-0.26</v>
+        <v>0.43</v>
       </c>
       <c r="H12" t="n">
         <v>0</v>
@@ -855,17 +861,17 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>102.207</v>
+        <v>102.116</v>
       </c>
       <c r="F13" t="n">
-        <v>0.027</v>
+        <v>-0.434</v>
       </c>
       <c r="G13" t="n">
-        <v>0.03</v>
+        <v>-0.42</v>
       </c>
       <c r="H13" t="n">
         <v>0</v>
@@ -893,13 +899,13 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>157.933</v>
+        <v>157.853</v>
       </c>
       <c r="F14" t="n">
-        <v>-0.389</v>
+        <v>-0.469</v>
       </c>
       <c r="G14" t="n">
-        <v>-0.25</v>
+        <v>-0.3</v>
       </c>
       <c r="H14" t="n">
         <v>0</v>
@@ -923,17 +929,17 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>0.519</v>
+        <v>0.5054</v>
       </c>
       <c r="F15" t="n">
-        <v>-0.0027</v>
+        <v>-0.0136</v>
       </c>
       <c r="G15" t="n">
-        <v>-0.52</v>
+        <v>-2.62</v>
       </c>
       <c r="H15" t="n">
         <v>0</v>
@@ -957,17 +963,17 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>0.5525</v>
+        <v>0.5391</v>
       </c>
       <c r="F16" t="n">
-        <v>-0.0038</v>
+        <v>-0.0134</v>
       </c>
       <c r="G16" t="n">
-        <v>-0.68</v>
+        <v>-2.43</v>
       </c>
       <c r="H16" t="n">
         <v>0</v>
@@ -991,17 +997,17 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>0.4085</v>
+        <v>0.4077</v>
       </c>
       <c r="F17" t="n">
-        <v>0.0028</v>
+        <v>-0.0008</v>
       </c>
       <c r="G17" t="n">
-        <v>0.6899999999999999</v>
+        <v>-0.2</v>
       </c>
       <c r="H17" t="n">
         <v>0</v>
@@ -1028,11 +1034,17 @@
           <t>2026-10-14</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
+      <c r="E18" t="n">
+        <v>78.89</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0.66</v>
+      </c>
       <c r="H18" t="n">
-        <v>50953748</v>
+        <v>50909600</v>
       </c>
     </row>
     <row r="19">
@@ -1056,11 +1068,17 @@
           <t>2026-10-14</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
+      <c r="E19" t="n">
+        <v>76.81</v>
+      </c>
+      <c r="F19" t="n">
+        <v>-0.28</v>
+      </c>
+      <c r="G19" t="n">
+        <v>-0.36</v>
+      </c>
       <c r="H19" t="n">
-        <v>63579674</v>
+        <v>63579700</v>
       </c>
     </row>
     <row r="20">
@@ -1081,20 +1099,20 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>4133.1001</v>
+        <v>4165.2998</v>
       </c>
       <c r="F20" t="n">
-        <v>-44.1997</v>
+        <v>57.3999</v>
       </c>
       <c r="G20" t="n">
-        <v>-1.06</v>
+        <v>1.4</v>
       </c>
       <c r="H20" t="n">
-        <v>6554</v>
+        <v>91221</v>
       </c>
     </row>
     <row r="21">
@@ -1115,20 +1133,20 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>94.77</v>
+        <v>94.18000000000001</v>
       </c>
       <c r="F21" t="n">
-        <v>0.63</v>
+        <v>-0.91</v>
       </c>
       <c r="G21" t="n">
-        <v>0.67</v>
+        <v>-0.96</v>
       </c>
       <c r="H21" t="n">
-        <v>2481</v>
+        <v>82304</v>
       </c>
     </row>
     <row r="22">
@@ -1149,20 +1167,20 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="E22" t="n">
-        <v>105.63</v>
+        <v>104.59</v>
       </c>
       <c r="F22" t="n">
-        <v>-0.06</v>
+        <v>-1.47</v>
       </c>
       <c r="G22" t="n">
-        <v>-0.06</v>
+        <v>-1.39</v>
       </c>
       <c r="H22" t="n">
-        <v>164</v>
+        <v>24050</v>
       </c>
     </row>
     <row r="23">
@@ -1183,20 +1201,20 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="E23" t="n">
-        <v>6.61</v>
+        <v>6.5425</v>
       </c>
       <c r="F23" t="n">
-        <v>-0.068</v>
+        <v>-0.06900000000000001</v>
       </c>
       <c r="G23" t="n">
-        <v>-1.02</v>
+        <v>-1.04</v>
       </c>
       <c r="H23" t="n">
-        <v>754</v>
+        <v>36101</v>
       </c>
     </row>
     <row r="24">
@@ -1220,11 +1238,17 @@
           <t>2026-10-14</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr"/>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr"/>
+      <c r="E24" t="n">
+        <v>64.39</v>
+      </c>
+      <c r="F24" t="n">
+        <v>-1.35</v>
+      </c>
+      <c r="G24" t="n">
+        <v>-2.05</v>
+      </c>
       <c r="H24" t="n">
-        <v>21163577</v>
+        <v>21169200</v>
       </c>
     </row>
     <row r="25">
@@ -1245,17 +1269,17 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="E25" t="n">
-        <v>16.87</v>
+        <v>17.47</v>
       </c>
       <c r="F25" t="n">
-        <v>1.6</v>
+        <v>0.6</v>
       </c>
       <c r="G25" t="n">
-        <v>10.48</v>
+        <v>3.56</v>
       </c>
       <c r="H25" t="n">
         <v>0</v>
@@ -1283,16 +1307,16 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>81650.47659999999</v>
+        <v>80418.07030000001</v>
       </c>
       <c r="F26" t="n">
-        <v>-1444.6484</v>
+        <v>-1144.4219</v>
       </c>
       <c r="G26" t="n">
-        <v>-1.74</v>
+        <v>-1.4</v>
       </c>
       <c r="H26" t="n">
-        <v>33361143808</v>
+        <v>40395726848</v>
       </c>
     </row>
     <row r="27">
@@ -1313,20 +1337,20 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="E27" t="n">
-        <v>1430</v>
+        <v>1420</v>
       </c>
       <c r="F27" t="n">
-        <v>120</v>
+        <v>-10</v>
       </c>
       <c r="G27" t="n">
-        <v>9.16</v>
+        <v>-0.7</v>
       </c>
       <c r="H27" t="n">
-        <v>182930700</v>
+        <v>87691800</v>
       </c>
     </row>
     <row r="28">
@@ -1347,20 +1371,20 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="E28" t="n">
-        <v>1500</v>
+        <v>1415</v>
       </c>
       <c r="F28" t="n">
-        <v>-20</v>
+        <v>-85</v>
       </c>
       <c r="G28" t="n">
-        <v>-1.32</v>
+        <v>-5.67</v>
       </c>
       <c r="H28" t="n">
-        <v>135916800</v>
+        <v>166054400</v>
       </c>
     </row>
     <row r="29">
@@ -1381,20 +1405,20 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="E29" t="n">
-        <v>665</v>
+        <v>630</v>
       </c>
       <c r="F29" t="n">
-        <v>0</v>
+        <v>-35</v>
       </c>
       <c r="G29" t="n">
-        <v>0</v>
+        <v>-5.26</v>
       </c>
       <c r="H29" t="n">
-        <v>380902600</v>
+        <v>285141100</v>
       </c>
     </row>
     <row r="30">
@@ -1415,20 +1439,20 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="E30" t="n">
-        <v>2320</v>
+        <v>2180</v>
       </c>
       <c r="F30" t="n">
-        <v>-110</v>
+        <v>-140</v>
       </c>
       <c r="G30" t="n">
-        <v>-4.53</v>
+        <v>-6.03</v>
       </c>
       <c r="H30" t="n">
-        <v>25909400</v>
+        <v>18298600</v>
       </c>
     </row>
     <row r="31">
@@ -1449,20 +1473,20 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="E31" t="n">
-        <v>4120</v>
+        <v>3920</v>
       </c>
       <c r="F31" t="n">
-        <v>-60</v>
+        <v>-200</v>
       </c>
       <c r="G31" t="n">
-        <v>-1.44</v>
+        <v>-4.85</v>
       </c>
       <c r="H31" t="n">
-        <v>44581400</v>
+        <v>47973300</v>
       </c>
     </row>
     <row r="32">
@@ -1483,20 +1507,20 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="E32" t="n">
-        <v>500</v>
+        <v>474</v>
       </c>
       <c r="F32" t="n">
-        <v>0</v>
+        <v>-26</v>
       </c>
       <c r="G32" t="n">
-        <v>0</v>
+        <v>-5.2</v>
       </c>
       <c r="H32" t="n">
-        <v>35585800</v>
+        <v>48900700</v>
       </c>
     </row>
     <row r="33">
@@ -1517,20 +1541,20 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="E33" t="n">
-        <v>595</v>
+        <v>575</v>
       </c>
       <c r="F33" t="n">
-        <v>-10</v>
+        <v>-20</v>
       </c>
       <c r="G33" t="n">
-        <v>-1.65</v>
+        <v>-3.36</v>
       </c>
       <c r="H33" t="n">
-        <v>41452100</v>
+        <v>70117600</v>
       </c>
     </row>
     <row r="34">
@@ -1551,20 +1575,20 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="E34" t="n">
-        <v>3620</v>
+        <v>3480</v>
       </c>
       <c r="F34" t="n">
-        <v>-90</v>
+        <v>-140</v>
       </c>
       <c r="G34" t="n">
-        <v>-2.43</v>
+        <v>-3.87</v>
       </c>
       <c r="H34" t="n">
-        <v>1895800</v>
+        <v>4822700</v>
       </c>
     </row>
     <row r="35">
@@ -1585,20 +1609,20 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="E35" t="n">
-        <v>520</v>
+        <v>470</v>
       </c>
       <c r="F35" t="n">
-        <v>-2</v>
+        <v>-50</v>
       </c>
       <c r="G35" t="n">
-        <v>-0.38</v>
+        <v>-9.619999999999999</v>
       </c>
       <c r="H35" t="n">
-        <v>119209400</v>
+        <v>143573800</v>
       </c>
     </row>
     <row r="36">
@@ -1619,20 +1643,20 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="E36" t="n">
-        <v>195</v>
+        <v>184</v>
       </c>
       <c r="F36" t="n">
-        <v>-4</v>
+        <v>-11</v>
       </c>
       <c r="G36" t="n">
-        <v>-2.01</v>
+        <v>-5.64</v>
       </c>
       <c r="H36" t="n">
-        <v>14683300</v>
+        <v>36831100</v>
       </c>
     </row>
     <row r="37">
@@ -1653,20 +1677,20 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="E37" t="n">
-        <v>14550</v>
+        <v>14075</v>
       </c>
       <c r="F37" t="n">
-        <v>300</v>
+        <v>-475</v>
       </c>
       <c r="G37" t="n">
-        <v>2.11</v>
+        <v>-3.26</v>
       </c>
       <c r="H37" t="n">
-        <v>10912400</v>
+        <v>10820200</v>
       </c>
     </row>
   </sheetData>
@@ -1725,22 +1749,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Pengganti LPG 3 Kg Mulai Dijual 2027, Tabungnya dari China</t>
+          <t>10.070 Kopdes Mulai Operasi Hari Ini</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Thu, 15 Oct 2026 06:55:00 +0700</t>
+          <t>Thu, 15 Oct 2026 20:00:41 +0700</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2021/12/14/cng-gaslink-1_169.jpeg?w=360&amp;amp;q=90" /&gt; Program CNG 3 kg sebagai pengganti LPG akan diluncurkan pada 2027. Uji coba telah dilakukan, dengan 100 ribu tabung dari China siap didistribusikan.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/21/kopdes-merah-putih-bersiap-operasional-23-ribu-bangunan-telah-rampung-1789986171380_169.jpeg?w=360&amp;amp;q=90" /&gt; Distribusi pasokan pangan untuk operasional Koperasi Desa/Kelurahan Merah Putih (KDKMP) dipastikan sudah siap.</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8707229/pengganti-lpg-3-kg-mulai-dijual-2027-tabungnya-dari-china</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8709020/10-070-kopdes-mulai-operasi-hari-ini</t>
         </is>
       </c>
     </row>
@@ -1752,22 +1776,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Bos Agrinas soal Ratusan Manajer Kopdes Mundur: Tidak Ada yang Rugi!</t>
+          <t>DJP Siapkan Insentif Pajak buat BUMN, Ini Bocorannya</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Thu, 15 Oct 2026 06:25:00 +0700</t>
+          <t>Thu, 15 Oct 2026 19:30:12 +0700</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/03/31/direktur-utama-pt-agrinas-pangan-nusantara-joao-angelo-de-sousa-mota-1774938653280_169.jpeg?w=360&amp;amp;q=90" /&gt; Itu kan anak bangsa, tidak ada yang rugi. Kalau saya dibina boleh lah, tegas dia.</t>
+          <t xml:space="preserve">&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/15/direktur-jenderal-pajak-djp-bimo-wijayanto-1792062697952_169.jpeg?w=360&amp;amp;q=90" /&gt; Direktorat Jenderal Pajak (DJP) disebut telah menyiapkan aturan tentang insentif pajak bagi Badan Usaha Milik Negara (BUMN) yang melakukan aksi </t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8706911/bos-agrinas-soal-ratusan-manajer-kopdes-mundur-tidak-ada-yang-rugi</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8708986/djp-siapkan-insentif-pajak-buat-bumn-ini-bocorannya</t>
         </is>
       </c>
     </row>
@@ -1779,22 +1803,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Dirut PLN Diganti di Tengah Masalah Listrik Batam Padam</t>
+          <t>KRL Kerap Gangguan, INKA Minta Maaf</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Thu, 15 Oct 2026 05:55:00 +0700</t>
+          <t>Thu, 15 Oct 2026 19:00:11 +0700</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2022/07/22/kantor-pln_169.jpeg?w=360&amp;amp;q=90" /&gt; Suroso Isnandar diangkat sebagai Direktur Utama (Dirut) baru PLN. Suroso menggantikan Darmawan Prasodjo.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/14/krl-inka-gangguan-penumpang-di-stasiun-pasar-minggu-pindah-krl-dok-istimewa-1791983235827_169.jpeg?w=360&amp;amp;q=90" /&gt; PT Industri Kereta Api (Persero) atau INKA buka suara soal beberapa rangkaian KRL CLI-225 yang mengalami masala</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8707520/dirut-pln-diganti-di-tengah-masalah-listrik-batam-padam</t>
+          <t>https://finance.detik.com/infrastruktur/d-8708975/krl-kerap-gangguan-inka-minta-maaf</t>
         </is>
       </c>
     </row>
@@ -1806,22 +1830,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>IKN Dapat Investasi Proyek Rusun hingga Restoran, Ini Rinciannya</t>
+          <t>Penerimaan Pajak RI Segitu-gitu Aja, DJP Buka Suara</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Wed, 14 Oct 2026 22:54:21 +0700</t>
+          <t>Thu, 15 Oct 2026 18:30:45 +0700</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/14/otorita-ikn-teken-kerja-sama-dengan-badan-usaha-swasta-1791992731112_169.jpeg?w=360&amp;amp;q=90" /&gt; Otorita IKN menandatangani Perjanjian Kerja Sama proyek dengan Badan Usaha sektor perumahan dan investasi langsung swasta murni di G</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/15/direktur-jenderal-pajak-djp-bimo-wijayanto-1792062697871_169.jpeg?w=360&amp;amp;q=90" /&gt; Direktur Jenderal Pajak (DJP) Bimo Wijayanto, mengatakan baru sekali dalam sejarah pemerintah berani menargetkan penerimaan pajak 9% dari PDB da</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/infrastruktur/d-8707509/ikn-dapat-investasi-proyek-rusun-hingga-restoran-ini-rinciannya</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8708906/penerimaan-pajak-ri-segitu-gitu-aja-djp-buka-suara</t>
         </is>
       </c>
     </row>
@@ -1833,22 +1857,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Kontraktor Swasta Diprioritaskan Garap Proyek Rp 50-100 Miliar</t>
+          <t>MR.D.I.Y., Kemenperin &amp;amp; CIMB Niaga Dorong IKM Perkuat Bisnis Berkelanjutan</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Wed, 14 Oct 2026 22:29:36 +0700</t>
+          <t>Thu, 15 Oct 2026 18:15:54 +0700</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/09/07/bi-prediksi-ekonomi-ri-2026-tumbuh-53-1757231809204_169.jpeg?w=360&amp;amp;q=90" /&gt; Pengusaha konstruksi dapat angin segara dengan Peraturan Menteri Pekerjaan Umum nomor 6 tahun 2025.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/15/mrdiy-kemenperin-cimb-niaga-dorong-ikm-perkuat-bisnis-berkelanjutan-1792062894911.jpeg?w=360&amp;amp;q=90" /&gt; PT Daya Intiguna Yasa Tbk dan CIMB Niaga gelar pelatihan manajemen keuangan untuk 100 IKM. Fokus pada keberlanjutan dan pen</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/infrastruktur/d-8707496/kontraktor-swasta-diprioritaskan-garap-proyek-rp-50-100-miliar</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8708914/mr-d-i-y-kemenperin-cimb-niaga-dorong-ikm-perkuat-bisnis-berkelanjutan</t>
         </is>
       </c>
     </row>
@@ -1860,22 +1884,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Pertamina Genjot Pasokan BBM ke Bali hingga 57,9 Juta Liter</t>
+          <t>Perang Arab Saudi Vs Houthi, Garuda Alihkan Rute-Tunda Penerbangan</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Wed, 14 Oct 2026 22:07:00 +0700</t>
+          <t>Thu, 15 Oct 2026 18:03:46 +0700</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/14/pertamina-genjot-pasokan-bbm-ke-bali-1791990343415_169.jpeg?w=360&amp;amp;q=90" /&gt; Pertamina Patra Niaga mengerahkan berbagai upaya untuk mempercepat pemulihan layanan Bahan Bakar Minyak (BBM) di Bali.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/07/19/pesawat-garuda-indonesia-1752916632356_169.jpeg?w=360&amp;amp;q=90" /&gt; Situasi geopolitik di kawasan Timur Tengah berpotensi berdampak pada operasi penerbangan dari dan menuju Arab Saudi.</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8707483/pertamina-genjot-pasokan-bbm-ke-bali-hingga-57-9-juta-liter</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8708883/perang-arab-saudi-vs-houthi-garuda-alihkan-rute-tunda-penerbangan</t>
         </is>
       </c>
     </row>
@@ -1887,22 +1911,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Profil Suroso Isnandar Dirut Baru PLN Pengganti Darmawan Prasodjo</t>
+          <t>Dilantik Jadi Wamentan, Alim Setiawan Dapat Tugas Apa dari Prabowo?</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Wed, 14 Oct 2026 21:16:32 +0700</t>
+          <t>Thu, 15 Oct 2026 17:29:58 +0700</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/14/dirut-baru-pln-suroso-isnandar-1791987368272_43.jpeg?w=360&amp;amp;q=90" /&gt; Suroso Isnandar ditunjuk menjadi Direktur Utama PT PLN (Persero) menggantikan Darmawan Prasodjo.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/15/ipb-1792047319407_169.jpeg?w=360&amp;amp;q=90" /&gt; Presiden Prabowo Subianto melantik Alim Setiawan Slamet menjadi Wakil Menteri Pertanian.</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8707441/profil-suroso-isnandar-dirut-baru-pln-pengganti-darmawan-prasodjo</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8708763/dilantik-jadi-wamentan-alim-setiawan-dapat-tugas-apa-dari-prabowo</t>
         </is>
       </c>
     </row>
@@ -1914,22 +1938,22 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Menkop Sudah Ajukan ke Kemenkeu Gaji PNS Dibayar Lewat Kopdes</t>
+          <t>Ada Harta Karun di Bawah Jakarta! Terungkap Saat Gali Jalur MRT</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Wed, 14 Oct 2026 21:01:16 +0700</t>
+          <t>Thu, 15 Oct 2026 17:24:29 +0700</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/03/10/menteri-koperasi-menkop-ferry-juliantono-1773142898217_169.jpeg?w=360&amp;amp;q=90" /&gt; Pemerintah menyiapkan skema pembayaran gaji pegawai negeri sipil (PNS) melalui Koperasi Desa/Kelurahan Merah Putih (Kopdes Merah Putih).</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/15/harta-karun-mrt-1792059689770_169.jpeg?w=360&amp;amp;q=90" /&gt; Proyek MRT Jakarta Fase 2 menemukan ribuan artefak sejarah, termasuk keramik kuno dan saluran air terakota, menantang proses konstruksi dan pelestarian budaya.</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8707426/menkop-sudah-ajukan-ke-kemenkeu-gaji-pns-dibayar-lewat-kopdes</t>
+          <t>https://finance.detik.com/infrastruktur/d-8708754/ada-harta-karun-di-bawah-jakarta-terungkap-saat-gali-jalur-mrt</t>
         </is>
       </c>
     </row>
@@ -1941,22 +1965,22 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Perluas Pasar Ekspor, APP Group Teken 5 Kesepakatan Dagang di TEI</t>
+          <t>Seharian di Zona Merah, IHSG Ditutup di Level 5.863</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Wed, 14 Oct 2026 20:55:33 +0700</t>
+          <t>Thu, 15 Oct 2026 17:09:50 +0700</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/14/dukung-penguatan-ekspor-nasional-app-group-perluas-kerja-sama-perdagangan-di-tei-2026-1791985685053.jpeg?w=360&amp;amp;q=90" /&gt; APP Group memperkuat kontribusi ekspor nasional di TEI 2026 dengan kesepakatan perdagangan internasional.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/05/18/ihsg-anjlok-ke-zona-merah-bursa-saham-melemah-tajam-1779098741262_169.jpeg?w=360&amp;amp;q=90" /&gt; Indeks Harga Saham Gabungan (IHSG) ditutup di zona merah sore ini.</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8707400/perluas-pasar-ekspor-app-group-teken-5-kesepakatan-dagang-di-tei</t>
+          <t>https://finance.detik.com/bursa-dan-valas/d-8708712/seharian-di-zona-merah-ihsg-ditutup-di-level-5-863</t>
         </is>
       </c>
     </row>
@@ -1968,22 +1992,22 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Danantara Indonesia Tegaskan Komitmen Peningkatan Layanan PLN</t>
+          <t>Subsidi LPG Bengkak dari Rp 87 T, Kini Tembus Rp 100 T</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Wed, 14 Oct 2026 20:24:45 +0700</t>
+          <t>Thu, 15 Oct 2026 17:04:34 +0700</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/06/26/dony-oskaria-1782464979898.jpeg?w=360&amp;amp;q=90" /&gt; Danantara Indonesia berkomitmen meningkatkan layanan PLN, khususnya di Batam, untuk keandalan pasokan listrik dan respons terhadap kebutuhan pelanggan.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/14/bahlil-lahadalia-rolandodetikcom-1791978307056_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Bahlil mengungkap subsidi LPG membengkak di atas Rp 100 triliun saat ICP naik. Pemerintah kembangkan CNG 3 kg untuk kurangi impor LPG.</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8707372/danantara-indonesia-tegaskan-komitmen-peningkatan-layanan-pln</t>
+          <t>https://finance.detik.com/energi/d-8708710/subsidi-lpg-bengkak-dari-rp-87-t-kini-tembus-rp-100-t</t>
         </is>
       </c>
     </row>
@@ -1995,22 +2019,22 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Darmawan Prasodjo Diganti, Ini Dia Dirut Baru PLN</t>
+          <t>Wamenkeu Tegaskan Kripto Bukan Mata Uang, Tetap Kena Pajak</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Wed, 14 Oct 2026 20:00:30 +0700</t>
+          <t>Thu, 15 Oct 2026 16:57:39 +0700</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2022/07/22/kantor-pln-1_169.jpeg?w=360&amp;amp;q=90" /&gt; Darmawan Prasodjo dicopot dari posisi Direktur Utama PT PLN (Persero).</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2022/07/11/ilustrasi-aset-kripto-bitcoin-dan-xrp_169.jpeg?w=360&amp;amp;q=90" /&gt; Wakil Menteri Keuangan (Wamenkeu) Nurkholisoh Ibnu Aman menegaskan, aset kripto bukan alat pembayaran yang sah di Indonesia.</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8707339/darmawan-prasodjo-diganti-ini-dia-dirut-baru-pln</t>
+          <t>https://finance.detik.com/fintech/d-8708701/wamenkeu-tegaskan-kripto-bukan-mata-uang-tetap-kena-pajak</t>
         </is>
       </c>
     </row>
@@ -2022,22 +2046,22 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>BBM di Bali Langka Picu Antrean Panjang, Bahlil: Dirut Pertamina Sudah di Sana</t>
+          <t>Ada 291 Ribu Lowongan Kerja di Luar Negeri, Baru Terisi 25%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Wed, 14 Oct 2026 19:47:02 +0700</t>
+          <t>Thu, 15 Oct 2026 16:53:22 +0700</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/11/18/antrean-kendaraan-di-salah-satu-spbu-di-kuta-selatan-badung-bali-selasa-18112025-foto-fabiola-dianiradetikbali-1763454407219_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Koordinator Hilirisasi dan Transisi Energi sekaligus Menteri ESDM Ba</t>
+          <t xml:space="preserve">&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/08/14/menteri-pelindungan-pekerja-migran-indonesia-p2mi-mukhtarudin-1786690624296_169.jpeg?w=360&amp;amp;q=90" /&gt; Kementerian Pelindungan Pekerja Migran Indonesia (P2MI) mencatat ada sekitar 291 ribu peluang kerja di luar negeri sepanjang </t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8707324/bbm-di-bali-langka-picu-antrean-panjang-bahlil-dirut-pertamina-sudah-di-sana</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8708692/ada-291-ribu-lowongan-kerja-di-luar-negeri-baru-terisi-25</t>
         </is>
       </c>
     </row>
@@ -2049,22 +2073,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Mendag Pede Harga Pangan Turun di Akhir Tahun, Ini Alasannya</t>
+          <t>Kurangi Impor Bensin, Bahlil Minta Lahan Tidur Ditanami Singkong</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Wed, 14 Oct 2026 19:30:01 +0700</t>
+          <t>Thu, 15 Oct 2026 16:18:36 +0700</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/14/menteri-perdagangan-mendag-budi-santoso-1791961572700_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Perdagangan (Mendag) Budi Santoso optimistis harga pangan berangsur turun menjelang akhir tahun.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/12/bahlil-lahadalia-1791784854378_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Bahlil Lahadalia dorong penggunaan etanol E20-E50 untuk kurangi impor bensin. Bahan baku etanol dari jagung, singkong, dan tebu.</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8707220/mendag-pede-harga-pangan-turun-di-akhir-tahun-ini-alasannya</t>
+          <t>https://finance.detik.com/energi/d-8708587/kurangi-impor-bensin-bahlil-minta-lahan-tidur-ditanami-singkong</t>
         </is>
       </c>
     </row>
@@ -2076,22 +2100,22 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Bahlil Ungkap Biang Kerok Listrik Padam di Batam: Petir hingga Kelelawar</t>
+          <t>Menag soal Fatwa Kripto: Hari Ini Mungkin Haram, Besok Bisa Jadi Halal</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Wed, 14 Oct 2026 19:16:02 +0700</t>
+          <t>Thu, 15 Oct 2026 16:12:32 +0700</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/04/28/menteri-esdm-bahlil-lahadalia-1777385212721_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Koordinator Bidang Hilirisasi dan Transisi Energi sekaligus Menteri ESDM Bahlil Lahadalia buka suara soal listrik padam di Batam</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/15/menteri-agama-menag-nasaruddin-umar-1792055500316_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Agama (Menag) Nasaruddin Umar menilai fatwa haram Majelis Ulama Indonesia (MUI) terkait aset kripto tidak bersifat permanen.</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8707278/bahlil-ungkap-biang-kerok-listrik-padam-di-batam-petir-hingga-kelelawar</t>
+          <t>https://finance.detik.com/fintech/d-8708586/menag-soal-fatwa-kripto-hari-ini-mungkin-haram-besok-bisa-jadi-halal</t>
         </is>
       </c>
     </row>
@@ -2103,22 +2127,22 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Mendag Harap Tak Ada Impor KRL Bekas Jepang, Minta Pakai Produk RI</t>
+          <t>Bahlil Resmikan Kilang LPG Cilamaya, Mampu Produksi 160 Ton per Hari</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Wed, 14 Oct 2026 19:00:14 +0700</t>
+          <t>Thu, 15 Oct 2026 16:09:06 +0700</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/14/menteri-perdagangan-mendag-budi-santoso-1791961572700_169.jpeg?w=360&amp;amp;q=90" /&gt; Kalau kami sih berharapnya ya produksi dalam negeri kan sudah ada. Jadi, saya berharap tidak ada impor bekas ya, kata Budi.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/06/26/menteri-esdm-1782487092560_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Bahlil meresmikan Kilang LPG Cilamaya di Karawang, mampu produksi 160 ton/hari. Ini langkah optimalkan energi dan kurangi impor LPG Indonesia.</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8707212/mendag-harap-tak-ada-impor-krl-bekas-jepang-minta-pakai-produk-ri</t>
+          <t>https://finance.detik.com/energi/d-8708568/bahlil-resmikan-kilang-lpg-cilamaya-mampu-produksi-160-ton-per-hari</t>
         </is>
       </c>
     </row>
@@ -2130,22 +2154,22 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Husniah Talenrang Dipecat sebagai Bupati Gowa</t>
+          <t>OTT KPK di Klaten, 20 Orang Termasuk Bupati Ditangkap</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Thu, 15 Oct 2026 06:52:20 +0700</t>
+          <t>Thu, 15 Oct 2026 20:06:37 +0700</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Wakil Bupati Gowa, Darmawangsyah Muin ditunjuk sebagai Plt.</t>
+          <t>KPK OTT di Klaten dan Jakarta, sebanyak 20 orang diamankan termasuk Bupati Klaten Hamenang Wajar Ismoyo.</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8313504/husniah-talenrang-dipecat-sebagai-bupati-gowa</t>
+          <t>https://www.liputan6.com/news/read/8314239/ott-kpk-di-klaten-20-orang-termasuk-bupati-ditangkap</t>
         </is>
       </c>
     </row>
@@ -2157,22 +2181,22 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Pemerintah Tambah 70.000 Polisi Hutan, Bantu Cegah Karhutla dan Lindungi Satwa</t>
+          <t>Sosok Hamenang Wajar Ismoyo, Bupati Klaten yang Kena OTT KPK</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Thu, 15 Oct 2026 06:35:27 +0700</t>
+          <t>Thu, 15 Oct 2026 19:57:16 +0700</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Polhut ke depan diharapkan tak hanya menindak, tetapi melakukan upaya pencegahan karhutla dan perlindungan satwa liar.</t>
+          <t>Bupati Klaten Hamenang Wajar Ismoyo terjaring OTT KPK pada Kamis (15/10/2026) pagi. Berikut profil dan perjalanan kariernya.</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8313497/pemerintah-tambah-70000-polisi-hutan-bantu-cegah-karhutla-dan-lindungi-satwa</t>
+          <t>https://www.liputan6.com/news/read/8313895/sosok-hamenang-wajar-ismoyo-bupati-klaten-yang-kena-ott-kpk</t>
         </is>
       </c>
     </row>
@@ -2184,22 +2208,22 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>PKS Ingin Gabungkan Wacana Dapil Nasional dan Sistem Proporsional Terbuka</t>
+          <t>Wiyagus Soroti Peran Forkopimda dalam Antisipasi Kebakaran Hutan Kaltim</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Thu, 15 Oct 2026 06:34:41 +0700</t>
+          <t>Thu, 15 Oct 2026 19:33:14 +0700</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Konsep dari dapil nasional ini adalah untuk mengakomodasi suara pemilih yang tidak terkonversi menjadi kursi DPR RI.</t>
+          <t>Wamendagri juga meminta pemerintah daerah tidak ragu menindak tegas pembakar hutan dan lahan.</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8313496/pks-ingin-gabungkan-wacana-dapil-nasional-dan-sistem-proporsional-terbuka</t>
+          <t>https://www.liputan6.com/news/read/8314218/wiyagus-soroti-peran-forkopimda-dalam-antisipasi-kebakaran-hutan-kaltim</t>
         </is>
       </c>
     </row>
@@ -2211,22 +2235,22 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Febrie Adriansyah yang Bersikukuh Tak Pernah Salah</t>
+          <t>KPK Benarkan OTT Bupati Klaten Hamenang Wajar Ismoyo</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Wed, 14 Oct 2026 22:41:49 +0700</t>
+          <t>Thu, 15 Oct 2026 19:33:37 +0700</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Febrie ingin majelis hakim mengembalikan berkas perkara dan barang bukti kepada jaksa penuntut umum (JPU), serta membebaskannya dari tahanan.</t>
+          <t>Ketua KPK Setyo Budiyanto membenarkan operasi tersebut menyasar Bupati Klaten Hamenang Wajar Ismoyo.</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8313411/febrie-adriansyah-yang-bersikukuh-tak-pernah-salah</t>
+          <t>https://www.liputan6.com/news/read/8314220/kpk-benarkan-ott-bupati-klaten-hamenang-wajar-ismoyo</t>
         </is>
       </c>
     </row>
@@ -2238,22 +2262,22 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Ledakan di Pasar Cimanggis Tewaskan 2 Orang, Dipastikan Bukan Bom</t>
+          <t>Menko Yusril: Beda Tafsir Undang-Undang Bisa Kacaukan Hukum</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Thu, 15 Oct 2026 05:53:42 +0700</t>
+          <t>Thu, 15 Oct 2026 19:03:00 +0700</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Belasan orang juga mengalai luka-luka.</t>
+          <t>Yusril memperingatkan perbedaan tafsir undang-undang di kalangan aparat penegak hukum dapat memicu kekacauan. Dia juga mempertanyakan praktik pembedaan putusan bebas murni dan tidak murni.</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8313491/ledakan-di-pasar-cimanggis-tewaskan-2-orang-dipastikan-bukan-bom</t>
+          <t>https://www.liputan6.com/news/read/8314166/menko-yusril-beda-tafsir-undang-undang-bisa-kacaukan-hukum</t>
         </is>
       </c>
     </row>
@@ -2265,22 +2289,22 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Mengurai Benang Kusut Kebakaran Hutan dan Lahan yang Terus Berulang</t>
+          <t>Australia dan Finlandia Bisa Jadi Rujukan Indonesia Tangani Kebakaran Hutan</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Thu, 15 Oct 2026 05:00:42 +0700</t>
+          <t>Thu, 15 Oct 2026 18:55:00 +0700</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Mengatasi kebakaran hutan dan lahan yang berulang membutuhkan lebih dari sekadar pemadaman api.</t>
+          <t>BRIN menyoroti pentingnya deteksi dini, pemetaan, dan koordinasi antarlembaga.</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8313474/mengurai-benang-kusut-kebakaran-hutan-dan-lahan-yang-terus-berulang</t>
+          <t>https://www.liputan6.com/news/read/8314183/australia-dan-finlandia-bisa-jadi-rujukan-indonesia-tangani-kebakaran-hutan</t>
         </is>
       </c>
     </row>
@@ -2292,22 +2316,22 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Klarifikasi Pemerintah Soal Bantuan Kebakaran Hutan Malaysia dan Jepang</t>
+          <t>BNPB Kaji Penetapan Status Bencana Nasional untuk Kebakaran Hutan</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Thu, 15 Oct 2026 01:28:51 +0700</t>
+          <t>Thu, 15 Oct 2026 18:53:59 +0700</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Kemenko Polkam membantah Indonesia menolak tawaran bantuan Malaysia untuk mengatasi karhutla.</t>
+          <t>Kepala BNPB Kristomei Sianturi akan mengkaji status penanganan karhutla di enam provinsi.</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8313473/klarifikasi-pemerintah-soal-bantuan-kebakaran-hutan-malaysia-dan-jepang</t>
+          <t>https://www.liputan6.com/news/read/8314184/bnpb-kaji-penetapan-status-bencana-nasional-untuk-kebakaran-hutan</t>
         </is>
       </c>
     </row>
@@ -2319,22 +2343,22 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Cairan Pemadam Brasil Diuji di Kebakaran Hutan, Ini Hasil Awalnya</t>
+          <t>Bupati Gowa Husniah Talenrang Diberhentikan, Wabup Jadi Plt</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Thu, 15 Oct 2026 01:19:35 +0700</t>
+          <t>Thu, 15 Oct 2026 18:37:03 +0700</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Cairan pemadam Brasil diharapkan membantu memadamkan api dan mengurangi asap karhutla.</t>
+          <t>Tito Karnavian memberhentikan Bupati Gowa Sitti Husniah Talenrang dan menunjuk Darmawangsyah Muin sebagai Plt.</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8313466/cairan-pemadam-brasil-diuji-di-kebakaran-hutan-ini-hasil-awalnya</t>
+          <t>https://www.liputan6.com/news/read/8314167/bupati-gowa-husniah-talenrang-diberhentikan-wabup-jadi-plt</t>
         </is>
       </c>
     </row>
@@ -2346,22 +2370,22 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Transformasi Digital PERURI, dari Mencetak Rupiah hingga Mengamankan Data Masyarakat</t>
+          <t>6 Kasus Korupsi Bantuan Bencana, dari Donggala hingga BNPB</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Wed, 14 Oct 2026 19:20:09 +0700</t>
+          <t>Thu, 15 Oct 2026 18:21:27 +0700</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Kenali transformasi digital PERURI melalui e-Meterai, Peruri Sign, dan dukungan GovTech untuk menjaga kedaulatan serta kepercayaan masyarakat.</t>
+          <t>Bantuan yang semestinya meringankan korban bencana justru dikorupsi, berikut daftarnya.</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8312930/transformasi-digital-peruri-dari-mencetak-rupiah-hingga-mengamankan-data-masyarakat</t>
+          <t>https://www.liputan6.com/news/read/8314155/6-kasus-korupsi-bantuan-bencana-dari-donggala-hingga-bnpb</t>
         </is>
       </c>
     </row>
@@ -2373,22 +2397,22 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Kejagung Buka Lelang Batu Bara Sitaan Kasus Samin Tan</t>
+          <t>Gempa Magnitudo 4,1 Guncang Bogor</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Wed, 14 Oct 2026 23:52:04 +0700</t>
+          <t>Thu, 15 Oct 2026 18:26:49 +0700</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Lelang batu bara sitaan kasus PT Asmin Koalindo Tuhup digelar secara daring melalui mekanisme open bidding.</t>
+          <t>Gempa bermagnitudo 4,1 mengguncang Bogor pada Kamis sore, getaran dirasakan di Pamijahan dan Kabandungan.</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8313447/kejagung-buka-lelang-batu-bara-sitaan-kasus-samin-tan</t>
+          <t>https://www.liputan6.com/news/read/8314161/gempa-magnitudo-41-guncang-bogor</t>
         </is>
       </c>
     </row>
@@ -2400,22 +2424,22 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Infografis: Rekam Jejak Kebakaran Hutan dan Lahan dalam 6 Tahun</t>
+          <t>Kepala BNPB Baru Janji Bersih-Bersih Internal Usai OTT KPK</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Wed, 14 Oct 2026 23:03:20 +0700</t>
+          <t>Thu, 15 Oct 2026 17:40:47 +0700</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Kalbar, Kalteng, Kalsel, Kaltim, Sumsel, Riau, dan Jambi menjadi wilayah prioritas penanganan karhutla.</t>
+          <t>Kepala BNPB Kristomei Sianturi merespons soal operasi tangkap tangan (OTT) KPK.</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8313425/infografis-rekam-jejak-kebakaran-hutan-dan-lahan-dalam-6-tahun</t>
+          <t>https://www.liputan6.com/news/read/8314116/kepala-bnpb-baru-janji-bersih-bersih-internal-usai-ott-kpk</t>
         </is>
       </c>
     </row>
@@ -2427,22 +2451,22 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Diduga Terkait LPG, Polisi Selidiki Ledakan di Pasar Cimanggis</t>
+          <t>Banjir Kembali Melanda Wilayah Sumatera, Pemulihan Infrastruktur Terganggu</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Wed, 14 Oct 2026 22:53:09 +0700</t>
+          <t>Thu, 15 Oct 2026 17:38:02 +0700</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Polisi masih mendalami penyebab ledakan di sebuah pertokoan di Pasar Cimanggis, Ciputat, Tangerang Selatan.</t>
+          <t>Sejumlah wilayah di Sumatera kembali dilanda banjir saat rehabilitasi dan rekonstruksi pascabencana masih berlangsung.</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8313420/diduga-terkait-lpg-polisi-selidiki-ledakan-di-pasar-cimanggis</t>
+          <t>https://www.liputan6.com/news/read/8314111/banjir-kembali-melanda-wilayah-sumatera-pemulihan-infrastruktur-terganggu</t>
         </is>
       </c>
     </row>
@@ -2454,22 +2478,22 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Gegana Tangani Ledakan di Pasar Cimanggis</t>
+          <t>Strategi Polisi Gerebek Kos Diduga Sarang Narkoba di Kampung Ambon</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Wed, 14 Oct 2026 22:45:14 +0700</t>
+          <t>Thu, 15 Oct 2026 17:21:04 +0700</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Polisi masih melakukan evakuasi, sterilisasi, dan olah TKP setelah ledakan terjadi di kawasan Pasar Cimanggis, Tangsel.</t>
+          <t>Penggerebekan kos di Kampung Ambon berujung pada pengamanan tujuh orang.</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8313410/gegana-tangani-ledakan-di-pasar-cimanggis</t>
+          <t>https://www.liputan6.com/news/read/8314100/strategi-polisi-gerebek-kos-diduga-sarang-narkoba-di-kampung-ambon</t>
         </is>
       </c>
     </row>
@@ -2481,22 +2505,22 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Hotspot Sumsel Naik 92 Persen, Begini Aksi Kemenhut</t>
+          <t>Rekam Jejak Maulana Bungaran, Wamen Imipas Baru</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Wed, 14 Oct 2026 22:13:45 +0700</t>
+          <t>Thu, 15 Oct 2026 17:14:43 +0700</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Kemenhut menerapkan pemindahan personel untuk memperkuat penanganan karhutla</t>
+          <t>Maulana Bungaran pernah aktif di Partai Gerindra dan memiliki rekam jejak kuat sebagai pengacara.</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8313400/hotspot-sumsel-naik-92-persen-begini-aksi-kemenhut</t>
+          <t>https://www.liputan6.com/news/read/8314065/rekam-jejak-maulana-bungaran-wamen-imipas-baru</t>
         </is>
       </c>
     </row>
@@ -2508,22 +2532,22 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Ledakan di Pasar Cimanggis Ciputat, 8 Orang Dilarikan ke RS</t>
+          <t>Rekam Jejak Jenderal Tandyo Budi, dari Wakil Panglima Jadi KSAD</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Wed, 14 Oct 2026 22:03:16 +0700</t>
+          <t>Thu, 15 Oct 2026 16:16:36 +0700</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Saat ini fokus utama yaitu menyelamatkan korban akibat ledakan tersebut.</t>
+          <t>Tandyo menggantikan Maruli pada saat bersamaan dilantik Prabowo menjadi Wakil Panglima TNI dan Kepala Badan Nasional Pengelola Perbatasan dan Daerah Terpencil.</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8313396/ledakan-di-pasar-cimanggis-ciputat-8-orang-dilarikan-ke-rs</t>
+          <t>https://www.liputan6.com/news/read/8314028/rekam-jejak-jenderal-tandyo-budi-dari-wakil-panglima-jadi-ksad</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data pasar & berita - 2026-10-15 23:56 UTC
</commit_message>
<xml_diff>
--- a/data/market_news_latest.xlsx
+++ b/data/market_news_latest.xlsx
@@ -422,7 +422,7 @@
     <col width="26" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
   </cols>
@@ -487,20 +487,20 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>5863.7798</v>
+        <v>5943.0239</v>
       </c>
       <c r="F2" t="n">
-        <v>-79.2441</v>
+        <v>17.0479</v>
       </c>
       <c r="G2" t="n">
-        <v>-1.33</v>
+        <v>0.29</v>
       </c>
       <c r="H2" t="n">
-        <v>0</v>
+        <v>270876900</v>
       </c>
     </row>
     <row r="3">
@@ -521,20 +521,20 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>7718.9399</v>
+        <v>7744.0601</v>
       </c>
       <c r="F3" t="n">
-        <v>-86.5103</v>
+        <v>25.1201</v>
       </c>
       <c r="G3" t="n">
-        <v>-1.11</v>
+        <v>0.33</v>
       </c>
       <c r="H3" t="n">
-        <v>5955580000</v>
+        <v>3428090000</v>
       </c>
     </row>
     <row r="4">
@@ -555,20 +555,20 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>51621.4805</v>
+        <v>52177.6914</v>
       </c>
       <c r="F4" t="n">
-        <v>-48.6211</v>
+        <v>556.2109</v>
       </c>
       <c r="G4" t="n">
-        <v>-0.09</v>
+        <v>1.08</v>
       </c>
       <c r="H4" t="n">
-        <v>442520000</v>
+        <v>500690219</v>
       </c>
     </row>
     <row r="5">
@@ -589,20 +589,20 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>26692.8691</v>
+        <v>26713.0254</v>
       </c>
       <c r="F5" t="n">
-        <v>-511.5117</v>
+        <v>20.1562</v>
       </c>
       <c r="G5" t="n">
-        <v>-1.88</v>
+        <v>0.08</v>
       </c>
       <c r="H5" t="n">
-        <v>8568280000</v>
+        <v>9708091000</v>
       </c>
     </row>
     <row r="6">
@@ -623,20 +623,20 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>64425.9492</v>
+        <v>67744.28909999999</v>
       </c>
       <c r="F6" t="n">
-        <v>-3318.3398</v>
+        <v>-33.2344</v>
       </c>
       <c r="G6" t="n">
-        <v>-4.9</v>
+        <v>-0.05</v>
       </c>
       <c r="H6" t="n">
-        <v>0</v>
+        <v>152100000</v>
       </c>
     </row>
     <row r="7">
@@ -657,20 +657,20 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>24062.7207</v>
+        <v>24314.1699</v>
       </c>
       <c r="F7" t="n">
-        <v>-251.4492</v>
+        <v>-31.0508</v>
       </c>
       <c r="G7" t="n">
-        <v>-1.03</v>
+        <v>-0.13</v>
       </c>
       <c r="H7" t="n">
-        <v>0</v>
+        <v>2804100000</v>
       </c>
     </row>
     <row r="8">
@@ -694,15 +694,9 @@
           <t>2026-10-15</t>
         </is>
       </c>
-      <c r="E8" t="n">
-        <v>3707.4761</v>
-      </c>
-      <c r="F8" t="n">
-        <v>-59.751</v>
-      </c>
-      <c r="G8" t="n">
-        <v>-1.59</v>
-      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
       <c r="H8" t="n">
         <v>3771678644</v>
       </c>
@@ -725,20 +719,20 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>10832.4697</v>
+        <v>10724.9004</v>
       </c>
       <c r="F9" t="n">
-        <v>107.5693</v>
+        <v>74.6006</v>
       </c>
       <c r="G9" t="n">
-        <v>1</v>
+        <v>0.7</v>
       </c>
       <c r="H9" t="n">
-        <v>0</v>
+        <v>610957900</v>
       </c>
     </row>
     <row r="10">
@@ -759,20 +753,20 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>25261.1094</v>
+        <v>25298.6094</v>
       </c>
       <c r="F10" t="n">
-        <v>-37.5</v>
+        <v>38.709</v>
       </c>
       <c r="G10" t="n">
-        <v>-0.15</v>
+        <v>0.15</v>
       </c>
       <c r="H10" t="n">
-        <v>0</v>
+        <v>56498200</v>
       </c>
     </row>
     <row r="11">
@@ -793,20 +787,20 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>5403.5</v>
+        <v>5423.3301</v>
       </c>
       <c r="F11" t="n">
-        <v>-19.8301</v>
+        <v>-7.1699</v>
       </c>
       <c r="G11" t="n">
-        <v>-0.37</v>
+        <v>-0.13</v>
       </c>
       <c r="H11" t="n">
-        <v>0</v>
+        <v>256903700</v>
       </c>
     </row>
     <row r="12">
@@ -831,13 +825,13 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>17943</v>
+        <v>17823.6992</v>
       </c>
       <c r="F12" t="n">
-        <v>76.5</v>
+        <v>-42.8008</v>
       </c>
       <c r="G12" t="n">
-        <v>0.43</v>
+        <v>-0.24</v>
       </c>
       <c r="H12" t="n">
         <v>0</v>
@@ -865,13 +859,13 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>102.116</v>
+        <v>102.046</v>
       </c>
       <c r="F13" t="n">
-        <v>-0.434</v>
+        <v>-0.504</v>
       </c>
       <c r="G13" t="n">
-        <v>-0.42</v>
+        <v>-0.49</v>
       </c>
       <c r="H13" t="n">
         <v>0</v>
@@ -895,17 +889,17 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>157.853</v>
+        <v>158.13</v>
       </c>
       <c r="F14" t="n">
-        <v>-0.469</v>
+        <v>0.173</v>
       </c>
       <c r="G14" t="n">
-        <v>-0.3</v>
+        <v>0.11</v>
       </c>
       <c r="H14" t="n">
         <v>0</v>
@@ -933,13 +927,13 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>0.5054</v>
+        <v>0.5089</v>
       </c>
       <c r="F15" t="n">
-        <v>-0.0136</v>
+        <v>-0.0101</v>
       </c>
       <c r="G15" t="n">
-        <v>-2.62</v>
+        <v>-1.95</v>
       </c>
       <c r="H15" t="n">
         <v>0</v>
@@ -967,13 +961,13 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>0.5391</v>
+        <v>0.5429</v>
       </c>
       <c r="F16" t="n">
-        <v>-0.0134</v>
+        <v>-0.009599999999999999</v>
       </c>
       <c r="G16" t="n">
-        <v>-2.43</v>
+        <v>-1.74</v>
       </c>
       <c r="H16" t="n">
         <v>0</v>
@@ -1001,13 +995,13 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>0.4077</v>
+        <v>0.4088</v>
       </c>
       <c r="F17" t="n">
-        <v>-0.0008</v>
+        <v>0.0003</v>
       </c>
       <c r="G17" t="n">
-        <v>-0.2</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="H17" t="n">
         <v>0</v>
@@ -1031,20 +1025,20 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>78.89</v>
+        <v>79.97</v>
       </c>
       <c r="F18" t="n">
-        <v>0.52</v>
+        <v>1.08</v>
       </c>
       <c r="G18" t="n">
-        <v>0.66</v>
+        <v>1.37</v>
       </c>
       <c r="H18" t="n">
-        <v>50909600</v>
+        <v>86228050</v>
       </c>
     </row>
     <row r="19">
@@ -1065,20 +1059,20 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>76.81</v>
+        <v>77.13</v>
       </c>
       <c r="F19" t="n">
-        <v>-0.28</v>
+        <v>0.32</v>
       </c>
       <c r="G19" t="n">
-        <v>-0.36</v>
+        <v>0.42</v>
       </c>
       <c r="H19" t="n">
-        <v>63579700</v>
+        <v>80514689</v>
       </c>
     </row>
     <row r="20">
@@ -1103,16 +1097,16 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>4165.2998</v>
+        <v>4178.2998</v>
       </c>
       <c r="F20" t="n">
-        <v>57.3999</v>
+        <v>70.3999</v>
       </c>
       <c r="G20" t="n">
-        <v>1.4</v>
+        <v>1.71</v>
       </c>
       <c r="H20" t="n">
-        <v>91221</v>
+        <v>3066</v>
       </c>
     </row>
     <row r="21">
@@ -1137,16 +1131,16 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>94.18000000000001</v>
+        <v>96.18000000000001</v>
       </c>
       <c r="F21" t="n">
-        <v>-0.91</v>
+        <v>1.09</v>
       </c>
       <c r="G21" t="n">
-        <v>-0.96</v>
+        <v>1.15</v>
       </c>
       <c r="H21" t="n">
-        <v>82304</v>
+        <v>2138</v>
       </c>
     </row>
     <row r="22">
@@ -1171,16 +1165,16 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>104.59</v>
+        <v>105.74</v>
       </c>
       <c r="F22" t="n">
-        <v>-1.47</v>
+        <v>-0.32</v>
       </c>
       <c r="G22" t="n">
-        <v>-1.39</v>
+        <v>-0.3</v>
       </c>
       <c r="H22" t="n">
-        <v>24050</v>
+        <v>209</v>
       </c>
     </row>
     <row r="23">
@@ -1205,16 +1199,16 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>6.5425</v>
+        <v>6.5515</v>
       </c>
       <c r="F23" t="n">
-        <v>-0.06900000000000001</v>
+        <v>-0.06</v>
       </c>
       <c r="G23" t="n">
-        <v>-1.04</v>
+        <v>-0.91</v>
       </c>
       <c r="H23" t="n">
-        <v>36101</v>
+        <v>247</v>
       </c>
     </row>
     <row r="24">
@@ -1235,20 +1229,20 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="E24" t="n">
-        <v>64.39</v>
+        <v>63.96</v>
       </c>
       <c r="F24" t="n">
-        <v>-1.35</v>
+        <v>-0.43</v>
       </c>
       <c r="G24" t="n">
-        <v>-2.05</v>
+        <v>-0.67</v>
       </c>
       <c r="H24" t="n">
-        <v>21169200</v>
+        <v>23159834</v>
       </c>
     </row>
     <row r="25">
@@ -1273,13 +1267,13 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>17.47</v>
+        <v>16.46</v>
       </c>
       <c r="F25" t="n">
-        <v>0.6</v>
+        <v>-0.41</v>
       </c>
       <c r="G25" t="n">
-        <v>3.56</v>
+        <v>-2.43</v>
       </c>
       <c r="H25" t="n">
         <v>0</v>
@@ -1307,16 +1301,16 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>80418.07030000001</v>
+        <v>82135.75</v>
       </c>
       <c r="F26" t="n">
-        <v>-1144.4219</v>
+        <v>573.2578</v>
       </c>
       <c r="G26" t="n">
-        <v>-1.4</v>
+        <v>0.7</v>
       </c>
       <c r="H26" t="n">
-        <v>40395726848</v>
+        <v>41975259136</v>
       </c>
     </row>
     <row r="27">
@@ -1749,22 +1743,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>10.070 Kopdes Mulai Operasi Hari Ini</t>
+          <t>Ritel Modern Tak Wajib Lagi Jual 30% Produk UMKM</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Thu, 15 Oct 2026 20:00:41 +0700</t>
+          <t>Fri, 16 Oct 2026 06:25:00 +0700</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/21/kopdes-merah-putih-bersiap-operasional-23-ribu-bangunan-telah-rampung-1789986171380_169.jpeg?w=360&amp;amp;q=90" /&gt; Distribusi pasokan pangan untuk operasional Koperasi Desa/Kelurahan Merah Putih (KDKMP) dipastikan sudah siap.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2023/04/03/ilustrasi-belanja-di-alfamart_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Perdagangan Budi Santoso menyampaikan pemerintah tak lagi mewajibkan produk usaha mikro kecil dan menengah (UMKM) memenuhi porsi 30% di ritel modern.</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8709020/10-070-kopdes-mulai-operasi-hari-ini</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8709142/ritel-modern-tak-wajib-lagi-jual-30-produk-umkm</t>
         </is>
       </c>
     </row>
@@ -1776,22 +1770,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>DJP Siapkan Insentif Pajak buat BUMN, Ini Bocorannya</t>
+          <t>Serapan Tenaga Kerja Menyusut Meski Ekonomi Tumbuh</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Thu, 15 Oct 2026 19:30:12 +0700</t>
+          <t>Fri, 16 Oct 2026 05:55:00 +0700</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/15/direktur-jenderal-pajak-djp-bimo-wijayanto-1792062697952_169.jpeg?w=360&amp;amp;q=90" /&gt; Direktorat Jenderal Pajak (DJP) disebut telah menyiapkan aturan tentang insentif pajak bagi Badan Usaha Milik Negara (BUMN) yang melakukan aksi </t>
+          <t xml:space="preserve">&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/03/berburu-lowongan-kerja-di-ragunan-career-fest-jadi-harapan-1788414921572_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Perindustrian (Menperin) Muhammad Sarmuji menyoroti semakin terbatasnya penciptaan lapangan kerja di tengah pertumbuhan </t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8708986/djp-siapkan-insentif-pajak-buat-bumn-ini-bocorannya</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8709116/serapan-tenaga-kerja-menyusut-meski-ekonomi-tumbuh</t>
         </is>
       </c>
     </row>
@@ -1803,22 +1797,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>KRL Kerap Gangguan, INKA Minta Maaf</t>
+          <t>Pertamina Patra Niaga Ungkap Layanan SPBU di Bali Berangsur Pulih</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Thu, 15 Oct 2026 19:00:11 +0700</t>
+          <t>Thu, 15 Oct 2026 22:35:01 +0700</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/14/krl-inka-gangguan-penumpang-di-stasiun-pasar-minggu-pindah-krl-dok-istimewa-1791983235827_169.jpeg?w=360&amp;amp;q=90" /&gt; PT Industri Kereta Api (Persero) atau INKA buka suara soal beberapa rangkaian KRL CLI-225 yang mengalami masala</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/15/pertamina-patra-niaga-1792078465155.jpeg?w=360&amp;amp;q=90" /&gt; PT Pertamina Patra Niaga memperkuat pasokan dan distribusi BBM di Bali dengan penambahan suplai dan operasional 24 jam.</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/infrastruktur/d-8708975/krl-kerap-gangguan-inka-minta-maaf</t>
+          <t>https://finance.detik.com/energi/d-8709219/pertamina-patra-niaga-ungkap-layanan-spbu-di-bali-berangsur-pulih</t>
         </is>
       </c>
     </row>
@@ -1830,22 +1824,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Penerimaan Pajak RI Segitu-gitu Aja, DJP Buka Suara</t>
+          <t>Pariwisata Andalan RI Genjot Ekonomi, Segini Kontribusinya</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Thu, 15 Oct 2026 18:30:45 +0700</t>
+          <t>Thu, 15 Oct 2026 22:25:00 +0700</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/15/direktur-jenderal-pajak-djp-bimo-wijayanto-1792062697871_169.jpeg?w=360&amp;amp;q=90" /&gt; Direktur Jenderal Pajak (DJP) Bimo Wijayanto, mengatakan baru sekali dalam sejarah pemerintah berani menargetkan penerimaan pajak 9% dari PDB da</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2019/03/18/c12187aa-58c0-47af-adc7-725abd129e54_169.jpeg?w=360&amp;amp;q=90" /&gt; Pemerintah terus menjaga momentum pertumbuhan pariwisata Indonesia sekaligus memperluas peluang usaha dan investasi.</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8708906/penerimaan-pajak-ri-segitu-gitu-aja-djp-buka-suara</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8709204/pariwisata-andalan-ri-genjot-ekonomi-segini-kontribusinya</t>
         </is>
       </c>
     </row>
@@ -1857,22 +1851,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>MR.D.I.Y., Kemenperin &amp;amp; CIMB Niaga Dorong IKM Perkuat Bisnis Berkelanjutan</t>
+          <t>Taspen Ikut Arahan Pemerintah soal Koperasi Jadi Penyalur Dana Pensiunan</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Thu, 15 Oct 2026 18:15:54 +0700</t>
+          <t>Thu, 15 Oct 2026 21:55:59 +0700</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/15/mrdiy-kemenperin-cimb-niaga-dorong-ikm-perkuat-bisnis-berkelanjutan-1792062894911.jpeg?w=360&amp;amp;q=90" /&gt; PT Daya Intiguna Yasa Tbk dan CIMB Niaga gelar pelatihan manajemen keuangan untuk 100 IKM. Fokus pada keberlanjutan dan pen</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/05/21/ilustrasi-layanan-taspen-1747810258404_169.jpeg?w=360&amp;amp;q=90" /&gt; PT Taspen (Persero) mengikuti arahan pemerintah terkait penyaluran dana pensiun aparatur sipil negara (ASN).</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8708914/mr-d-i-y-kemenperin-cimb-niaga-dorong-ikm-perkuat-bisnis-berkelanjutan</t>
+          <t>https://finance.detik.com/moneter/d-8709195/taspen-ikut-arahan-pemerintah-soal-koperasi-jadi-penyalur-dana-pensiunan</t>
         </is>
       </c>
     </row>
@@ -1884,22 +1878,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Perang Arab Saudi Vs Houthi, Garuda Alihkan Rute-Tunda Penerbangan</t>
+          <t>Genjot Pasokan di Bali, Pertamina Ingatkan Jangan Beli Pertalite buat Dijual Lagi</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Thu, 15 Oct 2026 18:03:46 +0700</t>
+          <t>Thu, 15 Oct 2026 21:47:06 +0700</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/07/19/pesawat-garuda-indonesia-1752916632356_169.jpeg?w=360&amp;amp;q=90" /&gt; Situasi geopolitik di kawasan Timur Tengah berpotensi berdampak pada operasi penerbangan dari dan menuju Arab Saudi.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/14/pertamina-genjot-pasokan-bbm-ke-bali-1791990343502_169.jpeg?w=360&amp;amp;q=90" /&gt; PT Pertamina Patra Niaga terus menggenjot penyaluran bahan bakar minyak (BBM) ke wilayah Bali</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8708883/perang-arab-saudi-vs-houthi-garuda-alihkan-rute-tunda-penerbangan</t>
+          <t>https://finance.detik.com/energi/d-8709161/genjot-pasokan-di-bali-pertamina-ingatkan-jangan-beli-pertalite-buat-dijual-lagi</t>
         </is>
       </c>
     </row>
@@ -1911,22 +1905,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Dilantik Jadi Wamentan, Alim Setiawan Dapat Tugas Apa dari Prabowo?</t>
+          <t>Danantara Siapkan Rp 1,7 Triliun/ Tahun buat Kesehatan, Pendidikan, Sanitasi</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Thu, 15 Oct 2026 17:29:58 +0700</t>
+          <t>Thu, 15 Oct 2026 20:55:00 +0700</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/15/ipb-1792047319407_169.jpeg?w=360&amp;amp;q=90" /&gt; Presiden Prabowo Subianto melantik Alim Setiawan Slamet menjadi Wakil Menteri Pertanian.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/07/01/wisma-danantara-indonesia-1751345496674_169.jpeg?w=360&amp;amp;q=90" /&gt; Danantara akan mengalokasikan US$ 100 juta atau Rp 1,7 triliun (kurs Rp 17.900) setiap tahun untuk mendukung program sosial melalui Danantara Trust.</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8708763/dilantik-jadi-wamentan-alim-setiawan-dapat-tugas-apa-dari-prabowo</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8709105/danantara-siapkan-rp-1-7-triliun-tahun-buat-kesehatan-pendidikan-sanitasi</t>
         </is>
       </c>
     </row>
@@ -1938,22 +1932,22 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Ada Harta Karun di Bawah Jakarta! Terungkap Saat Gali Jalur MRT</t>
+          <t>DJP Targetkan Setoran Pajak Digital Naik Sampai 50%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Thu, 15 Oct 2026 17:24:29 +0700</t>
+          <t>Thu, 15 Oct 2026 20:30:47 +0700</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/15/harta-karun-mrt-1792059689770_169.jpeg?w=360&amp;amp;q=90" /&gt; Proyek MRT Jakarta Fase 2 menemukan ribuan artefak sejarah, termasuk keramik kuno dan saluran air terakota, menantang proses konstruksi dan pelestarian budaya.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2024/12/11/ilustrasi-pajak_169.jpeg?w=360&amp;amp;q=90" /&gt; Direktur Jenderal Pajak Bimo Wijayanto memperkirakan penerimaan pajak dari aktivitas ekonomi digital bisa tumbuh 50%, menjadi sekitar Rp 16 triliun.</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/infrastruktur/d-8708754/ada-harta-karun-di-bawah-jakarta-terungkap-saat-gali-jalur-mrt</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8709031/djp-targetkan-setoran-pajak-digital-naik-sampai-50</t>
         </is>
       </c>
     </row>
@@ -1965,22 +1959,22 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Seharian di Zona Merah, IHSG Ditutup di Level 5.863</t>
+          <t>Mau Investasi Bitcoin? Pahami Cara Beli, Strategi, dan Risiko Kripto</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Thu, 15 Oct 2026 17:09:50 +0700</t>
+          <t>Thu, 15 Oct 2026 20:29:22 +0700</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/05/18/ihsg-anjlok-ke-zona-merah-bursa-saham-melemah-tajam-1779098741262_169.jpeg?w=360&amp;amp;q=90" /&gt; Indeks Harga Saham Gabungan (IHSG) ditutup di zona merah sore ini.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/15/magnific-1792070910370.jpeg?w=360&amp;amp;q=90" /&gt; Bitcoin semakin populer di kalangan investor. Pelajari cara berinvestasi, pilih platform seperti Pintu, dan terapkan strategi menabung untuk hasil optimal.</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/bursa-dan-valas/d-8708712/seharian-di-zona-merah-ihsg-ditutup-di-level-5-863</t>
+          <t>https://finance.detik.com/fintech/d-8709107/mau-investasi-bitcoin-pahami-cara-beli-strategi-dan-risiko-kripto</t>
         </is>
       </c>
     </row>
@@ -1992,22 +1986,22 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Subsidi LPG Bengkak dari Rp 87 T, Kini Tembus Rp 100 T</t>
+          <t>10.070 Kopdes Mulai Operasi Hari Ini</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Thu, 15 Oct 2026 17:04:34 +0700</t>
+          <t>Thu, 15 Oct 2026 20:00:41 +0700</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/14/bahlil-lahadalia-rolandodetikcom-1791978307056_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Bahlil mengungkap subsidi LPG membengkak di atas Rp 100 triliun saat ICP naik. Pemerintah kembangkan CNG 3 kg untuk kurangi impor LPG.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/21/kopdes-merah-putih-bersiap-operasional-23-ribu-bangunan-telah-rampung-1789986171380_169.jpeg?w=360&amp;amp;q=90" /&gt; Distribusi pasokan pangan untuk operasional Koperasi Desa/Kelurahan Merah Putih (KDKMP) dipastikan sudah siap.</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8708710/subsidi-lpg-bengkak-dari-rp-87-t-kini-tembus-rp-100-t</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8709020/10-070-kopdes-mulai-operasi-hari-ini</t>
         </is>
       </c>
     </row>
@@ -2019,22 +2013,22 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Wamenkeu Tegaskan Kripto Bukan Mata Uang, Tetap Kena Pajak</t>
+          <t>DJP Siapkan Insentif Pajak buat BUMN, Ini Bocorannya</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Thu, 15 Oct 2026 16:57:39 +0700</t>
+          <t>Thu, 15 Oct 2026 19:30:12 +0700</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2022/07/11/ilustrasi-aset-kripto-bitcoin-dan-xrp_169.jpeg?w=360&amp;amp;q=90" /&gt; Wakil Menteri Keuangan (Wamenkeu) Nurkholisoh Ibnu Aman menegaskan, aset kripto bukan alat pembayaran yang sah di Indonesia.</t>
+          <t xml:space="preserve">&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/15/direktur-jenderal-pajak-djp-bimo-wijayanto-1792062697952_169.jpeg?w=360&amp;amp;q=90" /&gt; Direktorat Jenderal Pajak (DJP) disebut telah menyiapkan aturan tentang insentif pajak bagi Badan Usaha Milik Negara (BUMN) yang melakukan aksi </t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/fintech/d-8708701/wamenkeu-tegaskan-kripto-bukan-mata-uang-tetap-kena-pajak</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8708986/djp-siapkan-insentif-pajak-buat-bumn-ini-bocorannya</t>
         </is>
       </c>
     </row>
@@ -2046,22 +2040,22 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Ada 291 Ribu Lowongan Kerja di Luar Negeri, Baru Terisi 25%</t>
+          <t>KRL Kerap Gangguan, INKA Minta Maaf</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Thu, 15 Oct 2026 16:53:22 +0700</t>
+          <t>Thu, 15 Oct 2026 19:00:11 +0700</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/08/14/menteri-pelindungan-pekerja-migran-indonesia-p2mi-mukhtarudin-1786690624296_169.jpeg?w=360&amp;amp;q=90" /&gt; Kementerian Pelindungan Pekerja Migran Indonesia (P2MI) mencatat ada sekitar 291 ribu peluang kerja di luar negeri sepanjang </t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/14/krl-inka-gangguan-penumpang-di-stasiun-pasar-minggu-pindah-krl-dok-istimewa-1791983235827_169.jpeg?w=360&amp;amp;q=90" /&gt; PT Industri Kereta Api (Persero) atau INKA buka suara soal beberapa rangkaian KRL CLI-225 yang mengalami masala</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8708692/ada-291-ribu-lowongan-kerja-di-luar-negeri-baru-terisi-25</t>
+          <t>https://finance.detik.com/infrastruktur/d-8708975/krl-kerap-gangguan-inka-minta-maaf</t>
         </is>
       </c>
     </row>
@@ -2073,22 +2067,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Kurangi Impor Bensin, Bahlil Minta Lahan Tidur Ditanami Singkong</t>
+          <t>Penerimaan Pajak RI Segitu-gitu Aja, DJP Buka Suara</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Thu, 15 Oct 2026 16:18:36 +0700</t>
+          <t>Thu, 15 Oct 2026 18:30:45 +0700</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/12/bahlil-lahadalia-1791784854378_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Bahlil Lahadalia dorong penggunaan etanol E20-E50 untuk kurangi impor bensin. Bahan baku etanol dari jagung, singkong, dan tebu.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/15/direktur-jenderal-pajak-djp-bimo-wijayanto-1792062697871_169.jpeg?w=360&amp;amp;q=90" /&gt; Direktur Jenderal Pajak (DJP) Bimo Wijayanto, mengatakan baru sekali dalam sejarah pemerintah berani menargetkan penerimaan pajak 9% dari PDB da</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8708587/kurangi-impor-bensin-bahlil-minta-lahan-tidur-ditanami-singkong</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8708906/penerimaan-pajak-ri-segitu-gitu-aja-djp-buka-suara</t>
         </is>
       </c>
     </row>
@@ -2100,22 +2094,22 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Menag soal Fatwa Kripto: Hari Ini Mungkin Haram, Besok Bisa Jadi Halal</t>
+          <t>MR.D.I.Y., Kemenperin &amp;amp; CIMB Niaga Dorong IKM Perkuat Bisnis Berkelanjutan</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Thu, 15 Oct 2026 16:12:32 +0700</t>
+          <t>Thu, 15 Oct 2026 18:15:54 +0700</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/15/menteri-agama-menag-nasaruddin-umar-1792055500316_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Agama (Menag) Nasaruddin Umar menilai fatwa haram Majelis Ulama Indonesia (MUI) terkait aset kripto tidak bersifat permanen.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/15/mrdiy-kemenperin-cimb-niaga-dorong-ikm-perkuat-bisnis-berkelanjutan-1792062894911.jpeg?w=360&amp;amp;q=90" /&gt; PT Daya Intiguna Yasa Tbk dan CIMB Niaga gelar pelatihan manajemen keuangan untuk 100 IKM. Fokus pada keberlanjutan dan pen</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/fintech/d-8708586/menag-soal-fatwa-kripto-hari-ini-mungkin-haram-besok-bisa-jadi-halal</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8708914/mr-d-i-y-kemenperin-cimb-niaga-dorong-ikm-perkuat-bisnis-berkelanjutan</t>
         </is>
       </c>
     </row>
@@ -2127,22 +2121,22 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Bahlil Resmikan Kilang LPG Cilamaya, Mampu Produksi 160 Ton per Hari</t>
+          <t>Perang Arab Saudi Vs Houthi, Garuda Alihkan Rute-Tunda Penerbangan</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Thu, 15 Oct 2026 16:09:06 +0700</t>
+          <t>Thu, 15 Oct 2026 18:03:46 +0700</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/06/26/menteri-esdm-1782487092560_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Bahlil meresmikan Kilang LPG Cilamaya di Karawang, mampu produksi 160 ton/hari. Ini langkah optimalkan energi dan kurangi impor LPG Indonesia.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/07/19/pesawat-garuda-indonesia-1752916632356_169.jpeg?w=360&amp;amp;q=90" /&gt; Situasi geopolitik di kawasan Timur Tengah berpotensi berdampak pada operasi penerbangan dari dan menuju Arab Saudi.</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8708568/bahlil-resmikan-kilang-lpg-cilamaya-mampu-produksi-160-ton-per-hari</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8708883/perang-arab-saudi-vs-houthi-garuda-alihkan-rute-tunda-penerbangan</t>
         </is>
       </c>
     </row>
@@ -2154,22 +2148,22 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>OTT KPK di Klaten, 20 Orang Termasuk Bupati Ditangkap</t>
+          <t>Cerita Menkum Supratman Saat Diminta Prabowo Pangkas Aturan Berbelit</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Thu, 15 Oct 2026 20:06:37 +0700</t>
+          <t>Fri, 16 Oct 2026 06:37:26 +0700</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>KPK OTT di Klaten dan Jakarta, sebanyak 20 orang diamankan termasuk Bupati Klaten Hamenang Wajar Ismoyo.</t>
+          <t>Menkum mengaku telah memangkas 195 Permenkum jadi 34.</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8314239/ott-kpk-di-klaten-20-orang-termasuk-bupati-ditangkap</t>
+          <t>https://www.liputan6.com/news/read/8314405/cerita-menkum-supratman-saat-diminta-prabowo-pangkas-aturan-berbelit</t>
         </is>
       </c>
     </row>
@@ -2181,22 +2175,22 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Sosok Hamenang Wajar Ismoyo, Bupati Klaten yang Kena OTT KPK</t>
+          <t>Menteri Imipas Sanksi Pegawai Terlibat Jual Beli Remisi</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Thu, 15 Oct 2026 19:57:16 +0700</t>
+          <t>Fri, 16 Oct 2026 06:32:28 +0700</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Bupati Klaten Hamenang Wajar Ismoyo terjaring OTT KPK pada Kamis (15/10/2026) pagi. Berikut profil dan perjalanan kariernya.</t>
+          <t>Agus belum merinci jenis sanksi yang dijatuhkan.</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8313895/sosok-hamenang-wajar-ismoyo-bupati-klaten-yang-kena-ott-kpk</t>
+          <t>https://www.liputan6.com/news/read/8314404/menteri-imipas-sanksi-pegawai-terlibat-jual-beli-remisi</t>
         </is>
       </c>
     </row>
@@ -2208,22 +2202,22 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Wiyagus Soroti Peran Forkopimda dalam Antisipasi Kebakaran Hutan Kaltim</t>
+          <t>Polisi Tetapkan 9 Tersangka TPPO ABK KM Maulana 23</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Thu, 15 Oct 2026 19:33:14 +0700</t>
+          <t>Fri, 16 Oct 2026 06:03:49 +0700</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Wamendagri juga meminta pemerintah daerah tidak ragu menindak tegas pembakar hutan dan lahan.</t>
+          <t>Penetapan tersebut dilakukan setelah penyidik menjalankan serangkaian proses penyelidikan dan penyidikan.</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8314218/wiyagus-soroti-peran-forkopimda-dalam-antisipasi-kebakaran-hutan-kaltim</t>
+          <t>https://www.liputan6.com/news/read/8314399/polisi-tetapkan-9-tersangka-tppo-abk-km-maulana-23</t>
         </is>
       </c>
     </row>
@@ -2235,22 +2229,22 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>KPK Benarkan OTT Bupati Klaten Hamenang Wajar Ismoyo</t>
+          <t>Bongkar Pasang Kabinet Prabowo untuk Kedelapan Kalinya</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Thu, 15 Oct 2026 19:33:37 +0700</t>
+          <t>Fri, 16 Oct 2026 06:00:00 +0700</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Ketua KPK Setyo Budiyanto membenarkan operasi tersebut menyasar Bupati Klaten Hamenang Wajar Ismoyo.</t>
+          <t>Dalam reshuffle kali ini, jajaran pimpinan strategis di sektor pertahanan, keamanan, kementerian, hingga lembaga nonkementerian mengalami penataan ulang.</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8314220/kpk-benarkan-ott-bupati-klaten-hamenang-wajar-ismoyo</t>
+          <t>https://www.liputan6.com/news/read/8314365/bongkar-pasang-kabinet-prabowo-untuk-kedelapan-kalinya</t>
         </is>
       </c>
     </row>
@@ -2262,22 +2256,22 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Menko Yusril: Beda Tafsir Undang-Undang Bisa Kacaukan Hukum</t>
+          <t>Menko Yusril: Terlalu Banyak Peraturan Kita Buat, Bikin Pusing</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Thu, 15 Oct 2026 19:03:00 +0700</t>
+          <t>Fri, 16 Oct 2026 05:30:55 +0700</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Yusril memperingatkan perbedaan tafsir undang-undang di kalangan aparat penegak hukum dapat memicu kekacauan. Dia juga mempertanyakan praktik pembedaan putusan bebas murni dan tidak murni.</t>
+          <t>Alih-alih menyelesaikan persoalan, aturan yang terus bertambah justru bisa membuat pelaksanaannya semakin rumit.</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8314166/menko-yusril-beda-tafsir-undang-undang-bisa-kacaukan-hukum</t>
+          <t>https://www.liputan6.com/news/read/8314394/menko-yusril-terlalu-banyak-peraturan-kita-buat-bikin-pusing</t>
         </is>
       </c>
     </row>
@@ -2289,22 +2283,22 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Australia dan Finlandia Bisa Jadi Rujukan Indonesia Tangani Kebakaran Hutan</t>
+          <t>Titik Api Kebakaran Hutan dan Lahan Menggila di Sumatra</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Thu, 15 Oct 2026 18:55:00 +0700</t>
+          <t>Fri, 16 Oct 2026 05:00:47 +0700</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>BRIN menyoroti pentingnya deteksi dini, pemetaan, dan koordinasi antarlembaga.</t>
+          <t>Dampak karhutla di Sumatra meluas hingga mengganggu aktivitas masyarakat.</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8314183/australia-dan-finlandia-bisa-jadi-rujukan-indonesia-tangani-kebakaran-hutan</t>
+          <t>https://www.liputan6.com/news/read/8314384/titik-api-kebakaran-hutan-dan-lahan-menggila-di-sumatra</t>
         </is>
       </c>
     </row>
@@ -2316,22 +2310,22 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>BNPB Kaji Penetapan Status Bencana Nasional untuk Kebakaran Hutan</t>
+          <t>Kepala BPK Jateng Turut Terjaring OTT KPK di Klaten</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Thu, 15 Oct 2026 18:53:59 +0700</t>
+          <t>Fri, 16 Oct 2026 00:26:44 +0700</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Kepala BNPB Kristomei Sianturi akan mengkaji status penanganan karhutla di enam provinsi.</t>
+          <t>KPK mengamankan 20 orang dalam OTT di Klaten, termasuk Bupati Hamenang Wajar Ismoyo dan Kepala Perwakilan BPK Jawa Tengah.</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8314184/bnpb-kaji-penetapan-status-bencana-nasional-untuk-kebakaran-hutan</t>
+          <t>https://www.liputan6.com/news/read/8314370/kepala-bpk-jateng-turut-terjaring-ott-kpk-di-klaten</t>
         </is>
       </c>
     </row>
@@ -2343,22 +2337,22 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Bupati Gowa Husniah Talenrang Diberhentikan, Wabup Jadi Plt</t>
+          <t>Baru Dilantik, Kepala BNPB Langsung Verifikasi Data Kebakaran Hutan</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Thu, 15 Oct 2026 18:37:03 +0700</t>
+          <t>Thu, 15 Oct 2026 23:50:08 +0700</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Tito Karnavian memberhentikan Bupati Gowa Sitti Husniah Talenrang dan menunjuk Darmawangsyah Muin sebagai Plt.</t>
+          <t>Kepala BNPB Kristomei Sianturi akan membandingkan data SiPongi dan pemantauan NASA untuk memverifikasi luas lahan terbakar akibat karhutla.</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8314167/bupati-gowa-husniah-talenrang-diberhentikan-wabup-jadi-plt</t>
+          <t>https://www.liputan6.com/news/read/8314357/baru-dilantik-kepala-bnpb-langsung-verifikasi-data-kebakaran-hutan</t>
         </is>
       </c>
     </row>
@@ -2370,22 +2364,22 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>6 Kasus Korupsi Bantuan Bencana, dari Donggala hingga BNPB</t>
+          <t>Infografis: 9 Pejabat Baru yang Dilantik dari Reshuffle Kabinet Prabowo</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Thu, 15 Oct 2026 18:21:27 +0700</t>
+          <t>Thu, 15 Oct 2026 22:56:00 +0700</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Bantuan yang semestinya meringankan korban bencana justru dikorupsi, berikut daftarnya.</t>
+          <t>Prabowo melantik sembilan pejabat baru dalam reshuffle Kabinet Merah Putih pada 15 Oktober 2026. Simak daftar nama dan jabatan yang mereka emban.</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8314155/6-kasus-korupsi-bantuan-bencana-dari-donggala-hingga-bnpb</t>
+          <t>https://www.liputan6.com/news/read/8314329/infografis-9-pejabat-baru-yang-dilantik-dari-reshuffle-kabinet-prabowo</t>
         </is>
       </c>
     </row>
@@ -2397,22 +2391,22 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Gempa Magnitudo 4,1 Guncang Bogor</t>
+          <t>Pramono Beberkan Ketimpangan Sosial Jakarta, Hunian Jadi Sorotan</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Thu, 15 Oct 2026 18:26:49 +0700</t>
+          <t>Thu, 15 Oct 2026 22:07:04 +0700</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Gempa bermagnitudo 4,1 mengguncang Bogor pada Kamis sore, getaran dirasakan di Pamijahan dan Kabandungan.</t>
+          <t>Di tengah perputaran ekonomi Jakarta, masih ada warga yang tinggal di rumah berukuran 3 x 4 meter bersama belasan orang.</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8314161/gempa-magnitudo-41-guncang-bogor</t>
+          <t>https://www.liputan6.com/news/read/8314305/pramono-beberkan-ketimpangan-sosial-jakarta-hunian-jadi-sorotan</t>
         </is>
       </c>
     </row>
@@ -2424,22 +2418,22 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Kepala BNPB Baru Janji Bersih-Bersih Internal Usai OTT KPK</t>
+          <t>Kasus Korupsi Nikel, Dirut PT CNI Jadi Tersangka Baru</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Thu, 15 Oct 2026 17:40:47 +0700</t>
+          <t>Thu, 15 Oct 2026 21:46:58 +0700</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Kepala BNPB Kristomei Sianturi merespons soal operasi tangkap tangan (OTT) KPK.</t>
+          <t>Dalam perkara dugaan korupsi tata kelola nikel, kerugian negara berdasarkan penghitungan BPKP disebut mencapai sekitar Rp 401 miliar.</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8314116/kepala-bnpb-baru-janji-bersih-bersih-internal-usai-ott-kpk</t>
+          <t>https://www.liputan6.com/news/read/8314297/kasus-korupsi-nikel-dirut-pt-cni-jadi-tersangka-baru</t>
         </is>
       </c>
     </row>
@@ -2451,22 +2445,22 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Banjir Kembali Melanda Wilayah Sumatera, Pemulihan Infrastruktur Terganggu</t>
+          <t>KPK Sita Rp 1 M dalam OTT Bupati Klaten</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Thu, 15 Oct 2026 17:38:02 +0700</t>
+          <t>Thu, 15 Oct 2026 20:47:53 +0700</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Sejumlah wilayah di Sumatera kembali dilanda banjir saat rehabilitasi dan rekonstruksi pascabencana masih berlangsung.</t>
+          <t>KPK masih memeriksa pihak-pihak yang diamankan dalam OTT di Klaten.</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8314111/banjir-kembali-melanda-wilayah-sumatera-pemulihan-infrastruktur-terganggu</t>
+          <t>https://www.liputan6.com/news/read/8314267/kpk-sita-rp-1-m-dalam-ott-bupati-klaten</t>
         </is>
       </c>
     </row>
@@ -2478,22 +2472,22 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Strategi Polisi Gerebek Kos Diduga Sarang Narkoba di Kampung Ambon</t>
+          <t>Jabat KSAD, Tandyo Budi Ungkap Tugas Khusus dari Prabowo</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Thu, 15 Oct 2026 17:21:04 +0700</t>
+          <t>Thu, 15 Oct 2026 20:29:36 +0700</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Penggerebekan kos di Kampung Ambon berujung pada pengamanan tujuh orang.</t>
+          <t>Tandyo mengatakan dirinya diminta Prabowo untuk mempercepat operasional sejumlah program strategis pemerintahan.</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8314100/strategi-polisi-gerebek-kos-diduga-sarang-narkoba-di-kampung-ambon</t>
+          <t>https://www.liputan6.com/news/read/8314262/jabat-ksad-tandyo-budi-ungkap-tugas-khusus-dari-prabowo</t>
         </is>
       </c>
     </row>
@@ -2505,22 +2499,22 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Rekam Jejak Maulana Bungaran, Wamen Imipas Baru</t>
+          <t>Terungkap, Dugaan Perkara di Balik OTT Bupati Klaten</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Thu, 15 Oct 2026 17:14:43 +0700</t>
+          <t>Thu, 15 Oct 2026 21:43:38 +0700</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Maulana Bungaran pernah aktif di Partai Gerindra dan memiliki rekam jejak kuat sebagai pengacara.</t>
+          <t>Giat tangkap tangan dilakukan berkaitan dengan penerimaan oleh Bupati Klaten dari pihak lain.</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8314065/rekam-jejak-maulana-bungaran-wamen-imipas-baru</t>
+          <t>https://www.liputan6.com/news/read/8314258/terungkap-dugaan-perkara-di-balik-ott-bupati-klaten</t>
         </is>
       </c>
     </row>
@@ -2532,22 +2526,22 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Rekam Jejak Jenderal Tandyo Budi, dari Wakil Panglima Jadi KSAD</t>
+          <t>Cegah Kebakaran Gambut Berulang, BPGMN Andalkan Sains dan Pemetaan Risiko</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Thu, 15 Oct 2026 16:16:36 +0700</t>
+          <t>Thu, 15 Oct 2026 20:19:00 +0700</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Tandyo menggantikan Maruli pada saat bersamaan dilantik Prabowo menjadi Wakil Panglima TNI dan Kepala Badan Nasional Pengelola Perbatasan dan Daerah Terpencil.</t>
+          <t>BPGMN akan memperkuat pemetaan risiko kebakaran dan melibatkan para ahli untuk memulihkan ekosistem gambut serta mangrove.</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8314028/rekam-jejak-jenderal-tandyo-budi-dari-wakil-panglima-jadi-ksad</t>
+          <t>https://www.liputan6.com/news/read/8314255/cegah-kebakaran-gambut-berulang-bpgmn-andalkan-sains-dan-pemetaan-risiko</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data pasar & berita - 2026-10-16 13:07 UTC
</commit_message>
<xml_diff>
--- a/data/market_news_latest.xlsx
+++ b/data/market_news_latest.xlsx
@@ -487,20 +487,20 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>5943.0239</v>
+        <v>5185.105</v>
       </c>
       <c r="F2" t="n">
-        <v>17.0479</v>
+        <v>-678.6748</v>
       </c>
       <c r="G2" t="n">
-        <v>0.29</v>
+        <v>-11.57</v>
       </c>
       <c r="H2" t="n">
-        <v>270876900</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -534,7 +534,7 @@
         <v>0.33</v>
       </c>
       <c r="H3" t="n">
-        <v>3428090000</v>
+        <v>6055670000</v>
       </c>
     </row>
     <row r="4">
@@ -568,7 +568,7 @@
         <v>1.08</v>
       </c>
       <c r="H4" t="n">
-        <v>500690219</v>
+        <v>500690000</v>
       </c>
     </row>
     <row r="5">
@@ -593,16 +593,16 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>26713.0254</v>
+        <v>26713.0293</v>
       </c>
       <c r="F5" t="n">
-        <v>20.1562</v>
+        <v>20.1602</v>
       </c>
       <c r="G5" t="n">
         <v>0.08</v>
       </c>
       <c r="H5" t="n">
-        <v>9708091000</v>
+        <v>10869960000</v>
       </c>
     </row>
     <row r="6">
@@ -623,20 +623,20 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>67744.28909999999</v>
+        <v>65324.2891</v>
       </c>
       <c r="F6" t="n">
-        <v>-33.2344</v>
+        <v>898.3398</v>
       </c>
       <c r="G6" t="n">
-        <v>-0.05</v>
+        <v>1.39</v>
       </c>
       <c r="H6" t="n">
-        <v>152100000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -657,20 +657,20 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>24314.1699</v>
+        <v>24186.8301</v>
       </c>
       <c r="F7" t="n">
-        <v>-31.0508</v>
+        <v>124.1094</v>
       </c>
       <c r="G7" t="n">
-        <v>-0.13</v>
+        <v>0.52</v>
       </c>
       <c r="H7" t="n">
-        <v>2804100000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -691,14 +691,20 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>3716.2842</v>
+      </c>
+      <c r="F8" t="n">
+        <v>8.8081</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0.24</v>
+      </c>
       <c r="H8" t="n">
-        <v>3771678644</v>
+        <v>18575544</v>
       </c>
     </row>
     <row r="9">
@@ -719,20 +725,20 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>10724.9004</v>
+        <v>10849.6904</v>
       </c>
       <c r="F9" t="n">
-        <v>74.6006</v>
+        <v>9.289999999999999</v>
       </c>
       <c r="G9" t="n">
-        <v>0.7</v>
+        <v>0.09</v>
       </c>
       <c r="H9" t="n">
-        <v>610957900</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -753,20 +759,20 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>25298.6094</v>
+        <v>25636.8496</v>
       </c>
       <c r="F10" t="n">
-        <v>38.709</v>
+        <v>254.2305</v>
       </c>
       <c r="G10" t="n">
-        <v>0.15</v>
+        <v>1</v>
       </c>
       <c r="H10" t="n">
-        <v>56498200</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -787,20 +793,20 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>5423.3301</v>
+        <v>5415.5298</v>
       </c>
       <c r="F11" t="n">
-        <v>-7.1699</v>
+        <v>12.0298</v>
       </c>
       <c r="G11" t="n">
-        <v>-0.13</v>
+        <v>0.22</v>
       </c>
       <c r="H11" t="n">
-        <v>256903700</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -821,17 +827,17 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>17823.6992</v>
+        <v>18000</v>
       </c>
       <c r="F12" t="n">
-        <v>-42.8008</v>
+        <v>176.3008</v>
       </c>
       <c r="G12" t="n">
-        <v>-0.24</v>
+        <v>0.99</v>
       </c>
       <c r="H12" t="n">
         <v>0</v>
@@ -855,17 +861,17 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>102.046</v>
+        <v>101.789</v>
       </c>
       <c r="F13" t="n">
-        <v>-0.504</v>
+        <v>-0.211</v>
       </c>
       <c r="G13" t="n">
-        <v>-0.49</v>
+        <v>-0.21</v>
       </c>
       <c r="H13" t="n">
         <v>0</v>
@@ -893,13 +899,13 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>158.13</v>
+        <v>158.037</v>
       </c>
       <c r="F14" t="n">
-        <v>0.173</v>
+        <v>0.08</v>
       </c>
       <c r="G14" t="n">
-        <v>0.11</v>
+        <v>0.05</v>
       </c>
       <c r="H14" t="n">
         <v>0</v>
@@ -923,17 +929,17 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>0.5089</v>
+        <v>0.5114</v>
       </c>
       <c r="F15" t="n">
-        <v>-0.0101</v>
+        <v>0.0025</v>
       </c>
       <c r="G15" t="n">
-        <v>-1.95</v>
+        <v>0.49</v>
       </c>
       <c r="H15" t="n">
         <v>0</v>
@@ -957,17 +963,17 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>0.5429</v>
+        <v>0.5445</v>
       </c>
       <c r="F16" t="n">
-        <v>-0.009599999999999999</v>
+        <v>0.0016</v>
       </c>
       <c r="G16" t="n">
-        <v>-1.74</v>
+        <v>0.29</v>
       </c>
       <c r="H16" t="n">
         <v>0</v>
@@ -991,17 +997,17 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>0.4088</v>
+        <v>0.4068</v>
       </c>
       <c r="F17" t="n">
-        <v>0.0003</v>
+        <v>-0.002</v>
       </c>
       <c r="G17" t="n">
-        <v>0.07000000000000001</v>
+        <v>-0.49</v>
       </c>
       <c r="H17" t="n">
         <v>0</v>
@@ -1038,7 +1044,7 @@
         <v>1.37</v>
       </c>
       <c r="H18" t="n">
-        <v>86228050</v>
+        <v>86514400</v>
       </c>
     </row>
     <row r="19">
@@ -1072,7 +1078,7 @@
         <v>0.42</v>
       </c>
       <c r="H19" t="n">
-        <v>80514689</v>
+        <v>80597700</v>
       </c>
     </row>
     <row r="20">
@@ -1093,20 +1099,20 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>4178.2998</v>
+        <v>4185.3999</v>
       </c>
       <c r="F20" t="n">
-        <v>70.3999</v>
+        <v>15.2998</v>
       </c>
       <c r="G20" t="n">
-        <v>1.71</v>
+        <v>0.37</v>
       </c>
       <c r="H20" t="n">
-        <v>3066</v>
+        <v>58728</v>
       </c>
     </row>
     <row r="21">
@@ -1127,20 +1133,20 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>96.18000000000001</v>
+        <v>95.78</v>
       </c>
       <c r="F21" t="n">
-        <v>1.09</v>
+        <v>-2.19</v>
       </c>
       <c r="G21" t="n">
-        <v>1.15</v>
+        <v>-2.24</v>
       </c>
       <c r="H21" t="n">
-        <v>2138</v>
+        <v>81042</v>
       </c>
     </row>
     <row r="22">
@@ -1161,20 +1167,20 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="E22" t="n">
-        <v>105.74</v>
+        <v>105.93</v>
       </c>
       <c r="F22" t="n">
-        <v>-0.32</v>
+        <v>0.01</v>
       </c>
       <c r="G22" t="n">
-        <v>-0.3</v>
+        <v>0.01</v>
       </c>
       <c r="H22" t="n">
-        <v>209</v>
+        <v>9046</v>
       </c>
     </row>
     <row r="23">
@@ -1195,20 +1201,20 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="E23" t="n">
-        <v>6.5515</v>
+        <v>6.6255</v>
       </c>
       <c r="F23" t="n">
-        <v>-0.06</v>
+        <v>0.114</v>
       </c>
       <c r="G23" t="n">
-        <v>-0.91</v>
+        <v>1.75</v>
       </c>
       <c r="H23" t="n">
-        <v>247</v>
+        <v>15894</v>
       </c>
     </row>
     <row r="24">
@@ -1242,7 +1248,7 @@
         <v>-0.67</v>
       </c>
       <c r="H24" t="n">
-        <v>23159834</v>
+        <v>23240000</v>
       </c>
     </row>
     <row r="25">
@@ -1263,17 +1269,17 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="E25" t="n">
-        <v>16.46</v>
+        <v>15.98</v>
       </c>
       <c r="F25" t="n">
-        <v>-0.41</v>
+        <v>-0.48</v>
       </c>
       <c r="G25" t="n">
-        <v>-2.43</v>
+        <v>-2.92</v>
       </c>
       <c r="H25" t="n">
         <v>0</v>
@@ -1297,20 +1303,20 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="E26" t="n">
-        <v>82135.75</v>
+        <v>81888.4219</v>
       </c>
       <c r="F26" t="n">
-        <v>573.2578</v>
+        <v>-253.0391</v>
       </c>
       <c r="G26" t="n">
-        <v>0.7</v>
+        <v>-0.31</v>
       </c>
       <c r="H26" t="n">
-        <v>41975259136</v>
+        <v>30546599936</v>
       </c>
     </row>
     <row r="27">
@@ -1331,20 +1337,20 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="E27" t="n">
-        <v>1420</v>
+        <v>1210</v>
       </c>
       <c r="F27" t="n">
-        <v>-10</v>
+        <v>-210</v>
       </c>
       <c r="G27" t="n">
-        <v>-0.7</v>
+        <v>-14.79</v>
       </c>
       <c r="H27" t="n">
-        <v>87691800</v>
+        <v>202008600</v>
       </c>
     </row>
     <row r="28">
@@ -1365,20 +1371,20 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="E28" t="n">
-        <v>1415</v>
+        <v>1205</v>
       </c>
       <c r="F28" t="n">
-        <v>-85</v>
+        <v>-210</v>
       </c>
       <c r="G28" t="n">
-        <v>-5.67</v>
+        <v>-14.84</v>
       </c>
       <c r="H28" t="n">
-        <v>166054400</v>
+        <v>79092200</v>
       </c>
     </row>
     <row r="29">
@@ -1399,20 +1405,20 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="E29" t="n">
-        <v>630</v>
+        <v>540</v>
       </c>
       <c r="F29" t="n">
-        <v>-35</v>
+        <v>-90</v>
       </c>
       <c r="G29" t="n">
-        <v>-5.26</v>
+        <v>-14.29</v>
       </c>
       <c r="H29" t="n">
-        <v>285141100</v>
+        <v>69411800</v>
       </c>
     </row>
     <row r="30">
@@ -1433,20 +1439,20 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="E30" t="n">
-        <v>2180</v>
+        <v>1855</v>
       </c>
       <c r="F30" t="n">
-        <v>-140</v>
+        <v>-325</v>
       </c>
       <c r="G30" t="n">
-        <v>-6.03</v>
+        <v>-14.91</v>
       </c>
       <c r="H30" t="n">
-        <v>18298600</v>
+        <v>40971900</v>
       </c>
     </row>
     <row r="31">
@@ -1467,20 +1473,20 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="E31" t="n">
-        <v>3920</v>
+        <v>3340</v>
       </c>
       <c r="F31" t="n">
-        <v>-200</v>
+        <v>-580</v>
       </c>
       <c r="G31" t="n">
-        <v>-4.85</v>
+        <v>-14.8</v>
       </c>
       <c r="H31" t="n">
-        <v>47973300</v>
+        <v>24196600</v>
       </c>
     </row>
     <row r="32">
@@ -1501,20 +1507,20 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="E32" t="n">
-        <v>474</v>
+        <v>404</v>
       </c>
       <c r="F32" t="n">
-        <v>-26</v>
+        <v>-70</v>
       </c>
       <c r="G32" t="n">
-        <v>-5.2</v>
+        <v>-14.77</v>
       </c>
       <c r="H32" t="n">
-        <v>48900700</v>
+        <v>65698800</v>
       </c>
     </row>
     <row r="33">
@@ -1535,20 +1541,20 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="E33" t="n">
-        <v>575</v>
+        <v>490</v>
       </c>
       <c r="F33" t="n">
-        <v>-20</v>
+        <v>-85</v>
       </c>
       <c r="G33" t="n">
-        <v>-3.36</v>
+        <v>-14.78</v>
       </c>
       <c r="H33" t="n">
-        <v>70117600</v>
+        <v>22779700</v>
       </c>
     </row>
     <row r="34">
@@ -1569,20 +1575,20 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="E34" t="n">
-        <v>3480</v>
+        <v>2960</v>
       </c>
       <c r="F34" t="n">
-        <v>-140</v>
+        <v>-520</v>
       </c>
       <c r="G34" t="n">
-        <v>-3.87</v>
+        <v>-14.94</v>
       </c>
       <c r="H34" t="n">
-        <v>4822700</v>
+        <v>7958900</v>
       </c>
     </row>
     <row r="35">
@@ -1603,20 +1609,20 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="E35" t="n">
-        <v>470</v>
+        <v>400</v>
       </c>
       <c r="F35" t="n">
-        <v>-50</v>
+        <v>-70</v>
       </c>
       <c r="G35" t="n">
-        <v>-9.619999999999999</v>
+        <v>-14.89</v>
       </c>
       <c r="H35" t="n">
-        <v>143573800</v>
+        <v>27349300</v>
       </c>
     </row>
     <row r="36">
@@ -1637,20 +1643,20 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="E36" t="n">
-        <v>184</v>
+        <v>157</v>
       </c>
       <c r="F36" t="n">
-        <v>-11</v>
+        <v>-27</v>
       </c>
       <c r="G36" t="n">
-        <v>-5.64</v>
+        <v>-14.67</v>
       </c>
       <c r="H36" t="n">
-        <v>36831100</v>
+        <v>100522400</v>
       </c>
     </row>
     <row r="37">
@@ -1671,20 +1677,20 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="E37" t="n">
-        <v>14075</v>
+        <v>11975</v>
       </c>
       <c r="F37" t="n">
-        <v>-475</v>
+        <v>-2100</v>
       </c>
       <c r="G37" t="n">
-        <v>-3.26</v>
+        <v>-14.92</v>
       </c>
       <c r="H37" t="n">
-        <v>10820200</v>
+        <v>1347700</v>
       </c>
     </row>
   </sheetData>
@@ -1743,22 +1749,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Ritel Modern Tak Wajib Lagi Jual 30% Produk UMKM</t>
+          <t>Intip Pembuatan Perahu Fiber untuk Nelayan di Kampung Nelayan Merah Putih</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Fri, 16 Oct 2026 06:25:00 +0700</t>
+          <t>Fri, 16 Oct 2026 20:00:11 +0700</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2023/04/03/ilustrasi-belanja-di-alfamart_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Perdagangan Budi Santoso menyampaikan pemerintah tak lagi mewajibkan produk usaha mikro kecil dan menengah (UMKM) memenuhi porsi 30% di ritel modern.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/16/intip-pembuatan-perahu-fiber-untuk-nelayan-di-kampung-nelayan-merah-putih-1792117410032_169.jpeg?w=360&amp;amp;q=90" /&gt; Pekerja membuat perahu nelayan berbahan fiber di galangan Kampung Nelayan Merah Putih, Manokwari, Papua Barat.</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8709142/ritel-modern-tak-wajib-lagi-jual-30-produk-umkm</t>
+          <t>https://finance.detik.com/foto-bisnis/d-8709506/intip-pembuatan-perahu-fiber-untuk-nelayan-di-kampung-nelayan-merah-putih</t>
         </is>
       </c>
     </row>
@@ -1770,22 +1776,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Serapan Tenaga Kerja Menyusut Meski Ekonomi Tumbuh</t>
+          <t>Rincian Total Denda Rp 2,1 Triliun buat  DSSA hingga BREN</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Fri, 16 Oct 2026 05:55:00 +0700</t>
+          <t>Fri, 16 Oct 2026 19:32:59 +0700</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/03/berburu-lowongan-kerja-di-ragunan-career-fest-jadi-harapan-1788414921572_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Perindustrian (Menperin) Muhammad Sarmuji menyoroti semakin terbatasnya penciptaan lapangan kerja di tengah pertumbuhan </t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/16/ihsg-ambruk-1157-ditutup-di-level-5185-1792144638939_169.jpeg?w=360&amp;amp;q=90" /&gt; Denda itu ditetapkan atas pelanggaran di bidang pasar modal yang dilakukan tiga emiten.</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8709116/serapan-tenaga-kerja-menyusut-meski-ekonomi-tumbuh</t>
+          <t>https://finance.detik.com/bursa-dan-valas/d-8710708/rincian-total-denda-rp-2-1-triliun-buat-dssa-hingga-bren</t>
         </is>
       </c>
     </row>
@@ -1797,22 +1803,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Pertamina Patra Niaga Ungkap Layanan SPBU di Bali Berangsur Pulih</t>
+          <t>1.550 Manajer Kopdes Minta Offering Ulang, Kemenkop: Mereka Menyesal Menolak</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Thu, 15 Oct 2026 22:35:01 +0700</t>
+          <t>Fri, 16 Oct 2026 19:00:42 +0700</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/15/pertamina-patra-niaga-1792078465155.jpeg?w=360&amp;amp;q=90" /&gt; PT Pertamina Patra Niaga memperkuat pasokan dan distribusi BBM di Bali dengan penambahan suplai dan operasional 24 jam.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/04/18/penyerahan-truk-kdmp-di-temanggung-1776489684625_169.jpeg?w=360&amp;amp;q=90" /&gt; Kemenkop mencatat 1.550 manajer Koperasi Desa/Kelurahan Merah Putih (KDKMP) terkendala proses administrasi karena melewati batas waktu penandatanganan k</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8709219/pertamina-patra-niaga-ungkap-layanan-spbu-di-bali-berangsur-pulih</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8710664/1-550-manajer-kopdes-minta-offering-ulang-kemenkop-mereka-menyesal-menolak</t>
         </is>
       </c>
     </row>
@@ -1824,22 +1830,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Pariwisata Andalan RI Genjot Ekonomi, Segini Kontribusinya</t>
+          <t>Perkuat Ekosistem Wakaf Produktif, BSI Dorong Potensi Rp 180 Triliun</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Thu, 15 Oct 2026 22:25:00 +0700</t>
+          <t>Fri, 16 Oct 2026 18:20:02 +0700</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2019/03/18/c12187aa-58c0-47af-adc7-725abd129e54_169.jpeg?w=360&amp;amp;q=90" /&gt; Pemerintah terus menjaga momentum pertumbuhan pariwisata Indonesia sekaligus memperluas peluang usaha dan investasi.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/16/bsi-1792149584130.jpeg?w=360&amp;amp;q=90" /&gt; PT Bank Syariah Indonesia (BSI) dorong pengembangan wakaf produktif di GLOW 2026. BSI optimis wakaf bisa tingkatkan kesejahteraan dan ketahanan ekonomi umat.</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8709204/pariwisata-andalan-ri-genjot-ekonomi-segini-kontribusinya</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8710593/perkuat-ekosistem-wakaf-produktif-bsi-dorong-potensi-rp-180-triliun</t>
         </is>
       </c>
     </row>
@@ -1851,22 +1857,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Taspen Ikut Arahan Pemerintah soal Koperasi Jadi Penyalur Dana Pensiunan</t>
+          <t>Dukung Ekspor UMKM, Astra Pamerkan Produk Lokal Unggulan di TEI 2026</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Thu, 15 Oct 2026 21:55:59 +0700</t>
+          <t>Fri, 16 Oct 2026 18:19:50 +0700</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/05/21/ilustrasi-layanan-taspen-1747810258404_169.jpeg?w=360&amp;amp;q=90" /&gt; PT Taspen (Persero) mengikuti arahan pemerintah terkait penyaluran dana pensiun aparatur sipil negara (ASN).</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/16/dukung-ekspor-umkm-astra-pamerkan-produk-lokal-unggulan-di-tei-2026-1792149478736_169.jpeg?w=360&amp;amp;q=90" /&gt; PT Astra International mendukung ekspor UMKM di Trade Expo Indonesia 2026. 30 peserta tampilkan produk unggulan dari De</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/moneter/d-8709195/taspen-ikut-arahan-pemerintah-soal-koperasi-jadi-penyalur-dana-pensiunan</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8710592/dukung-ekspor-umkm-astra-pamerkan-produk-lokal-unggulan-di-tei-2026</t>
         </is>
       </c>
     </row>
@@ -1878,22 +1884,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Genjot Pasokan di Bali, Pertamina Ingatkan Jangan Beli Pertalite buat Dijual Lagi</t>
+          <t>IHSG Ambruk 11,57%, Ditutup di Level 5.185</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Thu, 15 Oct 2026 21:47:06 +0700</t>
+          <t>Fri, 16 Oct 2026 18:04:47 +0700</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/14/pertamina-genjot-pasokan-bbm-ke-bali-1791990343502_169.jpeg?w=360&amp;amp;q=90" /&gt; PT Pertamina Patra Niaga terus menggenjot penyaluran bahan bakar minyak (BBM) ke wilayah Bali</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/16/ihsg-ambruk-1157-ditutup-di-level-5185-1792144639064.jpeg?w=360&amp;amp;q=90" /&gt; IHSG anjlok 11,57% ke level 5.185,11, di tengah konsultasi publik MSCI terkait rencana reklasifikasi pasar saham Indonesia menjadi Standalone Market.</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8709161/genjot-pasokan-di-bali-pertamina-ingatkan-jangan-beli-pertalite-buat-dijual-lagi</t>
+          <t>https://finance.detik.com/foto-bisnis/d-8710404/ihsg-ambruk-11-57-ditutup-di-level-5-185</t>
         </is>
       </c>
     </row>
@@ -1905,22 +1911,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Danantara Siapkan Rp 1,7 Triliun/ Tahun buat Kesehatan, Pendidikan, Sanitasi</t>
+          <t>Pemerintah Belum Putuskan Pembelian Pertalite Pakai Desil 9-10</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Thu, 15 Oct 2026 20:55:00 +0700</t>
+          <t>Fri, 16 Oct 2026 17:44:41 +0700</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/07/01/wisma-danantara-indonesia-1751345496674_169.jpeg?w=360&amp;amp;q=90" /&gt; Danantara akan mengalokasikan US$ 100 juta atau Rp 1,7 triliun (kurs Rp 17.900) setiap tahun untuk mendukung program sosial melalui Danantara Trust.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/15/warga-blitar-antre-panjang-untuk-mendapatkan-pertalite-1792054696805_169.jpeg?w=360&amp;amp;q=90" /&gt; Pemerintah belum memutuskan pembelian Pertalite untuk desil 9-10. Rencana ini masih dalam pengkajian dan diskusi, dengan kemungkinan</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8709105/danantara-siapkan-rp-1-7-triliun-tahun-buat-kesehatan-pendidikan-sanitasi</t>
+          <t>https://finance.detik.com/energi/d-8710521/pemerintah-belum-putuskan-pembelian-pertalite-pakai-desil-9-10</t>
         </is>
       </c>
     </row>
@@ -1932,22 +1938,22 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>DJP Targetkan Setoran Pajak Digital Naik Sampai 50%</t>
+          <t>Bahlil Sebut Penyusunan DIM RUU Migas Sudah 90%</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Thu, 15 Oct 2026 20:30:47 +0700</t>
+          <t>Fri, 16 Oct 2026 17:26:01 +0700</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2024/12/11/ilustrasi-pajak_169.jpeg?w=360&amp;amp;q=90" /&gt; Direktur Jenderal Pajak Bimo Wijayanto memperkirakan penerimaan pajak dari aktivitas ekonomi digital bisa tumbuh 50%, menjadi sekitar Rp 16 triliun.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/07/16/menteri-esdm-bahlil-lahadalia-1784186781817_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri ESDM Bahlil mengungkapkan RUU Migas hampir rampung, dengan progres 90%. Pembentukan Badan Usaha Khusus jadi fokus utama. Target DIM selesai 22 Oktobe</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8709031/djp-targetkan-setoran-pajak-digital-naik-sampai-50</t>
+          <t>https://finance.detik.com/energi/d-8710446/bahlil-sebut-penyusunan-dim-ruu-migas-sudah-90</t>
         </is>
       </c>
     </row>
@@ -1959,22 +1965,22 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Mau Investasi Bitcoin? Pahami Cara Beli, Strategi, dan Risiko Kripto</t>
+          <t>Pengguna Pertamax Ramai-ramai Pindah ke Pertalite, Stok Ikut Turun</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Thu, 15 Oct 2026 20:29:22 +0700</t>
+          <t>Fri, 16 Oct 2026 16:58:49 +0700</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/15/magnific-1792070910370.jpeg?w=360&amp;amp;q=90" /&gt; Bitcoin semakin populer di kalangan investor. Pelajari cara berinvestasi, pilih platform seperti Pintu, dan terapkan strategi menabung untuk hasil optimal.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/01/bahlil-lahadalia-1790850102759_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri ESDM Bahlil mengonfirmasi penurunan stok Pertalite menjadi 16-18 hari akibat pergeseran konsumsi. Ia memastikan stok aman dan normal dalam seminggu.</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/fintech/d-8709107/mau-investasi-bitcoin-pahami-cara-beli-strategi-dan-risiko-kripto</t>
+          <t>https://finance.detik.com/energi/d-8710388/pengguna-pertamax-ramai-ramai-pindah-ke-pertalite-stok-ikut-turun</t>
         </is>
       </c>
     </row>
@@ -1986,22 +1992,22 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>10.070 Kopdes Mulai Operasi Hari Ini</t>
+          <t>Manajer Kopdes Merah Putih Jadi Pegawai Koperasi Usai Dikontrak 2 Tahun</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Thu, 15 Oct 2026 20:00:41 +0700</t>
+          <t>Fri, 16 Oct 2026 16:51:48 +0700</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/21/kopdes-merah-putih-bersiap-operasional-23-ribu-bangunan-telah-rampung-1789986171380_169.jpeg?w=360&amp;amp;q=90" /&gt; Distribusi pasokan pangan untuk operasional Koperasi Desa/Kelurahan Merah Putih (KDKMP) dipastikan sudah siap.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/16/deputi-bidang-pengembangan-talenta-dan-daya-saing-koperasi-destry-anna-sari-1792139643262_169.jpeg?w=360&amp;amp;q=90" /&gt; Ya, jadi pegawai koperasi. Pegawai koperasi itu keren loh, ujar Destry.</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8709020/10-070-kopdes-mulai-operasi-hari-ini</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8710380/manajer-kopdes-merah-putih-jadi-pegawai-koperasi-usai-dikontrak-2-tahun</t>
         </is>
       </c>
     </row>
@@ -2013,22 +2019,22 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>DJP Siapkan Insentif Pajak buat BUMN, Ini Bocorannya</t>
+          <t>IHSG Ambruk 11,57% ke 5.185 Dibayangi Ancaman Downgrade MSCI</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Thu, 15 Oct 2026 19:30:12 +0700</t>
+          <t>Fri, 16 Oct 2026 16:34:54 +0700</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/15/direktur-jenderal-pajak-djp-bimo-wijayanto-1792062697952_169.jpeg?w=360&amp;amp;q=90" /&gt; Direktorat Jenderal Pajak (DJP) disebut telah menyiapkan aturan tentang insentif pajak bagi Badan Usaha Milik Negara (BUMN) yang melakukan aksi </t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/05/18/ihsg-anjlok-ke-zona-merah-bursa-saham-melemah-tajam-1779098741262_169.jpeg?w=360&amp;amp;q=90" /&gt; Indeks Harga Saham Gabungan (IHSG) ditutup anjlok 678,67 poin (11,57%) ke 5.185 atau anjlok 678,67 poin (11,57%).</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8708986/djp-siapkan-insentif-pajak-buat-bumn-ini-bocorannya</t>
+          <t>https://finance.detik.com/bursa-dan-valas/d-8710354/ihsg-ambruk-11-57-ke-5-185-dibayangi-ancaman-downgrade-msci</t>
         </is>
       </c>
     </row>
@@ -2040,22 +2046,22 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>KRL Kerap Gangguan, INKA Minta Maaf</t>
+          <t>Hadapi Tantangan Global, CIMB Gelar Acara Bahas AI hingga Supply Chain</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Thu, 15 Oct 2026 19:00:11 +0700</t>
+          <t>Fri, 16 Oct 2026 16:17:33 +0700</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/14/krl-inka-gangguan-penumpang-di-stasiun-pasar-minggu-pindah-krl-dok-istimewa-1791983235827_169.jpeg?w=360&amp;amp;q=90" /&gt; PT Industri Kereta Api (Persero) atau INKA buka suara soal beberapa rangkaian KRL CLI-225 yang mengalami masala</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/16/cimb-1792142228196_169.jpeg?w=360&amp;amp;q=90" /&gt; CIMB Niaga menggelar Business Summit 2026 untuk bahas tantangan ekonomi global, AI, dan supply chain.</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/infrastruktur/d-8708975/krl-kerap-gangguan-inka-minta-maaf</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8710321/hadapi-tantangan-global-cimb-gelar-acara-bahas-ai-hingga-supply-chain</t>
         </is>
       </c>
     </row>
@@ -2067,22 +2073,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Penerimaan Pajak RI Segitu-gitu Aja, DJP Buka Suara</t>
+          <t>Bareskrim Polri Turun Tangan Awasi Pelanggaran di Bursa</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Thu, 15 Oct 2026 18:30:45 +0700</t>
+          <t>Fri, 16 Oct 2026 16:17:15 +0700</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/15/direktur-jenderal-pajak-djp-bimo-wijayanto-1792062697871_169.jpeg?w=360&amp;amp;q=90" /&gt; Direktur Jenderal Pajak (DJP) Bimo Wijayanto, mengatakan baru sekali dalam sejarah pemerintah berani menargetkan penerimaan pajak 9% dari PDB da</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/01/30/ihsg-rebound-usai-dua-hari-anjlok-seiring-pengunduran-diri-dirut-bei-1769748663323_169.jpeg?w=360&amp;amp;q=90" /&gt; Kapolri Suyudi Ario Seto menyatakan Bareskrim Polri bakal turun tangan mengawasi langsung Bursa Efek Indonesia.</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8708906/penerimaan-pajak-ri-segitu-gitu-aja-djp-buka-suara</t>
+          <t>https://finance.detik.com/bursa-dan-valas/d-8710320/bareskrim-polri-turun-tangan-awasi-pelanggaran-di-bursa</t>
         </is>
       </c>
     </row>
@@ -2094,22 +2100,22 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>MR.D.I.Y., Kemenperin &amp;amp; CIMB Niaga Dorong IKM Perkuat Bisnis Berkelanjutan</t>
+          <t>Manajer Tetap Digaji Meski Kopdes Belum Beroperasi</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Thu, 15 Oct 2026 18:15:54 +0700</t>
+          <t>Fri, 16 Oct 2026 16:09:15 +0700</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/15/mrdiy-kemenperin-cimb-niaga-dorong-ikm-perkuat-bisnis-berkelanjutan-1792062894911.jpeg?w=360&amp;amp;q=90" /&gt; PT Daya Intiguna Yasa Tbk dan CIMB Niaga gelar pelatihan manajemen keuangan untuk 100 IKM. Fokus pada keberlanjutan dan pen</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/16/deputi-bidang-pengembangan-talenta-dan-daya-saing-koperasi-destry-anna-sari-1792139643262_169.jpeg?w=360&amp;amp;q=90" /&gt; Kementerian Koperasi (Kemenkop) memastikan semua manajer Koperasi Desa/Kelurahan Merah Putih (KDKMP) yang telah</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8708914/mr-d-i-y-kemenperin-cimb-niaga-dorong-ikm-perkuat-bisnis-berkelanjutan</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8710302/manajer-tetap-digaji-meski-kopdes-belum-beroperasi</t>
         </is>
       </c>
     </row>
@@ -2121,22 +2127,22 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Perang Arab Saudi Vs Houthi, Garuda Alihkan Rute-Tunda Penerbangan</t>
+          <t>IHSG Ambles 11%, Bos Danantara Lihat Peluang Borong Saham</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Thu, 15 Oct 2026 18:03:46 +0700</t>
+          <t>Fri, 16 Oct 2026 16:05:50 +0700</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/07/19/pesawat-garuda-indonesia-1752916632356_169.jpeg?w=360&amp;amp;q=90" /&gt; Situasi geopolitik di kawasan Timur Tengah berpotensi berdampak pada operasi penerbangan dari dan menuju Arab Saudi.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/02/menteri-investasi-dan-hilirisasikepala-bkpm-sekaligus-ceo-badan-pengelola-investasi-bpi-danantara-rosan-roeslani-di-sebuah-hot-1790942979284_169.jpeg?w=360&amp;amp;q=90" /&gt; CEO Danantara, Rosan Roeslani, menanggapi penurunan IHSG 11%</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8708883/perang-arab-saudi-vs-houthi-garuda-alihkan-rute-tunda-penerbangan</t>
+          <t>https://finance.detik.com/bursa-dan-valas/d-8710294/ihsg-ambles-11-bos-danantara-lihat-peluang-borong-saham</t>
         </is>
       </c>
     </row>
@@ -2148,22 +2154,22 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Cerita Menkum Supratman Saat Diminta Prabowo Pangkas Aturan Berbelit</t>
+          <t>Penampakan Bupati Klaten Hamenang Usai Diperiksa KPK</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Fri, 16 Oct 2026 06:37:26 +0700</t>
+          <t>Fri, 16 Oct 2026 19:42:50 +0700</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Menkum mengaku telah memangkas 195 Permenkum jadi 34.</t>
+          <t>Bupati Klaten Hamenang mengenakan rompi oranye khas tahanan KPK saat keluar dari Gedung Merah Putih KPK.</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8314405/cerita-menkum-supratman-saat-diminta-prabowo-pangkas-aturan-berbelit</t>
+          <t>https://www.liputan6.com/news/read/8315024/penampakan-bupati-klaten-hamenang-usai-diperiksa-kpk</t>
         </is>
       </c>
     </row>
@@ -2175,22 +2181,22 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Menteri Imipas Sanksi Pegawai Terlibat Jual Beli Remisi</t>
+          <t>Kasus Dugaan Kekerasan Dipicu Kembang Api, Pelapor Dipanggil Polisi</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Fri, 16 Oct 2026 06:32:28 +0700</t>
+          <t>Fri, 16 Oct 2026 19:31:21 +0700</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Agus belum merinci jenis sanksi yang dijatuhkan.</t>
+          <t>Amanda Andono memenuhi panggilan Polda Metro Jaya untuk menjelaskan kronologi dugaan kekerasan yang dialaminya di Pondok Pinang.</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8314404/menteri-imipas-sanksi-pegawai-terlibat-jual-beli-remisi</t>
+          <t>https://www.liputan6.com/news/read/8315009/kasus-dugaan-kekerasan-dipicu-kembang-api-pelapor-dipanggil-polisi</t>
         </is>
       </c>
     </row>
@@ -2202,22 +2208,22 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Polisi Tetapkan 9 Tersangka TPPO ABK KM Maulana 23</t>
+          <t>Putusan MK Buka Jalan Pengusutan Kasus Andrie Yunus di Peradilan Umum</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Fri, 16 Oct 2026 06:03:49 +0700</t>
+          <t>Fri, 16 Oct 2026 19:25:00 +0700</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Penetapan tersebut dilakukan setelah penyidik menjalankan serangkaian proses penyelidikan dan penyidikan.</t>
+          <t>Tim Advokasi mendesak Polda Metro Jaya mengusut 16 orang terkait kasus Andrie Yunus.</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8314399/polisi-tetapkan-9-tersangka-tppo-abk-km-maulana-23</t>
+          <t>https://www.liputan6.com/news/read/8315000/putusan-mk-buka-jalan-pengusutan-kasus-andrie-yunus-di-peradilan-umum</t>
         </is>
       </c>
     </row>
@@ -2229,22 +2235,22 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Bongkar Pasang Kabinet Prabowo untuk Kedelapan Kalinya</t>
+          <t>DPR Desak Kemenhut Gerak Cepat Tangani Kebakaran Hutan</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Fri, 16 Oct 2026 06:00:00 +0700</t>
+          <t>Fri, 16 Oct 2026 19:05:52 +0700</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Dalam reshuffle kali ini, jajaran pimpinan strategis di sektor pertahanan, keamanan, kementerian, hingga lembaga nonkementerian mengalami penataan ulang.</t>
+          <t>Desakan ini muncul setelah jumlah titik panas nasional mencapai 799 titik pada 15 Oktober 2026.</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8314365/bongkar-pasang-kabinet-prabowo-untuk-kedelapan-kalinya</t>
+          <t>https://www.liputan6.com/news/read/8314914/dpr-desak-kemenhut-gerak-cepat-tangani-kebakaran-hutan</t>
         </is>
       </c>
     </row>
@@ -2256,22 +2262,22 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Menko Yusril: Terlalu Banyak Peraturan Kita Buat, Bikin Pusing</t>
+          <t>Terungkap Identitas Terduga Pelaku Pencambukan di KPPG Bogor</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Fri, 16 Oct 2026 05:30:55 +0700</t>
+          <t>Fri, 16 Oct 2026 19:14:07 +0700</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Alih-alih menyelesaikan persoalan, aturan yang terus bertambah justru bisa membuat pelaksanaannya semakin rumit.</t>
+          <t>Identitas keduanya terungkap usai polisi mendatangi lokasi kejadian dan memeriksa sejumlah saksi.</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8314394/menko-yusril-terlalu-banyak-peraturan-kita-buat-bikin-pusing</t>
+          <t>https://www.liputan6.com/news/read/8314997/terungkap-identitas-terduga-pelaku-pencambukan-di-kppg-bogor</t>
         </is>
       </c>
     </row>
@@ -2283,22 +2289,22 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Titik Api Kebakaran Hutan dan Lahan Menggila di Sumatra</t>
+          <t>Mengenal Dana Bencana yang Terseret Kasus Korupsi BNPB</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Fri, 16 Oct 2026 05:00:47 +0700</t>
+          <t>Fri, 16 Oct 2026 18:13:59 +0700</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Dampak karhutla di Sumatra meluas hingga mengganggu aktivitas masyarakat.</t>
+          <t>KPK membeberkan dugaan penyalahgunaan dana kebencanaan BNPB melalui pengadaan barang dan jasa.</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8314384/titik-api-kebakaran-hutan-dan-lahan-menggila-di-sumatra</t>
+          <t>https://www.liputan6.com/news/read/8314950/mengenal-dana-bencana-yang-terseret-kasus-korupsi-bnpb</t>
         </is>
       </c>
     </row>
@@ -2310,22 +2316,22 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Kepala BPK Jateng Turut Terjaring OTT KPK di Klaten</t>
+          <t>Asap Karhutla Kalimantan Masuk Atmosfer Jakarta, Ini yang Perlu Dilakukan</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Fri, 16 Oct 2026 00:26:44 +0700</t>
+          <t>Fri, 16 Oct 2026 18:06:00 +0700</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>KPK mengamankan 20 orang dalam OTT di Klaten, termasuk Bupati Hamenang Wajar Ismoyo dan Kepala Perwakilan BPK Jawa Tengah.</t>
+          <t>Warga diimbau batasi aktivitas luar ruangan dan wajib memakai masker.</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8314370/kepala-bpk-jateng-turut-terjaring-ott-kpk-di-klaten</t>
+          <t>https://www.liputan6.com/news/read/8314949/asap-karhutla-kalimantan-masuk-atmosfer-jakarta-ini-yang-perlu-dilakukan</t>
         </is>
       </c>
     </row>
@@ -2337,22 +2343,22 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Baru Dilantik, Kepala BNPB Langsung Verifikasi Data Kebakaran Hutan</t>
+          <t>Kopdes Merah Putih Bisa Jual Obat Bebas, Skema Distribusi Disiapkan</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Thu, 15 Oct 2026 23:50:08 +0700</t>
+          <t>Fri, 16 Oct 2026 17:37:21 +0700</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Kepala BNPB Kristomei Sianturi akan membandingkan data SiPongi dan pemantauan NASA untuk memverifikasi luas lahan terbakar akibat karhutla.</t>
+          <t>Gerai Kopdes Merah Putih disiapkan menjadi alternatif akses obat bagi masyarakat.</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8314357/baru-dilantik-kepala-bnpb-langsung-verifikasi-data-kebakaran-hutan</t>
+          <t>https://www.liputan6.com/news/read/8314923/kopdes-merah-putih-bisa-jual-obat-bebas-skema-distribusi-disiapkan</t>
         </is>
       </c>
     </row>
@@ -2364,22 +2370,22 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Infografis: 9 Pejabat Baru yang Dilantik dari Reshuffle Kabinet Prabowo</t>
+          <t>Kongkalikong Tilap Dana Bencana: KPK Bongkar 2 Klaster Korupsi BNPB</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Thu, 15 Oct 2026 22:56:00 +0700</t>
+          <t>Fri, 16 Oct 2026 17:31:21 +0700</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Prabowo melantik sembilan pejabat baru dalam reshuffle Kabinet Merah Putih pada 15 Oktober 2026. Simak daftar nama dan jabatan yang mereka emban.</t>
+          <t>KPK membongkar ada dua klaster korupsi dana bencana di BNPB.</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8314329/infografis-9-pejabat-baru-yang-dilantik-dari-reshuffle-kabinet-prabowo</t>
+          <t>https://www.liputan6.com/news/read/8314913/kongkalikong-tilap-dana-bencana-kpk-bongkar-2-klaster-korupsi-bnpb</t>
         </is>
       </c>
     </row>
@@ -2391,22 +2397,22 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Pramono Beberkan Ketimpangan Sosial Jakarta, Hunian Jadi Sorotan</t>
+          <t>KPK: Dana Bencana BNPB Diduga Dipakai Beli Saham Rp 30,98 Miliar</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Thu, 15 Oct 2026 22:07:04 +0700</t>
+          <t>Fri, 16 Oct 2026 17:22:20 +0700</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Di tengah perputaran ekonomi Jakarta, masih ada warga yang tinggal di rumah berukuran 3 x 4 meter bersama belasan orang.</t>
+          <t>Kepemilikan saham tercatat mencapai 150,4 juta lembar atau setara 1,07 persen.</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8314305/pramono-beberkan-ketimpangan-sosial-jakarta-hunian-jadi-sorotan</t>
+          <t>https://www.liputan6.com/news/read/8314910/kpk-dana-bencana-bnpb-diduga-dipakai-beli-saham-rp-3098-miliar</t>
         </is>
       </c>
     </row>
@@ -2418,22 +2424,22 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Kasus Korupsi Nikel, Dirut PT CNI Jadi Tersangka Baru</t>
+          <t>Korupsi BNPB: Dana Karhutla Kalimantan, Gempa NTT Hingga Banjir Sumatra</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Thu, 15 Oct 2026 21:46:58 +0700</t>
+          <t>Fri, 16 Oct 2026 17:09:04 +0700</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Dalam perkara dugaan korupsi tata kelola nikel, kerugian negara berdasarkan penghitungan BPKP disebut mencapai sekitar Rp 401 miliar.</t>
+          <t>Dana darurat untuk penanganan bencana seperti Karhutla Kalimantan dan Gempa NTT ini diduga disalahgunakan melalui suap dan konflik kepentingan.</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8314297/kasus-korupsi-nikel-dirut-pt-cni-jadi-tersangka-baru</t>
+          <t>https://www.liputan6.com/news/read/8314899/korupsi-bnpb-dana-karhutla-kalimantan-gempa-ntt-hingga-banjir-sumatra</t>
         </is>
       </c>
     </row>
@@ -2445,22 +2451,22 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>KPK Sita Rp 1 M dalam OTT Bupati Klaten</t>
+          <t>OTT BNPB, KPK Sita Uang Asing hingga Kepingan Emas Senilai Rp 5,47 miliar</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Thu, 15 Oct 2026 20:47:53 +0700</t>
+          <t>Fri, 16 Oct 2026 17:07:41 +0700</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>KPK masih memeriksa pihak-pihak yang diamankan dalam OTT di Klaten.</t>
+          <t>KPK menyita barang bukti lebih kurang mencapai Rp 5,47 miliar dari OTT di Badan Nasional Penanggulangan Bencana (BNPB).</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8314267/kpk-sita-rp-1-m-dalam-ott-bupati-klaten</t>
+          <t>https://www.liputan6.com/news/read/8314897/ott-bnpb-kpk-sita-uang-asing-hingga-kepingan-emas-senilai-rp-547-miliar</t>
         </is>
       </c>
     </row>
@@ -2472,22 +2478,22 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Jabat KSAD, Tandyo Budi Ungkap Tugas Khusus dari Prabowo</t>
+          <t>KPK Tetapkan 5 Tersangka Kasus Korupsi Dana Bencana BNPB</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Thu, 15 Oct 2026 20:29:36 +0700</t>
+          <t>Fri, 16 Oct 2026 16:59:27 +0700</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Tandyo mengatakan dirinya diminta Prabowo untuk mempercepat operasional sejumlah program strategis pemerintahan.</t>
+          <t>KPK juga mengamankan barang bukti dengan nilai total sekitar Rp 5,47 miliar.</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8314262/jabat-ksad-tandyo-budi-ungkap-tugas-khusus-dari-prabowo</t>
+          <t>https://www.liputan6.com/news/read/8314889/kpk-tetapkan-5-tersangka-kasus-korupsi-dana-bencana-bnpb</t>
         </is>
       </c>
     </row>
@@ -2499,22 +2505,22 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Terungkap, Dugaan Perkara di Balik OTT Bupati Klaten</t>
+          <t>Penjelasan BMKG soal Sebaran Asap Kebakaran Hutan Terdeteksi di Jakarta</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Thu, 15 Oct 2026 21:43:38 +0700</t>
+          <t>Fri, 16 Oct 2026 16:02:00 +0700</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Giat tangkap tangan dilakukan berkaitan dengan penerimaan oleh Bupati Klaten dari pihak lain.</t>
+          <t>Arah angin membawa asap ini melintasi wilayah Jawa.</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8314258/terungkap-dugaan-perkara-di-balik-ott-bupati-klaten</t>
+          <t>https://www.liputan6.com/news/read/8314841/penjelasan-bmkg-soal-sebaran-asap-kebakaran-hutan-terdeteksi-di-jakarta</t>
         </is>
       </c>
     </row>
@@ -2526,22 +2532,22 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Cegah Kebakaran Gambut Berulang, BPGMN Andalkan Sains dan Pemetaan Risiko</t>
+          <t>Kapolri Usut Dugaan Pidana Pasar Modal Imbas IHSG Anjlok</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Thu, 15 Oct 2026 20:19:00 +0700</t>
+          <t>Fri, 16 Oct 2026 15:58:20 +0700</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>BPGMN akan memperkuat pemetaan risiko kebakaran dan melibatkan para ahli untuk memulihkan ekosistem gambut serta mangrove.</t>
+          <t>Penyidik Polri akan mengumpulkan alat bukti sebelum mengambil tindakan hukum.</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8314255/cegah-kebakaran-gambut-berulang-bpgmn-andalkan-sains-dan-pemetaan-risiko</t>
+          <t>https://www.liputan6.com/news/read/8314833/kapolri-usut-dugaan-pidana-pasar-modal-imbas-ihsg-anjlok</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data pasar & berita - 2026-10-18 23:45 UTC
</commit_message>
<xml_diff>
--- a/data/market_news_latest.xlsx
+++ b/data/market_news_latest.xlsx
@@ -500,7 +500,7 @@
         <v>-11.57</v>
       </c>
       <c r="H2" t="n">
-        <v>0</v>
+        <v>650917300</v>
       </c>
     </row>
     <row r="3">
@@ -521,20 +521,20 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>7744.0601</v>
+        <v>7659.4399</v>
       </c>
       <c r="F3" t="n">
-        <v>25.1201</v>
+        <v>-84.62009999999999</v>
       </c>
       <c r="G3" t="n">
-        <v>0.33</v>
+        <v>-1.09</v>
       </c>
       <c r="H3" t="n">
-        <v>6055670000</v>
+        <v>5482060000</v>
       </c>
     </row>
     <row r="4">
@@ -555,20 +555,20 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>52177.6914</v>
+        <v>52002.4102</v>
       </c>
       <c r="F4" t="n">
-        <v>556.2109</v>
+        <v>-175.2812</v>
       </c>
       <c r="G4" t="n">
-        <v>1.08</v>
+        <v>-0.34</v>
       </c>
       <c r="H4" t="n">
-        <v>500690000</v>
+        <v>488090000</v>
       </c>
     </row>
     <row r="5">
@@ -589,20 +589,20 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>26713.0293</v>
+        <v>26140.0293</v>
       </c>
       <c r="F5" t="n">
-        <v>20.1602</v>
+        <v>-573</v>
       </c>
       <c r="G5" t="n">
-        <v>0.08</v>
+        <v>-2.15</v>
       </c>
       <c r="H5" t="n">
-        <v>10869960000</v>
+        <v>9505000000</v>
       </c>
     </row>
     <row r="6">
@@ -636,7 +636,7 @@
         <v>1.39</v>
       </c>
       <c r="H6" t="n">
-        <v>0</v>
+        <v>168700000</v>
       </c>
     </row>
     <row r="7">
@@ -670,7 +670,7 @@
         <v>0.52</v>
       </c>
       <c r="H7" t="n">
-        <v>0</v>
+        <v>2773000000</v>
       </c>
     </row>
     <row r="8">
@@ -695,16 +695,16 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>3716.2842</v>
+        <v>3716.2839</v>
       </c>
       <c r="F8" t="n">
-        <v>8.8081</v>
+        <v>8.8079</v>
       </c>
       <c r="G8" t="n">
         <v>0.24</v>
       </c>
       <c r="H8" t="n">
-        <v>18575544</v>
+        <v>472600</v>
       </c>
     </row>
     <row r="9">
@@ -729,16 +729,16 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>10849.6904</v>
+        <v>10881.9004</v>
       </c>
       <c r="F9" t="n">
-        <v>9.289999999999999</v>
+        <v>41.5</v>
       </c>
       <c r="G9" t="n">
-        <v>0.09</v>
+        <v>0.38</v>
       </c>
       <c r="H9" t="n">
-        <v>0</v>
+        <v>876343700</v>
       </c>
     </row>
     <row r="10">
@@ -763,16 +763,16 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>25636.8496</v>
+        <v>25622.6094</v>
       </c>
       <c r="F10" t="n">
-        <v>254.2305</v>
+        <v>239.9902</v>
       </c>
       <c r="G10" t="n">
-        <v>1</v>
+        <v>0.95</v>
       </c>
       <c r="H10" t="n">
-        <v>0</v>
+        <v>59759400</v>
       </c>
     </row>
     <row r="11">
@@ -806,7 +806,7 @@
         <v>0.22</v>
       </c>
       <c r="H11" t="n">
-        <v>0</v>
+        <v>305854400</v>
       </c>
     </row>
     <row r="12">
@@ -827,17 +827,17 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>18000</v>
+        <v>17943</v>
       </c>
       <c r="F12" t="n">
-        <v>176.3008</v>
+        <v>-77.0996</v>
       </c>
       <c r="G12" t="n">
-        <v>0.99</v>
+        <v>-0.43</v>
       </c>
       <c r="H12" t="n">
         <v>0</v>
@@ -861,17 +861,17 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>101.789</v>
+        <v>101.88</v>
       </c>
       <c r="F13" t="n">
-        <v>-0.211</v>
+        <v>0.04</v>
       </c>
       <c r="G13" t="n">
-        <v>-0.21</v>
+        <v>0.04</v>
       </c>
       <c r="H13" t="n">
         <v>0</v>
@@ -895,17 +895,17 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>158.037</v>
+        <v>157.807</v>
       </c>
       <c r="F14" t="n">
-        <v>0.08</v>
+        <v>-0.336</v>
       </c>
       <c r="G14" t="n">
-        <v>0.05</v>
+        <v>-0.21</v>
       </c>
       <c r="H14" t="n">
         <v>0</v>
@@ -933,13 +933,13 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>0.5114</v>
+        <v>0.5098</v>
       </c>
       <c r="F15" t="n">
-        <v>0.0025</v>
+        <v>0.0009</v>
       </c>
       <c r="G15" t="n">
-        <v>0.49</v>
+        <v>0.18</v>
       </c>
       <c r="H15" t="n">
         <v>0</v>
@@ -967,13 +967,13 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>0.5445</v>
+        <v>0.5436</v>
       </c>
       <c r="F16" t="n">
-        <v>0.0016</v>
+        <v>0.0007</v>
       </c>
       <c r="G16" t="n">
-        <v>0.29</v>
+        <v>0.13</v>
       </c>
       <c r="H16" t="n">
         <v>0</v>
@@ -1001,13 +1001,13 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>0.4068</v>
+        <v>0.407</v>
       </c>
       <c r="F17" t="n">
-        <v>-0.002</v>
+        <v>-0.0018</v>
       </c>
       <c r="G17" t="n">
-        <v>-0.49</v>
+        <v>-0.44</v>
       </c>
       <c r="H17" t="n">
         <v>0</v>
@@ -1031,20 +1031,20 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>79.97</v>
+        <v>80.05</v>
       </c>
       <c r="F18" t="n">
-        <v>1.08</v>
+        <v>0.08</v>
       </c>
       <c r="G18" t="n">
-        <v>1.37</v>
+        <v>0.1</v>
       </c>
       <c r="H18" t="n">
-        <v>86514400</v>
+        <v>42297400</v>
       </c>
     </row>
     <row r="19">
@@ -1065,20 +1065,20 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>77.13</v>
+        <v>76.86</v>
       </c>
       <c r="F19" t="n">
-        <v>0.32</v>
+        <v>-0.27</v>
       </c>
       <c r="G19" t="n">
-        <v>0.42</v>
+        <v>-0.35</v>
       </c>
       <c r="H19" t="n">
-        <v>80597700</v>
+        <v>76938700</v>
       </c>
     </row>
     <row r="20">
@@ -1099,20 +1099,20 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>4185.3999</v>
+        <v>4202.2998</v>
       </c>
       <c r="F20" t="n">
-        <v>15.2998</v>
+        <v>21.1997</v>
       </c>
       <c r="G20" t="n">
-        <v>0.37</v>
+        <v>0.51</v>
       </c>
       <c r="H20" t="n">
-        <v>58728</v>
+        <v>5386</v>
       </c>
     </row>
     <row r="21">
@@ -1133,20 +1133,20 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>95.78</v>
+        <v>97.93000000000001</v>
       </c>
       <c r="F21" t="n">
-        <v>-2.19</v>
+        <v>-3.48</v>
       </c>
       <c r="G21" t="n">
-        <v>-2.24</v>
+        <v>-3.43</v>
       </c>
       <c r="H21" t="n">
-        <v>81042</v>
+        <v>6387</v>
       </c>
     </row>
     <row r="22">
@@ -1167,20 +1167,20 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="E22" t="n">
-        <v>105.93</v>
+        <v>108.49</v>
       </c>
       <c r="F22" t="n">
-        <v>0.01</v>
+        <v>-1.37</v>
       </c>
       <c r="G22" t="n">
-        <v>0.01</v>
+        <v>-1.25</v>
       </c>
       <c r="H22" t="n">
-        <v>9046</v>
+        <v>588</v>
       </c>
     </row>
     <row r="23">
@@ -1201,20 +1201,20 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="E23" t="n">
-        <v>6.6255</v>
+        <v>6.5725</v>
       </c>
       <c r="F23" t="n">
-        <v>0.114</v>
+        <v>0.0415</v>
       </c>
       <c r="G23" t="n">
-        <v>1.75</v>
+        <v>0.64</v>
       </c>
       <c r="H23" t="n">
-        <v>15894</v>
+        <v>359</v>
       </c>
     </row>
     <row r="24">
@@ -1235,20 +1235,20 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="E24" t="n">
-        <v>63.96</v>
+        <v>62.85</v>
       </c>
       <c r="F24" t="n">
-        <v>-0.43</v>
+        <v>-1.11</v>
       </c>
       <c r="G24" t="n">
-        <v>-0.67</v>
+        <v>-1.74</v>
       </c>
       <c r="H24" t="n">
-        <v>23240000</v>
+        <v>31508800</v>
       </c>
     </row>
     <row r="25">
@@ -1273,13 +1273,13 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>15.98</v>
+        <v>19.99</v>
       </c>
       <c r="F25" t="n">
-        <v>-0.48</v>
+        <v>3.53</v>
       </c>
       <c r="G25" t="n">
-        <v>-2.92</v>
+        <v>21.45</v>
       </c>
       <c r="H25" t="n">
         <v>0</v>
@@ -1303,20 +1303,20 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="E26" t="n">
-        <v>81888.4219</v>
+        <v>81973.0938</v>
       </c>
       <c r="F26" t="n">
-        <v>-253.0391</v>
+        <v>590.9453</v>
       </c>
       <c r="G26" t="n">
-        <v>-0.31</v>
+        <v>0.73</v>
       </c>
       <c r="H26" t="n">
-        <v>30546599936</v>
+        <v>18388713472</v>
       </c>
     </row>
     <row r="27">
@@ -1350,7 +1350,7 @@
         <v>-14.79</v>
       </c>
       <c r="H27" t="n">
-        <v>202008600</v>
+        <v>206590200</v>
       </c>
     </row>
     <row r="28">
@@ -1384,7 +1384,7 @@
         <v>-14.84</v>
       </c>
       <c r="H28" t="n">
-        <v>79092200</v>
+        <v>89153400</v>
       </c>
     </row>
     <row r="29">
@@ -1418,7 +1418,7 @@
         <v>-14.29</v>
       </c>
       <c r="H29" t="n">
-        <v>69411800</v>
+        <v>86042800</v>
       </c>
     </row>
     <row r="30">
@@ -1452,7 +1452,7 @@
         <v>-14.91</v>
       </c>
       <c r="H30" t="n">
-        <v>40971900</v>
+        <v>41687500</v>
       </c>
     </row>
     <row r="31">
@@ -1486,7 +1486,7 @@
         <v>-14.8</v>
       </c>
       <c r="H31" t="n">
-        <v>24196600</v>
+        <v>25530400</v>
       </c>
     </row>
     <row r="32">
@@ -1520,7 +1520,7 @@
         <v>-14.77</v>
       </c>
       <c r="H32" t="n">
-        <v>65698800</v>
+        <v>71038700</v>
       </c>
     </row>
     <row r="33">
@@ -1554,7 +1554,7 @@
         <v>-14.78</v>
       </c>
       <c r="H33" t="n">
-        <v>22779700</v>
+        <v>25592500</v>
       </c>
     </row>
     <row r="34">
@@ -1588,7 +1588,7 @@
         <v>-14.94</v>
       </c>
       <c r="H34" t="n">
-        <v>7958900</v>
+        <v>8168700</v>
       </c>
     </row>
     <row r="35">
@@ -1622,7 +1622,7 @@
         <v>-14.89</v>
       </c>
       <c r="H35" t="n">
-        <v>27349300</v>
+        <v>44001300</v>
       </c>
     </row>
     <row r="36">
@@ -1656,7 +1656,7 @@
         <v>-14.67</v>
       </c>
       <c r="H36" t="n">
-        <v>100522400</v>
+        <v>107257500</v>
       </c>
     </row>
     <row r="37">
@@ -1690,7 +1690,7 @@
         <v>-14.92</v>
       </c>
       <c r="H37" t="n">
-        <v>1347700</v>
+        <v>1615300</v>
       </c>
     </row>
   </sheetData>
@@ -1749,22 +1749,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Intip Pembuatan Perahu Fiber untuk Nelayan di Kampung Nelayan Merah Putih</t>
+          <t>MSCI Soroti Masalah Bahasa-Transparansi Pasar Modal RI</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Fri, 16 Oct 2026 20:00:11 +0700</t>
+          <t>Mon, 19 Oct 2026 06:30:52 +0700</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/16/intip-pembuatan-perahu-fiber-untuk-nelayan-di-kampung-nelayan-merah-putih-1792117410032_169.jpeg?w=360&amp;amp;q=90" /&gt; Pekerja membuat perahu nelayan berbahan fiber di galangan Kampung Nelayan Merah Putih, Manokwari, Papua Barat.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/05/18/ihsg-anjlok-ke-zona-merah-bursa-saham-melemah-tajam-1779098741437_169.jpeg?w=360&amp;amp;q=90" /&gt; Lembaga penyedia indeks saham global, MSCI, buka-bukaan soal aksesibilitas pasar modal Indonesia.</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/foto-bisnis/d-8709506/intip-pembuatan-perahu-fiber-untuk-nelayan-di-kampung-nelayan-merah-putih</t>
+          <t>https://finance.detik.com/bursa-dan-valas/d-8713143/msci-soroti-masalah-bahasa-transparansi-pasar-modal-ri</t>
         </is>
       </c>
     </row>
@@ -1776,22 +1776,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Rincian Total Denda Rp 2,1 Triliun buat  DSSA hingga BREN</t>
+          <t>Persiapan Giant Sea Wall Pantura, Struktur Pemecah Ombak Disiapkan di Demak</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Fri, 16 Oct 2026 19:32:59 +0700</t>
+          <t>Mon, 19 Oct 2026 06:00:47 +0700</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/16/ihsg-ambruk-1157-ditutup-di-level-5185-1792144638939_169.jpeg?w=360&amp;amp;q=90" /&gt; Denda itu ditetapkan atas pelanggaran di bidang pasar modal yang dilakukan tiga emiten.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/18/persiapan-giant-sea-wall-pantura-struktur-pemecah-ombak-disiapkan-di-demak-1792305303554_169.jpeg?w=360&amp;amp;q=90" /&gt; Pekerja memasang Hex-Brick untuk pemecah ombak semipermeabel di pesisir Demak. Upaya ini menjadi bagian dari per</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/bursa-dan-valas/d-8710708/rincian-total-denda-rp-2-1-triliun-buat-dssa-hingga-bren</t>
+          <t>https://finance.detik.com/foto-bisnis/d-8712466/persiapan-giant-sea-wall-pantura-struktur-pemecah-ombak-disiapkan-di-demak</t>
         </is>
       </c>
     </row>
@@ -1803,22 +1803,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>1.550 Manajer Kopdes Minta Offering Ulang, Kemenkop: Mereka Menyesal Menolak</t>
+          <t>Perusahaan Haji Isam Gadai Saham, Duitnya buat Apa?</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Fri, 16 Oct 2026 19:00:42 +0700</t>
+          <t>Mon, 19 Oct 2026 05:55:54 +0700</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/04/18/penyerahan-truk-kdmp-di-temanggung-1776489684625_169.jpeg?w=360&amp;amp;q=90" /&gt; Kemenkop mencatat 1.550 manajer Koperasi Desa/Kelurahan Merah Putih (KDKMP) terkendala proses administrasi karena melewati batas waktu penandatanganan k</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/16/ihsg-ambruk-1157-ditutup-di-level-5185-1792144638939_169.jpeg?w=360&amp;amp;q=90" /&gt; PT Bank Mandiri (Persero) Tbk (BMRI) buka-bukaan soal alokasi kredit dari aksi gadai saham dua perusahaan milik Andi Syamsuddin Arsyad alias Haji Is</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8710664/1-550-manajer-kopdes-minta-offering-ulang-kemenkop-mereka-menyesal-menolak</t>
+          <t>https://finance.detik.com/bursa-dan-valas/d-8712880/perusahaan-haji-isam-gadai-saham-duitnya-buat-apa</t>
         </is>
       </c>
     </row>
@@ -1830,22 +1830,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Perkuat Ekosistem Wakaf Produktif, BSI Dorong Potensi Rp 180 Triliun</t>
+          <t>Menyesap Harum Kopi Indonesia di Tokyo</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Fri, 16 Oct 2026 18:20:02 +0700</t>
+          <t>Mon, 19 Oct 2026 00:00:00 +0700</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/16/bsi-1792149584130.jpeg?w=360&amp;amp;q=90" /&gt; PT Bank Syariah Indonesia (BSI) dorong pengembangan wakaf produktif di GLOW 2026. BSI optimis wakaf bisa tingkatkan kesejahteraan dan ketahanan ekonomi umat.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/18/adv-bank-indonesi-1792334493519.jpeg?w=360&amp;amp;q=90" /&gt; Tepat pukul 10.00 tanggal 14 Oktober 2026, pameran Specialty Coffee Association of Japan (SCAJ) World Specialty Coffee Conference and Exhibition 2026</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8710593/perkuat-ekosistem-wakaf-produktif-bsi-dorong-potensi-rp-180-triliun</t>
+          <t>https://finance.detik.com/advertorial-news-block/d-8713009/menyesap-harum-kopi-indonesia-di-tokyo</t>
         </is>
       </c>
     </row>
@@ -1857,22 +1857,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Dukung Ekspor UMKM, Astra Pamerkan Produk Lokal Unggulan di TEI 2026</t>
+          <t>Perajin Batik Rifaiyah Batang Didorong Naik Kelas Lewat Kenduri Batik 2026</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Fri, 16 Oct 2026 18:19:50 +0700</t>
+          <t>Sun, 18 Oct 2026 22:30:51 +0700</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/16/dukung-ekspor-umkm-astra-pamerkan-produk-lokal-unggulan-di-tei-2026-1792149478736_169.jpeg?w=360&amp;amp;q=90" /&gt; PT Astra International mendukung ekspor UMKM di Trade Expo Indonesia 2026. 30 peserta tampilkan produk unggulan dari De</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/18/perajin-batik-rifaiyah-batang-didorong-naik-kelas-lewat-kenduri-batik-2026-1792304249394_169.jpeg?w=360&amp;amp;q=90" /&gt; Kenduri Batik Batang 2026 menjadi wadah perajin Batik Rifaiyah mengembangkan usaha. Kegiatan ini mendorong inova</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8710592/dukung-ekspor-umkm-astra-pamerkan-produk-lokal-unggulan-di-tei-2026</t>
+          <t>https://finance.detik.com/foto-bisnis/d-8712436/perajin-batik-rifaiyah-batang-didorong-naik-kelas-lewat-kenduri-batik-2026</t>
         </is>
       </c>
     </row>
@@ -1884,22 +1884,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>IHSG Ambruk 11,57%, Ditutup di Level 5.185</t>
+          <t>3 Cara Maksimalkan Penggunaan QRIS untuk Bantu Bisnis Berkembang</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Fri, 16 Oct 2026 18:04:47 +0700</t>
+          <t>Sun, 18 Oct 2026 22:00:51 +0700</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/16/ihsg-ambruk-1157-ditutup-di-level-5185-1792144639064.jpeg?w=360&amp;amp;q=90" /&gt; IHSG anjlok 11,57% ke level 5.185,11, di tengah konsultasi publik MSCI terkait rencana reklasifikasi pasar saham Indonesia menjadi Standalone Market.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/18/ilustrasi-qr-1792334198806.jpeg?w=360&amp;amp;q=90" /&gt; Optimalkan bisnis Anda dengan QRIS! Pelajari cara mempermudah transaksi, manfaatkan MDR 0%, dan daftar DANA Bisnis untuk keuntungan maksimal.</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/foto-bisnis/d-8710404/ihsg-ambruk-11-57-ditutup-di-level-5-185</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8713018/3-cara-maksimalkan-penggunaan-qris-untuk-bantu-bisnis-berkembang</t>
         </is>
       </c>
     </row>
@@ -1911,22 +1911,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Pemerintah Belum Putuskan Pembelian Pertalite Pakai Desil 9-10</t>
+          <t>Kilang Plaju Produksi Avtur 295 Ribu Barel hingga September</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Fri, 16 Oct 2026 17:44:41 +0700</t>
+          <t>Sun, 18 Oct 2026 22:00:07 +0700</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/15/warga-blitar-antre-panjang-untuk-mendapatkan-pertalite-1792054696805_169.jpeg?w=360&amp;amp;q=90" /&gt; Pemerintah belum memutuskan pembelian Pertalite untuk desil 9-10. Rencana ini masih dalam pengkajian dan diskusi, dengan kemungkinan</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/10/25/perwira-pertamina-perempuan-di-kilang-plaju-saat-melakukan-tugasnya-memonitor-mesin-produksi-polypropylene-1761406552564_169.jpeg?w=360&amp;amp;q=90" /&gt; Kilang Plaju mencatat produksi bahan bakar pesawat atau avtur sebesar 295.263 ba</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8710521/pemerintah-belum-putuskan-pembelian-pertalite-pakai-desil-9-10</t>
+          <t>https://finance.detik.com/energi/d-8712759/kilang-plaju-produksi-avtur-295-ribu-barel-hingga-september</t>
         </is>
       </c>
     </row>
@@ -1938,22 +1938,22 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Bahlil Sebut Penyusunan DIM RUU Migas Sudah 90%</t>
+          <t>Mau Pakai QRIS untuk Jualan? Cek Cara Ini biar Tak Kena Potongan Biaya</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Fri, 16 Oct 2026 17:26:01 +0700</t>
+          <t>Sun, 18 Oct 2026 21:48:34 +0700</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/07/16/menteri-esdm-bahlil-lahadalia-1784186781817_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri ESDM Bahlil mengungkapkan RUU Migas hampir rampung, dengan progres 90%. Pembentukan Badan Usaha Khusus jadi fokus utama. Target DIM selesai 22 Oktobe</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/21/ilustrasi-qris-1789973868497.png?w=360&amp;amp;q=90" /&gt; Pembayaran QRIS semakin mudah, dengan program MDR 0% untuk UMKM. Nikmati transaksi tanpa potongan biaya dan tingkatkan efisiensi bisnis Anda.</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8710446/bahlil-sebut-penyusunan-dim-ruu-migas-sudah-90</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8713015/mau-pakai-qris-untuk-jualan-cek-cara-ini-biar-tak-kena-potongan-biaya</t>
         </is>
       </c>
     </row>
@@ -1965,22 +1965,22 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Pengguna Pertamax Ramai-ramai Pindah ke Pertalite, Stok Ikut Turun</t>
+          <t>Tanjung Perak Jadi Lokasi Pertama Uji Coba Penertiban Kendaraan ODOL</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Fri, 16 Oct 2026 16:58:49 +0700</t>
+          <t>Sun, 18 Oct 2026 21:00:38 +0700</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/01/bahlil-lahadalia-1790850102759_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri ESDM Bahlil mengonfirmasi penurunan stok Pertalite menjadi 16-18 hari akibat pergeseran konsumsi. Ia memastikan stok aman dan normal dalam seminggu.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/06/20/ratusan-truk-blokade-jalur-pantura-alas-roban-batang-1750397214314_169.jpeg?w=360&amp;amp;q=90" /&gt; Pelabuhan Tanjung Perak, Surabaya akan menjadi lokasi pertama dalam penertiban kendaraan Over Dimension Over Loading (ODOL) yang diang</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8710388/pengguna-pertamax-ramai-ramai-pindah-ke-pertalite-stok-ikut-turun</t>
+          <t>https://finance.detik.com/infrastruktur/d-8712817/tanjung-perak-jadi-lokasi-pertama-uji-coba-penertiban-kendaraan-odol</t>
         </is>
       </c>
     </row>
@@ -1992,22 +1992,22 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Manajer Kopdes Merah Putih Jadi Pegawai Koperasi Usai Dikontrak 2 Tahun</t>
+          <t>BI Dorong Transaksi Pakai Mata Uang Lokal di Pertemuan IMF-Bank Dunia</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Fri, 16 Oct 2026 16:51:48 +0700</t>
+          <t>Sun, 18 Oct 2026 20:00:30 +0700</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/16/deputi-bidang-pengembangan-talenta-dan-daya-saing-koperasi-destry-anna-sari-1792139643262_169.jpeg?w=360&amp;amp;q=90" /&gt; Ya, jadi pegawai koperasi. Pegawai koperasi itu keren loh, ujar Destry.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/23/bi-pertahankan-suku-bunga-575-persen-fokus-jaga-stabilitas-rupiah-1790154587213_169.jpeg?w=360&amp;amp;q=90" /&gt; Bank Indonesia mendorong perluasan penggunaan mata mata uang lokal (Local Currency Transaction/LCT) dalam perdagangan dan</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8710380/manajer-kopdes-merah-putih-jadi-pegawai-koperasi-usai-dikontrak-2-tahun</t>
+          <t>https://finance.detik.com/moneter/d-8712864/bi-dorong-transaksi-pakai-mata-uang-lokal-di-pertemuan-imf-bank-dunia</t>
         </is>
       </c>
     </row>
@@ -2019,22 +2019,22 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>IHSG Ambruk 11,57% ke 5.185 Dibayangi Ancaman Downgrade MSCI</t>
+          <t>Transaksi Trade Expo Indonesia Tembus Rp 414 Triliun</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Fri, 16 Oct 2026 16:34:54 +0700</t>
+          <t>Sun, 18 Oct 2026 19:31:01 +0700</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/05/18/ihsg-anjlok-ke-zona-merah-bursa-saham-melemah-tajam-1779098741262_169.jpeg?w=360&amp;amp;q=90" /&gt; Indeks Harga Saham Gabungan (IHSG) ditutup anjlok 678,67 poin (11,57%) ke 5.185 atau anjlok 678,67 poin (11,57%).</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/18/menteri-perdagangan-budi-santoso-1792326567826_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Perdagangan Budi Santoso menyampaikan nilai transaksi Trade Expo Indonesia (TEI) ke-41 mencapai US$ 22,94 miliar atau setara sekitar Rp 414 triliu</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/bursa-dan-valas/d-8710354/ihsg-ambruk-11-57-ke-5-185-dibayangi-ancaman-downgrade-msci</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8712868/transaksi-trade-expo-indonesia-tembus-rp-414-triliun</t>
         </is>
       </c>
     </row>
@@ -2046,22 +2046,22 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Hadapi Tantangan Global, CIMB Gelar Acara Bahas AI hingga Supply Chain</t>
+          <t>34 Lembaga Keuangan Berminat Biayai Proyek Sampah Jadi Listrik</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Fri, 16 Oct 2026 16:17:33 +0700</t>
+          <t>Sun, 18 Oct 2026 19:00:27 +0700</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/16/cimb-1792142228196_169.jpeg?w=360&amp;amp;q=90" /&gt; CIMB Niaga menggelar Business Summit 2026 untuk bahas tantangan ekonomi global, AI, dan supply chain.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/07/01/wisma-danantara-indonesia-1751345496063_169.jpeg?w=360&amp;amp;q=90" /&gt; Danantara menetapkan 34 institusi keuangan sebagai anggota lenders panel untuk program Pengolahan Sampah menjadi Energi Listrik (PSEL).</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8710321/hadapi-tantangan-global-cimb-gelar-acara-bahas-ai-hingga-supply-chain</t>
+          <t>https://finance.detik.com/energi/d-8712594/34-lembaga-keuangan-berminat-biayai-proyek-sampah-jadi-listrik</t>
         </is>
       </c>
     </row>
@@ -2073,22 +2073,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Bareskrim Polri Turun Tangan Awasi Pelanggaran di Bursa</t>
+          <t>OJK &amp;amp; BEI Kumpulkan AB-Analis Usai IHSG Rontok Imbas Pengumuman MSCI</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Fri, 16 Oct 2026 16:17:15 +0700</t>
+          <t>Sun, 18 Oct 2026 17:43:11 +0700</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/01/30/ihsg-rebound-usai-dua-hari-anjlok-seiring-pengunduran-diri-dirut-bei-1769748663323_169.jpeg?w=360&amp;amp;q=90" /&gt; Kapolri Suyudi Ario Seto menyatakan Bareskrim Polri bakal turun tangan mengawasi langsung Bursa Efek Indonesia.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/06/03/ihsg-anjlok-411-persen-ke-level-5941-1780494579470_169.jpeg?w=360&amp;amp;q=90" /&gt; Otoritas Jasa Keuangan (OJK) dan Bursa Efek Indonesia (BEI) mengumpulkan analis dan anggota bursa (AB) hari ini, Minggu (18/10/2026).</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/bursa-dan-valas/d-8710320/bareskrim-polri-turun-tangan-awasi-pelanggaran-di-bursa</t>
+          <t>https://finance.detik.com/bursa-dan-valas/d-8712753/ojk-bei-kumpulkan-ab-analis-usai-ihsg-rontok-imbas-pengumuman-msci</t>
         </is>
       </c>
     </row>
@@ -2100,22 +2100,22 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Manajer Tetap Digaji Meski Kopdes Belum Beroperasi</t>
+          <t>IHSG Masih Diprediksi Rawan Longsor Usai Pengumuman MSCI</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Fri, 16 Oct 2026 16:09:15 +0700</t>
+          <t>Sun, 18 Oct 2026 17:00:46 +0700</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/16/deputi-bidang-pengembangan-talenta-dan-daya-saing-koperasi-destry-anna-sari-1792139643262_169.jpeg?w=360&amp;amp;q=90" /&gt; Kementerian Koperasi (Kemenkop) memastikan semua manajer Koperasi Desa/Kelurahan Merah Putih (KDKMP) yang telah</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/01/28/bei-terapkan-trading-halt-imbas-ihsg-anjlok-1769587530913_169.jpeg?w=360&amp;amp;q=90" /&gt; Indeks Harga Saham Gabungan (IHSG) berpotensi melanjutkan pelemahan di perdagangan Senin (19/10/2026).</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8710302/manajer-tetap-digaji-meski-kopdes-belum-beroperasi</t>
+          <t>https://finance.detik.com/bursa-dan-valas/d-8712545/ihsg-masih-diprediksi-rawan-longsor-usai-pengumuman-msci</t>
         </is>
       </c>
     </row>
@@ -2127,22 +2127,22 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>IHSG Ambles 11%, Bos Danantara Lihat Peluang Borong Saham</t>
+          <t>Harga Emas Antam Anjlok dalam Sepekan, Begini Pergerakannya</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Fri, 16 Oct 2026 16:05:50 +0700</t>
+          <t>Sun, 18 Oct 2026 16:00:10 +0700</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/02/menteri-investasi-dan-hilirisasikepala-bkpm-sekaligus-ceo-badan-pengelola-investasi-bpi-danantara-rosan-roeslani-di-sebuah-hot-1790942979284_169.jpeg?w=360&amp;amp;q=90" /&gt; CEO Danantara, Rosan Roeslani, menanggapi penurunan IHSG 11%</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/10/22/harga-emas-terjun-bebas-pasar-cikini-langsung-diserbu-pembeli-1761123863171_169.jpeg?w=360&amp;amp;q=90" /&gt; Harga emas Antam 24 karat sepanjang perdagangan 12-17 Oktober 2026 turun sebesar Rp 22.000 per gram.</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/bursa-dan-valas/d-8710294/ihsg-ambles-11-bos-danantara-lihat-peluang-borong-saham</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8712537/harga-emas-antam-anjlok-dalam-sepekan-begini-pergerakannya</t>
         </is>
       </c>
     </row>
@@ -2154,22 +2154,22 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Penampakan Bupati Klaten Hamenang Usai Diperiksa KPK</t>
+          <t>Bertemu Prabowo, Sekjen PBB Apresiasi Peran Indonesia untuk Palestina</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Fri, 16 Oct 2026 19:42:50 +0700</t>
+          <t>Mon, 19 Oct 2026 06:32:47 +0700</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Bupati Klaten Hamenang mengenakan rompi oranye khas tahanan KPK saat keluar dari Gedung Merah Putih KPK.</t>
+          <t>Sekjen PBB António Guterres berpamitan kepada Presiden Prabowo menjelang akhir masa jabatannya pada Desember 2026 dan mengapresiasi dukungan Indonesia bagi Palestina serta misi perdamaian PBB.</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8315024/penampakan-bupati-klaten-hamenang-usai-diperiksa-kpk</t>
+          <t>https://www.liputan6.com/news/read/8316023/bertemu-prabowo-sekjen-pbb-apresiasi-peran-indonesia-untuk-palestina</t>
         </is>
       </c>
     </row>
@@ -2181,22 +2181,22 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Kasus Dugaan Kekerasan Dipicu Kembang Api, Pelapor Dipanggil Polisi</t>
+          <t>DPR Buka-bukaan soal Polemik Syarat Pendidikan Capres-Cawapres di PKPU</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Fri, 16 Oct 2026 19:31:21 +0700</t>
+          <t>Mon, 19 Oct 2026 06:00:39 +0700</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Amanda Andono memenuhi panggilan Polda Metro Jaya untuk menjelaskan kronologi dugaan kekerasan yang dialaminya di Pondok Pinang.</t>
+          <t>Ahmad Doli Kurnia menyatakan Pasal 18 ayat (3) PKPU Nomor 19 Tahun 2023 tidak tercantum dalam draf yang dibahas Komisi II DPR saat konsultasi penyusunan aturan tersebut.</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8315009/kasus-dugaan-kekerasan-dipicu-kembang-api-pelapor-dipanggil-polisi</t>
+          <t>https://www.liputan6.com/news/read/8316016/dpr-buka-bukaan-soal-polemik-syarat-pendidikan-capres-cawapres-di-pkpu</t>
         </is>
       </c>
     </row>
@@ -2208,22 +2208,22 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Putusan MK Buka Jalan Pengusutan Kasus Andrie Yunus di Peradilan Umum</t>
+          <t>7 Perjalanan KRL Bogor Dibatalkan Hari Ini, Cek Jadwalnya</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Fri, 16 Oct 2026 19:25:00 +0700</t>
+          <t>Mon, 19 Oct 2026 05:35:40 +0700</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Tim Advokasi mendesak Polda Metro Jaya mengusut 16 orang terkait kasus Andrie Yunus.</t>
+          <t>KAI Commuter membatalkan tujuh perjalanan lintas Bogor pada Senin (19/10/2026) karena dua rangkaian kereta masih diperbaiki. Pengguna diminta mengecek jadwal dan alternatif perjalanan.</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8315000/putusan-mk-buka-jalan-pengusutan-kasus-andrie-yunus-di-peradilan-umum</t>
+          <t>https://www.liputan6.com/news/read/8316013/7-perjalanan-krl-bogor-dibatalkan-hari-ini-cek-jadwalnya</t>
         </is>
       </c>
     </row>
@@ -2235,22 +2235,22 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>DPR Desak Kemenhut Gerak Cepat Tangani Kebakaran Hutan</t>
+          <t>Prakiraan Cuaca Jakarta 19 Oktober: Jaksel dan Jaktim Berpotensi Hujan</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Fri, 16 Oct 2026 19:05:52 +0700</t>
+          <t>Mon, 19 Oct 2026 05:20:05 +0700</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Desakan ini muncul setelah jumlah titik panas nasional mencapai 799 titik pada 15 Oktober 2026.</t>
+          <t>BMKG memprakirakan hujan ringan berpotensi mengguyur Jakarta Selatan dan Jakarta Timur pada sore hingga malam hari, sementara wilayah lainnya cenderung berawan hingga cerah berawan.</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8314914/dpr-desak-kemenhut-gerak-cepat-tangani-kebakaran-hutan</t>
+          <t>https://www.liputan6.com/news/read/8316012/prakiraan-cuaca-jakarta-19-oktober-jaksel-dan-jaktim-berpotensi-hujan</t>
         </is>
       </c>
     </row>
@@ -2262,22 +2262,22 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Terungkap Identitas Terduga Pelaku Pencambukan di KPPG Bogor</t>
+          <t>Kronologi Bharada Valdo Tewas Ditembak Rekan Sesama Polisi</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Fri, 16 Oct 2026 19:14:07 +0700</t>
+          <t>Mon, 19 Oct 2026 05:08:04 +0700</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Identitas keduanya terungkap usai polisi mendatangi lokasi kejadian dan memeriksa sejumlah saksi.</t>
+          <t>Bharada Valdo tewas dalam insiden penembakan di Markas Polairud Pondok Cabe. Pengacara keluarga menduga pembunuhan berencana dan meminta penyidik mendalami kemungkinan keterlibatan pihak lain.</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8314997/terungkap-identitas-terduga-pelaku-pencambukan-di-kppg-bogor</t>
+          <t>https://www.liputan6.com/news/read/8316006/kronologi-bharada-valdo-tewas-ditembak-rekan-sesama-polisi</t>
         </is>
       </c>
     </row>
@@ -2289,22 +2289,22 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Mengenal Dana Bencana yang Terseret Kasus Korupsi BNPB</t>
+          <t>Kronologi Tawuran di Manggarai hingga Kios Dibakar, 6 Orang Ditangkap</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Fri, 16 Oct 2026 18:13:59 +0700</t>
+          <t>Mon, 19 Oct 2026 00:27:21 +0700</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>KPK membeberkan dugaan penyalahgunaan dana kebencanaan BNPB melalui pengadaan barang dan jasa.</t>
+          <t>Keenam orang itu masih menjalani pemeriksaan untuk mendalami peran masing-masing.</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8314950/mengenal-dana-bencana-yang-terseret-kasus-korupsi-bnpb</t>
+          <t>https://www.liputan6.com/news/read/8315986/kronologi-tawuran-di-manggarai-hingga-kios-dibakar-6-orang-ditangkap</t>
         </is>
       </c>
     </row>
@@ -2316,22 +2316,22 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Asap Karhutla Kalimantan Masuk Atmosfer Jakarta, Ini yang Perlu Dilakukan</t>
+          <t>Survei PPI, Erick Thohir Masuk 3 Besar Menteri Berkinerja Terbaik</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Fri, 16 Oct 2026 18:06:00 +0700</t>
+          <t>Sun, 18 Oct 2026 22:32:43 +0700</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Warga diimbau batasi aktivitas luar ruangan dan wajib memakai masker.</t>
+          <t>Erick Thohir dinilai berkinerja baik terutama karena performa Timnas Indonesia yang dianggap semakin meningkat.</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8314949/asap-karhutla-kalimantan-masuk-atmosfer-jakarta-ini-yang-perlu-dilakukan</t>
+          <t>https://www.liputan6.com/news/read/8315941/survei-ppi-erick-thohir-masuk-3-besar-menteri-berkinerja-terbaik</t>
         </is>
       </c>
     </row>
@@ -2343,22 +2343,22 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Kopdes Merah Putih Bisa Jual Obat Bebas, Skema Distribusi Disiapkan</t>
+          <t>Satgas Damai Cartenz Bongkar Markas KKB, Temukan 559 Selongsong Peluru</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Fri, 16 Oct 2026 17:37:21 +0700</t>
+          <t>Sun, 18 Oct 2026 21:48:21 +0700</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Gerai Kopdes Merah Putih disiapkan menjadi alternatif akses obat bagi masyarakat.</t>
+          <t>Di dalam honai ditemukan 559 selongsong peluru kaliber 5,56 mm dan sejumlah barang bukti lainnya.</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8314923/kopdes-merah-putih-bisa-jual-obat-bebas-skema-distribusi-disiapkan</t>
+          <t>https://www.liputan6.com/news/read/8315923/satgas-damai-cartenz-bongkar-markas-kkb-temukan-559-selongsong-peluru</t>
         </is>
       </c>
     </row>
@@ -2370,22 +2370,22 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Kongkalikong Tilap Dana Bencana: KPK Bongkar 2 Klaster Korupsi BNPB</t>
+          <t>Polisi Tembak Polisi di Markas Polairud Tangsel</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Fri, 16 Oct 2026 17:31:21 +0700</t>
+          <t>Sun, 18 Oct 2026 21:01:25 +0700</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>KPK membongkar ada dua klaster korupsi dana bencana di BNPB.</t>
+          <t>Tersangka berinisial AR, yang juga merupakan anggota Polri, telah diamankan.</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8314913/kongkalikong-tilap-dana-bencana-kpk-bongkar-2-klaster-korupsi-bnpb</t>
+          <t>https://www.liputan6.com/news/read/8315898/polisi-tembak-polisi-di-markas-polairud-tangsel</t>
         </is>
       </c>
     </row>
@@ -2397,22 +2397,22 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>KPK: Dana Bencana BNPB Diduga Dipakai Beli Saham Rp 30,98 Miliar</t>
+          <t>Sekjen PBB Temui Prabowo di Hambalang, Ini yang Dibahas</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Fri, 16 Oct 2026 17:22:20 +0700</t>
+          <t>Sun, 18 Oct 2026 19:22:20 +0700</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Kepemilikan saham tercatat mencapai 150,4 juta lembar atau setara 1,07 persen.</t>
+          <t>Prabowo menyambut langsung kedatangan Guterres saat turun dari kendaraan. Guterres dan rombongan terlihat kompak mengenakan batik.</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8314910/kpk-dana-bencana-bnpb-diduga-dipakai-beli-saham-rp-3098-miliar</t>
+          <t>https://www.liputan6.com/news/read/8315845/sekjen-pbb-temui-prabowo-di-hambalang-ini-yang-dibahas</t>
         </is>
       </c>
     </row>
@@ -2424,22 +2424,22 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Korupsi BNPB: Dana Karhutla Kalimantan, Gempa NTT Hingga Banjir Sumatra</t>
+          <t>Wamendagri Bima Arya Dorong Humas Pemerintah Lebih Dekat dengan Rakyat</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Fri, 16 Oct 2026 17:09:04 +0700</t>
+          <t>Sun, 18 Oct 2026 18:47:00 +0700</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Dana darurat untuk penanganan bencana seperti Karhutla Kalimantan dan Gempa NTT ini diduga disalahgunakan melalui suap dan konflik kepentingan.</t>
+          <t>Bima menjelaskan bahwa komunikasi publik perlu didasarkan pada pemahaman terhadap kebutuhan dan aspirasi masyarakat.</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8314899/korupsi-bnpb-dana-karhutla-kalimantan-gempa-ntt-hingga-banjir-sumatra</t>
+          <t>https://www.liputan6.com/news/read/8315833/wamendagri-bima-arya-dorong-humas-pemerintah-lebih-dekat-dengan-rakyat</t>
         </is>
       </c>
     </row>
@@ -2451,22 +2451,22 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>OTT BNPB, KPK Sita Uang Asing hingga Kepingan Emas Senilai Rp 5,47 miliar</t>
+          <t>Kronologi Pelari ITB Ultra Marathon Meninggal Saat Melintas di Cianjur</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Fri, 16 Oct 2026 17:07:41 +0700</t>
+          <t>Sun, 18 Oct 2026 18:43:59 +0700</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>KPK menyita barang bukti lebih kurang mencapai Rp 5,47 miliar dari OTT di Badan Nasional Penanggulangan Bencana (BNPB).</t>
+          <t>Pihak kampus dan panitia menyampaikan belasungkawa.</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8314897/ott-bnpb-kpk-sita-uang-asing-hingga-kepingan-emas-senilai-rp-547-miliar</t>
+          <t>https://www.liputan6.com/news/read/8315832/kronologi-pelari-itb-ultra-marathon-meninggal-saat-melintas-di-cianjur</t>
         </is>
       </c>
     </row>
@@ -2478,22 +2478,22 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>KPK Tetapkan 5 Tersangka Kasus Korupsi Dana Bencana BNPB</t>
+          <t>Kemensos Gelar Anugerah Jurnalistik Sekolah Rakyat 2026, Gus Ipul Soroti Peran Penting Media</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Fri, 16 Oct 2026 16:59:27 +0700</t>
+          <t>Sun, 18 Oct 2026 18:08:15 +0700</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>KPK juga mengamankan barang bukti dengan nilai total sekitar Rp 5,47 miliar.</t>
+          <t>BRI Peduli melibatkan 500 relawan dan menyediakan RVM untuk mendukung pengelolaan sampah selama MotoGP Mandalika 2026.</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8314889/kpk-tetapkan-5-tersangka-kasus-korupsi-dana-bencana-bnpb</t>
+          <t>https://www.liputan6.com/news/read/8315820/kemensos-gelar-anugerah-jurnalistik-sekolah-rakyat-2026-gus-ipul-soroti-peran-penting-media</t>
         </is>
       </c>
     </row>
@@ -2505,22 +2505,22 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Penjelasan BMKG soal Sebaran Asap Kebakaran Hutan Terdeteksi di Jakarta</t>
+          <t>Seskab Teddy Masuk Dua Besar Menteri Terbaik Versi Survei PPI</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Fri, 16 Oct 2026 16:02:00 +0700</t>
+          <t>Sun, 18 Oct 2026 22:01:03 +0700</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Arah angin membawa asap ini melintasi wilayah Jawa.</t>
+          <t>Di bawah mereka, Menteri Sosial Saifullah Yusuf memperoleh 4,5 persen, Menteri Koordinator Bidang Hilirisasi dan Investasi Bahlil Lahadalia 3,2 persen.</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8314841/penjelasan-bmkg-soal-sebaran-asap-kebakaran-hutan-terdeteksi-di-jakarta</t>
+          <t>https://www.liputan6.com/news/read/8315807/seskab-teddy-masuk-dua-besar-menteri-terbaik-versi-survei-ppi</t>
         </is>
       </c>
     </row>
@@ -2532,22 +2532,22 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Kapolri Usut Dugaan Pidana Pasar Modal Imbas IHSG Anjlok</t>
+          <t>Mantan Kadivhubinter Polri Napoleon Bonaparte Meninggal Dunia</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Fri, 16 Oct 2026 15:58:20 +0700</t>
+          <t>Sun, 18 Oct 2026 15:29:43 +0700</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Penyidik Polri akan mengumpulkan alat bukti sebelum mengambil tindakan hukum.</t>
+          <t>Napoleon Bonaparte dikabarkan meninggal akibat sakit.</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8314833/kapolri-usut-dugaan-pidana-pasar-modal-imbas-ihsg-anjlok</t>
+          <t>https://www.liputan6.com/news/read/8315754/mantan-kadivhubinter-polri-napoleon-bonaparte-meninggal-dunia</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data pasar & berita - 2026-10-19 15:25 UTC
</commit_message>
<xml_diff>
--- a/data/market_news_latest.xlsx
+++ b/data/market_news_latest.xlsx
@@ -487,20 +487,20 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>5185.105</v>
+        <v>4996.6089</v>
       </c>
       <c r="F2" t="n">
-        <v>-678.6748</v>
+        <v>-188.4961</v>
       </c>
       <c r="G2" t="n">
-        <v>-11.57</v>
+        <v>-3.64</v>
       </c>
       <c r="H2" t="n">
-        <v>650917300</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -521,20 +521,20 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>7659.4399</v>
+        <v>7723.46</v>
       </c>
       <c r="F3" t="n">
-        <v>-84.62009999999999</v>
+        <v>64.02</v>
       </c>
       <c r="G3" t="n">
-        <v>-1.09</v>
+        <v>0.84</v>
       </c>
       <c r="H3" t="n">
-        <v>5482060000</v>
+        <v>742614434</v>
       </c>
     </row>
     <row r="4">
@@ -555,20 +555,20 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>52002.4102</v>
+        <v>52095.4219</v>
       </c>
       <c r="F4" t="n">
-        <v>-175.2812</v>
+        <v>93.0117</v>
       </c>
       <c r="G4" t="n">
-        <v>-0.34</v>
+        <v>0.18</v>
       </c>
       <c r="H4" t="n">
-        <v>488090000</v>
+        <v>130641455</v>
       </c>
     </row>
     <row r="5">
@@ -589,20 +589,20 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>26140.0293</v>
+        <v>26576.4297</v>
       </c>
       <c r="F5" t="n">
-        <v>-573</v>
+        <v>436.4004</v>
       </c>
       <c r="G5" t="n">
-        <v>-2.15</v>
+        <v>1.67</v>
       </c>
       <c r="H5" t="n">
-        <v>9505000000</v>
+        <v>2719384000</v>
       </c>
     </row>
     <row r="6">
@@ -691,20 +691,20 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>3716.2839</v>
+        <v>3730.9199</v>
       </c>
       <c r="F8" t="n">
-        <v>8.8079</v>
+        <v>14.636</v>
       </c>
       <c r="G8" t="n">
-        <v>0.24</v>
+        <v>0.39</v>
       </c>
       <c r="H8" t="n">
-        <v>472600</v>
+        <v>3124419136</v>
       </c>
     </row>
     <row r="9">
@@ -725,20 +725,20 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>10881.9004</v>
+        <v>10730.4805</v>
       </c>
       <c r="F9" t="n">
-        <v>41.5</v>
+        <v>-151.4199</v>
       </c>
       <c r="G9" t="n">
-        <v>0.38</v>
+        <v>-1.39</v>
       </c>
       <c r="H9" t="n">
-        <v>876343700</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -759,20 +759,20 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>25622.6094</v>
+        <v>25211.3906</v>
       </c>
       <c r="F10" t="n">
-        <v>239.9902</v>
+        <v>-411.2188</v>
       </c>
       <c r="G10" t="n">
-        <v>0.95</v>
+        <v>-1.6</v>
       </c>
       <c r="H10" t="n">
-        <v>59759400</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -793,20 +793,20 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>5415.5298</v>
+        <v>5412</v>
       </c>
       <c r="F11" t="n">
-        <v>12.0298</v>
+        <v>-3.5298</v>
       </c>
       <c r="G11" t="n">
-        <v>0.22</v>
+        <v>-0.07000000000000001</v>
       </c>
       <c r="H11" t="n">
-        <v>305854400</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -861,17 +861,17 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>101.88</v>
+        <v>101.939</v>
       </c>
       <c r="F13" t="n">
-        <v>0.04</v>
+        <v>0.099</v>
       </c>
       <c r="G13" t="n">
-        <v>0.04</v>
+        <v>0.1</v>
       </c>
       <c r="H13" t="n">
         <v>0</v>
@@ -899,13 +899,13 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>157.807</v>
+        <v>158.41</v>
       </c>
       <c r="F14" t="n">
-        <v>-0.336</v>
+        <v>0.267</v>
       </c>
       <c r="G14" t="n">
-        <v>-0.21</v>
+        <v>0.17</v>
       </c>
       <c r="H14" t="n">
         <v>0</v>
@@ -929,17 +929,17 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>0.5098</v>
+        <v>0.5127</v>
       </c>
       <c r="F15" t="n">
-        <v>0.0009</v>
+        <v>0.0029</v>
       </c>
       <c r="G15" t="n">
-        <v>0.18</v>
+        <v>0.57</v>
       </c>
       <c r="H15" t="n">
         <v>0</v>
@@ -963,17 +963,17 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>0.5436</v>
+        <v>0.5465</v>
       </c>
       <c r="F16" t="n">
-        <v>0.0007</v>
+        <v>0.0029</v>
       </c>
       <c r="G16" t="n">
-        <v>0.13</v>
+        <v>0.53</v>
       </c>
       <c r="H16" t="n">
         <v>0</v>
@@ -997,17 +997,17 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>0.407</v>
+        <v>0.4077</v>
       </c>
       <c r="F17" t="n">
-        <v>-0.0018</v>
+        <v>0.0007</v>
       </c>
       <c r="G17" t="n">
-        <v>-0.44</v>
+        <v>0.17</v>
       </c>
       <c r="H17" t="n">
         <v>0</v>
@@ -1031,20 +1031,20 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>80.05</v>
+        <v>79.61499999999999</v>
       </c>
       <c r="F18" t="n">
-        <v>0.08</v>
+        <v>-0.435</v>
       </c>
       <c r="G18" t="n">
-        <v>0.1</v>
+        <v>-0.54</v>
       </c>
       <c r="H18" t="n">
-        <v>42297400</v>
+        <v>10128450</v>
       </c>
     </row>
     <row r="19">
@@ -1065,20 +1065,20 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>76.86</v>
+        <v>76.905</v>
       </c>
       <c r="F19" t="n">
-        <v>-0.27</v>
+        <v>0.045</v>
       </c>
       <c r="G19" t="n">
-        <v>-0.35</v>
+        <v>0.06</v>
       </c>
       <c r="H19" t="n">
-        <v>76938700</v>
+        <v>9681941</v>
       </c>
     </row>
     <row r="20">
@@ -1099,20 +1099,20 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>4202.2998</v>
+        <v>4165.7002</v>
       </c>
       <c r="F20" t="n">
-        <v>21.1997</v>
+        <v>-15.3999</v>
       </c>
       <c r="G20" t="n">
-        <v>0.51</v>
+        <v>-0.37</v>
       </c>
       <c r="H20" t="n">
-        <v>5386</v>
+        <v>93751</v>
       </c>
     </row>
     <row r="21">
@@ -1133,20 +1133,20 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>97.93000000000001</v>
+        <v>97.56</v>
       </c>
       <c r="F21" t="n">
-        <v>-3.48</v>
+        <v>-3.85</v>
       </c>
       <c r="G21" t="n">
-        <v>-3.43</v>
+        <v>-3.8</v>
       </c>
       <c r="H21" t="n">
-        <v>6387</v>
+        <v>151070</v>
       </c>
     </row>
     <row r="22">
@@ -1167,20 +1167,20 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="E22" t="n">
-        <v>108.49</v>
+        <v>108.02</v>
       </c>
       <c r="F22" t="n">
-        <v>-1.37</v>
+        <v>-1.84</v>
       </c>
       <c r="G22" t="n">
-        <v>-1.25</v>
+        <v>-1.67</v>
       </c>
       <c r="H22" t="n">
-        <v>588</v>
+        <v>19029</v>
       </c>
     </row>
     <row r="23">
@@ -1201,20 +1201,20 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="E23" t="n">
-        <v>6.5725</v>
+        <v>6.5475</v>
       </c>
       <c r="F23" t="n">
-        <v>0.0415</v>
+        <v>0.0165</v>
       </c>
       <c r="G23" t="n">
-        <v>0.64</v>
+        <v>0.25</v>
       </c>
       <c r="H23" t="n">
-        <v>359</v>
+        <v>24396</v>
       </c>
     </row>
     <row r="24">
@@ -1235,20 +1235,20 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="E24" t="n">
-        <v>62.85</v>
+        <v>63.67</v>
       </c>
       <c r="F24" t="n">
-        <v>-1.11</v>
+        <v>0.82</v>
       </c>
       <c r="G24" t="n">
-        <v>-1.74</v>
+        <v>1.3</v>
       </c>
       <c r="H24" t="n">
-        <v>31508800</v>
+        <v>8356721</v>
       </c>
     </row>
     <row r="25">
@@ -1269,17 +1269,17 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="E25" t="n">
-        <v>19.99</v>
+        <v>17.73</v>
       </c>
       <c r="F25" t="n">
-        <v>3.53</v>
+        <v>-2.26</v>
       </c>
       <c r="G25" t="n">
-        <v>21.45</v>
+        <v>-11.31</v>
       </c>
       <c r="H25" t="n">
         <v>0</v>
@@ -1303,20 +1303,20 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="E26" t="n">
-        <v>81973.0938</v>
+        <v>82372.99219999999</v>
       </c>
       <c r="F26" t="n">
-        <v>590.9453</v>
+        <v>355.3906</v>
       </c>
       <c r="G26" t="n">
-        <v>0.73</v>
+        <v>0.43</v>
       </c>
       <c r="H26" t="n">
-        <v>18388713472</v>
+        <v>26750234624</v>
       </c>
     </row>
     <row r="27">
@@ -1337,20 +1337,20 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="E27" t="n">
-        <v>1210</v>
+        <v>1195</v>
       </c>
       <c r="F27" t="n">
-        <v>-210</v>
+        <v>-15</v>
       </c>
       <c r="G27" t="n">
-        <v>-14.79</v>
+        <v>-1.24</v>
       </c>
       <c r="H27" t="n">
-        <v>206590200</v>
+        <v>335441300</v>
       </c>
     </row>
     <row r="28">
@@ -1371,20 +1371,20 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="E28" t="n">
-        <v>1205</v>
+        <v>1125</v>
       </c>
       <c r="F28" t="n">
-        <v>-210</v>
+        <v>-80</v>
       </c>
       <c r="G28" t="n">
-        <v>-14.84</v>
+        <v>-6.64</v>
       </c>
       <c r="H28" t="n">
-        <v>89153400</v>
+        <v>34059600</v>
       </c>
     </row>
     <row r="29">
@@ -1405,20 +1405,20 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="E29" t="n">
-        <v>540</v>
+        <v>505</v>
       </c>
       <c r="F29" t="n">
-        <v>-90</v>
+        <v>-35</v>
       </c>
       <c r="G29" t="n">
-        <v>-14.29</v>
+        <v>-6.48</v>
       </c>
       <c r="H29" t="n">
-        <v>86042800</v>
+        <v>184792800</v>
       </c>
     </row>
     <row r="30">
@@ -1439,20 +1439,20 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="E30" t="n">
-        <v>1855</v>
+        <v>1835</v>
       </c>
       <c r="F30" t="n">
-        <v>-325</v>
+        <v>-20</v>
       </c>
       <c r="G30" t="n">
-        <v>-14.91</v>
+        <v>-1.08</v>
       </c>
       <c r="H30" t="n">
-        <v>41687500</v>
+        <v>49854400</v>
       </c>
     </row>
     <row r="31">
@@ -1473,20 +1473,20 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="E31" t="n">
-        <v>3340</v>
+        <v>3110</v>
       </c>
       <c r="F31" t="n">
-        <v>-580</v>
+        <v>-230</v>
       </c>
       <c r="G31" t="n">
-        <v>-14.8</v>
+        <v>-6.89</v>
       </c>
       <c r="H31" t="n">
-        <v>25530400</v>
+        <v>3615400</v>
       </c>
     </row>
     <row r="32">
@@ -1507,20 +1507,20 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="E32" t="n">
-        <v>404</v>
+        <v>376</v>
       </c>
       <c r="F32" t="n">
-        <v>-70</v>
+        <v>-28</v>
       </c>
       <c r="G32" t="n">
-        <v>-14.77</v>
+        <v>-6.93</v>
       </c>
       <c r="H32" t="n">
-        <v>71038700</v>
+        <v>157927200</v>
       </c>
     </row>
     <row r="33">
@@ -1541,20 +1541,20 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="E33" t="n">
-        <v>490</v>
+        <v>456</v>
       </c>
       <c r="F33" t="n">
-        <v>-85</v>
+        <v>-34</v>
       </c>
       <c r="G33" t="n">
-        <v>-14.78</v>
+        <v>-6.94</v>
       </c>
       <c r="H33" t="n">
-        <v>25592500</v>
+        <v>17562200</v>
       </c>
     </row>
     <row r="34">
@@ -1575,20 +1575,20 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="E34" t="n">
-        <v>2960</v>
+        <v>2760</v>
       </c>
       <c r="F34" t="n">
-        <v>-520</v>
+        <v>-200</v>
       </c>
       <c r="G34" t="n">
-        <v>-14.94</v>
+        <v>-6.76</v>
       </c>
       <c r="H34" t="n">
-        <v>8168700</v>
+        <v>2824700</v>
       </c>
     </row>
     <row r="35">
@@ -1609,20 +1609,20 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="E35" t="n">
-        <v>400</v>
+        <v>372</v>
       </c>
       <c r="F35" t="n">
-        <v>-70</v>
+        <v>-28</v>
       </c>
       <c r="G35" t="n">
-        <v>-14.89</v>
+        <v>-7</v>
       </c>
       <c r="H35" t="n">
-        <v>44001300</v>
+        <v>4155400</v>
       </c>
     </row>
     <row r="36">
@@ -1643,20 +1643,20 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="E36" t="n">
-        <v>157</v>
+        <v>147</v>
       </c>
       <c r="F36" t="n">
-        <v>-27</v>
+        <v>-10</v>
       </c>
       <c r="G36" t="n">
-        <v>-14.67</v>
+        <v>-6.37</v>
       </c>
       <c r="H36" t="n">
-        <v>107257500</v>
+        <v>10013700</v>
       </c>
     </row>
     <row r="37">
@@ -1677,20 +1677,20 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="E37" t="n">
-        <v>11975</v>
+        <v>11150</v>
       </c>
       <c r="F37" t="n">
-        <v>-2100</v>
+        <v>-825</v>
       </c>
       <c r="G37" t="n">
-        <v>-14.92</v>
+        <v>-6.89</v>
       </c>
       <c r="H37" t="n">
-        <v>1615300</v>
+        <v>215900</v>
       </c>
     </row>
   </sheetData>
@@ -1749,22 +1749,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>MSCI Soroti Masalah Bahasa-Transparansi Pasar Modal RI</t>
+          <t>IHSG Melorot ke Bawah 5.000, Danantara Mau Borong Saham BUMN</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Mon, 19 Oct 2026 06:30:52 +0700</t>
+          <t>Mon, 19 Oct 2026 22:13:04 +0700</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/05/18/ihsg-anjlok-ke-zona-merah-bursa-saham-melemah-tajam-1779098741437_169.jpeg?w=360&amp;amp;q=90" /&gt; Lembaga penyedia indeks saham global, MSCI, buka-bukaan soal aksesibilitas pasar modal Indonesia.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/03/11/rosan-roeslani-firda-cynthia-anggrainy-al-djokyadetikcom-1741681299971_169.jpeg?w=360&amp;amp;q=90" /&gt; CEO Danantara Rosan Roeslani menanggapi Indeks Harga Saham Gabungan (IHSG) yang turun hingga ke bawah level 5.000.</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/bursa-dan-valas/d-8713143/msci-soroti-masalah-bahasa-transparansi-pasar-modal-ri</t>
+          <t>https://finance.detik.com/bursa-dan-valas/d-8714705/ihsg-melorot-ke-bawah-5-000-danantara-mau-borong-saham-bumn</t>
         </is>
       </c>
     </row>
@@ -1776,22 +1776,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Persiapan Giant Sea Wall Pantura, Struktur Pemecah Ombak Disiapkan di Demak</t>
+          <t>Penyebab Listrik Batam Padam Diusut, Bos PLN Pastikan Bukan Sabotase</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Mon, 19 Oct 2026 06:00:47 +0700</t>
+          <t>Mon, 19 Oct 2026 21:54:44 +0700</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/18/persiapan-giant-sea-wall-pantura-struktur-pemecah-ombak-disiapkan-di-demak-1792305303554_169.jpeg?w=360&amp;amp;q=90" /&gt; Pekerja memasang Hex-Brick untuk pemecah ombak semipermeabel di pesisir Demak. Upaya ini menjadi bagian dari per</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2023/01/01/pembangkit-listrik-pln-batam-foto-dok-pln_169.jpeg?w=360&amp;amp;q=90" /&gt; PLN sedang menyelidiki lebih dalam penyebab listrik padam di Batam, Kepulauan Riau, beberapa hari lalu.</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/foto-bisnis/d-8712466/persiapan-giant-sea-wall-pantura-struktur-pemecah-ombak-disiapkan-di-demak</t>
+          <t>https://finance.detik.com/energi/d-8714688/penyebab-listrik-batam-padam-diusut-bos-pln-pastikan-bukan-sabotase</t>
         </is>
       </c>
     </row>
@@ -1803,22 +1803,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Perusahaan Haji Isam Gadai Saham, Duitnya buat Apa?</t>
+          <t>Dua Tahun Prabowo: Investasi Rp 3.923 Triliun, 5,4 Juta Tenaga Kerja Terserap</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Mon, 19 Oct 2026 05:55:54 +0700</t>
+          <t>Mon, 19 Oct 2026 21:40:16 +0700</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/16/ihsg-ambruk-1157-ditutup-di-level-5185-1792144638939_169.jpeg?w=360&amp;amp;q=90" /&gt; PT Bank Mandiri (Persero) Tbk (BMRI) buka-bukaan soal alokasi kredit dari aksi gadai saham dua perusahaan milik Andi Syamsuddin Arsyad alias Haji Is</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/08/06/presiden-prabowo-subianto-menggelar-sidang-kabinet-rabu-682025-1754475097038_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Investasi dan Hilirisasi/Kepala BKPM Rosan Roeslani mengatakan total investasi dalam 2 tahun capai Rp 3.923 triliun.</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/bursa-dan-valas/d-8712880/perusahaan-haji-isam-gadai-saham-duitnya-buat-apa</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8714675/dua-tahun-prabowo-investasi-rp-3-923-triliun-5-4-juta-tenaga-kerja-terserap</t>
         </is>
       </c>
     </row>
@@ -1830,22 +1830,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Menyesap Harum Kopi Indonesia di Tokyo</t>
+          <t>5 Besar Investor Asing di Indonesia, Singapura Masih Rajanya</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Mon, 19 Oct 2026 00:00:00 +0700</t>
+          <t>Mon, 19 Oct 2026 21:25:48 +0700</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/18/adv-bank-indonesi-1792334493519.jpeg?w=360&amp;amp;q=90" /&gt; Tepat pukul 10.00 tanggal 14 Oktober 2026, pameran Specialty Coffee Association of Japan (SCAJ) World Specialty Coffee Conference and Exhibition 2026</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2023/03/28/ilustrasi-pertumbuhan-ekonomi_169.jpeg?w=360&amp;amp;q=90" /&gt; Realisasi investasi di Indonesia sepanjang Januari-September 2026 mencapai Rp 1.539,2 triliun atau 75,4% dari target. Singapura masih investor asing terbesar</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/advertorial-news-block/d-8713009/menyesap-harum-kopi-indonesia-di-tokyo</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8714667/5-besar-investor-asing-di-indonesia-singapura-masih-rajanya</t>
         </is>
       </c>
     </row>
@@ -1857,22 +1857,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Perajin Batik Rifaiyah Batang Didorong Naik Kelas Lewat Kenduri Batik 2026</t>
+          <t>Biang Kerok Masalah BBM di Bali: Kapal dari Jawa Terlambat Masuk</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Sun, 18 Oct 2026 22:30:51 +0700</t>
+          <t>Mon, 19 Oct 2026 21:13:33 +0700</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/18/perajin-batik-rifaiyah-batang-didorong-naik-kelas-lewat-kenduri-batik-2026-1792304249394_169.jpeg?w=360&amp;amp;q=90" /&gt; Kenduri Batik Batang 2026 menjadi wadah perajin Batik Rifaiyah mengembangkan usaha. Kegiatan ini mendorong inova</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/19/kondisi-antrean-pengisian-bbm-bersubsidi-yang-sudah-normal-kembali-di-spbu-besang-semarapura-tengah-klungkung-bali-senin-19102-1792374026464_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Energi dan Sumber Daya Mineral (ESDM) Bahlil Lahadal</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/foto-bisnis/d-8712436/perajin-batik-rifaiyah-batang-didorong-naik-kelas-lewat-kenduri-batik-2026</t>
+          <t>https://finance.detik.com/energi/d-8714655/biang-kerok-masalah-bbm-di-bali-kapal-dari-jawa-terlambat-masuk</t>
         </is>
       </c>
     </row>
@@ -1884,22 +1884,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>3 Cara Maksimalkan Penggunaan QRIS untuk Bantu Bisnis Berkembang</t>
+          <t>Inovasi Pertanian Ramah Lingkungan di Pasar Minggu</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Sun, 18 Oct 2026 22:00:51 +0700</t>
+          <t>Mon, 19 Oct 2026 21:12:34 +0700</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/18/ilustrasi-qr-1792334198806.jpeg?w=360&amp;amp;q=90" /&gt; Optimalkan bisnis Anda dengan QRIS! Pelajari cara mempermudah transaksi, manfaatkan MDR 0%, dan daftar DANA Bisnis untuk keuntungan maksimal.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/19/pemanfaatan-limbah-galon-untuk-tanam-padi-di-jakarta-1792418941312_169.jpeg?w=360&amp;amp;q=90" /&gt; Posyantek Kreya Loka memanfaatkan 1.500 galon plastik bekas untuk menanam padi di RPTRA Belimbing, Jakarta Selatan, sebagai inovasi ke</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8713018/3-cara-maksimalkan-penggunaan-qris-untuk-bantu-bisnis-berkembang</t>
+          <t>https://finance.detik.com/foto-bisnis/d-8714649/inovasi-pertanian-ramah-lingkungan-di-pasar-minggu</t>
         </is>
       </c>
     </row>
@@ -1911,22 +1911,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Kilang Plaju Produksi Avtur 295 Ribu Barel hingga September</t>
+          <t>Menjaga Asa Ekonomi Lewat Martabak Mini</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Sun, 18 Oct 2026 22:00:07 +0700</t>
+          <t>Mon, 19 Oct 2026 21:03:22 +0700</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/10/25/perwira-pertamina-perempuan-di-kilang-plaju-saat-melakukan-tugasnya-memonitor-mesin-produksi-polypropylene-1761406552564_169.jpeg?w=360&amp;amp;q=90" /&gt; Kilang Plaju mencatat produksi bahan bakar pesawat atau avtur sebesar 295.263 ba</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/19/kisah-sri-bertahan-jualan-martabak-mini-sejak-pandemi-1792418064215_169.jpeg?w=360&amp;amp;q=90" /&gt; Sejak pandemi COVID-19, Sri Rahayu (52) tekun berjualan martabak mini di Bekasi. Beromzet sekitar Rp 300 ribu sehari, usaha ini menja</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8712759/kilang-plaju-produksi-avtur-295-ribu-barel-hingga-september</t>
+          <t>https://finance.detik.com/foto-bisnis/d-8714627/menjaga-asa-ekonomi-lewat-martabak-mini</t>
         </is>
       </c>
     </row>
@@ -1938,22 +1938,22 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Mau Pakai QRIS untuk Jualan? Cek Cara Ini biar Tak Kena Potongan Biaya</t>
+          <t>Harga Minyak Tembus US$ 100/ Barel, Bahlil: Kondisi Global Makin Tak Menentu</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Sun, 18 Oct 2026 21:48:34 +0700</t>
+          <t>Mon, 19 Oct 2026 20:50:01 +0700</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/21/ilustrasi-qris-1789973868497.png?w=360&amp;amp;q=90" /&gt; Pembayaran QRIS semakin mudah, dengan program MDR 0% untuk UMKM. Nikmati transaksi tanpa potongan biaya dan tingkatkan efisiensi bisnis Anda.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/08/04/bahlil-lahadalia-1785840108228_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri ESDM Bahlil Lahadalia mengungkapkan harga minyak mentah Indonesia melonjak tajam seiring kenaikan harga minyak dunia.</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8713015/mau-pakai-qris-untuk-jualan-cek-cara-ini-biar-tak-kena-potongan-biaya</t>
+          <t>https://finance.detik.com/energi/d-8714613/harga-minyak-tembus-us-100-barel-bahlil-kondisi-global-makin-tak-menentu</t>
         </is>
       </c>
     </row>
@@ -1965,22 +1965,22 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Tanjung Perak Jadi Lokasi Pertama Uji Coba Penertiban Kendaraan ODOL</t>
+          <t>Bos OJK Buka Suara Usai Lapor Kondisi Bursa Saham ke Prabowo</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Sun, 18 Oct 2026 21:00:38 +0700</t>
+          <t>Mon, 19 Oct 2026 20:32:43 +0700</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/06/20/ratusan-truk-blokade-jalur-pantura-alas-roban-batang-1750397214314_169.jpeg?w=360&amp;amp;q=90" /&gt; Pelabuhan Tanjung Perak, Surabaya akan menjadi lokasi pertama dalam penertiban kendaraan Over Dimension Over Loading (ODOL) yang diang</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/08/03/frederica-widyasari-dewi-1785765447950_169.jpeg?w=360&amp;amp;q=90" /&gt; Pengumuman lembaga pemeringkatan MSCI soal potensi penurunan bursa saham Indonesia ke Standalone Market menimbulkan sentimen negatif.</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/infrastruktur/d-8712817/tanjung-perak-jadi-lokasi-pertama-uji-coba-penertiban-kendaraan-odol</t>
+          <t>https://finance.detik.com/bursa-dan-valas/d-8714572/bos-ojk-buka-suara-usai-lapor-kondisi-bursa-saham-ke-prabowo</t>
         </is>
       </c>
     </row>
@@ -1992,22 +1992,22 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>BI Dorong Transaksi Pakai Mata Uang Lokal di Pertemuan IMF-Bank Dunia</t>
+          <t>Investasi Tembus Rp 1.539,2 Triliun, Serap 2,19 Juta Tenaga Kerja</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Sun, 18 Oct 2026 20:00:30 +0700</t>
+          <t>Mon, 19 Oct 2026 20:22:05 +0700</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/23/bi-pertahankan-suku-bunga-575-persen-fokus-jaga-stabilitas-rupiah-1790154587213_169.jpeg?w=360&amp;amp;q=90" /&gt; Bank Indonesia mendorong perluasan penggunaan mata mata uang lokal (Local Currency Transaction/LCT) dalam perdagangan dan</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/11/20/menteri-investasi-dan-hilirisasikepala-bkpm-rosan-roeslani-1763634019135_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Investasi dan Hilirisasi/Kepala BKPM Rosan Roeslani mencatat realisasi investasi sepanjang periode Januari-September men</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/moneter/d-8712864/bi-dorong-transaksi-pakai-mata-uang-lokal-di-pertemuan-imf-bank-dunia</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8714565/investasi-tembus-rp-1-539-2-triliun-serap-2-19-juta-tenaga-kerja</t>
         </is>
       </c>
     </row>
@@ -2019,22 +2019,22 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Transaksi Trade Expo Indonesia Tembus Rp 414 Triliun</t>
+          <t>Ekspor dari Berbagai Sektor Bakal Digenjot</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Sun, 18 Oct 2026 19:31:01 +0700</t>
+          <t>Mon, 19 Oct 2026 20:09:58 +0700</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/18/menteri-perdagangan-budi-santoso-1792326567826_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Perdagangan Budi Santoso menyampaikan nilai transaksi Trade Expo Indonesia (TEI) ke-41 mencapai US$ 22,94 miliar atau setara sekitar Rp 414 triliu</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/06/09/tanjung-priok-tetap-sibuk-di-tengah-tekanan-dolar-harapan-ekspor-menguat-1780979464280_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Koordinator Perekonomian Airlangga Hartarto mengatakan pemerintah menggenjot kinerja ekspor nasional</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8712868/transaksi-trade-expo-indonesia-tembus-rp-414-triliun</t>
+          <t>https://finance.detik.com/ekonomi-bisnis/d-8714554/ekspor-dari-berbagai-sektor-bakal-digenjot</t>
         </is>
       </c>
     </row>
@@ -2046,22 +2046,22 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>34 Lembaga Keuangan Berminat Biayai Proyek Sampah Jadi Listrik</t>
+          <t>Kedai Inspirasi Bekasi, Ruang Difabel Merajut Kemandirian Ekonomi</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Sun, 18 Oct 2026 19:00:27 +0700</t>
+          <t>Mon, 19 Oct 2026 19:51:09 +0700</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/07/01/wisma-danantara-indonesia-1751345496063_169.jpeg?w=360&amp;amp;q=90" /&gt; Danantara menetapkan 34 institusi keuangan sebagai anggota lenders panel untuk program Pengolahan Sampah menjadi Energi Listrik (PSEL).</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/19/kedai-inspirasi-bekasi-ruang-difabel-merajut-kemandirian-ekonomi-1792395314234.jpeg?w=360&amp;amp;q=90" /&gt; Kedai Inspirasi menjadi ruang bagi penyandang disabilitas untuk mengembangkan keterampilan kerja dan membangun kemandirian eko</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8712594/34-lembaga-keuangan-berminat-biayai-proyek-sampah-jadi-listrik</t>
+          <t>https://finance.detik.com/foto-bisnis/d-8713877/kedai-inspirasi-bekasi-ruang-difabel-merajut-kemandirian-ekonomi</t>
         </is>
       </c>
     </row>
@@ -2073,22 +2073,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>OJK &amp;amp; BEI Kumpulkan AB-Analis Usai IHSG Rontok Imbas Pengumuman MSCI</t>
+          <t>131 CEO Global Kumpul di Jakarta, Danantara Incar Kesepakatan Besar</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Sun, 18 Oct 2026 17:43:11 +0700</t>
+          <t>Mon, 19 Oct 2026 19:00:20 +0700</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/06/03/ihsg-anjlok-411-persen-ke-level-5941-1780494579470_169.jpeg?w=360&amp;amp;q=90" /&gt; Otoritas Jasa Keuangan (OJK) dan Bursa Efek Indonesia (BEI) mengumpulkan analis dan anggota bursa (AB) hari ini, Minggu (18/10/2026).</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/19/danantara-1792409910587_169.jpeg?w=360&amp;amp;q=90" /&gt; Danantara Indonesia akan menggelar DTIIF 2026 pada 26-28 Oktober di Jakarta.</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/bursa-dan-valas/d-8712753/ojk-bei-kumpulkan-ab-analis-usai-ihsg-rontok-imbas-pengumuman-msci</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8714447/131-ceo-global-kumpul-di-jakarta-danantara-incar-kesepakatan-besar</t>
         </is>
       </c>
     </row>
@@ -2100,22 +2100,22 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>IHSG Masih Diprediksi Rawan Longsor Usai Pengumuman MSCI</t>
+          <t>IHSG Seharian Melemah, Ditutup ke Level 4.900</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Sun, 18 Oct 2026 17:00:46 +0700</t>
+          <t>Mon, 19 Oct 2026 18:34:09 +0700</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/01/28/bei-terapkan-trading-halt-imbas-ihsg-anjlok-1769587530913_169.jpeg?w=360&amp;amp;q=90" /&gt; Indeks Harga Saham Gabungan (IHSG) berpotensi melanjutkan pelemahan di perdagangan Senin (19/10/2026).</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/19/ihsg-dibuka-anjlok-431-bei-berlakukan-arb-7-1792382663303_169.jpeg?w=360&amp;amp;q=90" /&gt; IHSG ditutup melemah di zona merah, turun 188,49 poin ke 5.936,14. Ini merupakan level terendah dalam 10 tahun terakhir.</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/bursa-dan-valas/d-8712545/ihsg-masih-diprediksi-rawan-longsor-usai-pengumuman-msci</t>
+          <t>https://finance.detik.com/bursa-dan-valas/d-8714438/ihsg-seharian-melemah-ditutup-ke-level-4-900</t>
         </is>
       </c>
     </row>
@@ -2127,22 +2127,22 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Harga Emas Antam Anjlok dalam Sepekan, Begini Pergerakannya</t>
+          <t>Pasar Nikel Global Diproyeksi Tumbuh 21,39% hingga 2031</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Sun, 18 Oct 2026 16:00:10 +0700</t>
+          <t>Mon, 19 Oct 2026 18:25:08 +0700</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/10/22/harga-emas-terjun-bebas-pasar-cikini-langsung-diserbu-pembeli-1761123863171_169.jpeg?w=360&amp;amp;q=90" /&gt; Harga emas Antam 24 karat sepanjang perdagangan 12-17 Oktober 2026 turun sebesar Rp 22.000 per gram.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/19/mind-id-1792409058599_169.jpeg?w=360&amp;amp;q=90" /&gt; Prospek pasar nikel global meningkat, membuka peluang bagi Indonesia untuk memperdalam hilirisasi industri. Fokus pada produk akhir untuk nilai tambah maksimal.</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8712537/harga-emas-antam-anjlok-dalam-sepekan-begini-pergerakannya</t>
+          <t>https://finance.detik.com/energi/d-8714423/pasar-nikel-global-diproyeksi-tumbuh-21-39-hingga-2031</t>
         </is>
       </c>
     </row>
@@ -2154,22 +2154,22 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Bertemu Prabowo, Sekjen PBB Apresiasi Peran Indonesia untuk Palestina</t>
+          <t>Menag Soroti Kebakaran Hutan, Singgung Dosa Merusak Alam</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Mon, 19 Oct 2026 06:32:47 +0700</t>
+          <t>Mon, 19 Oct 2026 22:02:46 +0700</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Sekjen PBB António Guterres berpamitan kepada Presiden Prabowo menjelang akhir masa jabatannya pada Desember 2026 dan mengapresiasi dukungan Indonesia bagi Palestina serta misi perdamaian PBB.</t>
+          <t>Nasaruddin mengatakan, pendekatan ekoteologi dapat menjadi salah satu upaya untuk mendorong kepedulian masyarakat terhadap kelestarian lingkungan.</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8316023/bertemu-prabowo-sekjen-pbb-apresiasi-peran-indonesia-untuk-palestina</t>
+          <t>https://www.liputan6.com/news/read/8316740/menag-soroti-kebakaran-hutan-singgung-dosa-merusak-alam</t>
         </is>
       </c>
     </row>
@@ -2181,22 +2181,22 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>DPR Buka-bukaan soal Polemik Syarat Pendidikan Capres-Cawapres di PKPU</t>
+          <t>PKS Ingatkan Kader Hati-Hati Bicara di Medsos</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Mon, 19 Oct 2026 06:00:39 +0700</t>
+          <t>Mon, 19 Oct 2026 21:31:18 +0700</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Ahmad Doli Kurnia menyatakan Pasal 18 ayat (3) PKPU Nomor 19 Tahun 2023 tidak tercantum dalam draf yang dibahas Komisi II DPR saat konsultasi penyusunan aturan tersebut.</t>
+          <t>PKS berharap pejabat publik memiliki kesadaran bahwa cara menyampaikan pesan harus disesuaikan dengan perkembangan teknologi dan karakter ruang digital.</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8316016/dpr-buka-bukaan-soal-polemik-syarat-pendidikan-capres-cawapres-di-pkpu</t>
+          <t>https://www.liputan6.com/news/read/8316737/pks-ingatkan-kader-hati-hati-bicara-di-medsos</t>
         </is>
       </c>
     </row>
@@ -2208,22 +2208,22 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>7 Perjalanan KRL Bogor Dibatalkan Hari Ini, Cek Jadwalnya</t>
+          <t>Mantan KSAD Subagyo HS Meninggal Dunia</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Mon, 19 Oct 2026 05:35:40 +0700</t>
+          <t>Mon, 19 Oct 2026 21:06:13 +0700</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>KAI Commuter membatalkan tujuh perjalanan lintas Bogor pada Senin (19/10/2026) karena dua rangkaian kereta masih diperbaiki. Pengguna diminta mengecek jadwal dan alternatif perjalanan.</t>
+          <t>Subagyo HS meninggal dunia di RS Panti Rapih, Yogyakarta, Senin (19/10/2026) sore.</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8316013/7-perjalanan-krl-bogor-dibatalkan-hari-ini-cek-jadwalnya</t>
+          <t>https://www.liputan6.com/news/read/8316722/mantan-ksad-subagyo-hs-meninggal-dunia</t>
         </is>
       </c>
     </row>
@@ -2235,22 +2235,22 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Prakiraan Cuaca Jakarta 19 Oktober: Jaksel dan Jaktim Berpotensi Hujan</t>
+          <t>Prabowo Soroti Kinerja ASN-Polri</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Mon, 19 Oct 2026 05:20:05 +0700</t>
+          <t>Mon, 19 Oct 2026 20:52:56 +0700</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>BMKG memprakirakan hujan ringan berpotensi mengguyur Jakarta Selatan dan Jakarta Timur pada sore hingga malam hari, sementara wilayah lainnya cenderung berawan hingga cerah berawan.</t>
+          <t>Prabowo menyampaikan terkait pentingnya profesionalisme, integritas, dan kompetensi aparatur negara dalam penyelenggaraan pemerintahan.</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8316012/prakiraan-cuaca-jakarta-19-oktober-jaksel-dan-jaktim-berpotensi-hujan</t>
+          <t>https://www.liputan6.com/news/read/8316715/prabowo-soroti-kinerja-asn-polri</t>
         </is>
       </c>
     </row>
@@ -2262,22 +2262,22 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Kronologi Bharada Valdo Tewas Ditembak Rekan Sesama Polisi</t>
+          <t>Ini Hasil Tes Urine Sopir Pajero Tabrak Remaja hingga Tewas di Jaksel</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Mon, 19 Oct 2026 05:08:04 +0700</t>
+          <t>Mon, 19 Oct 2026 20:14:42 +0700</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Bharada Valdo tewas dalam insiden penembakan di Markas Polairud Pondok Cabe. Pengacara keluarga menduga pembunuhan berencana dan meminta penyidik mendalami kemungkinan keterlibatan pihak lain.</t>
+          <t>Hasil tes urine dilakukan kepolisian menunjukkan sopir negatif dari penyalahgunaan narkoba.</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8316006/kronologi-bharada-valdo-tewas-ditembak-rekan-sesama-polisi</t>
+          <t>https://www.liputan6.com/news/read/8316696/ini-hasil-tes-urine-sopir-pajero-tabrak-remaja-hingga-tewas-di-jaksel</t>
         </is>
       </c>
     </row>
@@ -2289,22 +2289,22 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Kronologi Tawuran di Manggarai hingga Kios Dibakar, 6 Orang Ditangkap</t>
+          <t>Nadiem Makarim Ajukan Kasasi, Ini Permintaannya ke Hakim</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Mon, 19 Oct 2026 00:27:21 +0700</t>
+          <t>Mon, 19 Oct 2026 20:13:26 +0700</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Keenam orang itu masih menjalani pemeriksaan untuk mendalami peran masing-masing.</t>
+          <t>Nadiem beberkan lima alasan Nadiem ajukan kasasi.</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8315986/kronologi-tawuran-di-manggarai-hingga-kios-dibakar-6-orang-ditangkap</t>
+          <t>https://www.liputan6.com/news/read/8316695/nadiem-makarim-ajukan-kasasi-ini-permintaannya-ke-hakim</t>
         </is>
       </c>
     </row>
@@ -2316,22 +2316,22 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Survei PPI, Erick Thohir Masuk 3 Besar Menteri Berkinerja Terbaik</t>
+          <t>Kronologi Bharatu Valdo Ditembak Rekan Sesama Polisi Versi Pengacara</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Sun, 18 Oct 2026 22:32:43 +0700</t>
+          <t>Mon, 19 Oct 2026 19:50:36 +0700</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Erick Thohir dinilai berkinerja baik terutama karena performa Timnas Indonesia yang dianggap semakin meningkat.</t>
+          <t>Penyidik menyampaikan bahwa tersangka diduga melampiaskan kemarahan karena teman-teman seangkatan korban disebut kerap melakukan perundungan.</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8315941/survei-ppi-erick-thohir-masuk-3-besar-menteri-berkinerja-terbaik</t>
+          <t>https://www.liputan6.com/news/read/8316686/kronologi-bharatu-valdo-ditembak-rekan-sesama-polisi-versi-pengacara</t>
         </is>
       </c>
     </row>
@@ -2343,22 +2343,22 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Satgas Damai Cartenz Bongkar Markas KKB, Temukan 559 Selongsong Peluru</t>
+          <t>Dudung soal Karhutla Belum jadi Bencana Nasional: Negara Masih Sanggup</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Sun, 18 Oct 2026 21:48:21 +0700</t>
+          <t>Mon, 19 Oct 2026 19:23:41 +0700</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Di dalam honai ditemukan 559 selongsong peluru kaliber 5,56 mm dan sejumlah barang bukti lainnya.</t>
+          <t>Dudung juga menjawab tawaran Malaysia untuk mengirimkan tiga helikopter.</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8315923/satgas-damai-cartenz-bongkar-markas-kkb-temukan-559-selongsong-peluru</t>
+          <t>https://www.liputan6.com/news/read/8316670/dudung-soal-karhutla-belum-jadi-bencana-nasional-negara-masih-sanggup</t>
         </is>
       </c>
     </row>
@@ -2370,22 +2370,22 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Polisi Tembak Polisi di Markas Polairud Tangsel</t>
+          <t>Dudung Ungkap Tawaran Malaysia dan Singapura Tangani Kebakaran Hutan</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Sun, 18 Oct 2026 21:01:25 +0700</t>
+          <t>Mon, 19 Oct 2026 19:16:35 +0700</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Tersangka berinisial AR, yang juga merupakan anggota Polri, telah diamankan.</t>
+          <t>Pemerintah Indonesia telah merespons usulan bantuan tersebut. Adapun teknis pelaksanaan bantuan masih perlu dikoordinasikan lebih lanjut.</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8315898/polisi-tembak-polisi-di-markas-polairud-tangsel</t>
+          <t>https://www.liputan6.com/news/read/8316667/dudung-ungkap-tawaran-malaysia-dan-singapura-tangani-kebakaran-hutan</t>
         </is>
       </c>
     </row>
@@ -2397,22 +2397,22 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Sekjen PBB Temui Prabowo di Hambalang, Ini yang Dibahas</t>
+          <t>Survei Terbaru Poltracking: 55,3% Responden Puas Kinerja Pemerintahan Prabowo-Gibran</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Sun, 18 Oct 2026 19:22:20 +0700</t>
+          <t>Mon, 19 Oct 2026 19:05:36 +0700</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Prabowo menyambut langsung kedatangan Guterres saat turun dari kendaraan. Guterres dan rombongan terlihat kompak mengenakan batik.</t>
+          <t>Survei Poltracking berlangsung pada 30 September hingga 7 Oktober 2026.</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8315845/sekjen-pbb-temui-prabowo-di-hambalang-ini-yang-dibahas</t>
+          <t>https://www.liputan6.com/news/read/8316660/survei-terbaru-poltracking-553-responden-puas-kinerja-pemerintahan-prabowo-gibran</t>
         </is>
       </c>
     </row>
@@ -2424,22 +2424,22 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Wamendagri Bima Arya Dorong Humas Pemerintah Lebih Dekat dengan Rakyat</t>
+          <t>Polisi Tembak Polisi, Pengacara Bharatu Valdo Pertanyakan Asal Senjata</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Sun, 18 Oct 2026 18:47:00 +0700</t>
+          <t>Mon, 19 Oct 2026 19:05:13 +0700</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Bima menjelaskan bahwa komunikasi publik perlu didasarkan pada pemahaman terhadap kebutuhan dan aspirasi masyarakat.</t>
+          <t>Kubu Bharatu Valdo mempertanyakan pengawasan senjata diperoleh pelaku penembakan di markas polairud, Pondok Cabe, Pamulang, Tangerang Selatan.</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8315833/wamendagri-bima-arya-dorong-humas-pemerintah-lebih-dekat-dengan-rakyat</t>
+          <t>https://www.liputan6.com/news/read/8316659/polisi-tembak-polisi-pengacara-bharatu-valdo-pertanyakan-asal-senjata</t>
         </is>
       </c>
     </row>
@@ -2451,22 +2451,22 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Kronologi Pelari ITB Ultra Marathon Meninggal Saat Melintas di Cianjur</t>
+          <t>Survei Poltracking: Gerindra 22,9 Persen, PDIP 13,4 Persen</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Sun, 18 Oct 2026 18:43:59 +0700</t>
+          <t>Mon, 19 Oct 2026 19:02:02 +0700</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Pihak kampus dan panitia menyampaikan belasungkawa.</t>
+          <t>Sejumlah partai berpotensi kembali lolos ke parlemen apabila ambang batas parlemen atau parliamentary threshold tetap ditetapkan sebesar 4%.</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8315832/kronologi-pelari-itb-ultra-marathon-meninggal-saat-melintas-di-cianjur</t>
+          <t>https://www.liputan6.com/news/read/8316649/survei-poltracking-gerindra-229-persen-pdip-134-persen</t>
         </is>
       </c>
     </row>
@@ -2478,22 +2478,22 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Kemensos Gelar Anugerah Jurnalistik Sekolah Rakyat 2026, Gus Ipul Soroti Peran Penting Media</t>
+          <t>Dua Strategi Pemprov Jakarta Antisipasi Asap Kebakaran Hutan</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Sun, 18 Oct 2026 18:08:15 +0700</t>
+          <t>Mon, 19 Oct 2026 18:36:15 +0700</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>BRI Peduli melibatkan 500 relawan dan menyediakan RVM untuk mendukung pengelolaan sampah selama MotoGP Mandalika 2026.</t>
+          <t>Strategi ini dilakukan Pemprov DKI Jakarta, mengantisipasi penyebaran asap kebakaran hutan dan lahan dari Sumatera dan Kalimantan sejak Jumat (16/10/2026).</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8315820/kemensos-gelar-anugerah-jurnalistik-sekolah-rakyat-2026-gus-ipul-soroti-peran-penting-media</t>
+          <t>https://www.liputan6.com/news/read/8316647/dua-strategi-pemprov-jakarta-antisipasi-asap-kebakaran-hutan</t>
         </is>
       </c>
     </row>
@@ -2505,22 +2505,22 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Seskab Teddy Masuk Dua Besar Menteri Terbaik Versi Survei PPI</t>
+          <t>Dari Apartemen di India, Rocky si Orangutan Akhirnya Pulang ke Indonesia</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Sun, 18 Oct 2026 22:01:03 +0700</t>
+          <t>Mon, 19 Oct 2026 18:17:40 +0700</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Di bawah mereka, Menteri Sosial Saifullah Yusuf memperoleh 4,5 persen, Menteri Koordinator Bidang Hilirisasi dan Investasi Bahlil Lahadalia 3,2 persen.</t>
+          <t>Rocky korban kejahatan perdagangan ilegal satwa liar lintas negara saat masih berusia 18-20 bulan.</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8315807/seskab-teddy-masuk-dua-besar-menteri-terbaik-versi-survei-ppi</t>
+          <t>https://www.liputan6.com/news/read/8316632/dari-apartemen-di-india-rocky-si-orangutan-akhirnya-pulang-ke-indonesia</t>
         </is>
       </c>
     </row>
@@ -2532,22 +2532,22 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Mantan Kadivhubinter Polri Napoleon Bonaparte Meninggal Dunia</t>
+          <t>Dudung Ungkap Arahan Prabowo untuk Perkuat Penanganan Karhutla</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Sun, 18 Oct 2026 15:29:43 +0700</t>
+          <t>Mon, 19 Oct 2026 18:01:41 +0700</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Napoleon Bonaparte dikabarkan meninggal akibat sakit.</t>
+          <t>Prabowo memerintahkan pengerahan pesawat Hercules dan personel untuk memperkuat penanganan karhutla.</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8315754/mantan-kadivhubinter-polri-napoleon-bonaparte-meninggal-dunia</t>
+          <t>https://www.liputan6.com/news/read/8316615/dudung-ungkap-arahan-prabowo-untuk-perkuat-penanganan-karhutla</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data pasar & berita - 2026-10-20 00:45 UTC
</commit_message>
<xml_diff>
--- a/data/market_news_latest.xlsx
+++ b/data/market_news_latest.xlsx
@@ -487,20 +487,20 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>4996.6089</v>
+        <v>5185.105</v>
       </c>
       <c r="F2" t="n">
-        <v>-188.4961</v>
+        <v>-678.6748</v>
       </c>
       <c r="G2" t="n">
-        <v>-3.64</v>
+        <v>-11.57</v>
       </c>
       <c r="H2" t="n">
-        <v>0</v>
+        <v>650917300</v>
       </c>
     </row>
     <row r="3">
@@ -525,16 +525,16 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>7723.46</v>
+        <v>7690.73</v>
       </c>
       <c r="F3" t="n">
-        <v>64.02</v>
+        <v>31.29</v>
       </c>
       <c r="G3" t="n">
-        <v>0.84</v>
+        <v>0.41</v>
       </c>
       <c r="H3" t="n">
-        <v>742614434</v>
+        <v>2634321000</v>
       </c>
     </row>
     <row r="4">
@@ -559,16 +559,16 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>52095.4219</v>
+        <v>51966.0312</v>
       </c>
       <c r="F4" t="n">
-        <v>93.0117</v>
+        <v>-36.3789</v>
       </c>
       <c r="G4" t="n">
-        <v>0.18</v>
+        <v>-0.07000000000000001</v>
       </c>
       <c r="H4" t="n">
-        <v>130641455</v>
+        <v>394068742</v>
       </c>
     </row>
     <row r="5">
@@ -593,16 +593,16 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>26576.4297</v>
+        <v>26430.8867</v>
       </c>
       <c r="F5" t="n">
-        <v>436.4004</v>
+        <v>290.8574</v>
       </c>
       <c r="G5" t="n">
-        <v>1.67</v>
+        <v>1.11</v>
       </c>
       <c r="H5" t="n">
-        <v>2719384000</v>
+        <v>6737330000</v>
       </c>
     </row>
     <row r="6">
@@ -623,20 +623,20 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>65324.2891</v>
+        <v>64333.5391</v>
       </c>
       <c r="F6" t="n">
-        <v>898.3398</v>
+        <v>-990.75</v>
       </c>
       <c r="G6" t="n">
-        <v>1.39</v>
+        <v>-1.52</v>
       </c>
       <c r="H6" t="n">
-        <v>168700000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -694,15 +694,9 @@
           <t>2026-10-19</t>
         </is>
       </c>
-      <c r="E8" t="n">
-        <v>3730.9199</v>
-      </c>
-      <c r="F8" t="n">
-        <v>14.636</v>
-      </c>
-      <c r="G8" t="n">
-        <v>0.39</v>
-      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
       <c r="H8" t="n">
         <v>3124419136</v>
       </c>
@@ -725,20 +719,20 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>10730.4805</v>
+        <v>10881.9004</v>
       </c>
       <c r="F9" t="n">
-        <v>-151.4199</v>
+        <v>41.5</v>
       </c>
       <c r="G9" t="n">
-        <v>-1.39</v>
+        <v>0.38</v>
       </c>
       <c r="H9" t="n">
-        <v>0</v>
+        <v>876343700</v>
       </c>
     </row>
     <row r="10">
@@ -759,20 +753,20 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>25211.3906</v>
+        <v>25622.6094</v>
       </c>
       <c r="F10" t="n">
-        <v>-411.2188</v>
+        <v>239.9902</v>
       </c>
       <c r="G10" t="n">
-        <v>-1.6</v>
+        <v>0.95</v>
       </c>
       <c r="H10" t="n">
-        <v>0</v>
+        <v>59759400</v>
       </c>
     </row>
     <row r="11">
@@ -793,20 +787,20 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>5412</v>
+        <v>5415.5298</v>
       </c>
       <c r="F11" t="n">
-        <v>-3.5298</v>
+        <v>12.0298</v>
       </c>
       <c r="G11" t="n">
-        <v>-0.07000000000000001</v>
+        <v>0.22</v>
       </c>
       <c r="H11" t="n">
-        <v>0</v>
+        <v>305854400</v>
       </c>
     </row>
     <row r="12">
@@ -831,13 +825,13 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>17943</v>
+        <v>18056</v>
       </c>
       <c r="F12" t="n">
-        <v>-77.0996</v>
+        <v>35.9004</v>
       </c>
       <c r="G12" t="n">
-        <v>-0.43</v>
+        <v>0.2</v>
       </c>
       <c r="H12" t="n">
         <v>0</v>
@@ -865,13 +859,13 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>101.939</v>
+        <v>101.925</v>
       </c>
       <c r="F13" t="n">
-        <v>0.099</v>
+        <v>0.08500000000000001</v>
       </c>
       <c r="G13" t="n">
-        <v>0.1</v>
+        <v>0.08</v>
       </c>
       <c r="H13" t="n">
         <v>0</v>
@@ -895,17 +889,17 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>158.41</v>
+        <v>158.554</v>
       </c>
       <c r="F14" t="n">
-        <v>0.267</v>
+        <v>0.748</v>
       </c>
       <c r="G14" t="n">
-        <v>0.17</v>
+        <v>0.47</v>
       </c>
       <c r="H14" t="n">
         <v>0</v>
@@ -933,13 +927,13 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>0.5127</v>
+        <v>0.5135999999999999</v>
       </c>
       <c r="F15" t="n">
-        <v>0.0029</v>
+        <v>0.0038</v>
       </c>
       <c r="G15" t="n">
-        <v>0.57</v>
+        <v>0.75</v>
       </c>
       <c r="H15" t="n">
         <v>0</v>
@@ -967,13 +961,13 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>0.5465</v>
+        <v>0.5472</v>
       </c>
       <c r="F16" t="n">
-        <v>0.0029</v>
+        <v>0.0036</v>
       </c>
       <c r="G16" t="n">
-        <v>0.53</v>
+        <v>0.66</v>
       </c>
       <c r="H16" t="n">
         <v>0</v>
@@ -1001,13 +995,13 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>0.4077</v>
+        <v>0.4075</v>
       </c>
       <c r="F17" t="n">
-        <v>0.0007</v>
+        <v>0.0005</v>
       </c>
       <c r="G17" t="n">
-        <v>0.17</v>
+        <v>0.12</v>
       </c>
       <c r="H17" t="n">
         <v>0</v>
@@ -1034,17 +1028,11 @@
           <t>2026-10-19</t>
         </is>
       </c>
-      <c r="E18" t="n">
-        <v>79.61499999999999</v>
-      </c>
-      <c r="F18" t="n">
-        <v>-0.435</v>
-      </c>
-      <c r="G18" t="n">
-        <v>-0.54</v>
-      </c>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
       <c r="H18" t="n">
-        <v>10128450</v>
+        <v>30938119</v>
       </c>
     </row>
     <row r="19">
@@ -1068,17 +1056,11 @@
           <t>2026-10-19</t>
         </is>
       </c>
-      <c r="E19" t="n">
-        <v>76.905</v>
-      </c>
-      <c r="F19" t="n">
-        <v>0.045</v>
-      </c>
-      <c r="G19" t="n">
-        <v>0.06</v>
-      </c>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr"/>
       <c r="H19" t="n">
-        <v>9681941</v>
+        <v>30721779</v>
       </c>
     </row>
     <row r="20">
@@ -1103,16 +1085,16 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>4165.7002</v>
+        <v>4151</v>
       </c>
       <c r="F20" t="n">
-        <v>-15.3999</v>
+        <v>-30.1001</v>
       </c>
       <c r="G20" t="n">
-        <v>-0.37</v>
+        <v>-0.72</v>
       </c>
       <c r="H20" t="n">
-        <v>93751</v>
+        <v>5080</v>
       </c>
     </row>
     <row r="21">
@@ -1137,16 +1119,16 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>97.56</v>
+        <v>98.40000000000001</v>
       </c>
       <c r="F21" t="n">
-        <v>-3.85</v>
+        <v>-3.01</v>
       </c>
       <c r="G21" t="n">
-        <v>-3.8</v>
+        <v>-2.97</v>
       </c>
       <c r="H21" t="n">
-        <v>151070</v>
+        <v>4142</v>
       </c>
     </row>
     <row r="22">
@@ -1171,16 +1153,16 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>108.02</v>
+        <v>109.34</v>
       </c>
       <c r="F22" t="n">
-        <v>-1.84</v>
+        <v>-0.52</v>
       </c>
       <c r="G22" t="n">
-        <v>-1.67</v>
+        <v>-0.47</v>
       </c>
       <c r="H22" t="n">
-        <v>19029</v>
+        <v>309</v>
       </c>
     </row>
     <row r="23">
@@ -1205,16 +1187,16 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>6.5475</v>
+        <v>6.5635</v>
       </c>
       <c r="F23" t="n">
-        <v>0.0165</v>
+        <v>0.0325</v>
       </c>
       <c r="G23" t="n">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="H23" t="n">
-        <v>24396</v>
+        <v>866</v>
       </c>
     </row>
     <row r="24">
@@ -1238,17 +1220,11 @@
           <t>2026-10-19</t>
         </is>
       </c>
-      <c r="E24" t="n">
-        <v>63.67</v>
-      </c>
-      <c r="F24" t="n">
-        <v>0.82</v>
-      </c>
-      <c r="G24" t="n">
-        <v>1.3</v>
-      </c>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr"/>
       <c r="H24" t="n">
-        <v>8356721</v>
+        <v>22046286</v>
       </c>
     </row>
     <row r="25">
@@ -1273,13 +1249,13 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>17.73</v>
+        <v>18.44</v>
       </c>
       <c r="F25" t="n">
-        <v>-2.26</v>
+        <v>-1.55</v>
       </c>
       <c r="G25" t="n">
-        <v>-11.31</v>
+        <v>-7.75</v>
       </c>
       <c r="H25" t="n">
         <v>0</v>
@@ -1303,20 +1279,20 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="E26" t="n">
-        <v>82372.99219999999</v>
+        <v>81545.8906</v>
       </c>
       <c r="F26" t="n">
-        <v>355.3906</v>
+        <v>-471.7109</v>
       </c>
       <c r="G26" t="n">
-        <v>0.43</v>
+        <v>-0.58</v>
       </c>
       <c r="H26" t="n">
-        <v>26750234624</v>
+        <v>24411439104</v>
       </c>
     </row>
     <row r="27">
@@ -1749,22 +1725,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>IHSG Melorot ke Bawah 5.000, Danantara Mau Borong Saham BUMN</t>
+          <t>Prancis Membara Dilanda Kerusuhan, 1.500 Toko Dijarah</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Mon, 19 Oct 2026 22:13:04 +0700</t>
+          <t>Tue, 20 Oct 2026 07:25:00 +0700</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/03/11/rosan-roeslani-firda-cynthia-anggrainy-al-djokyadetikcom-1741681299971_169.jpeg?w=360&amp;amp;q=90" /&gt; CEO Danantara Rosan Roeslani menanggapi Indeks Harga Saham Gabungan (IHSG) yang turun hingga ke bawah level 5.000.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2023/07/02/kerusuhan-di-prancis-kian-memanas-1000-orang-ditangkap-6_169.jpeg?w=360&amp;amp;q=90" /&gt; Ratusan ribu pengunjuk rasa di Prancis menyuarakan ketidakpuasan mereka atas kenaikan biaya hidup, upah rendah, dan pemangkasan anggaran pendidi</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/bursa-dan-valas/d-8714705/ihsg-melorot-ke-bawah-5-000-danantara-mau-borong-saham-bumn</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8714785/prancis-membara-dilanda-kerusuhan-1-500-toko-dijarah</t>
         </is>
       </c>
     </row>
@@ -1776,22 +1752,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Penyebab Listrik Batam Padam Diusut, Bos PLN Pastikan Bukan Sabotase</t>
+          <t>Lapangan Multiguna Bekasi Ditata Ulang untuk Sambut Ajang Olahraga Jabar</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Mon, 19 Oct 2026 21:54:44 +0700</t>
+          <t>Tue, 20 Oct 2026 07:15:51 +0700</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2023/01/01/pembangkit-listrik-pln-batam-foto-dok-pln_169.jpeg?w=360&amp;amp;q=90" /&gt; PLN sedang menyelidiki lebih dalam penyebab listrik padam di Batam, Kepulauan Riau, beberapa hari lalu.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/19/pemkot-bekasi-kebut-renovasi-lapangan-multiguna-siap-sambut-porprov-jabar-2026-1792426174773_169.jpeg?w=360&amp;amp;q=90" /&gt; Pemerintah Kota Bekasi mempercepat pembenahan Lapangan Multiguna untuk menyambut Porprov XV Jawa Barat. Proy</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8714688/penyebab-listrik-batam-padam-diusut-bos-pln-pastikan-bukan-sabotase</t>
+          <t>https://finance.detik.com/foto-bisnis/d-8714760/lapangan-multiguna-bekasi-ditata-ulang-untuk-sambut-ajang-olahraga-jabar</t>
         </is>
       </c>
     </row>
@@ -1803,22 +1779,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Dua Tahun Prabowo: Investasi Rp 3.923 Triliun, 5,4 Juta Tenaga Kerja Terserap</t>
+          <t>Bos BEI Ungkap Alasan RI Layak Bertahan di Emerging Market</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Mon, 19 Oct 2026 21:40:16 +0700</t>
+          <t>Tue, 20 Oct 2026 06:55:00 +0700</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/08/06/presiden-prabowo-subianto-menggelar-sidang-kabinet-rabu-682025-1754475097038_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Investasi dan Hilirisasi/Kepala BKPM Rosan Roeslani mengatakan total investasi dalam 2 tahun capai Rp 3.923 triliun.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/16/ihsg-ambruk-1157-ditutup-di-level-5185-1792144638939_169.jpeg?w=360&amp;amp;q=90" /&gt; Bursa Efek Indonesia (BEI) menegaskan Indonesia masih layak menyandang status Emerging Market.</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8714675/dua-tahun-prabowo-investasi-rp-3-923-triliun-5-4-juta-tenaga-kerja-terserap</t>
+          <t>https://finance.detik.com/bursa-dan-valas/d-8714782/bos-bei-ungkap-alasan-ri-layak-bertahan-di-emerging-market</t>
         </is>
       </c>
     </row>
@@ -1830,22 +1806,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>5 Besar Investor Asing di Indonesia, Singapura Masih Rajanya</t>
+          <t>Dugaan Permainan Harga Ayam dan Telur Mulai Terendus</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Mon, 19 Oct 2026 21:25:48 +0700</t>
+          <t>Tue, 20 Oct 2026 06:25:00 +0700</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2023/03/28/ilustrasi-pertumbuhan-ekonomi_169.jpeg?w=360&amp;amp;q=90" /&gt; Realisasi investasi di Indonesia sepanjang Januari-September 2026 mencapai Rp 1.539,2 triliun atau 75,4% dari target. Singapura masih investor asing terbesar</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/06/11/produksi-telur-berlimpah-peternak-hadapi-tantangan-harga-1781149160668_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Pertanian buka suara soal permainan harga ayam dan telur.</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8714667/5-besar-investor-asing-di-indonesia-singapura-masih-rajanya</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8714771/dugaan-permainan-harga-ayam-dan-telur-mulai-terendus</t>
         </is>
       </c>
     </row>
@@ -1857,22 +1833,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Biang Kerok Masalah BBM di Bali: Kapal dari Jawa Terlambat Masuk</t>
+          <t>Warga Karet Kuningan Olah Sampah Plastik Jadi BBM Alternatif</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Mon, 19 Oct 2026 21:13:33 +0700</t>
+          <t>Tue, 20 Oct 2026 06:00:13 +0700</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/19/kondisi-antrean-pengisian-bbm-bersubsidi-yang-sudah-normal-kembali-di-spbu-besang-semarapura-tengah-klungkung-bali-senin-19102-1792374026464_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Energi dan Sumber Daya Mineral (ESDM) Bahlil Lahadal</t>
+          <t xml:space="preserve">&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/19/warga-karet-kuningan-olah-sampah-plastik-jadi-bbm-alternatif-1-kg-hasilkan-09-liter-1792404845273_169.jpeg?w=360&amp;amp;q=90" /&gt; Warga Karet Kuningan, Jakarta Selatan, mengolah sampah plastik menjadi BBM alternatif bernama Petasol. </t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8714655/biang-kerok-masalah-bbm-di-bali-kapal-dari-jawa-terlambat-masuk</t>
+          <t>https://finance.detik.com/foto-bisnis/d-8714727/warga-karet-kuningan-olah-sampah-plastik-jadi-bbm-alternatif</t>
         </is>
       </c>
     </row>
@@ -1884,22 +1860,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Inovasi Pertanian Ramah Lingkungan di Pasar Minggu</t>
+          <t>Bakal Didepak Bursa dari Perhitungan IHSG, Ini Daftar 80 Saham HSC</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Mon, 19 Oct 2026 21:12:34 +0700</t>
+          <t>Tue, 20 Oct 2026 05:55:00 +0700</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/19/pemanfaatan-limbah-galon-untuk-tanam-padi-di-jakarta-1792418941312_169.jpeg?w=360&amp;amp;q=90" /&gt; Posyantek Kreya Loka memanfaatkan 1.500 galon plastik bekas untuk menanam padi di RPTRA Belimbing, Jakarta Selatan, sebagai inovasi ke</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/19/ihsg-dibuka-anjlok-431-bei-berlakukan-arb-7-1792382663579_169.jpeg?w=360&amp;amp;q=90" /&gt; BEI tidak lagi memperhitungkan saham-saham dengan kepemilikan terkonsentrasi tinggi atau high shareholding concentration (HSC) dalam perhitunga</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/foto-bisnis/d-8714649/inovasi-pertanian-ramah-lingkungan-di-pasar-minggu</t>
+          <t>https://finance.detik.com/bursa-dan-valas/d-8714769/bakal-didepak-bursa-dari-perhitungan-ihsg-ini-daftar-80-saham-hsc</t>
         </is>
       </c>
     </row>
@@ -1911,22 +1887,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Menjaga Asa Ekonomi Lewat Martabak Mini</t>
+          <t>Eks Menteri Kritik Singapura soal Karhutla: 4 dari 7 Perusahaan Tercatat di Sana!</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Mon, 19 Oct 2026 21:03:22 +0700</t>
+          <t>Tue, 20 Oct 2026 05:25:00 +0700</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/19/kisah-sri-bertahan-jualan-martabak-mini-sejak-pandemi-1792418064215_169.jpeg?w=360&amp;amp;q=90" /&gt; Sejak pandemi COVID-19, Sri Rahayu (52) tekun berjualan martabak mini di Bekasi. Beromzet sekitar Rp 300 ribu sehari, usaha ini menja</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/03/lahan-gambut-banjar-terbakar-petugas-berjibaku-jinakkan-api-1788405575337_169.jpeg?w=360&amp;amp;q=90" /&gt; Mantan Menteri Perdagangan Muhammad Lutfi mengkritik Singapura soal teguran ke 7 perusahaan yang dianggap bertanggung jawab ata</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/foto-bisnis/d-8714627/menjaga-asa-ekonomi-lewat-martabak-mini</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8714756/eks-menteri-kritik-singapura-soal-karhutla-4-dari-7-perusahaan-tercatat-di-sana</t>
         </is>
       </c>
     </row>
@@ -1938,22 +1914,22 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Harga Minyak Tembus US$ 100/ Barel, Bahlil: Kondisi Global Makin Tak Menentu</t>
+          <t>Bahlil Sebut Pabrik Baterai CATL di Karawang Segera Diresmikan</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Mon, 19 Oct 2026 20:50:01 +0700</t>
+          <t>Mon, 19 Oct 2026 22:54:03 +0700</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/08/04/bahlil-lahadalia-1785840108228_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri ESDM Bahlil Lahadalia mengungkapkan harga minyak mentah Indonesia melonjak tajam seiring kenaikan harga minyak dunia.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/08/04/bahlil-lahadalia-1785840108228_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Koordinator Bidang Hilirisasi dan Transisi Energi Bahlil Lahadalia mengatakan pabrik baterai CATL di Karawang akan diresmikan dalam waktu dekat.</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8714613/harga-minyak-tembus-us-100-barel-bahlil-kondisi-global-makin-tak-menentu</t>
+          <t>https://finance.detik.com/energi/d-8714738/bahlil-sebut-pabrik-baterai-catl-di-karawang-segera-diresmikan</t>
         </is>
       </c>
     </row>
@@ -1965,22 +1941,22 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Bos OJK Buka Suara Usai Lapor Kondisi Bursa Saham ke Prabowo</t>
+          <t>Wanti-wanti buat Pemerintah, Inflasi Pangan Bisa Melonjak ke 5%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Mon, 19 Oct 2026 20:32:43 +0700</t>
+          <t>Mon, 19 Oct 2026 22:43:15 +0700</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/08/03/frederica-widyasari-dewi-1785765447950_169.jpeg?w=360&amp;amp;q=90" /&gt; Pengumuman lembaga pemeringkatan MSCI soal potensi penurunan bursa saham Indonesia ke Standalone Market menimbulkan sentimen negatif.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/02/09/pedagang-bahan-pangan-di-pasar-lakessi-1770618996980_169.jpeg?w=360&amp;amp;q=90" /&gt; Gubernur Bank Indonesia (BI) Destry Damayanti mewanti-wanti soal inflasi pangan.</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/bursa-dan-valas/d-8714572/bos-ojk-buka-suara-usai-lapor-kondisi-bursa-saham-ke-prabowo</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8714725/wanti-wanti-buat-pemerintah-inflasi-pangan-bisa-melonjak-ke-5</t>
         </is>
       </c>
     </row>
@@ -1992,22 +1968,22 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Investasi Tembus Rp 1.539,2 Triliun, Serap 2,19 Juta Tenaga Kerja</t>
+          <t>Tetap Ada Efisiensi, Belanja Kuartal IV Disiapkan Rp 1.300 Triliun</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Mon, 19 Oct 2026 20:22:05 +0700</t>
+          <t>Mon, 19 Oct 2026 22:36:47 +0700</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/11/20/menteri-investasi-dan-hilirisasikepala-bkpm-rosan-roeslani-1763634019135_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Investasi dan Hilirisasi/Kepala BKPM Rosan Roeslani mencatat realisasi investasi sepanjang periode Januari-September men</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/09/apbn-defisit-rp319-triliun-menkeu-sebut-masih-sesuai-target-1791525967190_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Keuangan (Menkeu) Suahasil Nazara buka suara soal belanja anggaran pemerintah, termasuk soal efisiensi.</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8714565/investasi-tembus-rp-1-539-2-triliun-serap-2-19-juta-tenaga-kerja</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8714721/tetap-ada-efisiensi-belanja-kuartal-iv-disiapkan-rp-1-300-triliun</t>
         </is>
       </c>
     </row>
@@ -2019,22 +1995,22 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Ekspor dari Berbagai Sektor Bakal Digenjot</t>
+          <t>Suku Bunga Bank Sentral AS Diprediksi Naik, Bagaimana Nasib Rupiah?</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Mon, 19 Oct 2026 20:09:58 +0700</t>
+          <t>Mon, 19 Oct 2026 22:23:40 +0700</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/06/09/tanjung-priok-tetap-sibuk-di-tengah-tekanan-dolar-harapan-ekspor-menguat-1780979464280_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Koordinator Perekonomian Airlangga Hartarto mengatakan pemerintah menggenjot kinerja ekspor nasional</t>
+          <t xml:space="preserve">&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/07/08/rupiah-melemah-lagi-dolar-as-kembali-bertengger-di-rp18000-1783502390635_169.jpeg?w=360&amp;amp;q=90" /&gt; Gubernur Bank Indonesia (BI) Destry Damayanti memprediksi suku bunga bank sentral Amerika Serikat (AS) atau The Federal Reserve </t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/ekonomi-bisnis/d-8714554/ekspor-dari-berbagai-sektor-bakal-digenjot</t>
+          <t>https://finance.detik.com/bursa-dan-valas/d-8714711/suku-bunga-bank-sentral-as-diprediksi-naik-bagaimana-nasib-rupiah</t>
         </is>
       </c>
     </row>
@@ -2046,22 +2022,22 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Kedai Inspirasi Bekasi, Ruang Difabel Merajut Kemandirian Ekonomi</t>
+          <t>IHSG Melorot ke Bawah 5.000, Danantara Mau Borong Saham BUMN</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Mon, 19 Oct 2026 19:51:09 +0700</t>
+          <t>Mon, 19 Oct 2026 22:13:04 +0700</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/19/kedai-inspirasi-bekasi-ruang-difabel-merajut-kemandirian-ekonomi-1792395314234.jpeg?w=360&amp;amp;q=90" /&gt; Kedai Inspirasi menjadi ruang bagi penyandang disabilitas untuk mengembangkan keterampilan kerja dan membangun kemandirian eko</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/03/11/rosan-roeslani-firda-cynthia-anggrainy-al-djokyadetikcom-1741681299971_169.jpeg?w=360&amp;amp;q=90" /&gt; CEO Danantara Rosan Roeslani menanggapi Indeks Harga Saham Gabungan (IHSG) yang turun hingga ke bawah level 5.000.</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/foto-bisnis/d-8713877/kedai-inspirasi-bekasi-ruang-difabel-merajut-kemandirian-ekonomi</t>
+          <t>https://finance.detik.com/bursa-dan-valas/d-8714705/ihsg-melorot-ke-bawah-5-000-danantara-mau-borong-saham-bumn</t>
         </is>
       </c>
     </row>
@@ -2073,22 +2049,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>131 CEO Global Kumpul di Jakarta, Danantara Incar Kesepakatan Besar</t>
+          <t>Penyebab Listrik Batam Padam Diusut, Bos PLN Pastikan Bukan Sabotase</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Mon, 19 Oct 2026 19:00:20 +0700</t>
+          <t>Mon, 19 Oct 2026 21:54:44 +0700</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/19/danantara-1792409910587_169.jpeg?w=360&amp;amp;q=90" /&gt; Danantara Indonesia akan menggelar DTIIF 2026 pada 26-28 Oktober di Jakarta.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2023/01/01/pembangkit-listrik-pln-batam-foto-dok-pln_169.jpeg?w=360&amp;amp;q=90" /&gt; PLN sedang menyelidiki lebih dalam penyebab listrik padam di Batam, Kepulauan Riau, beberapa hari lalu.</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8714447/131-ceo-global-kumpul-di-jakarta-danantara-incar-kesepakatan-besar</t>
+          <t>https://finance.detik.com/energi/d-8714688/penyebab-listrik-batam-padam-diusut-bos-pln-pastikan-bukan-sabotase</t>
         </is>
       </c>
     </row>
@@ -2100,22 +2076,22 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>IHSG Seharian Melemah, Ditutup ke Level 4.900</t>
+          <t>Dua Tahun Prabowo: Investasi Rp 3.923 Triliun, 5,4 Juta Tenaga Kerja Terserap</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Mon, 19 Oct 2026 18:34:09 +0700</t>
+          <t>Mon, 19 Oct 2026 21:40:16 +0700</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/19/ihsg-dibuka-anjlok-431-bei-berlakukan-arb-7-1792382663303_169.jpeg?w=360&amp;amp;q=90" /&gt; IHSG ditutup melemah di zona merah, turun 188,49 poin ke 5.936,14. Ini merupakan level terendah dalam 10 tahun terakhir.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/08/06/presiden-prabowo-subianto-menggelar-sidang-kabinet-rabu-682025-1754475097038_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Investasi dan Hilirisasi/Kepala BKPM Rosan Roeslani mengatakan total investasi dalam 2 tahun capai Rp 3.923 triliun.</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/bursa-dan-valas/d-8714438/ihsg-seharian-melemah-ditutup-ke-level-4-900</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8714675/dua-tahun-prabowo-investasi-rp-3-923-triliun-5-4-juta-tenaga-kerja-terserap</t>
         </is>
       </c>
     </row>
@@ -2127,22 +2103,22 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Pasar Nikel Global Diproyeksi Tumbuh 21,39% hingga 2031</t>
+          <t>5 Besar Investor Asing di Indonesia, Singapura Masih Rajanya</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Mon, 19 Oct 2026 18:25:08 +0700</t>
+          <t>Mon, 19 Oct 2026 21:25:48 +0700</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/19/mind-id-1792409058599_169.jpeg?w=360&amp;amp;q=90" /&gt; Prospek pasar nikel global meningkat, membuka peluang bagi Indonesia untuk memperdalam hilirisasi industri. Fokus pada produk akhir untuk nilai tambah maksimal.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2023/03/28/ilustrasi-pertumbuhan-ekonomi_169.jpeg?w=360&amp;amp;q=90" /&gt; Realisasi investasi di Indonesia sepanjang Januari-September 2026 mencapai Rp 1.539,2 triliun atau 75,4% dari target. Singapura masih investor asing terbesar</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8714423/pasar-nikel-global-diproyeksi-tumbuh-21-39-hingga-2031</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8714667/5-besar-investor-asing-di-indonesia-singapura-masih-rajanya</t>
         </is>
       </c>
     </row>
@@ -2154,22 +2130,22 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Menag Soroti Kebakaran Hutan, Singgung Dosa Merusak Alam</t>
+          <t>Ada Demo di Jakarta Hari Ini, Cek Rekayasa Lalu Lintas dan Rute Alternatif</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Mon, 19 Oct 2026 22:02:46 +0700</t>
+          <t>Tue, 20 Oct 2026 07:36:03 +0700</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Nasaruddin mengatakan, pendekatan ekoteologi dapat menjadi salah satu upaya untuk mendorong kepedulian masyarakat terhadap kelestarian lingkungan.</t>
+          <t>Aksi demo bagai digelar di sejumlah titik di wilayah Jakarta hari ini, Selasa (20/10/2026).</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8316740/menag-soroti-kebakaran-hutan-singgung-dosa-merusak-alam</t>
+          <t>https://www.liputan6.com/news/read/8316844/ada-demo-di-jakarta-hari-ini-cek-rekayasa-lalu-lintas-dan-rute-alternatif</t>
         </is>
       </c>
     </row>
@@ -2181,22 +2157,22 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>PKS Ingatkan Kader Hati-Hati Bicara di Medsos</t>
+          <t>Cegah Pelajar Demo ke Jakarta, Dindik Tangerang Keluarkan Surat Edaran</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Mon, 19 Oct 2026 21:31:18 +0700</t>
+          <t>Tue, 20 Oct 2026 07:04:02 +0700</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>PKS berharap pejabat publik memiliki kesadaran bahwa cara menyampaikan pesan harus disesuaikan dengan perkembangan teknologi dan karakter ruang digital.</t>
+          <t>Dinas Pendidikan Kabupaten Tangerang mengeluarkan surat edaran mencegah siswa tak ikut aksi unjuk rasa dua tahun Prabowo di Jakarta.</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8316737/pks-ingatkan-kader-hati-hati-bicara-di-medsos</t>
+          <t>https://www.liputan6.com/news/read/8316834/cegah-pelajar-demo-ke-jakarta-dindik-tangerang-keluarkan-surat-edaran</t>
         </is>
       </c>
     </row>
@@ -2208,22 +2184,22 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Mantan KSAD Subagyo HS Meninggal Dunia</t>
+          <t>Benih Lobster Rp 5,8 Miliar Gagal Diselundupkan ke Luar Negeri</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Mon, 19 Oct 2026 21:06:13 +0700</t>
+          <t>Tue, 20 Oct 2026 06:55:06 +0700</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Subagyo HS meninggal dunia di RS Panti Rapih, Yogyakarta, Senin (19/10/2026) sore.</t>
+          <t>Penyelundupan benih lobster senilai Rp 5,8 miliar berhasil digagalkan. Tercium upaya pencucian uang dari hasil tindak pelanggaran ini.</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8316722/mantan-ksad-subagyo-hs-meninggal-dunia</t>
+          <t>https://www.liputan6.com/news/read/8316833/benih-lobster-rp-58-miliar-gagal-diselundupkan-ke-luar-negeri</t>
         </is>
       </c>
     </row>
@@ -2235,22 +2211,22 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Prabowo Soroti Kinerja ASN-Polri</t>
+          <t>Siapa Perusahaan Dibidik Biang Kerok Karhutla</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Mon, 19 Oct 2026 20:52:56 +0700</t>
+          <t>Tue, 20 Oct 2026 06:05:45 +0700</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Prabowo menyampaikan terkait pentingnya profesionalisme, integritas, dan kompetensi aparatur negara dalam penyelenggaraan pemerintahan.</t>
+          <t>Aparat kini membidik pertanggungjawaban korporasi, termasuk kemungkinan menelusuri pemilik perusahaan hingga pemegang saham</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8316715/prabowo-soroti-kinerja-asn-polri</t>
+          <t>https://www.liputan6.com/news/read/8316812/siapa-perusahaan-dibidik-biang-kerok-karhutla</t>
         </is>
       </c>
     </row>
@@ -2262,22 +2238,22 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Ini Hasil Tes Urine Sopir Pajero Tabrak Remaja hingga Tewas di Jaksel</t>
+          <t>Mengurai Fakta di Balik Kasus Polisi Tembak Polisi di Markas Polairud</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Mon, 19 Oct 2026 20:14:42 +0700</t>
+          <t>Tue, 20 Oct 2026 05:00:05 +0700</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Hasil tes urine dilakukan kepolisian menunjukkan sopir negatif dari penyalahgunaan narkoba.</t>
+          <t>Bharatu Valdo tewas dalam insiden yang melibatkan Bharada Andika Rahmadani. Dugaan motif terkait persoalan pribadi.</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8316696/ini-hasil-tes-urine-sopir-pajero-tabrak-remaja-hingga-tewas-di-jaksel</t>
+          <t>https://www.liputan6.com/news/read/8316808/mengurai-fakta-di-balik-kasus-polisi-tembak-polisi-di-markas-polairud</t>
         </is>
       </c>
     </row>
@@ -2289,22 +2265,22 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Nadiem Makarim Ajukan Kasasi, Ini Permintaannya ke Hakim</t>
+          <t>Subagyo HS, KSAD yang Pernah Mengabdi di Era Tiga Presiden</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Mon, 19 Oct 2026 20:13:26 +0700</t>
+          <t>Tue, 20 Oct 2026 00:00:49 +0700</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Nadiem beberkan lima alasan Nadiem ajukan kasasi.</t>
+          <t>Subagyo HS merupakan perwira TNI lulusan Akabri Magelang tahun 1970.</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8316695/nadiem-makarim-ajukan-kasasi-ini-permintaannya-ke-hakim</t>
+          <t>https://www.liputan6.com/news/read/8316777/subagyo-hs-ksad-yang-pernah-mengabdi-di-era-tiga-presiden</t>
         </is>
       </c>
     </row>
@@ -2316,22 +2292,22 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Kronologi Bharatu Valdo Ditembak Rekan Sesama Polisi Versi Pengacara</t>
+          <t>Wamenag Dorong Hukuman Maksimal Pelaku Kekerasan Seksual</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Mon, 19 Oct 2026 19:50:36 +0700</t>
+          <t>Mon, 19 Oct 2026 23:58:49 +0700</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Penyidik menyampaikan bahwa tersangka diduga melampiaskan kemarahan karena teman-teman seangkatan korban disebut kerap melakukan perundungan.</t>
+          <t>Kemenag telah membangun sistem penanganan kasus kekerasan di lingkungan pendidikan keagamaan.</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8316686/kronologi-bharatu-valdo-ditembak-rekan-sesama-polisi-versi-pengacara</t>
+          <t>https://www.liputan6.com/news/read/8316795/wamenag-dorong-hukuman-maksimal-pelaku-kekerasan-seksual</t>
         </is>
       </c>
     </row>
@@ -2343,22 +2319,22 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Dudung soal Karhutla Belum jadi Bencana Nasional: Negara Masih Sanggup</t>
+          <t>Catat, Ini Rute Alternatif Hindari Macet saat Demo di Jakarta Besok</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Mon, 19 Oct 2026 19:23:41 +0700</t>
+          <t>Mon, 19 Oct 2026 23:54:26 +0700</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Dudung juga menjawab tawaran Malaysia untuk mengirimkan tiga helikopter.</t>
+          <t>Pengguna jalan diharapkan menyesuaikan waktu keberangkatan, memanfaatkan rute alternatif, dan menghindari kawasan tersebut</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8316670/dudung-soal-karhutla-belum-jadi-bencana-nasional-negara-masih-sanggup</t>
+          <t>https://www.liputan6.com/news/read/8316794/catat-ini-rute-alternatif-hindari-macet-saat-demo-di-jakarta-besok</t>
         </is>
       </c>
     </row>
@@ -2370,22 +2346,22 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Dudung Ungkap Tawaran Malaysia dan Singapura Tangani Kebakaran Hutan</t>
+          <t>Ketua Komisi III Wanti-wanti RUU Perampasan Aset: Rentan Jadi Bumerang</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Mon, 19 Oct 2026 19:16:35 +0700</t>
+          <t>Mon, 19 Oct 2026 23:00:16 +0700</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Pemerintah Indonesia telah merespons usulan bantuan tersebut. Adapun teknis pelaksanaan bantuan masih perlu dikoordinasikan lebih lanjut.</t>
+          <t>Habiburokhman mengingatkan RUU Perampasan Aset harus memiliki perlindungan hukum agar tidak disalahgunakan.</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8316667/dudung-ungkap-tawaran-malaysia-dan-singapura-tangani-kebakaran-hutan</t>
+          <t>https://www.liputan6.com/news/read/8316733/ketua-komisi-iii-wanti-wanti-ruu-perampasan-aset-rentan-jadi-bumerang</t>
         </is>
       </c>
     </row>
@@ -2397,22 +2373,22 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Survei Terbaru Poltracking: 55,3% Responden Puas Kinerja Pemerintahan Prabowo-Gibran</t>
+          <t>Menag Soroti Kebakaran Hutan, Singgung Dosa Merusak Alam</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Mon, 19 Oct 2026 19:05:36 +0700</t>
+          <t>Mon, 19 Oct 2026 22:02:46 +0700</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Survei Poltracking berlangsung pada 30 September hingga 7 Oktober 2026.</t>
+          <t>Nasaruddin mengatakan, pendekatan ekoteologi dapat menjadi salah satu upaya untuk mendorong kepedulian masyarakat terhadap kelestarian lingkungan.</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8316660/survei-terbaru-poltracking-553-responden-puas-kinerja-pemerintahan-prabowo-gibran</t>
+          <t>https://www.liputan6.com/news/read/8316740/menag-soroti-kebakaran-hutan-singgung-dosa-merusak-alam</t>
         </is>
       </c>
     </row>
@@ -2424,22 +2400,22 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Polisi Tembak Polisi, Pengacara Bharatu Valdo Pertanyakan Asal Senjata</t>
+          <t>PKS Ingatkan Kader Hati-Hati Bicara di Medsos</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Mon, 19 Oct 2026 19:05:13 +0700</t>
+          <t>Mon, 19 Oct 2026 21:31:18 +0700</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Kubu Bharatu Valdo mempertanyakan pengawasan senjata diperoleh pelaku penembakan di markas polairud, Pondok Cabe, Pamulang, Tangerang Selatan.</t>
+          <t>PKS berharap pejabat publik memiliki kesadaran bahwa cara menyampaikan pesan harus disesuaikan dengan perkembangan teknologi dan karakter ruang digital.</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8316659/polisi-tembak-polisi-pengacara-bharatu-valdo-pertanyakan-asal-senjata</t>
+          <t>https://www.liputan6.com/news/read/8316737/pks-ingatkan-kader-hati-hati-bicara-di-medsos</t>
         </is>
       </c>
     </row>
@@ -2451,22 +2427,22 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Survei Poltracking: Gerindra 22,9 Persen, PDIP 13,4 Persen</t>
+          <t>Mantan KSAD Subagyo HS Meninggal Dunia</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Mon, 19 Oct 2026 19:02:02 +0700</t>
+          <t>Mon, 19 Oct 2026 21:06:13 +0700</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Sejumlah partai berpotensi kembali lolos ke parlemen apabila ambang batas parlemen atau parliamentary threshold tetap ditetapkan sebesar 4%.</t>
+          <t>Subagyo HS meninggal dunia di RS Panti Rapih, Yogyakarta, Senin (19/10/2026) sore.</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8316649/survei-poltracking-gerindra-229-persen-pdip-134-persen</t>
+          <t>https://www.liputan6.com/news/read/8316722/mantan-ksad-subagyo-hs-meninggal-dunia</t>
         </is>
       </c>
     </row>
@@ -2478,22 +2454,22 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Dua Strategi Pemprov Jakarta Antisipasi Asap Kebakaran Hutan</t>
+          <t>Prabowo Soroti Kinerja ASN-Polri</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Mon, 19 Oct 2026 18:36:15 +0700</t>
+          <t>Mon, 19 Oct 2026 20:52:56 +0700</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Strategi ini dilakukan Pemprov DKI Jakarta, mengantisipasi penyebaran asap kebakaran hutan dan lahan dari Sumatera dan Kalimantan sejak Jumat (16/10/2026).</t>
+          <t>Prabowo menyampaikan terkait pentingnya profesionalisme, integritas, dan kompetensi aparatur negara dalam penyelenggaraan pemerintahan.</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8316647/dua-strategi-pemprov-jakarta-antisipasi-asap-kebakaran-hutan</t>
+          <t>https://www.liputan6.com/news/read/8316715/prabowo-soroti-kinerja-asn-polri</t>
         </is>
       </c>
     </row>
@@ -2505,22 +2481,22 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Dari Apartemen di India, Rocky si Orangutan Akhirnya Pulang ke Indonesia</t>
+          <t>Ini Hasil Tes Urine Sopir Pajero Tabrak Remaja hingga Tewas di Jaksel</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Mon, 19 Oct 2026 18:17:40 +0700</t>
+          <t>Mon, 19 Oct 2026 20:14:42 +0700</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Rocky korban kejahatan perdagangan ilegal satwa liar lintas negara saat masih berusia 18-20 bulan.</t>
+          <t>Hasil tes urine dilakukan kepolisian menunjukkan sopir negatif dari penyalahgunaan narkoba.</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8316632/dari-apartemen-di-india-rocky-si-orangutan-akhirnya-pulang-ke-indonesia</t>
+          <t>https://www.liputan6.com/news/read/8316696/ini-hasil-tes-urine-sopir-pajero-tabrak-remaja-hingga-tewas-di-jaksel</t>
         </is>
       </c>
     </row>
@@ -2532,22 +2508,22 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Dudung Ungkap Arahan Prabowo untuk Perkuat Penanganan Karhutla</t>
+          <t>Nadiem Makarim Ajukan Kasasi, Ini Permintaannya ke Hakim</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Mon, 19 Oct 2026 18:01:41 +0700</t>
+          <t>Mon, 19 Oct 2026 20:13:26 +0700</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Prabowo memerintahkan pengerahan pesawat Hercules dan personel untuk memperkuat penanganan karhutla.</t>
+          <t>Nadiem beberkan lima alasan Nadiem ajukan kasasi.</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8316615/dudung-ungkap-arahan-prabowo-untuk-perkuat-penanganan-karhutla</t>
+          <t>https://www.liputan6.com/news/read/8316695/nadiem-makarim-ajukan-kasasi-ini-permintaannya-ke-hakim</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data pasar & berita - 2026-10-20 13:28 UTC
</commit_message>
<xml_diff>
--- a/data/market_news_latest.xlsx
+++ b/data/market_news_latest.xlsx
@@ -487,20 +487,20 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>5185.105</v>
+        <v>5278.8882</v>
       </c>
       <c r="F2" t="n">
-        <v>-678.6748</v>
+        <v>282.2793</v>
       </c>
       <c r="G2" t="n">
-        <v>-11.57</v>
+        <v>5.65</v>
       </c>
       <c r="H2" t="n">
-        <v>650917300</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -534,7 +534,7 @@
         <v>0.41</v>
       </c>
       <c r="H3" t="n">
-        <v>2634321000</v>
+        <v>4587260000</v>
       </c>
     </row>
     <row r="4">
@@ -568,7 +568,7 @@
         <v>-0.07000000000000001</v>
       </c>
       <c r="H4" t="n">
-        <v>394068742</v>
+        <v>394060000</v>
       </c>
     </row>
     <row r="5">
@@ -593,16 +593,16 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>26430.8867</v>
+        <v>26430.8906</v>
       </c>
       <c r="F5" t="n">
-        <v>290.8574</v>
+        <v>290.8613</v>
       </c>
       <c r="G5" t="n">
         <v>1.11</v>
       </c>
       <c r="H5" t="n">
-        <v>6737330000</v>
+        <v>7537660000</v>
       </c>
     </row>
     <row r="6">
@@ -627,13 +627,13 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>64333.5391</v>
+        <v>64075.4219</v>
       </c>
       <c r="F6" t="n">
-        <v>-990.75</v>
+        <v>-841.2773</v>
       </c>
       <c r="G6" t="n">
-        <v>-1.52</v>
+        <v>-1.3</v>
       </c>
       <c r="H6" t="n">
         <v>0</v>
@@ -657,20 +657,20 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>24186.8301</v>
+        <v>23867.7402</v>
       </c>
       <c r="F7" t="n">
-        <v>124.1094</v>
+        <v>-319.0898</v>
       </c>
       <c r="G7" t="n">
-        <v>0.52</v>
+        <v>-1.32</v>
       </c>
       <c r="H7" t="n">
-        <v>2773000000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -691,14 +691,20 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>3735.3704</v>
+      </c>
+      <c r="F8" t="n">
+        <v>4.4504</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0.12</v>
+      </c>
       <c r="H8" t="n">
-        <v>3124419136</v>
+        <v>2214600536</v>
       </c>
     </row>
     <row r="9">
@@ -719,20 +725,20 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>10881.9004</v>
+        <v>10684.6299</v>
       </c>
       <c r="F9" t="n">
-        <v>41.5</v>
+        <v>-80.0703</v>
       </c>
       <c r="G9" t="n">
-        <v>0.38</v>
+        <v>-0.74</v>
       </c>
       <c r="H9" t="n">
-        <v>876343700</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -753,20 +759,20 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>25622.6094</v>
+        <v>25122.25</v>
       </c>
       <c r="F10" t="n">
-        <v>239.9902</v>
+        <v>-197.5195</v>
       </c>
       <c r="G10" t="n">
-        <v>0.95</v>
+        <v>-0.78</v>
       </c>
       <c r="H10" t="n">
-        <v>59759400</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -787,20 +793,20 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>5415.5298</v>
+        <v>5404.02</v>
       </c>
       <c r="F11" t="n">
-        <v>12.0298</v>
+        <v>-7.98</v>
       </c>
       <c r="G11" t="n">
-        <v>0.22</v>
+        <v>-0.15</v>
       </c>
       <c r="H11" t="n">
-        <v>305854400</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -821,17 +827,17 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>18056</v>
+        <v>17943</v>
       </c>
       <c r="F12" t="n">
-        <v>35.9004</v>
+        <v>-113</v>
       </c>
       <c r="G12" t="n">
-        <v>0.2</v>
+        <v>-0.63</v>
       </c>
       <c r="H12" t="n">
         <v>0</v>
@@ -855,17 +861,17 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>101.925</v>
+        <v>101.749</v>
       </c>
       <c r="F13" t="n">
-        <v>0.08500000000000001</v>
+        <v>-0.231</v>
       </c>
       <c r="G13" t="n">
-        <v>0.08</v>
+        <v>-0.23</v>
       </c>
       <c r="H13" t="n">
         <v>0</v>
@@ -893,13 +899,13 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>158.554</v>
+        <v>157.996</v>
       </c>
       <c r="F14" t="n">
-        <v>0.748</v>
+        <v>0.19</v>
       </c>
       <c r="G14" t="n">
-        <v>0.47</v>
+        <v>0.12</v>
       </c>
       <c r="H14" t="n">
         <v>0</v>
@@ -923,17 +929,17 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>0.5135999999999999</v>
+        <v>0.5109</v>
       </c>
       <c r="F15" t="n">
-        <v>0.0038</v>
+        <v>-0.0027</v>
       </c>
       <c r="G15" t="n">
-        <v>0.75</v>
+        <v>-0.53</v>
       </c>
       <c r="H15" t="n">
         <v>0</v>
@@ -957,17 +963,17 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>0.5472</v>
+        <v>0.543</v>
       </c>
       <c r="F16" t="n">
-        <v>0.0036</v>
+        <v>-0.0042</v>
       </c>
       <c r="G16" t="n">
-        <v>0.66</v>
+        <v>-0.77</v>
       </c>
       <c r="H16" t="n">
         <v>0</v>
@@ -991,17 +997,17 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>0.4075</v>
+        <v>0.4085</v>
       </c>
       <c r="F17" t="n">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="G17" t="n">
-        <v>0.12</v>
+        <v>0.25</v>
       </c>
       <c r="H17" t="n">
         <v>0</v>
@@ -1028,11 +1034,17 @@
           <t>2026-10-19</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
+      <c r="E18" t="n">
+        <v>79.45999999999999</v>
+      </c>
+      <c r="F18" t="n">
+        <v>-0.59</v>
+      </c>
+      <c r="G18" t="n">
+        <v>-0.74</v>
+      </c>
       <c r="H18" t="n">
-        <v>30938119</v>
+        <v>30956200</v>
       </c>
     </row>
     <row r="19">
@@ -1056,11 +1068,17 @@
           <t>2026-10-19</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
+      <c r="E19" t="n">
+        <v>76.83</v>
+      </c>
+      <c r="F19" t="n">
+        <v>-0.03</v>
+      </c>
+      <c r="G19" t="n">
+        <v>-0.04</v>
+      </c>
       <c r="H19" t="n">
-        <v>30721779</v>
+        <v>31221800</v>
       </c>
     </row>
     <row r="20">
@@ -1081,20 +1099,20 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>4151</v>
+        <v>4136.7998</v>
       </c>
       <c r="F20" t="n">
-        <v>-30.1001</v>
+        <v>-23.3003</v>
       </c>
       <c r="G20" t="n">
-        <v>-0.72</v>
+        <v>-0.5600000000000001</v>
       </c>
       <c r="H20" t="n">
-        <v>5080</v>
+        <v>84848</v>
       </c>
     </row>
     <row r="21">
@@ -1115,20 +1133,20 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>98.40000000000001</v>
+        <v>99.70999999999999</v>
       </c>
       <c r="F21" t="n">
-        <v>-3.01</v>
+        <v>-3.95</v>
       </c>
       <c r="G21" t="n">
-        <v>-2.97</v>
+        <v>-3.81</v>
       </c>
       <c r="H21" t="n">
-        <v>4142</v>
+        <v>134576</v>
       </c>
     </row>
     <row r="22">
@@ -1149,20 +1167,20 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="E22" t="n">
-        <v>109.34</v>
+        <v>110.41</v>
       </c>
       <c r="F22" t="n">
-        <v>-0.52</v>
+        <v>0.86</v>
       </c>
       <c r="G22" t="n">
-        <v>-0.47</v>
+        <v>0.79</v>
       </c>
       <c r="H22" t="n">
-        <v>309</v>
+        <v>18835</v>
       </c>
     </row>
     <row r="23">
@@ -1183,20 +1201,20 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="E23" t="n">
-        <v>6.5635</v>
+        <v>6.579</v>
       </c>
       <c r="F23" t="n">
-        <v>0.0325</v>
+        <v>0.041</v>
       </c>
       <c r="G23" t="n">
-        <v>0.5</v>
+        <v>0.63</v>
       </c>
       <c r="H23" t="n">
-        <v>866</v>
+        <v>15266</v>
       </c>
     </row>
     <row r="24">
@@ -1220,11 +1238,17 @@
           <t>2026-10-19</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr"/>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr"/>
+      <c r="E24" t="n">
+        <v>63.31</v>
+      </c>
+      <c r="F24" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="G24" t="n">
+        <v>0.73</v>
+      </c>
       <c r="H24" t="n">
-        <v>22046286</v>
+        <v>22118900</v>
       </c>
     </row>
     <row r="25">
@@ -1245,17 +1269,17 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="E25" t="n">
-        <v>18.44</v>
+        <v>18.67</v>
       </c>
       <c r="F25" t="n">
-        <v>-1.55</v>
+        <v>0.23</v>
       </c>
       <c r="G25" t="n">
-        <v>-7.75</v>
+        <v>1.25</v>
       </c>
       <c r="H25" t="n">
         <v>0</v>
@@ -1283,16 +1307,16 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>81545.8906</v>
+        <v>81304.39840000001</v>
       </c>
       <c r="F26" t="n">
-        <v>-471.7109</v>
+        <v>-549.1405999999999</v>
       </c>
       <c r="G26" t="n">
-        <v>-0.58</v>
+        <v>-0.67</v>
       </c>
       <c r="H26" t="n">
-        <v>24411439104</v>
+        <v>22612764672</v>
       </c>
     </row>
     <row r="27">
@@ -1313,20 +1337,20 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="E27" t="n">
-        <v>1195</v>
+        <v>1435</v>
       </c>
       <c r="F27" t="n">
-        <v>-15</v>
+        <v>240</v>
       </c>
       <c r="G27" t="n">
-        <v>-1.24</v>
+        <v>20.08</v>
       </c>
       <c r="H27" t="n">
-        <v>335441300</v>
+        <v>232157200</v>
       </c>
     </row>
     <row r="28">
@@ -1347,20 +1371,20 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="E28" t="n">
-        <v>1125</v>
+        <v>1275</v>
       </c>
       <c r="F28" t="n">
-        <v>-80</v>
+        <v>150</v>
       </c>
       <c r="G28" t="n">
-        <v>-6.64</v>
+        <v>13.33</v>
       </c>
       <c r="H28" t="n">
-        <v>34059600</v>
+        <v>436758300</v>
       </c>
     </row>
     <row r="29">
@@ -1381,20 +1405,20 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="E29" t="n">
         <v>505</v>
       </c>
       <c r="F29" t="n">
-        <v>-35</v>
+        <v>0</v>
       </c>
       <c r="G29" t="n">
-        <v>-6.48</v>
+        <v>0</v>
       </c>
       <c r="H29" t="n">
-        <v>184792800</v>
+        <v>1225572700</v>
       </c>
     </row>
     <row r="30">
@@ -1415,20 +1439,20 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="E30" t="n">
-        <v>1835</v>
+        <v>2000</v>
       </c>
       <c r="F30" t="n">
-        <v>-20</v>
+        <v>165</v>
       </c>
       <c r="G30" t="n">
-        <v>-1.08</v>
+        <v>8.99</v>
       </c>
       <c r="H30" t="n">
-        <v>49854400</v>
+        <v>36611300</v>
       </c>
     </row>
     <row r="31">
@@ -1449,20 +1473,20 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="E31" t="n">
-        <v>3110</v>
+        <v>3150</v>
       </c>
       <c r="F31" t="n">
-        <v>-230</v>
+        <v>40</v>
       </c>
       <c r="G31" t="n">
-        <v>-6.89</v>
+        <v>1.29</v>
       </c>
       <c r="H31" t="n">
-        <v>3615400</v>
+        <v>199842000</v>
       </c>
     </row>
     <row r="32">
@@ -1483,20 +1507,20 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="E32" t="n">
-        <v>376</v>
+        <v>426</v>
       </c>
       <c r="F32" t="n">
-        <v>-28</v>
+        <v>50</v>
       </c>
       <c r="G32" t="n">
-        <v>-6.93</v>
+        <v>13.3</v>
       </c>
       <c r="H32" t="n">
-        <v>157927200</v>
+        <v>116844400</v>
       </c>
     </row>
     <row r="33">
@@ -1517,20 +1541,20 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="E33" t="n">
-        <v>456</v>
+        <v>484</v>
       </c>
       <c r="F33" t="n">
-        <v>-34</v>
+        <v>28</v>
       </c>
       <c r="G33" t="n">
-        <v>-6.94</v>
+        <v>6.14</v>
       </c>
       <c r="H33" t="n">
-        <v>17562200</v>
+        <v>168412600</v>
       </c>
     </row>
     <row r="34">
@@ -1551,20 +1575,20 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="E34" t="n">
-        <v>2760</v>
+        <v>2670</v>
       </c>
       <c r="F34" t="n">
-        <v>-200</v>
+        <v>-90</v>
       </c>
       <c r="G34" t="n">
-        <v>-6.76</v>
+        <v>-3.26</v>
       </c>
       <c r="H34" t="n">
-        <v>2824700</v>
+        <v>19202000</v>
       </c>
     </row>
     <row r="35">
@@ -1585,20 +1609,20 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="E35" t="n">
-        <v>372</v>
+        <v>346</v>
       </c>
       <c r="F35" t="n">
-        <v>-28</v>
+        <v>-26</v>
       </c>
       <c r="G35" t="n">
-        <v>-7</v>
+        <v>-6.99</v>
       </c>
       <c r="H35" t="n">
-        <v>4155400</v>
+        <v>21358700</v>
       </c>
     </row>
     <row r="36">
@@ -1619,20 +1643,20 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="E36" t="n">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="F36" t="n">
-        <v>-10</v>
+        <v>-1</v>
       </c>
       <c r="G36" t="n">
-        <v>-6.37</v>
+        <v>-0.68</v>
       </c>
       <c r="H36" t="n">
-        <v>10013700</v>
+        <v>38082800</v>
       </c>
     </row>
     <row r="37">
@@ -1653,20 +1677,20 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="E37" t="n">
-        <v>11150</v>
+        <v>10375</v>
       </c>
       <c r="F37" t="n">
-        <v>-825</v>
+        <v>-775</v>
       </c>
       <c r="G37" t="n">
-        <v>-6.89</v>
+        <v>-6.95</v>
       </c>
       <c r="H37" t="n">
-        <v>215900</v>
+        <v>1053100</v>
       </c>
     </row>
   </sheetData>
@@ -1725,22 +1749,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Prancis Membara Dilanda Kerusuhan, 1.500 Toko Dijarah</t>
+          <t>Luhut Usul ke Prabowo Kerugian Negara Bukan Pidana Korupsi</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Tue, 20 Oct 2026 07:25:00 +0700</t>
+          <t>Tue, 20 Oct 2026 20:14:23 +0700</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2023/07/02/kerusuhan-di-prancis-kian-memanas-1000-orang-ditangkap-6_169.jpeg?w=360&amp;amp;q=90" /&gt; Ratusan ribu pengunjuk rasa di Prancis menyuarakan ketidakpuasan mereka atas kenaikan biaya hidup, upah rendah, dan pemangkasan anggaran pendidi</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/06/09/luhut-hingga-chatib-basri-temui-prabowo-di-istana-1781007630172_169.jpeg?w=360&amp;amp;q=90" /&gt; Ketua Dewan Ekonomi Nasional (DEN) Luhut Binsar Pandjaitan mengusulkan kajian untuk mengubah definisi tindak pidana korupsi di Indonesia.</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8714785/prancis-membara-dilanda-kerusuhan-1-500-toko-dijarah</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8716297/luhut-usul-ke-prabowo-kerugian-negara-bukan-pidana-korupsi</t>
         </is>
       </c>
     </row>
@@ -1752,22 +1776,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Lapangan Multiguna Bekasi Ditata Ulang untuk Sambut Ajang Olahraga Jabar</t>
+          <t>MUI Tak Setuju Wajib Halal Diundur, Ini Alasannya</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Tue, 20 Oct 2026 07:15:51 +0700</t>
+          <t>Tue, 20 Oct 2026 20:00:41 +0700</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/19/pemkot-bekasi-kebut-renovasi-lapangan-multiguna-siap-sambut-porprov-jabar-2026-1792426174773_169.jpeg?w=360&amp;amp;q=90" /&gt; Pemerintah Kota Bekasi mempercepat pembenahan Lapangan Multiguna untuk menyambut Porprov XV Jawa Barat. Proy</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/01/17/logo-halal-resmi-di-negara-asean-6_169.png?w=360&amp;amp;q=90" /&gt; Awalnya, kewajiban sertifikasi halal dijadwalkan mulai berlaku 18 Oktober 2026.</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/foto-bisnis/d-8714760/lapangan-multiguna-bekasi-ditata-ulang-untuk-sambut-ajang-olahraga-jabar</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8716229/mui-tak-setuju-wajib-halal-diundur-ini-alasannya</t>
         </is>
       </c>
     </row>
@@ -1779,22 +1803,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Bos BEI Ungkap Alasan RI Layak Bertahan di Emerging Market</t>
+          <t>Respons Bos BEI soal Isu Singapura di Balik IHSG Rontok Usai Pernyataan MSCI</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Tue, 20 Oct 2026 06:55:00 +0700</t>
+          <t>Tue, 20 Oct 2026 19:56:21 +0700</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/16/ihsg-ambruk-1157-ditutup-di-level-5185-1792144638939_169.jpeg?w=360&amp;amp;q=90" /&gt; Bursa Efek Indonesia (BEI) menegaskan Indonesia masih layak menyandang status Emerging Market.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/28/direktur-utama-bei-jeffrey-hendrik-1790588485860_169.jpeg?w=360&amp;amp;q=90" /&gt; Bursa Efek Indonesia (BEI) buka suara terkait dugaan intervensi Singapura di balik usulan MSCI menurunkan status bursa saham Indonesia ke standalone mar</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/bursa-dan-valas/d-8714782/bos-bei-ungkap-alasan-ri-layak-bertahan-di-emerging-market</t>
+          <t>https://finance.detik.com/bursa-dan-valas/d-8716255/respons-bos-bei-soal-isu-singapura-di-balik-ihsg-rontok-usai-pernyataan-msci</t>
         </is>
       </c>
     </row>
@@ -1806,22 +1830,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Dugaan Permainan Harga Ayam dan Telur Mulai Terendus</t>
+          <t>6 Lembaga Tempatkan Mentan Amran Posisi Atas di Dua Tahun Prabowo-Gibran</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Tue, 20 Oct 2026 06:25:00 +0700</t>
+          <t>Tue, 20 Oct 2026 19:42:04 +0700</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/06/11/produksi-telur-berlimpah-peternak-hadapi-tantangan-harga-1781149160668_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Pertanian buka suara soal permainan harga ayam dan telur.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/11/08/ilustrasi-swasembada-pangan-1762593423685.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Pertanian Andi Amran Sulaiman meraih pengakuan tinggi dari enam lembaga independen. Program swasembada pangan sukses, meningkatkan kesejahteraan petani.</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8714771/dugaan-permainan-harga-ayam-dan-telur-mulai-terendus</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8716249/6-lembaga-tempatkan-mentan-amran-posisi-atas-di-dua-tahun-prabowo-gibran</t>
         </is>
       </c>
     </row>
@@ -1833,22 +1857,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Warga Karet Kuningan Olah Sampah Plastik Jadi BBM Alternatif</t>
+          <t>Suahasil Pastikan Penyaluran Gaji PNS Tak Lewat Koperasi</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Tue, 20 Oct 2026 06:00:13 +0700</t>
+          <t>Tue, 20 Oct 2026 19:33:10 +0700</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/19/warga-karet-kuningan-olah-sampah-plastik-jadi-bbm-alternatif-1-kg-hasilkan-09-liter-1792404845273_169.jpeg?w=360&amp;amp;q=90" /&gt; Warga Karet Kuningan, Jakarta Selatan, mengolah sampah plastik menjadi BBM alternatif bernama Petasol. </t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/20/menteri-keuangan-suahasil-nazara-1792487454171_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Keuangan Suahasil Nazara memastikan mekanisme gaji Aparatur Sipil Negara (ASN) tidak akan mengalami perubahan.</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/foto-bisnis/d-8714727/warga-karet-kuningan-olah-sampah-plastik-jadi-bbm-alternatif</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8716223/suahasil-pastikan-penyaluran-gaji-pns-tak-lewat-koperasi</t>
         </is>
       </c>
     </row>
@@ -1860,22 +1884,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Bakal Didepak Bursa dari Perhitungan IHSG, Ini Daftar 80 Saham HSC</t>
+          <t>Waspada Penipuan Digital, blu Hadirkan Podcast Cerita Camping di BIK</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Tue, 20 Oct 2026 05:55:00 +0700</t>
+          <t>Tue, 20 Oct 2026 19:27:46 +0700</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/19/ihsg-dibuka-anjlok-431-bei-berlakukan-arb-7-1792382663579_169.jpeg?w=360&amp;amp;q=90" /&gt; BEI tidak lagi memperhitungkan saham-saham dengan kepemilikan terkonsentrasi tinggi atau high shareholding concentration (HSC) dalam perhitunga</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/20/podcast-cerita-camping-1792498495627.png?w=360&amp;amp;q=90" /&gt; Blu by BCA Digital luncurkan podcast Cerita Camping untuk edukasi literasi keuangan digital. Dapatkan tips mengenali penipuan dan menjaga keamanan finansial.</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/bursa-dan-valas/d-8714769/bakal-didepak-bursa-dari-perhitungan-ihsg-ini-daftar-80-saham-hsc</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8716220/waspada-penipuan-digital-blu-hadirkan-podcast-cerita-camping-di-bik</t>
         </is>
       </c>
     </row>
@@ -1887,22 +1911,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Eks Menteri Kritik Singapura soal Karhutla: 4 dari 7 Perusahaan Tercatat di Sana!</t>
+          <t>OJK Periksa Saham-saham HSC!</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Tue, 20 Oct 2026 05:25:00 +0700</t>
+          <t>Tue, 20 Oct 2026 19:18:18 +0700</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/03/lahan-gambut-banjar-terbakar-petugas-berjibaku-jinakkan-api-1788405575337_169.jpeg?w=360&amp;amp;q=90" /&gt; Mantan Menteri Perdagangan Muhammad Lutfi mengkritik Singapura soal teguran ke 7 perusahaan yang dianggap bertanggung jawab ata</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/01/30/ihsg-rebound-usai-dua-hari-anjlok-seiring-pengunduran-diri-dirut-bei-1769748663323_169.jpeg?w=360&amp;amp;q=90" /&gt; OJK memeriksa saham-saham dengan tingkat konsentrasi kepemilikan tinggi atau High Shareholding Concentration (HSC) ter</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8714756/eks-menteri-kritik-singapura-soal-karhutla-4-dari-7-perusahaan-tercatat-di-sana</t>
+          <t>https://finance.detik.com/bursa-dan-valas/d-8716201/ojk-periksa-saham-saham-hsc</t>
         </is>
       </c>
     </row>
@@ -1914,22 +1938,22 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Bahlil Sebut Pabrik Baterai CATL di Karawang Segera Diresmikan</t>
+          <t>Bos OJK Ngaku Belum Istirahat Sejak MSCI Sebut Bursa RI Bisa Turun Kasta</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Mon, 19 Oct 2026 22:54:03 +0700</t>
+          <t>Tue, 20 Oct 2026 19:00:45 +0700</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/08/04/bahlil-lahadalia-1785840108228_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Koordinator Bidang Hilirisasi dan Transisi Energi Bahlil Lahadalia mengatakan pabrik baterai CATL di Karawang akan diresmikan dalam waktu dekat.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/20/ketua-dewan-komisioner-otoritas-jasa-keuangan-ojk-friderica-widyasari-dewi-1792489087006_169.jpeg?w=360&amp;amp;q=90" /&gt; Ketua Dewan Komisioner Otoritas Jasa Keuangan (OJK), Friderica Widyasari Dewi mengaku belum beristirahat sejak a</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8714738/bahlil-sebut-pabrik-baterai-catl-di-karawang-segera-diresmikan</t>
+          <t>https://finance.detik.com/bursa-dan-valas/d-8716117/bos-ojk-ngaku-belum-istirahat-sejak-msci-sebut-bursa-ri-bisa-turun-kasta</t>
         </is>
       </c>
     </row>
@@ -1941,22 +1965,22 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Wanti-wanti buat Pemerintah, Inflasi Pangan Bisa Melonjak ke 5%</t>
+          <t>Buyback Saham, BNI Jalankan Aksi Korporasi Terukur &amp;amp; Fundamental Tetap Kuat</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Mon, 19 Oct 2026 22:43:15 +0700</t>
+          <t>Tue, 20 Oct 2026 18:46:46 +0700</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/02/09/pedagang-bahan-pangan-di-pasar-lakessi-1770618996980_169.jpeg?w=360&amp;amp;q=90" /&gt; Gubernur Bank Indonesia (BI) Destry Damayanti mewanti-wanti soal inflasi pangan.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2023/09/16/gedung-bni.png?w=360&amp;amp;q=90" /&gt; PT BNI melanjutkan aksi korporasi melalui buyback saham hingga 26 Oktober 2026, dengan fokus pada pertumbuhan bisnis dan kepentingan pemegang saham.</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8714725/wanti-wanti-buat-pemerintah-inflasi-pangan-bisa-melonjak-ke-5</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8716160/buyback-saham-bni-jalankan-aksi-korporasi-terukur-fundamental-tetap-kuat</t>
         </is>
       </c>
     </row>
@@ -1968,22 +1992,22 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Tetap Ada Efisiensi, Belanja Kuartal IV Disiapkan Rp 1.300 Triliun</t>
+          <t>Bos OJK Buka Suara soal Singapura di Balik Ancaman Bursa RI Turun Kasta</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Mon, 19 Oct 2026 22:36:47 +0700</t>
+          <t>Tue, 20 Oct 2026 18:14:54 +0700</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/09/apbn-defisit-rp319-triliun-menkeu-sebut-masih-sesuai-target-1791525967190_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Keuangan (Menkeu) Suahasil Nazara buka suara soal belanja anggaran pemerintah, termasuk soal efisiensi.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/02/ketua-dewan-komisioner-ojk-friderica-widyasari-dewi-1790924890094_169.jpeg?w=360&amp;amp;q=90" /&gt; Perempuan yang akrab disapa Kiki ini menyatakan, sebagai regulator pihaknya akan fokus kerja.</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8714721/tetap-ada-efisiensi-belanja-kuartal-iv-disiapkan-rp-1-300-triliun</t>
+          <t>https://finance.detik.com/bursa-dan-valas/d-8716094/bos-ojk-buka-suara-soal-singapura-di-balik-ancaman-bursa-ri-turun-kasta</t>
         </is>
       </c>
     </row>
@@ -1995,22 +2019,22 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Suku Bunga Bank Sentral AS Diprediksi Naik, Bagaimana Nasib Rupiah?</t>
+          <t>Bos OJK Tepis Tudingan Beres-beres di Bursa Gegara Ancaman Turun Kasta</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Mon, 19 Oct 2026 22:23:40 +0700</t>
+          <t>Tue, 20 Oct 2026 17:59:02 +0700</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/07/08/rupiah-melemah-lagi-dolar-as-kembali-bertengger-di-rp18000-1783502390635_169.jpeg?w=360&amp;amp;q=90" /&gt; Gubernur Bank Indonesia (BI) Destry Damayanti memprediksi suku bunga bank sentral Amerika Serikat (AS) atau The Federal Reserve </t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/20/ketua-dewan-komisioner-otoritas-jasa-keuangan-ojk-friderica-widyasari-dewi-1792489086929_169.jpeg?w=360&amp;amp;q=90" /&gt; Ketua Dewan Komisioner OJK Friderica Widyasari Dewi menepis anggapan reformasi pasar modal Indonesia baru berjal</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/bursa-dan-valas/d-8714711/suku-bunga-bank-sentral-as-diprediksi-naik-bagaimana-nasib-rupiah</t>
+          <t>https://finance.detik.com/bursa-dan-valas/d-8716070/bos-ojk-tepis-tudingan-beres-beres-di-bursa-gegara-ancaman-turun-kasta</t>
         </is>
       </c>
     </row>
@@ -2022,22 +2046,22 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>IHSG Melorot ke Bawah 5.000, Danantara Mau Borong Saham BUMN</t>
+          <t>Kemarau Panjang Bikin Air Bendungan Menyusut, Kementerian PU Lakukan Ini</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Mon, 19 Oct 2026 22:13:04 +0700</t>
+          <t>Tue, 20 Oct 2026 17:01:07 +0700</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/03/11/rosan-roeslani-firda-cynthia-anggrainy-al-djokyadetikcom-1741681299971_169.jpeg?w=360&amp;amp;q=90" /&gt; CEO Danantara Rosan Roeslani menanggapi Indeks Harga Saham Gabungan (IHSG) yang turun hingga ke bawah level 5.000.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/02/07/wakil-menteri-pu-diana-kusumastuti-5_169.jpeg?w=360&amp;amp;q=90" /&gt; Kementerian Pekerjaan Umum (PU) menyiapkan sejumlah solusi, termasuk melalui operasi modifikasi cuaca dan pengaturan pola operasi waduk.</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/bursa-dan-valas/d-8714705/ihsg-melorot-ke-bawah-5-000-danantara-mau-borong-saham-bumn</t>
+          <t>https://finance.detik.com/infrastruktur/d-8715929/kemarau-panjang-bikin-air-bendungan-menyusut-kementerian-pu-lakukan-ini</t>
         </is>
       </c>
     </row>
@@ -2049,22 +2073,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Penyebab Listrik Batam Padam Diusut, Bos PLN Pastikan Bukan Sabotase</t>
+          <t>Pascapenjarahan, Toko-toko Mewah Prancis Dipasangi Pembatas</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Mon, 19 Oct 2026 21:54:44 +0700</t>
+          <t>Tue, 20 Oct 2026 16:52:56 +0700</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2023/01/01/pembangkit-listrik-pln-batam-foto-dok-pln_169.jpeg?w=360&amp;amp;q=90" /&gt; PLN sedang menyelidiki lebih dalam penyebab listrik padam di Batam, Kepulauan Riau, beberapa hari lalu.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/20/pascapenjarahan-toko-rolex-hingga-louis-vuitton-pancis-dipasangi-pembatas-1792473296412.jpeg?w=360&amp;amp;q=90" /&gt; Sejumlah toko mewah di Marseille dipasangi pembatas usai aksi penjarahan saat demonstrasi. Kerusuhan tersebut berakar</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8714688/penyebab-listrik-batam-padam-diusut-bos-pln-pastikan-bukan-sabotase</t>
+          <t>https://finance.detik.com/foto-bisnis/d-8715291/pascapenjarahan-toko-toko-mewah-prancis-dipasangi-pembatas</t>
         </is>
       </c>
     </row>
@@ -2076,22 +2100,22 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Dua Tahun Prabowo: Investasi Rp 3.923 Triliun, 5,4 Juta Tenaga Kerja Terserap</t>
+          <t>Bos OJK Ungkap Alasan Baru Beri Sanksi DSSA, BREN, dan CUAN</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Mon, 19 Oct 2026 21:40:16 +0700</t>
+          <t>Tue, 20 Oct 2026 16:44:27 +0700</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/08/06/presiden-prabowo-subianto-menggelar-sidang-kabinet-rabu-682025-1754475097038_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Investasi dan Hilirisasi/Kepala BKPM Rosan Roeslani mengatakan total investasi dalam 2 tahun capai Rp 3.923 triliun.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/20/ketua-dewan-komisioner-otoritas-jasa-keuangan-ojk-friderica-widyasari-dewi-1792489086929_169.jpeg?w=360&amp;amp;q=90" /&gt; Otoritas Jasa Keuangan (OJK) mengungkapkan alasan pengenaan sanksi administratif berupa denda dengan total Rp 2,</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8714675/dua-tahun-prabowo-investasi-rp-3-923-triliun-5-4-juta-tenaga-kerja-terserap</t>
+          <t>https://finance.detik.com/bursa-dan-valas/d-8715906/bos-ojk-ungkap-alasan-baru-beri-sanksi-dssa-bren-dan-cuan</t>
         </is>
       </c>
     </row>
@@ -2103,22 +2127,22 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>5 Besar Investor Asing di Indonesia, Singapura Masih Rajanya</t>
+          <t>IHSG Parkir di Level 5.278, Naik 5,65%</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Mon, 19 Oct 2026 21:25:48 +0700</t>
+          <t>Tue, 20 Oct 2026 16:39:06 +0700</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2023/03/28/ilustrasi-pertumbuhan-ekonomi_169.jpeg?w=360&amp;amp;q=90" /&gt; Realisasi investasi di Indonesia sepanjang Januari-September 2026 mencapai Rp 1.539,2 triliun atau 75,4% dari target. Singapura masih investor asing terbesar</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/16/ihsg-ambruk-1157-ditutup-di-level-5185-1792144638939_169.jpeg?w=360&amp;amp;q=90" /&gt; Indeks Harga Saham Gabungan (IHSG) mengalami perbaikan hari ini.</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8714667/5-besar-investor-asing-di-indonesia-singapura-masih-rajanya</t>
+          <t>https://finance.detik.com/bursa-dan-valas/d-8715889/ihsg-parkir-di-level-5-278-naik-5-65</t>
         </is>
       </c>
     </row>
@@ -2130,22 +2154,22 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Ada Demo di Jakarta Hari Ini, Cek Rekayasa Lalu Lintas dan Rute Alternatif</t>
+          <t>Demo di Tugu Tani Usai, Massa Sempat Bakar Flare</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Tue, 20 Oct 2026 07:36:03 +0700</t>
+          <t>Tue, 20 Oct 2026 20:15:36 +0700</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Aksi demo bagai digelar di sejumlah titik di wilayah Jakarta hari ini, Selasa (20/10/2026).</t>
+          <t>Massa bubar perlahan usai memasang spanduk berisi lima tuntutan kepada pemerintah.</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8316844/ada-demo-di-jakarta-hari-ini-cek-rekayasa-lalu-lintas-dan-rute-alternatif</t>
+          <t>https://www.liputan6.com/news/read/8317613/demo-di-tugu-tani-usai-massa-sempat-bakar-flare</t>
         </is>
       </c>
     </row>
@@ -2157,22 +2181,22 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Cegah Pelajar Demo ke Jakarta, Dindik Tangerang Keluarkan Surat Edaran</t>
+          <t>Kebakaran Hutan Arjuno-Ringgit Meluas, Api Mendekati Permukiman Warga</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Tue, 20 Oct 2026 07:04:02 +0700</t>
+          <t>Tue, 20 Oct 2026 20:03:39 +0700</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Dinas Pendidikan Kabupaten Tangerang mengeluarkan surat edaran mencegah siswa tak ikut aksi unjuk rasa dua tahun Prabowo di Jakarta.</t>
+          <t>Api dilaporkan merembet ke arah selatan menuju Kecamatan Singosari, Kabupaten Malang.</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8316834/cegah-pelajar-demo-ke-jakarta-dindik-tangerang-keluarkan-surat-edaran</t>
+          <t>https://www.liputan6.com/news/read/8317604/kebakaran-hutan-arjuno-ringgit-meluas-api-mendekati-permukiman-warga</t>
         </is>
       </c>
     </row>
@@ -2184,22 +2208,22 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Benih Lobster Rp 5,8 Miliar Gagal Diselundupkan ke Luar Negeri</t>
+          <t>Panjat Patung HI, 6 Aktivis Greenpeace Tunggu Kepastian Hukum</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Tue, 20 Oct 2026 06:55:06 +0700</t>
+          <t>Tue, 20 Oct 2026 19:44:09 +0700</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Penyelundupan benih lobster senilai Rp 5,8 miliar berhasil digagalkan. Tercium upaya pencucian uang dari hasil tindak pelanggaran ini.</t>
+          <t>Enam aktivis Greenpeace masih berada di Polda Metro Jaya. Tim advokasi mempertanyakan kejelasan status hukum mereka.</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8316833/benih-lobster-rp-58-miliar-gagal-diselundupkan-ke-luar-negeri</t>
+          <t>https://www.liputan6.com/news/read/8317582/panjat-patung-hi-6-aktivis-greenpeace-tunggu-kepastian-hukum</t>
         </is>
       </c>
     </row>
@@ -2211,22 +2235,22 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Siapa Perusahaan Dibidik Biang Kerok Karhutla</t>
+          <t>Ogah Dipalak, Siswa SMP di Sukabumi Dianiaya Kakak Kelas</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Tue, 20 Oct 2026 06:05:45 +0700</t>
+          <t>Tue, 20 Oct 2026 18:56:47 +0700</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Aparat kini membidik pertanggungjawaban korporasi, termasuk kemungkinan menelusuri pemilik perusahaan hingga pemegang saham</t>
+          <t>Korban mengalami cedera serius hingga kesulitan berjalan.</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8316812/siapa-perusahaan-dibidik-biang-kerok-karhutla</t>
+          <t>https://www.liputan6.com/news/read/8317557/ogah-dipalak-siswa-smp-di-sukabumi-dianiaya-kakak-kelas</t>
         </is>
       </c>
     </row>
@@ -2238,22 +2262,22 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Mengurai Fakta di Balik Kasus Polisi Tembak Polisi di Markas Polairud</t>
+          <t>Mahasiswa Pasang Spanduk Raksasa 5 Tuntutan di Monumen Tugu Tani</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Tue, 20 Oct 2026 05:00:05 +0700</t>
+          <t>Tue, 20 Oct 2026 18:40:57 +0700</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Bharatu Valdo tewas dalam insiden yang melibatkan Bharada Andika Rahmadani. Dugaan motif terkait persoalan pribadi.</t>
+          <t>Pembentangan spanduk dilakukan sekitar pukul 17.50 WIB.</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8316808/mengurai-fakta-di-balik-kasus-polisi-tembak-polisi-di-markas-polairud</t>
+          <t>https://www.liputan6.com/news/read/8317542/mahasiswa-pasang-spanduk-raksasa-5-tuntutan-di-monumen-tugu-tani</t>
         </is>
       </c>
     </row>
@@ -2265,22 +2289,22 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Subagyo HS, KSAD yang Pernah Mengabdi di Era Tiga Presiden</t>
+          <t>KPK Tetapkan 2 Tersangka Baru Kasus Suap Rejang Lebong</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Tue, 20 Oct 2026 00:00:49 +0700</t>
+          <t>Tue, 20 Oct 2026 18:34:09 +0700</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Subagyo HS merupakan perwira TNI lulusan Akabri Magelang tahun 1970.</t>
+          <t>Pengumuman tersangka baru itu setelah KPK memerika keduanya pada hari ini, Selasa (20/10/2026).</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8316777/subagyo-hs-ksad-yang-pernah-mengabdi-di-era-tiga-presiden</t>
+          <t>https://www.liputan6.com/news/read/8317535/kpk-tetapkan-2-tersangka-baru-kasus-suap-rejang-lebong</t>
         </is>
       </c>
     </row>
@@ -2292,22 +2316,22 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Wamenag Dorong Hukuman Maksimal Pelaku Kekerasan Seksual</t>
+          <t>Imigrasi Bidik Agen Perekrut WNI Jadi Tentara Bayaran Rusia</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Mon, 19 Oct 2026 23:58:49 +0700</t>
+          <t>Tue, 20 Oct 2026 18:21:29 +0700</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Kemenag telah membangun sistem penanganan kasus kekerasan di lingkungan pendidikan keagamaan.</t>
+          <t>Penegakan hukum disiapkan terhadap para perekrut dan agen yang terlibat dalam jaringan tersebut.</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8316795/wamenag-dorong-hukuman-maksimal-pelaku-kekerasan-seksual</t>
+          <t>https://www.liputan6.com/news/read/8317527/imigrasi-bidik-agen-perekrut-wni-jadi-tentara-bayaran-rusia</t>
         </is>
       </c>
     </row>
@@ -2319,22 +2343,22 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Catat, Ini Rute Alternatif Hindari Macet saat Demo di Jakarta Besok</t>
+          <t>Kejagung Kembalikan Rp 229,4 Miliar ke Korban KSP Indosurya</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Mon, 19 Oct 2026 23:54:26 +0700</t>
+          <t>Tue, 20 Oct 2026 18:09:27 +0700</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Pengguna jalan diharapkan menyesuaikan waktu keberangkatan, memanfaatkan rute alternatif, dan menghindari kawasan tersebut</t>
+          <t>Pengembalian tahap pertama ini dilakukan secara proporsional kepada para korban.</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8316794/catat-ini-rute-alternatif-hindari-macet-saat-demo-di-jakarta-besok</t>
+          <t>https://www.liputan6.com/news/read/8317508/kejagung-kembalikan-rp-2294-miliar-ke-korban-ksp-indosurya</t>
         </is>
       </c>
     </row>
@@ -2346,22 +2370,22 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Ketua Komisi III Wanti-wanti RUU Perampasan Aset: Rentan Jadi Bumerang</t>
+          <t>Prajurit TNI di Palangka Raya Aniaya Istri Usai Dipergoki Selingkuh</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Mon, 19 Oct 2026 23:00:16 +0700</t>
+          <t>Tue, 20 Oct 2026 17:33:45 +0700</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Habiburokhman mengingatkan RUU Perampasan Aset harus memiliki perlindungan hukum agar tidak disalahgunakan.</t>
+          <t>Dugaan penganiayaan itu viral di media sosial Threads pada Senin (19/10/2026).</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8316733/ketua-komisi-iii-wanti-wanti-ruu-perampasan-aset-rentan-jadi-bumerang</t>
+          <t>https://www.liputan6.com/news/read/8317471/prajurit-tni-di-palangka-raya-aniaya-istri-usai-dipergoki-selingkuh</t>
         </is>
       </c>
     </row>
@@ -2373,22 +2397,22 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Menag Soroti Kebakaran Hutan, Singgung Dosa Merusak Alam</t>
+          <t>Warga Bagikan Makanan Gratis untuk Mahasiswa Demo di Tugu Tani</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Mon, 19 Oct 2026 22:02:46 +0700</t>
+          <t>Tue, 20 Oct 2026 17:15:33 +0700</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Nasaruddin mengatakan, pendekatan ekoteologi dapat menjadi salah satu upaya untuk mendorong kepedulian masyarakat terhadap kelestarian lingkungan.</t>
+          <t>Warga terlihat membagikan roti dan minuman yang seluruhnya berasal dari sumbangan masyarakat.</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8316740/menag-soroti-kebakaran-hutan-singgung-dosa-merusak-alam</t>
+          <t>https://www.liputan6.com/news/read/8317452/warga-bagikan-makanan-gratis-untuk-mahasiswa-demo-di-tugu-tani</t>
         </is>
       </c>
     </row>
@@ -2400,22 +2424,22 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>PKS Ingatkan Kader Hati-Hati Bicara di Medsos</t>
+          <t>Alasan BEM UI Tak Pakai Almamater Saat Demo di Tugu Tani</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Mon, 19 Oct 2026 21:31:18 +0700</t>
+          <t>Tue, 20 Oct 2026 17:14:16 +0700</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>PKS berharap pejabat publik memiliki kesadaran bahwa cara menyampaikan pesan harus disesuaikan dengan perkembangan teknologi dan karakter ruang digital.</t>
+          <t>BEM UI mencoba pendekatan berbeda dalam aksi di Tugu Tani.</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8316737/pks-ingatkan-kader-hati-hati-bicara-di-medsos</t>
+          <t>https://www.liputan6.com/news/read/8317450/alasan-bem-ui-tak-pakai-almamater-saat-demo-di-tugu-tani</t>
         </is>
       </c>
     </row>
@@ -2427,22 +2451,22 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Mantan KSAD Subagyo HS Meninggal Dunia</t>
+          <t>BEM UI Ungkap Alasan Pilih Tugu Tani untuk Demo</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Mon, 19 Oct 2026 21:06:13 +0700</t>
+          <t>Tue, 20 Oct 2026 17:01:00 +0700</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Subagyo HS meninggal dunia di RS Panti Rapih, Yogyakarta, Senin (19/10/2026) sore.</t>
+          <t>Mahasiswa ingin menyuarakan tuntutan terkait karhutla dan ketimpangan sosial.</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8316722/mantan-ksad-subagyo-hs-meninggal-dunia</t>
+          <t>https://www.liputan6.com/news/read/8317401/bem-ui-ungkap-alasan-pilih-tugu-tani-untuk-demo</t>
         </is>
       </c>
     </row>
@@ -2454,22 +2478,22 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Prabowo Soroti Kinerja ASN-Polri</t>
+          <t>Detik-Detik Pajero Tabrak Siswa SMP di Jaksel hingga Tewas</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Mon, 19 Oct 2026 20:52:56 +0700</t>
+          <t>Tue, 20 Oct 2026 16:54:57 +0700</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Prabowo menyampaikan terkait pentingnya profesionalisme, integritas, dan kompetensi aparatur negara dalam penyelenggaraan pemerintahan.</t>
+          <t>Korban bahkan sempat bangun dan duduk sebelum dibawa ke rumah sakit. Namun, nyawanya tidak tertolong.</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8316715/prabowo-soroti-kinerja-asn-polri</t>
+          <t>https://www.liputan6.com/news/read/8317396/detik-detik-pajero-tabrak-siswa-smp-di-jaksel-hingga-tewas</t>
         </is>
       </c>
     </row>
@@ -2481,22 +2505,22 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Ini Hasil Tes Urine Sopir Pajero Tabrak Remaja hingga Tewas di Jaksel</t>
+          <t>Demo di Tugu Tani, BEM UI Bawa Lima Tuntutan</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Mon, 19 Oct 2026 20:14:42 +0700</t>
+          <t>Tue, 20 Oct 2026 16:21:38 +0700</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Hasil tes urine dilakukan kepolisian menunjukkan sopir negatif dari penyalahgunaan narkoba.</t>
+          <t>BEM UI menyatakan demo kali ini dirancang dengan pendekatan berbeda dari aksi-aksi sebelumnya.</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8316696/ini-hasil-tes-urine-sopir-pajero-tabrak-remaja-hingga-tewas-di-jaksel</t>
+          <t>https://www.liputan6.com/news/read/8317327/demo-di-tugu-tani-bem-ui-bawa-lima-tuntutan</t>
         </is>
       </c>
     </row>
@@ -2508,22 +2532,22 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Nadiem Makarim Ajukan Kasasi, Ini Permintaannya ke Hakim</t>
+          <t>Transformasi Kemenpora Dua Tahun Pemerintahan Prabowo-Gibran</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Mon, 19 Oct 2026 20:13:26 +0700</t>
+          <t>Tue, 20 Oct 2026 16:02:28 +0700</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Nadiem beberkan lima alasan Nadiem ajukan kasasi.</t>
+          <t>Salah satu terobosan fundamental adalah deregulasi 191 Peraturan Menteri Pemuda dan Olahraga menjadi empat Permenpora.</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8316695/nadiem-makarim-ajukan-kasasi-ini-permintaannya-ke-hakim</t>
+          <t>https://www.liputan6.com/news/read/8317288/transformasi-kemenpora-dua-tahun-pemerintahan-prabowo-gibran</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data pasar & berita - 2026-10-21 00:12 UTC
</commit_message>
<xml_diff>
--- a/data/market_news_latest.xlsx
+++ b/data/market_news_latest.xlsx
@@ -487,20 +487,20 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>5278.8882</v>
+        <v>4996.6089</v>
       </c>
       <c r="F2" t="n">
-        <v>282.2793</v>
+        <v>-188.4961</v>
       </c>
       <c r="G2" t="n">
-        <v>5.65</v>
+        <v>-3.64</v>
       </c>
       <c r="H2" t="n">
-        <v>0</v>
+        <v>279060000</v>
       </c>
     </row>
     <row r="3">
@@ -521,20 +521,20 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>7690.73</v>
+        <v>7712.5698</v>
       </c>
       <c r="F3" t="n">
-        <v>31.29</v>
+        <v>21.8398</v>
       </c>
       <c r="G3" t="n">
-        <v>0.41</v>
+        <v>0.28</v>
       </c>
       <c r="H3" t="n">
-        <v>4587260000</v>
+        <v>2721619000</v>
       </c>
     </row>
     <row r="4">
@@ -555,20 +555,20 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>51966.0312</v>
+        <v>52495.8789</v>
       </c>
       <c r="F4" t="n">
-        <v>-36.3789</v>
+        <v>529.8477</v>
       </c>
       <c r="G4" t="n">
-        <v>-0.07000000000000001</v>
+        <v>1.02</v>
       </c>
       <c r="H4" t="n">
-        <v>394060000</v>
+        <v>368648006</v>
       </c>
     </row>
     <row r="5">
@@ -589,20 +589,20 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>26430.8906</v>
+        <v>26424.8164</v>
       </c>
       <c r="F5" t="n">
-        <v>290.8613</v>
+        <v>-6.0742</v>
       </c>
       <c r="G5" t="n">
-        <v>1.11</v>
+        <v>-0.02</v>
       </c>
       <c r="H5" t="n">
-        <v>7537660000</v>
+        <v>6999145000</v>
       </c>
     </row>
     <row r="6">
@@ -623,20 +623,20 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>64075.4219</v>
+        <v>64916.6992</v>
       </c>
       <c r="F6" t="n">
-        <v>-841.2773</v>
+        <v>-407.5898</v>
       </c>
       <c r="G6" t="n">
-        <v>-1.3</v>
+        <v>-0.62</v>
       </c>
       <c r="H6" t="n">
-        <v>0</v>
+        <v>148000000</v>
       </c>
     </row>
     <row r="7">
@@ -657,20 +657,20 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>23867.7402</v>
+        <v>24186.8301</v>
       </c>
       <c r="F7" t="n">
-        <v>-319.0898</v>
+        <v>124.1094</v>
       </c>
       <c r="G7" t="n">
-        <v>-1.32</v>
+        <v>0.52</v>
       </c>
       <c r="H7" t="n">
-        <v>0</v>
+        <v>2773000000</v>
       </c>
     </row>
     <row r="8">
@@ -694,15 +694,9 @@
           <t>2026-10-20</t>
         </is>
       </c>
-      <c r="E8" t="n">
-        <v>3735.3704</v>
-      </c>
-      <c r="F8" t="n">
-        <v>4.4504</v>
-      </c>
-      <c r="G8" t="n">
-        <v>0.12</v>
-      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
       <c r="H8" t="n">
         <v>2214600536</v>
       </c>
@@ -725,20 +719,20 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>10684.6299</v>
+        <v>10764.7002</v>
       </c>
       <c r="F9" t="n">
-        <v>-80.0703</v>
+        <v>-117.2002</v>
       </c>
       <c r="G9" t="n">
-        <v>-0.74</v>
+        <v>-1.08</v>
       </c>
       <c r="H9" t="n">
-        <v>0</v>
+        <v>540130200</v>
       </c>
     </row>
     <row r="10">
@@ -759,20 +753,20 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>25122.25</v>
+        <v>25319.7695</v>
       </c>
       <c r="F10" t="n">
-        <v>-197.5195</v>
+        <v>-302.8398</v>
       </c>
       <c r="G10" t="n">
-        <v>-0.78</v>
+        <v>-1.18</v>
       </c>
       <c r="H10" t="n">
-        <v>0</v>
+        <v>45760800</v>
       </c>
     </row>
     <row r="11">
@@ -793,20 +787,20 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>5404.02</v>
+        <v>5412</v>
       </c>
       <c r="F11" t="n">
-        <v>-7.98</v>
+        <v>-3.5298</v>
       </c>
       <c r="G11" t="n">
-        <v>-0.15</v>
+        <v>-0.07000000000000001</v>
       </c>
       <c r="H11" t="n">
-        <v>0</v>
+        <v>265257200</v>
       </c>
     </row>
     <row r="12">
@@ -831,13 +825,13 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>17943</v>
+        <v>18041</v>
       </c>
       <c r="F12" t="n">
-        <v>-113</v>
+        <v>-15</v>
       </c>
       <c r="G12" t="n">
-        <v>-0.63</v>
+        <v>-0.08</v>
       </c>
       <c r="H12" t="n">
         <v>0</v>
@@ -865,13 +859,13 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>101.749</v>
+        <v>101.783</v>
       </c>
       <c r="F13" t="n">
-        <v>-0.231</v>
+        <v>-0.197</v>
       </c>
       <c r="G13" t="n">
-        <v>-0.23</v>
+        <v>-0.19</v>
       </c>
       <c r="H13" t="n">
         <v>0</v>
@@ -895,17 +889,17 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>157.996</v>
+        <v>158.328</v>
       </c>
       <c r="F14" t="n">
-        <v>0.19</v>
+        <v>-0.195</v>
       </c>
       <c r="G14" t="n">
-        <v>0.12</v>
+        <v>-0.12</v>
       </c>
       <c r="H14" t="n">
         <v>0</v>
@@ -933,13 +927,13 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>0.5109</v>
+        <v>0.5117</v>
       </c>
       <c r="F15" t="n">
-        <v>-0.0027</v>
+        <v>-0.0019</v>
       </c>
       <c r="G15" t="n">
-        <v>-0.53</v>
+        <v>-0.37</v>
       </c>
       <c r="H15" t="n">
         <v>0</v>
@@ -967,13 +961,13 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>0.543</v>
+        <v>0.5425</v>
       </c>
       <c r="F16" t="n">
-        <v>-0.0042</v>
+        <v>-0.0047</v>
       </c>
       <c r="G16" t="n">
-        <v>-0.77</v>
+        <v>-0.86</v>
       </c>
       <c r="H16" t="n">
         <v>0</v>
@@ -1001,13 +995,13 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>0.4085</v>
+        <v>0.408</v>
       </c>
       <c r="F17" t="n">
-        <v>0.001</v>
+        <v>0.0005</v>
       </c>
       <c r="G17" t="n">
-        <v>0.25</v>
+        <v>0.12</v>
       </c>
       <c r="H17" t="n">
         <v>0</v>
@@ -1031,20 +1025,14 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
-        </is>
-      </c>
-      <c r="E18" t="n">
-        <v>79.45999999999999</v>
-      </c>
-      <c r="F18" t="n">
-        <v>-0.59</v>
-      </c>
-      <c r="G18" t="n">
-        <v>-0.74</v>
-      </c>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
       <c r="H18" t="n">
-        <v>30956200</v>
+        <v>28348438</v>
       </c>
     </row>
     <row r="19">
@@ -1065,20 +1053,14 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
-        </is>
-      </c>
-      <c r="E19" t="n">
-        <v>76.83</v>
-      </c>
-      <c r="F19" t="n">
-        <v>-0.03</v>
-      </c>
-      <c r="G19" t="n">
-        <v>-0.04</v>
-      </c>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr"/>
       <c r="H19" t="n">
-        <v>31221800</v>
+        <v>42701539</v>
       </c>
     </row>
     <row r="20">
@@ -1103,16 +1085,16 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>4136.7998</v>
+        <v>4131.6001</v>
       </c>
       <c r="F20" t="n">
-        <v>-23.3003</v>
+        <v>-28.5</v>
       </c>
       <c r="G20" t="n">
-        <v>-0.5600000000000001</v>
+        <v>-0.6899999999999999</v>
       </c>
       <c r="H20" t="n">
-        <v>84848</v>
+        <v>5090</v>
       </c>
     </row>
     <row r="21">
@@ -1137,16 +1119,16 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>99.70999999999999</v>
+        <v>98.45</v>
       </c>
       <c r="F21" t="n">
-        <v>-3.95</v>
+        <v>-5.21</v>
       </c>
       <c r="G21" t="n">
-        <v>-3.81</v>
+        <v>-5.03</v>
       </c>
       <c r="H21" t="n">
-        <v>134576</v>
+        <v>3276</v>
       </c>
     </row>
     <row r="22">
@@ -1171,16 +1153,16 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>110.41</v>
+        <v>109.41</v>
       </c>
       <c r="F22" t="n">
-        <v>0.86</v>
+        <v>-0.14</v>
       </c>
       <c r="G22" t="n">
-        <v>0.79</v>
+        <v>-0.13</v>
       </c>
       <c r="H22" t="n">
-        <v>18835</v>
+        <v>315</v>
       </c>
     </row>
     <row r="23">
@@ -1205,16 +1187,16 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>6.579</v>
+        <v>6.609</v>
       </c>
       <c r="F23" t="n">
-        <v>0.041</v>
+        <v>0.07099999999999999</v>
       </c>
       <c r="G23" t="n">
-        <v>0.63</v>
+        <v>1.09</v>
       </c>
       <c r="H23" t="n">
-        <v>15266</v>
+        <v>501</v>
       </c>
     </row>
     <row r="24">
@@ -1235,20 +1217,14 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
-        </is>
-      </c>
-      <c r="E24" t="n">
-        <v>63.31</v>
-      </c>
-      <c r="F24" t="n">
-        <v>0.46</v>
-      </c>
-      <c r="G24" t="n">
-        <v>0.73</v>
-      </c>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr"/>
       <c r="H24" t="n">
-        <v>22118900</v>
+        <v>16515629</v>
       </c>
     </row>
     <row r="25">
@@ -1273,13 +1249,13 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>18.67</v>
+        <v>17.31</v>
       </c>
       <c r="F25" t="n">
-        <v>0.23</v>
+        <v>-1.13</v>
       </c>
       <c r="G25" t="n">
-        <v>1.25</v>
+        <v>-6.13</v>
       </c>
       <c r="H25" t="n">
         <v>0</v>
@@ -1303,20 +1279,20 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="E26" t="n">
-        <v>81304.39840000001</v>
+        <v>82918.42969999999</v>
       </c>
       <c r="F26" t="n">
-        <v>-549.1405999999999</v>
+        <v>1064.8906</v>
       </c>
       <c r="G26" t="n">
-        <v>-0.67</v>
+        <v>1.3</v>
       </c>
       <c r="H26" t="n">
-        <v>22612764672</v>
+        <v>26845833216</v>
       </c>
     </row>
     <row r="27">
@@ -1749,22 +1725,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Luhut Usul ke Prabowo Kerugian Negara Bukan Pidana Korupsi</t>
+          <t>Raksasa Keuangan Dunia Prediksi Ratusan Triliun Kabur Jika Bursa RI Turun Kasta</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Tue, 20 Oct 2026 20:14:23 +0700</t>
+          <t>Wed, 21 Oct 2026 06:25:00 +0700</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/06/09/luhut-hingga-chatib-basri-temui-prabowo-di-istana-1781007630172_169.jpeg?w=360&amp;amp;q=90" /&gt; Ketua Dewan Ekonomi Nasional (DEN) Luhut Binsar Pandjaitan mengusulkan kajian untuk mengubah definisi tindak pidana korupsi di Indonesia.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/16/ihsg-ambruk-1157-ditutup-di-level-5185-1792144639064_169.jpeg?w=360&amp;amp;q=90" /&gt; Raksasa institusi keuangan dunia memperkirakan pasar modal Indonesia bisa kehilangan aliran dana asing hingga ratusan triliun.</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8716297/luhut-usul-ke-prabowo-kerugian-negara-bukan-pidana-korupsi</t>
+          <t>https://finance.detik.com/bursa-dan-valas/d-8716442/raksasa-keuangan-dunia-prediksi-ratusan-triliun-kabur-jika-bursa-ri-turun-kasta</t>
         </is>
       </c>
     </row>
@@ -1776,22 +1752,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>MUI Tak Setuju Wajib Halal Diundur, Ini Alasannya</t>
+          <t>Kejar Pertumbuhan, Pemerintah Guyur Rp 1.300 T Genjot Belanja Akhir Tahun</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Tue, 20 Oct 2026 20:00:41 +0700</t>
+          <t>Wed, 21 Oct 2026 05:55:00 +0700</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/01/17/logo-halal-resmi-di-negara-asean-6_169.png?w=360&amp;amp;q=90" /&gt; Awalnya, kewajiban sertifikasi halal dijadwalkan mulai berlaku 18 Oktober 2026.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2015/12/17/00d5a8dc-da3d-483a-bd2e-e78ce08f1d66_169.jpg?w=360&amp;amp;q=90" /&gt; Menteri Keuangan Suahasil Nazara mengungkapkan pemerintah akan menggenjot belanja di akhir tahun untuk mempercepat pertumbuhan ekonomi.</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8716229/mui-tak-setuju-wajib-halal-diundur-ini-alasannya</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8716424/kejar-pertumbuhan-pemerintah-guyur-rp-1-300-t-genjot-belanja-akhir-tahun</t>
         </is>
       </c>
     </row>
@@ -1803,22 +1779,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Respons Bos BEI soal Isu Singapura di Balik IHSG Rontok Usai Pernyataan MSCI</t>
+          <t>180 Insulator di Jalur KRL Diganti, 513,926 Km Jaringan Listrik Atas Dirawat</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Tue, 20 Oct 2026 19:56:21 +0700</t>
+          <t>Tue, 20 Oct 2026 22:58:08 +0700</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/28/direktur-utama-bei-jeffrey-hendrik-1790588485860_169.jpeg?w=360&amp;amp;q=90" /&gt; Bursa Efek Indonesia (BEI) buka suara terkait dugaan intervensi Singapura di balik usulan MSCI menurunkan status bursa saham Indonesia ke standalone mar</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/20/perawatan-jaringan-listrik-krl-1792511606245_169.jpeg?w=360&amp;amp;q=90" /&gt; KAI melakukan perawatan jaringan listrik aliaran atas pada kereta rel listrik (KRL) berikut lokasi dan prosesnya.</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/bursa-dan-valas/d-8716255/respons-bos-bei-soal-isu-singapura-di-balik-ihsg-rontok-usai-pernyataan-msci</t>
+          <t>https://finance.detik.com/infrastruktur/d-8716475/180-insulator-di-jalur-krl-diganti-513-926-km-jaringan-listrik-atas-dirawat</t>
         </is>
       </c>
     </row>
@@ -1830,22 +1806,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>6 Lembaga Tempatkan Mentan Amran Posisi Atas di Dua Tahun Prabowo-Gibran</t>
+          <t>Nilai Ekspor Hilirisasi Mineral Diprediksi Tembus Rp 898 Triliun</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Tue, 20 Oct 2026 19:42:04 +0700</t>
+          <t>Tue, 20 Oct 2026 22:34:40 +0700</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/11/08/ilustrasi-swasembada-pangan-1762593423685.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Pertanian Andi Amran Sulaiman meraih pengakuan tinggi dari enam lembaga independen. Program swasembada pangan sukses, meningkatkan kesejahteraan petani.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/11/07/energi-bersih-dari-danau-toba-yang-menyalakan-industri-aluminium-nasional-1762530334223_169.jpeg?w=360&amp;amp;q=90" /&gt; Dewan Ekonomi Nasional (DEN) memprediksi ekspor hilirisasi mineral kritis dapat menyentuh US$ 50 miliar atau seki</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8716249/6-lembaga-tempatkan-mentan-amran-posisi-atas-di-dua-tahun-prabowo-gibran</t>
+          <t>https://finance.detik.com/energi/d-8716457/nilai-ekspor-hilirisasi-mineral-diprediksi-tembus-rp-898-triliun</t>
         </is>
       </c>
     </row>
@@ -1857,22 +1833,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Suahasil Pastikan Penyaluran Gaji PNS Tak Lewat Koperasi</t>
+          <t>Saran buat Pemerintah Usai MSCI Buka Opsi Bursa RI Turun Kasta</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Tue, 20 Oct 2026 19:33:10 +0700</t>
+          <t>Tue, 20 Oct 2026 22:11:55 +0700</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/20/menteri-keuangan-suahasil-nazara-1792487454171_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Keuangan Suahasil Nazara memastikan mekanisme gaji Aparatur Sipil Negara (ASN) tidak akan mengalami perubahan.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/05/18/ihsg-anjlok-ke-zona-merah-bursa-saham-melemah-tajam-1779098741437_169.jpeg?w=360&amp;amp;q=90" /&gt; Dewan Ekonomi Nasional ikut menyoroti masalah yang terjadi pada Bursa Efek Indonesia (BEI).</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8716223/suahasil-pastikan-penyaluran-gaji-pns-tak-lewat-koperasi</t>
+          <t>https://finance.detik.com/bursa-dan-valas/d-8716445/saran-buat-pemerintah-usai-msci-buka-opsi-bursa-ri-turun-kasta</t>
         </is>
       </c>
     </row>
@@ -1884,22 +1860,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Waspada Penipuan Digital, blu Hadirkan Podcast Cerita Camping di BIK</t>
+          <t>Serapan Gabah Bulog Jateng Tembus 108 Persen dari Target Tahunan</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Tue, 20 Oct 2026 19:27:46 +0700</t>
+          <t>Tue, 20 Oct 2026 21:55:30 +0700</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/20/podcast-cerita-camping-1792498495627.png?w=360&amp;amp;q=90" /&gt; Blu by BCA Digital luncurkan podcast Cerita Camping untuk edukasi literasi keuangan digital. Dapatkan tips mengenali penipuan dan menjaga keamanan finansial.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/20/realisasi-serapan-gabah-petani-di-jateng-1792470462877.jpeg?w=360&amp;amp;q=90" /&gt; Bulog Jawa Tengah mencatat serapan gabah petani mencapai 406.253 ton setara beras hingga Oktober 2026, atau 108,43% dari target tahunan.</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8716220/waspada-penipuan-digital-blu-hadirkan-podcast-cerita-camping-di-bik</t>
+          <t>https://finance.detik.com/foto-bisnis/d-8715178/serapan-gabah-bulog-jateng-tembus-108-persen-dari-target-tahunan</t>
         </is>
       </c>
     </row>
@@ -1911,22 +1887,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>OJK Periksa Saham-saham HSC!</t>
+          <t>Tak Lagi Barang, Bansos Bakal Lewat Transfer Uang Tunai</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Tue, 20 Oct 2026 19:18:18 +0700</t>
+          <t>Tue, 20 Oct 2026 21:30:19 +0700</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/01/30/ihsg-rebound-usai-dua-hari-anjlok-seiring-pengunduran-diri-dirut-bei-1769748663323_169.jpeg?w=360&amp;amp;q=90" /&gt; OJK memeriksa saham-saham dengan tingkat konsentrasi kepemilikan tinggi atau High Shareholding Concentration (HSC) ter</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2021/07/30/cara-cek-bansos-tunai-kemensos-simak-disini_169.jpeg?w=360&amp;amp;q=90" /&gt; Ketua Dewan Ekonomi Nasional (DEN) Luhut Binsar Pandjaitan menyatakan bantuan sosial (bansos) ke depannya tak lagi dalam bentuk barang</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/bursa-dan-valas/d-8716201/ojk-periksa-saham-saham-hsc</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8716403/tak-lagi-barang-bansos-bakal-lewat-transfer-uang-tunai</t>
         </is>
       </c>
     </row>
@@ -1938,22 +1914,22 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Bos OJK Ngaku Belum Istirahat Sejak MSCI Sebut Bursa RI Bisa Turun Kasta</t>
+          <t>Ungkap Kronologi, Bos ASDP Minta Maaf Insiden Kebakaran KMP Batumandi</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Tue, 20 Oct 2026 19:00:45 +0700</t>
+          <t>Tue, 20 Oct 2026 21:13:24 +0700</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/20/ketua-dewan-komisioner-otoritas-jasa-keuangan-ojk-friderica-widyasari-dewi-1792489087006_169.jpeg?w=360&amp;amp;q=90" /&gt; Ketua Dewan Komisioner Otoritas Jasa Keuangan (OJK), Friderica Widyasari Dewi mengaku belum beristirahat sejak a</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/20/proses-evakuasi-penumpang-kmp-batumandi-yang-terbakar-1792501886942_169.jpeg?w=360&amp;amp;q=90" /&gt; Direktur Utama ASDP Heru Widodo menyampaikan permohonan maaf atas insiden yang terjadi dan menegaskan keselamatan penumpang serta awa</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/bursa-dan-valas/d-8716117/bos-ojk-ngaku-belum-istirahat-sejak-msci-sebut-bursa-ri-bisa-turun-kasta</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8716386/ungkap-kronologi-bos-asdp-minta-maaf-insiden-kebakaran-kmp-batumandi</t>
         </is>
       </c>
     </row>
@@ -1965,22 +1941,22 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Buyback Saham, BNI Jalankan Aksi Korporasi Terukur &amp;amp; Fundamental Tetap Kuat</t>
+          <t>RI Mau Contoh Jepang &amp;amp; Italia Bikin MBG Prasmanan</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Tue, 20 Oct 2026 18:46:46 +0700</t>
+          <t>Tue, 20 Oct 2026 21:00:03 +0700</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2023/09/16/gedung-bni.png?w=360&amp;amp;q=90" /&gt; PT BNI melanjutkan aksi korporasi melalui buyback saham hingga 26 Oktober 2026, dengan fokus pada pertumbuhan bisnis dan kepentingan pemegang saham.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/20/penerima-manfaat-mbg-dalam-dua-tahun-pemerintahan-prabowo-1792479756787_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Koordinator Bidang Pangan Zulkifli Hasan buka-bukaan soal empat prioritas pembenahan program Makan Bergizi Gratis (MBG).</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8716160/buyback-saham-bni-jalankan-aksi-korporasi-terukur-fundamental-tetap-kuat</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8716171/ri-mau-contoh-jepang-italia-bikin-mbg-prasmanan</t>
         </is>
       </c>
     </row>
@@ -1992,22 +1968,22 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Bos OJK Buka Suara soal Singapura di Balik Ancaman Bursa RI Turun Kasta</t>
+          <t>2 Tahun Prabowo-Gibran, BULOG Luncurkan Kemasan Baru Beras SPHP</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Tue, 20 Oct 2026 18:14:54 +0700</t>
+          <t>Tue, 20 Oct 2026 20:30:23 +0700</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/02/ketua-dewan-komisioner-ojk-friderica-widyasari-dewi-1790924890094_169.jpeg?w=360&amp;amp;q=90" /&gt; Perempuan yang akrab disapa Kiki ini menyatakan, sebagai regulator pihaknya akan fokus kerja.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/20/2-tahun-prabowogibran-bulog-luncurkan-kemasan-baru-beras-sphp-1792502990466.jpeg?w=360&amp;amp;q=90" /&gt; Perum BULOG luncurkan kemasan baru 'Beras Kita Medium' untuk stabilisasi pangan. Inovasi ini dukung ketahanan pangan dan harga te</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/bursa-dan-valas/d-8716094/bos-ojk-buka-suara-soal-singapura-di-balik-ancaman-bursa-ri-turun-kasta</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8716335/2-tahun-prabowo-gibran-bulog-luncurkan-kemasan-baru-beras-sphp</t>
         </is>
       </c>
     </row>
@@ -2019,22 +1995,22 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Bos OJK Tepis Tudingan Beres-beres di Bursa Gegara Ancaman Turun Kasta</t>
+          <t>Luhut Usul ke Prabowo Kerugian Negara Bukan Pidana Korupsi</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Tue, 20 Oct 2026 17:59:02 +0700</t>
+          <t>Tue, 20 Oct 2026 20:14:23 +0700</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/20/ketua-dewan-komisioner-otoritas-jasa-keuangan-ojk-friderica-widyasari-dewi-1792489086929_169.jpeg?w=360&amp;amp;q=90" /&gt; Ketua Dewan Komisioner OJK Friderica Widyasari Dewi menepis anggapan reformasi pasar modal Indonesia baru berjal</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/06/09/luhut-hingga-chatib-basri-temui-prabowo-di-istana-1781007630172_169.jpeg?w=360&amp;amp;q=90" /&gt; Ketua Dewan Ekonomi Nasional (DEN) Luhut Binsar Pandjaitan mengusulkan kajian untuk mengubah definisi tindak pidana korupsi di Indonesia.</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/bursa-dan-valas/d-8716070/bos-ojk-tepis-tudingan-beres-beres-di-bursa-gegara-ancaman-turun-kasta</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8716297/luhut-usul-ke-prabowo-kerugian-negara-bukan-pidana-korupsi</t>
         </is>
       </c>
     </row>
@@ -2046,22 +2022,22 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Kemarau Panjang Bikin Air Bendungan Menyusut, Kementerian PU Lakukan Ini</t>
+          <t>MUI Tak Setuju Wajib Halal Diundur, Ini Alasannya</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Tue, 20 Oct 2026 17:01:07 +0700</t>
+          <t>Tue, 20 Oct 2026 20:00:41 +0700</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/02/07/wakil-menteri-pu-diana-kusumastuti-5_169.jpeg?w=360&amp;amp;q=90" /&gt; Kementerian Pekerjaan Umum (PU) menyiapkan sejumlah solusi, termasuk melalui operasi modifikasi cuaca dan pengaturan pola operasi waduk.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/01/17/logo-halal-resmi-di-negara-asean-6_169.png?w=360&amp;amp;q=90" /&gt; Awalnya, kewajiban sertifikasi halal dijadwalkan mulai berlaku 18 Oktober 2026.</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/infrastruktur/d-8715929/kemarau-panjang-bikin-air-bendungan-menyusut-kementerian-pu-lakukan-ini</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8716229/mui-tak-setuju-wajib-halal-diundur-ini-alasannya</t>
         </is>
       </c>
     </row>
@@ -2073,22 +2049,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Pascapenjarahan, Toko-toko Mewah Prancis Dipasangi Pembatas</t>
+          <t>Respons Bos BEI soal Isu Singapura di Balik IHSG Rontok Usai Pernyataan MSCI</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Tue, 20 Oct 2026 16:52:56 +0700</t>
+          <t>Tue, 20 Oct 2026 19:56:21 +0700</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/20/pascapenjarahan-toko-rolex-hingga-louis-vuitton-pancis-dipasangi-pembatas-1792473296412.jpeg?w=360&amp;amp;q=90" /&gt; Sejumlah toko mewah di Marseille dipasangi pembatas usai aksi penjarahan saat demonstrasi. Kerusuhan tersebut berakar</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/28/direktur-utama-bei-jeffrey-hendrik-1790588485860_169.jpeg?w=360&amp;amp;q=90" /&gt; Bursa Efek Indonesia (BEI) buka suara terkait dugaan intervensi Singapura di balik usulan MSCI menurunkan status bursa saham Indonesia ke standalone mar</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/foto-bisnis/d-8715291/pascapenjarahan-toko-toko-mewah-prancis-dipasangi-pembatas</t>
+          <t>https://finance.detik.com/bursa-dan-valas/d-8716255/respons-bos-bei-soal-isu-singapura-di-balik-ihsg-rontok-usai-pernyataan-msci</t>
         </is>
       </c>
     </row>
@@ -2100,22 +2076,22 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Bos OJK Ungkap Alasan Baru Beri Sanksi DSSA, BREN, dan CUAN</t>
+          <t>6 Lembaga Tempatkan Mentan Amran Posisi Atas di Dua Tahun Prabowo-Gibran</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Tue, 20 Oct 2026 16:44:27 +0700</t>
+          <t>Tue, 20 Oct 2026 19:42:04 +0700</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/20/ketua-dewan-komisioner-otoritas-jasa-keuangan-ojk-friderica-widyasari-dewi-1792489086929_169.jpeg?w=360&amp;amp;q=90" /&gt; Otoritas Jasa Keuangan (OJK) mengungkapkan alasan pengenaan sanksi administratif berupa denda dengan total Rp 2,</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/11/08/ilustrasi-swasembada-pangan-1762593423685.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Pertanian Andi Amran Sulaiman meraih pengakuan tinggi dari enam lembaga independen. Program swasembada pangan sukses, meningkatkan kesejahteraan petani.</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/bursa-dan-valas/d-8715906/bos-ojk-ungkap-alasan-baru-beri-sanksi-dssa-bren-dan-cuan</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8716249/6-lembaga-tempatkan-mentan-amran-posisi-atas-di-dua-tahun-prabowo-gibran</t>
         </is>
       </c>
     </row>
@@ -2127,22 +2103,22 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>IHSG Parkir di Level 5.278, Naik 5,65%</t>
+          <t>Suahasil Pastikan Penyaluran Gaji PNS Tak Lewat Koperasi</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Tue, 20 Oct 2026 16:39:06 +0700</t>
+          <t>Tue, 20 Oct 2026 19:33:10 +0700</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/16/ihsg-ambruk-1157-ditutup-di-level-5185-1792144638939_169.jpeg?w=360&amp;amp;q=90" /&gt; Indeks Harga Saham Gabungan (IHSG) mengalami perbaikan hari ini.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/20/menteri-keuangan-suahasil-nazara-1792487454171_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Keuangan Suahasil Nazara memastikan mekanisme gaji Aparatur Sipil Negara (ASN) tidak akan mengalami perubahan.</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/bursa-dan-valas/d-8715889/ihsg-parkir-di-level-5-278-naik-5-65</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8716223/suahasil-pastikan-penyaluran-gaji-pns-tak-lewat-koperasi</t>
         </is>
       </c>
     </row>
@@ -2154,22 +2130,22 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Demo di Tugu Tani Usai, Massa Sempat Bakar Flare</t>
+          <t>KPK Duga Ada Keterlibatan TNI Aktif di Kasus Korupsi Dana Bencana</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Tue, 20 Oct 2026 20:15:36 +0700</t>
+          <t>Wed, 21 Oct 2026 07:07:38 +0700</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Massa bubar perlahan usai memasang spanduk berisi lima tuntutan kepada pemerintah.</t>
+          <t>Apa yang lebih jahat dari korupsi dana bencana?</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8317613/demo-di-tugu-tani-usai-massa-sempat-bakar-flare</t>
+          <t>https://www.liputan6.com/news/read/8317763/kpk-duga-ada-keterlibatan-tni-aktif-di-kasus-korupsi-dana-bencana</t>
         </is>
       </c>
     </row>
@@ -2181,22 +2157,22 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Kebakaran Hutan Arjuno-Ringgit Meluas, Api Mendekati Permukiman Warga</t>
+          <t>Koperasi Pegawai Diduga Kelola Potongan Insentif di Pemkab Bogor</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Tue, 20 Oct 2026 20:03:39 +0700</t>
+          <t>Wed, 21 Oct 2026 06:25:01 +0700</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Api dilaporkan merembet ke arah selatan menuju Kecamatan Singosari, Kabupaten Malang.</t>
+          <t>KPK mendalami dugaan potongan insentif yang dikelola melalui koperasi pegawai Pemkab Bogor dan diduga mengalir kepada penyelenggara negara.</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8317604/kebakaran-hutan-arjuno-ringgit-meluas-api-mendekati-permukiman-warga</t>
+          <t>https://www.liputan6.com/news/read/8317754/koperasi-pegawai-diduga-kelola-potongan-insentif-di-pemkab-bogor</t>
         </is>
       </c>
     </row>
@@ -2208,22 +2184,22 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Panjat Patung HI, 6 Aktivis Greenpeace Tunggu Kepastian Hukum</t>
+          <t>Maruli Simanjuntak Minta Program Ekonomi Perbatasan Tak Berbelit</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Tue, 20 Oct 2026 19:44:09 +0700</t>
+          <t>Wed, 21 Oct 2026 06:07:31 +0700</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Enam aktivis Greenpeace masih berada di Polda Metro Jaya. Tim advokasi mempertanyakan kejelasan status hukum mereka.</t>
+          <t>BNPPDT memprioritaskan program ekonomi berbiaya terjangkau yang bisa segera dijalankan untuk masyarakat perbatasan dan daerah terpencil.</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8317582/panjat-patung-hi-6-aktivis-greenpeace-tunggu-kepastian-hukum</t>
+          <t>https://www.liputan6.com/news/read/8317751/maruli-simanjuntak-minta-program-ekonomi-perbatasan-tak-berbelit</t>
         </is>
       </c>
     </row>
@@ -2235,22 +2211,22 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Ogah Dipalak, Siswa SMP di Sukabumi Dianiaya Kakak Kelas</t>
+          <t>ASI: Kepercayaan ke Prabowo-Gibran 61,4 Persen, Kepuasan Beda Angka</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Tue, 20 Oct 2026 18:56:47 +0700</t>
+          <t>Wed, 21 Oct 2026 05:40:04 +0700</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Korban mengalami cedera serius hingga kesulitan berjalan.</t>
+          <t>Survei ASI mencatat kepercayaan terhadap pemerintahan Prabowo-Gibran sebesar 61,4 persen. Namun, kepuasan terhadap kinerja keduanya berbeda.</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8317557/ogah-dipalak-siswa-smp-di-sukabumi-dianiaya-kakak-kelas</t>
+          <t>https://www.liputan6.com/news/read/8317746/asi-kepercayaan-ke-prabowo-gibran-614-persen-kepuasan-beda-angka</t>
         </is>
       </c>
     </row>
@@ -2262,22 +2238,22 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Mahasiswa Pasang Spanduk Raksasa 5 Tuntutan di Monumen Tugu Tani</t>
+          <t>KPK Sita Rp 250 Juta dari PCNU Nias, Diduga Terkait Muktamar NU</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Tue, 20 Oct 2026 18:40:57 +0700</t>
+          <t>Wed, 21 Oct 2026 01:03:49 +0700</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Pembentangan spanduk dilakukan sekitar pukul 17.50 WIB.</t>
+          <t>KPK turut menelusuri keterkaitan uang tersebut dengan kasus korupsi di Kementerian ATR/BPN.</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8317542/mahasiswa-pasang-spanduk-raksasa-5-tuntutan-di-monumen-tugu-tani</t>
+          <t>https://www.liputan6.com/news/read/8317727/kpk-sita-rp-250-juta-dari-pcnu-nias-diduga-terkait-muktamar-nu</t>
         </is>
       </c>
     </row>
@@ -2289,22 +2265,22 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>KPK Tetapkan 2 Tersangka Baru Kasus Suap Rejang Lebong</t>
+          <t>Prabowo Terima DEN, Bahas Antisipasi El Nino hingga Kebakaran Hutan</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Tue, 20 Oct 2026 18:34:09 +0700</t>
+          <t>Wed, 21 Oct 2026 00:33:52 +0700</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Pengumuman tersangka baru itu setelah KPK memerika keduanya pada hari ini, Selasa (20/10/2026).</t>
+          <t>Dewan Ekonomi Nasional merekomendasikan sejumlah hal kepada pemerintah.</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8317535/kpk-tetapkan-2-tersangka-baru-kasus-suap-rejang-lebong</t>
+          <t>https://www.liputan6.com/news/read/8317713/prabowo-terima-den-bahas-antisipasi-el-nino-hingga-kebakaran-hutan</t>
         </is>
       </c>
     </row>
@@ -2316,22 +2292,22 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Imigrasi Bidik Agen Perekrut WNI Jadi Tentara Bayaran Rusia</t>
+          <t>KPK Sita Uang hingga Perhiasan di Rumah Dinas Bupati Klaten</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Tue, 20 Oct 2026 18:21:29 +0700</t>
+          <t>Wed, 21 Oct 2026 00:08:34 +0700</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Penegakan hukum disiapkan terhadap para perekrut dan agen yang terlibat dalam jaringan tersebut.</t>
+          <t>Penyidik akan menelaah seluruh barang yang telah disita untuk kepentingan penyidikan.</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8317527/imigrasi-bidik-agen-perekrut-wni-jadi-tentara-bayaran-rusia</t>
+          <t>https://www.liputan6.com/news/read/8317721/kpk-sita-uang-hingga-perhiasan-di-rumah-dinas-bupati-klaten</t>
         </is>
       </c>
     </row>
@@ -2343,22 +2319,22 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Kejagung Kembalikan Rp 229,4 Miliar ke Korban KSP Indosurya</t>
+          <t>Tak Hanya Aset Henry Surya, Kejagung Telusuri Peminjam Dana Indosurya</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Tue, 20 Oct 2026 18:09:27 +0700</t>
+          <t>Tue, 20 Oct 2026 23:32:55 +0700</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Pengembalian tahap pertama ini dilakukan secara proporsional kepada para korban.</t>
+          <t>Upaya tersebut dilakukan untuk mengoptimalkan pemulihan kerugian ribuan korban melalui perampasan dan pelelangan aset.</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8317508/kejagung-kembalikan-rp-2294-miliar-ke-korban-ksp-indosurya</t>
+          <t>https://www.liputan6.com/news/read/8317669/tak-hanya-aset-henry-surya-kejagung-telusuri-peminjam-dana-indosurya</t>
         </is>
       </c>
     </row>
@@ -2370,22 +2346,22 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Prajurit TNI di Palangka Raya Aniaya Istri Usai Dipergoki Selingkuh</t>
+          <t>6 Aktivis Greenpeace Dibebaskan Usai Diperiksa 8 Jam</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Tue, 20 Oct 2026 17:33:45 +0700</t>
+          <t>Tue, 20 Oct 2026 23:03:32 +0700</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Dugaan penganiayaan itu viral di media sosial Threads pada Senin (19/10/2026).</t>
+          <t>Para aktivis Greenpeace tersebut dibebaskan sekitar pukul 20.30 WIB.</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8317471/prajurit-tni-di-palangka-raya-aniaya-istri-usai-dipergoki-selingkuh</t>
+          <t>https://www.liputan6.com/news/read/8317698/6-aktivis-greenpeace-dibebaskan-usai-diperiksa-8-jam</t>
         </is>
       </c>
     </row>
@@ -2397,22 +2373,22 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Warga Bagikan Makanan Gratis untuk Mahasiswa Demo di Tugu Tani</t>
+          <t>Pemerintah Respons Aksi Greenpeace soal Krisis Iklim dan Biaya Hidup</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Tue, 20 Oct 2026 17:15:33 +0700</t>
+          <t>Tue, 20 Oct 2026 22:12:37 +0700</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Warga terlihat membagikan roti dan minuman yang seluruhnya berasal dari sumbangan masyarakat.</t>
+          <t>Greenpeace membentangkan spanduk kritik di kawasan Bundaran Hotel Indonesia (HI), Jakarta.</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8317452/warga-bagikan-makanan-gratis-untuk-mahasiswa-demo-di-tugu-tani</t>
+          <t>https://www.liputan6.com/news/read/8317664/pemerintah-respons-aksi-greenpeace-soal-krisis-iklim-dan-biaya-hidup</t>
         </is>
       </c>
     </row>
@@ -2424,22 +2400,22 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Alasan BEM UI Tak Pakai Almamater Saat Demo di Tugu Tani</t>
+          <t>DEN: 95 Persen Siswa Lebih Semangat Belajar Jika MBG Berkualitas</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Tue, 20 Oct 2026 17:14:16 +0700</t>
+          <t>Tue, 20 Oct 2026 21:27:47 +0700</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>BEM UI mencoba pendekatan berbeda dalam aksi di Tugu Tani.</t>
+          <t>Presiden Prabowo menerima rekomendasi DEN untuk meningkatkan perhatian terhadap kualitas menu MBG.</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8317450/alasan-bem-ui-tak-pakai-almamater-saat-demo-di-tugu-tani</t>
+          <t>https://www.liputan6.com/news/read/8317655/den-95-persen-siswa-lebih-semangat-belajar-jika-mbg-berkualitas</t>
         </is>
       </c>
     </row>
@@ -2451,22 +2427,22 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>BEM UI Ungkap Alasan Pilih Tugu Tani untuk Demo</t>
+          <t>Perjalanan 6 Tahun Korban KSP Indosurya Tagih Ganti Rugi</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Tue, 20 Oct 2026 17:01:00 +0700</t>
+          <t>Tue, 20 Oct 2026 21:08:29 +0700</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Mahasiswa ingin menyuarakan tuntutan terkait karhutla dan ketimpangan sosial.</t>
+          <t>Pengembalian dana tahap pertama kasus KSP Indosurya menjadi titik terang setelah bertahun-tahun menanti.</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8317401/bem-ui-ungkap-alasan-pilih-tugu-tani-untuk-demo</t>
+          <t>https://www.liputan6.com/news/read/8317643/perjalanan-6-tahun-korban-ksp-indosurya-tagih-ganti-rugi</t>
         </is>
       </c>
     </row>
@@ -2478,22 +2454,22 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Detik-Detik Pajero Tabrak Siswa SMP di Jaksel hingga Tewas</t>
+          <t>Mekanisme Penyaluran Rp 229,4 Miliar Ganti Rugi Korban Indosurya</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Tue, 20 Oct 2026 16:54:57 +0700</t>
+          <t>Tue, 20 Oct 2026 20:43:30 +0700</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Korban bahkan sempat bangun dan duduk sebelum dibawa ke rumah sakit. Namun, nyawanya tidak tertolong.</t>
+          <t>Penyaluran tahap pertama ini merupakan bagian dari pelaksanaan putusan terhadap terpidana Henry Surya dengan total dana sebesar Rp 229,4 miliar.</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8317396/detik-detik-pajero-tabrak-siswa-smp-di-jaksel-hingga-tewas</t>
+          <t>https://www.liputan6.com/news/read/8317623/mekanisme-penyaluran-rp-2294-miliar-ganti-rugi-korban-indosurya</t>
         </is>
       </c>
     </row>
@@ -2505,22 +2481,22 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Demo di Tugu Tani, BEM UI Bawa Lima Tuntutan</t>
+          <t>Demo di Tugu Tani Usai, Massa Sempat Bakar Flare</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Tue, 20 Oct 2026 16:21:38 +0700</t>
+          <t>Tue, 20 Oct 2026 20:15:36 +0700</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>BEM UI menyatakan demo kali ini dirancang dengan pendekatan berbeda dari aksi-aksi sebelumnya.</t>
+          <t>Massa bubar perlahan usai memasang spanduk berisi lima tuntutan kepada pemerintah.</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8317327/demo-di-tugu-tani-bem-ui-bawa-lima-tuntutan</t>
+          <t>https://www.liputan6.com/news/read/8317613/demo-di-tugu-tani-usai-massa-sempat-bakar-flare</t>
         </is>
       </c>
     </row>
@@ -2532,22 +2508,22 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Transformasi Kemenpora Dua Tahun Pemerintahan Prabowo-Gibran</t>
+          <t>Kebakaran Hutan Arjuno-Ringgit Meluas, Api Mendekati Permukiman Warga</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Tue, 20 Oct 2026 16:02:28 +0700</t>
+          <t>Tue, 20 Oct 2026 20:03:39 +0700</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Salah satu terobosan fundamental adalah deregulasi 191 Peraturan Menteri Pemuda dan Olahraga menjadi empat Permenpora.</t>
+          <t>Api dilaporkan merembet ke arah selatan menuju Kecamatan Singosari, Kabupaten Malang.</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8317288/transformasi-kemenpora-dua-tahun-pemerintahan-prabowo-gibran</t>
+          <t>https://www.liputan6.com/news/read/8317604/kebakaran-hutan-arjuno-ringgit-meluas-api-mendekati-permukiman-warga</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data pasar & berita - 2026-10-21 13:37 UTC
</commit_message>
<xml_diff>
--- a/data/market_news_latest.xlsx
+++ b/data/market_news_latest.xlsx
@@ -487,20 +487,20 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>4996.6089</v>
+        <v>5328.3599</v>
       </c>
       <c r="F2" t="n">
-        <v>-188.4961</v>
+        <v>49.4717</v>
       </c>
       <c r="G2" t="n">
-        <v>-3.64</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="H2" t="n">
-        <v>279060000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -521,20 +521,20 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>7712.5698</v>
+        <v>7727.0698</v>
       </c>
       <c r="F3" t="n">
-        <v>21.8398</v>
+        <v>14.5</v>
       </c>
       <c r="G3" t="n">
-        <v>0.28</v>
+        <v>0.19</v>
       </c>
       <c r="H3" t="n">
-        <v>2721619000</v>
+        <v>180674661</v>
       </c>
     </row>
     <row r="4">
@@ -555,20 +555,20 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>52495.8789</v>
+        <v>52503.5117</v>
       </c>
       <c r="F4" t="n">
-        <v>529.8477</v>
+        <v>7.6328</v>
       </c>
       <c r="G4" t="n">
-        <v>1.02</v>
+        <v>0.01</v>
       </c>
       <c r="H4" t="n">
-        <v>368648006</v>
+        <v>28472368</v>
       </c>
     </row>
     <row r="5">
@@ -589,20 +589,20 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>26424.8164</v>
+        <v>26548.4805</v>
       </c>
       <c r="F5" t="n">
-        <v>-6.0742</v>
+        <v>123.6602</v>
       </c>
       <c r="G5" t="n">
-        <v>-0.02</v>
+        <v>0.47</v>
       </c>
       <c r="H5" t="n">
-        <v>6999145000</v>
+        <v>1182947000</v>
       </c>
     </row>
     <row r="6">
@@ -623,20 +623,20 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>64916.6992</v>
+        <v>64621.2383</v>
       </c>
       <c r="F6" t="n">
-        <v>-407.5898</v>
+        <v>545.8164</v>
       </c>
       <c r="G6" t="n">
-        <v>-0.62</v>
+        <v>0.85</v>
       </c>
       <c r="H6" t="n">
-        <v>148000000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -657,20 +657,20 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>24186.8301</v>
+        <v>23651.8691</v>
       </c>
       <c r="F7" t="n">
-        <v>124.1094</v>
+        <v>-215.8711</v>
       </c>
       <c r="G7" t="n">
-        <v>0.52</v>
+        <v>-0.9</v>
       </c>
       <c r="H7" t="n">
-        <v>2773000000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -691,14 +691,20 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>3713.0276</v>
+      </c>
+      <c r="F8" t="n">
+        <v>-22.3425</v>
+      </c>
+      <c r="G8" t="n">
+        <v>-0.6</v>
+      </c>
       <c r="H8" t="n">
-        <v>2214600536</v>
+        <v>3468900532</v>
       </c>
     </row>
     <row r="9">
@@ -719,20 +725,20 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>10764.7002</v>
+        <v>10770.4902</v>
       </c>
       <c r="F9" t="n">
-        <v>-117.2002</v>
+        <v>37.4902</v>
       </c>
       <c r="G9" t="n">
-        <v>-1.08</v>
+        <v>0.35</v>
       </c>
       <c r="H9" t="n">
-        <v>540130200</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -753,20 +759,20 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>25319.7695</v>
+        <v>25660.8906</v>
       </c>
       <c r="F10" t="n">
-        <v>-302.8398</v>
+        <v>356.4707</v>
       </c>
       <c r="G10" t="n">
-        <v>-1.18</v>
+        <v>1.41</v>
       </c>
       <c r="H10" t="n">
-        <v>45760800</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -787,20 +793,20 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>5412</v>
+        <v>5437.9902</v>
       </c>
       <c r="F11" t="n">
-        <v>-3.5298</v>
+        <v>33.9702</v>
       </c>
       <c r="G11" t="n">
-        <v>-0.07000000000000001</v>
+        <v>0.63</v>
       </c>
       <c r="H11" t="n">
-        <v>265257200</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -821,17 +827,17 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>18041</v>
+        <v>17943</v>
       </c>
       <c r="F12" t="n">
-        <v>-15</v>
+        <v>-98</v>
       </c>
       <c r="G12" t="n">
-        <v>-0.08</v>
+        <v>-0.54</v>
       </c>
       <c r="H12" t="n">
         <v>0</v>
@@ -855,17 +861,17 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>101.783</v>
+        <v>101.685</v>
       </c>
       <c r="F13" t="n">
-        <v>-0.197</v>
+        <v>-0.045</v>
       </c>
       <c r="G13" t="n">
-        <v>-0.19</v>
+        <v>-0.04</v>
       </c>
       <c r="H13" t="n">
         <v>0</v>
@@ -893,13 +899,13 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>158.328</v>
+        <v>157.983</v>
       </c>
       <c r="F14" t="n">
-        <v>-0.195</v>
+        <v>-0.54</v>
       </c>
       <c r="G14" t="n">
-        <v>-0.12</v>
+        <v>-0.34</v>
       </c>
       <c r="H14" t="n">
         <v>0</v>
@@ -923,17 +929,17 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>0.5117</v>
+        <v>0.5094</v>
       </c>
       <c r="F15" t="n">
-        <v>-0.0019</v>
+        <v>-0.0023</v>
       </c>
       <c r="G15" t="n">
-        <v>-0.37</v>
+        <v>-0.45</v>
       </c>
       <c r="H15" t="n">
         <v>0</v>
@@ -957,17 +963,17 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>0.5425</v>
+        <v>0.5406</v>
       </c>
       <c r="F16" t="n">
-        <v>-0.0047</v>
+        <v>-0.0019</v>
       </c>
       <c r="G16" t="n">
-        <v>-0.86</v>
+        <v>-0.35</v>
       </c>
       <c r="H16" t="n">
         <v>0</v>
@@ -991,17 +997,17 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>0.408</v>
+        <v>0.407</v>
       </c>
       <c r="F17" t="n">
-        <v>0.0005</v>
+        <v>-0.001</v>
       </c>
       <c r="G17" t="n">
-        <v>0.12</v>
+        <v>-0.25</v>
       </c>
       <c r="H17" t="n">
         <v>0</v>
@@ -1025,14 +1031,20 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>80.34</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0.26</v>
+      </c>
       <c r="H18" t="n">
-        <v>28348438</v>
+        <v>1976433</v>
       </c>
     </row>
     <row r="19">
@@ -1053,14 +1065,20 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>76.95999999999999</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0.17</v>
+      </c>
       <c r="H19" t="n">
-        <v>42701539</v>
+        <v>1743667</v>
       </c>
     </row>
     <row r="20">
@@ -1081,20 +1099,20 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>4131.6001</v>
+        <v>4155.7002</v>
       </c>
       <c r="F20" t="n">
-        <v>-28.5</v>
+        <v>13.1001</v>
       </c>
       <c r="G20" t="n">
-        <v>-0.6899999999999999</v>
+        <v>0.32</v>
       </c>
       <c r="H20" t="n">
-        <v>5090</v>
+        <v>77851</v>
       </c>
     </row>
     <row r="21">
@@ -1115,20 +1133,20 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>98.45</v>
+        <v>97.28</v>
       </c>
       <c r="F21" t="n">
-        <v>-5.21</v>
+        <v>-4.51</v>
       </c>
       <c r="G21" t="n">
-        <v>-5.03</v>
+        <v>-4.43</v>
       </c>
       <c r="H21" t="n">
-        <v>3276</v>
+        <v>128159</v>
       </c>
     </row>
     <row r="22">
@@ -1149,20 +1167,20 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="E22" t="n">
-        <v>109.41</v>
+        <v>108.29</v>
       </c>
       <c r="F22" t="n">
-        <v>-0.14</v>
+        <v>-0.5</v>
       </c>
       <c r="G22" t="n">
-        <v>-0.13</v>
+        <v>-0.46</v>
       </c>
       <c r="H22" t="n">
-        <v>315</v>
+        <v>16896</v>
       </c>
     </row>
     <row r="23">
@@ -1183,20 +1201,20 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="E23" t="n">
-        <v>6.609</v>
+        <v>6.553</v>
       </c>
       <c r="F23" t="n">
-        <v>0.07099999999999999</v>
+        <v>-0.0135</v>
       </c>
       <c r="G23" t="n">
-        <v>1.09</v>
+        <v>-0.21</v>
       </c>
       <c r="H23" t="n">
-        <v>501</v>
+        <v>21092</v>
       </c>
     </row>
     <row r="24">
@@ -1217,14 +1235,20 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr"/>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr"/>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>63.565</v>
+      </c>
+      <c r="F24" t="n">
+        <v>0.245</v>
+      </c>
+      <c r="G24" t="n">
+        <v>0.39</v>
+      </c>
       <c r="H24" t="n">
-        <v>16515629</v>
+        <v>546239</v>
       </c>
     </row>
     <row r="25">
@@ -1245,17 +1269,17 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="E25" t="n">
-        <v>17.31</v>
+        <v>16.96</v>
       </c>
       <c r="F25" t="n">
-        <v>-1.13</v>
+        <v>-0.35</v>
       </c>
       <c r="G25" t="n">
-        <v>-6.13</v>
+        <v>-2.02</v>
       </c>
       <c r="H25" t="n">
         <v>0</v>
@@ -1283,16 +1307,16 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>82918.42969999999</v>
+        <v>83250.77340000001</v>
       </c>
       <c r="F26" t="n">
-        <v>1064.8906</v>
+        <v>309.7734</v>
       </c>
       <c r="G26" t="n">
-        <v>1.3</v>
+        <v>0.37</v>
       </c>
       <c r="H26" t="n">
-        <v>26845833216</v>
+        <v>26857611264</v>
       </c>
     </row>
     <row r="27">
@@ -1313,20 +1337,20 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="E27" t="n">
-        <v>1435</v>
+        <v>1485</v>
       </c>
       <c r="F27" t="n">
-        <v>240</v>
+        <v>50</v>
       </c>
       <c r="G27" t="n">
-        <v>20.08</v>
+        <v>3.48</v>
       </c>
       <c r="H27" t="n">
-        <v>232157200</v>
+        <v>171835800</v>
       </c>
     </row>
     <row r="28">
@@ -1347,20 +1371,20 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="E28" t="n">
-        <v>1275</v>
+        <v>1340</v>
       </c>
       <c r="F28" t="n">
-        <v>150</v>
+        <v>65</v>
       </c>
       <c r="G28" t="n">
-        <v>13.33</v>
+        <v>5.1</v>
       </c>
       <c r="H28" t="n">
-        <v>436758300</v>
+        <v>234603700</v>
       </c>
     </row>
     <row r="29">
@@ -1381,7 +1405,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="E29" t="n">
@@ -1394,7 +1418,7 @@
         <v>0</v>
       </c>
       <c r="H29" t="n">
-        <v>1225572700</v>
+        <v>453295000</v>
       </c>
     </row>
     <row r="30">
@@ -1415,20 +1439,20 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="E30" t="n">
-        <v>2000</v>
+        <v>2160</v>
       </c>
       <c r="F30" t="n">
-        <v>165</v>
+        <v>160</v>
       </c>
       <c r="G30" t="n">
-        <v>8.99</v>
+        <v>8</v>
       </c>
       <c r="H30" t="n">
-        <v>36611300</v>
+        <v>54437200</v>
       </c>
     </row>
     <row r="31">
@@ -1449,20 +1473,20 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="E31" t="n">
-        <v>3150</v>
+        <v>3060</v>
       </c>
       <c r="F31" t="n">
-        <v>40</v>
+        <v>-90</v>
       </c>
       <c r="G31" t="n">
-        <v>1.29</v>
+        <v>-2.86</v>
       </c>
       <c r="H31" t="n">
-        <v>199842000</v>
+        <v>70704200</v>
       </c>
     </row>
     <row r="32">
@@ -1483,20 +1507,20 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="E32" t="n">
-        <v>426</v>
+        <v>420</v>
       </c>
       <c r="F32" t="n">
-        <v>50</v>
+        <v>-6</v>
       </c>
       <c r="G32" t="n">
-        <v>13.3</v>
+        <v>-1.41</v>
       </c>
       <c r="H32" t="n">
-        <v>116844400</v>
+        <v>46513200</v>
       </c>
     </row>
     <row r="33">
@@ -1517,20 +1541,20 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="E33" t="n">
-        <v>484</v>
+        <v>470</v>
       </c>
       <c r="F33" t="n">
-        <v>28</v>
+        <v>-14</v>
       </c>
       <c r="G33" t="n">
-        <v>6.14</v>
+        <v>-2.89</v>
       </c>
       <c r="H33" t="n">
-        <v>168412600</v>
+        <v>86486800</v>
       </c>
     </row>
     <row r="34">
@@ -1551,20 +1575,20 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="E34" t="n">
-        <v>2670</v>
+        <v>2490</v>
       </c>
       <c r="F34" t="n">
-        <v>-90</v>
+        <v>-180</v>
       </c>
       <c r="G34" t="n">
-        <v>-3.26</v>
+        <v>-6.74</v>
       </c>
       <c r="H34" t="n">
-        <v>19202000</v>
+        <v>12531700</v>
       </c>
     </row>
     <row r="35">
@@ -1585,20 +1609,20 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="E35" t="n">
-        <v>346</v>
+        <v>322</v>
       </c>
       <c r="F35" t="n">
-        <v>-26</v>
+        <v>-24</v>
       </c>
       <c r="G35" t="n">
-        <v>-6.99</v>
+        <v>-6.94</v>
       </c>
       <c r="H35" t="n">
-        <v>21358700</v>
+        <v>539236300</v>
       </c>
     </row>
     <row r="36">
@@ -1619,20 +1643,20 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="E36" t="n">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="F36" t="n">
-        <v>-1</v>
+        <v>-2</v>
       </c>
       <c r="G36" t="n">
-        <v>-0.68</v>
+        <v>-1.37</v>
       </c>
       <c r="H36" t="n">
-        <v>38082800</v>
+        <v>19569300</v>
       </c>
     </row>
     <row r="37">
@@ -1653,20 +1677,20 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="E37" t="n">
-        <v>10375</v>
+        <v>9650</v>
       </c>
       <c r="F37" t="n">
-        <v>-775</v>
+        <v>-725</v>
       </c>
       <c r="G37" t="n">
-        <v>-6.95</v>
+        <v>-6.99</v>
       </c>
       <c r="H37" t="n">
-        <v>1053100</v>
+        <v>60687900</v>
       </c>
     </row>
   </sheetData>
@@ -1725,22 +1749,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Raksasa Keuangan Dunia Prediksi Ratusan Triliun Kabur Jika Bursa RI Turun Kasta</t>
+          <t>Bocoran Penetapan &amp;amp; Formula UMP 2027</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Wed, 21 Oct 2026 06:25:00 +0700</t>
+          <t>Wed, 21 Oct 2026 20:05:42 +0700</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/16/ihsg-ambruk-1157-ditutup-di-level-5185-1792144639064_169.jpeg?w=360&amp;amp;q=90" /&gt; Raksasa institusi keuangan dunia memperkirakan pasar modal Indonesia bisa kehilangan aliran dana asing hingga ratusan triliun.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/01/12/ilustrasi-rupiah-atau-upah-minimum-provinsi-ump-1768195061169_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Ketenagakerjaan (Menaker) Yassierli buka suara penetapan Upah Minimum Provinsi (UMP) 2027.</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/bursa-dan-valas/d-8716442/raksasa-keuangan-dunia-prediksi-ratusan-triliun-kabur-jika-bursa-ri-turun-kasta</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8717972/bocoran-penetapan-formula-ump-2027</t>
         </is>
       </c>
     </row>
@@ -1752,22 +1776,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Kejar Pertumbuhan, Pemerintah Guyur Rp 1.300 T Genjot Belanja Akhir Tahun</t>
+          <t>Soal Gaji PNS Lewat Kopdes Merah Putih, Menkop Ajak Menkeu Duduk Bareng</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Wed, 21 Oct 2026 05:55:00 +0700</t>
+          <t>Wed, 21 Oct 2026 19:54:39 +0700</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2015/12/17/00d5a8dc-da3d-483a-bd2e-e78ce08f1d66_169.jpg?w=360&amp;amp;q=90" /&gt; Menteri Keuangan Suahasil Nazara mengungkapkan pemerintah akan menggenjot belanja di akhir tahun untuk mempercepat pertumbuhan ekonomi.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/03/10/menteri-koperasi-menkop-ferry-juliantono-1773150156348_169.jpeg?w=360&amp;amp;q=90" /&gt; Menkop Ferry Juliantono menyampaikan pembayaran gaji PNS hingga pensiunan melalui Kopdes Merah Putih akan dibahas dengan Menteri Keuangan Suahasil</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8716424/kejar-pertumbuhan-pemerintah-guyur-rp-1-300-t-genjot-belanja-akhir-tahun</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8717963/soal-gaji-pns-lewat-kopdes-merah-putih-menkop-ajak-menkeu-duduk-bareng</t>
         </is>
       </c>
     </row>
@@ -1779,22 +1803,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>180 Insulator di Jalur KRL Diganti, 513,926 Km Jaringan Listrik Atas Dirawat</t>
+          <t>Respons Bos OJK Usai Prabowo Pidato RI Tidak Takut MSCI</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Tue, 20 Oct 2026 22:58:08 +0700</t>
+          <t>Wed, 21 Oct 2026 19:28:14 +0700</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/20/perawatan-jaringan-listrik-krl-1792511606245_169.jpeg?w=360&amp;amp;q=90" /&gt; KAI melakukan perawatan jaringan listrik aliaran atas pada kereta rel listrik (KRL) berikut lokasi dan prosesnya.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/02/ketua-dewan-komisioner-ojk-friderica-widyasari-dewi-1790924890094_169.jpeg?w=360&amp;amp;q=90" /&gt; Otoritas Jasa Keuangan (OJK) menegaskan reformasi pasar modal akan tetap berlanjut.</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/infrastruktur/d-8716475/180-insulator-di-jalur-krl-diganti-513-926-km-jaringan-listrik-atas-dirawat</t>
+          <t>https://finance.detik.com/bursa-dan-valas/d-8717918/respons-bos-ojk-usai-prabowo-pidato-ri-tidak-takut-msci</t>
         </is>
       </c>
     </row>
@@ -1806,22 +1830,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Nilai Ekspor Hilirisasi Mineral Diprediksi Tembus Rp 898 Triliun</t>
+          <t>Menperin Usul Mobil Hybrid Bebas Ganjil Genap &amp;amp; Dapat Parkir Khusus</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Tue, 20 Oct 2026 22:34:40 +0700</t>
+          <t>Wed, 21 Oct 2026 19:12:04 +0700</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/11/07/energi-bersih-dari-danau-toba-yang-menyalakan-industri-aluminium-nasional-1762530334223_169.jpeg?w=360&amp;amp;q=90" /&gt; Dewan Ekonomi Nasional (DEN) memprediksi ekspor hilirisasi mineral kritis dapat menyentuh US$ 50 miliar atau seki</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/15/menteri-perindustrian-menperin-muhammad-sarmuji-1792046444534_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Perindustrian (Menperin) Muhammad Sarmuji mengusulkan mobil hybrid bisa mendapat insentif berupa pembebasan ganjil genap hingga par</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8716457/nilai-ekspor-hilirisasi-mineral-diprediksi-tembus-rp-898-triliun</t>
+          <t>https://finance.detik.com/industri/d-8717905/menperin-usul-mobil-hybrid-bebas-ganjil-genap-dapat-parkir-khusus</t>
         </is>
       </c>
     </row>
@@ -1833,22 +1857,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Saran buat Pemerintah Usai MSCI Buka Opsi Bursa RI Turun Kasta</t>
+          <t>China Geber Energi Hijau, Bangun PLTS di Karawang hingga Afrika</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Tue, 20 Oct 2026 22:11:55 +0700</t>
+          <t>Wed, 21 Oct 2026 19:00:16 +0700</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/05/18/ihsg-anjlok-ke-zona-merah-bursa-saham-melemah-tajam-1779098741437_169.jpeg?w=360&amp;amp;q=90" /&gt; Dewan Ekonomi Nasional ikut menyoroti masalah yang terjadi pada Bursa Efek Indonesia (BEI).</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/10/19/plts-sengkol-1760877825671_169.jpeg?w=360&amp;amp;q=90" /&gt; Sejumlah negara berkembang disebut mulai memanfaatkan teknologi dan keahlian dari China untuk mempercepat transisi energi terbarukan.</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/bursa-dan-valas/d-8716445/saran-buat-pemerintah-usai-msci-buka-opsi-bursa-ri-turun-kasta</t>
+          <t>https://finance.detik.com/energi/d-8717876/china-geber-energi-hijau-bangun-plts-di-karawang-hingga-afrika</t>
         </is>
       </c>
     </row>
@@ -1860,22 +1884,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Serapan Gabah Bulog Jateng Tembus 108 Persen dari Target Tahunan</t>
+          <t>Luhut Buka-bukaan soal Usulan Kerugian Negara Bukan Korupsi</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Tue, 20 Oct 2026 21:55:30 +0700</t>
+          <t>Wed, 21 Oct 2026 18:13:10 +0700</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/20/realisasi-serapan-gabah-petani-di-jateng-1792470462877.jpeg?w=360&amp;amp;q=90" /&gt; Bulog Jawa Tengah mencatat serapan gabah petani mencapai 406.253 ton setara beras hingga Oktober 2026, atau 108,43% dari target tahunan.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/21/dewan-ekonomi-nasional-den-melakukan-pertemuan-dengan-presiden-prabowo-subianto-1792553489489_169.jpeg?w=360&amp;amp;q=90" /&gt; Ketua Dewan Ekonomi Nasional (DEN) Luhut Binsar Pandjaitan memberikan penjelasan soal usulan kerugian negar</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/foto-bisnis/d-8715178/serapan-gabah-bulog-jateng-tembus-108-persen-dari-target-tahunan</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8717857/luhut-buka-bukaan-soal-usulan-kerugian-negara-bukan-korupsi</t>
         </is>
       </c>
     </row>
@@ -1887,22 +1911,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Tak Lagi Barang, Bansos Bakal Lewat Transfer Uang Tunai</t>
+          <t>Jaga Fundamental Bisnis, Jasa Marga Buka Opsi Buyback Saham</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Tue, 20 Oct 2026 21:30:19 +0700</t>
+          <t>Wed, 21 Oct 2026 17:51:22 +0700</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2021/07/30/cara-cek-bansos-tunai-kemensos-simak-disini_169.jpeg?w=360&amp;amp;q=90" /&gt; Ketua Dewan Ekonomi Nasional (DEN) Luhut Binsar Pandjaitan menyatakan bantuan sosial (bansos) ke depannya tak lagi dalam bentuk barang</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/21/pt-jasa-marga-persero-tbk-1792579833359.jpeg?w=360&amp;amp;q=90" /&gt; Jasa Marga memantau pasar modal dan mempertimbangkan opsi buyback saham untuk mendukung pertumbuhan jangka panjang dan menjaga fundamental perusahaan.</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8716403/tak-lagi-barang-bansos-bakal-lewat-transfer-uang-tunai</t>
+          <t>https://finance.detik.com/bursa-dan-valas/d-8717806/jaga-fundamental-bisnis-jasa-marga-buka-opsi-buyback-saham</t>
         </is>
       </c>
     </row>
@@ -1914,22 +1938,22 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Ungkap Kronologi, Bos ASDP Minta Maaf Insiden Kebakaran KMP Batumandi</t>
+          <t>Bos BI Terus Pantau Pergerakan Modal Asing Usai Pengumuman MSCI</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Tue, 20 Oct 2026 21:13:24 +0700</t>
+          <t>Wed, 21 Oct 2026 17:23:22 +0700</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/20/proses-evakuasi-penumpang-kmp-batumandi-yang-terbakar-1792501886942_169.jpeg?w=360&amp;amp;q=90" /&gt; Direktur Utama ASDP Heru Widodo menyampaikan permohonan maaf atas insiden yang terjadi dan menegaskan keselamatan penumpang serta awa</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/21/bank-indonesia-bi-memutuskan-menaikkan-suku-bunga-deposit-facility-sebesar-25-basis-poin-bps-menjadi-5-keputusan-tersebut-diam-1792576096896_169.jpeg?w=360&amp;amp;q=90" /&gt; Imbas pengumuman ini, rupiah juga sempat tercatat melemah se</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8716386/ungkap-kronologi-bos-asdp-minta-maaf-insiden-kebakaran-kmp-batumandi</t>
+          <t>https://finance.detik.com/moneter/d-8717743/bos-bi-terus-pantau-pergerakan-modal-asing-usai-pengumuman-msci</t>
         </is>
       </c>
     </row>
@@ -1941,22 +1965,22 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>RI Mau Contoh Jepang &amp;amp; Italia Bikin MBG Prasmanan</t>
+          <t>Beredar Kabar CIMB Niaga Bakal Cabut dari Bursa, Dirut Buka Suara</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Tue, 20 Oct 2026 21:00:03 +0700</t>
+          <t>Wed, 21 Oct 2026 17:02:27 +0700</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/20/penerima-manfaat-mbg-dalam-dua-tahun-pemerintahan-prabowo-1792479756787_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Koordinator Bidang Pangan Zulkifli Hasan buka-bukaan soal empat prioritas pembenahan program Makan Bergizi Gratis (MBG).</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/01/31/cimb-niaga-1769845465946_169.png?w=360&amp;amp;q=90" /&gt; PT Bank CIMB Niaga Tbk (BNGA) dikabarkan akan melakukan pembatalan pencatatan saham atau delisting dari Bursa Efek Indonesia (BEI).</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8716171/ri-mau-contoh-jepang-italia-bikin-mbg-prasmanan</t>
+          <t>https://finance.detik.com/bursa-dan-valas/d-8717687/beredar-kabar-cimb-niaga-bakal-cabut-dari-bursa-dirut-buka-suara</t>
         </is>
       </c>
     </row>
@@ -1968,22 +1992,22 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2 Tahun Prabowo-Gibran, BULOG Luncurkan Kemasan Baru Beras SPHP</t>
+          <t>BI Naikkan Suku Bunga Deposit Facility Jadi 5 Persen, BI Rate Tetap 5,75 Persen</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Tue, 20 Oct 2026 20:30:23 +0700</t>
+          <t>Wed, 21 Oct 2026 17:01:39 +0700</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/20/2-tahun-prabowogibran-bulog-luncurkan-kemasan-baru-beras-sphp-1792502990466.jpeg?w=360&amp;amp;q=90" /&gt; Perum BULOG luncurkan kemasan baru 'Beras Kita Medium' untuk stabilisasi pangan. Inovasi ini dukung ketahanan pangan dan harga te</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/21/bank-indonesia-bi-memutuskan-menaikkan-suku-bunga-deposit-facility-sebesar-25-basis-poin-bps-menjadi-5-keputusan-tersebut-diam-1792576096521_169.jpeg?w=360&amp;amp;q=90" /&gt; Bank Indonesia menaikkan suku bunga Deposit Facility menjadi</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8716335/2-tahun-prabowo-gibran-bulog-luncurkan-kemasan-baru-beras-sphp</t>
+          <t>https://finance.detik.com/foto-bisnis/d-8717658/bi-naikkan-suku-bunga-deposit-facility-jadi-5-persen-bi-rate-tetap-5-75-persen</t>
         </is>
       </c>
     </row>
@@ -1995,22 +2019,22 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Luhut Usul ke Prabowo Kerugian Negara Bukan Pidana Korupsi</t>
+          <t>Prabowo: Prestasi Kita Paling Utama Swasembada Pangan dalam Waktu Cepat</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Tue, 20 Oct 2026 20:14:23 +0700</t>
+          <t>Wed, 21 Oct 2026 16:53:03 +0700</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/06/09/luhut-hingga-chatib-basri-temui-prabowo-di-istana-1781007630172_169.jpeg?w=360&amp;amp;q=90" /&gt; Ketua Dewan Ekonomi Nasional (DEN) Luhut Binsar Pandjaitan mengusulkan kajian untuk mengubah definisi tindak pidana korupsi di Indonesia.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/21/prabowo-pimpin-sidang-kabinet-2-tahun-pemerintahan-di-istana-jakarta-rabu-21102026-1792574488043_169.jpeg?w=360&amp;amp;q=90" /&gt; Presiden Prabowo Subianto bersyukur Indonesia berhasil swasembada pangan.</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8716297/luhut-usul-ke-prabowo-kerugian-negara-bukan-pidana-korupsi</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8717656/prabowo-prestasi-kita-paling-utama-swasembada-pangan-dalam-waktu-cepat</t>
         </is>
       </c>
     </row>
@@ -2022,22 +2046,22 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>MUI Tak Setuju Wajib Halal Diundur, Ini Alasannya</t>
+          <t>Sebut Korporasi Jadi Biang Kerok Karhutla, Prabowo: Ini Terorisme Lingkungan!</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Tue, 20 Oct 2026 20:00:41 +0700</t>
+          <t>Wed, 21 Oct 2026 16:50:49 +0700</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/01/17/logo-halal-resmi-di-negara-asean-6_169.png?w=360&amp;amp;q=90" /&gt; Awalnya, kewajiban sertifikasi halal dijadwalkan mulai berlaku 18 Oktober 2026.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/21/prabowo-pimpin-sidang-kabinet-2-tahun-pemerintahan-di-istana-jakarta-rabu-21102026-1792574488128_169.jpeg?w=360&amp;amp;q=90" /&gt; Presiden Prabowo Subianto menyatakan karhutla di Indonesia akibat campur tangan manusia dan korporasi.</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8716229/mui-tak-setuju-wajib-halal-diundur-ini-alasannya</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8717649/sebut-korporasi-jadi-biang-kerok-karhutla-prabowo-ini-terorisme-lingkungan</t>
         </is>
       </c>
     </row>
@@ -2049,22 +2073,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Respons Bos BEI soal Isu Singapura di Balik IHSG Rontok Usai Pernyataan MSCI</t>
+          <t>IHSG Ditutup di Level 5.328, Naik 0,94%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Tue, 20 Oct 2026 19:56:21 +0700</t>
+          <t>Wed, 21 Oct 2026 16:43:59 +0700</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/28/direktur-utama-bei-jeffrey-hendrik-1790588485860_169.jpeg?w=360&amp;amp;q=90" /&gt; Bursa Efek Indonesia (BEI) buka suara terkait dugaan intervensi Singapura di balik usulan MSCI menurunkan status bursa saham Indonesia ke standalone mar</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/01/30/ihsg-rebound-usai-dua-hari-anjlok-seiring-pengunduran-diri-dirut-bei-1769748663323_169.jpeg?w=360&amp;amp;q=90" /&gt; Indeks Harga Saham Gabungan (IHSG) ditutup menguat pada perdagangan hari ini, Rabu (21/10/2026).</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/bursa-dan-valas/d-8716255/respons-bos-bei-soal-isu-singapura-di-balik-ihsg-rontok-usai-pernyataan-msci</t>
+          <t>https://finance.detik.com/bursa-dan-valas/d-8717606/ihsg-ditutup-di-level-5-328-naik-0-94</t>
         </is>
       </c>
     </row>
@@ -2076,22 +2100,22 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>6 Lembaga Tempatkan Mentan Amran Posisi Atas di Dua Tahun Prabowo-Gibran</t>
+          <t>BI Ancam Cabut Izin Merchant yang Pakai QRIS buat Judol</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Tue, 20 Oct 2026 19:42:04 +0700</t>
+          <t>Wed, 21 Oct 2026 16:38:11 +0700</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/11/08/ilustrasi-swasembada-pangan-1762593423685.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Pertanian Andi Amran Sulaiman meraih pengakuan tinggi dari enam lembaga independen. Program swasembada pangan sukses, meningkatkan kesejahteraan petani.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/08/01/ilustrasi-qris-1785553518914_169.png?w=360&amp;amp;q=90" /&gt; Bank Indonesia (BI) tak segan mencabut izin merchant atau Penyedia Jasa Pembayaran (PJP) yang terbukti menggunakan QRIS dalam transaksi judi online (judol).</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8716249/6-lembaga-tempatkan-mentan-amran-posisi-atas-di-dua-tahun-prabowo-gibran</t>
+          <t>https://finance.detik.com/moneter/d-8717592/bi-ancam-cabut-izin-merchant-yang-pakai-qris-buat-judol</t>
         </is>
       </c>
     </row>
@@ -2103,22 +2127,22 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Suahasil Pastikan Penyaluran Gaji PNS Tak Lewat Koperasi</t>
+          <t>Prabowo Pede RI Tak Perlu Impor BBM Berkat B50 &amp;amp; E50</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Tue, 20 Oct 2026 19:33:10 +0700</t>
+          <t>Wed, 21 Oct 2026 16:38:04 +0700</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/20/menteri-keuangan-suahasil-nazara-1792487454171_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Keuangan Suahasil Nazara memastikan mekanisme gaji Aparatur Sipil Negara (ASN) tidak akan mengalami perubahan.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/21/prabowo-pimpin-sidang-kabinet-2-tahun-pemerintahan-di-istana-jakarta-rabu-21102026-1792574488043_169.jpeg?w=360&amp;amp;q=90" /&gt; Presiden Prabowo Subianto optimistis Indonesia tidak perlu lagi mengimpor bahan bakar minyak (BBM).</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8716223/suahasil-pastikan-penyaluran-gaji-pns-tak-lewat-koperasi</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8717598/prabowo-pede-ri-tak-perlu-impor-bbm-berkat-b50-e50</t>
         </is>
       </c>
     </row>
@@ -2130,22 +2154,22 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>KPK Duga Ada Keterlibatan TNI Aktif di Kasus Korupsi Dana Bencana</t>
+          <t>KPK Buka Suara soal Usulan Hapus Unsur Kerugian Negara dalam Definisi Korupsi</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Wed, 21 Oct 2026 07:07:38 +0700</t>
+          <t>Wed, 21 Oct 2026 20:23:25 +0700</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Apa yang lebih jahat dari korupsi dana bencana?</t>
+          <t>KPK menilai diskursus kerugian keuangan negara sudah firm. Lebih penting membahas penguatan pemberantasan korupsi.</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8317763/kpk-duga-ada-keterlibatan-tni-aktif-di-kasus-korupsi-dana-bencana</t>
+          <t>https://www.liputan6.com/news/read/8318490/kpk-buka-suara-soal-usulan-hapus-unsur-kerugian-negara-dalam-definisi-korupsi</t>
         </is>
       </c>
     </row>
@@ -2157,22 +2181,22 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Koperasi Pegawai Diduga Kelola Potongan Insentif di Pemkab Bogor</t>
+          <t>Prabowo ke Jajaran Kabinet: Saya Bangga Menjadi Presidenmu</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Wed, 21 Oct 2026 06:25:01 +0700</t>
+          <t>Wed, 21 Oct 2026 20:09:37 +0700</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>KPK mendalami dugaan potongan insentif yang dikelola melalui koperasi pegawai Pemkab Bogor dan diduga mengalir kepada penyelenggara negara.</t>
+          <t>Presiden Prabowo menyampaikan apresiasi kepada jajaran Kabinet Merah Putih.</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8317754/koperasi-pegawai-diduga-kelola-potongan-insentif-di-pemkab-bogor</t>
+          <t>https://www.liputan6.com/news/read/8318479/prabowo-ke-jajaran-kabinet-saya-bangga-menjadi-presidenmu</t>
         </is>
       </c>
     </row>
@@ -2184,22 +2208,22 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Maruli Simanjuntak Minta Program Ekonomi Perbatasan Tak Berbelit</t>
+          <t>KPK Bidik 2 Prajurit TNI Aktif di Kasus Korupsi BNPB</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Wed, 21 Oct 2026 06:07:31 +0700</t>
+          <t>Wed, 21 Oct 2026 19:35:55 +0700</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>BNPPDT memprioritaskan program ekonomi berbiaya terjangkau yang bisa segera dijalankan untuk masyarakat perbatasan dan daerah terpencil.</t>
+          <t>KPK libatkan Puspom TNI dalam penyelidikan kasus korupsi BNPB.</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8317751/maruli-simanjuntak-minta-program-ekonomi-perbatasan-tak-berbelit</t>
+          <t>https://www.liputan6.com/news/read/8318445/kpk-bidik-2-prajurit-tni-aktif-di-kasus-korupsi-bnpb</t>
         </is>
       </c>
     </row>
@@ -2211,22 +2235,22 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>ASI: Kepercayaan ke Prabowo-Gibran 61,4 Persen, Kepuasan Beda Angka</t>
+          <t>Syahganda Nainggolan Siap Kawal Kepastian Status Pengemudi Ojol</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Wed, 21 Oct 2026 05:40:04 +0700</t>
+          <t>Wed, 21 Oct 2026 19:26:12 +0700</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Survei ASI mencatat kepercayaan terhadap pemerintahan Prabowo-Gibran sebesar 61,4 persen. Namun, kepuasan terhadap kinerja keduanya berbeda.</t>
+          <t>Kejelasan mengenai kedudukan pengemudi penting driver ojol.</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8317746/asi-kepercayaan-ke-prabowo-gibran-614-persen-kepuasan-beda-angka</t>
+          <t>https://www.liputan6.com/news/read/8318434/syahganda-nainggolan-siap-kawal-kepastian-status-pengemudi-ojol</t>
         </is>
       </c>
     </row>
@@ -2238,22 +2262,22 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>KPK Sita Rp 250 Juta dari PCNU Nias, Diduga Terkait Muktamar NU</t>
+          <t>Pemerintah Tegaskan Pro Buruh, Upah Naik hingga 6,5% dan Ojol Terima 92%</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Wed, 21 Oct 2026 01:03:49 +0700</t>
+          <t>Wed, 21 Oct 2026 19:24:37 +0700</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>KPK turut menelusuri keterkaitan uang tersebut dengan kasus korupsi di Kementerian ATR/BPN.</t>
+          <t>Kepala Bakom Syahganda Nainggolan menegaskan pemerintah sangat berpihak kepada buruh.</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8317727/kpk-sita-rp-250-juta-dari-pcnu-nias-diduga-terkait-muktamar-nu</t>
+          <t>https://www.liputan6.com/news/read/8318431/pemerintah-tegaskan-pro-buruh-upah-naik-hingga-65-dan-ojol-terima-92</t>
         </is>
       </c>
     </row>
@@ -2265,22 +2289,22 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Prabowo Terima DEN, Bahas Antisipasi El Nino hingga Kebakaran Hutan</t>
+          <t>Bareskrim Usut Dugaan Beras Fortifikasi Tak Sesuai Label</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Wed, 21 Oct 2026 00:33:52 +0700</t>
+          <t>Wed, 21 Oct 2026 19:14:37 +0700</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Dewan Ekonomi Nasional merekomendasikan sejumlah hal kepada pemerintah.</t>
+          <t>Penyidik menyita 1.194 kemasan beras dari lima merek berbeda.</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8317713/prabowo-terima-den-bahas-antisipasi-el-nino-hingga-kebakaran-hutan</t>
+          <t>https://www.liputan6.com/news/read/8318426/bareskrim-usut-dugaan-beras-fortifikasi-tak-sesuai-label</t>
         </is>
       </c>
     </row>
@@ -2292,22 +2316,22 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>KPK Sita Uang hingga Perhiasan di Rumah Dinas Bupati Klaten</t>
+          <t>Kabakom Janji Sampaikan 'Suara' Buruh soal Upah hingga PHK ke Presiden</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Wed, 21 Oct 2026 00:08:34 +0700</t>
+          <t>Wed, 21 Oct 2026 19:26:38 +0700</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Penyidik akan menelaah seluruh barang yang telah disita untuk kepentingan penyidikan.</t>
+          <t>Kabakom pastikan pemerintah berpihak pada buruh.</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8317721/kpk-sita-uang-hingga-perhiasan-di-rumah-dinas-bupati-klaten</t>
+          <t>https://www.liputan6.com/news/read/8318414/kabakom-janji-sampaikan-suara-buruh-soal-upah-hingga-phk-ke-presiden</t>
         </is>
       </c>
     </row>
@@ -2319,22 +2343,22 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Tak Hanya Aset Henry Surya, Kejagung Telusuri Peminjam Dana Indosurya</t>
+          <t>Jaksa Beberkan Kelemahan Eksepsi Don Ritto</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Tue, 20 Oct 2026 23:32:55 +0700</t>
+          <t>Wed, 21 Oct 2026 18:51:22 +0700</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Upaya tersebut dilakukan untuk mengoptimalkan pemulihan kerugian ribuan korban melalui perampasan dan pelelangan aset.</t>
+          <t>Jaksa menilai sebagian besar keberatan diajukan Don Ritto telah memasuki materi pokok perkara harus dibuktikan dalam persidangan.</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8317669/tak-hanya-aset-henry-surya-kejagung-telusuri-peminjam-dana-indosurya</t>
+          <t>https://www.liputan6.com/news/read/8318409/jaksa-beberkan-kelemahan-eksepsi-don-ritto</t>
         </is>
       </c>
     </row>
@@ -2346,22 +2370,22 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>6 Aktivis Greenpeace Dibebaskan Usai Diperiksa 8 Jam</t>
+          <t>Bakom Pastikan Pemerintah Terus Evaluasi MBG dan Perkuat Pengawasan</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Tue, 20 Oct 2026 23:03:32 +0700</t>
+          <t>Wed, 21 Oct 2026 18:33:00 +0700</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Para aktivis Greenpeace tersebut dibebaskan sekitar pukul 20.30 WIB.</t>
+          <t>Syahganda menegaskan aspek kebersihan, penyimpanan bahan pangan, dan pengawasan menjadi bagian penting dalam evaluasi MBG.</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8317698/6-aktivis-greenpeace-dibebaskan-usai-diperiksa-8-jam</t>
+          <t>https://www.liputan6.com/news/read/8318388/bakom-pastikan-pemerintah-terus-evaluasi-mbg-dan-perkuat-pengawasan</t>
         </is>
       </c>
     </row>
@@ -2373,22 +2397,22 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Pemerintah Respons Aksi Greenpeace soal Krisis Iklim dan Biaya Hidup</t>
+          <t>Said Abdullah Soroti Kekeringan dan Kebakaran Hutan Berulang Tiap Tahun</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Tue, 20 Oct 2026 22:12:37 +0700</t>
+          <t>Wed, 21 Oct 2026 18:16:01 +0700</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Greenpeace membentangkan spanduk kritik di kawasan Bundaran Hotel Indonesia (HI), Jakarta.</t>
+          <t>Menurut Said, Karhutla dan kekeringan saling berhubungan. Hutan adalah penyangga kehidupan dan daerah tangkapan air.</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8317664/pemerintah-respons-aksi-greenpeace-soal-krisis-iklim-dan-biaya-hidup</t>
+          <t>https://www.liputan6.com/news/read/8318374/said-abdullah-soroti-kekeringan-dan-kebakaran-hutan-berulang-tiap-tahun</t>
         </is>
       </c>
     </row>
@@ -2400,22 +2424,22 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>DEN: 95 Persen Siswa Lebih Semangat Belajar Jika MBG Berkualitas</t>
+          <t>Apresiasi Transformasi Pertanian Mentan Amran, Wakil Ketua Komisi IV DPR Soroti Mekanisasi hingga Harga Gabah</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Tue, 20 Oct 2026 21:27:47 +0700</t>
+          <t>Wed, 21 Oct 2026 18:08:51 +0700</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Presiden Prabowo menerima rekomendasi DEN untuk meningkatkan perhatian terhadap kualitas menu MBG.</t>
+          <t>Hanan A Rozak menyoroti peran mekanisasi, pupuk bersubsidi, irigasi, dan kebijakan harga dalam mendukung produksi serta swasembada pangan.</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8317655/den-95-persen-siswa-lebih-semangat-belajar-jika-mbg-berkualitas</t>
+          <t>https://www.liputan6.com/news/read/8318371/apresiasi-transformasi-pertanian-mentan-amran-wakil-ketua-komisi-iv-dpr-soroti-mekanisasi-hingga-harga-gabah</t>
         </is>
       </c>
     </row>
@@ -2427,22 +2451,22 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Perjalanan 6 Tahun Korban KSP Indosurya Tagih Ganti Rugi</t>
+          <t>Kapolri Buka Suara Penyidikan Kasus Polisi Tembak Polisi</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Tue, 20 Oct 2026 21:08:29 +0700</t>
+          <t>Wed, 21 Oct 2026 18:19:30 +0700</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Pengembalian dana tahap pertama kasus KSP Indosurya menjadi titik terang setelah bertahun-tahun menanti.</t>
+          <t>Motif penembakan masih misteri.</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8317643/perjalanan-6-tahun-korban-ksp-indosurya-tagih-ganti-rugi</t>
+          <t>https://www.liputan6.com/news/read/8318368/kapolri-buka-suara-penyidikan-kasus-polisi-tembak-polisi</t>
         </is>
       </c>
     </row>
@@ -2454,22 +2478,22 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Mekanisme Penyaluran Rp 229,4 Miliar Ganti Rugi Korban Indosurya</t>
+          <t>Prabowo Jawab Kritik Kabinet Gemuk</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Tue, 20 Oct 2026 20:43:30 +0700</t>
+          <t>Wed, 21 Oct 2026 18:06:23 +0700</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Penyaluran tahap pertama ini merupakan bagian dari pelaksanaan putusan terhadap terpidana Henry Surya dengan total dana sebesar Rp 229,4 miliar.</t>
+          <t>Prabowo menanggapi kritik terhadap jumlah anggota Kabinet Merah Putih yang dinilai terlalu besar dan tidak efisien.</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8317623/mekanisme-penyaluran-rp-2294-miliar-ganti-rugi-korban-indosurya</t>
+          <t>https://www.liputan6.com/news/read/8318367/prabowo-jawab-kritik-kabinet-gemuk</t>
         </is>
       </c>
     </row>
@@ -2481,22 +2505,22 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Demo di Tugu Tani Usai, Massa Sempat Bakar Flare</t>
+          <t>Ancaman Prabowo ke Korporasi Terlibat Kebakaran Hutan</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Tue, 20 Oct 2026 20:15:36 +0700</t>
+          <t>Wed, 21 Oct 2026 17:45:00 +0700</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Massa bubar perlahan usai memasang spanduk berisi lima tuntutan kepada pemerintah.</t>
+          <t>Prabowo menuturkan, berdasarkan hasil penyelidikan di lapangan, fenomena karhutla tidak semata-mata alamiah, namun juga ada campur tangan manusia.</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8317613/demo-di-tugu-tani-usai-massa-sempat-bakar-flare</t>
+          <t>https://www.liputan6.com/news/read/8318352/ancaman-prabowo-ke-korporasi-terlibat-kebakaran-hutan</t>
         </is>
       </c>
     </row>
@@ -2508,22 +2532,22 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Kebakaran Hutan Arjuno-Ringgit Meluas, Api Mendekati Permukiman Warga</t>
+          <t>Finger Heart Rocky Gerung untuk Dua Tahun Prabowo-Gibran</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Tue, 20 Oct 2026 20:03:39 +0700</t>
+          <t>Wed, 21 Oct 2026 17:39:35 +0700</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Api dilaporkan merembet ke arah selatan menuju Kecamatan Singosari, Kabupaten Malang.</t>
+          <t>Rocky menyampaikan penilaian tersebut saat menghadiri sidang kabinet paripurna di Istana.</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8317604/kebakaran-hutan-arjuno-ringgit-meluas-api-mendekati-permukiman-warga</t>
+          <t>https://www.liputan6.com/news/read/8318349/finger-heart-rocky-gerung-untuk-dua-tahun-prabowo-gibran</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data pasar & berita - 2026-10-22 00:16 UTC
</commit_message>
<xml_diff>
--- a/data/market_news_latest.xlsx
+++ b/data/market_news_latest.xlsx
@@ -487,20 +487,20 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>5328.3599</v>
+        <v>5278.8882</v>
       </c>
       <c r="F2" t="n">
-        <v>49.4717</v>
+        <v>282.2793</v>
       </c>
       <c r="G2" t="n">
-        <v>0.9399999999999999</v>
+        <v>5.65</v>
       </c>
       <c r="H2" t="n">
-        <v>0</v>
+        <v>534990700</v>
       </c>
     </row>
     <row r="3">
@@ -525,16 +525,16 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>7727.0698</v>
+        <v>7757.1699</v>
       </c>
       <c r="F3" t="n">
-        <v>14.5</v>
+        <v>44.6001</v>
       </c>
       <c r="G3" t="n">
-        <v>0.19</v>
+        <v>0.58</v>
       </c>
       <c r="H3" t="n">
-        <v>180674661</v>
+        <v>2889474000</v>
       </c>
     </row>
     <row r="4">
@@ -559,16 +559,16 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>52503.5117</v>
+        <v>52856.0898</v>
       </c>
       <c r="F4" t="n">
-        <v>7.6328</v>
+        <v>360.2109</v>
       </c>
       <c r="G4" t="n">
-        <v>0.01</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="H4" t="n">
-        <v>28472368</v>
+        <v>359385262</v>
       </c>
     </row>
     <row r="5">
@@ -593,16 +593,16 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>26548.4805</v>
+        <v>26702.8574</v>
       </c>
       <c r="F5" t="n">
-        <v>123.6602</v>
+        <v>278.0371</v>
       </c>
       <c r="G5" t="n">
-        <v>0.47</v>
+        <v>1.05</v>
       </c>
       <c r="H5" t="n">
-        <v>1182947000</v>
+        <v>6898345000</v>
       </c>
     </row>
     <row r="6">
@@ -623,17 +623,17 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>64621.2383</v>
+        <v>64746.4883</v>
       </c>
       <c r="F6" t="n">
-        <v>545.8164</v>
+        <v>671.0664</v>
       </c>
       <c r="G6" t="n">
-        <v>0.85</v>
+        <v>1.05</v>
       </c>
       <c r="H6" t="n">
         <v>0</v>
@@ -657,20 +657,20 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>23651.8691</v>
+        <v>23867.7402</v>
       </c>
       <c r="F7" t="n">
-        <v>-215.8711</v>
+        <v>-319.0898</v>
       </c>
       <c r="G7" t="n">
-        <v>-0.9</v>
+        <v>-1.32</v>
       </c>
       <c r="H7" t="n">
-        <v>0</v>
+        <v>2650200000</v>
       </c>
     </row>
     <row r="8">
@@ -694,15 +694,9 @@
           <t>2026-10-21</t>
         </is>
       </c>
-      <c r="E8" t="n">
-        <v>3713.0276</v>
-      </c>
-      <c r="F8" t="n">
-        <v>-22.3425</v>
-      </c>
-      <c r="G8" t="n">
-        <v>-0.6</v>
-      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
       <c r="H8" t="n">
         <v>3468900532</v>
       </c>
@@ -725,20 +719,20 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>10770.4902</v>
+        <v>10733</v>
       </c>
       <c r="F9" t="n">
-        <v>37.4902</v>
+        <v>-31.7002</v>
       </c>
       <c r="G9" t="n">
-        <v>0.35</v>
+        <v>-0.29</v>
       </c>
       <c r="H9" t="n">
-        <v>0</v>
+        <v>848274600</v>
       </c>
     </row>
     <row r="10">
@@ -759,20 +753,20 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>25660.8906</v>
+        <v>25304.4199</v>
       </c>
       <c r="F10" t="n">
-        <v>356.4707</v>
+        <v>-15.3496</v>
       </c>
       <c r="G10" t="n">
-        <v>1.41</v>
+        <v>-0.06</v>
       </c>
       <c r="H10" t="n">
-        <v>0</v>
+        <v>52913300</v>
       </c>
     </row>
     <row r="11">
@@ -793,20 +787,20 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>5437.9902</v>
+        <v>5404.02</v>
       </c>
       <c r="F11" t="n">
-        <v>33.9702</v>
+        <v>-7.98</v>
       </c>
       <c r="G11" t="n">
-        <v>0.63</v>
+        <v>-0.15</v>
       </c>
       <c r="H11" t="n">
-        <v>0</v>
+        <v>249844900</v>
       </c>
     </row>
     <row r="12">
@@ -827,17 +821,17 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="E12" t="n">
         <v>17943</v>
       </c>
       <c r="F12" t="n">
-        <v>-98</v>
+        <v>-42.4004</v>
       </c>
       <c r="G12" t="n">
-        <v>-0.54</v>
+        <v>-0.24</v>
       </c>
       <c r="H12" t="n">
         <v>0</v>
@@ -865,10 +859,10 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>101.685</v>
+        <v>101.687</v>
       </c>
       <c r="F13" t="n">
-        <v>-0.045</v>
+        <v>-0.043</v>
       </c>
       <c r="G13" t="n">
         <v>-0.04</v>
@@ -895,17 +889,17 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>157.983</v>
+        <v>158.185</v>
       </c>
       <c r="F14" t="n">
-        <v>-0.54</v>
+        <v>-0.083</v>
       </c>
       <c r="G14" t="n">
-        <v>-0.34</v>
+        <v>-0.05</v>
       </c>
       <c r="H14" t="n">
         <v>0</v>
@@ -933,13 +927,13 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>0.5094</v>
+        <v>0.5145999999999999</v>
       </c>
       <c r="F15" t="n">
-        <v>-0.0023</v>
+        <v>0.0029</v>
       </c>
       <c r="G15" t="n">
-        <v>-0.45</v>
+        <v>0.57</v>
       </c>
       <c r="H15" t="n">
         <v>0</v>
@@ -967,13 +961,13 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>0.5406</v>
+        <v>0.5439000000000001</v>
       </c>
       <c r="F16" t="n">
-        <v>-0.0019</v>
+        <v>0.0014</v>
       </c>
       <c r="G16" t="n">
-        <v>-0.35</v>
+        <v>0.26</v>
       </c>
       <c r="H16" t="n">
         <v>0</v>
@@ -1001,13 +995,13 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>0.407</v>
+        <v>0.4063</v>
       </c>
       <c r="F17" t="n">
-        <v>-0.001</v>
+        <v>-0.0017</v>
       </c>
       <c r="G17" t="n">
-        <v>-0.25</v>
+        <v>-0.42</v>
       </c>
       <c r="H17" t="n">
         <v>0</v>
@@ -1034,17 +1028,11 @@
           <t>2026-10-21</t>
         </is>
       </c>
-      <c r="E18" t="n">
-        <v>80.34</v>
-      </c>
-      <c r="F18" t="n">
-        <v>0.21</v>
-      </c>
-      <c r="G18" t="n">
-        <v>0.26</v>
-      </c>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
       <c r="H18" t="n">
-        <v>1976433</v>
+        <v>35949645</v>
       </c>
     </row>
     <row r="19">
@@ -1068,17 +1056,11 @@
           <t>2026-10-21</t>
         </is>
       </c>
-      <c r="E19" t="n">
-        <v>76.95999999999999</v>
-      </c>
-      <c r="F19" t="n">
-        <v>0.13</v>
-      </c>
-      <c r="G19" t="n">
-        <v>0.17</v>
-      </c>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr"/>
       <c r="H19" t="n">
-        <v>1743667</v>
+        <v>35880008</v>
       </c>
     </row>
     <row r="20">
@@ -1103,16 +1085,16 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>4155.7002</v>
+        <v>4140.6001</v>
       </c>
       <c r="F20" t="n">
-        <v>13.1001</v>
+        <v>-2</v>
       </c>
       <c r="G20" t="n">
-        <v>0.32</v>
+        <v>-0.05</v>
       </c>
       <c r="H20" t="n">
-        <v>77851</v>
+        <v>5102</v>
       </c>
     </row>
     <row r="21">
@@ -1137,16 +1119,16 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>97.28</v>
+        <v>97.97</v>
       </c>
       <c r="F21" t="n">
-        <v>-4.51</v>
+        <v>-3.82</v>
       </c>
       <c r="G21" t="n">
-        <v>-4.43</v>
+        <v>-3.75</v>
       </c>
       <c r="H21" t="n">
-        <v>128159</v>
+        <v>4424</v>
       </c>
     </row>
     <row r="22">
@@ -1171,16 +1153,16 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>108.29</v>
+        <v>109.98</v>
       </c>
       <c r="F22" t="n">
-        <v>-0.5</v>
+        <v>1.19</v>
       </c>
       <c r="G22" t="n">
-        <v>-0.46</v>
+        <v>1.09</v>
       </c>
       <c r="H22" t="n">
-        <v>16896</v>
+        <v>240</v>
       </c>
     </row>
     <row r="23">
@@ -1205,16 +1187,16 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>6.553</v>
+        <v>6.558</v>
       </c>
       <c r="F23" t="n">
-        <v>-0.0135</v>
+        <v>-0.008500000000000001</v>
       </c>
       <c r="G23" t="n">
-        <v>-0.21</v>
+        <v>-0.13</v>
       </c>
       <c r="H23" t="n">
-        <v>21092</v>
+        <v>828</v>
       </c>
     </row>
     <row r="24">
@@ -1238,17 +1220,11 @@
           <t>2026-10-21</t>
         </is>
       </c>
-      <c r="E24" t="n">
-        <v>63.565</v>
-      </c>
-      <c r="F24" t="n">
-        <v>0.245</v>
-      </c>
-      <c r="G24" t="n">
-        <v>0.39</v>
-      </c>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr"/>
       <c r="H24" t="n">
-        <v>546239</v>
+        <v>17733563</v>
       </c>
     </row>
     <row r="25">
@@ -1273,13 +1249,13 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>16.96</v>
+        <v>16.68</v>
       </c>
       <c r="F25" t="n">
-        <v>-0.35</v>
+        <v>-0.63</v>
       </c>
       <c r="G25" t="n">
-        <v>-2.02</v>
+        <v>-3.64</v>
       </c>
       <c r="H25" t="n">
         <v>0</v>
@@ -1303,20 +1279,20 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="E26" t="n">
-        <v>83250.77340000001</v>
+        <v>84169.0312</v>
       </c>
       <c r="F26" t="n">
-        <v>309.7734</v>
+        <v>1228.0312</v>
       </c>
       <c r="G26" t="n">
-        <v>0.37</v>
+        <v>1.48</v>
       </c>
       <c r="H26" t="n">
-        <v>26857611264</v>
+        <v>30698053632</v>
       </c>
     </row>
     <row r="27">
@@ -1749,22 +1725,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Bocoran Penetapan &amp;amp; Formula UMP 2027</t>
+          <t>Dua Menteri Pastikan Gaji PNS Tidak Lewat Kopdes, Menkop Buka Suara</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Wed, 21 Oct 2026 20:05:42 +0700</t>
+          <t>Thu, 22 Oct 2026 07:00:00 +0700</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/01/12/ilustrasi-rupiah-atau-upah-minimum-provinsi-ump-1768195061169_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Ketenagakerjaan (Menaker) Yassierli buka suara penetapan Upah Minimum Provinsi (UMP) 2027.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/18/17288-koperasi-desa-merah-putih-siap-beroperasi-ditargetkan-oktober-2026-1789704926087_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Keuangan dan PANRB memastikan gaji PNS tetap dibayar langsung ke rekening, bukan melalui Koperasi Desa.</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8717972/bocoran-penetapan-formula-ump-2027</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8718189/dua-menteri-pastikan-gaji-pns-tidak-lewat-kopdes-menkop-buka-suara</t>
         </is>
       </c>
     </row>
@@ -1776,22 +1752,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Soal Gaji PNS Lewat Kopdes Merah Putih, Menkop Ajak Menkeu Duduk Bareng</t>
+          <t>Cihuy! DP 0% Rumah &amp;amp; Kendaraan Masih Lanjut</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Wed, 21 Oct 2026 19:54:39 +0700</t>
+          <t>Thu, 22 Oct 2026 06:25:00 +0700</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/03/10/menteri-koperasi-menkop-ferry-juliantono-1773150156348_169.jpeg?w=360&amp;amp;q=90" /&gt; Menkop Ferry Juliantono menyampaikan pembayaran gaji PNS hingga pensiunan melalui Kopdes Merah Putih akan dibahas dengan Menteri Keuangan Suahasil</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/21/bank-indonesia-bi-memutuskan-menaikkan-suku-bunga-deposit-facility-sebesar-25-basis-poin-bps-menjadi-5-keputusan-tersebut-diam-1792576096825_169.jpeg?w=360&amp;amp;q=90" /&gt; Bank Indonesia (BI) memperpanjang kebijakan uang muka atau d</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8717963/soal-gaji-pns-lewat-kopdes-merah-putih-menkop-ajak-menkeu-duduk-bareng</t>
+          <t>https://finance.detik.com/moneter/d-8717984/cihuy-dp-0-rumah-kendaraan-masih-lanjut</t>
         </is>
       </c>
     </row>
@@ -1803,22 +1779,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Respons Bos OJK Usai Prabowo Pidato RI Tidak Takut MSCI</t>
+          <t>Prabowo Beri Pesan Keras buat MSCI</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Wed, 21 Oct 2026 19:28:14 +0700</t>
+          <t>Thu, 22 Oct 2026 05:55:09 +0700</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/02/ketua-dewan-komisioner-ojk-friderica-widyasari-dewi-1790924890094_169.jpeg?w=360&amp;amp;q=90" /&gt; Otoritas Jasa Keuangan (OJK) menegaskan reformasi pasar modal akan tetap berlanjut.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/21/sidang-kabinet-paripurna-di-istana-kepresidenan-1792580318733_169.jpeg?w=360&amp;amp;q=90" /&gt; Pesan keras disampaikan Presiden Prabowo Subianto kepada MSCI.</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/bursa-dan-valas/d-8717918/respons-bos-ojk-usai-prabowo-pidato-ri-tidak-takut-msci</t>
+          <t>https://finance.detik.com/bursa-dan-valas/d-8717980/prabowo-beri-pesan-keras-buat-msci</t>
         </is>
       </c>
     </row>
@@ -1830,22 +1806,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Menperin Usul Mobil Hybrid Bebas Ganjil Genap &amp;amp; Dapat Parkir Khusus</t>
+          <t>Saat Pembayaran QRIS Telah Melintasi Batas Negara</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Wed, 21 Oct 2026 19:12:04 +0700</t>
+          <t>Thu, 22 Oct 2026 00:00:00 +0700</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/15/menteri-perindustrian-menperin-muhammad-sarmuji-1792046444534_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Perindustrian (Menperin) Muhammad Sarmuji mengusulkan mobil hybrid bisa mendapat insentif berupa pembebasan ganjil genap hingga par</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/21/adv-1792558313107.jpeg?w=360&amp;amp;q=90" /&gt; Saat Pembayaran QRIS Telah Melintasi Batas Negara</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/industri/d-8717905/menperin-usul-mobil-hybrid-bebas-ganjil-genap-dapat-parkir-khusus</t>
+          <t>https://finance.detik.com/advertorial-news-block/d-8716941/saat-pembayaran-qris-telah-melintasi-batas-negara</t>
         </is>
       </c>
     </row>
@@ -1857,22 +1833,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>China Geber Energi Hijau, Bangun PLTS di Karawang hingga Afrika</t>
+          <t>Rp 31,8 Triliun Disiapkan buat BSU, Beras 10 Kg, hingga Diskon Nataru</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Wed, 21 Oct 2026 19:00:16 +0700</t>
+          <t>Wed, 21 Oct 2026 23:00:36 +0700</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/10/19/plts-sengkol-1760877825671_169.jpeg?w=360&amp;amp;q=90" /&gt; Sejumlah negara berkembang disebut mulai memanfaatkan teknologi dan keahlian dari China untuk mempercepat transisi energi terbarukan.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/13/ilustrasi-bsu-2026-1791879636208_169.jpeg?w=360&amp;amp;q=90" /&gt; Pemerintah menyiapkan 4 program andalan</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8717876/china-geber-energi-hijau-bangun-plts-di-karawang-hingga-afrika</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8718185/rp-31-8-triliun-disiapkan-buat-bsu-beras-10-kg-hingga-diskon-nataru</t>
         </is>
       </c>
     </row>
@@ -1884,22 +1860,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Luhut Buka-bukaan soal Usulan Kerugian Negara Bukan Korupsi</t>
+          <t>Bos Otorita Pastikan Tak Ada Korporasi Terlibat Karhutla Sekitar Kawasan IKN</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Wed, 21 Oct 2026 18:13:10 +0700</t>
+          <t>Wed, 21 Oct 2026 22:55:00 +0700</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/21/dewan-ekonomi-nasional-den-melakukan-pertemuan-dengan-presiden-prabowo-subianto-1792553489489_169.jpeg?w=360&amp;amp;q=90" /&gt; Ketua Dewan Ekonomi Nasional (DEN) Luhut Binsar Pandjaitan memberikan penjelasan soal usulan kerugian negar</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/11/04/kepala-otorita-ikn-basuki-hadimuljono-1762234920793_169.jpeg?w=360&amp;amp;q=90" /&gt; Kepala OIKN Basuki Hadimuljono memastikan tidak ada indikasi keterlibatan korporasi dalam kebakaran hutan dan lahan (karhutla) di sekitar kawasan IKN</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8717857/luhut-buka-bukaan-soal-usulan-kerugian-negara-bukan-korupsi</t>
+          <t>https://finance.detik.com/infrastruktur/d-8718175/bos-otorita-pastikan-tak-ada-korporasi-terlibat-karhutla-sekitar-kawasan-ikn</t>
         </is>
       </c>
     </row>
@@ -1911,22 +1887,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Jaga Fundamental Bisnis, Jasa Marga Buka Opsi Buyback Saham</t>
+          <t>Tips Menghindari Penipuan Berkedok Rekrutmen untuk Para Jobseekers</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Wed, 21 Oct 2026 17:51:22 +0700</t>
+          <t>Wed, 21 Oct 2026 22:48:08 +0700</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/21/pt-jasa-marga-persero-tbk-1792579833359.jpeg?w=360&amp;amp;q=90" /&gt; Jasa Marga memantau pasar modal dan mempertimbangkan opsi buyback saham untuk mendukung pertumbuhan jangka panjang dan menjaga fundamental perusahaan.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/21/tips-menghindari-penipuan-berkedok-rekrutmen-untuk-para-jobseekers-1792597627341.jpeg?w=360&amp;amp;q=90" /&gt; Di era digital, penipuan rekrutmen semakin marak. Direktur Pegadaian berbagi tips untuk jobseeker agar terhindar dari penipu</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/bursa-dan-valas/d-8717806/jaga-fundamental-bisnis-jasa-marga-buka-opsi-buyback-saham</t>
+          <t>https://finance.detik.com/lainnya/d-8718172/tips-menghindari-penipuan-berkedok-rekrutmen-untuk-para-jobseekers</t>
         </is>
       </c>
     </row>
@@ -1938,22 +1914,22 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Bos BI Terus Pantau Pergerakan Modal Asing Usai Pengumuman MSCI</t>
+          <t>Karhutla di Sekitar Kawasan IKN 1.600 Ha Padam, Tidak Ganggu Proyek</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Wed, 21 Oct 2026 17:23:22 +0700</t>
+          <t>Wed, 21 Oct 2026 22:42:37 +0700</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/21/bank-indonesia-bi-memutuskan-menaikkan-suku-bunga-deposit-facility-sebesar-25-basis-poin-bps-menjadi-5-keputusan-tersebut-diam-1792576096896_169.jpeg?w=360&amp;amp;q=90" /&gt; Imbas pengumuman ini, rupiah juga sempat tercatat melemah se</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/08/15/kawasan-inti-pusat-pemerintahan-ibu-kota-nusantara-ikn-1786797746713_169.jpeg?w=360&amp;amp;q=90" /&gt; Otorita Ibu Kota Nusantara memastikan insiden kebakaran hutan dan lahan kurang lebih 1.600 hektare di sekitar kawasan IKN telah berh</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/moneter/d-8717743/bos-bi-terus-pantau-pergerakan-modal-asing-usai-pengumuman-msci</t>
+          <t>https://finance.detik.com/infrastruktur/d-8718166/karhutla-di-sekitar-kawasan-ikn-1-600-ha-padam-tidak-ganggu-proyek</t>
         </is>
       </c>
     </row>
@@ -1965,22 +1941,22 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Beredar Kabar CIMB Niaga Bakal Cabut dari Bursa, Dirut Buka Suara</t>
+          <t>Megaproyek IKN Tetap Jalan, Investasi Rp 4 Triliun Baru Masuk</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Wed, 21 Oct 2026 17:02:27 +0700</t>
+          <t>Wed, 21 Oct 2026 22:21:05 +0700</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/01/31/cimb-niaga-1769845465946_169.png?w=360&amp;amp;q=90" /&gt; PT Bank CIMB Niaga Tbk (BNGA) dikabarkan akan melakukan pembatalan pencatatan saham atau delisting dari Bursa Efek Indonesia (BEI).</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2024/12/10/kepala-otorita-ikn-basuki-hadimuljono_169.jpeg?w=360&amp;amp;q=90" /&gt; Pembangunan infrastruktur strategis di kawasan megaproyek Ibu Kota Nusantara (IKN), Kalimantan Timur terus berjalan.</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/bursa-dan-valas/d-8717687/beredar-kabar-cimb-niaga-bakal-cabut-dari-bursa-dirut-buka-suara</t>
+          <t>https://finance.detik.com/infrastruktur/d-8718134/megaproyek-ikn-tetap-jalan-investasi-rp-4-triliun-baru-masuk</t>
         </is>
       </c>
     </row>
@@ -1992,22 +1968,22 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>BI Naikkan Suku Bunga Deposit Facility Jadi 5 Persen, BI Rate Tetap 5,75 Persen</t>
+          <t>Bahlil Buka Opsi Setop Ekspor Gas ke Negara Tetangga</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Wed, 21 Oct 2026 17:01:39 +0700</t>
+          <t>Wed, 21 Oct 2026 21:58:32 +0700</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/21/bank-indonesia-bi-memutuskan-menaikkan-suku-bunga-deposit-facility-sebesar-25-basis-poin-bps-menjadi-5-keputusan-tersebut-diam-1792576096521_169.jpeg?w=360&amp;amp;q=90" /&gt; Bank Indonesia menaikkan suku bunga Deposit Facility menjadi</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/08/04/bahlil-lahadalia-1785840108228_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Energi dan Sumber Daya Mineral (ESDM) Bahlil Lahadalia membuka opsi setop ekspor gas ke negara tetangga.</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/foto-bisnis/d-8717658/bi-naikkan-suku-bunga-deposit-facility-jadi-5-persen-bi-rate-tetap-5-75-persen</t>
+          <t>https://finance.detik.com/energi/d-8718097/bahlil-buka-opsi-setop-ekspor-gas-ke-negara-tetangga</t>
         </is>
       </c>
     </row>
@@ -2019,22 +1995,22 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Prabowo: Prestasi Kita Paling Utama Swasembada Pangan dalam Waktu Cepat</t>
+          <t>Terbongkar Pihak-pihak di Balik Kasus Saham DSSA, BREN, dan CUAN</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Wed, 21 Oct 2026 16:53:03 +0700</t>
+          <t>Wed, 21 Oct 2026 21:32:53 +0700</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/21/prabowo-pimpin-sidang-kabinet-2-tahun-pemerintahan-di-istana-jakarta-rabu-21102026-1792574488043_169.jpeg?w=360&amp;amp;q=90" /&gt; Presiden Prabowo Subianto bersyukur Indonesia berhasil swasembada pangan.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/05/18/ihsg-anjlok-ke-zona-merah-bursa-saham-melemah-tajam-1779098741437_169.jpeg?w=360&amp;amp;q=90" /&gt; OJK menjatuhkan denda kepada tiga emiten di pasar modal Indonesia, yakni DSSA, BREN, dan CUAN.</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8717656/prabowo-prestasi-kita-paling-utama-swasembada-pangan-dalam-waktu-cepat</t>
+          <t>https://finance.detik.com/bursa-dan-valas/d-8718072/terbongkar-pihak-pihak-di-balik-kasus-saham-dssa-bren-dan-cuan</t>
         </is>
       </c>
     </row>
@@ -2046,22 +2022,22 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Sebut Korporasi Jadi Biang Kerok Karhutla, Prabowo: Ini Terorisme Lingkungan!</t>
+          <t>Bima Arya: Mengejar Pertumbuhan Ekonomi Harus Peduli pada Lingkungan</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Wed, 21 Oct 2026 16:50:49 +0700</t>
+          <t>Wed, 21 Oct 2026 21:23:46 +0700</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/21/prabowo-pimpin-sidang-kabinet-2-tahun-pemerintahan-di-istana-jakarta-rabu-21102026-1792574488128_169.jpeg?w=360&amp;amp;q=90" /&gt; Presiden Prabowo Subianto menyatakan karhutla di Indonesia akibat campur tangan manusia dan korporasi.</t>
+          <t xml:space="preserve">&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/21/wakil-menteri-dalam-negeri-wamendagri-bima-arya-sugiarto-1792592599172.jpeg?w=360&amp;amp;q=90" /&gt; Wamendagri Bima Arya dorong Pemda selaraskan pertumbuhan ekonomi dengan pelestarian lingkungan. Pentingnya partisipasi masyarakat dan </t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8717649/sebut-korporasi-jadi-biang-kerok-karhutla-prabowo-ini-terorisme-lingkungan</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8718060/bima-arya-mengejar-pertumbuhan-ekonomi-harus-peduli-pada-lingkungan</t>
         </is>
       </c>
     </row>
@@ -2073,22 +2049,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>IHSG Ditutup di Level 5.328, Naik 0,94%</t>
+          <t>Harga Minyak Meroket, Pertalite Dipastikan Tidak Naik</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Wed, 21 Oct 2026 16:43:59 +0700</t>
+          <t>Wed, 21 Oct 2026 21:03:01 +0700</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/01/30/ihsg-rebound-usai-dua-hari-anjlok-seiring-pengunduran-diri-dirut-bei-1769748663323_169.jpeg?w=360&amp;amp;q=90" /&gt; Indeks Harga Saham Gabungan (IHSG) ditutup menguat pada perdagangan hari ini, Rabu (21/10/2026).</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/08/20/pemerintah-perketat-penyaluran-pertalite-mulai-2027-1787210254552_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Energi dan Sumber Daya Mineral (ESDM) Bahlil Lahadalia menegaskan pemerintah tidak menaikkan harga bahan bakar minyak (BBM) sub</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/bursa-dan-valas/d-8717606/ihsg-ditutup-di-level-5-328-naik-0-94</t>
+          <t>https://finance.detik.com/energi/d-8718032/harga-minyak-meroket-pertalite-dipastikan-tidak-naik</t>
         </is>
       </c>
     </row>
@@ -2100,22 +2076,22 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>BI Ancam Cabut Izin Merchant yang Pakai QRIS buat Judol</t>
+          <t>Prabowo: Prestasi Kita Paling Utama Swasembada Pangan dalam Waktu Cepat</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Wed, 21 Oct 2026 16:38:11 +0700</t>
+          <t>Wed, 21 Oct 2026 20:59:39 +0700</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/08/01/ilustrasi-qris-1785553518914_169.png?w=360&amp;amp;q=90" /&gt; Bank Indonesia (BI) tak segan mencabut izin merchant atau Penyedia Jasa Pembayaran (PJP) yang terbukti menggunakan QRIS dalam transaksi judi online (judol).</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/21/presiden-prabowo-subianto-1792590961666.jpeg?w=360&amp;amp;q=90" /&gt; Presiden Prabowo menegaskan swasembada pangan sebagai prestasi utama pemerintah. Indonesia siap hadapi tantangan global dengan kemandirian pangan yang kuat.</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/moneter/d-8717592/bi-ancam-cabut-izin-merchant-yang-pakai-qris-buat-judol</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8718025/prabowo-prestasi-kita-paling-utama-swasembada-pangan-dalam-waktu-cepat</t>
         </is>
       </c>
     </row>
@@ -2127,22 +2103,22 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Prabowo Pede RI Tak Perlu Impor BBM Berkat B50 &amp;amp; E50</t>
+          <t>Krisis Gas di Taiz Yaman Memaksa Warga Antre Berjam-jam</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Wed, 21 Oct 2026 16:38:04 +0700</t>
+          <t>Wed, 21 Oct 2026 20:53:03 +0700</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/21/prabowo-pimpin-sidang-kabinet-2-tahun-pemerintahan-di-istana-jakarta-rabu-21102026-1792574488043_169.jpeg?w=360&amp;amp;q=90" /&gt; Presiden Prabowo Subianto optimistis Indonesia tidak perlu lagi mengimpor bahan bakar minyak (BBM).</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/21/krisis-gas-di-taiz-yaman-memaksa-warga-antre-berjam-jam-1792560778171.jpeg?w=360&amp;amp;q=90" /&gt; Warga Taiz di Yaman mengantre berjam-jam untuk mendapatkan gas memasak. Krisis pasokan kian memburuk imbas pengepungan dan penutupan ja</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8717598/prabowo-pede-ri-tak-perlu-impor-bbm-berkat-b50-e50</t>
+          <t>https://finance.detik.com/foto-bisnis/d-8717050/krisis-gas-di-taiz-yaman-memaksa-warga-antre-berjam-jam</t>
         </is>
       </c>
     </row>
@@ -2154,22 +2130,22 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>KPK Buka Suara soal Usulan Hapus Unsur Kerugian Negara dalam Definisi Korupsi</t>
+          <t>DPR Ingatkan Timsel KPU Sudah Bisa Dibentuk Tanpa Tunggu RUU Pemilu</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Wed, 21 Oct 2026 20:23:25 +0700</t>
+          <t>Thu, 22 Oct 2026 06:40:39 +0700</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>KPK menilai diskursus kerugian keuangan negara sudah firm. Lebih penting membahas penguatan pemberantasan korupsi.</t>
+          <t>Pembentukan timsel KPU periode berikutnya dapat dimulai tanpa menunggu RUU Pemilu.</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8318490/kpk-buka-suara-soal-usulan-hapus-unsur-kerugian-negara-dalam-definisi-korupsi</t>
+          <t>https://www.liputan6.com/news/read/8318626/dpr-ingatkan-timsel-kpu-sudah-bisa-dibentuk-tanpa-tunggu-ruu-pemilu</t>
         </is>
       </c>
     </row>
@@ -2181,22 +2157,22 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Prabowo ke Jajaran Kabinet: Saya Bangga Menjadi Presidenmu</t>
+          <t>Resolusi Jihad dan Api Perlawanan dari Pesantren</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Wed, 21 Oct 2026 20:09:37 +0700</t>
+          <t>Thu, 22 Oct 2026 06:34:29 +0700</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Presiden Prabowo menyampaikan apresiasi kepada jajaran Kabinet Merah Putih.</t>
+          <t>Resolusi Jihad 22 Oktober 1945 menjadi salah satu pemantik perlawanan ulama dan santri dalam mempertahankan kemerdekaan Indonesia.</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8318479/prabowo-ke-jajaran-kabinet-saya-bangga-menjadi-presidenmu</t>
+          <t>https://www.liputan6.com/news/read/8317894/resolusi-jihad-dan-api-perlawanan-dari-pesantren</t>
         </is>
       </c>
     </row>
@@ -2208,22 +2184,22 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>KPK Bidik 2 Prajurit TNI Aktif di Kasus Korupsi BNPB</t>
+          <t>Belanja APBD Jakarta 2026 Baru Terserap 54,39 Persen, Pramono Ingatkan Jajarannya</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Wed, 21 Oct 2026 19:35:55 +0700</t>
+          <t>Thu, 22 Oct 2026 06:21:52 +0700</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>KPK libatkan Puspom TNI dalam penyelidikan kasus korupsi BNPB.</t>
+          <t>Pramono Anung meminta perangkat daerah mempercepat kegiatan APBD 2026. Hingga akhir September, realisasi belanja Jakarta baru mencapai 54,39 persen dari pagu Rp 74,29 triliun.</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8318445/kpk-bidik-2-prajurit-tni-aktif-di-kasus-korupsi-bnpb</t>
+          <t>https://www.liputan6.com/news/read/8318625/belanja-apbd-jakarta-2026-baru-terserap-5439-persen-pramono-ingatkan-jajarannya</t>
         </is>
       </c>
     </row>
@@ -2235,22 +2211,22 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Syahganda Nainggolan Siap Kawal Kepastian Status Pengemudi Ojol</t>
+          <t>2 TNI Aktif di Pusaran Korupsi Dana Bencana BNPB</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Wed, 21 Oct 2026 19:26:12 +0700</t>
+          <t>Thu, 22 Oct 2026 06:06:10 +0700</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Kejelasan mengenai kedudukan pengemudi penting driver ojol.</t>
+          <t>KPK menggandeng Puspom TNI dalam penanganan perkara.</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8318434/syahganda-nainggolan-siap-kawal-kepastian-status-pengemudi-ojol</t>
+          <t>https://www.liputan6.com/news/read/8318601/2-tni-aktif-di-pusaran-korupsi-dana-bencana-bnpb</t>
         </is>
       </c>
     </row>
@@ -2262,22 +2238,22 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Pemerintah Tegaskan Pro Buruh, Upah Naik hingga 6,5% dan Ojol Terima 92%</t>
+          <t>Bapanas Ungkap Bahaya Beras Fortifikasi, Bikin Mual hingga Anemia</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Wed, 21 Oct 2026 19:24:37 +0700</t>
+          <t>Thu, 22 Oct 2026 05:42:37 +0700</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Kepala Bakom Syahganda Nainggolan menegaskan pemerintah sangat berpihak kepada buruh.</t>
+          <t>Beras fortifikasi mengandung Zinc yang berlebihan. Di pasaran beras fortifiksi medium sempat beredar bahkan dengan label premium.</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8318431/pemerintah-tegaskan-pro-buruh-upah-naik-hingga-65-dan-ojol-terima-92</t>
+          <t>https://www.liputan6.com/news/read/8318624/bapanas-ungkap-bahaya-beras-fortifikasi-bikin-mual-hingga-anemia</t>
         </is>
       </c>
     </row>
@@ -2289,22 +2265,22 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Bareskrim Usut Dugaan Beras Fortifikasi Tak Sesuai Label</t>
+          <t>Beras Fortifikasi Medium Dijual Premium, Masyarakat Rugi Rp 89 Triliun</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Wed, 21 Oct 2026 19:14:37 +0700</t>
+          <t>Thu, 22 Oct 2026 05:20:25 +0700</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Penyidik menyita 1.194 kemasan beras dari lima merek berbeda.</t>
+          <t>Beras fortifikasi kualitas medium ditulis kualitas premium dan dijual dengan harga selangit.</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8318426/bareskrim-usut-dugaan-beras-fortifikasi-tak-sesuai-label</t>
+          <t>https://www.liputan6.com/news/read/8318622/beras-fortifikasi-medium-dijual-premium-masyarakat-rugi-rp-89-triliun</t>
         </is>
       </c>
     </row>
@@ -2316,22 +2292,22 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Kabakom Janji Sampaikan 'Suara' Buruh soal Upah hingga PHK ke Presiden</t>
+          <t>Drama Nusron Wahid: Ditunggu di Gedung KPK, Muncul di Istana</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Wed, 21 Oct 2026 19:26:38 +0700</t>
+          <t>Thu, 22 Oct 2026 05:00:00 +0700</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Kabakom pastikan pemerintah berpihak pada buruh.</t>
+          <t>Nusron Wahid akhirnya terlihat di hadapan publik setelah dua kali tidak memenuhi panggilan KPK.</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8318414/kabakom-janji-sampaikan-suara-buruh-soal-upah-hingga-phk-ke-presiden</t>
+          <t>https://www.liputan6.com/news/read/8318602/drama-nusron-wahid-ditunggu-di-gedung-kpk-muncul-di-istana</t>
         </is>
       </c>
     </row>
@@ -2343,22 +2319,22 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Jaksa Beberkan Kelemahan Eksepsi Don Ritto</t>
+          <t>Yusril: Definisi Korupsi di Indonesia 20 Tahun Stagnan</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Wed, 21 Oct 2026 18:51:22 +0700</t>
+          <t>Wed, 21 Oct 2026 23:00:08 +0700</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Jaksa menilai sebagian besar keberatan diajukan Don Ritto telah memasuki materi pokok perkara harus dibuktikan dalam persidangan.</t>
+          <t>Menko Kumham Imipas Yusril Ihza Mahendra menilai definisi korupsi di Indonesia memang perlu direformasi.</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8318409/jaksa-beberkan-kelemahan-eksepsi-don-ritto</t>
+          <t>https://www.liputan6.com/news/read/8318574/yusril-definisi-korupsi-di-indonesia-20-tahun-stagnan</t>
         </is>
       </c>
     </row>
@@ -2370,22 +2346,22 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Bakom Pastikan Pemerintah Terus Evaluasi MBG dan Perkuat Pengawasan</t>
+          <t>Pemprov DKI Gelar Simulasi Gempa Serentak, Ini Tujuannya</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Wed, 21 Oct 2026 18:33:00 +0700</t>
+          <t>Wed, 21 Oct 2026 22:20:40 +0700</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Syahganda menegaskan aspek kebersihan, penyimpanan bahan pangan, dan pengawasan menjadi bagian penting dalam evaluasi MBG.</t>
+          <t>Simulasi gempa bumi ini digelar secara serentak pada Rabu (21/10/2026) pukul 10.00 WIB.</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8318388/bakom-pastikan-pemerintah-terus-evaluasi-mbg-dan-perkuat-pengawasan</t>
+          <t>https://www.liputan6.com/news/read/8318559/pemprov-dki-gelar-simulasi-gempa-serentak-ini-tujuannya</t>
         </is>
       </c>
     </row>
@@ -2397,22 +2373,22 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Said Abdullah Soroti Kekeringan dan Kebakaran Hutan Berulang Tiap Tahun</t>
+          <t>Nurman Herin Mengaku Diperalat Penyidik, Jaksa Minta Eksepsi Ditolak</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Wed, 21 Oct 2026 18:16:01 +0700</t>
+          <t>Wed, 21 Oct 2026 22:13:50 +0700</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Menurut Said, Karhutla dan kekeringan saling berhubungan. Hutan adalah penyangga kehidupan dan daerah tangkapan air.</t>
+          <t>Jaksa meminta majelis hakim menolak eksepsi terdakwa Nurman Herin di kasus korupsi dan TPPU Febrie Adriansyah.</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8318374/said-abdullah-soroti-kekeringan-dan-kebakaran-hutan-berulang-tiap-tahun</t>
+          <t>https://www.liputan6.com/news/read/8318552/nurman-herin-mengaku-diperalat-penyidik-jaksa-minta-eksepsi-ditolak</t>
         </is>
       </c>
     </row>
@@ -2424,22 +2400,22 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Apresiasi Transformasi Pertanian Mentan Amran, Wakil Ketua Komisi IV DPR Soroti Mekanisasi hingga Harga Gabah</t>
+          <t>Komitmen Pemrakarsa 98 Resolution Network Mengawal Pemerintah Prabowo-Gibran</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Wed, 21 Oct 2026 18:08:51 +0700</t>
+          <t>Wed, 21 Oct 2026 23:56:53 +0700</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Hanan A Rozak menyoroti peran mekanisasi, pupuk bersubsidi, irigasi, dan kebijakan harga dalam mendukung produksi serta swasembada pangan.</t>
+          <t>Pemrakarsa 98 Resolution Network menegaskan dua tahun pemerintahan Prabowo menjadi momentum memperkuat demokrasi ekonomi.</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8318371/apresiasi-transformasi-pertanian-mentan-amran-wakil-ketua-komisi-iv-dpr-soroti-mekanisasi-hingga-harga-gabah</t>
+          <t>https://www.liputan6.com/news/read/8318596/komitmen-pemrakarsa-98-resolution-network-mengawal-pemerintah-prabowo-gibran</t>
         </is>
       </c>
     </row>
@@ -2451,22 +2427,22 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Kapolri Buka Suara Penyidikan Kasus Polisi Tembak Polisi</t>
+          <t>Prabowo: Perbedaan dan Kritik Perlu, Tapi Persatuan Harus Dijaga</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Wed, 21 Oct 2026 18:19:30 +0700</t>
+          <t>Wed, 21 Oct 2026 23:28:47 +0700</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Motif penembakan masih misteri.</t>
+          <t>Presiden Prabowo menegaskan komitmennya menjalankan politik persatuan nasional dengan merangkul seluruh kekuatan.</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8318368/kapolri-buka-suara-penyidikan-kasus-polisi-tembak-polisi</t>
+          <t>https://www.liputan6.com/news/read/8318546/prabowo-perbedaan-dan-kritik-perlu-tapi-persatuan-harus-dijaga</t>
         </is>
       </c>
     </row>
@@ -2478,22 +2454,22 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Prabowo Jawab Kritik Kabinet Gemuk</t>
+          <t>Pramono Harap Jakarta Makin Berprestasi Jelang Usia 500 Tahun</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Wed, 21 Oct 2026 18:06:23 +0700</t>
+          <t>Wed, 21 Oct 2026 22:41:54 +0700</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Prabowo menanggapi kritik terhadap jumlah anggota Kabinet Merah Putih yang dinilai terlalu besar dan tidak efisien.</t>
+          <t>Gubernur DKI Jakarta Pramono Anung meminta masyarakat terus meningkatkan prestasi dan menjaga kerukunan.</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8318367/prabowo-jawab-kritik-kabinet-gemuk</t>
+          <t>https://www.liputan6.com/news/read/8318541/pramono-harap-jakarta-makin-berprestasi-jelang-usia-500-tahun</t>
         </is>
       </c>
     </row>
@@ -2505,22 +2481,22 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Ancaman Prabowo ke Korporasi Terlibat Kebakaran Hutan</t>
+          <t>Bahas Politik Luar Negeri, Prabowo Usung Good Neighbor Policy</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Wed, 21 Oct 2026 17:45:00 +0700</t>
+          <t>Wed, 21 Oct 2026 22:13:19 +0700</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Prabowo menuturkan, berdasarkan hasil penyelidikan di lapangan, fenomena karhutla tidak semata-mata alamiah, namun juga ada campur tangan manusia.</t>
+          <t>Indonesia berupaya membangun kerja sama dengan berbagai negara dan menjaga hubungan baik.</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8318352/ancaman-prabowo-ke-korporasi-terlibat-kebakaran-hutan</t>
+          <t>https://www.liputan6.com/news/read/8318525/bahas-politik-luar-negeri-prabowo-usung-good-neighbor-policy</t>
         </is>
       </c>
     </row>
@@ -2532,22 +2508,22 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Finger Heart Rocky Gerung untuk Dua Tahun Prabowo-Gibran</t>
+          <t>11 Korporasi Jadi Tersangka Kebakaran Hutan, 3 Perusahaan Asing</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Wed, 21 Oct 2026 17:39:35 +0700</t>
+          <t>Wed, 21 Oct 2026 21:42:18 +0700</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Rocky menyampaikan penilaian tersebut saat menghadiri sidang kabinet paripurna di Istana.</t>
+          <t>Kapolri menegaskan penyidik tidak menghadapi kendala dalam menangani kasus tersebut.</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8318349/finger-heart-rocky-gerung-untuk-dua-tahun-prabowo-gibran</t>
+          <t>https://www.liputan6.com/news/read/8318536/11-korporasi-jadi-tersangka-kebakaran-hutan-3-perusahaan-asing</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data pasar & berita - 2026-10-22 13:39 UTC
</commit_message>
<xml_diff>
--- a/data/market_news_latest.xlsx
+++ b/data/market_news_latest.xlsx
@@ -422,7 +422,7 @@
     <col width="26" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
   </cols>
@@ -487,20 +487,20 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>5278.8882</v>
+        <v>5387.9048</v>
       </c>
       <c r="F2" t="n">
-        <v>282.2793</v>
+        <v>59.5449</v>
       </c>
       <c r="G2" t="n">
-        <v>5.65</v>
+        <v>1.12</v>
       </c>
       <c r="H2" t="n">
-        <v>534990700</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -521,20 +521,20 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>7757.1699</v>
+        <v>7695.25</v>
       </c>
       <c r="F3" t="n">
-        <v>44.6001</v>
+        <v>-61.9199</v>
       </c>
       <c r="G3" t="n">
-        <v>0.58</v>
+        <v>-0.8</v>
       </c>
       <c r="H3" t="n">
-        <v>2889474000</v>
+        <v>203879799</v>
       </c>
     </row>
     <row r="4">
@@ -555,20 +555,20 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>52856.0898</v>
+        <v>52672.4102</v>
       </c>
       <c r="F4" t="n">
-        <v>360.2109</v>
+        <v>-183.6797</v>
       </c>
       <c r="G4" t="n">
-        <v>0.6899999999999999</v>
+        <v>-0.35</v>
       </c>
       <c r="H4" t="n">
-        <v>359385262</v>
+        <v>34507950</v>
       </c>
     </row>
     <row r="5">
@@ -589,20 +589,20 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>26702.8574</v>
+        <v>26325.4082</v>
       </c>
       <c r="F5" t="n">
-        <v>278.0371</v>
+        <v>-377.4512</v>
       </c>
       <c r="G5" t="n">
-        <v>1.05</v>
+        <v>-1.41</v>
       </c>
       <c r="H5" t="n">
-        <v>6898345000</v>
+        <v>1083109000</v>
       </c>
     </row>
     <row r="6">
@@ -627,13 +627,13 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>64746.4883</v>
+        <v>62907.8398</v>
       </c>
       <c r="F6" t="n">
-        <v>671.0664</v>
+        <v>-1713.3984</v>
       </c>
       <c r="G6" t="n">
-        <v>1.05</v>
+        <v>-2.65</v>
       </c>
       <c r="H6" t="n">
         <v>0</v>
@@ -657,20 +657,20 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>23867.7402</v>
+        <v>22934.6797</v>
       </c>
       <c r="F7" t="n">
-        <v>-319.0898</v>
+        <v>-717.1895</v>
       </c>
       <c r="G7" t="n">
-        <v>-1.32</v>
+        <v>-3.03</v>
       </c>
       <c r="H7" t="n">
-        <v>2650200000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -691,14 +691,20 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>3658.0256</v>
+      </c>
+      <c r="F8" t="n">
+        <v>-55.0024</v>
+      </c>
+      <c r="G8" t="n">
+        <v>-1.48</v>
+      </c>
       <c r="H8" t="n">
-        <v>3468900532</v>
+        <v>819523340</v>
       </c>
     </row>
     <row r="9">
@@ -719,20 +725,20 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>10733</v>
+        <v>10735.1201</v>
       </c>
       <c r="F9" t="n">
-        <v>-31.7002</v>
+        <v>-17.7803</v>
       </c>
       <c r="G9" t="n">
-        <v>-0.29</v>
+        <v>-0.17</v>
       </c>
       <c r="H9" t="n">
-        <v>848274600</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -753,20 +759,20 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>25304.4199</v>
+        <v>25516.6895</v>
       </c>
       <c r="F10" t="n">
-        <v>-15.3496</v>
+        <v>-128.3496</v>
       </c>
       <c r="G10" t="n">
-        <v>-0.06</v>
+        <v>-0.5</v>
       </c>
       <c r="H10" t="n">
-        <v>52913300</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -787,20 +793,20 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>5404.02</v>
+        <v>5415.1401</v>
       </c>
       <c r="F11" t="n">
-        <v>-7.98</v>
+        <v>-22.8501</v>
       </c>
       <c r="G11" t="n">
-        <v>-0.15</v>
+        <v>-0.42</v>
       </c>
       <c r="H11" t="n">
-        <v>249844900</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -855,17 +861,17 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>101.687</v>
+        <v>101.792</v>
       </c>
       <c r="F13" t="n">
-        <v>-0.043</v>
+        <v>0.012</v>
       </c>
       <c r="G13" t="n">
-        <v>-0.04</v>
+        <v>0.01</v>
       </c>
       <c r="H13" t="n">
         <v>0</v>
@@ -893,13 +899,13 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>158.185</v>
+        <v>157.269</v>
       </c>
       <c r="F14" t="n">
-        <v>-0.083</v>
+        <v>-0.999</v>
       </c>
       <c r="G14" t="n">
-        <v>-0.05</v>
+        <v>-0.63</v>
       </c>
       <c r="H14" t="n">
         <v>0</v>
@@ -923,17 +929,17 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>0.5145999999999999</v>
+        <v>0.5044</v>
       </c>
       <c r="F15" t="n">
-        <v>0.0029</v>
+        <v>-0.0102</v>
       </c>
       <c r="G15" t="n">
-        <v>0.57</v>
+        <v>-1.98</v>
       </c>
       <c r="H15" t="n">
         <v>0</v>
@@ -957,17 +963,17 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>0.5439000000000001</v>
+        <v>0.5352</v>
       </c>
       <c r="F16" t="n">
-        <v>0.0014</v>
+        <v>-0.008699999999999999</v>
       </c>
       <c r="G16" t="n">
-        <v>0.26</v>
+        <v>-1.6</v>
       </c>
       <c r="H16" t="n">
         <v>0</v>
@@ -991,17 +997,17 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>0.4063</v>
+        <v>0.404</v>
       </c>
       <c r="F17" t="n">
-        <v>-0.0017</v>
+        <v>-0.0023</v>
       </c>
       <c r="G17" t="n">
-        <v>-0.42</v>
+        <v>-0.57</v>
       </c>
       <c r="H17" t="n">
         <v>0</v>
@@ -1025,14 +1031,20 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>81</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0.95</v>
+      </c>
       <c r="H18" t="n">
-        <v>35949645</v>
+        <v>3841450</v>
       </c>
     </row>
     <row r="19">
@@ -1053,14 +1065,20 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>76.955</v>
+      </c>
+      <c r="F19" t="n">
+        <v>-0.025</v>
+      </c>
+      <c r="G19" t="n">
+        <v>-0.03</v>
+      </c>
       <c r="H19" t="n">
-        <v>35880008</v>
+        <v>2268810</v>
       </c>
     </row>
     <row r="20">
@@ -1081,20 +1099,20 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>4140.6001</v>
+        <v>4091.8999</v>
       </c>
       <c r="F20" t="n">
-        <v>-2</v>
+        <v>-58.1001</v>
       </c>
       <c r="G20" t="n">
-        <v>-0.05</v>
+        <v>-1.4</v>
       </c>
       <c r="H20" t="n">
-        <v>5102</v>
+        <v>116667</v>
       </c>
     </row>
     <row r="21">
@@ -1115,20 +1133,20 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>97.97</v>
+        <v>99.8</v>
       </c>
       <c r="F21" t="n">
-        <v>-3.82</v>
+        <v>2.65</v>
       </c>
       <c r="G21" t="n">
-        <v>-3.75</v>
+        <v>2.73</v>
       </c>
       <c r="H21" t="n">
-        <v>4424</v>
+        <v>117095</v>
       </c>
     </row>
     <row r="22">
@@ -1149,20 +1167,20 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="E22" t="n">
-        <v>109.98</v>
+        <v>112.3</v>
       </c>
       <c r="F22" t="n">
-        <v>1.19</v>
+        <v>3.48</v>
       </c>
       <c r="G22" t="n">
-        <v>1.09</v>
+        <v>3.2</v>
       </c>
       <c r="H22" t="n">
-        <v>240</v>
+        <v>19060</v>
       </c>
     </row>
     <row r="23">
@@ -1183,20 +1201,20 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="E23" t="n">
-        <v>6.558</v>
+        <v>6.439</v>
       </c>
       <c r="F23" t="n">
-        <v>-0.008500000000000001</v>
+        <v>-0.104</v>
       </c>
       <c r="G23" t="n">
-        <v>-0.13</v>
+        <v>-1.59</v>
       </c>
       <c r="H23" t="n">
-        <v>828</v>
+        <v>38078</v>
       </c>
     </row>
     <row r="24">
@@ -1217,14 +1235,20 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr"/>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr"/>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>62.25</v>
+      </c>
+      <c r="F24" t="n">
+        <v>-1.32</v>
+      </c>
+      <c r="G24" t="n">
+        <v>-2.08</v>
+      </c>
       <c r="H24" t="n">
-        <v>17733563</v>
+        <v>1373065</v>
       </c>
     </row>
     <row r="25">
@@ -1245,17 +1269,17 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="E25" t="n">
-        <v>16.68</v>
+        <v>18.07</v>
       </c>
       <c r="F25" t="n">
-        <v>-0.63</v>
+        <v>1.39</v>
       </c>
       <c r="G25" t="n">
-        <v>-3.64</v>
+        <v>8.33</v>
       </c>
       <c r="H25" t="n">
         <v>0</v>
@@ -1283,16 +1307,16 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>84169.0312</v>
+        <v>81540.0469</v>
       </c>
       <c r="F26" t="n">
-        <v>1228.0312</v>
+        <v>-2471.9219</v>
       </c>
       <c r="G26" t="n">
-        <v>1.48</v>
+        <v>-2.94</v>
       </c>
       <c r="H26" t="n">
-        <v>30698053632</v>
+        <v>38158757888</v>
       </c>
     </row>
     <row r="27">
@@ -1313,20 +1337,20 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="E27" t="n">
-        <v>1485</v>
+        <v>1440</v>
       </c>
       <c r="F27" t="n">
-        <v>50</v>
+        <v>-45</v>
       </c>
       <c r="G27" t="n">
-        <v>3.48</v>
+        <v>-3.03</v>
       </c>
       <c r="H27" t="n">
-        <v>171835800</v>
+        <v>115064900</v>
       </c>
     </row>
     <row r="28">
@@ -1347,20 +1371,20 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="E28" t="n">
         <v>1340</v>
       </c>
       <c r="F28" t="n">
-        <v>65</v>
+        <v>0</v>
       </c>
       <c r="G28" t="n">
-        <v>5.1</v>
+        <v>0</v>
       </c>
       <c r="H28" t="n">
-        <v>234603700</v>
+        <v>192500500</v>
       </c>
     </row>
     <row r="29">
@@ -1381,20 +1405,20 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="E29" t="n">
-        <v>505</v>
+        <v>496</v>
       </c>
       <c r="F29" t="n">
-        <v>0</v>
+        <v>-9</v>
       </c>
       <c r="G29" t="n">
-        <v>0</v>
+        <v>-1.78</v>
       </c>
       <c r="H29" t="n">
-        <v>453295000</v>
+        <v>486782800</v>
       </c>
     </row>
     <row r="30">
@@ -1415,20 +1439,20 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="E30" t="n">
-        <v>2160</v>
+        <v>2320</v>
       </c>
       <c r="F30" t="n">
         <v>160</v>
       </c>
       <c r="G30" t="n">
-        <v>8</v>
+        <v>7.41</v>
       </c>
       <c r="H30" t="n">
-        <v>54437200</v>
+        <v>23389400</v>
       </c>
     </row>
     <row r="31">
@@ -1449,20 +1473,20 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="E31" t="n">
-        <v>3060</v>
+        <v>3070</v>
       </c>
       <c r="F31" t="n">
-        <v>-90</v>
+        <v>10</v>
       </c>
       <c r="G31" t="n">
-        <v>-2.86</v>
+        <v>0.33</v>
       </c>
       <c r="H31" t="n">
-        <v>70704200</v>
+        <v>43534800</v>
       </c>
     </row>
     <row r="32">
@@ -1483,20 +1507,20 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="E32" t="n">
-        <v>420</v>
+        <v>424</v>
       </c>
       <c r="F32" t="n">
-        <v>-6</v>
+        <v>4</v>
       </c>
       <c r="G32" t="n">
-        <v>-1.41</v>
+        <v>0.95</v>
       </c>
       <c r="H32" t="n">
-        <v>46513200</v>
+        <v>43922700</v>
       </c>
     </row>
     <row r="33">
@@ -1517,20 +1541,20 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="E33" t="n">
-        <v>470</v>
+        <v>478</v>
       </c>
       <c r="F33" t="n">
-        <v>-14</v>
+        <v>8</v>
       </c>
       <c r="G33" t="n">
-        <v>-2.89</v>
+        <v>1.7</v>
       </c>
       <c r="H33" t="n">
-        <v>86486800</v>
+        <v>87778300</v>
       </c>
     </row>
     <row r="34">
@@ -1551,20 +1575,20 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="E34" t="n">
-        <v>2490</v>
+        <v>2520</v>
       </c>
       <c r="F34" t="n">
-        <v>-180</v>
+        <v>30</v>
       </c>
       <c r="G34" t="n">
-        <v>-6.74</v>
+        <v>1.2</v>
       </c>
       <c r="H34" t="n">
-        <v>12531700</v>
+        <v>9474800</v>
       </c>
     </row>
     <row r="35">
@@ -1585,20 +1609,20 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="E35" t="n">
-        <v>322</v>
+        <v>314</v>
       </c>
       <c r="F35" t="n">
-        <v>-24</v>
+        <v>-8</v>
       </c>
       <c r="G35" t="n">
-        <v>-6.94</v>
+        <v>-2.48</v>
       </c>
       <c r="H35" t="n">
-        <v>539236300</v>
+        <v>854759900</v>
       </c>
     </row>
     <row r="36">
@@ -1619,20 +1643,20 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="E36" t="n">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="F36" t="n">
-        <v>-2</v>
+        <v>4</v>
       </c>
       <c r="G36" t="n">
-        <v>-1.37</v>
+        <v>2.78</v>
       </c>
       <c r="H36" t="n">
-        <v>19569300</v>
+        <v>19327000</v>
       </c>
     </row>
     <row r="37">
@@ -1653,20 +1677,20 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="E37" t="n">
-        <v>9650</v>
+        <v>10000</v>
       </c>
       <c r="F37" t="n">
-        <v>-725</v>
+        <v>350</v>
       </c>
       <c r="G37" t="n">
-        <v>-6.99</v>
+        <v>3.63</v>
       </c>
       <c r="H37" t="n">
-        <v>60687900</v>
+        <v>33713400</v>
       </c>
     </row>
   </sheetData>
@@ -1725,22 +1749,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Dua Menteri Pastikan Gaji PNS Tidak Lewat Kopdes, Menkop Buka Suara</t>
+          <t>Menteri UMKM Ungkap Alasan Wajib Halal Ditunda</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Thu, 22 Oct 2026 07:00:00 +0700</t>
+          <t>Thu, 22 Oct 2026 20:30:00 +0700</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/18/17288-koperasi-desa-merah-putih-siap-beroperasi-ditargetkan-oktober-2026-1789704926087_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Keuangan dan PANRB memastikan gaji PNS tetap dibayar langsung ke rekening, bukan melalui Koperasi Desa.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/12/02/menteri-usaha-mikro-kecil-dan-menengah-umkm-maman-abdurrahman-1764677159466_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Usaha Mikro Kecil dan Menengah (UMKM) Maman Abdurrahman menyampaikan alasan kewajiban sertifikasi halal diundur menja</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8718189/dua-menteri-pastikan-gaji-pns-tidak-lewat-kopdes-menkop-buka-suara</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8719637/menteri-umkm-ungkap-alasan-wajib-halal-ditunda</t>
         </is>
       </c>
     </row>
@@ -1752,22 +1776,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Cihuy! DP 0% Rumah &amp;amp; Kendaraan Masih Lanjut</t>
+          <t>Bank Mandiri Tingkatkan Layanan Digital untuk Dorong Pertumbuhan Bisnis</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Thu, 22 Oct 2026 06:25:00 +0700</t>
+          <t>Thu, 22 Oct 2026 20:06:47 +0700</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/21/bank-indonesia-bi-memutuskan-menaikkan-suku-bunga-deposit-facility-sebesar-25-basis-poin-bps-menjadi-5-keputusan-tersebut-diam-1792576096825_169.jpeg?w=360&amp;amp;q=90" /&gt; Bank Indonesia (BI) memperpanjang kebijakan uang muka atau d</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/22/bank-mandiri-1792674027427.png?w=360&amp;amp;q=90" /&gt; Bank Mandiri terus tingkatkan layanan untuk memenuhi ekspektasi nasabah. Fokus pada pengalaman pelanggan dan integrasi layanan digital dalam satu aplikasi.</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/moneter/d-8717984/cihuy-dp-0-rumah-kendaraan-masih-lanjut</t>
+          <t>https://finance.detik.com/moneter/d-8719674/bank-mandiri-tingkatkan-layanan-digital-untuk-dorong-pertumbuhan-bisnis</t>
         </is>
       </c>
     </row>
@@ -1779,22 +1803,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Prabowo Beri Pesan Keras buat MSCI</t>
+          <t>Anggaran Rekening Gratis Turun dari Rp 3,84 T Jadi Rp 1,28 T</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Thu, 22 Oct 2026 05:55:09 +0700</t>
+          <t>Thu, 22 Oct 2026 20:00:20 +0700</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/21/sidang-kabinet-paripurna-di-istana-kepresidenan-1792580318733_169.jpeg?w=360&amp;amp;q=90" /&gt; Pesan keras disampaikan Presiden Prabowo Subianto kepada MSCI.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/10/27/bi-pertahankan-bi-rate-475-persen-untuk-jaga-stabilitas-rupiah-1761539775425_169.jpeg?w=360&amp;amp;q=90" /&gt; Pemerintah mengubah anggaran program rekening gratis dari Rp 3,84 triliun menjadi Rp 1,28 triliun, hal ini dilakukan setelah</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/bursa-dan-valas/d-8717980/prabowo-beri-pesan-keras-buat-msci</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8719657/anggaran-rekening-gratis-turun-dari-rp-3-84-t-jadi-rp-1-28-t</t>
         </is>
       </c>
     </row>
@@ -1806,22 +1830,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Saat Pembayaran QRIS Telah Melintasi Batas Negara</t>
+          <t>UMK Lokal Dapat Diskon 50% Biaya Administrasi Toko Online Selamanya</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Thu, 22 Oct 2026 00:00:00 +0700</t>
+          <t>Thu, 22 Oct 2026 20:00:17 +0700</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/21/adv-1792558313107.jpeg?w=360&amp;amp;q=90" /&gt; Saat Pembayaran QRIS Telah Melintasi Batas Negara</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/22/menteri-usaha-mikro-kecil-dan-menengah-umkm-maman-abdurrahman-1792667292505_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri UMKM Maman Abdurrahman menyampaikan kebijakan ini akan berlaku secara permanen.</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/advertorial-news-block/d-8716941/saat-pembayaran-qris-telah-melintasi-batas-negara</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8719617/umk-lokal-dapat-diskon-50-biaya-administrasi-toko-online-selamanya</t>
         </is>
       </c>
     </row>
@@ -1833,22 +1857,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Rp 31,8 Triliun Disiapkan buat BSU, Beras 10 Kg, hingga Diskon Nataru</t>
+          <t>Putri Tanjung Bicara Pentingnya Ekosistem Kreatif yang Sehat</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Wed, 21 Oct 2026 23:00:36 +0700</t>
+          <t>Thu, 22 Oct 2026 19:31:06 +0700</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/13/ilustrasi-bsu-2026-1791879636208_169.jpeg?w=360&amp;amp;q=90" /&gt; Pemerintah menyiapkan 4 program andalan</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/22/putri-tanjung-bicara-pentingnya-ekosistem-kreatif-yang-sehat-1792672229786_43.jpeg?w=360&amp;amp;q=90" /&gt; Putri Tanjung dorong penguatan ekosistem ekonomi kreatif Indonesia agar IP lokal bersaing global. Kolaborasi penting untuk kemb</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8718185/rp-31-8-triliun-disiapkan-buat-bsu-beras-10-kg-hingga-diskon-nataru</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8719633/putri-tanjung-bicara-pentingnya-ekosistem-kreatif-yang-sehat</t>
         </is>
       </c>
     </row>
@@ -1860,22 +1884,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Bos Otorita Pastikan Tak Ada Korporasi Terlibat Karhutla Sekitar Kawasan IKN</t>
+          <t>OJK Ungkap Progres Demutualisasi Bursa: BEI Gelar RUPS Akhir Oktober 2026</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Wed, 21 Oct 2026 22:55:00 +0700</t>
+          <t>Thu, 22 Oct 2026 19:30:11 +0700</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/11/04/kepala-otorita-ikn-basuki-hadimuljono-1762234920793_169.jpeg?w=360&amp;amp;q=90" /&gt; Kepala OIKN Basuki Hadimuljono memastikan tidak ada indikasi keterlibatan korporasi dalam kebakaran hutan dan lahan (karhutla) di sekitar kawasan IKN</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2016/12/30/ed5ec33a-5357-40f8-8f66-6713c06687ea_169.jpg?w=360&amp;amp;q=90" /&gt; OJK mengungkap progres demutualisasi BEI, dengan RUPS dijadwalkan pada 28 Oktober 2026 untuk membahas perubahan anggaran dasar dan langkah selanjutnya.</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/infrastruktur/d-8718175/bos-otorita-pastikan-tak-ada-korporasi-terlibat-karhutla-sekitar-kawasan-ikn</t>
+          <t>https://finance.detik.com/moneter/d-8719551/ojk-ungkap-progres-demutualisasi-bursa-bei-gelar-rups-akhir-oktober-2026</t>
         </is>
       </c>
     </row>
@@ -1887,22 +1911,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Tips Menghindari Penipuan Berkedok Rekrutmen untuk Para Jobseekers</t>
+          <t>BRI Siapkan Buyback Saham Tahap II Senilai Rp 1 Triliun</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Wed, 21 Oct 2026 22:48:08 +0700</t>
+          <t>Thu, 22 Oct 2026 19:12:42 +0700</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/21/tips-menghindari-penipuan-berkedok-rekrutmen-untuk-para-jobseekers-1792597627341.jpeg?w=360&amp;amp;q=90" /&gt; Di era digital, penipuan rekrutmen semakin marak. Direktur Pegadaian berbagi tips untuk jobseeker agar terhindar dari penipu</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/22/ilustrasi-gedung-bri-1792671138276.jpeg?w=360&amp;amp;q=90" /&gt; PT BRI umumkan rencana buyback saham Tahap II senilai Rp 1 triliun. Aksi ini bertujuan tingkatkan nilai pemegang saham dan dukung pertumbuhan jangka panjang.</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/lainnya/d-8718172/tips-menghindari-penipuan-berkedok-rekrutmen-untuk-para-jobseekers</t>
+          <t>https://finance.detik.com/bursa-dan-valas/d-8719613/bri-siapkan-buyback-saham-tahap-ii-senilai-rp-1-triliun</t>
         </is>
       </c>
     </row>
@@ -1914,22 +1938,22 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Karhutla di Sekitar Kawasan IKN 1.600 Ha Padam, Tidak Ganggu Proyek</t>
+          <t>Kementan Dorong Hilirisasi Hortikultura Lewat Inovasi KWT di Lombok</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Wed, 21 Oct 2026 22:42:37 +0700</t>
+          <t>Thu, 22 Oct 2026 19:11:30 +0700</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/08/15/kawasan-inti-pusat-pemerintahan-ibu-kota-nusantara-ikn-1786797746713_169.jpeg?w=360&amp;amp;q=90" /&gt; Otorita Ibu Kota Nusantara memastikan insiden kebakaran hutan dan lahan kurang lebih 1.600 hektare di sekitar kawasan IKN telah berh</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/22/kementan-dorong-hilirisasi-hortikultura-lewat-inovasi-kwt-di-lombok-1792671077202.jpeg?w=360&amp;amp;q=90" /&gt; Kementan dorong hilirisasi hortikultura melalui pengembangan produk olahan lokal. KWT Sasak Maiq jadi contoh sukses dalam m</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/infrastruktur/d-8718166/karhutla-di-sekitar-kawasan-ikn-1-600-ha-padam-tidak-ganggu-proyek</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8719610/kementan-dorong-hilirisasi-hortikultura-lewat-inovasi-kwt-di-lombok</t>
         </is>
       </c>
     </row>
@@ -1941,22 +1965,22 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Megaproyek IKN Tetap Jalan, Investasi Rp 4 Triliun Baru Masuk</t>
+          <t>336 Investor Asing Colek OJK Usai MSCI Buka Opsi Bursa RI Turun Kasta</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Wed, 21 Oct 2026 22:21:05 +0700</t>
+          <t>Thu, 22 Oct 2026 19:00:35 +0700</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2024/12/10/kepala-otorita-ikn-basuki-hadimuljono_169.jpeg?w=360&amp;amp;q=90" /&gt; Pembangunan infrastruktur strategis di kawasan megaproyek Ibu Kota Nusantara (IKN), Kalimantan Timur terus berjalan.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/06/04/ihsg-terpuruk-kekhawatiran-pasar-meningkat-1780558039793_169.jpeg?w=360&amp;amp;q=90" /&gt; Sebanyak 336 investor asing meminta klarifikasi OJK dan BEI terkait pengumuman MSCI.</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/infrastruktur/d-8718134/megaproyek-ikn-tetap-jalan-investasi-rp-4-triliun-baru-masuk</t>
+          <t>https://finance.detik.com/bursa-dan-valas/d-8719580/336-investor-asing-colek-ojk-usai-msci-buka-opsi-bursa-ri-turun-kasta</t>
         </is>
       </c>
     </row>
@@ -1968,22 +1992,22 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Bahlil Buka Opsi Setop Ekspor Gas ke Negara Tetangga</t>
+          <t>Penyaluran KUR Tembus Rp 260 T ke 4 Juta Debitur</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Wed, 21 Oct 2026 21:58:32 +0700</t>
+          <t>Thu, 22 Oct 2026 19:00:28 +0700</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/08/04/bahlil-lahadalia-1785840108228_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Energi dan Sumber Daya Mineral (ESDM) Bahlil Lahadalia membuka opsi setop ekspor gas ke negara tetangga.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/22/menteri-usaha-mikro-kecil-dan-menengah-umkm-maman-abdurrahman-1792667292505_169.jpeg?w=360&amp;amp;q=90" /&gt; Kementerian Usaha Mikro Kecil dan Menengah (UMKM) melaporkan realisasi penyaluran kredit usaha rakyat (KUR) mencapai Rp 260,8</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8718097/bahlil-buka-opsi-setop-ekspor-gas-ke-negara-tetangga</t>
+          <t>https://finance.detik.com/moneter/d-8719524/penyaluran-kur-tembus-rp-260-t-ke-4-juta-debitur</t>
         </is>
       </c>
     </row>
@@ -1995,22 +2019,22 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Terbongkar Pihak-pihak di Balik Kasus Saham DSSA, BREN, dan CUAN</t>
+          <t>Bayan Buka Suara Sahamnya Diborong Haji Isam di Harga Murah</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Wed, 21 Oct 2026 21:32:53 +0700</t>
+          <t>Thu, 22 Oct 2026 18:31:25 +0700</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/05/18/ihsg-anjlok-ke-zona-merah-bursa-saham-melemah-tajam-1779098741437_169.jpeg?w=360&amp;amp;q=90" /&gt; OJK menjatuhkan denda kepada tiga emiten di pasar modal Indonesia, yakni DSSA, BREN, dan CUAN.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/16/ihsg-ambruk-1157-ditutup-di-level-5185-1792144638880_169.jpeg?w=360&amp;amp;q=90" /&gt; PT Bayan Resources buka suara sahamnya diborong murah oleh Haji Isam.</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/bursa-dan-valas/d-8718072/terbongkar-pihak-pihak-di-balik-kasus-saham-dssa-bren-dan-cuan</t>
+          <t>https://finance.detik.com/bursa-dan-valas/d-8719560/bayan-buka-suara-sahamnya-diborong-haji-isam-di-harga-murah</t>
         </is>
       </c>
     </row>
@@ -2022,22 +2046,22 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Bima Arya: Mengejar Pertumbuhan Ekonomi Harus Peduli pada Lingkungan</t>
+          <t>WIKA Bakal Siapkan Layanan Avtur Terintegrasi di Bandara Kertajati</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Wed, 21 Oct 2026 21:23:46 +0700</t>
+          <t>Thu, 22 Oct 2026 18:30:33 +0700</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/21/wakil-menteri-dalam-negeri-wamendagri-bima-arya-sugiarto-1792592599172.jpeg?w=360&amp;amp;q=90" /&gt; Wamendagri Bima Arya dorong Pemda selaraskan pertumbuhan ekonomi dengan pelestarian lingkungan. Pentingnya partisipasi masyarakat dan </t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/22/wika-finalisasi-commissioning-aft-kertajati-siapkan-layanan-avtur-terintegrasi-di-bandara-kertajati-1792668571401.jpeg?w=360&amp;amp;q=90" /&gt; PT Wijaya Karya (WIKA) hampir menyelesaikan commissioning Aviation Fuel Terminal di Kertaja</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8718060/bima-arya-mengejar-pertumbuhan-ekonomi-harus-peduli-pada-lingkungan</t>
+          <t>https://finance.detik.com/infrastruktur/d-8719559/wika-bakal-siapkan-layanan-avtur-terintegrasi-di-bandara-kertajati</t>
         </is>
       </c>
     </row>
@@ -2049,22 +2073,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Harga Minyak Meroket, Pertalite Dipastikan Tidak Naik</t>
+          <t>bank bjb Ajak Masyarakat Ikuti Semarang 10K, Cuma Nabung Bisa Dapat Tiket</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Wed, 21 Oct 2026 21:03:01 +0700</t>
+          <t>Thu, 22 Oct 2026 17:44:44 +0700</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/08/20/pemerintah-perketat-penyaluran-pertalite-mulai-2027-1787210254552_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Energi dan Sumber Daya Mineral (ESDM) Bahlil Lahadalia menegaskan pemerintah tidak menaikkan harga bahan bakar minyak (BBM) sub</t>
+          <t xml:space="preserve">&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/22/bank-bjb-ajak-masyarakat-ikuti-semarang-10k-cuma-nabung-bisa-dapat-tiket-1792665852462.jpeg?w=360&amp;amp;q=90" /&gt; Bank bjb luncurkan program promo Semarang 10K 2026, menggabungkan gaya hidup sehat dan perencanaan keuangan. Dapatkan </t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8718032/harga-minyak-meroket-pertalite-dipastikan-tidak-naik</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8719477/bank-bjb-ajak-masyarakat-ikuti-semarang-10k-cuma-nabung-bisa-dapat-tiket</t>
         </is>
       </c>
     </row>
@@ -2076,22 +2100,22 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Prabowo: Prestasi Kita Paling Utama Swasembada Pangan dalam Waktu Cepat</t>
+          <t>bank bjb Raih Pengakuan Top 50 Emiten MidCap dalam IICD CG Award 2026</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Wed, 21 Oct 2026 20:59:39 +0700</t>
+          <t>Thu, 22 Oct 2026 17:35:40 +0700</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/21/presiden-prabowo-subianto-1792590961666.jpeg?w=360&amp;amp;q=90" /&gt; Presiden Prabowo menegaskan swasembada pangan sebagai prestasi utama pemerintah. Indonesia siap hadapi tantangan global dengan kemandirian pangan yang kuat.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/22/bank-bjb-raih-pengakuan-top-50-emiten-midcap-dalam-iicd-cg-award-2026-1792664414280_43.jpeg?w=360&amp;amp;q=90" /&gt; bank bjb meraih penghargaan GCG dari IICD sebagai Top 50 Emiten MidCap. Pengakuan ini memperkuat komitmen bank dalam m</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8718025/prabowo-prestasi-kita-paling-utama-swasembada-pangan-dalam-waktu-cepat</t>
+          <t>https://finance.detik.com/moneter/d-8719434/bank-bjb-raih-pengakuan-top-50-emiten-midcap-dalam-iicd-cg-award-2026</t>
         </is>
       </c>
     </row>
@@ -2103,22 +2127,22 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Krisis Gas di Taiz Yaman Memaksa Warga Antre Berjam-jam</t>
+          <t>Pencari Kerja Berburu 12 Ribu Lowongan di Karir Jakarta Expo 2026</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Wed, 21 Oct 2026 20:53:03 +0700</t>
+          <t>Thu, 22 Oct 2026 17:30:45 +0700</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/21/krisis-gas-di-taiz-yaman-memaksa-warga-antre-berjam-jam-1792560778171.jpeg?w=360&amp;amp;q=90" /&gt; Warga Taiz di Yaman mengantre berjam-jam untuk mendapatkan gas memasak. Krisis pasokan kian memburuk imbas pengepungan dan penutupan ja</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/22/pencari-kerja-berburu-12-ribu-lowongan-di-karir-jakarta-expo-2026-1792655486514.jpeg?w=360&amp;amp;q=90" /&gt; Pemprov DKI Jakarta menggelar Karir Jakarta Expo 2026 di SMESCO. Bursa kerja gratis ini menyediakan 12 ribu lowongan dari rat</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/foto-bisnis/d-8717050/krisis-gas-di-taiz-yaman-memaksa-warga-antre-berjam-jam</t>
+          <t>https://finance.detik.com/foto-bisnis/d-8719100/pencari-kerja-berburu-12-ribu-lowongan-di-karir-jakarta-expo-2026</t>
         </is>
       </c>
     </row>
@@ -2130,22 +2154,22 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>DPR Ingatkan Timsel KPU Sudah Bisa Dibentuk Tanpa Tunggu RUU Pemilu</t>
+          <t>Kemendagri Minta Pemda Evaluasi Aturan yang Bebani Warga</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Thu, 22 Oct 2026 06:40:39 +0700</t>
+          <t>Thu, 22 Oct 2026 20:36:21 +0700</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Pembentukan timsel KPU periode berikutnya dapat dimulai tanpa menunggu RUU Pemilu.</t>
+          <t>Sejumlah tahapan perlu dikaji agar dapat dilaksanakan secara paralel sehingga pelayanan menjadi lebih sederhana, cepat, dan efisien.</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8318626/dpr-ingatkan-timsel-kpu-sudah-bisa-dibentuk-tanpa-tunggu-ruu-pemilu</t>
+          <t>https://www.liputan6.com/news/read/8319345/kemendagri-minta-pemda-evaluasi-aturan-yang-bebani-warga</t>
         </is>
       </c>
     </row>
@@ -2157,22 +2181,22 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Resolusi Jihad dan Api Perlawanan dari Pesantren</t>
+          <t>Santri Tak Cuma Soal Sarung dan Kitab Kuning</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Thu, 22 Oct 2026 06:34:29 +0700</t>
+          <t>Thu, 22 Oct 2026 20:05:19 +0700</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Resolusi Jihad 22 Oktober 1945 menjadi salah satu pemantik perlawanan ulama dan santri dalam mempertahankan kemerdekaan Indonesia.</t>
+          <t>Santri masa kini tak hanya belajar agama, tetapi juga mengembangkan diri untuk menghadapi tantangan zaman.</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8317894/resolusi-jihad-dan-api-perlawanan-dari-pesantren</t>
+          <t>https://www.liputan6.com/news/read/8319318/santri-tak-cuma-soal-sarung-dan-kitab-kuning</t>
         </is>
       </c>
     </row>
@@ -2184,22 +2208,22 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Belanja APBD Jakarta 2026 Baru Terserap 54,39 Persen, Pramono Ingatkan Jajarannya</t>
+          <t>Pria Tanpa Identitas Ditemukan Tewas di Warung Kosong Bekasi</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Thu, 22 Oct 2026 06:21:52 +0700</t>
+          <t>Thu, 22 Oct 2026 19:59:45 +0700</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Pramono Anung meminta perangkat daerah mempercepat kegiatan APBD 2026. Hingga akhir September, realisasi belanja Jakarta baru mencapai 54,39 persen dari pagu Rp 74,29 triliun.</t>
+          <t>Saksi sempat mencium bau tak sedap beberapa hari sebelumnya.</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8318625/belanja-apbd-jakarta-2026-baru-terserap-5439-persen-pramono-ingatkan-jajarannya</t>
+          <t>https://www.liputan6.com/news/read/8319326/pria-tanpa-identitas-ditemukan-tewas-di-warung-kosong-bekasi</t>
         </is>
       </c>
     </row>
@@ -2211,22 +2235,22 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2 TNI Aktif di Pusaran Korupsi Dana Bencana BNPB</t>
+          <t>Momen Haru Hari Santri, Siswa Sekolah Rakyat Ungkap Mimpi Lewat Puisi</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Thu, 22 Oct 2026 06:06:10 +0700</t>
+          <t>Thu, 22 Oct 2026 19:35:00 +0700</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>KPK menggandeng Puspom TNI dalam penanganan perkara.</t>
+          <t>Siswa Sekolah Rakyat Terintegrasi 1 Jombang melafalkan bait demi bait puisi dipersembahkan dalam rangka memperingati Hari Santri Nasional 2026.</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8318601/2-tni-aktif-di-pusaran-korupsi-dana-bencana-bnpb</t>
+          <t>https://www.liputan6.com/news/read/8319308/momen-haru-hari-santri-siswa-sekolah-rakyat-ungkap-mimpi-lewat-puisi</t>
         </is>
       </c>
     </row>
@@ -2238,22 +2262,22 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Bapanas Ungkap Bahaya Beras Fortifikasi, Bikin Mual hingga Anemia</t>
+          <t>Prabowo soal Kebakaran Hutan: Ada Negara Mengolok-olok, Kita Cool Saja</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Thu, 22 Oct 2026 05:42:37 +0700</t>
+          <t>Thu, 22 Oct 2026 19:00:39 +0700</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Beras fortifikasi mengandung Zinc yang berlebihan. Di pasaran beras fortifiksi medium sempat beredar bahkan dengan label premium.</t>
+          <t>Padahal, kata Prabowo, perusahaan-perusahaan dari negara itu ikut terlibat dan bertanggung jawab atas karhutla.</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8318624/bapanas-ungkap-bahaya-beras-fortifikasi-bikin-mual-hingga-anemia</t>
+          <t>https://www.liputan6.com/news/read/8319290/prabowo-soal-kebakaran-hutan-ada-negara-mengolok-olok-kita-cool-saja</t>
         </is>
       </c>
     </row>
@@ -2265,22 +2289,22 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Beras Fortifikasi Medium Dijual Premium, Masyarakat Rugi Rp 89 Triliun</t>
+          <t>Prabowo: Saya Malu jadi Presiden Kalau Rakyat Miskin Terus</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Thu, 22 Oct 2026 05:20:25 +0700</t>
+          <t>Thu, 22 Oct 2026 18:53:07 +0700</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Beras fortifikasi kualitas medium ditulis kualitas premium dan dijual dengan harga selangit.</t>
+          <t>Prabowo berjanji akan lebih banyak menyalurkan alokasi anggaran ke daerah.</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8318622/beras-fortifikasi-medium-dijual-premium-masyarakat-rugi-rp-89-triliun</t>
+          <t>https://www.liputan6.com/news/read/8319287/prabowo-saya-malu-jadi-presiden-kalau-rakyat-miskin-terus</t>
         </is>
       </c>
     </row>
@@ -2292,22 +2316,22 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Drama Nusron Wahid: Ditunggu di Gedung KPK, Muncul di Istana</t>
+          <t>Kronologi Kecelakaan Maut Mobilio Tabrak Pikap di Rasuna Said</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Thu, 22 Oct 2026 05:00:00 +0700</t>
+          <t>Thu, 22 Oct 2026 18:24:54 +0700</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Nusron Wahid akhirnya terlihat di hadapan publik setelah dua kali tidak memenuhi panggilan KPK.</t>
+          <t>Polisi menduga kecelakaan yang terjadi pada dini hari tersebut dipicu oleh kecepatan tinggi Mobilio.</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8318602/drama-nusron-wahid-ditunggu-di-gedung-kpk-muncul-di-istana</t>
+          <t>https://www.liputan6.com/news/read/8319262/kronologi-kecelakaan-maut-mobilio-tabrak-pikap-di-rasuna-said</t>
         </is>
       </c>
     </row>
@@ -2319,22 +2343,22 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Yusril: Definisi Korupsi di Indonesia 20 Tahun Stagnan</t>
+          <t>Kronologi 45 WNA Diciduk Petugas Imigrasi di Apartemen Kalibata City</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Wed, 21 Oct 2026 23:00:08 +0700</t>
+          <t>Thu, 22 Oct 2026 18:21:55 +0700</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Menko Kumham Imipas Yusril Ihza Mahendra menilai definisi korupsi di Indonesia memang perlu direformasi.</t>
+          <t>Dalam operasi tersebut, petugas mengamankan 45 WNA untuk menjalani pemeriksaan lebih lanjut di Ditjen Imigrasi.</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8318574/yusril-definisi-korupsi-di-indonesia-20-tahun-stagnan</t>
+          <t>https://www.liputan6.com/news/read/8319261/kronologi-45-wna-diciduk-petugas-imigrasi-di-apartemen-kalibata-city</t>
         </is>
       </c>
     </row>
@@ -2346,22 +2370,22 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Pemprov DKI Gelar Simulasi Gempa Serentak, Ini Tujuannya</t>
+          <t>Gempa Magnitudo 5,2 Guncang Bengkulu</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Wed, 21 Oct 2026 22:20:40 +0700</t>
+          <t>Thu, 22 Oct 2026 18:11:53 +0700</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Simulasi gempa bumi ini digelar secara serentak pada Rabu (21/10/2026) pukul 10.00 WIB.</t>
+          <t>Gempa bumi magnitudo 5,2 terjadi di 6 km Barat Laut Lebong, Bengkulu, tanpa potensi tsunami.</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8318559/pemprov-dki-gelar-simulasi-gempa-serentak-ini-tujuannya</t>
+          <t>https://www.liputan6.com/news/read/8319252/gempa-magnitudo-52-guncang-bengkulu</t>
         </is>
       </c>
     </row>
@@ -2373,22 +2397,22 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Nurman Herin Mengaku Diperalat Penyidik, Jaksa Minta Eksepsi Ditolak</t>
+          <t>Pramono Targetkan Pengangguran Jakarta Turun jadi 3,5 Persen</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Wed, 21 Oct 2026 22:13:50 +0700</t>
+          <t>Thu, 22 Oct 2026 17:55:15 +0700</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Jaksa meminta majelis hakim menolak eksepsi terdakwa Nurman Herin di kasus korupsi dan TPPU Febrie Adriansyah.</t>
+          <t>Jika angka pengangguran Jakarta turun, Pramono berharap jadi contoh daerah lain.</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8318552/nurman-herin-mengaku-diperalat-penyidik-jaksa-minta-eksepsi-ditolak</t>
+          <t>https://www.liputan6.com/news/read/8319238/pramono-targetkan-pengangguran-jakarta-turun-jadi-35-persen</t>
         </is>
       </c>
     </row>
@@ -2400,22 +2424,22 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Komitmen Pemrakarsa 98 Resolution Network Mengawal Pemerintah Prabowo-Gibran</t>
+          <t>Prabowo Pimpin Langsung Dewan Nasional Kesejahteraan Keuangan</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Wed, 21 Oct 2026 23:56:53 +0700</t>
+          <t>Thu, 22 Oct 2026 17:41:20 +0700</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Pemrakarsa 98 Resolution Network menegaskan dua tahun pemerintahan Prabowo menjadi momentum memperkuat demokrasi ekonomi.</t>
+          <t>Presiden Prabowo meresmikan pembentukan Dewan Nasional Kesejahteraan Keuangan pada Kamis (22/10/2026).</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8318596/komitmen-pemrakarsa-98-resolution-network-mengawal-pemerintah-prabowo-gibran</t>
+          <t>https://www.liputan6.com/news/read/8319226/prabowo-pimpin-langsung-dewan-nasional-kesejahteraan-keuangan</t>
         </is>
       </c>
     </row>
@@ -2427,22 +2451,22 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Prabowo: Perbedaan dan Kritik Perlu, Tapi Persatuan Harus Dijaga</t>
+          <t>Prabowo: Banyak Perusahaan Asing Harus Bertanggung Jawab Kebakaran Hutan</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Wed, 21 Oct 2026 23:28:47 +0700</t>
+          <t>Thu, 22 Oct 2026 17:21:09 +0700</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Presiden Prabowo menegaskan komitmennya menjalankan politik persatuan nasional dengan merangkul seluruh kekuatan.</t>
+          <t>Presiden Prabowo mengancam akan mencabut izin konsesi perusahaan yang berulang kali melanggar aturan.</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8318546/prabowo-perbedaan-dan-kritik-perlu-tapi-persatuan-harus-dijaga</t>
+          <t>https://www.liputan6.com/news/read/8319215/prabowo-banyak-perusahaan-asing-harus-bertanggung-jawab-kebakaran-hutan</t>
         </is>
       </c>
     </row>
@@ -2454,22 +2478,22 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Pramono Harap Jakarta Makin Berprestasi Jelang Usia 500 Tahun</t>
+          <t>Hari Santri 2026, Prabowo Ungkap Peran Pesantren dalam Kemerdekaan Indonesia</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Wed, 21 Oct 2026 22:41:54 +0700</t>
+          <t>Thu, 22 Oct 2026 16:32:45 +0700</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Gubernur DKI Jakarta Pramono Anung meminta masyarakat terus meningkatkan prestasi dan menjaga kerukunan.</t>
+          <t>Prabowo berharap para santri dan santriwati semakin kompak dan hebat.</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8318541/pramono-harap-jakarta-makin-berprestasi-jelang-usia-500-tahun</t>
+          <t>https://www.liputan6.com/news/read/8319177/hari-santri-2026-prabowo-ungkap-peran-pesantren-dalam-kemerdekaan-indonesia</t>
         </is>
       </c>
     </row>
@@ -2481,22 +2505,22 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Bahas Politik Luar Negeri, Prabowo Usung Good Neighbor Policy</t>
+          <t>Tahun Depan, Warga Jakarta Bisa Naik Transportasi Gratis untuk Cari Kerja</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Wed, 21 Oct 2026 22:13:19 +0700</t>
+          <t>Thu, 22 Oct 2026 16:25:04 +0700</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Indonesia berupaya membangun kerja sama dengan berbagai negara dan menjaga hubungan baik.</t>
+          <t>Pencari kerja bakal masuk salah satu kategori penerima manfaat layanan transportasi umum gratis.</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8318525/bahas-politik-luar-negeri-prabowo-usung-good-neighbor-policy</t>
+          <t>https://www.liputan6.com/news/read/8319131/tahun-depan-warga-jakarta-bisa-naik-transportasi-gratis-untuk-cari-kerja</t>
         </is>
       </c>
     </row>
@@ -2508,22 +2532,22 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>11 Korporasi Jadi Tersangka Kebakaran Hutan, 3 Perusahaan Asing</t>
+          <t>Survei Voxpol: 63,1% Publik Percaya Pemerintahan Prabowo-Gibran</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Wed, 21 Oct 2026 21:42:18 +0700</t>
+          <t>Thu, 22 Oct 2026 16:00:55 +0700</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Kapolri menegaskan penyidik tidak menghadapi kendala dalam menangani kasus tersebut.</t>
+          <t>Voxpol menilai kepercayaan terhadap pemerintahan Prabowo-Gibran relatif kuat.</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8318536/11-korporasi-jadi-tersangka-kebakaran-hutan-3-perusahaan-asing</t>
+          <t>https://www.liputan6.com/news/read/8319099/survei-voxpol-631-publik-percaya-pemerintahan-prabowo-gibran</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data pasar & berita - 2026-10-23 00:13 UTC
</commit_message>
<xml_diff>
--- a/data/market_news_latest.xlsx
+++ b/data/market_news_latest.xlsx
@@ -487,20 +487,20 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>5387.9048</v>
+        <v>5328.3599</v>
       </c>
       <c r="F2" t="n">
-        <v>59.5449</v>
+        <v>49.4717</v>
       </c>
       <c r="G2" t="n">
-        <v>1.12</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="H2" t="n">
-        <v>0</v>
+        <v>292010300</v>
       </c>
     </row>
     <row r="3">
@@ -525,16 +525,16 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>7695.25</v>
+        <v>7663.4302</v>
       </c>
       <c r="F3" t="n">
-        <v>-61.9199</v>
+        <v>-93.7397</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.8</v>
+        <v>-1.21</v>
       </c>
       <c r="H3" t="n">
-        <v>203879799</v>
+        <v>3559453000</v>
       </c>
     </row>
     <row r="4">
@@ -559,16 +559,16 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>52672.4102</v>
+        <v>52867.9805</v>
       </c>
       <c r="F4" t="n">
-        <v>-183.6797</v>
+        <v>11.8906</v>
       </c>
       <c r="G4" t="n">
-        <v>-0.35</v>
+        <v>0.02</v>
       </c>
       <c r="H4" t="n">
-        <v>34507950</v>
+        <v>506198387</v>
       </c>
     </row>
     <row r="5">
@@ -593,16 +593,16 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>26325.4082</v>
+        <v>26008.8594</v>
       </c>
       <c r="F5" t="n">
-        <v>-377.4512</v>
+        <v>-694</v>
       </c>
       <c r="G5" t="n">
-        <v>-1.41</v>
+        <v>-2.6</v>
       </c>
       <c r="H5" t="n">
-        <v>1083109000</v>
+        <v>7832683000</v>
       </c>
     </row>
     <row r="6">
@@ -623,20 +623,20 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>62907.8398</v>
+        <v>64621.2383</v>
       </c>
       <c r="F6" t="n">
-        <v>-1713.3984</v>
+        <v>545.8164</v>
       </c>
       <c r="G6" t="n">
-        <v>-2.65</v>
+        <v>0.85</v>
       </c>
       <c r="H6" t="n">
-        <v>0</v>
+        <v>149800000</v>
       </c>
     </row>
     <row r="7">
@@ -657,20 +657,20 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>22934.6797</v>
+        <v>23651.8691</v>
       </c>
       <c r="F7" t="n">
-        <v>-717.1895</v>
+        <v>-215.8711</v>
       </c>
       <c r="G7" t="n">
-        <v>-3.03</v>
+        <v>-0.9</v>
       </c>
       <c r="H7" t="n">
-        <v>0</v>
+        <v>2484800000</v>
       </c>
     </row>
     <row r="8">
@@ -694,15 +694,9 @@
           <t>2026-10-22</t>
         </is>
       </c>
-      <c r="E8" t="n">
-        <v>3658.0256</v>
-      </c>
-      <c r="F8" t="n">
-        <v>-55.0024</v>
-      </c>
-      <c r="G8" t="n">
-        <v>-1.48</v>
-      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
       <c r="H8" t="n">
         <v>819523340</v>
       </c>
@@ -725,20 +719,20 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>10735.1201</v>
+        <v>10752.9004</v>
       </c>
       <c r="F9" t="n">
-        <v>-17.7803</v>
+        <v>19.9004</v>
       </c>
       <c r="G9" t="n">
-        <v>-0.17</v>
+        <v>0.19</v>
       </c>
       <c r="H9" t="n">
-        <v>0</v>
+        <v>727782000</v>
       </c>
     </row>
     <row r="10">
@@ -759,20 +753,20 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>25516.6895</v>
+        <v>25645.0391</v>
       </c>
       <c r="F10" t="n">
-        <v>-128.3496</v>
+        <v>340.6191</v>
       </c>
       <c r="G10" t="n">
-        <v>-0.5</v>
+        <v>1.35</v>
       </c>
       <c r="H10" t="n">
-        <v>0</v>
+        <v>54049700</v>
       </c>
     </row>
     <row r="11">
@@ -793,20 +787,20 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>5415.1401</v>
+        <v>5437.9902</v>
       </c>
       <c r="F11" t="n">
-        <v>-22.8501</v>
+        <v>33.9702</v>
       </c>
       <c r="G11" t="n">
-        <v>-0.42</v>
+        <v>0.63</v>
       </c>
       <c r="H11" t="n">
-        <v>0</v>
+        <v>276361800</v>
       </c>
     </row>
     <row r="12">
@@ -827,17 +821,17 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="E12" t="n">
         <v>17943</v>
       </c>
       <c r="F12" t="n">
-        <v>-42.4004</v>
+        <v>-65</v>
       </c>
       <c r="G12" t="n">
-        <v>-0.24</v>
+        <v>-0.36</v>
       </c>
       <c r="H12" t="n">
         <v>0</v>
@@ -865,13 +859,13 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>101.792</v>
+        <v>101.546</v>
       </c>
       <c r="F13" t="n">
-        <v>0.012</v>
+        <v>-0.234</v>
       </c>
       <c r="G13" t="n">
-        <v>0.01</v>
+        <v>-0.23</v>
       </c>
       <c r="H13" t="n">
         <v>0</v>
@@ -895,17 +889,17 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>157.269</v>
+        <v>156.198</v>
       </c>
       <c r="F14" t="n">
-        <v>-0.999</v>
+        <v>-1.934</v>
       </c>
       <c r="G14" t="n">
-        <v>-0.63</v>
+        <v>-1.22</v>
       </c>
       <c r="H14" t="n">
         <v>0</v>
@@ -933,13 +927,13 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>0.5044</v>
+        <v>0.4953</v>
       </c>
       <c r="F15" t="n">
-        <v>-0.0102</v>
+        <v>-0.0193</v>
       </c>
       <c r="G15" t="n">
-        <v>-1.98</v>
+        <v>-3.75</v>
       </c>
       <c r="H15" t="n">
         <v>0</v>
@@ -967,13 +961,13 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>0.5352</v>
+        <v>0.5286999999999999</v>
       </c>
       <c r="F16" t="n">
-        <v>-0.008699999999999999</v>
+        <v>-0.0152</v>
       </c>
       <c r="G16" t="n">
-        <v>-1.6</v>
+        <v>-2.79</v>
       </c>
       <c r="H16" t="n">
         <v>0</v>
@@ -1001,13 +995,13 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>0.404</v>
+        <v>0.4022</v>
       </c>
       <c r="F17" t="n">
-        <v>-0.0023</v>
+        <v>-0.0041</v>
       </c>
       <c r="G17" t="n">
-        <v>-0.57</v>
+        <v>-1.01</v>
       </c>
       <c r="H17" t="n">
         <v>0</v>
@@ -1034,17 +1028,11 @@
           <t>2026-10-22</t>
         </is>
       </c>
-      <c r="E18" t="n">
-        <v>81</v>
-      </c>
-      <c r="F18" t="n">
-        <v>0.76</v>
-      </c>
-      <c r="G18" t="n">
-        <v>0.95</v>
-      </c>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
       <c r="H18" t="n">
-        <v>3841450</v>
+        <v>65594889</v>
       </c>
     </row>
     <row r="19">
@@ -1068,17 +1056,11 @@
           <t>2026-10-22</t>
         </is>
       </c>
-      <c r="E19" t="n">
-        <v>76.955</v>
-      </c>
-      <c r="F19" t="n">
-        <v>-0.025</v>
-      </c>
-      <c r="G19" t="n">
-        <v>-0.03</v>
-      </c>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr"/>
       <c r="H19" t="n">
-        <v>2268810</v>
+        <v>47048939</v>
       </c>
     </row>
     <row r="20">
@@ -1103,16 +1085,16 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>4091.8999</v>
+        <v>4038.3</v>
       </c>
       <c r="F20" t="n">
-        <v>-58.1001</v>
+        <v>-111.7</v>
       </c>
       <c r="G20" t="n">
-        <v>-1.4</v>
+        <v>-2.69</v>
       </c>
       <c r="H20" t="n">
-        <v>116667</v>
+        <v>6660</v>
       </c>
     </row>
     <row r="21">
@@ -1137,16 +1119,16 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>99.8</v>
+        <v>99.38</v>
       </c>
       <c r="F21" t="n">
-        <v>2.65</v>
+        <v>2.23</v>
       </c>
       <c r="G21" t="n">
-        <v>2.73</v>
+        <v>2.3</v>
       </c>
       <c r="H21" t="n">
-        <v>117095</v>
+        <v>4018</v>
       </c>
     </row>
     <row r="22">
@@ -1171,16 +1153,16 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>112.3</v>
+        <v>113.1</v>
       </c>
       <c r="F22" t="n">
-        <v>3.48</v>
+        <v>4.28</v>
       </c>
       <c r="G22" t="n">
-        <v>3.2</v>
+        <v>3.93</v>
       </c>
       <c r="H22" t="n">
-        <v>19060</v>
+        <v>73</v>
       </c>
     </row>
     <row r="23">
@@ -1205,16 +1187,16 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>6.439</v>
+        <v>6.3995</v>
       </c>
       <c r="F23" t="n">
-        <v>-0.104</v>
+        <v>-0.1435</v>
       </c>
       <c r="G23" t="n">
-        <v>-1.59</v>
+        <v>-2.19</v>
       </c>
       <c r="H23" t="n">
-        <v>38078</v>
+        <v>685</v>
       </c>
     </row>
     <row r="24">
@@ -1238,17 +1220,11 @@
           <t>2026-10-22</t>
         </is>
       </c>
-      <c r="E24" t="n">
-        <v>62.25</v>
-      </c>
-      <c r="F24" t="n">
-        <v>-1.32</v>
-      </c>
-      <c r="G24" t="n">
-        <v>-2.08</v>
-      </c>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr"/>
       <c r="H24" t="n">
-        <v>1373065</v>
+        <v>28385465</v>
       </c>
     </row>
     <row r="25">
@@ -1273,13 +1249,13 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>18.07</v>
+        <v>19.03</v>
       </c>
       <c r="F25" t="n">
-        <v>1.39</v>
+        <v>2.35</v>
       </c>
       <c r="G25" t="n">
-        <v>8.33</v>
+        <v>14.09</v>
       </c>
       <c r="H25" t="n">
         <v>0</v>
@@ -1303,20 +1279,20 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="E26" t="n">
-        <v>81540.0469</v>
+        <v>81050.7812</v>
       </c>
       <c r="F26" t="n">
-        <v>-2471.9219</v>
+        <v>-2961.1875</v>
       </c>
       <c r="G26" t="n">
-        <v>-2.94</v>
+        <v>-3.52</v>
       </c>
       <c r="H26" t="n">
-        <v>38158757888</v>
+        <v>33452693504</v>
       </c>
     </row>
     <row r="27">
@@ -1749,22 +1725,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Menteri UMKM Ungkap Alasan Wajib Halal Ditunda</t>
+          <t>Prabowo Mau Tutup 700 BUMN sampai Desember 2026!</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Thu, 22 Oct 2026 20:30:00 +0700</t>
+          <t>Fri, 23 Oct 2026 07:00:23 +0700</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/12/02/menteri-usaha-mikro-kecil-dan-menengah-umkm-maman-abdurrahman-1764677159466_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Usaha Mikro Kecil dan Menengah (UMKM) Maman Abdurrahman menyampaikan alasan kewajiban sertifikasi halal diundur menja</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/08/28/presiden-prabowo-subianto-1756366417599_169.jpeg?w=360&amp;amp;q=90" /&gt; Presiden Prabowo Subianto menegaskan rencana penutupan 700 BUMN untuk efisiensi. Proses ini bertahap, fokus pada perusahaan yang merugikan negara.</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8719637/menteri-umkm-ungkap-alasan-wajib-halal-ditunda</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8719746/prabowo-mau-tutup-700-bumn-sampai-desember-2026</t>
         </is>
       </c>
     </row>
@@ -1776,22 +1752,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Bank Mandiri Tingkatkan Layanan Digital untuk Dorong Pertumbuhan Bisnis</t>
+          <t>Saham HSC Segera Ditendang dari Perhitungan IHSG, Ada Tanda Khusus</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Thu, 22 Oct 2026 20:06:47 +0700</t>
+          <t>Fri, 23 Oct 2026 06:25:00 +0700</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/22/bank-mandiri-1792674027427.png?w=360&amp;amp;q=90" /&gt; Bank Mandiri terus tingkatkan layanan untuk memenuhi ekspektasi nasabah. Fokus pada pengalaman pelanggan dan integrasi layanan digital dalam satu aplikasi.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/06/04/ihsg-terpuruk-kekhawatiran-pasar-meningkat-1780558039733_169.jpeg?w=360&amp;amp;q=90" /&gt; Bursa Efek Indonesia mengumumkan perubahan kriteria IHSG, mengeluarkan saham dengan konsentrasi kepemilikan tinggi mulai 2 November 2026.</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/moneter/d-8719674/bank-mandiri-tingkatkan-layanan-digital-untuk-dorong-pertumbuhan-bisnis</t>
+          <t>https://finance.detik.com/bursa-dan-valas/d-8719635/saham-hsc-segera-ditendang-dari-perhitungan-ihsg-ada-tanda-khusus</t>
         </is>
       </c>
     </row>
@@ -1803,22 +1779,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Anggaran Rekening Gratis Turun dari Rp 3,84 T Jadi Rp 1,28 T</t>
+          <t>Prabowo Dapat Laporan Ada Tambang Raksasa Senilai Rp 5.400 T</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Thu, 22 Oct 2026 20:00:20 +0700</t>
+          <t>Fri, 23 Oct 2026 05:55:00 +0700</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/10/27/bi-pertahankan-bi-rate-475-persen-untuk-jaga-stabilitas-rupiah-1761539775425_169.jpeg?w=360&amp;amp;q=90" /&gt; Pemerintah mengubah anggaran program rekening gratis dari Rp 3,84 triliun menjadi Rp 1,28 triliun, hal ini dilakukan setelah</t>
+          <t xml:space="preserve">&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/22/presiden-prabowo-di-rakornas-tim-percepatan-akses-keuangan-daerah-tpakd-jiexpo-kemayoran-jakarta-kamis-22102026-muchlis-jr-bir-1792664303215_169.jpeg?w=360&amp;amp;q=90" /&gt; Presiden Prabowo Subianto mengaku dapat laporan ada tambang </t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8719657/anggaran-rekening-gratis-turun-dari-rp-3-84-t-jadi-rp-1-28-t</t>
+          <t>https://finance.detik.com/energi/d-8719507/prabowo-dapat-laporan-ada-tambang-raksasa-senilai-rp-5-400-t</t>
         </is>
       </c>
     </row>
@@ -1830,22 +1806,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>UMK Lokal Dapat Diskon 50% Biaya Administrasi Toko Online Selamanya</t>
+          <t>Pertamina Pasang Oil Boom di Sekitar Kapal Batumandi</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Thu, 22 Oct 2026 20:00:17 +0700</t>
+          <t>Thu, 22 Oct 2026 22:46:34 +0700</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/22/menteri-usaha-mikro-kecil-dan-menengah-umkm-maman-abdurrahman-1792667292505_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri UMKM Maman Abdurrahman menyampaikan kebijakan ini akan berlaku secara permanen.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/22/pt-pertamina-trans-kontinental-ptk-1792683765501_169.jpeg?w=360&amp;amp;q=90" /&gt; Pertamina mengerahkan tim tanggap darurat Operasional Marine Tanjung Sekong dan Marine Tanjung Gerem untuk membantu penanganan kebakaran Kapal KMP Batum</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8719617/umk-lokal-dapat-diskon-50-biaya-administrasi-toko-online-selamanya</t>
+          <t>https://finance.detik.com/energi/d-8719830/pertamina-pasang-oil-boom-di-sekitar-kapal-batumandi</t>
         </is>
       </c>
     </row>
@@ -1857,22 +1833,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Putri Tanjung Bicara Pentingnya Ekosistem Kreatif yang Sehat</t>
+          <t>Rincian Stimulus Rp 31 Triliun Akhir Tahun: BSU hingga Rekening Gratis</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Thu, 22 Oct 2026 19:31:06 +0700</t>
+          <t>Thu, 22 Oct 2026 22:06:55 +0700</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/22/putri-tanjung-bicara-pentingnya-ekosistem-kreatif-yang-sehat-1792672229786_43.jpeg?w=360&amp;amp;q=90" /&gt; Putri Tanjung dorong penguatan ekosistem ekonomi kreatif Indonesia agar IP lokal bersaing global. Kolaborasi penting untuk kemb</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/02/ilustrasi-bsu-kemnaker-rp-900000-1790934696631_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Koordinator Perekonomian Airlangga Hartarto menyampaikan pemerintah menyiapkan stimulus ekonomi sebesar Rp 31 triliun untuk kuartal IV 2026.</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8719633/putri-tanjung-bicara-pentingnya-ekosistem-kreatif-yang-sehat</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8719796/rincian-stimulus-rp-31-triliun-akhir-tahun-bsu-hingga-rekening-gratis</t>
         </is>
       </c>
     </row>
@@ -1884,22 +1860,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>OJK Ungkap Progres Demutualisasi Bursa: BEI Gelar RUPS Akhir Oktober 2026</t>
+          <t>Potret Padatnya Pencari Kerja di Tengah Badai PHK</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Thu, 22 Oct 2026 19:30:11 +0700</t>
+          <t>Thu, 22 Oct 2026 21:30:07 +0700</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2016/12/30/ed5ec33a-5357-40f8-8f66-6713c06687ea_169.jpg?w=360&amp;amp;q=90" /&gt; OJK mengungkap progres demutualisasi BEI, dengan RUPS dijadwalkan pada 28 Oktober 2026 untuk membahas perubahan anggaran dasar dan langkah selanjutnya.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/22/potret-padatnya-pencari-kerja-di-tengah-badai-phk-1792676014221_169.jpeg?w=360&amp;amp;q=90" /&gt; Pencari kerja memadati Karir Jakarta Expo 2026 di Jakarta. Lebih dari 28 ribu orang mendaftar untuk 12 ribu lowongan.</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/moneter/d-8719551/ojk-ungkap-progres-demutualisasi-bursa-bei-gelar-rups-akhir-oktober-2026</t>
+          <t>https://finance.detik.com/foto-bisnis/d-8719703/potret-padatnya-pencari-kerja-di-tengah-badai-phk</t>
         </is>
       </c>
     </row>
@@ -1911,22 +1887,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>BRI Siapkan Buyback Saham Tahap II Senilai Rp 1 Triliun</t>
+          <t>Danantara Bakal Umumkan Investasi Data Center dan AI</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Thu, 22 Oct 2026 19:12:42 +0700</t>
+          <t>Thu, 22 Oct 2026 21:30:01 +0700</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/22/ilustrasi-gedung-bri-1792671138276.jpeg?w=360&amp;amp;q=90" /&gt; PT BRI umumkan rencana buyback saham Tahap II senilai Rp 1 triliun. Aksi ini bertujuan tingkatkan nilai pemegang saham dan dukung pertumbuhan jangka panjang.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/07/01/wisma-danantara-indonesia-1751345496255_169.jpeg?w=360&amp;amp;q=90" /&gt; Pengembangan infrastruktur digital dan AI menjadi salah satu prioritas investasi untuk meningkatkan daya saing dan kapasitas teknologi nasional.</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/bursa-dan-valas/d-8719613/bri-siapkan-buyback-saham-tahap-ii-senilai-rp-1-triliun</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8719620/danantara-bakal-umumkan-investasi-data-center-dan-ai</t>
         </is>
       </c>
     </row>
@@ -1938,22 +1914,22 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Kementan Dorong Hilirisasi Hortikultura Lewat Inovasi KWT di Lombok</t>
+          <t>7 Provinsi Terdampak Karhutla Dapat Bantuan, Total Rp 1,23 Triliun</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Thu, 22 Oct 2026 19:11:30 +0700</t>
+          <t>Thu, 22 Oct 2026 20:56:09 +0700</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/22/kementan-dorong-hilirisasi-hortikultura-lewat-inovasi-kwt-di-lombok-1792671077202.jpeg?w=360&amp;amp;q=90" /&gt; Kementan dorong hilirisasi hortikultura melalui pengembangan produk olahan lokal. KWT Sasak Maiq jadi contoh sukses dalam m</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/08/21/petugas-memadamkan-karhutla-di-kalimantan-1787304053622_169.jpeg?w=360&amp;amp;q=90" /&gt; Pemerintah mengirimkan bantuan dana ke tujuh provinsi terdampak kebakaran hutan dan lahan (karhutla). Total anggaran mencapai Rp 1,23 triliun.</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8719610/kementan-dorong-hilirisasi-hortikultura-lewat-inovasi-kwt-di-lombok</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8719722/7-provinsi-terdampak-karhutla-dapat-bantuan-total-rp-1-23-triliun</t>
         </is>
       </c>
     </row>
@@ -1965,22 +1941,22 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>336 Investor Asing Colek OJK Usai MSCI Buka Opsi Bursa RI Turun Kasta</t>
+          <t>Menteri UMKM Ungkap Alasan Wajib Halal Ditunda</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Thu, 22 Oct 2026 19:00:35 +0700</t>
+          <t>Thu, 22 Oct 2026 20:30:00 +0700</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/06/04/ihsg-terpuruk-kekhawatiran-pasar-meningkat-1780558039793_169.jpeg?w=360&amp;amp;q=90" /&gt; Sebanyak 336 investor asing meminta klarifikasi OJK dan BEI terkait pengumuman MSCI.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/12/02/menteri-usaha-mikro-kecil-dan-menengah-umkm-maman-abdurrahman-1764677159466_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Usaha Mikro Kecil dan Menengah (UMKM) Maman Abdurrahman menyampaikan alasan kewajiban sertifikasi halal diundur menja</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/bursa-dan-valas/d-8719580/336-investor-asing-colek-ojk-usai-msci-buka-opsi-bursa-ri-turun-kasta</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8719637/menteri-umkm-ungkap-alasan-wajib-halal-ditunda</t>
         </is>
       </c>
     </row>
@@ -1992,22 +1968,22 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Penyaluran KUR Tembus Rp 260 T ke 4 Juta Debitur</t>
+          <t>Bank Mandiri Tingkatkan Layanan Digital untuk Dorong Pertumbuhan Bisnis</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Thu, 22 Oct 2026 19:00:28 +0700</t>
+          <t>Thu, 22 Oct 2026 20:06:47 +0700</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/22/menteri-usaha-mikro-kecil-dan-menengah-umkm-maman-abdurrahman-1792667292505_169.jpeg?w=360&amp;amp;q=90" /&gt; Kementerian Usaha Mikro Kecil dan Menengah (UMKM) melaporkan realisasi penyaluran kredit usaha rakyat (KUR) mencapai Rp 260,8</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/22/bank-mandiri-1792674027427.png?w=360&amp;amp;q=90" /&gt; Bank Mandiri terus tingkatkan layanan untuk memenuhi ekspektasi nasabah. Fokus pada pengalaman pelanggan dan integrasi layanan digital dalam satu aplikasi.</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/moneter/d-8719524/penyaluran-kur-tembus-rp-260-t-ke-4-juta-debitur</t>
+          <t>https://finance.detik.com/moneter/d-8719674/bank-mandiri-tingkatkan-layanan-digital-untuk-dorong-pertumbuhan-bisnis</t>
         </is>
       </c>
     </row>
@@ -2019,22 +1995,22 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Bayan Buka Suara Sahamnya Diborong Haji Isam di Harga Murah</t>
+          <t>Anggaran Rekening Gratis Turun dari Rp 3,84 T Jadi Rp 1,28 T</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Thu, 22 Oct 2026 18:31:25 +0700</t>
+          <t>Thu, 22 Oct 2026 20:00:20 +0700</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/16/ihsg-ambruk-1157-ditutup-di-level-5185-1792144638880_169.jpeg?w=360&amp;amp;q=90" /&gt; PT Bayan Resources buka suara sahamnya diborong murah oleh Haji Isam.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/10/27/bi-pertahankan-bi-rate-475-persen-untuk-jaga-stabilitas-rupiah-1761539775425_169.jpeg?w=360&amp;amp;q=90" /&gt; Pemerintah mengubah anggaran program rekening gratis dari Rp 3,84 triliun menjadi Rp 1,28 triliun, hal ini dilakukan setelah</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/bursa-dan-valas/d-8719560/bayan-buka-suara-sahamnya-diborong-haji-isam-di-harga-murah</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8719657/anggaran-rekening-gratis-turun-dari-rp-3-84-t-jadi-rp-1-28-t</t>
         </is>
       </c>
     </row>
@@ -2046,22 +2022,22 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>WIKA Bakal Siapkan Layanan Avtur Terintegrasi di Bandara Kertajati</t>
+          <t>UMK Lokal Dapat Diskon 50% Biaya Administrasi Toko Online Selamanya</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Thu, 22 Oct 2026 18:30:33 +0700</t>
+          <t>Thu, 22 Oct 2026 20:00:17 +0700</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/22/wika-finalisasi-commissioning-aft-kertajati-siapkan-layanan-avtur-terintegrasi-di-bandara-kertajati-1792668571401.jpeg?w=360&amp;amp;q=90" /&gt; PT Wijaya Karya (WIKA) hampir menyelesaikan commissioning Aviation Fuel Terminal di Kertaja</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/22/menteri-usaha-mikro-kecil-dan-menengah-umkm-maman-abdurrahman-1792667292505_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri UMKM Maman Abdurrahman menyampaikan kebijakan ini akan berlaku secara permanen.</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/infrastruktur/d-8719559/wika-bakal-siapkan-layanan-avtur-terintegrasi-di-bandara-kertajati</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8719617/umk-lokal-dapat-diskon-50-biaya-administrasi-toko-online-selamanya</t>
         </is>
       </c>
     </row>
@@ -2073,22 +2049,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>bank bjb Ajak Masyarakat Ikuti Semarang 10K, Cuma Nabung Bisa Dapat Tiket</t>
+          <t>Putri Tanjung Bicara Pentingnya Ekosistem Kreatif yang Sehat</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Thu, 22 Oct 2026 17:44:44 +0700</t>
+          <t>Thu, 22 Oct 2026 19:31:06 +0700</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/22/bank-bjb-ajak-masyarakat-ikuti-semarang-10k-cuma-nabung-bisa-dapat-tiket-1792665852462.jpeg?w=360&amp;amp;q=90" /&gt; Bank bjb luncurkan program promo Semarang 10K 2026, menggabungkan gaya hidup sehat dan perencanaan keuangan. Dapatkan </t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/22/putri-tanjung-bicara-pentingnya-ekosistem-kreatif-yang-sehat-1792672229786_43.jpeg?w=360&amp;amp;q=90" /&gt; Putri Tanjung dorong penguatan ekosistem ekonomi kreatif Indonesia agar IP lokal bersaing global. Kolaborasi penting untuk kemb</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8719477/bank-bjb-ajak-masyarakat-ikuti-semarang-10k-cuma-nabung-bisa-dapat-tiket</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8719633/putri-tanjung-bicara-pentingnya-ekosistem-kreatif-yang-sehat</t>
         </is>
       </c>
     </row>
@@ -2100,22 +2076,22 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>bank bjb Raih Pengakuan Top 50 Emiten MidCap dalam IICD CG Award 2026</t>
+          <t>OJK Ungkap Progres Demutualisasi Bursa: BEI Gelar RUPS Akhir Oktober 2026</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Thu, 22 Oct 2026 17:35:40 +0700</t>
+          <t>Thu, 22 Oct 2026 19:30:11 +0700</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/22/bank-bjb-raih-pengakuan-top-50-emiten-midcap-dalam-iicd-cg-award-2026-1792664414280_43.jpeg?w=360&amp;amp;q=90" /&gt; bank bjb meraih penghargaan GCG dari IICD sebagai Top 50 Emiten MidCap. Pengakuan ini memperkuat komitmen bank dalam m</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2016/12/30/ed5ec33a-5357-40f8-8f66-6713c06687ea_169.jpg?w=360&amp;amp;q=90" /&gt; OJK mengungkap progres demutualisasi BEI, dengan RUPS dijadwalkan pada 28 Oktober 2026 untuk membahas perubahan anggaran dasar dan langkah selanjutnya.</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/moneter/d-8719434/bank-bjb-raih-pengakuan-top-50-emiten-midcap-dalam-iicd-cg-award-2026</t>
+          <t>https://finance.detik.com/moneter/d-8719551/ojk-ungkap-progres-demutualisasi-bursa-bei-gelar-rups-akhir-oktober-2026</t>
         </is>
       </c>
     </row>
@@ -2127,22 +2103,22 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Pencari Kerja Berburu 12 Ribu Lowongan di Karir Jakarta Expo 2026</t>
+          <t>BRI Siapkan Buyback Saham Tahap II Senilai Rp 1 Triliun</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Thu, 22 Oct 2026 17:30:45 +0700</t>
+          <t>Thu, 22 Oct 2026 19:12:42 +0700</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/22/pencari-kerja-berburu-12-ribu-lowongan-di-karir-jakarta-expo-2026-1792655486514.jpeg?w=360&amp;amp;q=90" /&gt; Pemprov DKI Jakarta menggelar Karir Jakarta Expo 2026 di SMESCO. Bursa kerja gratis ini menyediakan 12 ribu lowongan dari rat</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/22/ilustrasi-gedung-bri-1792671138276.jpeg?w=360&amp;amp;q=90" /&gt; PT BRI umumkan rencana buyback saham Tahap II senilai Rp 1 triliun. Aksi ini bertujuan tingkatkan nilai pemegang saham dan dukung pertumbuhan jangka panjang.</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/foto-bisnis/d-8719100/pencari-kerja-berburu-12-ribu-lowongan-di-karir-jakarta-expo-2026</t>
+          <t>https://finance.detik.com/bursa-dan-valas/d-8719613/bri-siapkan-buyback-saham-tahap-ii-senilai-rp-1-triliun</t>
         </is>
       </c>
     </row>
@@ -2154,22 +2130,22 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Kemendagri Minta Pemda Evaluasi Aturan yang Bebani Warga</t>
+          <t>Akses Penanjakan Bromo Dibuka Lagi Pascakebakaran, Simak Aturan dan Kuotanya</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Thu, 22 Oct 2026 20:36:21 +0700</t>
+          <t>Fri, 23 Oct 2026 06:30:16 +0700</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Sejumlah tahapan perlu dikaji agar dapat dilaksanakan secara paralel sehingga pelayanan menjadi lebih sederhana, cepat, dan efisien.</t>
+          <t>Pengunjung dan pelaku jasa wisata harus patuhi semua aturan demi mencegah titik api kembali muncul.</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8319345/kemendagri-minta-pemda-evaluasi-aturan-yang-bebani-warga</t>
+          <t>https://www.liputan6.com/news/read/8319478/akses-penanjakan-bromo-dibuka-lagi-pascakebakaran-simak-aturan-dan-kuotanya</t>
         </is>
       </c>
     </row>
@@ -2181,22 +2157,22 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Santri Tak Cuma Soal Sarung dan Kitab Kuning</t>
+          <t>Peringati Pink Month, Ribuan Warga Venezuela Turun ke Jalan</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Thu, 22 Oct 2026 20:05:19 +0700</t>
+          <t>Fri, 23 Oct 2026 06:00:56 +0700</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Santri masa kini tak hanya belajar agama, tetapi juga mengembangkan diri untuk menghadapi tantangan zaman.</t>
+          <t>Ribuan perempuan dan pegiat kesehatan memadati jalanan Caracas, Venezuela, Kamis (22/10/2026), dalam aksi memperingati Bulan Kesadaran Kanker Payudara atau Pink Month. Para peserta membawa balon merah muda, spanduk, dan bendera Venezuela sebagai bentuk solidaritas bagi pasien kanker payudara dan par</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8319318/santri-tak-cuma-soal-sarung-dan-kitab-kuning</t>
+          <t>https://www.liputan6.com/photo/read/8319472/peringati-pink-month-ribuan-warga-venezuela-turun-ke-jalan</t>
         </is>
       </c>
     </row>
@@ -2208,22 +2184,22 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Pria Tanpa Identitas Ditemukan Tewas di Warung Kosong Bekasi</t>
+          <t>Satgas PKH Cabut Izin Tambang PT KEL 3.500 Hektare di Papua</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Thu, 22 Oct 2026 19:59:45 +0700</t>
+          <t>Fri, 23 Oct 2026 05:39:32 +0700</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Saksi sempat mencium bau tak sedap beberapa hari sebelumnya.</t>
+          <t>Jaksa Agung menyebut PT KEL terbukti melakukan pertambangan emas secara ilegal baik di dalam maupun di luar Wilayah Izin Usaha Pertambangan.</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8319326/pria-tanpa-identitas-ditemukan-tewas-di-warung-kosong-bekasi</t>
+          <t>https://www.liputan6.com/news/read/8319469/satgas-pkh-cabut-izin-tambang-pt-kel-3500-hektare-di-papua</t>
         </is>
       </c>
     </row>
@@ -2235,22 +2211,22 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Momen Haru Hari Santri, Siswa Sekolah Rakyat Ungkap Mimpi Lewat Puisi</t>
+          <t>Jakarta International Literary Festival 2026 Resmi Dibuka</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Thu, 22 Oct 2026 19:35:00 +0700</t>
+          <t>Fri, 23 Oct 2026 05:30:48 +0700</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Siswa Sekolah Rakyat Terintegrasi 1 Jombang melafalkan bait demi bait puisi dipersembahkan dalam rangka memperingati Hari Santri Nasional 2026.</t>
+          <t>Mengusung tema 'Living Space', Jakarta International Literary Festival 2026 resmi dibuka di Graha Bhakti Budaya, Taman Ismail Marzuki.</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8319308/momen-haru-hari-santri-siswa-sekolah-rakyat-ungkap-mimpi-lewat-puisi</t>
+          <t>https://www.liputan6.com/news/read/8319467/jakarta-international-literary-festival-2026-resmi-dibuka</t>
         </is>
       </c>
     </row>
@@ -2262,22 +2238,22 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Prabowo soal Kebakaran Hutan: Ada Negara Mengolok-olok, Kita Cool Saja</t>
+          <t>40 Tokoh Ajukan 'Amicus Curiae' untuk Eks Ketua Ombudsman</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Thu, 22 Oct 2026 19:00:39 +0700</t>
+          <t>Fri, 23 Oct 2026 05:17:54 +0700</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Padahal, kata Prabowo, perusahaan-perusahaan dari negara itu ikut terlibat dan bertanggung jawab atas karhutla.</t>
+          <t>Perkara yang menjerat mantan Ketua Ombudsman RI Hery Susanto memasuki babak baru.</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8319290/prabowo-soal-kebakaran-hutan-ada-negara-mengolok-olok-kita-cool-saja</t>
+          <t>https://www.liputan6.com/news/read/8319466/40-tokoh-ajukan-amicus-curiae-untuk-eks-ketua-ombudsman</t>
         </is>
       </c>
     </row>
@@ -2289,22 +2265,22 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Prabowo: Saya Malu jadi Presiden Kalau Rakyat Miskin Terus</t>
+          <t>Bareskrim Bongkar Judi Online Bermodus Permainan di Jakbar</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Thu, 22 Oct 2026 18:53:07 +0700</t>
+          <t>Fri, 23 Oct 2026 00:48:31 +0700</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Prabowo berjanji akan lebih banyak menyalurkan alokasi anggaran ke daerah.</t>
+          <t>Empat tersangka ditangkap. Mereka memiliki peran sendiri-sendiri.</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8319287/prabowo-saya-malu-jadi-presiden-kalau-rakyat-miskin-terus</t>
+          <t>https://www.liputan6.com/news/read/8319448/bareskrim-bongkar-judi-online-bermodus-permainan-di-jakbar</t>
         </is>
       </c>
     </row>
@@ -2316,22 +2292,22 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Kronologi Kecelakaan Maut Mobilio Tabrak Pikap di Rasuna Said</t>
+          <t>Prabowo Sebut Indonesia Negara Ekonomi Terbesar ke-7 di Dunia</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Thu, 22 Oct 2026 18:24:54 +0700</t>
+          <t>Thu, 22 Oct 2026 22:40:48 +0700</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Polisi menduga kecelakaan yang terjadi pada dini hari tersebut dipicu oleh kecepatan tinggi Mobilio.</t>
+          <t>Prabowo menilai capaian tersebut menunjukkan kekuatan ekonomi Indonesia.</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8319262/kronologi-kecelakaan-maut-mobilio-tabrak-pikap-di-rasuna-said</t>
+          <t>https://www.liputan6.com/news/read/8319421/prabowo-sebut-indonesia-negara-ekonomi-terbesar-ke-7-di-dunia</t>
         </is>
       </c>
     </row>
@@ -2343,22 +2319,22 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Kronologi 45 WNA Diciduk Petugas Imigrasi di Apartemen Kalibata City</t>
+          <t>Prabowo Janji Tambah Anggaran untuk Provinsi dan Kabupaten</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Thu, 22 Oct 2026 18:21:55 +0700</t>
+          <t>Thu, 22 Oct 2026 23:00:34 +0700</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Dalam operasi tersebut, petugas mengamankan 45 WNA untuk menjalani pemeriksaan lebih lanjut di Ditjen Imigrasi.</t>
+          <t>Praboowo meyakini jumlah anggaran yang disalurkan ke daerah akan meningkat tahun depan.</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8319261/kronologi-45-wna-diciduk-petugas-imigrasi-di-apartemen-kalibata-city</t>
+          <t>https://www.liputan6.com/news/read/8319415/prabowo-janji-tambah-anggaran-untuk-provinsi-dan-kabupaten</t>
         </is>
       </c>
     </row>
@@ -2370,22 +2346,22 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Gempa Magnitudo 5,2 Guncang Bengkulu</t>
+          <t>KPK Tahan 7 Tersangka Baru Kasus Korupsi Proyek Jalan BBPJN Sumut</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Thu, 22 Oct 2026 18:11:53 +0700</t>
+          <t>Thu, 22 Oct 2026 22:04:43 +0700</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Gempa bumi magnitudo 5,2 terjadi di 6 km Barat Laut Lebong, Bengkulu, tanpa potensi tsunami.</t>
+          <t>Salah satu tersangka yang ditahan KPK adalah mantan Kepala BBPJN Sumut, Stanley Cicero Haggard Tuapattinaja.</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8319252/gempa-magnitudo-52-guncang-bengkulu</t>
+          <t>https://www.liputan6.com/news/read/8319397/kpk-tahan-7-tersangka-baru-kasus-korupsi-proyek-jalan-bbpjn-sumut</t>
         </is>
       </c>
     </row>
@@ -2397,22 +2373,22 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Pramono Targetkan Pengangguran Jakarta Turun jadi 3,5 Persen</t>
+          <t>Judi Online hingga Narkoba Disorot, Ini Pesan Polri di Kemah Kebangsaan</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Thu, 22 Oct 2026 17:55:15 +0700</t>
+          <t>Thu, 22 Oct 2026 22:01:42 +0700</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Jika angka pengangguran Jakarta turun, Pramono berharap jadi contoh daerah lain.</t>
+          <t>Pelajar dari berbagai sekolahan mengikuti kemah kebangsaan sebagai upaya menanamkan cinta Tanah Air.</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8319238/pramono-targetkan-pengangguran-jakarta-turun-jadi-35-persen</t>
+          <t>https://www.liputan6.com/news/read/8319395/judi-online-hingga-narkoba-disorot-ini-pesan-polri-di-kemah-kebangsaan</t>
         </is>
       </c>
     </row>
@@ -2424,22 +2400,22 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Prabowo Pimpin Langsung Dewan Nasional Kesejahteraan Keuangan</t>
+          <t>Prabowo Bidik Penyaluran Kredit Rakyat Rp 400 Triliun pada 2027</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Thu, 22 Oct 2026 17:41:20 +0700</t>
+          <t>Thu, 22 Oct 2026 21:17:26 +0700</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Presiden Prabowo meresmikan pembentukan Dewan Nasional Kesejahteraan Keuangan pada Kamis (22/10/2026).</t>
+          <t>Pembiayaan tersebut akan menyasar petani, nelayan, hingga masyarakat pedesaan dan kelompok berpenghasilan rendah.</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8319226/prabowo-pimpin-langsung-dewan-nasional-kesejahteraan-keuangan</t>
+          <t>https://www.liputan6.com/news/read/8319370/prabowo-bidik-penyaluran-kredit-rakyat-rp-400-triliun-pada-2027</t>
         </is>
       </c>
     </row>
@@ -2451,22 +2427,22 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Prabowo: Banyak Perusahaan Asing Harus Bertanggung Jawab Kebakaran Hutan</t>
+          <t>Hadiri Rakornas TPAKD, Mendagri Pastikan Bantuan Apresiasi Pemda TA 2027 Tetap Ada</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Thu, 22 Oct 2026 17:21:09 +0700</t>
+          <t>Thu, 22 Oct 2026 21:04:48 +0700</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Presiden Prabowo mengancam akan mencabut izin konsesi perusahaan yang berulang kali melanggar aturan.</t>
+          <t>Berdasarkan hasil koordinasi dengan Menteri Keuangan Suahasil Nazara, pemerintah menyiapkan Rp 2 triliun untuk TA 2027.</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8319215/prabowo-banyak-perusahaan-asing-harus-bertanggung-jawab-kebakaran-hutan</t>
+          <t>https://www.liputan6.com/news/read/8319365/hadiri-rakornas-tpakd-mendagri-pastikan-bantuan-apresiasi-pemda-ta-2027-tetap-ada</t>
         </is>
       </c>
     </row>
@@ -2478,22 +2454,22 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Hari Santri 2026, Prabowo Ungkap Peran Pesantren dalam Kemerdekaan Indonesia</t>
+          <t>Prabowo Minta Menteri Selektif Beri Konsesi Tambang</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Thu, 22 Oct 2026 16:32:45 +0700</t>
+          <t>Thu, 22 Oct 2026 20:44:29 +0700</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Prabowo berharap para santri dan santriwati semakin kompak dan hebat.</t>
+          <t>Prabowo meminta agar izin konsesi diberikan secara selektif dan memastikan pihak tersebut memiliki kemampuan untuk mengelola SDA secara optimal.</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8319177/hari-santri-2026-prabowo-ungkap-peran-pesantren-dalam-kemerdekaan-indonesia</t>
+          <t>https://www.liputan6.com/news/read/8319349/prabowo-minta-menteri-selektif-beri-konsesi-tambang</t>
         </is>
       </c>
     </row>
@@ -2505,22 +2481,22 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Tahun Depan, Warga Jakarta Bisa Naik Transportasi Gratis untuk Cari Kerja</t>
+          <t>Kemendagri Minta Pemda Evaluasi Aturan yang Bebani Warga</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Thu, 22 Oct 2026 16:25:04 +0700</t>
+          <t>Thu, 22 Oct 2026 20:36:21 +0700</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Pencari kerja bakal masuk salah satu kategori penerima manfaat layanan transportasi umum gratis.</t>
+          <t>Sejumlah tahapan perlu dikaji agar dapat dilaksanakan secara paralel sehingga pelayanan menjadi lebih sederhana, cepat, dan efisien.</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8319131/tahun-depan-warga-jakarta-bisa-naik-transportasi-gratis-untuk-cari-kerja</t>
+          <t>https://www.liputan6.com/news/read/8319345/kemendagri-minta-pemda-evaluasi-aturan-yang-bebani-warga</t>
         </is>
       </c>
     </row>
@@ -2532,22 +2508,22 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Survei Voxpol: 63,1% Publik Percaya Pemerintahan Prabowo-Gibran</t>
+          <t>Santri Tak Cuma Soal Sarung dan Kitab Kuning</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Thu, 22 Oct 2026 16:00:55 +0700</t>
+          <t>Thu, 22 Oct 2026 20:05:19 +0700</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Voxpol menilai kepercayaan terhadap pemerintahan Prabowo-Gibran relatif kuat.</t>
+          <t>Santri masa kini tak hanya belajar agama, tetapi juga mengembangkan diri untuk menghadapi tantangan zaman.</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8319099/survei-voxpol-631-publik-percaya-pemerintahan-prabowo-gibran</t>
+          <t>https://www.liputan6.com/news/read/8319318/santri-tak-cuma-soal-sarung-dan-kitab-kuning</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data pasar & berita - 2026-10-23 13:15 UTC
</commit_message>
<xml_diff>
--- a/data/market_news_latest.xlsx
+++ b/data/market_news_latest.xlsx
@@ -422,7 +422,7 @@
     <col width="26" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
   </cols>
@@ -487,20 +487,20 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>5328.3599</v>
+        <v>5439.2578</v>
       </c>
       <c r="F2" t="n">
-        <v>49.4717</v>
+        <v>51.353</v>
       </c>
       <c r="G2" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.95</v>
       </c>
       <c r="H2" t="n">
-        <v>292010300</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -534,7 +534,7 @@
         <v>-1.21</v>
       </c>
       <c r="H3" t="n">
-        <v>3559453000</v>
+        <v>5972620000</v>
       </c>
     </row>
     <row r="4">
@@ -568,7 +568,7 @@
         <v>0.02</v>
       </c>
       <c r="H4" t="n">
-        <v>506198387</v>
+        <v>506190000</v>
       </c>
     </row>
     <row r="5">
@@ -602,7 +602,7 @@
         <v>-2.6</v>
       </c>
       <c r="H5" t="n">
-        <v>7832683000</v>
+        <v>9012120000</v>
       </c>
     </row>
     <row r="6">
@@ -623,20 +623,20 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>64621.2383</v>
+        <v>62693.1602</v>
       </c>
       <c r="F6" t="n">
-        <v>545.8164</v>
+        <v>-214.6797</v>
       </c>
       <c r="G6" t="n">
-        <v>0.85</v>
+        <v>-0.34</v>
       </c>
       <c r="H6" t="n">
-        <v>149800000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -657,20 +657,20 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>23651.8691</v>
+        <v>23093.3691</v>
       </c>
       <c r="F7" t="n">
-        <v>-215.8711</v>
+        <v>158.6895</v>
       </c>
       <c r="G7" t="n">
-        <v>-0.9</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="H7" t="n">
-        <v>2484800000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -691,14 +691,20 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>3690.4753</v>
+      </c>
+      <c r="F8" t="n">
+        <v>32.4495</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0.89</v>
+      </c>
       <c r="H8" t="n">
-        <v>819523340</v>
+        <v>3744683648</v>
       </c>
     </row>
     <row r="9">
@@ -719,20 +725,20 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>10752.9004</v>
+        <v>10658.3203</v>
       </c>
       <c r="F9" t="n">
-        <v>19.9004</v>
+        <v>-66.6797</v>
       </c>
       <c r="G9" t="n">
-        <v>0.19</v>
+        <v>-0.62</v>
       </c>
       <c r="H9" t="n">
-        <v>727782000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -753,20 +759,20 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>25645.0391</v>
+        <v>25125.1406</v>
       </c>
       <c r="F10" t="n">
-        <v>340.6191</v>
+        <v>-246.6094</v>
       </c>
       <c r="G10" t="n">
-        <v>1.35</v>
+        <v>-0.97</v>
       </c>
       <c r="H10" t="n">
-        <v>54049700</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -787,20 +793,20 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>5437.9902</v>
+        <v>5422.1602</v>
       </c>
       <c r="F11" t="n">
-        <v>33.9702</v>
+        <v>7.02</v>
       </c>
       <c r="G11" t="n">
-        <v>0.63</v>
+        <v>0.13</v>
       </c>
       <c r="H11" t="n">
-        <v>276361800</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -825,13 +831,13 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>17943</v>
+        <v>18050</v>
       </c>
       <c r="F12" t="n">
-        <v>-65</v>
+        <v>42</v>
       </c>
       <c r="G12" t="n">
-        <v>-0.36</v>
+        <v>0.23</v>
       </c>
       <c r="H12" t="n">
         <v>0</v>
@@ -855,17 +861,17 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>101.546</v>
+        <v>101.686</v>
       </c>
       <c r="F13" t="n">
-        <v>-0.234</v>
+        <v>0.076</v>
       </c>
       <c r="G13" t="n">
-        <v>-0.23</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="H13" t="n">
         <v>0</v>
@@ -893,13 +899,13 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>156.198</v>
+        <v>156.391</v>
       </c>
       <c r="F14" t="n">
-        <v>-1.934</v>
+        <v>-1.741</v>
       </c>
       <c r="G14" t="n">
-        <v>-1.22</v>
+        <v>-1.1</v>
       </c>
       <c r="H14" t="n">
         <v>0</v>
@@ -923,17 +929,17 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>0.4953</v>
+        <v>0.4957</v>
       </c>
       <c r="F15" t="n">
-        <v>-0.0193</v>
+        <v>0.0004</v>
       </c>
       <c r="G15" t="n">
-        <v>-3.75</v>
+        <v>0.08</v>
       </c>
       <c r="H15" t="n">
         <v>0</v>
@@ -957,17 +963,17 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>0.5286999999999999</v>
+        <v>0.5281</v>
       </c>
       <c r="F16" t="n">
-        <v>-0.0152</v>
+        <v>-0.0005999999999999999</v>
       </c>
       <c r="G16" t="n">
-        <v>-2.79</v>
+        <v>-0.11</v>
       </c>
       <c r="H16" t="n">
         <v>0</v>
@@ -991,17 +997,17 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>0.4022</v>
+        <v>0.4037</v>
       </c>
       <c r="F17" t="n">
-        <v>-0.0041</v>
+        <v>0.0015</v>
       </c>
       <c r="G17" t="n">
-        <v>-1.01</v>
+        <v>0.37</v>
       </c>
       <c r="H17" t="n">
         <v>0</v>
@@ -1028,11 +1034,17 @@
           <t>2026-10-22</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
+      <c r="E18" t="n">
+        <v>81.73999999999999</v>
+      </c>
+      <c r="F18" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G18" t="n">
+        <v>1.87</v>
+      </c>
       <c r="H18" t="n">
-        <v>65594889</v>
+        <v>64652900</v>
       </c>
     </row>
     <row r="19">
@@ -1056,11 +1068,17 @@
           <t>2026-10-22</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
+      <c r="E19" t="n">
+        <v>77.09999999999999</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0.16</v>
+      </c>
       <c r="H19" t="n">
-        <v>47048939</v>
+        <v>47048900</v>
       </c>
     </row>
     <row r="20">
@@ -1081,20 +1099,20 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>4038.3</v>
+        <v>4041</v>
       </c>
       <c r="F20" t="n">
-        <v>-111.7</v>
+        <v>-19.3999</v>
       </c>
       <c r="G20" t="n">
-        <v>-2.69</v>
+        <v>-0.48</v>
       </c>
       <c r="H20" t="n">
-        <v>6660</v>
+        <v>89778</v>
       </c>
     </row>
     <row r="21">
@@ -1115,20 +1133,20 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>99.38</v>
+        <v>101.02</v>
       </c>
       <c r="F21" t="n">
-        <v>2.23</v>
+        <v>1.55</v>
       </c>
       <c r="G21" t="n">
-        <v>2.3</v>
+        <v>1.56</v>
       </c>
       <c r="H21" t="n">
-        <v>4018</v>
+        <v>106313</v>
       </c>
     </row>
     <row r="22">
@@ -1149,20 +1167,20 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="E22" t="n">
-        <v>113.1</v>
+        <v>110.06</v>
       </c>
       <c r="F22" t="n">
-        <v>4.28</v>
+        <v>-3.11</v>
       </c>
       <c r="G22" t="n">
-        <v>3.93</v>
+        <v>-2.75</v>
       </c>
       <c r="H22" t="n">
-        <v>73</v>
+        <v>14855</v>
       </c>
     </row>
     <row r="23">
@@ -1183,20 +1201,20 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="E23" t="n">
-        <v>6.3995</v>
+        <v>6.4655</v>
       </c>
       <c r="F23" t="n">
-        <v>-0.1435</v>
+        <v>0.103</v>
       </c>
       <c r="G23" t="n">
-        <v>-2.19</v>
+        <v>1.62</v>
       </c>
       <c r="H23" t="n">
-        <v>685</v>
+        <v>20732</v>
       </c>
     </row>
     <row r="24">
@@ -1220,11 +1238,17 @@
           <t>2026-10-22</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr"/>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr"/>
+      <c r="E24" t="n">
+        <v>61.72</v>
+      </c>
+      <c r="F24" t="n">
+        <v>-1.85</v>
+      </c>
+      <c r="G24" t="n">
+        <v>-2.91</v>
+      </c>
       <c r="H24" t="n">
-        <v>28385465</v>
+        <v>28385500</v>
       </c>
     </row>
     <row r="25">
@@ -1245,17 +1269,17 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="E25" t="n">
-        <v>19.03</v>
+        <v>20.22</v>
       </c>
       <c r="F25" t="n">
-        <v>2.35</v>
+        <v>1.19</v>
       </c>
       <c r="G25" t="n">
-        <v>14.09</v>
+        <v>6.25</v>
       </c>
       <c r="H25" t="n">
         <v>0</v>
@@ -1283,16 +1307,16 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>81050.7812</v>
+        <v>81533.47659999999</v>
       </c>
       <c r="F26" t="n">
-        <v>-2961.1875</v>
+        <v>221.5859</v>
       </c>
       <c r="G26" t="n">
-        <v>-3.52</v>
+        <v>0.27</v>
       </c>
       <c r="H26" t="n">
-        <v>33452693504</v>
+        <v>24775368704</v>
       </c>
     </row>
     <row r="27">
@@ -1313,20 +1337,20 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="E27" t="n">
         <v>1440</v>
       </c>
       <c r="F27" t="n">
-        <v>-45</v>
+        <v>0</v>
       </c>
       <c r="G27" t="n">
-        <v>-3.03</v>
+        <v>0</v>
       </c>
       <c r="H27" t="n">
-        <v>115064900</v>
+        <v>68976800</v>
       </c>
     </row>
     <row r="28">
@@ -1347,20 +1371,20 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="E28" t="n">
-        <v>1340</v>
+        <v>1330</v>
       </c>
       <c r="F28" t="n">
-        <v>0</v>
+        <v>-10</v>
       </c>
       <c r="G28" t="n">
-        <v>0</v>
+        <v>-0.75</v>
       </c>
       <c r="H28" t="n">
-        <v>192500500</v>
+        <v>136283100</v>
       </c>
     </row>
     <row r="29">
@@ -1381,20 +1405,20 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="E29" t="n">
-        <v>496</v>
+        <v>510</v>
       </c>
       <c r="F29" t="n">
-        <v>-9</v>
+        <v>14</v>
       </c>
       <c r="G29" t="n">
-        <v>-1.78</v>
+        <v>2.82</v>
       </c>
       <c r="H29" t="n">
-        <v>486782800</v>
+        <v>353645100</v>
       </c>
     </row>
     <row r="30">
@@ -1415,20 +1439,20 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="E30" t="n">
-        <v>2320</v>
+        <v>2380</v>
       </c>
       <c r="F30" t="n">
-        <v>160</v>
+        <v>60</v>
       </c>
       <c r="G30" t="n">
-        <v>7.41</v>
+        <v>2.59</v>
       </c>
       <c r="H30" t="n">
-        <v>23389400</v>
+        <v>20443500</v>
       </c>
     </row>
     <row r="31">
@@ -1449,20 +1473,20 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="E31" t="n">
-        <v>3070</v>
+        <v>3090</v>
       </c>
       <c r="F31" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="G31" t="n">
-        <v>0.33</v>
+        <v>0.65</v>
       </c>
       <c r="H31" t="n">
-        <v>43534800</v>
+        <v>27460600</v>
       </c>
     </row>
     <row r="32">
@@ -1483,20 +1507,20 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="E32" t="n">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="F32" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G32" t="n">
-        <v>0.95</v>
+        <v>0.47</v>
       </c>
       <c r="H32" t="n">
-        <v>43922700</v>
+        <v>24749800</v>
       </c>
     </row>
     <row r="33">
@@ -1517,20 +1541,20 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="E33" t="n">
-        <v>478</v>
+        <v>500</v>
       </c>
       <c r="F33" t="n">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="G33" t="n">
-        <v>1.7</v>
+        <v>4.6</v>
       </c>
       <c r="H33" t="n">
-        <v>87778300</v>
+        <v>154580300</v>
       </c>
     </row>
     <row r="34">
@@ -1551,20 +1575,20 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="E34" t="n">
-        <v>2520</v>
+        <v>2660</v>
       </c>
       <c r="F34" t="n">
-        <v>30</v>
+        <v>140</v>
       </c>
       <c r="G34" t="n">
-        <v>1.2</v>
+        <v>5.56</v>
       </c>
       <c r="H34" t="n">
-        <v>9474800</v>
+        <v>13319700</v>
       </c>
     </row>
     <row r="35">
@@ -1585,20 +1609,20 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="E35" t="n">
-        <v>314</v>
+        <v>378</v>
       </c>
       <c r="F35" t="n">
-        <v>-8</v>
+        <v>64</v>
       </c>
       <c r="G35" t="n">
-        <v>-2.48</v>
+        <v>20.38</v>
       </c>
       <c r="H35" t="n">
-        <v>854759900</v>
+        <v>791388800</v>
       </c>
     </row>
     <row r="36">
@@ -1619,20 +1643,20 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="E36" t="n">
-        <v>148</v>
+        <v>174</v>
       </c>
       <c r="F36" t="n">
-        <v>4</v>
+        <v>26</v>
       </c>
       <c r="G36" t="n">
-        <v>2.78</v>
+        <v>17.57</v>
       </c>
       <c r="H36" t="n">
-        <v>19327000</v>
+        <v>290939000</v>
       </c>
     </row>
     <row r="37">
@@ -1653,20 +1677,20 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="E37" t="n">
-        <v>10000</v>
+        <v>10300</v>
       </c>
       <c r="F37" t="n">
-        <v>350</v>
+        <v>300</v>
       </c>
       <c r="G37" t="n">
-        <v>3.63</v>
+        <v>3</v>
       </c>
       <c r="H37" t="n">
-        <v>33713400</v>
+        <v>13505800</v>
       </c>
     </row>
   </sheetData>
@@ -1725,22 +1749,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Prabowo Mau Tutup 700 BUMN sampai Desember 2026!</t>
+          <t>Forum Investasi Jateng Bahas Strategi KEK Batang Hadapi Persaingan Global</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Fri, 23 Oct 2026 07:00:23 +0700</t>
+          <t>Fri, 23 Oct 2026 20:00:09 +0700</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/08/28/presiden-prabowo-subianto-1756366417599_169.jpeg?w=360&amp;amp;q=90" /&gt; Presiden Prabowo Subianto menegaskan rencana penutupan 700 BUMN untuk efisiensi. Proses ini bertahap, fokus pada perusahaan yang merugikan negara.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/23/forum-investasi-jateng-bahas-strategi-kek-batang-hadapi-persaingan-global-1792756806815_169.jpeg?w=360&amp;amp;q=90" /&gt; Jawa Tengah memperkuat strategi menarik investasi melalui KEK Batang dan kolaborasi lintas instansi. Keamanan dan</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8719746/prabowo-mau-tutup-700-bumn-sampai-desember-2026</t>
+          <t>https://finance.detik.com/foto-bisnis/d-8721287/forum-investasi-jateng-bahas-strategi-kek-batang-hadapi-persaingan-global</t>
         </is>
       </c>
     </row>
@@ -1752,22 +1776,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Saham HSC Segera Ditendang dari Perhitungan IHSG, Ada Tanda Khusus</t>
+          <t>Bos OJK Lapor Prabowo Kondisi Bursa Usai MSCI Buka Opsi Turun Kasta</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Fri, 23 Oct 2026 06:25:00 +0700</t>
+          <t>Fri, 23 Oct 2026 20:00:05 +0700</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/06/04/ihsg-terpuruk-kekhawatiran-pasar-meningkat-1780558039733_169.jpeg?w=360&amp;amp;q=90" /&gt; Bursa Efek Indonesia mengumumkan perubahan kriteria IHSG, mengeluarkan saham dengan konsentrasi kepemilikan tinggi mulai 2 November 2026.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/08/03/frederica-widyasari-dewi-1785765447950_169.jpeg?w=360&amp;amp;q=90" /&gt; Ketua DK OJK Friderica Widyasari Dewi memberikan laporan ke Presiden Prabowo Subianto soal kondisi bursa efek.</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/bursa-dan-valas/d-8719635/saham-hsc-segera-ditendang-dari-perhitungan-ihsg-ada-tanda-khusus</t>
+          <t>https://finance.detik.com/bursa-dan-valas/d-8721341/bos-ojk-lapor-prabowo-kondisi-bursa-usai-msci-buka-opsi-turun-kasta</t>
         </is>
       </c>
     </row>
@@ -1779,22 +1803,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Prabowo Dapat Laporan Ada Tambang Raksasa Senilai Rp 5.400 T</t>
+          <t>Bank Mandiri Catat Laba Rp 45,5 T Hingga Kuartal III 2026</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Fri, 23 Oct 2026 05:55:00 +0700</t>
+          <t>Fri, 23 Oct 2026 19:31:15 +0700</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/22/presiden-prabowo-di-rakornas-tim-percepatan-akses-keuangan-daerah-tpakd-jiexpo-kemayoran-jakarta-kamis-22102026-muchlis-jr-bir-1792664303215_169.jpeg?w=360&amp;amp;q=90" /&gt; Presiden Prabowo Subianto mengaku dapat laporan ada tambang </t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/23/laba-bank-mandiri-tumbuh-207-persen-tembus-rp455-triliun-per-september-2026-1792754648866_169.jpeg?w=360&amp;amp;q=90" /&gt; Bank Mandiri mencatat laba bersih Rp45,5 triliun hingga September 2026, tumbuh 20,7 persen secara tahunan. Peny</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8719507/prabowo-dapat-laporan-ada-tambang-raksasa-senilai-rp-5-400-t</t>
+          <t>https://finance.detik.com/foto-bisnis/d-8721238/bank-mandiri-catat-laba-rp-45-5-t-hingga-kuartal-iii-2026</t>
         </is>
       </c>
     </row>
@@ -1806,22 +1830,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Pertamina Pasang Oil Boom di Sekitar Kapal Batumandi</t>
+          <t>Dukung Program B50, Agrinas Targetkan Kontribusi 600 Ribu KL Biodiesel</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Thu, 22 Oct 2026 22:46:34 +0700</t>
+          <t>Fri, 23 Oct 2026 19:23:29 +0700</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/22/pt-pertamina-trans-kontinental-ptk-1792683765501_169.jpeg?w=360&amp;amp;q=90" /&gt; Pertamina mengerahkan tim tanggap darurat Operasional Marine Tanjung Sekong dan Marine Tanjung Gerem untuk membantu penanganan kebakaran Kapal KMP Batum</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/23/agrinas-palma-1792756345406_169.jpeg?w=360&amp;amp;q=90" /&gt; PT Agrinas Palma Nusantara menargetkan kontribusi 600.000 kiloliter biodiesel untuk program B50 hingga Desember 2027, sambil mendampingi petani plasma.</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8719830/pertamina-pasang-oil-boom-di-sekitar-kapal-batumandi</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8721318/dukung-program-b50-agrinas-targetkan-kontribusi-600-ribu-kl-biodiesel</t>
         </is>
       </c>
     </row>
@@ -1833,22 +1857,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Rincian Stimulus Rp 31 Triliun Akhir Tahun: BSU hingga Rekening Gratis</t>
+          <t>Masuk PSN, Agrinas Palma Rencanakan Peremajaan Sawit di Torganda</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Thu, 22 Oct 2026 22:06:55 +0700</t>
+          <t>Fri, 23 Oct 2026 19:03:22 +0700</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/02/ilustrasi-bsu-kemnaker-rp-900000-1790934696631_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Koordinator Perekonomian Airlangga Hartarto menyampaikan pemerintah menyiapkan stimulus ekonomi sebesar Rp 31 triliun untuk kuartal IV 2026.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/23/agrinas-palma-1792756345345_169.jpeg?w=360&amp;amp;q=90" /&gt; PT Agrinas Palma Nusantara siapkan peremajaan kebun sawit 48.000 hektare setelah ditetapkan sebagai pelaksana Proyek Strategis Nasional.</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8719796/rincian-stimulus-rp-31-triliun-akhir-tahun-bsu-hingga-rekening-gratis</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8721281/masuk-psn-agrinas-palma-rencanakan-peremajaan-sawit-di-torganda</t>
         </is>
       </c>
     </row>
@@ -1860,22 +1884,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Potret Padatnya Pencari Kerja di Tengah Badai PHK</t>
+          <t>Bantu Suahasil Tambal Subsidi BBM, Bahlil Target PNBP Minerba Tembus Rp 165 T</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Thu, 22 Oct 2026 21:30:07 +0700</t>
+          <t>Fri, 23 Oct 2026 19:00:00 +0700</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/22/potret-padatnya-pencari-kerja-di-tengah-badai-phk-1792676014221_169.jpeg?w=360&amp;amp;q=90" /&gt; Pencari kerja memadati Karir Jakarta Expo 2026 di Jakarta. Lebih dari 28 ribu orang mendaftar untuk 12 ribu lowongan.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2024/01/04/kebutuhan-batu-bara-meningkat-begini-proses-bongkar-muat-di-pltu-tidore-1_169.jpeg?w=360&amp;amp;q=90" /&gt; Menko Hilirisasi dan Transisi Energi Bahlil Lahadalia menargetkan peningkatan PNBP mineral dan batu bara.</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/foto-bisnis/d-8719703/potret-padatnya-pencari-kerja-di-tengah-badai-phk</t>
+          <t>https://finance.detik.com/energi/d-8721264/bantu-suahasil-tambal-subsidi-bbm-bahlil-target-pnbp-minerba-tembus-rp-165-t</t>
         </is>
       </c>
     </row>
@@ -1887,22 +1911,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Danantara Bakal Umumkan Investasi Data Center dan AI</t>
+          <t>Indonesia Peringkat 14 Adopsi Kripto Global, Akun Tembus 22,93 Juta</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Thu, 22 Oct 2026 21:30:01 +0700</t>
+          <t>Fri, 23 Oct 2026 18:41:09 +0700</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/07/01/wisma-danantara-indonesia-1751345496255_169.jpeg?w=360&amp;amp;q=90" /&gt; Pengembangan infrastruktur digital dan AI menjadi salah satu prioritas investasi untuk meningkatkan daya saing dan kapasitas teknologi nasional.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/23/distrik-keuangan-jakarta-1792755401554.jpeg?w=360&amp;amp;q=90" /&gt; Indonesia menduduki peringkat ke-14 dalam adopsi kripto global. Meskipun turun, jumlah pengguna terus meningkat.</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8719620/danantara-bakal-umumkan-investasi-data-center-dan-ai</t>
+          <t>https://finance.detik.com/fintech/d-8721251/indonesia-peringkat-14-adopsi-kripto-global-akun-tembus-22-93-juta</t>
         </is>
       </c>
     </row>
@@ -1914,22 +1938,22 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>7 Provinsi Terdampak Karhutla Dapat Bantuan, Total Rp 1,23 Triliun</t>
+          <t>Terapkan Ekspor Satu Pintu Lewat DSI, Prabowo: Tindakan Survival!</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Thu, 22 Oct 2026 20:56:09 +0700</t>
+          <t>Fri, 23 Oct 2026 18:27:40 +0700</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/08/21/petugas-memadamkan-karhutla-di-kalimantan-1787304053622_169.jpeg?w=360&amp;amp;q=90" /&gt; Pemerintah mengirimkan bantuan dana ke tujuh provinsi terdampak kebakaran hutan dan lahan (karhutla). Total anggaran mencapai Rp 1,23 triliun.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/21/sidang-kabinet-paripurna-di-istana-kepresidenan-1792580318733_169.jpeg?w=360&amp;amp;q=90" /&gt; Presiden Prabowo Subianto menjelaskan kebijakan ekspor satu pintu adalah survival mode.</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8719722/7-provinsi-terdampak-karhutla-dapat-bantuan-total-rp-1-23-triliun</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8721226/terapkan-ekspor-satu-pintu-lewat-dsi-prabowo-tindakan-survival</t>
         </is>
       </c>
     </row>
@@ -1941,22 +1965,22 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Menteri UMKM Ungkap Alasan Wajib Halal Ditunda</t>
+          <t>Kemen PU &amp;amp; PT PP Tangani 31 Titik Longsor di Sumut, Progres Lampaui Target</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Thu, 22 Oct 2026 20:30:00 +0700</t>
+          <t>Fri, 23 Oct 2026 18:21:33 +0700</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/12/02/menteri-usaha-mikro-kecil-dan-menengah-umkm-maman-abdurrahman-1764677159466_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Usaha Mikro Kecil dan Menengah (UMKM) Maman Abdurrahman menyampaikan alasan kewajiban sertifikasi halal diundur menja</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/23/kemen-pu-pt-pp-tangani-31-titik-longsoran-di-sumut-progres-lampaui-target-1792754399461.jpeg?w=360&amp;amp;q=90" /&gt; PT PP (Persero) Tbk berkontribusi dalam pemulihan infrastruktur jalan pascabencana di Sumatera Utara dengan proyek se</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8719637/menteri-umkm-ungkap-alasan-wajib-halal-ditunda</t>
+          <t>https://finance.detik.com/infrastruktur/d-8721221/kemen-pu-pt-pp-tangani-31-titik-longsor-di-sumut-progres-lampaui-target</t>
         </is>
       </c>
     </row>
@@ -1968,22 +1992,22 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Bank Mandiri Tingkatkan Layanan Digital untuk Dorong Pertumbuhan Bisnis</t>
+          <t>Prabowo Minta KEK Bisa Sumbang Ekonomi RI hingga 1%</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Thu, 22 Oct 2026 20:06:47 +0700</t>
+          <t>Fri, 23 Oct 2026 17:51:49 +0700</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/22/bank-mandiri-1792674027427.png?w=360&amp;amp;q=90" /&gt; Bank Mandiri terus tingkatkan layanan untuk memenuhi ekspektasi nasabah. Fokus pada pengalaman pelanggan dan integrasi layanan digital dalam satu aplikasi.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/23/wakil-ketua-2-tim-pelaksana-dewan-kek-budi-santoso-1792752570074_169.jpeg?w=360&amp;amp;q=90" /&gt; Presiden Prabowo Subianto meminta agar Kawasan Ekonomi Khusus (KEK) dapat berkontribusi pada pertumbuhan ekonomi hingga 1% tahun depan.</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/moneter/d-8719674/bank-mandiri-tingkatkan-layanan-digital-untuk-dorong-pertumbuhan-bisnis</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8721158/prabowo-minta-kek-bisa-sumbang-ekonomi-ri-hingga-1</t>
         </is>
       </c>
     </row>
@@ -1995,22 +2019,22 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Anggaran Rekening Gratis Turun dari Rp 3,84 T Jadi Rp 1,28 T</t>
+          <t>Bayar Premi Asuransi Mulai Rp 1.000/Hari, Ini Proteksi yang Didapat</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Thu, 22 Oct 2026 20:00:20 +0700</t>
+          <t>Fri, 23 Oct 2026 17:35:24 +0700</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/10/27/bi-pertahankan-bi-rate-475-persen-untuk-jaga-stabilitas-rupiah-1761539775425_169.jpeg?w=360&amp;amp;q=90" /&gt; Pemerintah mengubah anggaran program rekening gratis dari Rp 3,84 triliun menjadi Rp 1,28 triliun, hal ini dilakukan setelah</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2022/02/04/ilustrasi-asuransi_169.jpeg?w=360&amp;amp;q=90" /&gt; PT Asuransi BRI Life meluncurkan produk asuransi Corporate Eazy (COZY) yang fleksibel, menawarkan manfaat dasar dan tambahan sesuai kebutuhan perusahaan.</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8719657/anggaran-rekening-gratis-turun-dari-rp-3-84-t-jadi-rp-1-28-t</t>
+          <t>https://finance.detik.com/moneter/d-8721176/bayar-premi-asuransi-mulai-rp-1-000-hari-ini-proteksi-yang-didapat</t>
         </is>
       </c>
     </row>
@@ -2022,22 +2046,22 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>UMK Lokal Dapat Diskon 50% Biaya Administrasi Toko Online Selamanya</t>
+          <t>TNI-Polri Siap Kawal Investasi di Jateng</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Thu, 22 Oct 2026 20:00:17 +0700</t>
+          <t>Fri, 23 Oct 2026 17:27:27 +0700</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/22/menteri-usaha-mikro-kecil-dan-menengah-umkm-maman-abdurrahman-1792667292505_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri UMKM Maman Abdurrahman menyampaikan kebijakan ini akan berlaku secara permanen.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/23/forum-investasi-jawa-tengah-1792743658262_169.png?w=360&amp;amp;q=90" /&gt; TNI-Polri ikut mengawal realisasi investasi di Jawa Tengah, begini upayanya.</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8719617/umk-lokal-dapat-diskon-50-biaya-administrasi-toko-online-selamanya</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8721112/tni-polri-siap-kawal-investasi-di-jateng</t>
         </is>
       </c>
     </row>
@@ -2049,22 +2073,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Putri Tanjung Bicara Pentingnya Ekosistem Kreatif yang Sehat</t>
+          <t>Eksplorasi Privilege Kesehatan MCU-Genomics dari BRI Private &amp;amp; Prioritas</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Thu, 22 Oct 2026 19:31:06 +0700</t>
+          <t>Fri, 23 Oct 2026 17:25:08 +0700</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/22/putri-tanjung-bicara-pentingnya-ekosistem-kreatif-yang-sehat-1792672229786_43.jpeg?w=360&amp;amp;q=90" /&gt; Putri Tanjung dorong penguatan ekosistem ekonomi kreatif Indonesia agar IP lokal bersaing global. Kolaborasi penting untuk kemb</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/23/prodia-1792751083734_169.jpeg?w=360&amp;amp;q=90" /&gt; BRI dan Prodia hadirkan layanan kesehatan eksklusif untuk nasabah Private dan Prioritas, termasuk pemeriksaan rutin, MCU, dan genomik dengan berbagai manfaat.</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8719633/putri-tanjung-bicara-pentingnya-ekosistem-kreatif-yang-sehat</t>
+          <t>https://finance.detik.com/moneter/d-8721108/eksplorasi-privilege-kesehatan-mcu-genomics-dari-bri-private-prioritas</t>
         </is>
       </c>
     </row>
@@ -2076,22 +2100,22 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>OJK Ungkap Progres Demutualisasi Bursa: BEI Gelar RUPS Akhir Oktober 2026</t>
+          <t>Gubernur Jateng Mau Jemput Investasi Vietnam</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Thu, 22 Oct 2026 19:30:11 +0700</t>
+          <t>Fri, 23 Oct 2026 17:01:55 +0700</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2016/12/30/ed5ec33a-5357-40f8-8f66-6713c06687ea_169.jpg?w=360&amp;amp;q=90" /&gt; OJK mengungkap progres demutualisasi BEI, dengan RUPS dijadwalkan pada 28 Oktober 2026 untuk membahas perubahan anggaran dasar dan langkah selanjutnya.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/23/gubernur-jateng-irjen-purn-ahmad-luthfi-1792743908471_169.png?w=360&amp;amp;q=90" /&gt; Gubernur Jateng Ahmad Luthfi bersiap untuk menjemput investasi ke Vietnam.</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/moneter/d-8719551/ojk-ungkap-progres-demutualisasi-bursa-bei-gelar-rups-akhir-oktober-2026</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8721034/gubernur-jateng-mau-jemput-investasi-vietnam</t>
         </is>
       </c>
     </row>
@@ -2103,22 +2127,22 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>BRI Siapkan Buyback Saham Tahap II Senilai Rp 1 Triliun</t>
+          <t>Prabowo Respons Antrean Panjang BBM di Bali, Kasih Titah Khusus ke Bahlil Cs</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Thu, 22 Oct 2026 19:12:42 +0700</t>
+          <t>Fri, 23 Oct 2026 16:42:52 +0700</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/22/ilustrasi-gedung-bri-1792671138276.jpeg?w=360&amp;amp;q=90" /&gt; PT BRI umumkan rencana buyback saham Tahap II senilai Rp 1 triliun. Aksi ini bertujuan tingkatkan nilai pemegang saham dan dukung pertumbuhan jangka panjang.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/21/presiden-prabowo-subianto-1792590961586_169.jpeg?w=360&amp;amp;q=90" /&gt; Presiden Prabowo Subianto memberikan titah khusus soal penanganan krisis BBM di Bali.</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/bursa-dan-valas/d-8719613/bri-siapkan-buyback-saham-tahap-ii-senilai-rp-1-triliun</t>
+          <t>https://finance.detik.com/energi/d-8721000/prabowo-respons-antrean-panjang-bbm-di-bali-kasih-titah-khusus-ke-bahlil-cs</t>
         </is>
       </c>
     </row>
@@ -2130,22 +2154,22 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Akses Penanjakan Bromo Dibuka Lagi Pascakebakaran, Simak Aturan dan Kuotanya</t>
+          <t>Rute Transjakarta Dialihkan Selama Jakarta Running Festival, Ini Daftarnya</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Fri, 23 Oct 2026 06:30:16 +0700</t>
+          <t>Fri, 23 Oct 2026 20:12:23 +0700</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Pengunjung dan pelaku jasa wisata harus patuhi semua aturan demi mencegah titik api kembali muncul.</t>
+          <t>Penyesuaian ini dilakukan agar mobilitas peserta festival dan pelanggan tetap berjalan lancar.</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8319478/akses-penanjakan-bromo-dibuka-lagi-pascakebakaran-simak-aturan-dan-kuotanya</t>
+          <t>https://www.liputan6.com/news/read/8320106/rute-transjakarta-dialihkan-selama-jakarta-running-festival-ini-daftarnya</t>
         </is>
       </c>
     </row>
@@ -2157,22 +2181,22 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Peringati Pink Month, Ribuan Warga Venezuela Turun ke Jalan</t>
+          <t>Kronologi Terbongkarnya Pabrik Sabu Blue Ice di Pidie Aceh</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Fri, 23 Oct 2026 06:00:56 +0700</t>
+          <t>Fri, 23 Oct 2026 19:57:43 +0700</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Ribuan perempuan dan pegiat kesehatan memadati jalanan Caracas, Venezuela, Kamis (22/10/2026), dalam aksi memperingati Bulan Kesadaran Kanker Payudara atau Pink Month. Para peserta membawa balon merah muda, spanduk, dan bendera Venezuela sebagai bentuk solidaritas bagi pasien kanker payudara dan par</t>
+          <t>Polri mengamankan barang bukti sabu kualias premiun alias Blue Ice seberat 1,2 ton.</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/photo/read/8319472/peringati-pink-month-ribuan-warga-venezuela-turun-ke-jalan</t>
+          <t>https://www.liputan6.com/news/read/8320099/kronologi-terbongkarnya-pabrik-sabu-blue-ice-di-pidie-aceh</t>
         </is>
       </c>
     </row>
@@ -2184,22 +2208,22 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Satgas PKH Cabut Izin Tambang PT KEL 3.500 Hektare di Papua</t>
+          <t>Pramono Berharap Warga Dukung JRF 2026 Akhir Pekan Ini</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Fri, 23 Oct 2026 05:39:32 +0700</t>
+          <t>Fri, 23 Oct 2026 19:46:00 +0700</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Jaksa Agung menyebut PT KEL terbukti melakukan pertambangan emas secara ilegal baik di dalam maupun di luar Wilayah Izin Usaha Pertambangan.</t>
+          <t>Pramono Anung pastikan Pemprov DKI sediakan fasilitas transportasi gratis dan pengaturan lalu lintas.</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8319469/satgas-pkh-cabut-izin-tambang-pt-kel-3500-hektare-di-papua</t>
+          <t>https://www.liputan6.com/news/read/8320094/pramono-berharap-warga-dukung-jrf-2026-akhir-pekan-ini</t>
         </is>
       </c>
     </row>
@@ -2211,22 +2235,22 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Jakarta International Literary Festival 2026 Resmi Dibuka</t>
+          <t>Penampakan 4 Mobil Sitaan KPK di Kasus Korupsi Dana Bencana BNPB</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Fri, 23 Oct 2026 05:30:48 +0700</t>
+          <t>Fri, 23 Oct 2026 19:25:20 +0700</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Mengusung tema 'Living Space', Jakarta International Literary Festival 2026 resmi dibuka di Graha Bhakti Budaya, Taman Ismail Marzuki.</t>
+          <t>Dengan penyitaan terbaru ini, total empat mobil telah diamankan penyidik KPK.</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8319467/jakarta-international-literary-festival-2026-resmi-dibuka</t>
+          <t>https://www.liputan6.com/news/read/8320080/penampakan-4-mobil-sitaan-kpk-di-kasus-korupsi-dana-bencana-bnpb</t>
         </is>
       </c>
     </row>
@@ -2238,22 +2262,22 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>40 Tokoh Ajukan 'Amicus Curiae' untuk Eks Ketua Ombudsman</t>
+          <t>Dilaporkan Tokoh Adat Papua, Sutradara Film Pesta Babi Dipanggil Polisi</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Fri, 23 Oct 2026 05:17:54 +0700</t>
+          <t>Fri, 23 Oct 2026 19:21:28 +0700</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Perkara yang menjerat mantan Ketua Ombudsman RI Hery Susanto memasuki babak baru.</t>
+          <t>Pemeriksaan dijadwalkan pada Selasa, 27 Oktober 2026.</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8319466/40-tokoh-ajukan-amicus-curiae-untuk-eks-ketua-ombudsman</t>
+          <t>https://www.liputan6.com/news/read/8320074/dilaporkan-tokoh-adat-papua-sutradara-film-pesta-babi-dipanggil-polisi</t>
         </is>
       </c>
     </row>
@@ -2265,22 +2289,22 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Bareskrim Bongkar Judi Online Bermodus Permainan di Jakbar</t>
+          <t>NasDem Soroti Kesehatan Mental Ibu, 57 Persen Alami Baby Blues</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Fri, 23 Oct 2026 00:48:31 +0700</t>
+          <t>Fri, 23 Oct 2026 18:36:29 +0700</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Empat tersangka ditangkap. Mereka memiliki peran sendiri-sendiri.</t>
+          <t>Kesehatan mental ibu di antaranya berlanjut dari baby blues menjadi depresi pascamelahirkan.</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8319448/bareskrim-bongkar-judi-online-bermodus-permainan-di-jakbar</t>
+          <t>https://www.liputan6.com/news/read/8320046/nasdem-soroti-kesehatan-mental-ibu-57-persen-alami-baby-blues</t>
         </is>
       </c>
     </row>
@@ -2292,22 +2316,22 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Prabowo Sebut Indonesia Negara Ekonomi Terbesar ke-7 di Dunia</t>
+          <t>Prabowo Beberkan Penindakan Pelanggaran MBG, Ini Hasillnya</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Thu, 22 Oct 2026 22:40:48 +0700</t>
+          <t>Fri, 23 Oct 2026 18:20:16 +0700</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Prabowo menilai capaian tersebut menunjukkan kekuatan ekonomi Indonesia.</t>
+          <t>Prabowo menyampaikan hal tersebut dalam Sidang Kabinet Paripurna di Kompleks Istana Kepresidenan.</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8319421/prabowo-sebut-indonesia-negara-ekonomi-terbesar-ke-7-di-dunia</t>
+          <t>https://www.liputan6.com/news/read/8320025/prabowo-beberkan-penindakan-pelanggaran-mbg-ini-hasillnya</t>
         </is>
       </c>
     </row>
@@ -2319,22 +2343,22 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Prabowo Janji Tambah Anggaran untuk Provinsi dan Kabupaten</t>
+          <t>Korban Pembacokan di Jaktim Ternyata Eks Anggota Kopassus</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Thu, 22 Oct 2026 23:00:34 +0700</t>
+          <t>Fri, 23 Oct 2026 17:52:34 +0700</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Praboowo meyakini jumlah anggaran yang disalurkan ke daerah akan meningkat tahun depan.</t>
+          <t>Korban bernama Muhammad Fahrul (48).</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8319415/prabowo-janji-tambah-anggaran-untuk-provinsi-dan-kabupaten</t>
+          <t>https://www.liputan6.com/news/read/8320002/korban-pembacokan-di-jaktim-ternyata-eks-anggota-kopassus</t>
         </is>
       </c>
     </row>
@@ -2346,22 +2370,22 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>KPK Tahan 7 Tersangka Baru Kasus Korupsi Proyek Jalan BBPJN Sumut</t>
+          <t>Kronologi Penyelundupan 1,16 Ton Ketamin di Perairan Belawan</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Thu, 22 Oct 2026 22:04:43 +0700</t>
+          <t>Fri, 23 Oct 2026 18:42:18 +0700</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Salah satu tersangka yang ditahan KPK adalah mantan Kepala BBPJN Sumut, Stanley Cicero Haggard Tuapattinaja.</t>
+          <t>Kapal terdeteksi melakukan pergerakan tidak biasa di Selat Malaka dan Laut Andaman.</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8319397/kpk-tahan-7-tersangka-baru-kasus-korupsi-proyek-jalan-bbpjn-sumut</t>
+          <t>https://www.liputan6.com/news/read/8319985/kronologi-penyelundupan-116-ton-ketamin-di-perairan-belawan</t>
         </is>
       </c>
     </row>
@@ -2373,22 +2397,22 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Judi Online hingga Narkoba Disorot, Ini Pesan Polri di Kemah Kebangsaan</t>
+          <t>Kasus Judi Online Boxkia, Terungkap Omzet Rp 2 Miliar Per Bulan</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Thu, 22 Oct 2026 22:01:42 +0700</t>
+          <t>Fri, 23 Oct 2026 17:17:39 +0700</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Pelajar dari berbagai sekolahan mengikuti kemah kebangsaan sebagai upaya menanamkan cinta Tanah Air.</t>
+          <t>Bareskrim Polri mengungkap praktik perjudian online melalui situs Boxkia.</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8319395/judi-online-hingga-narkoba-disorot-ini-pesan-polri-di-kemah-kebangsaan</t>
+          <t>https://www.liputan6.com/news/read/8319974/kasus-judi-online-boxkia-terungkap-omzet-rp-2-miliar-per-bulan</t>
         </is>
       </c>
     </row>
@@ -2400,22 +2424,22 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Prabowo Bidik Penyaluran Kredit Rakyat Rp 400 Triliun pada 2027</t>
+          <t>Kapolri Beberkan Data Perorangan dan Korporasi Terseret Kebakaran Hutan</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Thu, 22 Oct 2026 21:17:26 +0700</t>
+          <t>Fri, 23 Oct 2026 17:15:00 +0700</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Pembiayaan tersebut akan menyasar petani, nelayan, hingga masyarakat pedesaan dan kelompok berpenghasilan rendah.</t>
+          <t>Total 35.390 hektare lahan terbakar, dengan penegakan hukum terus berjalan.</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8319370/prabowo-bidik-penyaluran-kredit-rakyat-rp-400-triliun-pada-2027</t>
+          <t>https://www.liputan6.com/news/read/8319968/kapolri-beberkan-data-perorangan-dan-korporasi-terseret-kebakaran-hutan</t>
         </is>
       </c>
     </row>
@@ -2427,22 +2451,22 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Hadiri Rakornas TPAKD, Mendagri Pastikan Bantuan Apresiasi Pemda TA 2027 Tetap Ada</t>
+          <t>Infografis: 10 Negara dengan Pertumbuhan Orang Kaya Tertinggi</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Thu, 22 Oct 2026 21:04:48 +0700</t>
+          <t>Fri, 23 Oct 2026 17:02:12 +0700</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Berdasarkan hasil koordinasi dengan Menteri Keuangan Suahasil Nazara, pemerintah menyiapkan Rp 2 triliun untuk TA 2027.</t>
+          <t>Indonesia, Arab Saudi, dan Vietnam masuk dalam daftar negara dengan proyeksi pertumbuhan orang super kaya yang pesat.</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8319365/hadiri-rakornas-tpakd-mendagri-pastikan-bantuan-apresiasi-pemda-ta-2027-tetap-ada</t>
+          <t>https://www.liputan6.com/news/read/8319962/infografis-10-negara-dengan-pertumbuhan-orang-kaya-tertinggi</t>
         </is>
       </c>
     </row>
@@ -2454,22 +2478,22 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Prabowo Minta Menteri Selektif Beri Konsesi Tambang</t>
+          <t>Limbah Dibidik Jadi Sumber Energi Rendah Karbon</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Thu, 22 Oct 2026 20:44:29 +0700</t>
+          <t>Fri, 23 Oct 2026 16:50:50 +0700</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Prabowo meminta agar izin konsesi diberikan secara selektif dan memastikan pihak tersebut memiliki kemampuan untuk mengelola SDA secara optimal.</t>
+          <t>Limbah tak hanya menjadi residu tetapi bisa menjadi energi yang berpotensi memberikan nilai tambah.</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8319349/prabowo-minta-menteri-selektif-beri-konsesi-tambang</t>
+          <t>https://www.liputan6.com/news/read/8319948/limbah-dibidik-jadi-sumber-energi-rendah-karbon</t>
         </is>
       </c>
     </row>
@@ -2481,22 +2505,22 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Kemendagri Minta Pemda Evaluasi Aturan yang Bebani Warga</t>
+          <t>Ketika Kreativitas dan Olahraga Menggerakkan Roda Ekonomi Jakarta</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Thu, 22 Oct 2026 20:36:21 +0700</t>
+          <t>Fri, 23 Oct 2026 17:54:23 +0700</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Sejumlah tahapan perlu dikaji agar dapat dilaksanakan secara paralel sehingga pelayanan menjadi lebih sederhana, cepat, dan efisien.</t>
+          <t>Perputaran ekonomi Jakarta meningkat pesat berkat event kreatif dan olahraga.</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8319345/kemendagri-minta-pemda-evaluasi-aturan-yang-bebani-warga</t>
+          <t>https://www.liputan6.com/news/read/8319937/ketika-kreativitas-dan-olahraga-menggerakkan-roda-ekonomi-jakarta</t>
         </is>
       </c>
     </row>
@@ -2508,22 +2532,22 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Santri Tak Cuma Soal Sarung dan Kitab Kuning</t>
+          <t>Dua Tahun Prabowo-Gibran, Revitalisasi Sekolah Diperluas</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Thu, 22 Oct 2026 20:05:19 +0700</t>
+          <t>Fri, 23 Oct 2026 15:43:51 +0700</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Santri masa kini tak hanya belajar agama, tetapi juga mengembangkan diri untuk menghadapi tantangan zaman.</t>
+          <t>Revitalisasi ditujukan untuk memperbaiki fasilitas sekolah.</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8319318/santri-tak-cuma-soal-sarung-dan-kitab-kuning</t>
+          <t>https://www.liputan6.com/news/read/8319883/dua-tahun-prabowo-gibran-revitalisasi-sekolah-diperluas</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data pasar & berita - 2026-10-25 23:38 UTC
</commit_message>
<xml_diff>
--- a/data/market_news_latest.xlsx
+++ b/data/market_news_latest.xlsx
@@ -500,7 +500,7 @@
         <v>0.95</v>
       </c>
       <c r="H2" t="n">
-        <v>0</v>
+        <v>397036500</v>
       </c>
     </row>
     <row r="3">
@@ -521,20 +521,20 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>7663.4302</v>
+        <v>7623.6802</v>
       </c>
       <c r="F3" t="n">
-        <v>-93.7397</v>
+        <v>-39.75</v>
       </c>
       <c r="G3" t="n">
-        <v>-1.21</v>
+        <v>-0.52</v>
       </c>
       <c r="H3" t="n">
-        <v>5972620000</v>
+        <v>5062330000</v>
       </c>
     </row>
     <row r="4">
@@ -555,20 +555,20 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>52867.9805</v>
+        <v>52215.1602</v>
       </c>
       <c r="F4" t="n">
-        <v>11.8906</v>
+        <v>-652.8203</v>
       </c>
       <c r="G4" t="n">
-        <v>0.02</v>
+        <v>-1.23</v>
       </c>
       <c r="H4" t="n">
-        <v>506190000</v>
+        <v>348500000</v>
       </c>
     </row>
     <row r="5">
@@ -589,20 +589,20 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>26008.8594</v>
+        <v>25955.3398</v>
       </c>
       <c r="F5" t="n">
-        <v>-694</v>
+        <v>-53.5195</v>
       </c>
       <c r="G5" t="n">
-        <v>-2.6</v>
+        <v>-0.21</v>
       </c>
       <c r="H5" t="n">
-        <v>9012120000</v>
+        <v>6554790000</v>
       </c>
     </row>
     <row r="6">
@@ -636,7 +636,7 @@
         <v>-0.34</v>
       </c>
       <c r="H6" t="n">
-        <v>0</v>
+        <v>208600000</v>
       </c>
     </row>
     <row r="7">
@@ -670,7 +670,7 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="H7" t="n">
-        <v>0</v>
+        <v>3842800000</v>
       </c>
     </row>
     <row r="8">
@@ -695,16 +695,16 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>3690.4753</v>
+        <v>3690.4751</v>
       </c>
       <c r="F8" t="n">
-        <v>32.4495</v>
+        <v>32.4492</v>
       </c>
       <c r="G8" t="n">
         <v>0.89</v>
       </c>
       <c r="H8" t="n">
-        <v>3744683648</v>
+        <v>552800</v>
       </c>
     </row>
     <row r="9">
@@ -729,16 +729,16 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>10658.3203</v>
+        <v>10690.4004</v>
       </c>
       <c r="F9" t="n">
-        <v>-66.6797</v>
+        <v>-34.5996</v>
       </c>
       <c r="G9" t="n">
-        <v>-0.62</v>
+        <v>-0.32</v>
       </c>
       <c r="H9" t="n">
-        <v>0</v>
+        <v>697030600</v>
       </c>
     </row>
     <row r="10">
@@ -763,16 +763,16 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>25125.1406</v>
+        <v>25181.6504</v>
       </c>
       <c r="F10" t="n">
-        <v>-246.6094</v>
+        <v>-190.0996</v>
       </c>
       <c r="G10" t="n">
-        <v>-0.97</v>
+        <v>-0.75</v>
       </c>
       <c r="H10" t="n">
-        <v>0</v>
+        <v>58950600</v>
       </c>
     </row>
     <row r="11">
@@ -806,7 +806,7 @@
         <v>0.13</v>
       </c>
       <c r="H11" t="n">
-        <v>0</v>
+        <v>388429200</v>
       </c>
     </row>
     <row r="12">
@@ -827,17 +827,17 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>18050</v>
+        <v>17956</v>
       </c>
       <c r="F12" t="n">
-        <v>42</v>
+        <v>-97</v>
       </c>
       <c r="G12" t="n">
-        <v>0.23</v>
+        <v>-0.54</v>
       </c>
       <c r="H12" t="n">
         <v>0</v>
@@ -861,17 +861,17 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>101.686</v>
+        <v>101.765</v>
       </c>
       <c r="F13" t="n">
-        <v>0.076</v>
+        <v>-0.045</v>
       </c>
       <c r="G13" t="n">
-        <v>0.07000000000000001</v>
+        <v>-0.04</v>
       </c>
       <c r="H13" t="n">
         <v>0</v>
@@ -895,17 +895,17 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>156.391</v>
+        <v>156.888</v>
       </c>
       <c r="F14" t="n">
-        <v>-1.741</v>
+        <v>0.394</v>
       </c>
       <c r="G14" t="n">
-        <v>-1.1</v>
+        <v>0.25</v>
       </c>
       <c r="H14" t="n">
         <v>0</v>
@@ -933,13 +933,13 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>0.4957</v>
+        <v>0.4988</v>
       </c>
       <c r="F15" t="n">
-        <v>0.0004</v>
+        <v>0.0035</v>
       </c>
       <c r="G15" t="n">
-        <v>0.08</v>
+        <v>0.71</v>
       </c>
       <c r="H15" t="n">
         <v>0</v>
@@ -967,13 +967,13 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>0.5281</v>
+        <v>0.5315</v>
       </c>
       <c r="F16" t="n">
-        <v>-0.0005999999999999999</v>
+        <v>0.0028</v>
       </c>
       <c r="G16" t="n">
-        <v>-0.11</v>
+        <v>0.53</v>
       </c>
       <c r="H16" t="n">
         <v>0</v>
@@ -1001,13 +1001,13 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>0.4037</v>
+        <v>0.4032</v>
       </c>
       <c r="F17" t="n">
-        <v>0.0015</v>
+        <v>0.001</v>
       </c>
       <c r="G17" t="n">
-        <v>0.37</v>
+        <v>0.25</v>
       </c>
       <c r="H17" t="n">
         <v>0</v>
@@ -1031,20 +1031,20 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>81.73999999999999</v>
+        <v>81.34</v>
       </c>
       <c r="F18" t="n">
-        <v>1.5</v>
+        <v>-0.4</v>
       </c>
       <c r="G18" t="n">
-        <v>1.87</v>
+        <v>-0.49</v>
       </c>
       <c r="H18" t="n">
-        <v>64652900</v>
+        <v>35120900</v>
       </c>
     </row>
     <row r="19">
@@ -1065,20 +1065,20 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>77.09999999999999</v>
+        <v>77.05</v>
       </c>
       <c r="F19" t="n">
-        <v>0.12</v>
+        <v>-0.05</v>
       </c>
       <c r="G19" t="n">
-        <v>0.16</v>
+        <v>-0.06</v>
       </c>
       <c r="H19" t="n">
-        <v>47048900</v>
+        <v>56640900</v>
       </c>
     </row>
     <row r="20">
@@ -1099,20 +1099,20 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>4041</v>
+        <v>4012</v>
       </c>
       <c r="F20" t="n">
-        <v>-19.3999</v>
+        <v>4.1001</v>
       </c>
       <c r="G20" t="n">
-        <v>-0.48</v>
+        <v>0.1</v>
       </c>
       <c r="H20" t="n">
-        <v>89778</v>
+        <v>3340</v>
       </c>
     </row>
     <row r="21">
@@ -1133,20 +1133,20 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>101.02</v>
+        <v>102.29</v>
       </c>
       <c r="F21" t="n">
-        <v>1.55</v>
+        <v>-0.98</v>
       </c>
       <c r="G21" t="n">
-        <v>1.56</v>
+        <v>-0.95</v>
       </c>
       <c r="H21" t="n">
-        <v>106313</v>
+        <v>10295</v>
       </c>
     </row>
     <row r="22">
@@ -1167,20 +1167,20 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="E22" t="n">
-        <v>110.06</v>
+        <v>110.82</v>
       </c>
       <c r="F22" t="n">
-        <v>-3.11</v>
+        <v>-5.9</v>
       </c>
       <c r="G22" t="n">
-        <v>-2.75</v>
+        <v>-5.05</v>
       </c>
       <c r="H22" t="n">
-        <v>14855</v>
+        <v>741</v>
       </c>
     </row>
     <row r="23">
@@ -1201,20 +1201,20 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="E23" t="n">
-        <v>6.4655</v>
+        <v>6.4925</v>
       </c>
       <c r="F23" t="n">
-        <v>0.103</v>
+        <v>0.0165</v>
       </c>
       <c r="G23" t="n">
-        <v>1.62</v>
+        <v>0.25</v>
       </c>
       <c r="H23" t="n">
-        <v>20732</v>
+        <v>782</v>
       </c>
     </row>
     <row r="24">
@@ -1235,20 +1235,20 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="E24" t="n">
-        <v>61.72</v>
+        <v>62.01</v>
       </c>
       <c r="F24" t="n">
-        <v>-1.85</v>
+        <v>0.29</v>
       </c>
       <c r="G24" t="n">
-        <v>-2.91</v>
+        <v>0.47</v>
       </c>
       <c r="H24" t="n">
-        <v>28385500</v>
+        <v>22024100</v>
       </c>
     </row>
     <row r="25">
@@ -1273,13 +1273,13 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>20.22</v>
+        <v>19.45</v>
       </c>
       <c r="F25" t="n">
-        <v>1.19</v>
+        <v>0.42</v>
       </c>
       <c r="G25" t="n">
-        <v>6.25</v>
+        <v>2.21</v>
       </c>
       <c r="H25" t="n">
         <v>0</v>
@@ -1303,20 +1303,20 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="E26" t="n">
-        <v>81533.47659999999</v>
+        <v>80154.7031</v>
       </c>
       <c r="F26" t="n">
-        <v>221.5859</v>
+        <v>-636.1328</v>
       </c>
       <c r="G26" t="n">
-        <v>0.27</v>
+        <v>-0.79</v>
       </c>
       <c r="H26" t="n">
-        <v>24775368704</v>
+        <v>11814104064</v>
       </c>
     </row>
     <row r="27">
@@ -1749,22 +1749,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Forum Investasi Jateng Bahas Strategi KEK Batang Hadapi Persaingan Global</t>
+          <t>Serangan Rudal Rusia Hantam Kharkiv, Pusat Perbelanjaan Terbakar</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Fri, 23 Oct 2026 20:00:09 +0700</t>
+          <t>Mon, 26 Oct 2026 06:00:16 +0700</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/23/forum-investasi-jateng-bahas-strategi-kek-batang-hadapi-persaingan-global-1792756806815_169.jpeg?w=360&amp;amp;q=90" /&gt; Jawa Tengah memperkuat strategi menarik investasi melalui KEK Batang dan kolaborasi lintas instansi. Keamanan dan</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/25/serangan-rudal-rusia-hantam-kharkiv-pusat-perbelanjaan-terbakar-1792913695273_169.jpeg?w=360&amp;amp;q=90" /&gt; Serangan rudal Rusia menghantam pusat perbelanjaan di Kharkiv, Ukraina, memicu kebakaran dan merusak bangunan sipil.</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/foto-bisnis/d-8721287/forum-investasi-jateng-bahas-strategi-kek-batang-hadapi-persaingan-global</t>
+          <t>https://finance.detik.com/foto-bisnis/d-8723283/serangan-rudal-rusia-hantam-kharkiv-pusat-perbelanjaan-terbakar</t>
         </is>
       </c>
     </row>
@@ -1776,22 +1776,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Bos OJK Lapor Prabowo Kondisi Bursa Usai MSCI Buka Opsi Turun Kasta</t>
+          <t>Singapura Singgung soal Kontrak Usai RI Pangkas Ekspor Gas</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Fri, 23 Oct 2026 20:00:05 +0700</t>
+          <t>Mon, 26 Oct 2026 05:55:43 +0700</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/08/03/frederica-widyasari-dewi-1785765447950_169.jpeg?w=360&amp;amp;q=90" /&gt; Ketua DK OJK Friderica Widyasari Dewi memberikan laporan ke Presiden Prabowo Subianto soal kondisi bursa efek.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2024/05/16/sosok-lawrence-wong-perdana-menteri-baru-singapura-1_169.jpeg?w=360&amp;amp;q=90" /&gt; Perdana Menteri (PM) Singapura Lawrence Wong akhirnya angkat bicara merespons kebijakan Indonesia mengurangi ekspor gas.</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/bursa-dan-valas/d-8721341/bos-ojk-lapor-prabowo-kondisi-bursa-usai-msci-buka-opsi-turun-kasta</t>
+          <t>https://finance.detik.com/energi/d-8723774/singapura-singgung-soal-kontrak-usai-ri-pangkas-ekspor-gas</t>
         </is>
       </c>
     </row>
@@ -1803,22 +1803,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Bank Mandiri Catat Laba Rp 45,5 T Hingga Kuartal III 2026</t>
+          <t>Mentan Ungkap Anomali Harga Telur: Stok Melimpah, tapi Harga Naik</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Fri, 23 Oct 2026 19:31:15 +0700</t>
+          <t>Sun, 25 Oct 2026 22:00:44 +0700</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/23/laba-bank-mandiri-tumbuh-207-persen-tembus-rp455-triliun-per-september-2026-1792754648866_169.jpeg?w=360&amp;amp;q=90" /&gt; Bank Mandiri mencatat laba bersih Rp45,5 triliun hingga September 2026, tumbuh 20,7 persen secara tahunan. Peny</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/07/28/pemerintah-pastikan-beras-hingga-daging-ayam-dalam-kondisi-surplus-1785222178359_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Pertanian Amran Sulaiman mengungkapkan harga telur saat ini mengalami anomali.</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/foto-bisnis/d-8721238/bank-mandiri-catat-laba-rp-45-5-t-hingga-kuartal-iii-2026</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8723273/mentan-ungkap-anomali-harga-telur-stok-melimpah-tapi-harga-naik</t>
         </is>
       </c>
     </row>
@@ -1830,22 +1830,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Dukung Program B50, Agrinas Targetkan Kontribusi 600 Ribu KL Biodiesel</t>
+          <t>ESDM Buka Lowongan 108 Pengawal Energi, Gaji hingga Rp 6,5 Juta/Bulan</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Fri, 23 Oct 2026 19:23:29 +0700</t>
+          <t>Sun, 25 Oct 2026 21:00:16 +0700</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/23/agrinas-palma-1792756345406_169.jpeg?w=360&amp;amp;q=90" /&gt; PT Agrinas Palma Nusantara menargetkan kontribusi 600.000 kiloliter biodiesel untuk program B50 hingga Desember 2027, sambil mendampingi petani plasma.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/05/11/ilustrasi-job-fair-atau-lowongan-kerja-1746929349100_169.jpeg?w=360&amp;amp;q=90" /&gt; Kementerian Energi dan Sumber Daya Mineral (ESDM) membuka kesempatan kerja untuk posisi verifikator lapangan dan analis dalam Program Pengawal Energ</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8721318/dukung-program-b50-agrinas-targetkan-kontribusi-600-ribu-kl-biodiesel</t>
+          <t>https://finance.detik.com/energi/d-8723623/esdm-buka-lowongan-108-pengawal-energi-gaji-hingga-rp-6-5-juta-bulan</t>
         </is>
       </c>
     </row>
@@ -1857,22 +1857,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Masuk PSN, Agrinas Palma Rencanakan Peremajaan Sawit di Torganda</t>
+          <t>Mentan Lapor Prabowo 500 Ribu Ha Rawa Disulap Jadi Sawah</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Fri, 23 Oct 2026 19:03:22 +0700</t>
+          <t>Sun, 25 Oct 2026 20:00:40 +0700</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/23/agrinas-palma-1792756345345_169.jpeg?w=360&amp;amp;q=90" /&gt; PT Agrinas Palma Nusantara siapkan peremajaan kebun sawit 48.000 hektare setelah ditetapkan sebagai pelaksana Proyek Strategis Nasional.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/10/10/mentan-amran-sulaiman-1760077106363_169.jpeg?w=360&amp;amp;q=90" /&gt; Pemerintah terus menambah area tanam pangan untuk memenuhi kebutuhan pangan dalam negeri.</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8721281/masuk-psn-agrinas-palma-rencanakan-peremajaan-sawit-di-torganda</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8723304/mentan-lapor-prabowo-500-ribu-ha-rawa-disulap-jadi-sawah</t>
         </is>
       </c>
     </row>
@@ -1884,22 +1884,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Bantu Suahasil Tambal Subsidi BBM, Bahlil Target PNBP Minerba Tembus Rp 165 T</t>
+          <t>Petani Ungkap Biang Kerok Harga Cabai Masih Mahal</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Fri, 23 Oct 2026 19:00:00 +0700</t>
+          <t>Sun, 25 Oct 2026 19:00:31 +0700</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2024/01/04/kebutuhan-batu-bara-meningkat-begini-proses-bongkar-muat-di-pltu-tidore-1_169.jpeg?w=360&amp;amp;q=90" /&gt; Menko Hilirisasi dan Transisi Energi Bahlil Lahadalia menargetkan peningkatan PNBP mineral dan batu bara.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/14/cabai-rawit-1789368088062_169.jpeg?w=360&amp;amp;q=90" /&gt; Harga komoditas cabai masih mahal di tingkat konsumen. Bahkan harga cabai rawit merah menembus angka Rp 100.000 per kilogram (kg).</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8721264/bantu-suahasil-tambal-subsidi-bbm-bahlil-target-pnbp-minerba-tembus-rp-165-t</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8723492/petani-ungkap-biang-kerok-harga-cabai-masih-mahal</t>
         </is>
       </c>
     </row>
@@ -1911,22 +1911,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Indonesia Peringkat 14 Adopsi Kripto Global, Akun Tembus 22,93 Juta</t>
+          <t>Jurus Bank Digital dan Pindar Geber Penyaluran Kredit</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Fri, 23 Oct 2026 18:41:09 +0700</t>
+          <t>Sun, 25 Oct 2026 18:52:38 +0700</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/23/distrik-keuangan-jakarta-1792755401554.jpeg?w=360&amp;amp;q=90" /&gt; Indonesia menduduki peringkat ke-14 dalam adopsi kripto global. Meskipun turun, jumlah pengguna terus meningkat.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2022/12/24/ilustrasi-bank-digital_169.jpeg?w=360&amp;amp;q=90" /&gt; Krom Bank dan Easycash berkolaborasi untuk memperluas akses pembiayaan digital. Kemitraan ini mendukung pertumbuhan kredit yang sehat dan berkelanjutan.</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/fintech/d-8721251/indonesia-peringkat-14-adopsi-kripto-global-akun-tembus-22-93-juta</t>
+          <t>https://finance.detik.com/moneter/d-8723691/jurus-bank-digital-dan-pindar-geber-penyaluran-kredit</t>
         </is>
       </c>
     </row>
@@ -1938,22 +1938,22 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Terapkan Ekspor Satu Pintu Lewat DSI, Prabowo: Tindakan Survival!</t>
+          <t>Menteri Energi Singapura Jamin Pasokan Gas Aman Meski RI Pangkas Ekspor</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Fri, 23 Oct 2026 18:27:40 +0700</t>
+          <t>Sun, 25 Oct 2026 17:59:18 +0700</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/21/sidang-kabinet-paripurna-di-istana-kepresidenan-1792580318733_169.jpeg?w=360&amp;amp;q=90" /&gt; Presiden Prabowo Subianto menjelaskan kebijakan ekspor satu pintu adalah survival mode.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2018/12/02/8b875544-14e2-4c92-b965-208d6e58c75f_169.jpeg?w=360&amp;amp;q=90" /&gt; Ministry of Energy, Trade and Industry/METI memastikan pengurangan pasokan gas di Indonesia tidak mengganggu pelayanan energi nasional.</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8721226/terapkan-ekspor-satu-pintu-lewat-dsi-prabowo-tindakan-survival</t>
+          <t>https://finance.detik.com/energi/d-8723479/menteri-energi-singapura-jamin-pasokan-gas-aman-meski-ri-pangkas-ekspor</t>
         </is>
       </c>
     </row>
@@ -1965,22 +1965,22 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Kemen PU &amp;amp; PT PP Tangani 31 Titik Longsor di Sumut, Progres Lampaui Target</t>
+          <t>Anggota BPK Fathan Subchi Meninggal Saat Tugas di Moskow</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Fri, 23 Oct 2026 18:21:33 +0700</t>
+          <t>Sun, 25 Oct 2026 17:19:11 +0700</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/23/kemen-pu-pt-pp-tangani-31-titik-longsoran-di-sumut-progres-lampaui-target-1792754399461.jpeg?w=360&amp;amp;q=90" /&gt; PT PP (Persero) Tbk berkontribusi dalam pemulihan infrastruktur jalan pascabencana di Sumatera Utara dengan proyek se</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/25/anggota-vi-bpk-ri-fathan-subchi-dok-situs-resmi-bpk-ri-1792909744024_169.webp?w=360&amp;amp;q=90" /&gt; Kabar duka datang dari Badan Pemeriksa Keuangan (BPK). Anggota VI BPK Fathan Subchi meninggal dunia.</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/infrastruktur/d-8721221/kemen-pu-pt-pp-tangani-31-titik-longsor-di-sumut-progres-lampaui-target</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8723509/anggota-bpk-fathan-subchi-meninggal-saat-tugas-di-moskow</t>
         </is>
       </c>
     </row>
@@ -1992,22 +1992,22 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Prabowo Minta KEK Bisa Sumbang Ekonomi RI hingga 1%</t>
+          <t>Program Magang Nasional Lanjut Tahun Depan, Kuota 150 Ribu Orang</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Fri, 23 Oct 2026 17:51:49 +0700</t>
+          <t>Sun, 25 Oct 2026 17:00:21 +0700</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/23/wakil-ketua-2-tim-pelaksana-dewan-kek-budi-santoso-1792752570074_169.jpeg?w=360&amp;amp;q=90" /&gt; Presiden Prabowo Subianto meminta agar Kawasan Ekonomi Khusus (KEK) dapat berkontribusi pada pertumbuhan ekonomi hingga 1% tahun depan.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/22/kemenko-perekonomian-1792659032881_169.jpeg?w=360&amp;amp;q=90" /&gt; Pemerintah mulai menyiapkan sederet program stimulus ekonomi untuk diterapkan mulai tahun depan, Program Magang Nasional menjadi salah satunya.</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8721158/prabowo-minta-kek-bisa-sumbang-ekonomi-ri-hingga-1</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8723189/program-magang-nasional-lanjut-tahun-depan-kuota-150-ribu-orang</t>
         </is>
       </c>
     </row>
@@ -2019,22 +2019,22 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Bayar Premi Asuransi Mulai Rp 1.000/Hari, Ini Proteksi yang Didapat</t>
+          <t>Dari Batik hingga Kerajinan Kulit, UMKM Lokal Ini Tembus Pasar Global</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Fri, 23 Oct 2026 17:35:24 +0700</t>
+          <t>Sun, 25 Oct 2026 16:56:57 +0700</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2022/02/04/ilustrasi-asuransi_169.jpeg?w=360&amp;amp;q=90" /&gt; PT Asuransi BRI Life meluncurkan produk asuransi Corporate Eazy (COZY) yang fleksibel, menawarkan manfaat dasar dan tambahan sesuai kebutuhan perusahaan.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/25/umkm-1792924003903_169.jpeg?w=360&amp;amp;q=90" /&gt; Mereka melibatkan masyarakat dalam produksi dan pengembangan usaha.</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/moneter/d-8721176/bayar-premi-asuransi-mulai-rp-1-000-hari-ini-proteksi-yang-didapat</t>
+          <t>https://finance.detik.com/solusiukm/d-8723517/dari-batik-hingga-kerajinan-kulit-umkm-lokal-ini-tembus-pasar-global</t>
         </is>
       </c>
     </row>
@@ -2046,22 +2046,22 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>TNI-Polri Siap Kawal Investasi di Jateng</t>
+          <t>Bantu Petani di Lampung, Mentan Siapkan Benih hingga Alat Pertanian</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Fri, 23 Oct 2026 17:27:27 +0700</t>
+          <t>Sun, 25 Oct 2026 16:11:44 +0700</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/23/forum-investasi-jawa-tengah-1792743658262_169.png?w=360&amp;amp;q=90" /&gt; TNI-Polri ikut mengawal realisasi investasi di Jawa Tengah, begini upayanya.</t>
+          <t xml:space="preserve">&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/25/bantu-petani-di-lampung-mentan-siapkan-benih-hingga-alat-pertanian-1792919455925_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Pertanian Andi Amran Sulaiman menanggapi keluhan petani Lampung dengan dukungan benih dan alat pertanian, serta </t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8721112/tni-polri-siap-kawal-investasi-di-jateng</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8723415/bantu-petani-di-lampung-mentan-siapkan-benih-hingga-alat-pertanian</t>
         </is>
       </c>
     </row>
@@ -2073,22 +2073,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Eksplorasi Privilege Kesehatan MCU-Genomics dari BRI Private &amp;amp; Prioritas</t>
+          <t>Harga Cabai Rawit Masih Mahal, Tembus Rp 102 Ribu/Kg!</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Fri, 23 Oct 2026 17:25:08 +0700</t>
+          <t>Sun, 25 Oct 2026 15:56:26 +0700</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/23/prodia-1792751083734_169.jpeg?w=360&amp;amp;q=90" /&gt; BRI dan Prodia hadirkan layanan kesehatan eksklusif untuk nasabah Private dan Prioritas, termasuk pemeriksaan rutin, MCU, dan genomik dengan berbagai manfaat.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/21/harga-cabai-rawit-merah-tembus-rp70-ribu-per-kg-di-tangerang-1789977514373_169.jpeg?w=360&amp;amp;q=90" /&gt; Komoditas cabai masih dijual dengan harga tinggi, bahkan ada yang menyentuh Rp 100.000 per kilogram (kg).</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/moneter/d-8721108/eksplorasi-privilege-kesehatan-mcu-genomics-dari-bri-private-prioritas</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8723279/harga-cabai-rawit-masih-mahal-tembus-rp-102-ribu-kg</t>
         </is>
       </c>
     </row>
@@ -2100,22 +2100,22 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Gubernur Jateng Mau Jemput Investasi Vietnam</t>
+          <t>Ribuan Penggemar Padati Indonesia Game Expo 2026</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Fri, 23 Oct 2026 17:01:55 +0700</t>
+          <t>Sun, 25 Oct 2026 15:00:16 +0700</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/23/gubernur-jateng-irjen-purn-ahmad-luthfi-1792743908471_169.png?w=360&amp;amp;q=90" /&gt; Gubernur Jateng Ahmad Luthfi bersiap untuk menjemput investasi ke Vietnam.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/24/surga-pencinta-gim-dan-budaya-pop-di-indonesia-game-expo-2026-1792836890279.jpeg?w=360&amp;amp;q=90" /&gt; Indonesia Game Expo (IGE) 2026 di ICE BSD, Tangerang, menghadirkan lebih dari 200 booth gim, kartu koleksi, action figure, hingga</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8721034/gubernur-jateng-mau-jemput-investasi-vietnam</t>
+          <t>https://finance.detik.com/foto-bisnis/d-8722309/ribuan-penggemar-padati-indonesia-game-expo-2026</t>
         </is>
       </c>
     </row>
@@ -2127,22 +2127,22 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Prabowo Respons Antrean Panjang BBM di Bali, Kasih Titah Khusus ke Bahlil Cs</t>
+          <t>Rak Besi Banting Harga di Transmart Full Day Sale</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Fri, 23 Oct 2026 16:42:52 +0700</t>
+          <t>Sun, 25 Oct 2026 15:00:00 +0700</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/21/presiden-prabowo-subianto-1792590961586_169.jpeg?w=360&amp;amp;q=90" /&gt; Presiden Prabowo Subianto memberikan titah khusus soal penanganan krisis BBM di Bali.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/25/transmart-full-day-sale-1792899602865_169.png?w=360&amp;amp;q=90" /&gt; Pesta diskon Transmart Full Day Sale kembali digelar seharian penuh.</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8721000/prabowo-respons-antrean-panjang-bbm-di-bali-kasih-titah-khusus-ke-bahlil-cs</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8722992/rak-besi-banting-harga-di-transmart-full-day-sale</t>
         </is>
       </c>
     </row>
@@ -2154,22 +2154,22 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Rute Transjakarta Dialihkan Selama Jakarta Running Festival, Ini Daftarnya</t>
+          <t>KPK Usul Harta Pejabat Tak Dilaporkan di LHKPN Bisa Dirampas Negara</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Fri, 23 Oct 2026 20:12:23 +0700</t>
+          <t>Mon, 26 Oct 2026 00:46:08 +0700</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Penyesuaian ini dilakukan agar mobilitas peserta festival dan pelanggan tetap berjalan lancar.</t>
+          <t>Selain itu, KPK mengusulkan negara dapat merampas harta penyelenggara negara apabila kekayaan yang dimiliki ternyata melebihi jumlah di LHKPN</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8320106/rute-transjakarta-dialihkan-selama-jakarta-running-festival-ini-daftarnya</t>
+          <t>https://www.liputan6.com/news/read/8321071/kpk-usul-harta-pejabat-tak-dilaporkan-di-lhkpn-bisa-dirampas-negara</t>
         </is>
       </c>
     </row>
@@ -2181,22 +2181,22 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Kronologi Terbongkarnya Pabrik Sabu Blue Ice di Pidie Aceh</t>
+          <t>Gubernur URI Menghadap Prabowo di Hambalang, Ini yang Dilaporkan</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Fri, 23 Oct 2026 19:57:43 +0700</t>
+          <t>Sun, 25 Oct 2026 21:18:52 +0700</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Polri mengamankan barang bukti sabu kualias premiun alias Blue Ice seberat 1,2 ton.</t>
+          <t>Pertemuan tersebut juga membahas perkembangan pembangunan gedung URI.</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8320099/kronologi-terbongkarnya-pabrik-sabu-blue-ice-di-pidie-aceh</t>
+          <t>https://www.liputan6.com/news/read/8321012/gubernur-uri-menghadap-prabowo-di-hambalang-ini-yang-dilaporkan</t>
         </is>
       </c>
     </row>
@@ -2208,22 +2208,22 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Pramono Berharap Warga Dukung JRF 2026 Akhir Pekan Ini</t>
+          <t>Megawati: Anak Muda Harus Berani Lawan Ketidakadilan dan Bela Rakyat</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Fri, 23 Oct 2026 19:46:00 +0700</t>
+          <t>Sun, 25 Oct 2026 21:09:28 +0700</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Pramono Anung pastikan Pemprov DKI sediakan fasilitas transportasi gratis dan pengaturan lalu lintas.</t>
+          <t>Menurut Megawati, generasi muda tidak cukup hanya memiliki kecerdasan dan keterampilan.</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8320094/pramono-berharap-warga-dukung-jrf-2026-akhir-pekan-ini</t>
+          <t>https://www.liputan6.com/news/read/8321007/megawati-anak-muda-harus-berani-lawan-ketidakadilan-dan-bela-rakyat</t>
         </is>
       </c>
     </row>
@@ -2235,22 +2235,22 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Penampakan 4 Mobil Sitaan KPK di Kasus Korupsi Dana Bencana BNPB</t>
+          <t>Napak Tilas Sumpah Pemuda, 500 Anak Muda Susuri Jejak Sejarah Jakarta</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Fri, 23 Oct 2026 19:25:20 +0700</t>
+          <t>Sun, 25 Oct 2026 20:12:32 +0700</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Dengan penyitaan terbaru ini, total empat mobil telah diamankan penyidik KPK.</t>
+          <t>Sebanyak 500 pelajar dan pemuda menyusuri sejumlah lokasi bersejarah di Jakarta untuk mengenang semangat persatuan dalam Sumpah Pemuda 1928.</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8320080/penampakan-4-mobil-sitaan-kpk-di-kasus-korupsi-dana-bencana-bnpb</t>
+          <t>https://www.liputan6.com/news/read/8320963/napak-tilas-sumpah-pemuda-500-anak-muda-susuri-jejak-sejarah-jakarta</t>
         </is>
       </c>
     </row>
@@ -2262,22 +2262,22 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Dilaporkan Tokoh Adat Papua, Sutradara Film Pesta Babi Dipanggil Polisi</t>
+          <t>Pramono Klaim Modifikasi Cuaca Bantu Sukseskan Jakarta Running Festival</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Fri, 23 Oct 2026 19:21:28 +0700</t>
+          <t>Sun, 25 Oct 2026 19:04:02 +0700</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Pemeriksaan dijadwalkan pada Selasa, 27 Oktober 2026.</t>
+          <t>Pramono Anung menyebutmodifikasi cuaca  selama dua hari penyelenggaraan Jakarta Running Festival membantu menurunkan polusi udara dan mengantisipasi hujan di sejumlah wilayah.</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8320074/dilaporkan-tokoh-adat-papua-sutradara-film-pesta-babi-dipanggil-polisi</t>
+          <t>https://www.liputan6.com/news/read/8320953/pramono-klaim-modifikasi-cuaca-bantu-sukseskan-jakarta-running-festival</t>
         </is>
       </c>
     </row>
@@ -2289,22 +2289,22 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>NasDem Soroti Kesehatan Mental Ibu, 57 Persen Alami Baby Blues</t>
+          <t>Hasto Cerita Kebijakan Megawati Cegah Hutan Bekas Karhutla Jadi Kebun Sawit</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Fri, 23 Oct 2026 18:36:29 +0700</t>
+          <t>Sun, 25 Oct 2026 18:01:03 +0700</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Kesehatan mental ibu di antaranya berlanjut dari baby blues menjadi depresi pascamelahirkan.</t>
+          <t>Menurut Hasto, sanksi tegas diperlukan, terutama jika lahan yang dibakar kemudian dialihfungsikan menjadi kebun sawit.</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8320046/nasdem-soroti-kesehatan-mental-ibu-57-persen-alami-baby-blues</t>
+          <t>https://www.liputan6.com/news/read/8320941/hasto-cerita-kebijakan-megawati-cegah-hutan-bekas-karhutla-jadi-kebun-sawit</t>
         </is>
       </c>
     </row>
@@ -2316,22 +2316,22 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Prabowo Beberkan Penindakan Pelanggaran MBG, Ini Hasillnya</t>
+          <t>Muntaber Massal di Tangsel, Warga Tuntut Kompensasi Rp 539 Juta</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Fri, 23 Oct 2026 18:20:16 +0700</t>
+          <t>Sun, 25 Oct 2026 17:38:23 +0700</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Prabowo menyampaikan hal tersebut dalam Sidang Kabinet Paripurna di Kompleks Istana Kepresidenan.</t>
+          <t>Warga memberikan tenggat waktu hingga Selasa (27/10/2026) agar perusahaan memberikan kejelasan mengenai tuntutan ganti rugi.</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8320025/prabowo-beberkan-penindakan-pelanggaran-mbg-ini-hasillnya</t>
+          <t>https://www.liputan6.com/news/read/8320929/muntaber-massal-di-tangsel-warga-tuntut-kompensasi-rp-539-juta</t>
         </is>
       </c>
     </row>
@@ -2343,22 +2343,22 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Korban Pembacokan di Jaktim Ternyata Eks Anggota Kopassus</t>
+          <t>Indonesia Siapkan Forum Konservasi Terumbu Karang di AS</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Fri, 23 Oct 2026 17:52:34 +0700</t>
+          <t>Sun, 25 Oct 2026 17:33:52 +0700</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Korban bernama Muhammad Fahrul (48).</t>
+          <t>Indonesia menyiapkan forum internasional di Washington pada 2027 untuk memperluas dukungan pembiayaan dan kerja sama konservasi terumbu karang.</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8320002/korban-pembacokan-di-jaktim-ternyata-eks-anggota-kopassus</t>
+          <t>https://www.liputan6.com/news/read/8320927/indonesia-siapkan-forum-konservasi-terumbu-karang-di-as</t>
         </is>
       </c>
     </row>
@@ -2370,22 +2370,22 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Kronologi Penyelundupan 1,16 Ton Ketamin di Perairan Belawan</t>
+          <t>Anggota VI BPK Fathan Subchi Meninggal Dunia</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Fri, 23 Oct 2026 18:42:18 +0700</t>
+          <t>Sun, 25 Oct 2026 17:15:27 +0700</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Kapal terdeteksi melakukan pergerakan tidak biasa di Selat Malaka dan Laut Andaman.</t>
+          <t>Anggota VI BPK Fathan Subchi meninggal dunia pada usia 56 tahun saat menjalankan tugas pemeriksaan di Moskow, Rusia, Minggu (25/10/2026).</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8319985/kronologi-penyelundupan-116-ton-ketamin-di-perairan-belawan</t>
+          <t>https://www.liputan6.com/news/read/8320918/anggota-vi-bpk-fathan-subchi-meninggal-dunia</t>
         </is>
       </c>
     </row>
@@ -2397,22 +2397,22 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Kasus Judi Online Boxkia, Terungkap Omzet Rp 2 Miliar Per Bulan</t>
+          <t>SBY Kenang Pengabdian Widodo AS saat Indonesia Hadapi Krisis 1998</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Fri, 23 Oct 2026 17:17:39 +0700</t>
+          <t>Sun, 25 Oct 2026 17:12:01 +0700</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Bareskrim Polri mengungkap praktik perjudian online melalui situs Boxkia.</t>
+          <t>SBY mengenang mantan Panglima TNI Widodo AS sebagai prajurit dan negarawan yang berkomitmen menjaga konstitusi serta keutuhan bangsa.</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8319974/kasus-judi-online-boxkia-terungkap-omzet-rp-2-miliar-per-bulan</t>
+          <t>https://www.liputan6.com/news/read/8320914/sby-kenang-pengabdian-widodo-as-saat-indonesia-hadapi-krisis-1998</t>
         </is>
       </c>
     </row>
@@ -2424,22 +2424,22 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Kapolri Beberkan Data Perorangan dan Korporasi Terseret Kebakaran Hutan</t>
+          <t>Penataan Stasiun Karet dan Sudirman Baru Rampung Akhir 2026</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Fri, 23 Oct 2026 17:15:00 +0700</t>
+          <t>Sun, 25 Oct 2026 16:27:53 +0700</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Total 35.390 hektare lahan terbakar, dengan penegakan hukum terus berjalan.</t>
+          <t>KAI menargetkan penataan kawasan Stasiun Karet dan Sudirman Baru rampung 31 Desember 2026, dengan fasilitas baru untuk memudahkan mobilitas penumpang.</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8319968/kapolri-beberkan-data-perorangan-dan-korporasi-terseret-kebakaran-hutan</t>
+          <t>https://www.liputan6.com/news/read/8320894/penataan-stasiun-karet-dan-sudirman-baru-rampung-akhir-2026</t>
         </is>
       </c>
     </row>
@@ -2451,22 +2451,22 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Infografis: 10 Negara dengan Pertumbuhan Orang Kaya Tertinggi</t>
+          <t>Seruni dan Dekranas Dukung Pelestarian Tenun Gringsing</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Fri, 23 Oct 2026 17:02:12 +0700</t>
+          <t>Sun, 25 Oct 2026 15:57:26 +0700</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Indonesia, Arab Saudi, dan Vietnam masuk dalam daftar negara dengan proyeksi pertumbuhan orang super kaya yang pesat.</t>
+          <t>Penyerahan bantuan ini disertai pemeriksaan mata untuk mengetahui tingkat minus setiap penerima.</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8319962/infografis-10-negara-dengan-pertumbuhan-orang-kaya-tertinggi</t>
+          <t>https://www.liputan6.com/news/read/8320888/seruni-dan-dekranas-dukung-pelestarian-tenun-gringsing</t>
         </is>
       </c>
     </row>
@@ -2478,22 +2478,22 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Limbah Dibidik Jadi Sumber Energi Rendah Karbon</t>
+          <t>Demi Efisiensi, Tri Tito Karnavian Gabungkan Rapat Tiga Lembaga</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Fri, 23 Oct 2026 16:50:50 +0700</t>
+          <t>Sun, 25 Oct 2026 15:54:35 +0700</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Limbah tak hanya menjadi residu tetapi bisa menjadi energi yang berpotensi memberikan nilai tambah.</t>
+          <t>Tri Tito Karnavian menggabungkan rapat kerja Dekranas, TP PKK, dan TP Posyandu dalam satu forum untuk meningkatkan efisiensi anggaran dan koordinasi program.</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8319948/limbah-dibidik-jadi-sumber-energi-rendah-karbon</t>
+          <t>https://www.liputan6.com/news/read/8320886/demi-efisiensi-tri-tito-karnavian-gabungkan-rapat-tiga-lembaga</t>
         </is>
       </c>
     </row>
@@ -2505,22 +2505,22 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Ketika Kreativitas dan Olahraga Menggerakkan Roda Ekonomi Jakarta</t>
+          <t>Pramono: Izin Rumah Ibadah Harus Selesai dalam Dua Pekan</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Fri, 23 Oct 2026 17:54:23 +0700</t>
+          <t>Sun, 25 Oct 2026 15:41:01 +0700</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Perputaran ekonomi Jakarta meningkat pesat berkat event kreatif dan olahraga.</t>
+          <t>Pramono Anung meminta izin pembangunan rumah ibadah di Jakarta diselesaikan dalam satu hingga dua pekan setelah seluruh persyaratan administrasi terpenuhi.</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8319937/ketika-kreativitas-dan-olahraga-menggerakkan-roda-ekonomi-jakarta</t>
+          <t>https://www.liputan6.com/news/read/8320868/pramono-izin-rumah-ibadah-harus-selesai-dalam-dua-pekan</t>
         </is>
       </c>
     </row>
@@ -2532,22 +2532,22 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Dua Tahun Prabowo-Gibran, Revitalisasi Sekolah Diperluas</t>
+          <t>Kondisi Terkini Driver Ojol Dilindas BYD di Blok M</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Fri, 23 Oct 2026 15:43:51 +0700</t>
+          <t>Sun, 25 Oct 2026 15:27:27 +0700</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Revitalisasi ditujukan untuk memperbaiki fasilitas sekolah.</t>
+          <t>Korban berinisial HS (56) saat ini masih menjalani observasi di Rumah Sakit Fatmawati.</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8319883/dua-tahun-prabowo-gibran-revitalisasi-sekolah-diperluas</t>
+          <t>https://www.liputan6.com/news/read/8320875/kondisi-terkini-driver-ojol-dilindas-byd-di-blok-m</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data pasar & berita - 2026-10-26 15:02 UTC
</commit_message>
<xml_diff>
--- a/data/market_news_latest.xlsx
+++ b/data/market_news_latest.xlsx
@@ -487,20 +487,20 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>5439.2578</v>
+        <v>5373.0942</v>
       </c>
       <c r="F2" t="n">
-        <v>51.353</v>
+        <v>-66.1636</v>
       </c>
       <c r="G2" t="n">
-        <v>0.95</v>
+        <v>-1.22</v>
       </c>
       <c r="H2" t="n">
-        <v>397036500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -521,20 +521,20 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>7623.6802</v>
+        <v>7701.54</v>
       </c>
       <c r="F3" t="n">
-        <v>-39.75</v>
+        <v>77.8599</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.52</v>
+        <v>1.02</v>
       </c>
       <c r="H3" t="n">
-        <v>5062330000</v>
+        <v>659034209</v>
       </c>
     </row>
     <row r="4">
@@ -555,20 +555,20 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>52215.1602</v>
+        <v>52491.9609</v>
       </c>
       <c r="F4" t="n">
-        <v>-652.8203</v>
+        <v>276.8008</v>
       </c>
       <c r="G4" t="n">
-        <v>-1.23</v>
+        <v>0.53</v>
       </c>
       <c r="H4" t="n">
-        <v>348500000</v>
+        <v>98731755</v>
       </c>
     </row>
     <row r="5">
@@ -589,20 +589,20 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>25955.3398</v>
+        <v>26305.5059</v>
       </c>
       <c r="F5" t="n">
-        <v>-53.5195</v>
+        <v>350.166</v>
       </c>
       <c r="G5" t="n">
-        <v>-0.21</v>
+        <v>1.35</v>
       </c>
       <c r="H5" t="n">
-        <v>6554790000</v>
+        <v>2381854000</v>
       </c>
     </row>
     <row r="6">
@@ -657,20 +657,20 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>23093.3691</v>
+        <v>23211.8105</v>
       </c>
       <c r="F7" t="n">
-        <v>158.6895</v>
+        <v>118.4414</v>
       </c>
       <c r="G7" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.51</v>
       </c>
       <c r="H7" t="n">
-        <v>3842800000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -691,20 +691,20 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>3690.4751</v>
+        <v>3697.52</v>
       </c>
       <c r="F8" t="n">
-        <v>32.4492</v>
+        <v>7.0449</v>
       </c>
       <c r="G8" t="n">
-        <v>0.89</v>
+        <v>0.19</v>
       </c>
       <c r="H8" t="n">
-        <v>552800</v>
+        <v>329758840</v>
       </c>
     </row>
     <row r="9">
@@ -725,20 +725,20 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>10690.4004</v>
+        <v>10768.2695</v>
       </c>
       <c r="F9" t="n">
-        <v>-34.5996</v>
+        <v>77.8691</v>
       </c>
       <c r="G9" t="n">
-        <v>-0.32</v>
+        <v>0.73</v>
       </c>
       <c r="H9" t="n">
-        <v>697030600</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -759,20 +759,20 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>25181.6504</v>
+        <v>25497.0703</v>
       </c>
       <c r="F10" t="n">
-        <v>-190.0996</v>
+        <v>315.4199</v>
       </c>
       <c r="G10" t="n">
-        <v>-0.75</v>
+        <v>1.25</v>
       </c>
       <c r="H10" t="n">
-        <v>58950600</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -793,20 +793,20 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>5422.1602</v>
+        <v>5415.9102</v>
       </c>
       <c r="F11" t="n">
-        <v>7.02</v>
+        <v>-6.25</v>
       </c>
       <c r="G11" t="n">
-        <v>0.13</v>
+        <v>-0.12</v>
       </c>
       <c r="H11" t="n">
-        <v>388429200</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -827,17 +827,17 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>17956</v>
+        <v>17978</v>
       </c>
       <c r="F12" t="n">
-        <v>-97</v>
+        <v>-75</v>
       </c>
       <c r="G12" t="n">
-        <v>-0.54</v>
+        <v>-0.42</v>
       </c>
       <c r="H12" t="n">
         <v>0</v>
@@ -861,17 +861,17 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>101.765</v>
+        <v>101.99</v>
       </c>
       <c r="F13" t="n">
-        <v>-0.045</v>
+        <v>0.18</v>
       </c>
       <c r="G13" t="n">
-        <v>-0.04</v>
+        <v>0.18</v>
       </c>
       <c r="H13" t="n">
         <v>0</v>
@@ -895,17 +895,17 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>156.888</v>
+        <v>157.55</v>
       </c>
       <c r="F14" t="n">
-        <v>0.394</v>
+        <v>1.056</v>
       </c>
       <c r="G14" t="n">
-        <v>0.25</v>
+        <v>0.67</v>
       </c>
       <c r="H14" t="n">
         <v>0</v>
@@ -929,17 +929,17 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>0.4988</v>
+        <v>0.497</v>
       </c>
       <c r="F15" t="n">
-        <v>0.0035</v>
+        <v>-0.0018</v>
       </c>
       <c r="G15" t="n">
-        <v>0.71</v>
+        <v>-0.36</v>
       </c>
       <c r="H15" t="n">
         <v>0</v>
@@ -963,17 +963,17 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>0.5315</v>
+        <v>0.5285</v>
       </c>
       <c r="F16" t="n">
-        <v>0.0028</v>
+        <v>-0.003</v>
       </c>
       <c r="G16" t="n">
-        <v>0.53</v>
+        <v>-0.5600000000000001</v>
       </c>
       <c r="H16" t="n">
         <v>0</v>
@@ -997,17 +997,17 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>0.4032</v>
+        <v>0.4043</v>
       </c>
       <c r="F17" t="n">
-        <v>0.001</v>
+        <v>0.0011</v>
       </c>
       <c r="G17" t="n">
-        <v>0.25</v>
+        <v>0.27</v>
       </c>
       <c r="H17" t="n">
         <v>0</v>
@@ -1031,20 +1031,20 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>81.34</v>
+        <v>81.685</v>
       </c>
       <c r="F18" t="n">
-        <v>-0.4</v>
+        <v>0.345</v>
       </c>
       <c r="G18" t="n">
-        <v>-0.49</v>
+        <v>0.42</v>
       </c>
       <c r="H18" t="n">
-        <v>35120900</v>
+        <v>8768809</v>
       </c>
     </row>
     <row r="19">
@@ -1065,20 +1065,20 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>77.05</v>
+        <v>77.315</v>
       </c>
       <c r="F19" t="n">
-        <v>-0.05</v>
+        <v>0.265</v>
       </c>
       <c r="G19" t="n">
-        <v>-0.06</v>
+        <v>0.34</v>
       </c>
       <c r="H19" t="n">
-        <v>56640900</v>
+        <v>11317534</v>
       </c>
     </row>
     <row r="20">
@@ -1099,20 +1099,20 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>4012</v>
+        <v>4032.8</v>
       </c>
       <c r="F20" t="n">
-        <v>4.1001</v>
+        <v>24.9001</v>
       </c>
       <c r="G20" t="n">
-        <v>0.1</v>
+        <v>0.62</v>
       </c>
       <c r="H20" t="n">
-        <v>3340</v>
+        <v>86338</v>
       </c>
     </row>
     <row r="21">
@@ -1133,20 +1133,20 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>102.29</v>
+        <v>101.07</v>
       </c>
       <c r="F21" t="n">
-        <v>-0.98</v>
+        <v>-2.2</v>
       </c>
       <c r="G21" t="n">
-        <v>-0.95</v>
+        <v>-2.13</v>
       </c>
       <c r="H21" t="n">
-        <v>10295</v>
+        <v>141272</v>
       </c>
     </row>
     <row r="22">
@@ -1167,20 +1167,20 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="E22" t="n">
-        <v>110.82</v>
+        <v>110.14</v>
       </c>
       <c r="F22" t="n">
-        <v>-5.9</v>
+        <v>-6.58</v>
       </c>
       <c r="G22" t="n">
-        <v>-5.05</v>
+        <v>-5.64</v>
       </c>
       <c r="H22" t="n">
-        <v>741</v>
+        <v>20633</v>
       </c>
     </row>
     <row r="23">
@@ -1201,20 +1201,20 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="E23" t="n">
-        <v>6.4925</v>
+        <v>6.521</v>
       </c>
       <c r="F23" t="n">
-        <v>0.0165</v>
+        <v>0.045</v>
       </c>
       <c r="G23" t="n">
-        <v>0.25</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="H23" t="n">
-        <v>782</v>
+        <v>22262</v>
       </c>
     </row>
     <row r="24">
@@ -1235,20 +1235,20 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="E24" t="n">
-        <v>62.01</v>
+        <v>61.945</v>
       </c>
       <c r="F24" t="n">
-        <v>0.29</v>
+        <v>-0.065</v>
       </c>
       <c r="G24" t="n">
-        <v>0.47</v>
+        <v>-0.1</v>
       </c>
       <c r="H24" t="n">
-        <v>22024100</v>
+        <v>6265588</v>
       </c>
     </row>
     <row r="25">
@@ -1269,17 +1269,17 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="E25" t="n">
-        <v>19.45</v>
+        <v>17.99</v>
       </c>
       <c r="F25" t="n">
-        <v>0.42</v>
+        <v>-1.46</v>
       </c>
       <c r="G25" t="n">
-        <v>2.21</v>
+        <v>-7.51</v>
       </c>
       <c r="H25" t="n">
         <v>0</v>
@@ -1303,20 +1303,20 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="E26" t="n">
-        <v>80154.7031</v>
+        <v>80311.7188</v>
       </c>
       <c r="F26" t="n">
-        <v>-636.1328</v>
+        <v>287.7109</v>
       </c>
       <c r="G26" t="n">
-        <v>-0.79</v>
+        <v>0.36</v>
       </c>
       <c r="H26" t="n">
-        <v>11814104064</v>
+        <v>24188891136</v>
       </c>
     </row>
     <row r="27">
@@ -1337,20 +1337,20 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="E27" t="n">
-        <v>1440</v>
+        <v>1420</v>
       </c>
       <c r="F27" t="n">
-        <v>0</v>
+        <v>-20</v>
       </c>
       <c r="G27" t="n">
-        <v>0</v>
+        <v>-1.39</v>
       </c>
       <c r="H27" t="n">
-        <v>68976800</v>
+        <v>89907100</v>
       </c>
     </row>
     <row r="28">
@@ -1371,20 +1371,20 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="E28" t="n">
-        <v>1330</v>
+        <v>1445</v>
       </c>
       <c r="F28" t="n">
-        <v>-10</v>
+        <v>115</v>
       </c>
       <c r="G28" t="n">
-        <v>-0.75</v>
+        <v>8.65</v>
       </c>
       <c r="H28" t="n">
-        <v>136283100</v>
+        <v>448969700</v>
       </c>
     </row>
     <row r="29">
@@ -1405,20 +1405,20 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="E29" t="n">
-        <v>510</v>
+        <v>482</v>
       </c>
       <c r="F29" t="n">
-        <v>14</v>
+        <v>-28</v>
       </c>
       <c r="G29" t="n">
-        <v>2.82</v>
+        <v>-5.49</v>
       </c>
       <c r="H29" t="n">
-        <v>353645100</v>
+        <v>669467800</v>
       </c>
     </row>
     <row r="30">
@@ -1439,20 +1439,20 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="E30" t="n">
-        <v>2380</v>
+        <v>2320</v>
       </c>
       <c r="F30" t="n">
-        <v>60</v>
+        <v>-60</v>
       </c>
       <c r="G30" t="n">
-        <v>2.59</v>
+        <v>-2.52</v>
       </c>
       <c r="H30" t="n">
-        <v>20443500</v>
+        <v>14666400</v>
       </c>
     </row>
     <row r="31">
@@ -1473,20 +1473,20 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="E31" t="n">
-        <v>3090</v>
+        <v>3050</v>
       </c>
       <c r="F31" t="n">
-        <v>20</v>
+        <v>-40</v>
       </c>
       <c r="G31" t="n">
-        <v>0.65</v>
+        <v>-1.29</v>
       </c>
       <c r="H31" t="n">
-        <v>27460600</v>
+        <v>59198800</v>
       </c>
     </row>
     <row r="32">
@@ -1507,20 +1507,20 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="E32" t="n">
         <v>426</v>
       </c>
       <c r="F32" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G32" t="n">
-        <v>0.47</v>
+        <v>0</v>
       </c>
       <c r="H32" t="n">
-        <v>24749800</v>
+        <v>72384700</v>
       </c>
     </row>
     <row r="33">
@@ -1541,20 +1541,20 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="E33" t="n">
-        <v>500</v>
+        <v>472</v>
       </c>
       <c r="F33" t="n">
-        <v>22</v>
+        <v>-28</v>
       </c>
       <c r="G33" t="n">
-        <v>4.6</v>
+        <v>-5.6</v>
       </c>
       <c r="H33" t="n">
-        <v>154580300</v>
+        <v>95356100</v>
       </c>
     </row>
     <row r="34">
@@ -1575,20 +1575,20 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="E34" t="n">
-        <v>2660</v>
+        <v>2490</v>
       </c>
       <c r="F34" t="n">
-        <v>140</v>
+        <v>-170</v>
       </c>
       <c r="G34" t="n">
-        <v>5.56</v>
+        <v>-6.39</v>
       </c>
       <c r="H34" t="n">
-        <v>13319700</v>
+        <v>9056700</v>
       </c>
     </row>
     <row r="35">
@@ -1609,20 +1609,20 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="E35" t="n">
-        <v>378</v>
+        <v>376</v>
       </c>
       <c r="F35" t="n">
-        <v>64</v>
+        <v>-2</v>
       </c>
       <c r="G35" t="n">
-        <v>20.38</v>
+        <v>-0.53</v>
       </c>
       <c r="H35" t="n">
-        <v>791388800</v>
+        <v>715424300</v>
       </c>
     </row>
     <row r="36">
@@ -1643,20 +1643,20 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="E36" t="n">
-        <v>174</v>
+        <v>167</v>
       </c>
       <c r="F36" t="n">
-        <v>26</v>
+        <v>-7</v>
       </c>
       <c r="G36" t="n">
-        <v>17.57</v>
+        <v>-4.02</v>
       </c>
       <c r="H36" t="n">
-        <v>290939000</v>
+        <v>184085900</v>
       </c>
     </row>
     <row r="37">
@@ -1677,20 +1677,20 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="E37" t="n">
-        <v>10300</v>
+        <v>10200</v>
       </c>
       <c r="F37" t="n">
-        <v>300</v>
+        <v>-100</v>
       </c>
       <c r="G37" t="n">
-        <v>3</v>
+        <v>-0.97</v>
       </c>
       <c r="H37" t="n">
-        <v>13505800</v>
+        <v>13991200</v>
       </c>
     </row>
   </sheetData>
@@ -1749,22 +1749,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Serangan Rudal Rusia Hantam Kharkiv, Pusat Perbelanjaan Terbakar</t>
+          <t>Jurus Pemerintah Jaga Pasokan dan Harga Pangan Jelang Nataru</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Mon, 26 Oct 2026 06:00:16 +0700</t>
+          <t>Mon, 26 Oct 2026 21:36:17 +0700</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/25/serangan-rudal-rusia-hantam-kharkiv-pusat-perbelanjaan-terbakar-1792913695273_169.jpeg?w=360&amp;amp;q=90" /&gt; Serangan rudal Rusia menghantam pusat perbelanjaan di Kharkiv, Ukraina, memicu kebakaran dan merusak bangunan sipil.</t>
+          <t xml:space="preserve">&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/26/rapat-koordinasi-terbatas-rakortas-bidang-pangan-yang-dipimpin-menteri-koordinator-bidang-pangan-ri-menko-pangan-zulkifli-hasa-1793025343365.jpeg?w=360&amp;amp;q=90" /&gt; Pemerintah antisipasi stabilitas pangan menjelang Nataru dengan </t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/foto-bisnis/d-8723283/serangan-rudal-rusia-hantam-kharkiv-pusat-perbelanjaan-terbakar</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8725387/jurus-pemerintah-jaga-pasokan-dan-harga-pangan-jelang-nataru</t>
         </is>
       </c>
     </row>
@@ -1776,22 +1776,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Singapura Singgung soal Kontrak Usai RI Pangkas Ekspor Gas</t>
+          <t>3.030 Penerbangan Terdampak Karhutla Sejak Agustus, 1.700 Rute Dibatalkan</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Mon, 26 Oct 2026 05:55:43 +0700</t>
+          <t>Mon, 26 Oct 2026 21:30:00 +0700</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2024/05/16/sosok-lawrence-wong-perdana-menteri-baru-singapura-1_169.jpeg?w=360&amp;amp;q=90" /&gt; Perdana Menteri (PM) Singapura Lawrence Wong akhirnya angkat bicara merespons kebijakan Indonesia mengurangi ekspor gas.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2023/10/05/ngeri-kabut-asap-bikin-jarak-pandang-di-bandara-palangka-raya-terbatas-1_169.jpeg?w=360&amp;amp;q=90" /&gt; Kemenhub mencatat sebanyak 3.030 penerbangan terdampak oleh kabut asap akibat kebakaran hutan dan lahan (karhutla) sejak 14 Agus</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8723774/singapura-singgung-soal-kontrak-usai-ri-pangkas-ekspor-gas</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8725381/3-030-penerbangan-terdampak-karhutla-sejak-agustus-1-700-rute-dibatalkan</t>
         </is>
       </c>
     </row>
@@ -1803,22 +1803,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Mentan Ungkap Anomali Harga Telur: Stok Melimpah, tapi Harga Naik</t>
+          <t>Pertamina Dukung Perpres 107 Perkuat Ketahanan Energi Nasional</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Sun, 25 Oct 2026 22:00:44 +0700</t>
+          <t>Mon, 26 Oct 2026 21:27:35 +0700</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/07/28/pemerintah-pastikan-beras-hingga-daging-ayam-dalam-kondisi-surplus-1785222178359_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Pertanian Amran Sulaiman mengungkapkan harga telur saat ini mengalami anomali.</t>
+          <t xml:space="preserve">&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/26/pertamina-siap-jalankan-perpres-107-untuk-perkuat-ketahanan-energi-nasional-1793024805115.jpeg?w=360&amp;amp;q=90" /&gt; Pertamina mendukung Perpres 107/2026 untuk memperkuat pengadaan energi nasional. Komitmen menjaga ketersediaan BBM </t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8723273/mentan-ungkap-anomali-harga-telur-stok-melimpah-tapi-harga-naik</t>
+          <t>https://finance.detik.com/energi/d-8725384/pertamina-dukung-perpres-107-perkuat-ketahanan-energi-nasional</t>
         </is>
       </c>
     </row>
@@ -1830,22 +1830,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>ESDM Buka Lowongan 108 Pengawal Energi, Gaji hingga Rp 6,5 Juta/Bulan</t>
+          <t>Harga Tiket Pesawat Bakal Turun 11-13% Saat Libur Natal &amp;amp; Tahun Baru</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Sun, 25 Oct 2026 21:00:16 +0700</t>
+          <t>Mon, 26 Oct 2026 21:16:28 +0700</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/05/11/ilustrasi-job-fair-atau-lowongan-kerja-1746929349100_169.jpeg?w=360&amp;amp;q=90" /&gt; Kementerian Energi dan Sumber Daya Mineral (ESDM) membuka kesempatan kerja untuk posisi verifikator lapangan dan analis dalam Program Pengawal Energ</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2023/11/11/ilustrasi-harga-tiket-pesawat_169.png?w=360&amp;amp;q=90" /&gt; Kementerian Perhubungan (Kemenhub) menargetkan harga tiket pesawat dapat turun 11-13% selama periode Natal dan Tahun Baru (Nataru) 2026/2027.</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8723623/esdm-buka-lowongan-108-pengawal-energi-gaji-hingga-rp-6-5-juta-bulan</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8725373/harga-tiket-pesawat-bakal-turun-11-13-saat-libur-natal-tahun-baru</t>
         </is>
       </c>
     </row>
@@ -1857,22 +1857,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Mentan Lapor Prabowo 500 Ribu Ha Rawa Disulap Jadi Sawah</t>
+          <t>Impor KRL Bekas Jepang Tunggu Restu Kemenhub</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Sun, 25 Oct 2026 20:00:40 +0700</t>
+          <t>Mon, 26 Oct 2026 21:08:16 +0700</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/10/10/mentan-amran-sulaiman-1760077106363_169.jpeg?w=360&amp;amp;q=90" /&gt; Pemerintah terus menambah area tanam pangan untuk memenuhi kebutuhan pangan dalam negeri.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2014/06/27/7792aea3-ac73-4740-974a-e71dca1fea91_169.jpg?w=360&amp;amp;q=90" /&gt; Kementerian Perhubungan (Kemenhub) mempelajari proposal pengadaan Kereta Rel Listrik (KRL) bekas dari Jepang.</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8723304/mentan-lapor-prabowo-500-ribu-ha-rawa-disulap-jadi-sawah</t>
+          <t>https://finance.detik.com/infrastruktur/d-8725367/impor-krl-bekas-jepang-tunggu-restu-kemenhub</t>
         </is>
       </c>
     </row>
@@ -1884,22 +1884,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Petani Ungkap Biang Kerok Harga Cabai Masih Mahal</t>
+          <t>Karya Siswa Disabilitas di Bali Tembus Toko Oleh-Oleh, Harga Mulai Rp 10 Ribu</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Sun, 25 Oct 2026 19:00:31 +0700</t>
+          <t>Mon, 26 Oct 2026 21:00:41 +0700</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/14/cabai-rawit-1789368088062_169.jpeg?w=360&amp;amp;q=90" /&gt; Harga komoditas cabai masih mahal di tingkat konsumen. Bahkan harga cabai rawit merah menembus angka Rp 100.000 per kilogram (kg).</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/26/karya-siswa-disabilitas-di-bali-tembus-toko-oleh-oleh-harga-mulai-rp-10-ribu-1792999583884_169.jpeg?w=360&amp;amp;q=90" /&gt; Siswa tunarungu di SLB Negeri 1 Tabanan, Bali, membuat kerajinan tangan. Produk mereka dijual di toko oleh-ole</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8723492/petani-ungkap-biang-kerok-harga-cabai-masih-mahal</t>
+          <t>https://finance.detik.com/foto-bisnis/d-8724549/karya-siswa-disabilitas-di-bali-tembus-toko-oleh-oleh-harga-mulai-rp-10-ribu</t>
         </is>
       </c>
     </row>
@@ -1911,22 +1911,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Jurus Bank Digital dan Pindar Geber Penyaluran Kredit</t>
+          <t>Truk AMDK Diusulkan Dikecualikan dari Pembatasan Saat Nataru</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Sun, 25 Oct 2026 18:52:38 +0700</t>
+          <t>Mon, 26 Oct 2026 21:00:03 +0700</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2022/12/24/ilustrasi-bank-digital_169.jpeg?w=360&amp;amp;q=90" /&gt; Krom Bank dan Easycash berkolaborasi untuk memperluas akses pembiayaan digital. Kemitraan ini mendukung pertumbuhan kredit yang sehat dan berkelanjutan.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2023/06/23/pangsa-pasar-air-minum-kemasan-lokal-meningkat-2_169.jpeg?w=360&amp;amp;q=90" /&gt; Distribusi AMDK diminta dikecualikan dalam pembatasan truk saat libur Nataru.</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/moneter/d-8723691/jurus-bank-digital-dan-pindar-geber-penyaluran-kredit</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8725185/truk-amdk-diusulkan-dikecualikan-dari-pembatasan-saat-nataru</t>
         </is>
       </c>
     </row>
@@ -1938,22 +1938,22 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Menteri Energi Singapura Jamin Pasokan Gas Aman Meski RI Pangkas Ekspor</t>
+          <t>Tiga Penyebab Dana Operasional Dapur MBG Nggak Cair</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Sun, 25 Oct 2026 17:59:18 +0700</t>
+          <t>Mon, 26 Oct 2026 21:00:00 +0700</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2018/12/02/8b875544-14e2-4c92-b965-208d6e58c75f_169.jpeg?w=360&amp;amp;q=90" /&gt; Ministry of Energy, Trade and Industry/METI memastikan pengurangan pasokan gas di Indonesia tidak mengganggu pelayanan energi nasional.</t>
+          <t xml:space="preserve">&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/06/08/realisasi-anggaran-program-makanan-bergizi-gratis-1780905690949_169.jpeg?w=360&amp;amp;q=90" /&gt; BGN mengungkapkan penyebab dana operasional Satuan Pelayanan Pemenuhan Gizi (SPPG) atau Dapur Makan Bergizi Gratis (MBG) tidak cair pada </t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8723479/menteri-energi-singapura-jamin-pasokan-gas-aman-meski-ri-pangkas-ekspor</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8725276/tiga-penyebab-dana-operasional-dapur-mbg-nggak-cair</t>
         </is>
       </c>
     </row>
@@ -1965,22 +1965,22 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Anggota BPK Fathan Subchi Meninggal Saat Tugas di Moskow</t>
+          <t>Petinggi BUMN Dilarang Pakai Anggaran &amp;amp; Fasilitas Perusahaan buat Kegiatan Pribadi</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Sun, 25 Oct 2026 17:19:11 +0700</t>
+          <t>Mon, 26 Oct 2026 20:38:32 +0700</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/25/anggota-vi-bpk-ri-fathan-subchi-dok-situs-resmi-bpk-ri-1792909744024_169.webp?w=360&amp;amp;q=90" /&gt; Kabar duka datang dari Badan Pemeriksa Keuangan (BPK). Anggota VI BPK Fathan Subchi meninggal dunia.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2020/07/02/logo-baru-kementerian-bumn-1_169.jpeg?w=360&amp;amp;q=90" /&gt; Danantara melarang direksi dan dewan komisaris BUMN menggunakan anggaran maupun fasilitas perusahaan untuk hobi, olahraga hingga kegiatan pribadi</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8723509/anggota-bpk-fathan-subchi-meninggal-saat-tugas-di-moskow</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8725332/petinggi-bumn-dilarang-pakai-anggaran-fasilitas-perusahaan-buat-kegiatan-pribadi</t>
         </is>
       </c>
     </row>
@@ -1992,22 +1992,22 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Program Magang Nasional Lanjut Tahun Depan, Kuota 150 Ribu Orang</t>
+          <t>Bos Danantara Sebut Obligasi US$ 1,5 M Diserbu Investor Asing</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Sun, 25 Oct 2026 17:00:21 +0700</t>
+          <t>Mon, 26 Oct 2026 20:30:13 +0700</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/22/kemenko-perekonomian-1792659032881_169.jpeg?w=360&amp;amp;q=90" /&gt; Pemerintah mulai menyiapkan sederet program stimulus ekonomi untuk diterapkan mulai tahun depan, Program Magang Nasional menjadi salah satunya.</t>
+          <t xml:space="preserve">&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/22/chief-investment-officer-cio-danantara-indonesia-pandu-sjahrir-1792645980929_169.jpeg?w=360&amp;amp;q=90" /&gt; Danantara mengungkapkan penerbitan obligasi US$ 1,5 miliar atau sekitar Rp 27,15 triliun (kurs Rp 18.100) mendapat sambutan </t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8723189/program-magang-nasional-lanjut-tahun-depan-kuota-150-ribu-orang</t>
+          <t>https://finance.detik.com/bursa-dan-valas/d-8725114/bos-danantara-sebut-obligasi-us-1-5-m-diserbu-investor-asing</t>
         </is>
       </c>
     </row>
@@ -2019,22 +2019,22 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Dari Batik hingga Kerajinan Kulit, UMKM Lokal Ini Tembus Pasar Global</t>
+          <t>Bos-bos BUMN &amp;amp; Keluarga Dilarang Keras Pamer Gaya Hidup Mewah di Medsos</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Sun, 25 Oct 2026 16:56:57 +0700</t>
+          <t>Mon, 26 Oct 2026 20:12:07 +0700</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/25/umkm-1792924003903_169.jpeg?w=360&amp;amp;q=90" /&gt; Mereka melibatkan masyarakat dalam produksi dan pengembangan usaha.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2023/04/06/ilustrasi-flexing-keluarga-pejabat_169.jpeg?w=360&amp;amp;q=90" /&gt; Danantara melarang direksi dan dewan komisaris memamerkan gaya hidup mewah atau berlebihan hingga debat politik dan komentar partisan di media sosial (medsos).</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/solusiukm/d-8723517/dari-batik-hingga-kerajinan-kulit-umkm-lokal-ini-tembus-pasar-global</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8725293/bos-bos-bumn-keluarga-dilarang-keras-pamer-gaya-hidup-mewah-di-medsos</t>
         </is>
       </c>
     </row>
@@ -2046,22 +2046,22 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Bantu Petani di Lampung, Mentan Siapkan Benih hingga Alat Pertanian</t>
+          <t>Menjemput Asa Berburu Peluang Kerja</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Sun, 25 Oct 2026 16:11:44 +0700</t>
+          <t>Mon, 26 Oct 2026 20:00:40 +0700</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/25/bantu-petani-di-lampung-mentan-siapkan-benih-hingga-alat-pertanian-1792919455925_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Pertanian Andi Amran Sulaiman menanggapi keluhan petani Lampung dengan dukungan benih dan alat pertanian, serta </t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/26/menjemput-asa-berburu-peluang-kerja-1792994483182_169.jpeg?w=360&amp;amp;q=90" /&gt; Pencari kerja berburu peluang di bursa karier yang diikuti 46 perusahaan di Bandung. Bursa karier ini menyediakan ratusan lowongan.</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8723415/bantu-petani-di-lampung-mentan-siapkan-benih-hingga-alat-pertanian</t>
+          <t>https://finance.detik.com/foto-bisnis/d-8724380/menjemput-asa-berburu-peluang-kerja</t>
         </is>
       </c>
     </row>
@@ -2073,22 +2073,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Harga Cabai Rawit Masih Mahal, Tembus Rp 102 Ribu/Kg!</t>
+          <t>Bea Cukai Gagalkan Penyelundupan Ekspor Emas 402 Kg Senilai Rp 1,02 T di 2026</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Sun, 25 Oct 2026 15:56:26 +0700</t>
+          <t>Mon, 26 Oct 2026 20:00:00 +0700</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/21/harga-cabai-rawit-merah-tembus-rp70-ribu-per-kg-di-tangerang-1789977514373_169.jpeg?w=360&amp;amp;q=90" /&gt; Komoditas cabai masih dijual dengan harga tinggi, bahkan ada yang menyentuh Rp 100.000 per kilogram (kg).</t>
+          <t xml:space="preserve">&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/26/bea-cukai-gagalkan-penyelundupan-emas-2588-kg-ke-luar-negeri-1793002747999_169.jpeg?w=360&amp;amp;q=90" /&gt; Direktorat Jenderal Bea dan Cukai (DJBC) Kementerian Keuangan telah menindak penyelundupan ekspor emas secara ilegal 127 kali </t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8723279/harga-cabai-rawit-masih-mahal-tembus-rp-102-ribu-kg</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8725080/bea-cukai-gagalkan-penyelundupan-ekspor-emas-402-kg-senilai-rp-1-02-t-di-2026</t>
         </is>
       </c>
     </row>
@@ -2100,22 +2100,22 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Ribuan Penggemar Padati Indonesia Game Expo 2026</t>
+          <t>Bahlil Ungkap Lokasi PLTN: Batam-Halmahera</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Sun, 25 Oct 2026 15:00:16 +0700</t>
+          <t>Mon, 26 Oct 2026 19:45:25 +0700</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/24/surga-pencinta-gim-dan-budaya-pop-di-indonesia-game-expo-2026-1792836890279.jpeg?w=360&amp;amp;q=90" /&gt; Indonesia Game Expo (IGE) 2026 di ICE BSD, Tangerang, menghadirkan lebih dari 200 booth gim, kartu koleksi, action figure, hingga</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/15/kunjungan-menteri-esdm-bahlil-lahadalia-usai-meninjau-program-lisdes-di-karawang-1792058690303_169.jpeg?w=360&amp;amp;q=90" /&gt; Rencana pembangunan PLTN di Indonesia terungkap, Batam dan Halmahera masuk dalam kajian dan studi kelayaka</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/foto-bisnis/d-8722309/ribuan-penggemar-padati-indonesia-game-expo-2026</t>
+          <t>https://finance.detik.com/energi/d-8725233/bahlil-ungkap-lokasi-pltn-batam-halmahera</t>
         </is>
       </c>
     </row>
@@ -2127,22 +2127,22 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Rak Besi Banting Harga di Transmart Full Day Sale</t>
+          <t>Danantara Atur Ketat Perjalanan Dinas Bos-bos BUMN, Ini Isinya</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Sun, 25 Oct 2026 15:00:00 +0700</t>
+          <t>Mon, 26 Oct 2026 19:45:25 +0700</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/25/transmart-full-day-sale-1792899602865_169.png?w=360&amp;amp;q=90" /&gt; Pesta diskon Transmart Full Day Sale kembali digelar seharian penuh.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/07/01/wisma-danantara-indonesia-1751345496674_169.jpeg?w=360&amp;amp;q=90" /&gt; Badan Pengelola Investasi Daya Anagata Nusantara (BPI Danantara) menetapkan aturan ketat perjalanan dinas direksi dan dewan komisaris BUMN.</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8722992/rak-besi-banting-harga-di-transmart-full-day-sale</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8725269/danantara-atur-ketat-perjalanan-dinas-bos-bos-bumn-ini-isinya</t>
         </is>
       </c>
     </row>
@@ -2154,22 +2154,22 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>KPK Usul Harta Pejabat Tak Dilaporkan di LHKPN Bisa Dirampas Negara</t>
+          <t>KPK Panggil Lagi Nusron Wahid usai Dua Kali Mangkir</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Mon, 26 Oct 2026 00:46:08 +0700</t>
+          <t>Mon, 26 Oct 2026 21:21:18 +0700</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Selain itu, KPK mengusulkan negara dapat merampas harta penyelenggara negara apabila kekayaan yang dimiliki ternyata melebihi jumlah di LHKPN</t>
+          <t>Penyidik KPK membutuhkan keterangan Nusron untuk melengkapi proses penyidikan.</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8321071/kpk-usul-harta-pejabat-tak-dilaporkan-di-lhkpn-bisa-dirampas-negara</t>
+          <t>https://www.liputan6.com/news/read/8321772/kpk-panggil-lagi-nusron-wahid-usai-dua-kali-mangkir</t>
         </is>
       </c>
     </row>
@@ -2181,22 +2181,22 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Gubernur URI Menghadap Prabowo di Hambalang, Ini yang Dilaporkan</t>
+          <t>Penampakan WN Taiwan, Tersangka Kasus Penyelundupan 1,16 Ton Ketamin</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Sun, 25 Oct 2026 21:18:52 +0700</t>
+          <t>Mon, 26 Oct 2026 21:03:03 +0700</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Pertemuan tersebut juga membahas perkembangan pembangunan gedung URI.</t>
+          <t>Polri menetapkan WN Taiwan YCY sebagai tersangka utama kasus penyelundupan 1,16 ton ketamin.</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8321012/gubernur-uri-menghadap-prabowo-di-hambalang-ini-yang-dilaporkan</t>
+          <t>https://www.liputan6.com/news/read/8321764/penampakan-wn-taiwan-tersangka-kasus-penyelundupan-116-ton-ketamin</t>
         </is>
       </c>
     </row>
@@ -2208,22 +2208,22 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Megawati: Anak Muda Harus Berani Lawan Ketidakadilan dan Bela Rakyat</t>
+          <t>Pemotor Tewas Tabrak Pembatas Jalan di Depan PIM 2</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Sun, 25 Oct 2026 21:09:28 +0700</t>
+          <t>Mon, 26 Oct 2026 20:35:11 +0700</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Menurut Megawati, generasi muda tidak cukup hanya memiliki kecerdasan dan keterampilan.</t>
+          <t>Pengendara Honda Beat berusia 24 tahun meninggal dunia setelah menabrak pembatas jalan di depan PIM 2, Jakarta Selatan. Penyebab kecelakaan masih diselidiki polisi.</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8321007/megawati-anak-muda-harus-berani-lawan-ketidakadilan-dan-bela-rakyat</t>
+          <t>https://www.liputan6.com/news/read/8321754/pemotor-tewas-tabrak-pembatas-jalan-di-depan-pim-2</t>
         </is>
       </c>
     </row>
@@ -2235,22 +2235,22 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Napak Tilas Sumpah Pemuda, 500 Anak Muda Susuri Jejak Sejarah Jakarta</t>
+          <t>Menkomdigi: 45 Persen Anak Pernah Jadi Korban Perundungan Siber</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Sun, 25 Oct 2026 20:12:32 +0700</t>
+          <t>Mon, 26 Oct 2026 20:33:25 +0700</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Sebanyak 500 pelajar dan pemuda menyusuri sejumlah lokasi bersejarah di Jakarta untuk mengenang semangat persatuan dalam Sumpah Pemuda 1928.</t>
+          <t>Temuan tersebut menunjukkan pentingnya penguatan perlindungan anak di ruang digital.</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8320963/napak-tilas-sumpah-pemuda-500-anak-muda-susuri-jejak-sejarah-jakarta</t>
+          <t>https://www.liputan6.com/news/read/8321752/menkomdigi-45-persen-anak-pernah-jadi-korban-perundungan-siber</t>
         </is>
       </c>
     </row>
@@ -2262,22 +2262,22 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Pramono Klaim Modifikasi Cuaca Bantu Sukseskan Jakarta Running Festival</t>
+          <t>Prabowo Belum Setujui Usul Luhut soal Perubahan Definisi Korupsi, Ini Alasannya</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Sun, 25 Oct 2026 19:04:02 +0700</t>
+          <t>Mon, 26 Oct 2026 20:09:43 +0700</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Pramono Anung menyebutmodifikasi cuaca  selama dua hari penyelenggaraan Jakarta Running Festival membantu menurunkan polusi udara dan mengantisipasi hujan di sejumlah wilayah.</t>
+          <t>Yusril dan Prabowo berdiskusi mengenai usulan DEN untuk mengubah definisi korupsi dalam UU Tipikor.</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8320953/pramono-klaim-modifikasi-cuaca-bantu-sukseskan-jakarta-running-festival</t>
+          <t>https://www.liputan6.com/news/read/8321744/prabowo-belum-setujui-usul-luhut-soal-perubahan-definisi-korupsi-ini-alasannya</t>
         </is>
       </c>
     </row>
@@ -2289,22 +2289,22 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Hasto Cerita Kebijakan Megawati Cegah Hutan Bekas Karhutla Jadi Kebun Sawit</t>
+          <t>Bukan Sekadar Kurir, Bareskrim Incar Sumber Emas Ilegal</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Sun, 25 Oct 2026 18:01:03 +0700</t>
+          <t>Mon, 26 Oct 2026 20:05:00 +0700</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Menurut Hasto, sanksi tegas diperlukan, terutama jika lahan yang dibakar kemudian dialihfungsikan menjadi kebun sawit.</t>
+          <t>Upaya ini melibatkan koordinasi dengan Bea Cukai untuk mengungkap jaringan peredaran.</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8320941/hasto-cerita-kebijakan-megawati-cegah-hutan-bekas-karhutla-jadi-kebun-sawit</t>
+          <t>https://www.liputan6.com/news/read/8321740/bukan-sekadar-kurir-bareskrim-incar-sumber-emas-ilegal</t>
         </is>
       </c>
     </row>
@@ -2316,22 +2316,22 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Muntaber Massal di Tangsel, Warga Tuntut Kompensasi Rp 539 Juta</t>
+          <t>Titik Api Way Kambas Padam, Lokasi 14 Km dari Pusat Latihan Gajah</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Sun, 25 Oct 2026 17:38:23 +0700</t>
+          <t>Mon, 26 Oct 2026 19:12:36 +0700</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Warga memberikan tenggat waktu hingga Selasa (27/10/2026) agar perusahaan memberikan kejelasan mengenai tuntutan ganti rugi.</t>
+          <t>BPBD Lampung menyatakan titik karhutla yang ditangani di TN Way Kambas telah padam dan berjarak 14 kilometer dari Pusat Latihan Gajah. Pemadaman di titik lain masih berlanjut.</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8320929/muntaber-massal-di-tangsel-warga-tuntut-kompensasi-rp-539-juta</t>
+          <t>https://www.liputan6.com/news/read/8321696/titik-api-way-kambas-padam-lokasi-14-km-dari-pusat-latihan-gajah</t>
         </is>
       </c>
     </row>
@@ -2343,22 +2343,22 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Indonesia Siapkan Forum Konservasi Terumbu Karang di AS</t>
+          <t>Bukan Lagi Bentuk Padat, Ini Modus Baru Penyelundupan Emas Ilegal</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Sun, 25 Oct 2026 17:33:52 +0700</t>
+          <t>Mon, 26 Oct 2026 18:57:38 +0700</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Indonesia menyiapkan forum internasional di Washington pada 2027 untuk memperluas dukungan pembiayaan dan kerja sama konservasi terumbu karang.</t>
+          <t>Pelaku penyelundupan menggunakan beragam cara untuk menyembunyikan emas.</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8320927/indonesia-siapkan-forum-konservasi-terumbu-karang-di-as</t>
+          <t>https://www.liputan6.com/news/read/8321703/bukan-lagi-bentuk-padat-ini-modus-baru-penyelundupan-emas-ilegal</t>
         </is>
       </c>
     </row>
@@ -2370,22 +2370,22 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Anggota VI BPK Fathan Subchi Meninggal Dunia</t>
+          <t>Anggota DPR Tak Setuju Pansel Penyelenggara Pemilu Dibentuk Sekarang, Ini Alasannya</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Sun, 25 Oct 2026 17:15:27 +0700</t>
+          <t>Mon, 26 Oct 2026 18:52:36 +0700</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Anggota VI BPK Fathan Subchi meninggal dunia pada usia 56 tahun saat menjalankan tugas pemeriksaan di Moskow, Rusia, Minggu (25/10/2026).</t>
+          <t>Untuk mengatasi persoalan itu, Doli menawarkan dua opsi.</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8320918/anggota-vi-bpk-fathan-subchi-meninggal-dunia</t>
+          <t>https://www.liputan6.com/news/read/8321701/anggota-dpr-tak-setuju-pansel-penyelenggara-pemilu-dibentuk-sekarang-ini-alasannya</t>
         </is>
       </c>
     </row>
@@ -2397,22 +2397,22 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>SBY Kenang Pengabdian Widodo AS saat Indonesia Hadapi Krisis 1998</t>
+          <t>Doli Kurnia Tanggapi Mekanisme Pemakzulan</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Sun, 25 Oct 2026 17:12:01 +0700</t>
+          <t>Mon, 26 Oct 2026 18:39:35 +0700</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>SBY mengenang mantan Panglima TNI Widodo AS sebagai prajurit dan negarawan yang berkomitmen menjaga konstitusi serta keutuhan bangsa.</t>
+          <t>Mekanisme pemakzulan wakil presiden sendiri disebutnya telah diatur dalam konstitusi.</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8320914/sby-kenang-pengabdian-widodo-as-saat-indonesia-hadapi-krisis-1998</t>
+          <t>https://www.liputan6.com/news/read/8321689/doli-kurnia-tanggapi-mekanisme-pemakzulan</t>
         </is>
       </c>
     </row>
@@ -2424,22 +2424,22 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Penataan Stasiun Karet dan Sudirman Baru Rampung Akhir 2026</t>
+          <t>Target Walkot Bekasi Bangun 2 Halte Usai Disinggung Pramono</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Sun, 25 Oct 2026 16:27:53 +0700</t>
+          <t>Mon, 26 Oct 2026 18:26:06 +0700</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>KAI menargetkan penataan kawasan Stasiun Karet dan Sudirman Baru rampung 31 Desember 2026, dengan fasilitas baru untuk memudahkan mobilitas penumpang.</t>
+          <t>Pembangunan dua Halte Transjabodetabek di Bekasi ditargetkan rampung awal Desember 2026.</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8320894/penataan-stasiun-karet-dan-sudirman-baru-rampung-akhir-2026</t>
+          <t>https://www.liputan6.com/news/read/8321682/target-walkot-bekasi-bangun-2-halte-usai-disinggung-pramono</t>
         </is>
       </c>
     </row>
@@ -2451,22 +2451,22 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Seruni dan Dekranas Dukung Pelestarian Tenun Gringsing</t>
+          <t>Kemenkum Buat Program bagi 45 Ribu Napi, Dipekerjakan di Proyek Pemerintah</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Sun, 25 Oct 2026 15:57:26 +0700</t>
+          <t>Mon, 26 Oct 2026 18:22:31 +0700</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Penyerahan bantuan ini disertai pemeriksaan mata untuk mengetahui tingkat minus setiap penerima.</t>
+          <t>Kementerian Hukum menyiapkan program rehabilitasi dan reedukasi bagi 30.000–45.000 narapidana yang berpeluang dilibatkan dalam proyek kementerian dan lembaga.</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8320888/seruni-dan-dekranas-dukung-pelestarian-tenun-gringsing</t>
+          <t>https://www.liputan6.com/news/read/8321679/kemenkum-buat-program-bagi-45-ribu-napi-dipekerjakan-di-proyek-pemerintah</t>
         </is>
       </c>
     </row>
@@ -2478,22 +2478,22 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Demi Efisiensi, Tri Tito Karnavian Gabungkan Rapat Tiga Lembaga</t>
+          <t>Yusril Menghadap Prabowo, Bahas Perubahan Definisi Korupsi</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Sun, 25 Oct 2026 15:54:35 +0700</t>
+          <t>Mon, 26 Oct 2026 18:09:58 +0700</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Tri Tito Karnavian menggabungkan rapat kerja Dekranas, TP PKK, dan TP Posyandu dalam satu forum untuk meningkatkan efisiensi anggaran dan koordinasi program.</t>
+          <t>Menurut Yusril, terdapat sejumlah perbuatan yang merugikan negara, tetapi belum tentu dapat dikategorikan sebagai korupsi.</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8320886/demi-efisiensi-tri-tito-karnavian-gabungkan-rapat-tiga-lembaga</t>
+          <t>https://www.liputan6.com/news/read/8321672/yusril-menghadap-prabowo-bahas-perubahan-definisi-korupsi</t>
         </is>
       </c>
     </row>
@@ -2505,22 +2505,22 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Pramono: Izin Rumah Ibadah Harus Selesai dalam Dua Pekan</t>
+          <t>Bea Cukai Ungkap 127 Kasus Emas Ilegal, Nilainya Tembus Rp 1,02 Triliun</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Sun, 25 Oct 2026 15:41:01 +0700</t>
+          <t>Mon, 26 Oct 2026 18:04:22 +0700</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Pramono Anung meminta izin pembangunan rumah ibadah di Jakarta diselesaikan dalam satu hingga dua pekan setelah seluruh persyaratan administrasi terpenuhi.</t>
+          <t>Bea Cukai mencatat 127 penindakan pengeluaran emas ilegal hingga 26 Oktober 2026, dengan barang bukti 402,31 kg emas senilai Rp1,02 triliun.</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8320868/pramono-izin-rumah-ibadah-harus-selesai-dalam-dua-pekan</t>
+          <t>https://www.liputan6.com/news/read/8321638/bea-cukai-ungkap-127-kasus-emas-ilegal-nilainya-tembus-rp-102-triliun</t>
         </is>
       </c>
     </row>
@@ -2532,22 +2532,22 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Kondisi Terkini Driver Ojol Dilindas BYD di Blok M</t>
+          <t>Kampung Ambon Digerebek Empat Kali Dalam Sebulan, 7 Orang Ditangkap</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Sun, 25 Oct 2026 15:27:27 +0700</t>
+          <t>Mon, 26 Oct 2026 18:02:17 +0700</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Korban berinisial HS (56) saat ini masih menjalani observasi di Rumah Sakit Fatmawati.</t>
+          <t>Penggerebekan di Kampung Ambon tersebut menjadi operasi keempat sepanjang Oktober 2026</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8320875/kondisi-terkini-driver-ojol-dilindas-byd-di-blok-m</t>
+          <t>https://www.liputan6.com/news/read/8321662/kampung-ambon-digerebek-empat-kali-dalam-sebulan-7-orang-ditangkap</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data pasar & berita - 2026-10-27 00:57 UTC
</commit_message>
<xml_diff>
--- a/data/market_news_latest.xlsx
+++ b/data/market_news_latest.xlsx
@@ -487,20 +487,20 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>5373.0942</v>
+        <v>5439.2578</v>
       </c>
       <c r="F2" t="n">
-        <v>-66.1636</v>
+        <v>51.353</v>
       </c>
       <c r="G2" t="n">
-        <v>-1.22</v>
+        <v>0.95</v>
       </c>
       <c r="H2" t="n">
-        <v>0</v>
+        <v>397036500</v>
       </c>
     </row>
     <row r="3">
@@ -525,16 +525,16 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>7701.54</v>
+        <v>7676.77</v>
       </c>
       <c r="F3" t="n">
-        <v>77.8599</v>
+        <v>53.0898</v>
       </c>
       <c r="G3" t="n">
-        <v>1.02</v>
+        <v>0.7</v>
       </c>
       <c r="H3" t="n">
-        <v>659034209</v>
+        <v>2759066000</v>
       </c>
     </row>
     <row r="4">
@@ -559,16 +559,16 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>52491.9609</v>
+        <v>52361.5781</v>
       </c>
       <c r="F4" t="n">
-        <v>276.8008</v>
+        <v>146.418</v>
       </c>
       <c r="G4" t="n">
-        <v>0.53</v>
+        <v>0.28</v>
       </c>
       <c r="H4" t="n">
-        <v>98731755</v>
+        <v>387915369</v>
       </c>
     </row>
     <row r="5">
@@ -593,16 +593,16 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>26305.5059</v>
+        <v>26169.3809</v>
       </c>
       <c r="F5" t="n">
-        <v>350.166</v>
+        <v>214.041</v>
       </c>
       <c r="G5" t="n">
-        <v>1.35</v>
+        <v>0.82</v>
       </c>
       <c r="H5" t="n">
-        <v>2381854000</v>
+        <v>6508626000</v>
       </c>
     </row>
     <row r="6">
@@ -623,20 +623,20 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>62693.1602</v>
+        <v>63392.0312</v>
       </c>
       <c r="F6" t="n">
-        <v>-214.6797</v>
+        <v>698.8711</v>
       </c>
       <c r="G6" t="n">
-        <v>-0.34</v>
+        <v>1.11</v>
       </c>
       <c r="H6" t="n">
-        <v>208600000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -657,20 +657,20 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>23211.8105</v>
+        <v>23093.3691</v>
       </c>
       <c r="F7" t="n">
-        <v>118.4414</v>
+        <v>158.6895</v>
       </c>
       <c r="G7" t="n">
-        <v>0.51</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="H7" t="n">
-        <v>0</v>
+        <v>3842800000</v>
       </c>
     </row>
     <row r="8">
@@ -694,15 +694,9 @@
           <t>2026-10-26</t>
         </is>
       </c>
-      <c r="E8" t="n">
-        <v>3697.52</v>
-      </c>
-      <c r="F8" t="n">
-        <v>7.0449</v>
-      </c>
-      <c r="G8" t="n">
-        <v>0.19</v>
-      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
       <c r="H8" t="n">
         <v>329758840</v>
       </c>
@@ -725,20 +719,20 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>10768.2695</v>
+        <v>10690.4004</v>
       </c>
       <c r="F9" t="n">
-        <v>77.8691</v>
+        <v>-34.5996</v>
       </c>
       <c r="G9" t="n">
-        <v>0.73</v>
+        <v>-0.32</v>
       </c>
       <c r="H9" t="n">
-        <v>0</v>
+        <v>697030600</v>
       </c>
     </row>
     <row r="10">
@@ -759,20 +753,20 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>25497.0703</v>
+        <v>25181.6504</v>
       </c>
       <c r="F10" t="n">
-        <v>315.4199</v>
+        <v>-190.0996</v>
       </c>
       <c r="G10" t="n">
-        <v>1.25</v>
+        <v>-0.75</v>
       </c>
       <c r="H10" t="n">
-        <v>0</v>
+        <v>58950600</v>
       </c>
     </row>
     <row r="11">
@@ -793,20 +787,20 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>5415.9102</v>
+        <v>5422.1602</v>
       </c>
       <c r="F11" t="n">
-        <v>-6.25</v>
+        <v>7.02</v>
       </c>
       <c r="G11" t="n">
-        <v>-0.12</v>
+        <v>0.13</v>
       </c>
       <c r="H11" t="n">
-        <v>0</v>
+        <v>388429200</v>
       </c>
     </row>
     <row r="12">
@@ -831,13 +825,13 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>17978</v>
+        <v>18081</v>
       </c>
       <c r="F12" t="n">
-        <v>-75</v>
+        <v>28</v>
       </c>
       <c r="G12" t="n">
-        <v>-0.42</v>
+        <v>0.16</v>
       </c>
       <c r="H12" t="n">
         <v>0</v>
@@ -865,13 +859,13 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>101.99</v>
+        <v>102.034</v>
       </c>
       <c r="F13" t="n">
-        <v>0.18</v>
+        <v>0.224</v>
       </c>
       <c r="G13" t="n">
-        <v>0.18</v>
+        <v>0.22</v>
       </c>
       <c r="H13" t="n">
         <v>0</v>
@@ -895,17 +889,17 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>157.55</v>
+        <v>157.592</v>
       </c>
       <c r="F14" t="n">
-        <v>1.056</v>
+        <v>0.762</v>
       </c>
       <c r="G14" t="n">
-        <v>0.67</v>
+        <v>0.49</v>
       </c>
       <c r="H14" t="n">
         <v>0</v>
@@ -933,13 +927,13 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>0.497</v>
+        <v>0.4986</v>
       </c>
       <c r="F15" t="n">
-        <v>-0.0018</v>
+        <v>-0.0002</v>
       </c>
       <c r="G15" t="n">
-        <v>-0.36</v>
+        <v>-0.04</v>
       </c>
       <c r="H15" t="n">
         <v>0</v>
@@ -967,13 +961,13 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>0.5285</v>
+        <v>0.5301</v>
       </c>
       <c r="F16" t="n">
-        <v>-0.003</v>
+        <v>-0.0014</v>
       </c>
       <c r="G16" t="n">
-        <v>-0.5600000000000001</v>
+        <v>-0.26</v>
       </c>
       <c r="H16" t="n">
         <v>0</v>
@@ -1001,13 +995,13 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>0.4043</v>
+        <v>0.4025</v>
       </c>
       <c r="F17" t="n">
-        <v>0.0011</v>
+        <v>-0.0007</v>
       </c>
       <c r="G17" t="n">
-        <v>0.27</v>
+        <v>-0.17</v>
       </c>
       <c r="H17" t="n">
         <v>0</v>
@@ -1034,17 +1028,11 @@
           <t>2026-10-26</t>
         </is>
       </c>
-      <c r="E18" t="n">
-        <v>81.685</v>
-      </c>
-      <c r="F18" t="n">
-        <v>0.345</v>
-      </c>
-      <c r="G18" t="n">
-        <v>0.42</v>
-      </c>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
       <c r="H18" t="n">
-        <v>8768809</v>
+        <v>24127074</v>
       </c>
     </row>
     <row r="19">
@@ -1068,17 +1056,11 @@
           <t>2026-10-26</t>
         </is>
       </c>
-      <c r="E19" t="n">
-        <v>77.315</v>
-      </c>
-      <c r="F19" t="n">
-        <v>0.265</v>
-      </c>
-      <c r="G19" t="n">
-        <v>0.34</v>
-      </c>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr"/>
       <c r="H19" t="n">
-        <v>11317534</v>
+        <v>41292931</v>
       </c>
     </row>
     <row r="20">
@@ -1103,16 +1085,16 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>4032.8</v>
+        <v>4026</v>
       </c>
       <c r="F20" t="n">
-        <v>24.9001</v>
+        <v>18.1001</v>
       </c>
       <c r="G20" t="n">
-        <v>0.62</v>
+        <v>0.45</v>
       </c>
       <c r="H20" t="n">
-        <v>86338</v>
+        <v>7342</v>
       </c>
     </row>
     <row r="21">
@@ -1137,16 +1119,16 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>101.07</v>
+        <v>101.18</v>
       </c>
       <c r="F21" t="n">
-        <v>-2.2</v>
+        <v>-2.09</v>
       </c>
       <c r="G21" t="n">
-        <v>-2.13</v>
+        <v>-2.02</v>
       </c>
       <c r="H21" t="n">
-        <v>141272</v>
+        <v>4916</v>
       </c>
     </row>
     <row r="22">
@@ -1171,16 +1153,16 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>110.14</v>
+        <v>110.06</v>
       </c>
       <c r="F22" t="n">
-        <v>-6.58</v>
+        <v>-6.66</v>
       </c>
       <c r="G22" t="n">
-        <v>-5.64</v>
+        <v>-5.71</v>
       </c>
       <c r="H22" t="n">
-        <v>20633</v>
+        <v>698</v>
       </c>
     </row>
     <row r="23">
@@ -1205,16 +1187,16 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>6.521</v>
+        <v>6.572</v>
       </c>
       <c r="F23" t="n">
-        <v>0.045</v>
+        <v>0.096</v>
       </c>
       <c r="G23" t="n">
-        <v>0.6899999999999999</v>
+        <v>1.48</v>
       </c>
       <c r="H23" t="n">
-        <v>22262</v>
+        <v>681</v>
       </c>
     </row>
     <row r="24">
@@ -1238,17 +1220,11 @@
           <t>2026-10-26</t>
         </is>
       </c>
-      <c r="E24" t="n">
-        <v>61.945</v>
-      </c>
-      <c r="F24" t="n">
-        <v>-0.065</v>
-      </c>
-      <c r="G24" t="n">
-        <v>-0.1</v>
-      </c>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr"/>
       <c r="H24" t="n">
-        <v>6265588</v>
+        <v>17850668</v>
       </c>
     </row>
     <row r="25">
@@ -1273,13 +1249,13 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>17.99</v>
+        <v>18.39</v>
       </c>
       <c r="F25" t="n">
-        <v>-1.46</v>
+        <v>-1.06</v>
       </c>
       <c r="G25" t="n">
-        <v>-7.51</v>
+        <v>-5.45</v>
       </c>
       <c r="H25" t="n">
         <v>0</v>
@@ -1303,20 +1279,20 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="E26" t="n">
-        <v>80311.7188</v>
+        <v>80104.82030000001</v>
       </c>
       <c r="F26" t="n">
-        <v>287.7109</v>
+        <v>80.8125</v>
       </c>
       <c r="G26" t="n">
-        <v>0.36</v>
+        <v>0.1</v>
       </c>
       <c r="H26" t="n">
-        <v>24188891136</v>
+        <v>27099494400</v>
       </c>
     </row>
     <row r="27">
@@ -1749,22 +1725,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Jurus Pemerintah Jaga Pasokan dan Harga Pangan Jelang Nataru</t>
+          <t>Pendaftaran Magang Nasional Batch 3 Dibuka Hari Ini</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Mon, 26 Oct 2026 21:36:17 +0700</t>
+          <t>Tue, 27 Oct 2026 07:30:58 +0700</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/26/rapat-koordinasi-terbatas-rakortas-bidang-pangan-yang-dipimpin-menteri-koordinator-bidang-pangan-ri-menko-pangan-zulkifli-hasa-1793025343365.jpeg?w=360&amp;amp;q=90" /&gt; Pemerintah antisipasi stabilitas pangan menjelang Nataru dengan </t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2023/05/03/gedung-kemnaker_169.jpeg?w=360&amp;amp;q=90" /&gt; Kementerian Ketenagakerjaan (Kemnaker) resmi membuka pendaftaran Program Magang Nasional (MagangHub) Batch 3 Angkatan II mulai hari ini, Selasa (27/10).</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8725387/jurus-pemerintah-jaga-pasokan-dan-harga-pangan-jelang-nataru</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8725378/pendaftaran-magang-nasional-batch-3-dibuka-hari-ini</t>
         </is>
       </c>
     </row>
@@ -1776,22 +1752,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>3.030 Penerbangan Terdampak Karhutla Sejak Agustus, 1.700 Rute Dibatalkan</t>
+          <t>Rencana Baru BEI Sikat Saham Gorengan</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Mon, 26 Oct 2026 21:30:00 +0700</t>
+          <t>Tue, 27 Oct 2026 07:00:49 +0700</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2023/10/05/ngeri-kabut-asap-bikin-jarak-pandang-di-bandara-palangka-raya-terbatas-1_169.jpeg?w=360&amp;amp;q=90" /&gt; Kemenhub mencatat sebanyak 3.030 penerbangan terdampak oleh kabut asap akibat kebakaran hutan dan lahan (karhutla) sejak 14 Agus</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/07/13/direktur-utama-bei-jeffrey-hendrik-1783928734693_169.jpeg?w=360&amp;amp;q=90" /&gt; Bursa Efek Indonesia (BEI) memperketat pengawasan saham gorengan dengan langsung investigasi emiten yang terindikasi melakukan manipulasi harga.</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8725381/3-030-penerbangan-terdampak-karhutla-sejak-agustus-1-700-rute-dibatalkan</t>
+          <t>https://finance.detik.com/bursa-dan-valas/d-8725377/rencana-baru-bei-sikat-saham-gorengan</t>
         </is>
       </c>
     </row>
@@ -1803,22 +1779,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Pertamina Dukung Perpres 107 Perkuat Ketahanan Energi Nasional</t>
+          <t>Penyelundupan Emas 25 Kg Digagalkan di 5 Bandara, Ini Daftarnya</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Mon, 26 Oct 2026 21:27:35 +0700</t>
+          <t>Tue, 27 Oct 2026 06:30:53 +0700</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/26/pertamina-siap-jalankan-perpres-107-untuk-perkuat-ketahanan-energi-nasional-1793024805115.jpeg?w=360&amp;amp;q=90" /&gt; Pertamina mendukung Perpres 107/2026 untuk memperkuat pengadaan energi nasional. Komitmen menjaga ketersediaan BBM </t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/26/bea-cukai-gagalkan-penyelundupan-emas-2588-kg-ke-luar-negeri-1793002748135_169.jpeg?w=360&amp;amp;q=90" /&gt; Direktorat Jenderal Bea dan Cukai Kementerian Keuangan menggagalkan upaya penyelundupan ekspor emas secara ilegal dengan total</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8725384/pertamina-dukung-perpres-107-perkuat-ketahanan-energi-nasional</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8725372/penyelundupan-emas-25-kg-digagalkan-di-5-bandara-ini-daftarnya</t>
         </is>
       </c>
     </row>
@@ -1830,22 +1806,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Harga Tiket Pesawat Bakal Turun 11-13% Saat Libur Natal &amp;amp; Tahun Baru</t>
+          <t>Dua Penyebab RI Pangkas Ekspor Gas ke Singapura</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Mon, 26 Oct 2026 21:16:28 +0700</t>
+          <t>Tue, 27 Oct 2026 05:55:15 +0700</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2023/11/11/ilustrasi-harga-tiket-pesawat_169.png?w=360&amp;amp;q=90" /&gt; Kementerian Perhubungan (Kemenhub) menargetkan harga tiket pesawat dapat turun 11-13% selama periode Natal dan Tahun Baru (Nataru) 2026/2027.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/04/28/menteri-esdm-bahlil-lahadalia-1777385212647_169.jpeg?w=360&amp;amp;q=90" /&gt; Menko Hilirisasi dan Transisi Energi Bahlil Lahadalia menjelaskan alasan pemangkasan ekspor gas ke Singapura.</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8725373/harga-tiket-pesawat-bakal-turun-11-13-saat-libur-natal-tahun-baru</t>
+          <t>https://finance.detik.com/energi/d-8725370/dua-penyebab-ri-pangkas-ekspor-gas-ke-singapura</t>
         </is>
       </c>
     </row>
@@ -1857,22 +1833,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Impor KRL Bekas Jepang Tunggu Restu Kemenhub</t>
+          <t>Minyak Jelantah 'Disulap' Jadi 11 Juta Liter SAF</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Mon, 26 Oct 2026 21:08:16 +0700</t>
+          <t>Mon, 26 Oct 2026 22:30:00 +0700</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2014/06/27/7792aea3-ac73-4740-974a-e71dca1fea91_169.jpg?w=360&amp;amp;q=90" /&gt; Kementerian Perhubungan (Kemenhub) mempelajari proposal pengadaan Kereta Rel Listrik (KRL) bekas dari Jepang.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/08/21/pt-pertamina-persero-telah-mengembangkan-pertamina-sustainable-aviation-fuel-saf-1755754152640_169.jpeg?w=360&amp;amp;q=90" /&gt; Pertamina memproduksi minyak jelantah menjadi bahan bakar bioavtur atau bahan bakar penerbangan ramah ling</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/infrastruktur/d-8725367/impor-krl-bekas-jepang-tunggu-restu-kemenhub</t>
+          <t>https://finance.detik.com/energi/d-8725402/minyak-jelantah-disulap-jadi-11-juta-liter-saf</t>
         </is>
       </c>
     </row>
@@ -1884,22 +1860,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Karya Siswa Disabilitas di Bali Tembus Toko Oleh-Oleh, Harga Mulai Rp 10 Ribu</t>
+          <t>UMKM Didorong Perluas Pasar Lewat Rantai Pasok Makan Bergizi Gratis</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Mon, 26 Oct 2026 21:00:41 +0700</t>
+          <t>Mon, 26 Oct 2026 22:00:44 +0700</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/26/karya-siswa-disabilitas-di-bali-tembus-toko-oleh-oleh-harga-mulai-rp-10-ribu-1792999583884_169.jpeg?w=360&amp;amp;q=90" /&gt; Siswa tunarungu di SLB Negeri 1 Tabanan, Bali, membuat kerajinan tangan. Produk mereka dijual di toko oleh-ole</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/26/umkm-didorong-perluas-pasar-lewat-rantai-pasok-makan-bergizi-gratis-1792994912262_169.jpeg?w=360&amp;amp;q=90" /&gt; Sebanyak 68 ribu UMKM terhubung dalam rantai pasok program Makan Bergizi Gratis (MBG). Keterlibatan usaha lokal diharap</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/foto-bisnis/d-8724549/karya-siswa-disabilitas-di-bali-tembus-toko-oleh-oleh-harga-mulai-rp-10-ribu</t>
+          <t>https://finance.detik.com/foto-bisnis/d-8724402/umkm-didorong-perluas-pasar-lewat-rantai-pasok-makan-bergizi-gratis</t>
         </is>
       </c>
     </row>
@@ -1911,22 +1887,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Truk AMDK Diusulkan Dikecualikan dari Pembatasan Saat Nataru</t>
+          <t>Proses Pengadaan KRL Baru Sudah Sejauh Mana? Ini Jawaban Menhub</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Mon, 26 Oct 2026 21:00:03 +0700</t>
+          <t>Mon, 26 Oct 2026 22:00:00 +0700</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2023/06/23/pangsa-pasar-air-minum-kemasan-lokal-meningkat-2_169.jpeg?w=360&amp;amp;q=90" /&gt; Distribusi AMDK diminta dikecualikan dalam pembatasan truk saat libur Nataru.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/20/perawatan-jaringan-listrik-krl-1792511606131_169.jpeg?w=360&amp;amp;q=90" /&gt; Kementerian Perhubungan (Kemenhub) buka suara soal progres serta skema pelaksanaan pengadaan 30 rangkaian Kereta Rel Listrik (KRL) baru.</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8725185/truk-amdk-diusulkan-dikecualikan-dari-pembatasan-saat-nataru</t>
+          <t>https://finance.detik.com/infrastruktur/d-8725393/proses-pengadaan-krl-baru-sudah-sejauh-mana-ini-jawaban-menhub</t>
         </is>
       </c>
     </row>
@@ -1938,22 +1914,22 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Tiga Penyebab Dana Operasional Dapur MBG Nggak Cair</t>
+          <t>Jurus Pemerintah Jaga Pasokan dan Harga Pangan Jelang Nataru</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Mon, 26 Oct 2026 21:00:00 +0700</t>
+          <t>Mon, 26 Oct 2026 21:36:17 +0700</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/06/08/realisasi-anggaran-program-makanan-bergizi-gratis-1780905690949_169.jpeg?w=360&amp;amp;q=90" /&gt; BGN mengungkapkan penyebab dana operasional Satuan Pelayanan Pemenuhan Gizi (SPPG) atau Dapur Makan Bergizi Gratis (MBG) tidak cair pada </t>
+          <t xml:space="preserve">&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/26/rapat-koordinasi-terbatas-rakortas-bidang-pangan-yang-dipimpin-menteri-koordinator-bidang-pangan-ri-menko-pangan-zulkifli-hasa-1793025343365.jpeg?w=360&amp;amp;q=90" /&gt; Pemerintah antisipasi stabilitas pangan menjelang Nataru dengan </t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8725276/tiga-penyebab-dana-operasional-dapur-mbg-nggak-cair</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8725387/jurus-pemerintah-jaga-pasokan-dan-harga-pangan-jelang-nataru</t>
         </is>
       </c>
     </row>
@@ -1965,22 +1941,22 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Petinggi BUMN Dilarang Pakai Anggaran &amp;amp; Fasilitas Perusahaan buat Kegiatan Pribadi</t>
+          <t>3.030 Penerbangan Terdampak Karhutla Sejak Agustus, 1.700 Rute Dibatalkan</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Mon, 26 Oct 2026 20:38:32 +0700</t>
+          <t>Mon, 26 Oct 2026 21:30:00 +0700</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2020/07/02/logo-baru-kementerian-bumn-1_169.jpeg?w=360&amp;amp;q=90" /&gt; Danantara melarang direksi dan dewan komisaris BUMN menggunakan anggaran maupun fasilitas perusahaan untuk hobi, olahraga hingga kegiatan pribadi</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2023/10/05/ngeri-kabut-asap-bikin-jarak-pandang-di-bandara-palangka-raya-terbatas-1_169.jpeg?w=360&amp;amp;q=90" /&gt; Kemenhub mencatat sebanyak 3.030 penerbangan terdampak oleh kabut asap akibat kebakaran hutan dan lahan (karhutla) sejak 14 Agus</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8725332/petinggi-bumn-dilarang-pakai-anggaran-fasilitas-perusahaan-buat-kegiatan-pribadi</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8725381/3-030-penerbangan-terdampak-karhutla-sejak-agustus-1-700-rute-dibatalkan</t>
         </is>
       </c>
     </row>
@@ -1992,22 +1968,22 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Bos Danantara Sebut Obligasi US$ 1,5 M Diserbu Investor Asing</t>
+          <t>Pertamina Dukung Perpres 107 Perkuat Ketahanan Energi Nasional</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Mon, 26 Oct 2026 20:30:13 +0700</t>
+          <t>Mon, 26 Oct 2026 21:27:35 +0700</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/22/chief-investment-officer-cio-danantara-indonesia-pandu-sjahrir-1792645980929_169.jpeg?w=360&amp;amp;q=90" /&gt; Danantara mengungkapkan penerbitan obligasi US$ 1,5 miliar atau sekitar Rp 27,15 triliun (kurs Rp 18.100) mendapat sambutan </t>
+          <t xml:space="preserve">&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/26/pertamina-siap-jalankan-perpres-107-untuk-perkuat-ketahanan-energi-nasional-1793024805115.jpeg?w=360&amp;amp;q=90" /&gt; Pertamina mendukung Perpres 107/2026 untuk memperkuat pengadaan energi nasional. Komitmen menjaga ketersediaan BBM </t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/bursa-dan-valas/d-8725114/bos-danantara-sebut-obligasi-us-1-5-m-diserbu-investor-asing</t>
+          <t>https://finance.detik.com/energi/d-8725384/pertamina-dukung-perpres-107-perkuat-ketahanan-energi-nasional</t>
         </is>
       </c>
     </row>
@@ -2019,22 +1995,22 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Bos-bos BUMN &amp;amp; Keluarga Dilarang Keras Pamer Gaya Hidup Mewah di Medsos</t>
+          <t>Harga Tiket Pesawat Bakal Turun 11-13% Saat Libur Natal &amp;amp; Tahun Baru</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Mon, 26 Oct 2026 20:12:07 +0700</t>
+          <t>Mon, 26 Oct 2026 21:16:28 +0700</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2023/04/06/ilustrasi-flexing-keluarga-pejabat_169.jpeg?w=360&amp;amp;q=90" /&gt; Danantara melarang direksi dan dewan komisaris memamerkan gaya hidup mewah atau berlebihan hingga debat politik dan komentar partisan di media sosial (medsos).</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2023/11/11/ilustrasi-harga-tiket-pesawat_169.png?w=360&amp;amp;q=90" /&gt; Kementerian Perhubungan (Kemenhub) menargetkan harga tiket pesawat dapat turun 11-13% selama periode Natal dan Tahun Baru (Nataru) 2026/2027.</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8725293/bos-bos-bumn-keluarga-dilarang-keras-pamer-gaya-hidup-mewah-di-medsos</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8725373/harga-tiket-pesawat-bakal-turun-11-13-saat-libur-natal-tahun-baru</t>
         </is>
       </c>
     </row>
@@ -2046,22 +2022,22 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Menjemput Asa Berburu Peluang Kerja</t>
+          <t>Impor KRL Bekas Jepang Tunggu Restu Kemenhub</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Mon, 26 Oct 2026 20:00:40 +0700</t>
+          <t>Mon, 26 Oct 2026 21:08:16 +0700</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/26/menjemput-asa-berburu-peluang-kerja-1792994483182_169.jpeg?w=360&amp;amp;q=90" /&gt; Pencari kerja berburu peluang di bursa karier yang diikuti 46 perusahaan di Bandung. Bursa karier ini menyediakan ratusan lowongan.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2014/06/27/7792aea3-ac73-4740-974a-e71dca1fea91_169.jpg?w=360&amp;amp;q=90" /&gt; Kementerian Perhubungan (Kemenhub) mempelajari proposal pengadaan Kereta Rel Listrik (KRL) bekas dari Jepang.</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/foto-bisnis/d-8724380/menjemput-asa-berburu-peluang-kerja</t>
+          <t>https://finance.detik.com/infrastruktur/d-8725367/impor-krl-bekas-jepang-tunggu-restu-kemenhub</t>
         </is>
       </c>
     </row>
@@ -2073,22 +2049,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Bea Cukai Gagalkan Penyelundupan Ekspor Emas 402 Kg Senilai Rp 1,02 T di 2026</t>
+          <t>Karya Siswa Disabilitas di Bali Tembus Toko Oleh-Oleh, Harga Mulai Rp 10 Ribu</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Mon, 26 Oct 2026 20:00:00 +0700</t>
+          <t>Mon, 26 Oct 2026 21:00:41 +0700</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/26/bea-cukai-gagalkan-penyelundupan-emas-2588-kg-ke-luar-negeri-1793002747999_169.jpeg?w=360&amp;amp;q=90" /&gt; Direktorat Jenderal Bea dan Cukai (DJBC) Kementerian Keuangan telah menindak penyelundupan ekspor emas secara ilegal 127 kali </t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/26/karya-siswa-disabilitas-di-bali-tembus-toko-oleh-oleh-harga-mulai-rp-10-ribu-1792999583884_169.jpeg?w=360&amp;amp;q=90" /&gt; Siswa tunarungu di SLB Negeri 1 Tabanan, Bali, membuat kerajinan tangan. Produk mereka dijual di toko oleh-ole</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8725080/bea-cukai-gagalkan-penyelundupan-ekspor-emas-402-kg-senilai-rp-1-02-t-di-2026</t>
+          <t>https://finance.detik.com/foto-bisnis/d-8724549/karya-siswa-disabilitas-di-bali-tembus-toko-oleh-oleh-harga-mulai-rp-10-ribu</t>
         </is>
       </c>
     </row>
@@ -2100,22 +2076,22 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Bahlil Ungkap Lokasi PLTN: Batam-Halmahera</t>
+          <t>Truk AMDK Diusulkan Dikecualikan dari Pembatasan Saat Nataru</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Mon, 26 Oct 2026 19:45:25 +0700</t>
+          <t>Mon, 26 Oct 2026 21:00:03 +0700</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/15/kunjungan-menteri-esdm-bahlil-lahadalia-usai-meninjau-program-lisdes-di-karawang-1792058690303_169.jpeg?w=360&amp;amp;q=90" /&gt; Rencana pembangunan PLTN di Indonesia terungkap, Batam dan Halmahera masuk dalam kajian dan studi kelayaka</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2023/06/23/pangsa-pasar-air-minum-kemasan-lokal-meningkat-2_169.jpeg?w=360&amp;amp;q=90" /&gt; Distribusi AMDK diminta dikecualikan dalam pembatasan truk saat libur Nataru.</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8725233/bahlil-ungkap-lokasi-pltn-batam-halmahera</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8725185/truk-amdk-diusulkan-dikecualikan-dari-pembatasan-saat-nataru</t>
         </is>
       </c>
     </row>
@@ -2127,22 +2103,22 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Danantara Atur Ketat Perjalanan Dinas Bos-bos BUMN, Ini Isinya</t>
+          <t>Tiga Penyebab Dana Operasional Dapur MBG Nggak Cair</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Mon, 26 Oct 2026 19:45:25 +0700</t>
+          <t>Mon, 26 Oct 2026 21:00:00 +0700</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/07/01/wisma-danantara-indonesia-1751345496674_169.jpeg?w=360&amp;amp;q=90" /&gt; Badan Pengelola Investasi Daya Anagata Nusantara (BPI Danantara) menetapkan aturan ketat perjalanan dinas direksi dan dewan komisaris BUMN.</t>
+          <t xml:space="preserve">&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/06/08/realisasi-anggaran-program-makanan-bergizi-gratis-1780905690949_169.jpeg?w=360&amp;amp;q=90" /&gt; BGN mengungkapkan penyebab dana operasional Satuan Pelayanan Pemenuhan Gizi (SPPG) atau Dapur Makan Bergizi Gratis (MBG) tidak cair pada </t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8725269/danantara-atur-ketat-perjalanan-dinas-bos-bos-bumn-ini-isinya</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8725276/tiga-penyebab-dana-operasional-dapur-mbg-nggak-cair</t>
         </is>
       </c>
     </row>
@@ -2154,22 +2130,22 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>KPK Panggil Lagi Nusron Wahid usai Dua Kali Mangkir</t>
+          <t>KPK Jadwalkan Ulang Pemeriksaan Suami Fadia Arafiq</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Mon, 26 Oct 2026 21:21:18 +0700</t>
+          <t>Tue, 27 Oct 2026 06:36:11 +0700</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Penyidik KPK membutuhkan keterangan Nusron untuk melengkapi proses penyidikan.</t>
+          <t>Ashraff akan diperiksa sebagai saksi dalam pengembangan penyidikan kasus dugaan tindak pidana pencucian uang (TPPU).</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8321772/kpk-panggil-lagi-nusron-wahid-usai-dua-kali-mangkir</t>
+          <t>https://www.liputan6.com/news/read/8321864/kpk-jadwalkan-ulang-pemeriksaan-suami-fadia-arafiq</t>
         </is>
       </c>
     </row>
@@ -2181,22 +2157,22 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Penampakan WN Taiwan, Tersangka Kasus Penyelundupan 1,16 Ton Ketamin</t>
+          <t>Menkomdigi Minta Medsos Terapkan Klasifikasi Usia Pengguna</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Mon, 26 Oct 2026 21:03:03 +0700</t>
+          <t>Tue, 27 Oct 2026 06:12:38 +0700</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Polri menetapkan WN Taiwan YCY sebagai tersangka utama kasus penyelundupan 1,16 ton ketamin.</t>
+          <t>Meutya Hafid minta media sosial (medsos) bedakan pengguna anak dan dewasa demi perlindungan digital.</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8321764/penampakan-wn-taiwan-tersangka-kasus-penyelundupan-116-ton-ketamin</t>
+          <t>https://www.liputan6.com/news/read/8321860/menkomdigi-minta-medsos-terapkan-klasifikasi-usia-pengguna</t>
         </is>
       </c>
     </row>
@@ -2208,22 +2184,22 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Pemotor Tewas Tabrak Pembatas Jalan di Depan PIM 2</t>
+          <t>Praktik Licik di Balik Tunggakan Pajak McLaren Ratusan Juta</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Mon, 26 Oct 2026 20:35:11 +0700</t>
+          <t>Tue, 27 Oct 2026 06:01:23 +0700</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Pengendara Honda Beat berusia 24 tahun meninggal dunia setelah menabrak pembatas jalan di depan PIM 2, Jakarta Selatan. Penyebab kecelakaan masih diselidiki polisi.</t>
+          <t>Yudariansyah dinyatakan menunggak pajak mobil mewah jenis McLaren 570S AT.</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8321754/pemotor-tewas-tabrak-pembatas-jalan-di-depan-pim-2</t>
+          <t>https://www.liputan6.com/news/read/8321818/praktik-licik-di-balik-tunggakan-pajak-mclaren-ratusan-juta</t>
         </is>
       </c>
     </row>
@@ -2235,22 +2211,22 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Menkomdigi: 45 Persen Anak Pernah Jadi Korban Perundungan Siber</t>
+          <t>Ketika Kemenangan di Lapangan, Berujung Hilangnya Nyawa ARK</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Mon, 26 Oct 2026 20:33:25 +0700</t>
+          <t>Tue, 27 Oct 2026 05:00:48 +0700</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Temuan tersebut menunjukkan pentingnya penguatan perlindungan anak di ruang digital.</t>
+          <t>Polres Bogor telah menangkap seorang pelaku berinisial MR dan berkomitmen pada penyelidikan profesional.</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8321752/menkomdigi-45-persen-anak-pernah-jadi-korban-perundungan-siber</t>
+          <t>https://www.liputan6.com/news/read/8321831/ketika-kemenangan-di-lapangan-berujung-hilangnya-nyawa-ark</t>
         </is>
       </c>
     </row>
@@ -2262,22 +2238,22 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Prabowo Belum Setujui Usul Luhut soal Perubahan Definisi Korupsi, Ini Alasannya</t>
+          <t>Puan Soroti Lonjakan Pasien Karhutla, Rumah Sakit Diminta Siaga</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Mon, 26 Oct 2026 20:09:43 +0700</t>
+          <t>Tue, 27 Oct 2026 01:01:05 +0700</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Yusril dan Prabowo berdiskusi mengenai usulan DEN untuk mengubah definisi korupsi dalam UU Tipikor.</t>
+          <t>Data pasien dan kebutuhan rumah sakit harus diperbarui.</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8321744/prabowo-belum-setujui-usul-luhut-soal-perubahan-definisi-korupsi-ini-alasannya</t>
+          <t>https://www.liputan6.com/news/read/8321825/puan-soroti-lonjakan-pasien-karhutla-rumah-sakit-diminta-siaga</t>
         </is>
       </c>
     </row>
@@ -2289,22 +2265,22 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Bukan Sekadar Kurir, Bareskrim Incar Sumber Emas Ilegal</t>
+          <t>Awal Kecurigaan Polisi terhadap Kapal Pembawa 1,16 Ton Ketamin</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Mon, 26 Oct 2026 20:05:00 +0700</t>
+          <t>Tue, 27 Oct 2026 00:01:05 +0700</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Upaya ini melibatkan koordinasi dengan Bea Cukai untuk mengungkap jaringan peredaran.</t>
+          <t>Kecurigaan Polisi terhadap kapal MT Global 168 yang membawa 1,16 ton ketamin bermula dari anomali pergerakan di Laut Andaman.</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8321740/bukan-sekadar-kurir-bareskrim-incar-sumber-emas-ilegal</t>
+          <t>https://www.liputan6.com/news/read/8321806/awal-kecurigaan-polisi-terhadap-kapal-pembawa-116-ton-ketamin</t>
         </is>
       </c>
     </row>
@@ -2316,22 +2292,22 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Titik Api Way Kambas Padam, Lokasi 14 Km dari Pusat Latihan Gajah</t>
+          <t>Maruarar Temui Presiden Prabowo Bahas Target Program Bedah Rumah 2026</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Mon, 26 Oct 2026 19:12:36 +0700</t>
+          <t>Mon, 26 Oct 2026 23:41:00 +0700</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>BPBD Lampung menyatakan titik karhutla yang ditangani di TN Way Kambas telah padam dan berjarak 14 kilometer dari Pusat Latihan Gajah. Pemadaman di titik lain masih berlanjut.</t>
+          <t>Program ini meningkat signifikan menjadi 400.000 unit.</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8321696/titik-api-way-kambas-padam-lokasi-14-km-dari-pusat-latihan-gajah</t>
+          <t>https://www.liputan6.com/news/read/8321817/maruarar-temui-presiden-prabowo-bahas-target-program-bedah-rumah-2026</t>
         </is>
       </c>
     </row>
@@ -2343,22 +2319,22 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Bukan Lagi Bentuk Padat, Ini Modus Baru Penyelundupan Emas Ilegal</t>
+          <t>Letda Jihad Tewas Tertembak di Gudang Senjata, Kopassus Sebut Murni Kelalaian</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Mon, 26 Oct 2026 18:57:38 +0700</t>
+          <t>Mon, 26 Oct 2026 23:12:12 +0700</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Pelaku penyelundupan menggunakan beragam cara untuk menyembunyikan emas.</t>
+          <t>Insiden yang menewaskan Letda Jihad itu terjadi setelah pistol meledak di gudang senjata.</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8321703/bukan-lagi-bentuk-padat-ini-modus-baru-penyelundupan-emas-ilegal</t>
+          <t>https://www.liputan6.com/news/read/8321808/letda-jihad-tewas-tertembak-di-gudang-senjata-kopassus-sebut-murni-kelalaian</t>
         </is>
       </c>
     </row>
@@ -2370,22 +2346,22 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Anggota DPR Tak Setuju Pansel Penyelenggara Pemilu Dibentuk Sekarang, Ini Alasannya</t>
+          <t>Tersangka Pembacokan Suporter Hingga Tewas di Bogor Ditangkap</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Mon, 26 Oct 2026 18:52:36 +0700</t>
+          <t>Mon, 26 Oct 2026 22:39:00 +0700</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Untuk mengatasi persoalan itu, Doli menawarkan dua opsi.</t>
+          <t>Peristiwa tragis ini terjadi setelah pertandingan di Pakansari. Pelaku diancam 15 tahun penjara.</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8321701/anggota-dpr-tak-setuju-pansel-penyelenggara-pemilu-dibentuk-sekarang-ini-alasannya</t>
+          <t>https://www.liputan6.com/news/read/8321800/tersangka-pembacokan-suporter-hingga-tewas-di-bogor-ditangkap</t>
         </is>
       </c>
     </row>
@@ -2397,22 +2373,22 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Doli Kurnia Tanggapi Mekanisme Pemakzulan</t>
+          <t>Kala Walkot Bekasi Rayu Pramono Bantu Bangun Dua Flyover</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Mon, 26 Oct 2026 18:39:35 +0700</t>
+          <t>Mon, 26 Oct 2026 22:00:05 +0700</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Mekanisme pemakzulan wakil presiden sendiri disebutnya telah diatur dalam konstitusi.</t>
+          <t>Flyover tersebut diharapkan dapat mengurangi kemacetan di Kemang Pratama dan Pasar Bantargebang.</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8321689/doli-kurnia-tanggapi-mekanisme-pemakzulan</t>
+          <t>https://www.liputan6.com/news/read/8321756/kala-walkot-bekasi-rayu-pramono-bantu-bangun-dua-flyover</t>
         </is>
       </c>
     </row>
@@ -2424,22 +2400,22 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Target Walkot Bekasi Bangun 2 Halte Usai Disinggung Pramono</t>
+          <t>KPK Panggil Lagi Nusron Wahid usai Dua Kali Mangkir</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Mon, 26 Oct 2026 18:26:06 +0700</t>
+          <t>Mon, 26 Oct 2026 21:21:18 +0700</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Pembangunan dua Halte Transjabodetabek di Bekasi ditargetkan rampung awal Desember 2026.</t>
+          <t>Penyidik KPK membutuhkan keterangan Nusron untuk melengkapi proses penyidikan.</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8321682/target-walkot-bekasi-bangun-2-halte-usai-disinggung-pramono</t>
+          <t>https://www.liputan6.com/news/read/8321772/kpk-panggil-lagi-nusron-wahid-usai-dua-kali-mangkir</t>
         </is>
       </c>
     </row>
@@ -2451,22 +2427,22 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Kemenkum Buat Program bagi 45 Ribu Napi, Dipekerjakan di Proyek Pemerintah</t>
+          <t>Penampakan WN Taiwan, Tersangka Kasus Penyelundupan 1,16 Ton Ketamin</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Mon, 26 Oct 2026 18:22:31 +0700</t>
+          <t>Mon, 26 Oct 2026 21:03:03 +0700</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Kementerian Hukum menyiapkan program rehabilitasi dan reedukasi bagi 30.000–45.000 narapidana yang berpeluang dilibatkan dalam proyek kementerian dan lembaga.</t>
+          <t>Polri menetapkan WN Taiwan YCY sebagai tersangka utama kasus penyelundupan 1,16 ton ketamin.</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8321679/kemenkum-buat-program-bagi-45-ribu-napi-dipekerjakan-di-proyek-pemerintah</t>
+          <t>https://www.liputan6.com/news/read/8321764/penampakan-wn-taiwan-tersangka-kasus-penyelundupan-116-ton-ketamin</t>
         </is>
       </c>
     </row>
@@ -2478,22 +2454,22 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Yusril Menghadap Prabowo, Bahas Perubahan Definisi Korupsi</t>
+          <t>Pemotor Tewas Tabrak Pembatas Jalan di Depan PIM 2</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Mon, 26 Oct 2026 18:09:58 +0700</t>
+          <t>Mon, 26 Oct 2026 20:35:11 +0700</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Menurut Yusril, terdapat sejumlah perbuatan yang merugikan negara, tetapi belum tentu dapat dikategorikan sebagai korupsi.</t>
+          <t>Pengendara Honda Beat berusia 24 tahun meninggal dunia setelah menabrak pembatas jalan di depan PIM 2, Jakarta Selatan. Penyebab kecelakaan masih diselidiki polisi.</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8321672/yusril-menghadap-prabowo-bahas-perubahan-definisi-korupsi</t>
+          <t>https://www.liputan6.com/news/read/8321754/pemotor-tewas-tabrak-pembatas-jalan-di-depan-pim-2</t>
         </is>
       </c>
     </row>
@@ -2505,22 +2481,22 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Bea Cukai Ungkap 127 Kasus Emas Ilegal, Nilainya Tembus Rp 1,02 Triliun</t>
+          <t>Menkomdigi: 45 Persen Anak Pernah Jadi Korban Perundungan Siber</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Mon, 26 Oct 2026 18:04:22 +0700</t>
+          <t>Mon, 26 Oct 2026 20:33:25 +0700</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Bea Cukai mencatat 127 penindakan pengeluaran emas ilegal hingga 26 Oktober 2026, dengan barang bukti 402,31 kg emas senilai Rp1,02 triliun.</t>
+          <t>Temuan tersebut menunjukkan pentingnya penguatan perlindungan anak di ruang digital.</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8321638/bea-cukai-ungkap-127-kasus-emas-ilegal-nilainya-tembus-rp-102-triliun</t>
+          <t>https://www.liputan6.com/news/read/8321752/menkomdigi-45-persen-anak-pernah-jadi-korban-perundungan-siber</t>
         </is>
       </c>
     </row>
@@ -2532,22 +2508,22 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Kampung Ambon Digerebek Empat Kali Dalam Sebulan, 7 Orang Ditangkap</t>
+          <t>Prabowo Belum Setujui Usul Luhut soal Perubahan Definisi Korupsi, Ini Alasannya</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Mon, 26 Oct 2026 18:02:17 +0700</t>
+          <t>Mon, 26 Oct 2026 20:09:43 +0700</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Penggerebekan di Kampung Ambon tersebut menjadi operasi keempat sepanjang Oktober 2026</t>
+          <t>Yusril dan Prabowo berdiskusi mengenai usulan DEN untuk mengubah definisi korupsi dalam UU Tipikor.</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8321662/kampung-ambon-digerebek-empat-kali-dalam-sebulan-7-orang-ditangkap</t>
+          <t>https://www.liputan6.com/news/read/8321744/prabowo-belum-setujui-usul-luhut-soal-perubahan-definisi-korupsi-ini-alasannya</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data pasar & berita - 2026-10-27 14:16 UTC
</commit_message>
<xml_diff>
--- a/data/market_news_latest.xlsx
+++ b/data/market_news_latest.xlsx
@@ -487,20 +487,20 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>5439.2578</v>
+        <v>5266.1299</v>
       </c>
       <c r="F2" t="n">
-        <v>51.353</v>
+        <v>-106.9644</v>
       </c>
       <c r="G2" t="n">
-        <v>0.95</v>
+        <v>-1.99</v>
       </c>
       <c r="H2" t="n">
-        <v>397036500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -521,20 +521,20 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>7676.77</v>
+        <v>7682.2202</v>
       </c>
       <c r="F3" t="n">
-        <v>53.0898</v>
+        <v>5.4502</v>
       </c>
       <c r="G3" t="n">
-        <v>0.7</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="H3" t="n">
-        <v>2759066000</v>
+        <v>426744496</v>
       </c>
     </row>
     <row r="4">
@@ -555,20 +555,20 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>52361.5781</v>
+        <v>52320.3984</v>
       </c>
       <c r="F4" t="n">
-        <v>146.418</v>
+        <v>-41.1797</v>
       </c>
       <c r="G4" t="n">
-        <v>0.28</v>
+        <v>-0.08</v>
       </c>
       <c r="H4" t="n">
-        <v>387915369</v>
+        <v>63545576</v>
       </c>
     </row>
     <row r="5">
@@ -589,20 +589,20 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>26169.3809</v>
+        <v>26231.8379</v>
       </c>
       <c r="F5" t="n">
-        <v>214.041</v>
+        <v>62.457</v>
       </c>
       <c r="G5" t="n">
-        <v>0.82</v>
+        <v>0.24</v>
       </c>
       <c r="H5" t="n">
-        <v>6508626000</v>
+        <v>1900687000</v>
       </c>
     </row>
     <row r="6">
@@ -627,13 +627,13 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>63392.0312</v>
+        <v>63268.3711</v>
       </c>
       <c r="F6" t="n">
-        <v>698.8711</v>
+        <v>1078.7227</v>
       </c>
       <c r="G6" t="n">
-        <v>1.11</v>
+        <v>1.73</v>
       </c>
       <c r="H6" t="n">
         <v>0</v>
@@ -657,20 +657,20 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>23093.3691</v>
+        <v>23041.3203</v>
       </c>
       <c r="F7" t="n">
-        <v>158.6895</v>
+        <v>-170.4902</v>
       </c>
       <c r="G7" t="n">
-        <v>0.6899999999999999</v>
+        <v>-0.73</v>
       </c>
       <c r="H7" t="n">
-        <v>3842800000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -691,14 +691,20 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>3648.301</v>
+      </c>
+      <c r="F8" t="n">
+        <v>-49.219</v>
+      </c>
+      <c r="G8" t="n">
+        <v>-1.33</v>
+      </c>
       <c r="H8" t="n">
-        <v>329758840</v>
+        <v>3124247536</v>
       </c>
     </row>
     <row r="9">
@@ -719,20 +725,20 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>10690.4004</v>
+        <v>10659.6104</v>
       </c>
       <c r="F9" t="n">
-        <v>-34.5996</v>
+        <v>-107.6895</v>
       </c>
       <c r="G9" t="n">
-        <v>-0.32</v>
+        <v>-1</v>
       </c>
       <c r="H9" t="n">
-        <v>697030600</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -753,20 +759,20 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>25181.6504</v>
+        <v>25452.8496</v>
       </c>
       <c r="F10" t="n">
-        <v>-190.0996</v>
+        <v>42.0098</v>
       </c>
       <c r="G10" t="n">
-        <v>-0.75</v>
+        <v>0.17</v>
       </c>
       <c r="H10" t="n">
-        <v>58950600</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -787,20 +793,20 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>5422.1602</v>
+        <v>5397.0298</v>
       </c>
       <c r="F11" t="n">
-        <v>7.02</v>
+        <v>-18.8804</v>
       </c>
       <c r="G11" t="n">
-        <v>0.13</v>
+        <v>-0.35</v>
       </c>
       <c r="H11" t="n">
-        <v>388429200</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -821,17 +827,17 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>18081</v>
+        <v>18025</v>
       </c>
       <c r="F12" t="n">
-        <v>28</v>
+        <v>-56</v>
       </c>
       <c r="G12" t="n">
-        <v>0.16</v>
+        <v>-0.31</v>
       </c>
       <c r="H12" t="n">
         <v>0</v>
@@ -855,17 +861,17 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>102.034</v>
+        <v>102.231</v>
       </c>
       <c r="F13" t="n">
-        <v>0.224</v>
+        <v>0.271</v>
       </c>
       <c r="G13" t="n">
-        <v>0.22</v>
+        <v>0.27</v>
       </c>
       <c r="H13" t="n">
         <v>0</v>
@@ -893,13 +899,13 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>157.592</v>
+        <v>157.866</v>
       </c>
       <c r="F14" t="n">
-        <v>0.762</v>
+        <v>1.036</v>
       </c>
       <c r="G14" t="n">
-        <v>0.49</v>
+        <v>0.66</v>
       </c>
       <c r="H14" t="n">
         <v>0</v>
@@ -923,17 +929,17 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>0.4986</v>
+        <v>0.5003</v>
       </c>
       <c r="F15" t="n">
-        <v>-0.0002</v>
+        <v>0.0017</v>
       </c>
       <c r="G15" t="n">
-        <v>-0.04</v>
+        <v>0.34</v>
       </c>
       <c r="H15" t="n">
         <v>0</v>
@@ -957,17 +963,17 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>0.5301</v>
+        <v>0.5313</v>
       </c>
       <c r="F16" t="n">
-        <v>-0.0014</v>
+        <v>0.0012</v>
       </c>
       <c r="G16" t="n">
-        <v>-0.26</v>
+        <v>0.23</v>
       </c>
       <c r="H16" t="n">
         <v>0</v>
@@ -991,17 +997,17 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>0.4025</v>
+        <v>0.4043</v>
       </c>
       <c r="F17" t="n">
-        <v>-0.0007</v>
+        <v>0.0018</v>
       </c>
       <c r="G17" t="n">
-        <v>-0.17</v>
+        <v>0.45</v>
       </c>
       <c r="H17" t="n">
         <v>0</v>
@@ -1025,14 +1031,20 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>81.535</v>
+      </c>
+      <c r="F18" t="n">
+        <v>-0.145</v>
+      </c>
+      <c r="G18" t="n">
+        <v>-0.18</v>
+      </c>
       <c r="H18" t="n">
-        <v>24127074</v>
+        <v>2686833</v>
       </c>
     </row>
     <row r="19">
@@ -1053,14 +1065,20 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>77.31</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0.14</v>
+      </c>
       <c r="H19" t="n">
-        <v>41292931</v>
+        <v>6718650</v>
       </c>
     </row>
     <row r="20">
@@ -1081,20 +1099,20 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>4026</v>
+        <v>4047.5</v>
       </c>
       <c r="F20" t="n">
-        <v>18.1001</v>
+        <v>9.100099999999999</v>
       </c>
       <c r="G20" t="n">
-        <v>0.45</v>
+        <v>0.23</v>
       </c>
       <c r="H20" t="n">
-        <v>7342</v>
+        <v>87046</v>
       </c>
     </row>
     <row r="21">
@@ -1115,20 +1133,20 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>101.18</v>
+        <v>101.66</v>
       </c>
       <c r="F21" t="n">
-        <v>-2.09</v>
+        <v>-0.1</v>
       </c>
       <c r="G21" t="n">
-        <v>-2.02</v>
+        <v>-0.1</v>
       </c>
       <c r="H21" t="n">
-        <v>4916</v>
+        <v>122466</v>
       </c>
     </row>
     <row r="22">
@@ -1149,20 +1167,20 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="E22" t="n">
-        <v>110.06</v>
+        <v>110.77</v>
       </c>
       <c r="F22" t="n">
-        <v>-6.66</v>
+        <v>-5.04</v>
       </c>
       <c r="G22" t="n">
-        <v>-5.71</v>
+        <v>-4.35</v>
       </c>
       <c r="H22" t="n">
-        <v>698</v>
+        <v>22204</v>
       </c>
     </row>
     <row r="23">
@@ -1183,20 +1201,20 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="E23" t="n">
-        <v>6.572</v>
+        <v>6.609</v>
       </c>
       <c r="F23" t="n">
-        <v>0.096</v>
+        <v>0.101</v>
       </c>
       <c r="G23" t="n">
-        <v>1.48</v>
+        <v>1.55</v>
       </c>
       <c r="H23" t="n">
-        <v>681</v>
+        <v>21334</v>
       </c>
     </row>
     <row r="24">
@@ -1217,14 +1235,20 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr"/>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr"/>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>62.2</v>
+      </c>
+      <c r="F24" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="G24" t="n">
+        <v>0.61</v>
+      </c>
       <c r="H24" t="n">
-        <v>17850668</v>
+        <v>4088987</v>
       </c>
     </row>
     <row r="25">
@@ -1245,17 +1269,17 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="E25" t="n">
-        <v>18.39</v>
+        <v>18.03</v>
       </c>
       <c r="F25" t="n">
-        <v>-1.06</v>
+        <v>-0.36</v>
       </c>
       <c r="G25" t="n">
-        <v>-5.45</v>
+        <v>-1.96</v>
       </c>
       <c r="H25" t="n">
         <v>0</v>
@@ -1283,16 +1307,16 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>80104.82030000001</v>
+        <v>79947.4219</v>
       </c>
       <c r="F26" t="n">
-        <v>80.8125</v>
+        <v>-59.2344</v>
       </c>
       <c r="G26" t="n">
-        <v>0.1</v>
+        <v>-0.07000000000000001</v>
       </c>
       <c r="H26" t="n">
-        <v>27099494400</v>
+        <v>22821048320</v>
       </c>
     </row>
     <row r="27">
@@ -1313,20 +1337,20 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="E27" t="n">
-        <v>1420</v>
+        <v>1325</v>
       </c>
       <c r="F27" t="n">
-        <v>-20</v>
+        <v>-95</v>
       </c>
       <c r="G27" t="n">
-        <v>-1.39</v>
+        <v>-6.69</v>
       </c>
       <c r="H27" t="n">
-        <v>89907100</v>
+        <v>94747900</v>
       </c>
     </row>
     <row r="28">
@@ -1347,20 +1371,20 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="E28" t="n">
-        <v>1445</v>
+        <v>1360</v>
       </c>
       <c r="F28" t="n">
-        <v>115</v>
+        <v>-85</v>
       </c>
       <c r="G28" t="n">
-        <v>8.65</v>
+        <v>-5.88</v>
       </c>
       <c r="H28" t="n">
-        <v>448969700</v>
+        <v>552502700</v>
       </c>
     </row>
     <row r="29">
@@ -1381,20 +1405,20 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="E29" t="n">
-        <v>482</v>
+        <v>456</v>
       </c>
       <c r="F29" t="n">
-        <v>-28</v>
+        <v>-26</v>
       </c>
       <c r="G29" t="n">
-        <v>-5.49</v>
+        <v>-5.39</v>
       </c>
       <c r="H29" t="n">
-        <v>669467800</v>
+        <v>771278300</v>
       </c>
     </row>
     <row r="30">
@@ -1415,20 +1439,20 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="E30" t="n">
-        <v>2320</v>
+        <v>2160</v>
       </c>
       <c r="F30" t="n">
-        <v>-60</v>
+        <v>-160</v>
       </c>
       <c r="G30" t="n">
-        <v>-2.52</v>
+        <v>-6.9</v>
       </c>
       <c r="H30" t="n">
-        <v>14666400</v>
+        <v>9145800</v>
       </c>
     </row>
     <row r="31">
@@ -1449,20 +1473,20 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="E31" t="n">
-        <v>3050</v>
+        <v>2870</v>
       </c>
       <c r="F31" t="n">
-        <v>-40</v>
+        <v>-180</v>
       </c>
       <c r="G31" t="n">
-        <v>-1.29</v>
+        <v>-5.9</v>
       </c>
       <c r="H31" t="n">
-        <v>59198800</v>
+        <v>45857600</v>
       </c>
     </row>
     <row r="32">
@@ -1483,20 +1507,20 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="E32" t="n">
-        <v>426</v>
+        <v>398</v>
       </c>
       <c r="F32" t="n">
-        <v>0</v>
+        <v>-28</v>
       </c>
       <c r="G32" t="n">
-        <v>0</v>
+        <v>-6.57</v>
       </c>
       <c r="H32" t="n">
-        <v>72384700</v>
+        <v>46521100</v>
       </c>
     </row>
     <row r="33">
@@ -1517,20 +1541,20 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="E33" t="n">
-        <v>472</v>
+        <v>452</v>
       </c>
       <c r="F33" t="n">
-        <v>-28</v>
+        <v>-20</v>
       </c>
       <c r="G33" t="n">
-        <v>-5.6</v>
+        <v>-4.24</v>
       </c>
       <c r="H33" t="n">
-        <v>95356100</v>
+        <v>85657700</v>
       </c>
     </row>
     <row r="34">
@@ -1551,20 +1575,20 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="E34" t="n">
-        <v>2490</v>
+        <v>2320</v>
       </c>
       <c r="F34" t="n">
         <v>-170</v>
       </c>
       <c r="G34" t="n">
-        <v>-6.39</v>
+        <v>-6.83</v>
       </c>
       <c r="H34" t="n">
-        <v>9056700</v>
+        <v>9559800</v>
       </c>
     </row>
     <row r="35">
@@ -1585,20 +1609,20 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="E35" t="n">
-        <v>376</v>
+        <v>352</v>
       </c>
       <c r="F35" t="n">
-        <v>-2</v>
+        <v>-24</v>
       </c>
       <c r="G35" t="n">
-        <v>-0.53</v>
+        <v>-6.38</v>
       </c>
       <c r="H35" t="n">
-        <v>715424300</v>
+        <v>479646600</v>
       </c>
     </row>
     <row r="36">
@@ -1619,20 +1643,20 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="E36" t="n">
-        <v>167</v>
+        <v>156</v>
       </c>
       <c r="F36" t="n">
-        <v>-7</v>
+        <v>-11</v>
       </c>
       <c r="G36" t="n">
-        <v>-4.02</v>
+        <v>-6.59</v>
       </c>
       <c r="H36" t="n">
-        <v>184085900</v>
+        <v>47375000</v>
       </c>
     </row>
     <row r="37">
@@ -1653,20 +1677,20 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="E37" t="n">
-        <v>10200</v>
+        <v>10275</v>
       </c>
       <c r="F37" t="n">
-        <v>-100</v>
+        <v>75</v>
       </c>
       <c r="G37" t="n">
-        <v>-0.97</v>
+        <v>0.74</v>
       </c>
       <c r="H37" t="n">
-        <v>13991200</v>
+        <v>20401200</v>
       </c>
     </row>
   </sheetData>
@@ -1725,22 +1749,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Pendaftaran Magang Nasional Batch 3 Dibuka Hari Ini</t>
+          <t>Daerah Kesulitan Bayar Gaji Pegawai, Dua Menteri Prabowo Buka Suara</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Tue, 27 Oct 2026 07:30:58 +0700</t>
+          <t>Tue, 27 Oct 2026 20:31:18 +0700</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2023/05/03/gedung-kemnaker_169.jpeg?w=360&amp;amp;q=90" /&gt; Kementerian Ketenagakerjaan (Kemnaker) resmi membuka pendaftaran Program Magang Nasional (MagangHub) Batch 3 Angkatan II mulai hari ini, Selasa (27/10).</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/10/10/potret-asn-aparatur-sipil-negara-1760067743474_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Dalam Negeri Tito Karnavian dan Menteri Keuangan Suahasil Nazara buka suara soal daerah sulit bayar gaji pegawai.</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8725378/pendaftaran-magang-nasional-batch-3-dibuka-hari-ini</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8726936/daerah-kesulitan-bayar-gaji-pegawai-dua-menteri-prabowo-buka-suara</t>
         </is>
       </c>
     </row>
@@ -1752,22 +1776,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Rencana Baru BEI Sikat Saham Gorengan</t>
+          <t>Produk Lokal Mendunia, Ekspor UMKM Tembus Rp6,6 Triliun Lewat Marketplace</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Tue, 27 Oct 2026 07:00:49 +0700</t>
+          <t>Tue, 27 Oct 2026 20:30:50 +0700</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/07/13/direktur-utama-bei-jeffrey-hendrik-1783928734693_169.jpeg?w=360&amp;amp;q=90" /&gt; Bursa Efek Indonesia (BEI) memperketat pengawasan saham gorengan dengan langsung investigasi emiten yang terindikasi melakukan manipulasi harga.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/27/produk-lokal-mendunia-ekspor-umkm-tembus-rp66-triliun-lewat-marketplace-1793104069684_169.jpeg?w=360&amp;amp;q=90" /&gt; UMKM Indonesia kian menembus pasar global lewat marketplace. Perdagangan digital membuka peluang ekspor produk loka</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/bursa-dan-valas/d-8725377/rencana-baru-bei-sikat-saham-gorengan</t>
+          <t>https://finance.detik.com/foto-bisnis/d-8726838/produk-lokal-mendunia-ekspor-umkm-tembus-rp6-6-triliun-lewat-marketplace</t>
         </is>
       </c>
     </row>
@@ -1779,22 +1803,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Penyelundupan Emas 25 Kg Digagalkan di 5 Bandara, Ini Daftarnya</t>
+          <t>Siap Jadi Penyangga Jagung, BULOG Perkuat Kemitraan Petani-Peternak</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Tue, 27 Oct 2026 06:30:53 +0700</t>
+          <t>Tue, 27 Oct 2026 20:18:55 +0700</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/26/bea-cukai-gagalkan-penyelundupan-emas-2588-kg-ke-luar-negeri-1793002748135_169.jpeg?w=360&amp;amp;q=90" /&gt; Direktorat Jenderal Bea dan Cukai Kementerian Keuangan menggagalkan upaya penyelundupan ekspor emas secara ilegal dengan total</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/27/siap-jadi-penyangga-pasokan-jagung-bulog-perkuat-kemitraan-petani-peternak-1793106864647_169.jpeg?w=360&amp;amp;q=90" /&gt; Perum BULOG siap menjadi penyangga pasokan jagung nasional, memperkuat kemitraan antara petani dan peternak untu</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8725372/penyelundupan-emas-25-kg-digagalkan-di-5-bandara-ini-daftarnya</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8726924/siap-jadi-penyangga-jagung-bulog-perkuat-kemitraan-petani-peternak</t>
         </is>
       </c>
     </row>
@@ -1806,22 +1830,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Dua Penyebab RI Pangkas Ekspor Gas ke Singapura</t>
+          <t>Kinerja Semester I 2026 Positif, JAPFA Perkuat Inovasi dan Efisiensi</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Tue, 27 Oct 2026 05:55:15 +0700</t>
+          <t>Tue, 27 Oct 2026 20:01:48 +0700</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/04/28/menteri-esdm-bahlil-lahadalia-1777385212647_169.jpeg?w=360&amp;amp;q=90" /&gt; Menko Hilirisasi dan Transisi Energi Bahlil Lahadalia menjelaskan alasan pemangkasan ekspor gas ke Singapura.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/27/kinerja-semester-i-2026-positif-japfa-perkuat-inovasi-dan-efisiensi-1793105772143_169.jpeg?w=360&amp;amp;q=90" /&gt; PT Japfa Comfeed Indonesia Tbk mencatat laba Rp 2,68 triliun di Semester I-2026, didukung penjualan bersih Rp 35,36 tri</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8725370/dua-penyebab-ri-pangkas-ekspor-gas-ke-singapura</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8726903/kinerja-semester-i-2026-positif-japfa-perkuat-inovasi-dan-efisiensi</t>
         </is>
       </c>
     </row>
@@ -1833,22 +1857,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Minyak Jelantah 'Disulap' Jadi 11 Juta Liter SAF</t>
+          <t>Suntikan Dana Pusat ke Daerah Tembus Rp 720 Triliun</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Mon, 26 Oct 2026 22:30:00 +0700</t>
+          <t>Tue, 27 Oct 2026 19:58:37 +0700</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/08/21/pt-pertamina-persero-telah-mengembangkan-pertamina-sustainable-aviation-fuel-saf-1755754152640_169.jpeg?w=360&amp;amp;q=90" /&gt; Pertamina memproduksi minyak jelantah menjadi bahan bakar bioavtur atau bahan bakar penerbangan ramah ling</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2015/12/17/00d5a8dc-da3d-483a-bd2e-e78ce08f1d66_169.jpg?w=360&amp;amp;q=90" /&gt; Menteri Keuangan Suahasil Nazara mengungkapkan pemerintah telah menggelontorkan dana Transfer ke Daerah (TKD) hingga Rp 720 triliun.</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8725402/minyak-jelantah-disulap-jadi-11-juta-liter-saf</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8726899/suntikan-dana-pusat-ke-daerah-tembus-rp-720-triliun</t>
         </is>
       </c>
     </row>
@@ -1860,22 +1884,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>UMKM Didorong Perluas Pasar Lewat Rantai Pasok Makan Bergizi Gratis</t>
+          <t>Nikmati Akhir Pekan di WKND Market PIK2, Bisa Belanja hingga Ikut Workshop</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Mon, 26 Oct 2026 22:00:44 +0700</t>
+          <t>Tue, 27 Oct 2026 19:39:02 +0700</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/26/umkm-didorong-perluas-pasar-lewat-rantai-pasok-makan-bergizi-gratis-1792994912262_169.jpeg?w=360&amp;amp;q=90" /&gt; Sebanyak 68 ribu UMKM terhubung dalam rantai pasok program Makan Bergizi Gratis (MBG). Keterlibatan usaha lokal diharap</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/27/wknd-market-vol-6-hadir-di-lands-end-pik2-cek-jadwal-aksesnya-1793104614080_169.jpeg?w=360&amp;amp;q=90" /&gt; WKND Market Vol. 6 di Pantai Indah Kapuk 2 hadir 6-8 November 2026. Nikmati belanja produk lokal, workshop kreatif, olahraga,</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/foto-bisnis/d-8724402/umkm-didorong-perluas-pasar-lewat-rantai-pasok-makan-bergizi-gratis</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8726851/nikmati-akhir-pekan-di-wknd-market-pik2-bisa-belanja-hingga-ikut-workshop</t>
         </is>
       </c>
     </row>
@@ -1887,22 +1911,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Proses Pengadaan KRL Baru Sudah Sejauh Mana? Ini Jawaban Menhub</t>
+          <t>Proyek LNG Abadi Masela Ditargetkan Operasi 2029, Begini Progresnya</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Mon, 26 Oct 2026 22:00:00 +0700</t>
+          <t>Tue, 27 Oct 2026 18:10:02 +0700</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/20/perawatan-jaringan-listrik-krl-1792511606131_169.jpeg?w=360&amp;amp;q=90" /&gt; Kementerian Perhubungan (Kemenhub) buka suara soal progres serta skema pelaksanaan pengadaan 30 rangkaian Kereta Rel Listrik (KRL) baru.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/02/14/kepala-skk-migas-djoko-siswanto-1_169.jpeg?w=360&amp;amp;q=90" /&gt; INPEX Masela Ltd. selesaikan tahap FEED proyek LNG Abadi lebih cepat, proyek gas raksasa itu ditargetkan beroperasi paling cepat 2029.</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/infrastruktur/d-8725393/proses-pengadaan-krl-baru-sudah-sejauh-mana-ini-jawaban-menhub</t>
+          <t>https://finance.detik.com/energi/d-8726688/proyek-lng-abadi-masela-ditargetkan-operasi-2029-begini-progresnya</t>
         </is>
       </c>
     </row>
@@ -1914,22 +1938,22 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Jurus Pemerintah Jaga Pasokan dan Harga Pangan Jelang Nataru</t>
+          <t>Bansos Digital Meluncur 10 November, 100 Juta Warga Bakal Terdaftar</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Mon, 26 Oct 2026 21:36:17 +0700</t>
+          <t>Tue, 27 Oct 2026 17:50:31 +0700</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/26/rapat-koordinasi-terbatas-rakortas-bidang-pangan-yang-dipimpin-menteri-koordinator-bidang-pangan-ri-menko-pangan-zulkifli-hasa-1793025343365.jpeg?w=360&amp;amp;q=90" /&gt; Pemerintah antisipasi stabilitas pangan menjelang Nataru dengan </t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/27/pertemuan-ketua-den-dengan-menko-kumham-imipas-1793090271348_169.jpeg?w=360&amp;amp;q=90" /&gt; Dan kita harap nanti waktu roll out oleh Presiden tanggal 10 November itu sudah lebih 100 juta orang, kata Luhut.</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8725387/jurus-pemerintah-jaga-pasokan-dan-harga-pangan-jelang-nataru</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8726657/bansos-digital-meluncur-10-november-100-juta-warga-bakal-terdaftar</t>
         </is>
       </c>
     </row>
@@ -1941,22 +1965,22 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>3.030 Penerbangan Terdampak Karhutla Sejak Agustus, 1.700 Rute Dibatalkan</t>
+          <t>Waskita Karya Lanjutkan Pemulihan Pascabencana di Aceh, Progres Hampir 70%</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Mon, 26 Oct 2026 21:30:00 +0700</t>
+          <t>Tue, 27 Oct 2026 17:41:12 +0700</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2023/10/05/ngeri-kabut-asap-bikin-jarak-pandang-di-bandara-palangka-raya-terbatas-1_169.jpeg?w=360&amp;amp;q=90" /&gt; Kemenhub mencatat sebanyak 3.030 penerbangan terdampak oleh kabut asap akibat kebakaran hutan dan lahan (karhutla) sejak 14 Agus</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/27/waskita-karya-lanjutkan-pemulihan-pascabencana-di-aceh-progres-hampir-70-1793097636359.jpeg?w=360&amp;amp;q=90" /&gt; Waskita Karya terus berupaya memulihkan Aceh pascabencana dengan proyek penanganan infrastruktur dan penyediaan air be</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8725381/3-030-penerbangan-terdampak-karhutla-sejak-agustus-1-700-rute-dibatalkan</t>
+          <t>https://finance.detik.com/infrastruktur/d-8726642/waskita-karya-lanjutkan-pemulihan-pascabencana-di-aceh-progres-hampir-70</t>
         </is>
       </c>
     </row>
@@ -1968,22 +1992,22 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Pertamina Dukung Perpres 107 Perkuat Ketahanan Energi Nasional</t>
+          <t>BI Pangkas Kewajiban GWM, BCA Bidik Target Kredit Double Digit</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Mon, 26 Oct 2026 21:27:35 +0700</t>
+          <t>Tue, 27 Oct 2026 17:40:20 +0700</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/26/pertamina-siap-jalankan-perpres-107-untuk-perkuat-ketahanan-energi-nasional-1793024805115.jpeg?w=360&amp;amp;q=90" /&gt; Pertamina mendukung Perpres 107/2026 untuk memperkuat pengadaan energi nasional. Komitmen menjaga ketersediaan BBM </t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2016/04/28/4f6b9d13-dc5d-4f7b-944c-7dd26d554e82_169.jpg?w=360&amp;amp;q=90" /&gt; PT Bank Central Asia (BBCA) menyambut baik pelonggaran GWM oleh Bank Indonesia, yang mendukung pertumbuhan kredit BCA.</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8725384/pertamina-dukung-perpres-107-perkuat-ketahanan-energi-nasional</t>
+          <t>https://finance.detik.com/moneter/d-8726637/bi-pangkas-kewajiban-gwm-bca-bidik-target-kredit-double-digit</t>
         </is>
       </c>
     </row>
@@ -1995,22 +2019,22 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Harga Tiket Pesawat Bakal Turun 11-13% Saat Libur Natal &amp;amp; Tahun Baru</t>
+          <t>Stabilitas Perbankan di Tengah Gejolak Pasar Modal</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Mon, 26 Oct 2026 21:16:28 +0700</t>
+          <t>Tue, 27 Oct 2026 17:29:53 +0700</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2023/11/11/ilustrasi-harga-tiket-pesawat_169.png?w=360&amp;amp;q=90" /&gt; Kementerian Perhubungan (Kemenhub) menargetkan harga tiket pesawat dapat turun 11-13% selama periode Natal dan Tahun Baru (Nataru) 2026/2027.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/19/ihsg-dibuka-anjlok-431-bei-berlakukan-arb-7-1792382663806_169.jpeg?w=360&amp;amp;q=90" /&gt; OJK, bersama pemerintah dan BEI, memperkuat pasar modal Indonesia dengan reformasi untuk meningkatkan dan menjaga kepercayaan investor global.</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8725373/harga-tiket-pesawat-bakal-turun-11-13-saat-libur-natal-tahun-baru</t>
+          <t>https://finance.detik.com/moneter/d-8726613/stabilitas-perbankan-di-tengah-gejolak-pasar-modal</t>
         </is>
       </c>
     </row>
@@ -2022,22 +2046,22 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Impor KRL Bekas Jepang Tunggu Restu Kemenhub</t>
+          <t>blu by BCA Digital Ajak Anak Muda Eksplorasi Hal Baru Lewat #EksplorSemaumu</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Mon, 26 Oct 2026 21:08:16 +0700</t>
+          <t>Tue, 27 Oct 2026 17:22:45 +0700</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2014/06/27/7792aea3-ac73-4740-974a-e71dca1fea91_169.jpg?w=360&amp;amp;q=90" /&gt; Kementerian Perhubungan (Kemenhub) mempelajari proposal pengadaan Kereta Rel Listrik (KRL) bekas dari Jepang.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/27/blu-by-bca-digital-ajak-anak-muda-eksplorasi-hal-baru-lewat-eksplorsemaumu-1793096408008_169.png?w=360&amp;amp;q=90" /&gt; Blu by BCA Digital mengajak anak muda untuk #EksplorSemaumu, merayakan pengalaman unik dengan fitur perbankan dig</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/infrastruktur/d-8725367/impor-krl-bekas-jepang-tunggu-restu-kemenhub</t>
+          <t>https://finance.detik.com/moneter/d-8726594/blu-by-bca-digital-ajak-anak-muda-eksplorasi-hal-baru-lewat-eksplorsemaumu</t>
         </is>
       </c>
     </row>
@@ -2049,22 +2073,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Karya Siswa Disabilitas di Bali Tembus Toko Oleh-Oleh, Harga Mulai Rp 10 Ribu</t>
+          <t>RI Bakal Dapat Kiriman 30 Juta Barel Minyak dari UEA Bebas Ongkir</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Mon, 26 Oct 2026 21:00:41 +0700</t>
+          <t>Tue, 27 Oct 2026 17:16:56 +0700</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/26/karya-siswa-disabilitas-di-bali-tembus-toko-oleh-oleh-harga-mulai-rp-10-ribu-1792999583884_169.jpeg?w=360&amp;amp;q=90" /&gt; Siswa tunarungu di SLB Negeri 1 Tabanan, Bali, membuat kerajinan tangan. Produk mereka dijual di toko oleh-ole</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2021/04/16/infografis-indonesia-masih-impor-bbm-1_169.jpeg?w=360&amp;amp;q=90" /&gt; Pemerintah UEA akan mengirim 30 juta barel minyak ke Indonesia tanpa biaya modal kerja.</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/foto-bisnis/d-8724549/karya-siswa-disabilitas-di-bali-tembus-toko-oleh-oleh-harga-mulai-rp-10-ribu</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8726589/ri-bakal-dapat-kiriman-30-juta-barel-minyak-dari-uea-bebas-ongkir</t>
         </is>
       </c>
     </row>
@@ -2076,22 +2100,22 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Truk AMDK Diusulkan Dikecualikan dari Pembatasan Saat Nataru</t>
+          <t>Jamin Kredit UMKM-K Rp 271 T, Jamkrindo Raup Laba Rp 1,1 T per September 2026</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Mon, 26 Oct 2026 21:00:03 +0700</t>
+          <t>Tue, 27 Oct 2026 17:05:37 +0700</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2023/06/23/pangsa-pasar-air-minum-kemasan-lokal-meningkat-2_169.jpeg?w=360&amp;amp;q=90" /&gt; Distribusi AMDK diminta dikecualikan dalam pembatasan truk saat libur Nataru.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2023/04/27/jamkrindo_169.jpeg?w=360&amp;amp;q=90" /&gt; Jamkrindo laporkan penjaminan Rp 271,20 triliun hingga September 2026, dukung 2,97 juta UMKM dan 9,46 juta tenaga kerja. Laba sebelum pajak Rp 1,1 triliun.</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8725185/truk-amdk-diusulkan-dikecualikan-dari-pembatasan-saat-nataru</t>
+          <t>https://finance.detik.com/moneter/d-8726555/jamin-kredit-umkm-k-rp-271-t-jamkrindo-raup-laba-rp-1-1-t-per-september-2026</t>
         </is>
       </c>
     </row>
@@ -2103,22 +2127,22 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Tiga Penyebab Dana Operasional Dapur MBG Nggak Cair</t>
+          <t>Progres Tol Semarang-Demak Seksi 1 Capai 79,42 Persen</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Mon, 26 Oct 2026 21:00:00 +0700</t>
+          <t>Tue, 27 Oct 2026 17:02:44 +0700</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/06/08/realisasi-anggaran-program-makanan-bergizi-gratis-1780905690949_169.jpeg?w=360&amp;amp;q=90" /&gt; BGN mengungkapkan penyebab dana operasional Satuan Pelayanan Pemenuhan Gizi (SPPG) atau Dapur Makan Bergizi Gratis (MBG) tidak cair pada </t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/27/progres-pembangunan-jalan-tol-semarang-demak-seksi-1-1793081892794_169.jpeg?w=360&amp;amp;q=90" /&gt; Progres pembangunan Tol Semarang-Demak Seksi 1 mencapai 79,42 persen hingga 22 Oktober 2026 dan ditargetkan rampung pada akhir 2027.</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8725276/tiga-penyebab-dana-operasional-dapur-mbg-nggak-cair</t>
+          <t>https://finance.detik.com/foto-bisnis/d-8726052/progres-tol-semarang-demak-seksi-1-capai-79-42-persen</t>
         </is>
       </c>
     </row>
@@ -2130,22 +2154,22 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>KPK Jadwalkan Ulang Pemeriksaan Suami Fadia Arafiq</t>
+          <t>Wajah Baru SMPN 91 Jakarta, Ada Lift dan Panel Surya</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Tue, 27 Oct 2026 06:36:11 +0700</t>
+          <t>Tue, 27 Oct 2026 20:54:18 +0700</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Ashraff akan diperiksa sebagai saksi dalam pengembangan penyidikan kasus dugaan tindak pidana pencucian uang (TPPU).</t>
+          <t>Revitalisasi SMPN 91 Jakarta menambah ruang kelas dari delapan menjadi 21, dilengkapi lift, panel surya, dan papan interaktif digital.</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8321864/kpk-jadwalkan-ulang-pemeriksaan-suami-fadia-arafiq</t>
+          <t>https://www.liputan6.com/news/read/8322618/wajah-baru-smpn-91-jakarta-ada-lift-dan-panel-surya</t>
         </is>
       </c>
     </row>
@@ -2157,22 +2181,22 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Menkomdigi Minta Medsos Terapkan Klasifikasi Usia Pengguna</t>
+          <t>Bahagianya Siswa Belajar di Gedung Baru SMPN 91, Makin Betah di Sekolah</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Tue, 27 Oct 2026 06:12:38 +0700</t>
+          <t>Tue, 27 Oct 2026 20:57:14 +0700</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Meutya Hafid minta media sosial (medsos) bedakan pengguna anak dan dewasa demi perlindungan digital.</t>
+          <t>Di SMPN 91 Jakarta, revitalisasi tak hanya mengubah wajah bangunan.</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8321860/menkomdigi-minta-medsos-terapkan-klasifikasi-usia-pengguna</t>
+          <t>https://www.liputan6.com/news/read/8322627/bahagianya-siswa-belajar-di-gedung-baru-smpn-91-makin-betah-di-sekolah</t>
         </is>
       </c>
     </row>
@@ -2184,22 +2208,22 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Praktik Licik di Balik Tunggakan Pajak McLaren Ratusan Juta</t>
+          <t>KPK Buka Suara soal Kabar Panggil Nusron Wahid Besok</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Tue, 27 Oct 2026 06:01:23 +0700</t>
+          <t>Tue, 27 Oct 2026 21:00:27 +0700</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Yudariansyah dinyatakan menunggak pajak mobil mewah jenis McLaren 570S AT.</t>
+          <t>Nusron Wahid sebelumnya telah dua kali mangkir dari panggilan KPK</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8321818/praktik-licik-di-balik-tunggakan-pajak-mclaren-ratusan-juta</t>
+          <t>https://www.liputan6.com/news/read/8322629/kpk-buka-suara-soal-kabar-panggil-nusron-wahid-besok</t>
         </is>
       </c>
     </row>
@@ -2211,22 +2235,22 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Ketika Kemenangan di Lapangan, Berujung Hilangnya Nyawa ARK</t>
+          <t>KSPSI Ingatkan Massa Demo 28 Oktober Tak Anarkis dan Sebar Hoaks</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Tue, 27 Oct 2026 05:00:48 +0700</t>
+          <t>Tue, 27 Oct 2026 20:19:09 +0700</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Polres Bogor telah menangkap seorang pelaku berinisial MR dan berkomitmen pada penyelidikan profesional.</t>
+          <t>KSPSI mengajak masyarakat mengutamakan dialog dan musyawarah serta tidak menyebarkan informasi yang dapat memperkeruh suasana.</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8321831/ketika-kemenangan-di-lapangan-berujung-hilangnya-nyawa-ark</t>
+          <t>https://www.liputan6.com/news/read/8322599/kspsi-ingatkan-massa-demo-28-oktober-tak-anarkis-dan-sebar-hoaks</t>
         </is>
       </c>
     </row>
@@ -2238,22 +2262,22 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Puan Soroti Lonjakan Pasien Karhutla, Rumah Sakit Diminta Siaga</t>
+          <t>Sestama BNPB Dicecar KPK Soal Pengadaan Dana Bencana</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Tue, 27 Oct 2026 01:01:05 +0700</t>
+          <t>Tue, 27 Oct 2026 19:44:22 +0700</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Data pasien dan kebutuhan rumah sakit harus diperbarui.</t>
+          <t>Penyidik KPK mendalami dua persoalan dalam pemeriksaan tersebut.</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8321825/puan-soroti-lonjakan-pasien-karhutla-rumah-sakit-diminta-siaga</t>
+          <t>https://www.liputan6.com/news/read/8322572/sestama-bnpb-dicecar-kpk-soal-pengadaan-dana-bencana</t>
         </is>
       </c>
     </row>
@@ -2265,22 +2289,22 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Awal Kecurigaan Polisi terhadap Kapal Pembawa 1,16 Ton Ketamin</t>
+          <t>Demo 28 Oktober, Polisi Imbau Jaga Fasilitas Umum</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Tue, 27 Oct 2026 00:01:05 +0700</t>
+          <t>Tue, 27 Oct 2026 19:36:44 +0700</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Kecurigaan Polisi terhadap kapal MT Global 168 yang membawa 1,16 ton ketamin bermula dari anomali pergerakan di Laut Andaman.</t>
+          <t>Sejumlah aliansi mahasiswa akan menggelar aksi unjuk rasa di Jakarta, Rabu, 28 Oktober 2026.</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8321806/awal-kecurigaan-polisi-terhadap-kapal-pembawa-116-ton-ketamin</t>
+          <t>https://www.liputan6.com/news/read/8322565/demo-28-oktober-polisi-imbau-jaga-fasilitas-umum</t>
         </is>
       </c>
     </row>
@@ -2292,22 +2316,22 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Maruarar Temui Presiden Prabowo Bahas Target Program Bedah Rumah 2026</t>
+          <t>Penyebab KRL Berasap hingga Terdengar Ledakan di Stasiun Jakarta Kota</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Mon, 26 Oct 2026 23:41:00 +0700</t>
+          <t>Tue, 27 Oct 2026 19:37:10 +0700</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Program ini meningkat signifikan menjadi 400.000 unit.</t>
+          <t>KAI Commuter mengalihkan penumpang Commuter Line relasi Jakarta Kota-Bogor ke rangkaian lain imbas KRL berasap dan mengeluarkan percikan api.</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8321817/maruarar-temui-presiden-prabowo-bahas-target-program-bedah-rumah-2026</t>
+          <t>https://www.liputan6.com/news/read/8322567/penyebab-krl-berasap-hingga-terdengar-ledakan-di-stasiun-jakarta-kota</t>
         </is>
       </c>
     </row>
@@ -2319,22 +2343,22 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Letda Jihad Tewas Tertembak di Gudang Senjata, Kopassus Sebut Murni Kelalaian</t>
+          <t>Ada Ledakan dan Percikan Api di KRL Jakarta-Bogor, KAI Buka Suara</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Mon, 26 Oct 2026 23:12:12 +0700</t>
+          <t>Tue, 27 Oct 2026 19:27:47 +0700</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Insiden yang menewaskan Letda Jihad itu terjadi setelah pistol meledak di gudang senjata.</t>
+          <t>Kereta Commuter Line Jakarta–Bogor mengalami gangguan usai terdengar ledakan dan percikan api.</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8321808/letda-jihad-tewas-tertembak-di-gudang-senjata-kopassus-sebut-murni-kelalaian</t>
+          <t>https://www.liputan6.com/news/read/8322561/ada-ledakan-dan-percikan-api-di-krl-jakarta-bogor-kai-buka-suara</t>
         </is>
       </c>
     </row>
@@ -2346,22 +2370,22 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Tersangka Pembacokan Suporter Hingga Tewas di Bogor Ditangkap</t>
+          <t>Polri Jamin Penanganan Medis Ojol Korban Kecelakaan di Blok M</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Mon, 26 Oct 2026 22:39:00 +0700</t>
+          <t>Tue, 27 Oct 2026 19:27:25 +0700</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Peristiwa tragis ini terjadi setelah pertandingan di Pakansari. Pelaku diancam 15 tahun penjara.</t>
+          <t>Polri memberikan pendampingan kepada pengemudi ojol korban kecelakaan di Blok M.</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8321800/tersangka-pembacokan-suporter-hingga-tewas-di-bogor-ditangkap</t>
+          <t>https://www.liputan6.com/news/read/8322560/polri-jamin-penanganan-medis-ojol-korban-kecelakaan-di-blok-m</t>
         </is>
       </c>
     </row>
@@ -2373,22 +2397,22 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Kala Walkot Bekasi Rayu Pramono Bantu Bangun Dua Flyover</t>
+          <t>BRIN Punya 4 Kandidat Vaksin Malaria, Prabowo Minta Riset Dipercepat</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Mon, 26 Oct 2026 22:00:05 +0700</t>
+          <t>Tue, 27 Oct 2026 19:15:44 +0700</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Flyover tersebut diharapkan dapat mengurangi kemacetan di Kemang Pratama dan Pasar Bantargebang.</t>
+          <t>Prabowo ingin pengembangan vaksin malaria tersebut dapat selesai tiga tahun lebih cepat dari target awal.</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8321756/kala-walkot-bekasi-rayu-pramono-bantu-bangun-dua-flyover</t>
+          <t>https://www.liputan6.com/news/read/8322550/brin-punya-4-kandidat-vaksin-malaria-prabowo-minta-riset-dipercepat</t>
         </is>
       </c>
     </row>
@@ -2400,22 +2424,22 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>KPK Panggil Lagi Nusron Wahid usai Dua Kali Mangkir</t>
+          <t>Komite Sadar Gelar Aksi di Bundaran HI Besok, Ini Lima Tuntutannya</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Mon, 26 Oct 2026 21:21:18 +0700</t>
+          <t>Tue, 27 Oct 2026 19:05:00 +0700</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Penyidik KPK membutuhkan keterangan Nusron untuk melengkapi proses penyidikan.</t>
+          <t>Mereka mendesak pemerintah memenuhi lima tuntutan utama, termasuk penuntasan tata kelola lahan dan kebebasan bersuara.</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8321772/kpk-panggil-lagi-nusron-wahid-usai-dua-kali-mangkir</t>
+          <t>https://www.liputan6.com/news/read/8322542/komite-sadar-gelar-aksi-di-bundaran-hi-besok-ini-lima-tuntutannya</t>
         </is>
       </c>
     </row>
@@ -2427,22 +2451,22 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Penampakan WN Taiwan, Tersangka Kasus Penyelundupan 1,16 Ton Ketamin</t>
+          <t>Jelang Sumpah Pemuda, Masyarakat Diminta Waspadai Provokasi</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Mon, 26 Oct 2026 21:03:03 +0700</t>
+          <t>Tue, 27 Oct 2026 18:51:48 +0700</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Polri menetapkan WN Taiwan YCY sebagai tersangka utama kasus penyelundupan 1,16 ton ketamin.</t>
+          <t>Menjelang Sumpah Pemuda, Polri mengajak masyarakat memperkuat kolaborasi menjaga kamtibmas</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8321764/penampakan-wn-taiwan-tersangka-kasus-penyelundupan-116-ton-ketamin</t>
+          <t>https://www.liputan6.com/news/read/8322532/jelang-sumpah-pemuda-masyarakat-diminta-waspadai-provokasi</t>
         </is>
       </c>
     </row>
@@ -2454,22 +2478,22 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Pemotor Tewas Tabrak Pembatas Jalan di Depan PIM 2</t>
+          <t>Ada Demo Sumpah Pemuda Besok, TNI-Polri Kawal Jakarta</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Mon, 26 Oct 2026 20:35:11 +0700</t>
+          <t>Tue, 27 Oct 2026 18:48:40 +0700</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Pengendara Honda Beat berusia 24 tahun meninggal dunia setelah menabrak pembatas jalan di depan PIM 2, Jakarta Selatan. Penyebab kecelakaan masih diselidiki polisi.</t>
+          <t>Petugas akan ditempatkan di sejumlah titik kegiatan untuk mengawal peserta aksi</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8321754/pemotor-tewas-tabrak-pembatas-jalan-di-depan-pim-2</t>
+          <t>https://www.liputan6.com/news/read/8322530/ada-demo-sumpah-pemuda-besok-tni-polri-kawal-jakarta</t>
         </is>
       </c>
     </row>
@@ -2481,22 +2505,22 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Menkomdigi: 45 Persen Anak Pernah Jadi Korban Perundungan Siber</t>
+          <t>Kecelakaan Beruntun 4 Kendaraan di Tol Akses Tanjung Priok</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Mon, 26 Oct 2026 20:33:25 +0700</t>
+          <t>Tue, 27 Oct 2026 18:24:32 +0700</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Temuan tersebut menunjukkan pentingnya penguatan perlindungan anak di ruang digital.</t>
+          <t>Kecelakaan tersebut menyebabkan satu orang mengalami luka.</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8321752/menkomdigi-45-persen-anak-pernah-jadi-korban-perundungan-siber</t>
+          <t>https://www.liputan6.com/news/read/8322513/kecelakaan-beruntun-4-kendaraan-di-tol-akses-tanjung-priok</t>
         </is>
       </c>
     </row>
@@ -2508,22 +2532,22 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Prabowo Belum Setujui Usul Luhut soal Perubahan Definisi Korupsi, Ini Alasannya</t>
+          <t>Polri Jamin Kebebasan Berpendapat, Masyarakat Diimbau Tertib</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Mon, 26 Oct 2026 20:09:43 +0700</t>
+          <t>Tue, 27 Oct 2026 18:05:49 +0700</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Yusril dan Prabowo berdiskusi mengenai usulan DEN untuk mengubah definisi korupsi dalam UU Tipikor.</t>
+          <t>Polri mengajak masyarakat menjaga ruang demokrasi dan menghormati perbedaan pendapat.</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8321744/prabowo-belum-setujui-usul-luhut-soal-perubahan-definisi-korupsi-ini-alasannya</t>
+          <t>https://www.liputan6.com/news/read/8322499/polri-jamin-kebebasan-berpendapat-masyarakat-diimbau-tertib</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data pasar & berita - 2026-10-28 00:47 UTC
</commit_message>
<xml_diff>
--- a/data/market_news_latest.xlsx
+++ b/data/market_news_latest.xlsx
@@ -487,20 +487,20 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>5266.1299</v>
+        <v>5373.0942</v>
       </c>
       <c r="F2" t="n">
-        <v>-106.9644</v>
+        <v>-66.1636</v>
       </c>
       <c r="G2" t="n">
-        <v>-1.99</v>
+        <v>-1.22</v>
       </c>
       <c r="H2" t="n">
-        <v>0</v>
+        <v>280027100</v>
       </c>
     </row>
     <row r="3">
@@ -525,16 +525,16 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>7682.2202</v>
+        <v>7722.6001</v>
       </c>
       <c r="F3" t="n">
-        <v>5.4502</v>
+        <v>45.8301</v>
       </c>
       <c r="G3" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.6</v>
       </c>
       <c r="H3" t="n">
-        <v>426744496</v>
+        <v>2810939000</v>
       </c>
     </row>
     <row r="4">
@@ -559,16 +559,16 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>52320.3984</v>
+        <v>52377.5703</v>
       </c>
       <c r="F4" t="n">
-        <v>-41.1797</v>
+        <v>15.9922</v>
       </c>
       <c r="G4" t="n">
-        <v>-0.08</v>
+        <v>0.03</v>
       </c>
       <c r="H4" t="n">
-        <v>63545576</v>
+        <v>401210066</v>
       </c>
     </row>
     <row r="5">
@@ -593,16 +593,16 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>26231.8379</v>
+        <v>26477.8105</v>
       </c>
       <c r="F5" t="n">
-        <v>62.457</v>
+        <v>308.4297</v>
       </c>
       <c r="G5" t="n">
-        <v>0.24</v>
+        <v>1.18</v>
       </c>
       <c r="H5" t="n">
-        <v>1900687000</v>
+        <v>7116359000</v>
       </c>
     </row>
     <row r="6">
@@ -623,17 +623,17 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>63268.3711</v>
+        <v>63918.3594</v>
       </c>
       <c r="F6" t="n">
-        <v>1078.7227</v>
+        <v>1728.7109</v>
       </c>
       <c r="G6" t="n">
-        <v>1.73</v>
+        <v>2.78</v>
       </c>
       <c r="H6" t="n">
         <v>0</v>
@@ -657,20 +657,20 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>23041.3203</v>
+        <v>23211.8105</v>
       </c>
       <c r="F7" t="n">
-        <v>-170.4902</v>
+        <v>118.4414</v>
       </c>
       <c r="G7" t="n">
-        <v>-0.73</v>
+        <v>0.51</v>
       </c>
       <c r="H7" t="n">
-        <v>0</v>
+        <v>2494900000</v>
       </c>
     </row>
     <row r="8">
@@ -694,15 +694,9 @@
           <t>2026-10-27</t>
         </is>
       </c>
-      <c r="E8" t="n">
-        <v>3648.301</v>
-      </c>
-      <c r="F8" t="n">
-        <v>-49.219</v>
-      </c>
-      <c r="G8" t="n">
-        <v>-1.33</v>
-      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
       <c r="H8" t="n">
         <v>3124247536</v>
       </c>
@@ -725,20 +719,20 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>10659.6104</v>
+        <v>10767.2998</v>
       </c>
       <c r="F9" t="n">
-        <v>-107.6895</v>
+        <v>76.8994</v>
       </c>
       <c r="G9" t="n">
-        <v>-1</v>
+        <v>0.72</v>
       </c>
       <c r="H9" t="n">
-        <v>0</v>
+        <v>562995300</v>
       </c>
     </row>
     <row r="10">
@@ -759,20 +753,20 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>25452.8496</v>
+        <v>25410.8398</v>
       </c>
       <c r="F10" t="n">
-        <v>42.0098</v>
+        <v>229.1895</v>
       </c>
       <c r="G10" t="n">
-        <v>0.17</v>
+        <v>0.91</v>
       </c>
       <c r="H10" t="n">
-        <v>0</v>
+        <v>47950100</v>
       </c>
     </row>
     <row r="11">
@@ -793,20 +787,20 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>5397.0298</v>
+        <v>5415.9102</v>
       </c>
       <c r="F11" t="n">
-        <v>-18.8804</v>
+        <v>-6.25</v>
       </c>
       <c r="G11" t="n">
-        <v>-0.35</v>
+        <v>-0.12</v>
       </c>
       <c r="H11" t="n">
-        <v>0</v>
+        <v>264516700</v>
       </c>
     </row>
     <row r="12">
@@ -831,13 +825,13 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>18025</v>
+        <v>18144</v>
       </c>
       <c r="F12" t="n">
-        <v>-56</v>
+        <v>63</v>
       </c>
       <c r="G12" t="n">
-        <v>-0.31</v>
+        <v>0.35</v>
       </c>
       <c r="H12" t="n">
         <v>0</v>
@@ -865,13 +859,13 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>102.231</v>
+        <v>102.337</v>
       </c>
       <c r="F13" t="n">
-        <v>0.271</v>
+        <v>0.377</v>
       </c>
       <c r="G13" t="n">
-        <v>0.27</v>
+        <v>0.37</v>
       </c>
       <c r="H13" t="n">
         <v>0</v>
@@ -895,17 +889,17 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>157.866</v>
+        <v>157.857</v>
       </c>
       <c r="F14" t="n">
-        <v>1.036</v>
+        <v>0.329</v>
       </c>
       <c r="G14" t="n">
-        <v>0.66</v>
+        <v>0.21</v>
       </c>
       <c r="H14" t="n">
         <v>0</v>
@@ -933,13 +927,13 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>0.5003</v>
+        <v>0.4993</v>
       </c>
       <c r="F15" t="n">
-        <v>0.0017</v>
+        <v>0.0007</v>
       </c>
       <c r="G15" t="n">
-        <v>0.34</v>
+        <v>0.14</v>
       </c>
       <c r="H15" t="n">
         <v>0</v>
@@ -967,13 +961,13 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>0.5313</v>
+        <v>0.5305</v>
       </c>
       <c r="F16" t="n">
-        <v>0.0012</v>
+        <v>0.0004</v>
       </c>
       <c r="G16" t="n">
-        <v>0.23</v>
+        <v>0.08</v>
       </c>
       <c r="H16" t="n">
         <v>0</v>
@@ -1001,13 +995,13 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>0.4043</v>
+        <v>0.404</v>
       </c>
       <c r="F17" t="n">
-        <v>0.0018</v>
+        <v>0.0015</v>
       </c>
       <c r="G17" t="n">
-        <v>0.45</v>
+        <v>0.37</v>
       </c>
       <c r="H17" t="n">
         <v>0</v>
@@ -1034,17 +1028,11 @@
           <t>2026-10-27</t>
         </is>
       </c>
-      <c r="E18" t="n">
-        <v>81.535</v>
-      </c>
-      <c r="F18" t="n">
-        <v>-0.145</v>
-      </c>
-      <c r="G18" t="n">
-        <v>-0.18</v>
-      </c>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
       <c r="H18" t="n">
-        <v>2686833</v>
+        <v>19529180</v>
       </c>
     </row>
     <row r="19">
@@ -1068,17 +1056,11 @@
           <t>2026-10-27</t>
         </is>
       </c>
-      <c r="E19" t="n">
-        <v>77.31</v>
-      </c>
-      <c r="F19" t="n">
-        <v>0.11</v>
-      </c>
-      <c r="G19" t="n">
-        <v>0.14</v>
-      </c>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr"/>
       <c r="H19" t="n">
-        <v>6718650</v>
+        <v>54988363</v>
       </c>
     </row>
     <row r="20">
@@ -1103,16 +1085,16 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>4047.5</v>
+        <v>4075.2</v>
       </c>
       <c r="F20" t="n">
-        <v>9.100099999999999</v>
+        <v>36.8</v>
       </c>
       <c r="G20" t="n">
-        <v>0.23</v>
+        <v>0.91</v>
       </c>
       <c r="H20" t="n">
-        <v>87046</v>
+        <v>6054</v>
       </c>
     </row>
     <row r="21">
@@ -1137,16 +1119,16 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>101.66</v>
+        <v>100.5</v>
       </c>
       <c r="F21" t="n">
-        <v>-0.1</v>
+        <v>-1.26</v>
       </c>
       <c r="G21" t="n">
-        <v>-0.1</v>
+        <v>-1.24</v>
       </c>
       <c r="H21" t="n">
-        <v>122466</v>
+        <v>5845</v>
       </c>
     </row>
     <row r="22">
@@ -1171,16 +1153,16 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>110.77</v>
+        <v>109.87</v>
       </c>
       <c r="F22" t="n">
-        <v>-5.04</v>
+        <v>-5.94</v>
       </c>
       <c r="G22" t="n">
-        <v>-4.35</v>
+        <v>-5.13</v>
       </c>
       <c r="H22" t="n">
-        <v>22204</v>
+        <v>480</v>
       </c>
     </row>
     <row r="23">
@@ -1205,16 +1187,16 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>6.609</v>
+        <v>6.6585</v>
       </c>
       <c r="F23" t="n">
-        <v>0.101</v>
+        <v>0.1505</v>
       </c>
       <c r="G23" t="n">
-        <v>1.55</v>
+        <v>2.31</v>
       </c>
       <c r="H23" t="n">
-        <v>21334</v>
+        <v>507</v>
       </c>
     </row>
     <row r="24">
@@ -1238,17 +1220,11 @@
           <t>2026-10-27</t>
         </is>
       </c>
-      <c r="E24" t="n">
-        <v>62.2</v>
-      </c>
-      <c r="F24" t="n">
-        <v>0.38</v>
-      </c>
-      <c r="G24" t="n">
-        <v>0.61</v>
-      </c>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr"/>
       <c r="H24" t="n">
-        <v>4088987</v>
+        <v>23450109</v>
       </c>
     </row>
     <row r="25">
@@ -1273,13 +1249,13 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>18.03</v>
+        <v>17.52</v>
       </c>
       <c r="F25" t="n">
-        <v>-0.36</v>
+        <v>-0.87</v>
       </c>
       <c r="G25" t="n">
-        <v>-1.96</v>
+        <v>-4.73</v>
       </c>
       <c r="H25" t="n">
         <v>0</v>
@@ -1303,20 +1279,20 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="E26" t="n">
-        <v>79947.4219</v>
+        <v>80659.99219999999</v>
       </c>
       <c r="F26" t="n">
-        <v>-59.2344</v>
+        <v>653.3359</v>
       </c>
       <c r="G26" t="n">
-        <v>-0.07000000000000001</v>
+        <v>0.82</v>
       </c>
       <c r="H26" t="n">
-        <v>22821048320</v>
+        <v>22768437248</v>
       </c>
     </row>
     <row r="27">
@@ -1749,22 +1725,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Daerah Kesulitan Bayar Gaji Pegawai, Dua Menteri Prabowo Buka Suara</t>
+          <t>Bocoran Insentif Mobil Hybrid dari Menperin</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Tue, 27 Oct 2026 20:31:18 +0700</t>
+          <t>Wed, 28 Oct 2026 07:30:18 +0700</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/10/10/potret-asn-aparatur-sipil-negara-1760067743474_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Dalam Negeri Tito Karnavian dan Menteri Keuangan Suahasil Nazara buka suara soal daerah sulit bayar gaji pegawai.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/02/sertijab-menteri-perindustrian-sarmuji-gantikan-agus-gumiwang-1790919880231_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Perindustrian Sarmuji buka-bukaan bocoran insentif mobil hybrid.</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8726936/daerah-kesulitan-bayar-gaji-pegawai-dua-menteri-prabowo-buka-suara</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8726958/bocoran-insentif-mobil-hybrid-dari-menperin</t>
         </is>
       </c>
     </row>
@@ -1776,22 +1752,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Produk Lokal Mendunia, Ekspor UMKM Tembus Rp6,6 Triliun Lewat Marketplace</t>
+          <t>Sanksi Pajak Bisa Dihapus atau Dikurangi, Ini Rinciannya</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Tue, 27 Oct 2026 20:30:50 +0700</t>
+          <t>Wed, 28 Oct 2026 07:00:01 +0700</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/27/produk-lokal-mendunia-ekspor-umkm-tembus-rp66-triliun-lewat-marketplace-1793104069684_169.jpeg?w=360&amp;amp;q=90" /&gt; UMKM Indonesia kian menembus pasar global lewat marketplace. Perdagangan digital membuka peluang ekspor produk loka</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2024/11/22/ilustrasi-pajak-2026_169.jpeg?w=360&amp;amp;q=90" /&gt; Direktorat Jenderal Pajak (DJP) Kementerian Keuangan memberikan fasilitas pengurangan atau penghapusan sanksi administratif pajak.</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/foto-bisnis/d-8726838/produk-lokal-mendunia-ekspor-umkm-tembus-rp6-6-triliun-lewat-marketplace</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8726977/sanksi-pajak-bisa-dihapus-atau-dikurangi-ini-rinciannya</t>
         </is>
       </c>
     </row>
@@ -1803,22 +1779,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Siap Jadi Penyangga Jagung, BULOG Perkuat Kemitraan Petani-Peternak</t>
+          <t>Siap-siap, Akhir Tahun Bakal Ada WFH</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Tue, 27 Oct 2026 20:18:55 +0700</t>
+          <t>Wed, 28 Oct 2026 06:30:59 +0700</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/27/siap-jadi-penyangga-pasokan-jagung-bulog-perkuat-kemitraan-petani-peternak-1793106864647_169.jpeg?w=360&amp;amp;q=90" /&gt; Perum BULOG siap menjadi penyangga pasokan jagung nasional, memperkuat kemitraan antara petani dan peternak untu</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/10/28/ilustrasi-wfh-1761645496439_169.jpeg?w=360&amp;amp;q=90" /&gt; Kementerian Perhubungan (Kemenhub) mengusulkan work from home (WFH) selama jelang dan sesudah libur Natal 2026 dan Tahun Baru 2027 (Nataru).</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8726924/siap-jadi-penyangga-jagung-bulog-perkuat-kemitraan-petani-peternak</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8726954/siap-siap-akhir-tahun-bakal-ada-wfh</t>
         </is>
       </c>
     </row>
@@ -1830,22 +1806,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Kinerja Semester I 2026 Positif, JAPFA Perkuat Inovasi dan Efisiensi</t>
+          <t>Luhut Ungkap Isi Pembicaraan dengan Bahlil Usai Pangkas Gas ke Singapura</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Tue, 27 Oct 2026 20:01:48 +0700</t>
+          <t>Wed, 28 Oct 2026 05:55:08 +0700</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/27/kinerja-semester-i-2026-positif-japfa-perkuat-inovasi-dan-efisiensi-1793105772143_169.jpeg?w=360&amp;amp;q=90" /&gt; PT Japfa Comfeed Indonesia Tbk mencatat laba Rp 2,68 triliun di Semester I-2026, didukung penjualan bersih Rp 35,36 tri</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/27/pertemuan-ketua-den-dengan-menko-kumham-imipas-1793090271348_169.jpeg?w=360&amp;amp;q=90" /&gt; Nggak juga (tidak menyebabkan konflik) saya kira karena Pak Bahlil, juga tadi saya bicara sama beliau, ya beliau menyampaikan ini aja concer</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8726903/kinerja-semester-i-2026-positif-japfa-perkuat-inovasi-dan-efisiensi</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8726951/luhut-ungkap-isi-pembicaraan-dengan-bahlil-usai-pangkas-gas-ke-singapura</t>
         </is>
       </c>
     </row>
@@ -1857,22 +1833,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Suntikan Dana Pusat ke Daerah Tembus Rp 720 Triliun</t>
+          <t>Petinggi Mubadala Sambangi RI Lapor Progres Blok Andaman</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Tue, 27 Oct 2026 19:58:37 +0700</t>
+          <t>Tue, 27 Oct 2026 22:50:03 +0700</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2015/12/17/00d5a8dc-da3d-483a-bd2e-e78ce08f1d66_169.jpg?w=360&amp;amp;q=90" /&gt; Menteri Keuangan Suahasil Nazara mengungkapkan pemerintah telah menggelontorkan dana Transfer ke Daerah (TKD) hingga Rp 720 triliun.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2024/04/07/energi-di-bulan-suci-dari-pulau-besi-10_169.jpeg?w=360&amp;amp;q=90" /&gt; Perusahaan minyak dan gas (migas) Uni Emirat Arab (UEA), Mubadala Energy, akan terlibat dalam proyek gas di Andaman, lepas pantai Aceh.</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8726899/suntikan-dana-pusat-ke-daerah-tembus-rp-720-triliun</t>
+          <t>https://finance.detik.com/energi/d-8727069/petinggi-mubadala-sambangi-ri-lapor-progres-blok-andaman</t>
         </is>
       </c>
     </row>
@@ -1884,22 +1860,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Nikmati Akhir Pekan di WKND Market PIK2, Bisa Belanja hingga Ikut Workshop</t>
+          <t>Produksi Gas Blok Masela Paling Lambat Mulai 2030</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Tue, 27 Oct 2026 19:39:02 +0700</t>
+          <t>Tue, 27 Oct 2026 22:03:44 +0700</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/27/wknd-market-vol-6-hadir-di-lands-end-pik2-cek-jadwal-aksesnya-1793104614080_169.jpeg?w=360&amp;amp;q=90" /&gt; WKND Market Vol. 6 di Pantai Indah Kapuk 2 hadir 6-8 November 2026. Nikmati belanja produk lokal, workshop kreatif, olahraga,</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/04/09/inpex-rilis-desain-pabrik-pengolahan-lng-masela-1744182721026_169.jpeg?w=360&amp;amp;q=90" /&gt; Produksi gas di Blok Masela, Maluku, ditargetkan mulai berjalan 2030. Blok Masela nantinya akan memproduksi liquefied natural gas (LNG) ata</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8726851/nikmati-akhir-pekan-di-wknd-market-pik2-bisa-belanja-hingga-ikut-workshop</t>
+          <t>https://finance.detik.com/energi/d-8727029/produksi-gas-blok-masela-paling-lambat-mulai-2030</t>
         </is>
       </c>
     </row>
@@ -1911,22 +1887,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Proyek LNG Abadi Masela Ditargetkan Operasi 2029, Begini Progresnya</t>
+          <t>Perusahaan AS Bawa Rp 9 Triliun ke Batam, Garap Proyek Silika hingga AI</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Tue, 27 Oct 2026 18:10:02 +0700</t>
+          <t>Tue, 27 Oct 2026 21:19:43 +0700</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/02/14/kepala-skk-migas-djoko-siswanto-1_169.jpeg?w=360&amp;amp;q=90" /&gt; INPEX Masela Ltd. selesaikan tahap FEED proyek LNG Abadi lebih cepat, proyek gas raksasa itu ditargetkan beroperasi paling cepat 2029.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/04/04/ilustrasi-produksi-dan-kawasan-industri-di-batam-foto-dok-bp-batam-1743782355897_169.jpeg?w=360&amp;amp;q=90" /&gt; Proyek Strategis Nasional (PSN) WIRARAJA GESEIP resmi menggandeng investor asal Amerika Serikat, Tynergy Technology Grou</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8726688/proyek-lng-abadi-masela-ditargetkan-operasi-2029-begini-progresnya</t>
+          <t>https://finance.detik.com/industri/d-8726987/perusahaan-as-bawa-rp-9-triliun-ke-batam-garap-proyek-silika-hingga-ai</t>
         </is>
       </c>
     </row>
@@ -1938,22 +1914,22 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Bansos Digital Meluncur 10 November, 100 Juta Warga Bakal Terdaftar</t>
+          <t>Daerah Kesulitan Bayar Gaji Pegawai, Dua Menteri Prabowo Buka Suara</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Tue, 27 Oct 2026 17:50:31 +0700</t>
+          <t>Tue, 27 Oct 2026 20:31:18 +0700</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/27/pertemuan-ketua-den-dengan-menko-kumham-imipas-1793090271348_169.jpeg?w=360&amp;amp;q=90" /&gt; Dan kita harap nanti waktu roll out oleh Presiden tanggal 10 November itu sudah lebih 100 juta orang, kata Luhut.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/10/10/potret-asn-aparatur-sipil-negara-1760067743474_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Dalam Negeri Tito Karnavian dan Menteri Keuangan Suahasil Nazara buka suara soal daerah sulit bayar gaji pegawai.</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8726657/bansos-digital-meluncur-10-november-100-juta-warga-bakal-terdaftar</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8726936/daerah-kesulitan-bayar-gaji-pegawai-dua-menteri-prabowo-buka-suara</t>
         </is>
       </c>
     </row>
@@ -1965,22 +1941,22 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Waskita Karya Lanjutkan Pemulihan Pascabencana di Aceh, Progres Hampir 70%</t>
+          <t>Produk Lokal Mendunia, Ekspor UMKM Tembus Rp6,6 Triliun Lewat Marketplace</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Tue, 27 Oct 2026 17:41:12 +0700</t>
+          <t>Tue, 27 Oct 2026 20:30:50 +0700</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/27/waskita-karya-lanjutkan-pemulihan-pascabencana-di-aceh-progres-hampir-70-1793097636359.jpeg?w=360&amp;amp;q=90" /&gt; Waskita Karya terus berupaya memulihkan Aceh pascabencana dengan proyek penanganan infrastruktur dan penyediaan air be</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/27/produk-lokal-mendunia-ekspor-umkm-tembus-rp66-triliun-lewat-marketplace-1793104069684_169.jpeg?w=360&amp;amp;q=90" /&gt; UMKM Indonesia kian menembus pasar global lewat marketplace. Perdagangan digital membuka peluang ekspor produk loka</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/infrastruktur/d-8726642/waskita-karya-lanjutkan-pemulihan-pascabencana-di-aceh-progres-hampir-70</t>
+          <t>https://finance.detik.com/foto-bisnis/d-8726838/produk-lokal-mendunia-ekspor-umkm-tembus-rp6-6-triliun-lewat-marketplace</t>
         </is>
       </c>
     </row>
@@ -1992,22 +1968,22 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>BI Pangkas Kewajiban GWM, BCA Bidik Target Kredit Double Digit</t>
+          <t>Siap Jadi Penyangga Jagung, BULOG Perkuat Kemitraan Petani-Peternak</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Tue, 27 Oct 2026 17:40:20 +0700</t>
+          <t>Tue, 27 Oct 2026 20:18:55 +0700</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2016/04/28/4f6b9d13-dc5d-4f7b-944c-7dd26d554e82_169.jpg?w=360&amp;amp;q=90" /&gt; PT Bank Central Asia (BBCA) menyambut baik pelonggaran GWM oleh Bank Indonesia, yang mendukung pertumbuhan kredit BCA.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/27/siap-jadi-penyangga-pasokan-jagung-bulog-perkuat-kemitraan-petani-peternak-1793106864647_169.jpeg?w=360&amp;amp;q=90" /&gt; Perum BULOG siap menjadi penyangga pasokan jagung nasional, memperkuat kemitraan antara petani dan peternak untu</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/moneter/d-8726637/bi-pangkas-kewajiban-gwm-bca-bidik-target-kredit-double-digit</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8726924/siap-jadi-penyangga-jagung-bulog-perkuat-kemitraan-petani-peternak</t>
         </is>
       </c>
     </row>
@@ -2019,22 +1995,22 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Stabilitas Perbankan di Tengah Gejolak Pasar Modal</t>
+          <t>Kinerja Semester I 2026 Positif, JAPFA Perkuat Inovasi dan Efisiensi</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Tue, 27 Oct 2026 17:29:53 +0700</t>
+          <t>Tue, 27 Oct 2026 20:01:48 +0700</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/19/ihsg-dibuka-anjlok-431-bei-berlakukan-arb-7-1792382663806_169.jpeg?w=360&amp;amp;q=90" /&gt; OJK, bersama pemerintah dan BEI, memperkuat pasar modal Indonesia dengan reformasi untuk meningkatkan dan menjaga kepercayaan investor global.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/27/kinerja-semester-i-2026-positif-japfa-perkuat-inovasi-dan-efisiensi-1793105772143_169.jpeg?w=360&amp;amp;q=90" /&gt; PT Japfa Comfeed Indonesia Tbk mencatat laba Rp 2,68 triliun di Semester I-2026, didukung penjualan bersih Rp 35,36 tri</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/moneter/d-8726613/stabilitas-perbankan-di-tengah-gejolak-pasar-modal</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8726903/kinerja-semester-i-2026-positif-japfa-perkuat-inovasi-dan-efisiensi</t>
         </is>
       </c>
     </row>
@@ -2046,22 +2022,22 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>blu by BCA Digital Ajak Anak Muda Eksplorasi Hal Baru Lewat #EksplorSemaumu</t>
+          <t>Suntikan Dana Pusat ke Daerah Tembus Rp 720 Triliun</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Tue, 27 Oct 2026 17:22:45 +0700</t>
+          <t>Tue, 27 Oct 2026 19:58:37 +0700</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/27/blu-by-bca-digital-ajak-anak-muda-eksplorasi-hal-baru-lewat-eksplorsemaumu-1793096408008_169.png?w=360&amp;amp;q=90" /&gt; Blu by BCA Digital mengajak anak muda untuk #EksplorSemaumu, merayakan pengalaman unik dengan fitur perbankan dig</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2015/12/17/00d5a8dc-da3d-483a-bd2e-e78ce08f1d66_169.jpg?w=360&amp;amp;q=90" /&gt; Menteri Keuangan Suahasil Nazara mengungkapkan pemerintah telah menggelontorkan dana Transfer ke Daerah (TKD) hingga Rp 720 triliun.</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/moneter/d-8726594/blu-by-bca-digital-ajak-anak-muda-eksplorasi-hal-baru-lewat-eksplorsemaumu</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8726899/suntikan-dana-pusat-ke-daerah-tembus-rp-720-triliun</t>
         </is>
       </c>
     </row>
@@ -2073,22 +2049,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>RI Bakal Dapat Kiriman 30 Juta Barel Minyak dari UEA Bebas Ongkir</t>
+          <t>Nikmati Akhir Pekan di WKND Market PIK2, Bisa Belanja hingga Ikut Workshop</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Tue, 27 Oct 2026 17:16:56 +0700</t>
+          <t>Tue, 27 Oct 2026 19:39:02 +0700</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2021/04/16/infografis-indonesia-masih-impor-bbm-1_169.jpeg?w=360&amp;amp;q=90" /&gt; Pemerintah UEA akan mengirim 30 juta barel minyak ke Indonesia tanpa biaya modal kerja.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/27/wknd-market-vol-6-hadir-di-lands-end-pik2-cek-jadwal-aksesnya-1793104614080_169.jpeg?w=360&amp;amp;q=90" /&gt; WKND Market Vol. 6 di Pantai Indah Kapuk 2 hadir 6-8 November 2026. Nikmati belanja produk lokal, workshop kreatif, olahraga,</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8726589/ri-bakal-dapat-kiriman-30-juta-barel-minyak-dari-uea-bebas-ongkir</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8726851/nikmati-akhir-pekan-di-wknd-market-pik2-bisa-belanja-hingga-ikut-workshop</t>
         </is>
       </c>
     </row>
@@ -2100,22 +2076,22 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Jamin Kredit UMKM-K Rp 271 T, Jamkrindo Raup Laba Rp 1,1 T per September 2026</t>
+          <t>Proyek LNG Abadi Masela Ditargetkan Operasi 2029, Begini Progresnya</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Tue, 27 Oct 2026 17:05:37 +0700</t>
+          <t>Tue, 27 Oct 2026 18:10:02 +0700</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2023/04/27/jamkrindo_169.jpeg?w=360&amp;amp;q=90" /&gt; Jamkrindo laporkan penjaminan Rp 271,20 triliun hingga September 2026, dukung 2,97 juta UMKM dan 9,46 juta tenaga kerja. Laba sebelum pajak Rp 1,1 triliun.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/02/14/kepala-skk-migas-djoko-siswanto-1_169.jpeg?w=360&amp;amp;q=90" /&gt; INPEX Masela Ltd. selesaikan tahap FEED proyek LNG Abadi lebih cepat, proyek gas raksasa itu ditargetkan beroperasi paling cepat 2029.</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/moneter/d-8726555/jamin-kredit-umkm-k-rp-271-t-jamkrindo-raup-laba-rp-1-1-t-per-september-2026</t>
+          <t>https://finance.detik.com/energi/d-8726688/proyek-lng-abadi-masela-ditargetkan-operasi-2029-begini-progresnya</t>
         </is>
       </c>
     </row>
@@ -2127,22 +2103,22 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Progres Tol Semarang-Demak Seksi 1 Capai 79,42 Persen</t>
+          <t>Bansos Digital Meluncur 10 November, 100 Juta Warga Bakal Terdaftar</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Tue, 27 Oct 2026 17:02:44 +0700</t>
+          <t>Tue, 27 Oct 2026 17:50:31 +0700</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/27/progres-pembangunan-jalan-tol-semarang-demak-seksi-1-1793081892794_169.jpeg?w=360&amp;amp;q=90" /&gt; Progres pembangunan Tol Semarang-Demak Seksi 1 mencapai 79,42 persen hingga 22 Oktober 2026 dan ditargetkan rampung pada akhir 2027.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/27/pertemuan-ketua-den-dengan-menko-kumham-imipas-1793090271348_169.jpeg?w=360&amp;amp;q=90" /&gt; Dan kita harap nanti waktu roll out oleh Presiden tanggal 10 November itu sudah lebih 100 juta orang, kata Luhut.</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/foto-bisnis/d-8726052/progres-tol-semarang-demak-seksi-1-capai-79-42-persen</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8726657/bansos-digital-meluncur-10-november-100-juta-warga-bakal-terdaftar</t>
         </is>
       </c>
     </row>
@@ -2154,22 +2130,22 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Wajah Baru SMPN 91 Jakarta, Ada Lift dan Panel Surya</t>
+          <t>SMPN 2 Depok Berulang Kali Banjir, Disdik Siapkan Langkah Ini</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Tue, 27 Oct 2026 20:54:18 +0700</t>
+          <t>Wed, 28 Oct 2026 07:36:53 +0700</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Revitalisasi SMPN 91 Jakarta menambah ruang kelas dari delapan menjadi 21, dilengkapi lift, panel surya, dan papan interaktif digital.</t>
+          <t>Disdik Depok menyiapkan langkah jangka pendek dan menengah untuk mencegah banjir kembali merendam SMPN 2 Depok.</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8322618/wajah-baru-smpn-91-jakarta-ada-lift-dan-panel-surya</t>
+          <t>https://www.liputan6.com/news/read/8322781/smpn-2-depok-berulang-kali-banjir-disdik-siapkan-langkah-ini</t>
         </is>
       </c>
     </row>
@@ -2181,22 +2157,22 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Bahagianya Siswa Belajar di Gedung Baru SMPN 91, Makin Betah di Sekolah</t>
+          <t>Frugal Living dan Melambatnya Daya Beli Kelas Menengah</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Tue, 27 Oct 2026 20:57:14 +0700</t>
+          <t>Wed, 28 Oct 2026 07:06:02 +0700</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Di SMPN 91 Jakarta, revitalisasi tak hanya mengubah wajah bangunan.</t>
+          <t>Data Mandiri Spending Index (MSI) terbaru September 2026, menangkap gejala adanya pelambatan tren belanja di masyarakat.</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8322627/bahagianya-siswa-belajar-di-gedung-baru-smpn-91-makin-betah-di-sekolah</t>
+          <t>https://www.liputan6.com/news/read/8322236/frugal-living-dan-melambatnya-daya-beli-kelas-menengah</t>
         </is>
       </c>
     </row>
@@ -2208,22 +2184,22 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>KPK Buka Suara soal Kabar Panggil Nusron Wahid Besok</t>
+          <t>Mengapa Orang Ber-IQ Tinggi Seperti Dwi Martono Bisa Bertindak Keji?</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Tue, 27 Oct 2026 21:00:27 +0700</t>
+          <t>Wed, 28 Oct 2026 07:04:15 +0700</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Nusron Wahid sebelumnya telah dua kali mangkir dari panggilan KPK</t>
+          <t>Dwi menjadi sorotan publik setelah diduga membunuh istri sirinya, Dini Hardiyanti (30) dan anaknya di Madiun, Jawa Timur.</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8322629/kpk-buka-suara-soal-kabar-panggil-nusron-wahid-besok</t>
+          <t>https://www.liputan6.com/news/read/8322733/mengapa-orang-ber-iq-tinggi-seperti-dwi-martono-bisa-bertindak-keji</t>
         </is>
       </c>
     </row>
@@ -2235,22 +2211,22 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>KSPSI Ingatkan Massa Demo 28 Oktober Tak Anarkis dan Sebar Hoaks</t>
+          <t>Demo BEM UI, Ini Tuntutan yang Dibawa</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Tue, 27 Oct 2026 20:19:09 +0700</t>
+          <t>Wed, 28 Oct 2026 06:01:59 +0700</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>KSPSI mengajak masyarakat mengutamakan dialog dan musyawarah serta tidak menyebarkan informasi yang dapat memperkeruh suasana.</t>
+          <t>Mahasiswa telah menghimpun berbagai keresahan masyarakat yang dinilai belum mendapat respons memadai dari pemerintah.</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8322599/kspsi-ingatkan-massa-demo-28-oktober-tak-anarkis-dan-sebar-hoaks</t>
+          <t>https://www.liputan6.com/news/read/8322753/demo-bem-ui-ini-tuntutan-yang-dibawa</t>
         </is>
       </c>
     </row>
@@ -2262,22 +2238,22 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Sestama BNPB Dicecar KPK Soal Pengadaan Dana Bencana</t>
+          <t>Membidik Penyawer Ratusan Juta ke PCNU</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Tue, 27 Oct 2026 19:44:22 +0700</t>
+          <t>Wed, 28 Oct 2026 06:00:56 +0700</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Penyidik KPK mendalami dua persoalan dalam pemeriksaan tersebut.</t>
+          <t>Dugaan praktik risywah dalam Muktamar ke-35 NU di Jombang menjadi sorotan.</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8322572/sestama-bnpb-dicecar-kpk-soal-pengadaan-dana-bencana</t>
+          <t>https://www.liputan6.com/news/read/8322738/membidik-penyawer-ratusan-juta-ke-pcnu</t>
         </is>
       </c>
     </row>
@@ -2289,22 +2265,22 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Demo 28 Oktober, Polisi Imbau Jaga Fasilitas Umum</t>
+          <t>Lokasi Demo BEM UI, Hindari Jalan Ini</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Tue, 27 Oct 2026 19:36:44 +0700</t>
+          <t>Wed, 28 Oct 2026 05:51:22 +0700</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Sejumlah aliansi mahasiswa akan menggelar aksi unjuk rasa di Jakarta, Rabu, 28 Oktober 2026.</t>
+          <t>Aksi demo mahasiswa UI di Bundaran HI hari ini. Polisi siapkan rekayasa lalu lintas di sejumlah titik Jakarta.</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8322565/demo-28-oktober-polisi-imbau-jaga-fasilitas-umum</t>
+          <t>https://www.liputan6.com/news/read/8322759/lokasi-demo-bem-ui-hindari-jalan-ini</t>
         </is>
       </c>
     </row>
@@ -2316,22 +2292,22 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Penyebab KRL Berasap hingga Terdengar Ledakan di Stasiun Jakarta Kota</t>
+          <t>Ketika Cinta Dini Dibalas Pembunuhan Keji Dwi Martono</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Tue, 27 Oct 2026 19:37:10 +0700</t>
+          <t>Wed, 28 Oct 2026 05:06:09 +0700</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>KAI Commuter mengalihkan penumpang Commuter Line relasi Jakarta Kota-Bogor ke rangkaian lain imbas KRL berasap dan mengeluarkan percikan api.</t>
+          <t>Teka teki pembunuhan sadis Dini Hardiyanti (30) dan anak kandungnya, AGF (4) akhirnya terbongkar.</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8322567/penyebab-krl-berasap-hingga-terdengar-ledakan-di-stasiun-jakarta-kota</t>
+          <t>https://www.liputan6.com/news/read/8322710/ketika-cinta-dini-dibalas-pembunuhan-keji-dwi-martono</t>
         </is>
       </c>
     </row>
@@ -2343,22 +2319,22 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Ada Ledakan dan Percikan Api di KRL Jakarta-Bogor, KAI Buka Suara</t>
+          <t>Demo 28 Oktober, Presiden KSPN Ajak Massa Jaga Persatuan Sesuai Sumpah Pemuda</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Tue, 27 Oct 2026 19:27:47 +0700</t>
+          <t>Wed, 28 Oct 2026 03:06:57 +0700</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Kereta Commuter Line Jakarta–Bogor mengalami gangguan usai terdengar ledakan dan percikan api.</t>
+          <t>Ristadi mengingatkan, aksi yang bertepatan dengan peringatan Hari Sumpah Pemuda itu perlu mengedepankan semangat persatuan</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8322561/ada-ledakan-dan-percikan-api-di-krl-jakarta-bogor-kai-buka-suara</t>
+          <t>https://www.liputan6.com/news/read/8322689/demo-28-oktober-presiden-kspn-ajak-massa-jaga-persatuan-sesuai-sumpah-pemuda</t>
         </is>
       </c>
     </row>
@@ -2370,22 +2346,22 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Polri Jamin Penanganan Medis Ojol Korban Kecelakaan di Blok M</t>
+          <t>Ada Demo Hari Sumpah Pemuda di Jakarta, Hindari 4 Lokasi Ini</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Tue, 27 Oct 2026 19:27:25 +0700</t>
+          <t>Wed, 28 Oct 2026 00:57:38 +0700</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Polri memberikan pendampingan kepada pengemudi ojol korban kecelakaan di Blok M.</t>
+          <t>Polda Metro Jaya menyiapkan rekayasa lalu lintas secara situasional di sejumlah lokasi aksi.</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8322560/polri-jamin-penanganan-medis-ojol-korban-kecelakaan-di-blok-m</t>
+          <t>https://www.liputan6.com/news/read/8322734/ada-demo-hari-sumpah-pemuda-di-jakarta-hindari-4-lokasi-ini</t>
         </is>
       </c>
     </row>
@@ -2397,22 +2373,22 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>BRIN Punya 4 Kandidat Vaksin Malaria, Prabowo Minta Riset Dipercepat</t>
+          <t>Alokasi Transfer Daerah Ditambah Jadi Rp 720 T</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Tue, 27 Oct 2026 19:15:44 +0700</t>
+          <t>Wed, 28 Oct 2026 00:08:51 +0700</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Prabowo ingin pengembangan vaksin malaria tersebut dapat selesai tiga tahun lebih cepat dari target awal.</t>
+          <t>Menkeu Suahasil Tambah Alokasi Transfer Daerah Rp 720 T</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8322550/brin-punya-4-kandidat-vaksin-malaria-prabowo-minta-riset-dipercepat</t>
+          <t>https://www.liputan6.com/news/read/8322727/alokasi-transfer-daerah-ditambah-jadi-rp-720-t</t>
         </is>
       </c>
     </row>
@@ -2424,22 +2400,22 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Komite Sadar Gelar Aksi di Bundaran HI Besok, Ini Lima Tuntutannya</t>
+          <t>Menkeu dan Mendagri Bahas Anggaran Bencana hingga Insentif Daerah</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Tue, 27 Oct 2026 19:05:00 +0700</t>
+          <t>Tue, 27 Oct 2026 23:54:57 +0700</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Mereka mendesak pemerintah memenuhi lima tuntutan utama, termasuk penuntasan tata kelola lahan dan kebebasan bersuara.</t>
+          <t>Kemenkeu dan Kemendagri menyelaraskan APBN dan APBD agar program penanganan bencana.</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8322542/komite-sadar-gelar-aksi-di-bundaran-hi-besok-ini-lima-tuntutannya</t>
+          <t>https://www.liputan6.com/news/read/8322721/menkeu-dan-mendagri-bahas-anggaran-bencana-hingga-insentif-daerah</t>
         </is>
       </c>
     </row>
@@ -2451,22 +2427,22 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Jelang Sumpah Pemuda, Masyarakat Diminta Waspadai Provokasi</t>
+          <t>Rumput JIS Dikritik Shin Tae-yong dan Rizky Ridho, Pramono Buka Suara</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Tue, 27 Oct 2026 18:51:48 +0700</t>
+          <t>Tue, 27 Oct 2026 23:37:17 +0700</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Menjelang Sumpah Pemuda, Polri mengajak masyarakat memperkuat kolaborasi menjaga kamtibmas</t>
+          <t>Gubernur DKI Jakarta Pramono Anung mengakui kondisi rumput JIS masih belum sempurna</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8322532/jelang-sumpah-pemuda-masyarakat-diminta-waspadai-provokasi</t>
+          <t>https://www.liputan6.com/news/read/8322714/rumput-jis-dikritik-shin-tae-yong-dan-rizky-ridho-pramono-buka-suara</t>
         </is>
       </c>
     </row>
@@ -2478,22 +2454,22 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Ada Demo Sumpah Pemuda Besok, TNI-Polri Kawal Jakarta</t>
+          <t>265 Sekolah Rakyat Berdiri, Seskab Teddy: 45 Ribu Anak Jalanan Kembali Bersekolah</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Tue, 27 Oct 2026 18:48:40 +0700</t>
+          <t>Tue, 27 Oct 2026 23:00:36 +0700</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Petugas akan ditempatkan di sejumlah titik kegiatan untuk mengawal peserta aksi</t>
+          <t>Sekolah Rakyat tidak hanya menyediakan ruang belajar, tetapi juga menghadirkan lingkungan yang mendukung tumbuh kembang.</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8322530/ada-demo-sumpah-pemuda-besok-tni-polri-kawal-jakarta</t>
+          <t>https://www.liputan6.com/news/read/8322700/265-sekolah-rakyat-berdiri-seskab-teddy-45-ribu-anak-jalanan-kembali-bersekolah</t>
         </is>
       </c>
     </row>
@@ -2505,22 +2481,22 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Kecelakaan Beruntun 4 Kendaraan di Tol Akses Tanjung Priok</t>
+          <t>Tersangka Penyerang Bobotoh di Bogor Bukan Anggota Kelompok Suporter</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Tue, 27 Oct 2026 18:24:32 +0700</t>
+          <t>Tue, 27 Oct 2026 22:54:43 +0700</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Kecelakaan tersebut menyebabkan satu orang mengalami luka.</t>
+          <t>Polisi telah mengamankan tersangka yang diduga melakukan penyerangan hingga menyebabkan suporter meninggal.</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8322513/kecelakaan-beruntun-4-kendaraan-di-tol-akses-tanjung-priok</t>
+          <t>https://www.liputan6.com/news/read/8322698/tersangka-penyerang-bobotoh-di-bogor-bukan-anggota-kelompok-suporter</t>
         </is>
       </c>
     </row>
@@ -2532,22 +2508,22 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Polri Jamin Kebebasan Berpendapat, Masyarakat Diimbau Tertib</t>
+          <t>Nasib Obligasi Jakarta Usai Pramono Bertemu Menkeu</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Tue, 27 Oct 2026 18:05:49 +0700</t>
+          <t>Tue, 27 Oct 2026 22:21:46 +0700</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Polri mengajak masyarakat menjaga ruang demokrasi dan menghormati perbedaan pendapat.</t>
+          <t>Pemprov DKI Jakarta akan mengikuti keputusan pemerintah pusat.</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8322499/polri-jamin-kebebasan-berpendapat-masyarakat-diimbau-tertib</t>
+          <t>https://www.liputan6.com/news/read/8322673/nasib-obligasi-jakarta-usai-pramono-bertemu-menkeu</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data pasar & berita - 2026-10-28 14:58 UTC
</commit_message>
<xml_diff>
--- a/data/market_news_latest.xlsx
+++ b/data/market_news_latest.xlsx
@@ -487,20 +487,20 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>5373.0942</v>
+        <v>5282.312</v>
       </c>
       <c r="F2" t="n">
-        <v>-66.1636</v>
+        <v>16.1821</v>
       </c>
       <c r="G2" t="n">
-        <v>-1.22</v>
+        <v>0.31</v>
       </c>
       <c r="H2" t="n">
-        <v>280027100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -521,20 +521,20 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>7722.6001</v>
+        <v>7728.4302</v>
       </c>
       <c r="F3" t="n">
-        <v>45.8301</v>
+        <v>5.8301</v>
       </c>
       <c r="G3" t="n">
-        <v>0.6</v>
+        <v>0.08</v>
       </c>
       <c r="H3" t="n">
-        <v>2810939000</v>
+        <v>653802820</v>
       </c>
     </row>
     <row r="4">
@@ -555,20 +555,20 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>52377.5703</v>
+        <v>52471.5781</v>
       </c>
       <c r="F4" t="n">
-        <v>15.9922</v>
+        <v>94.0078</v>
       </c>
       <c r="G4" t="n">
-        <v>0.03</v>
+        <v>0.18</v>
       </c>
       <c r="H4" t="n">
-        <v>401210066</v>
+        <v>84875450</v>
       </c>
     </row>
     <row r="5">
@@ -589,20 +589,20 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>26477.8105</v>
+        <v>26437.6289</v>
       </c>
       <c r="F5" t="n">
-        <v>308.4297</v>
+        <v>-40.1816</v>
       </c>
       <c r="G5" t="n">
-        <v>1.18</v>
+        <v>-0.15</v>
       </c>
       <c r="H5" t="n">
-        <v>7116359000</v>
+        <v>2518702000</v>
       </c>
     </row>
     <row r="6">
@@ -627,13 +627,13 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>63918.3594</v>
+        <v>63954.1914</v>
       </c>
       <c r="F6" t="n">
-        <v>1728.7109</v>
+        <v>685.8203</v>
       </c>
       <c r="G6" t="n">
-        <v>2.78</v>
+        <v>1.08</v>
       </c>
       <c r="H6" t="n">
         <v>0</v>
@@ -657,20 +657,20 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>23211.8105</v>
+        <v>23094.8301</v>
       </c>
       <c r="F7" t="n">
-        <v>118.4414</v>
+        <v>53.5098</v>
       </c>
       <c r="G7" t="n">
-        <v>0.51</v>
+        <v>0.23</v>
       </c>
       <c r="H7" t="n">
-        <v>2494900000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -691,14 +691,20 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>3681.469</v>
+      </c>
+      <c r="F8" t="n">
+        <v>33.168</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0.91</v>
+      </c>
       <c r="H8" t="n">
-        <v>3124247536</v>
+        <v>412609940</v>
       </c>
     </row>
     <row r="9">
@@ -719,20 +725,20 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>10767.2998</v>
+        <v>10698.0801</v>
       </c>
       <c r="F9" t="n">
-        <v>76.8994</v>
+        <v>11.5801</v>
       </c>
       <c r="G9" t="n">
-        <v>0.72</v>
+        <v>0.11</v>
       </c>
       <c r="H9" t="n">
-        <v>562995300</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -753,20 +759,20 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>25410.8398</v>
+        <v>25684.5195</v>
       </c>
       <c r="F10" t="n">
-        <v>229.1895</v>
+        <v>93.75</v>
       </c>
       <c r="G10" t="n">
-        <v>0.91</v>
+        <v>0.37</v>
       </c>
       <c r="H10" t="n">
-        <v>47950100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -787,20 +793,20 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>5415.9102</v>
+        <v>5397.9102</v>
       </c>
       <c r="F11" t="n">
-        <v>-6.25</v>
+        <v>0.8804</v>
       </c>
       <c r="G11" t="n">
-        <v>-0.12</v>
+        <v>0.02</v>
       </c>
       <c r="H11" t="n">
-        <v>264516700</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -821,17 +827,17 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>18144</v>
+        <v>18183</v>
       </c>
       <c r="F12" t="n">
-        <v>63</v>
+        <v>39</v>
       </c>
       <c r="G12" t="n">
-        <v>0.35</v>
+        <v>0.21</v>
       </c>
       <c r="H12" t="n">
         <v>0</v>
@@ -855,17 +861,17 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>102.337</v>
+        <v>102.376</v>
       </c>
       <c r="F13" t="n">
-        <v>0.377</v>
+        <v>0.056</v>
       </c>
       <c r="G13" t="n">
-        <v>0.37</v>
+        <v>0.05</v>
       </c>
       <c r="H13" t="n">
         <v>0</v>
@@ -893,13 +899,13 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>157.857</v>
+        <v>158.147</v>
       </c>
       <c r="F14" t="n">
-        <v>0.329</v>
+        <v>0.619</v>
       </c>
       <c r="G14" t="n">
-        <v>0.21</v>
+        <v>0.39</v>
       </c>
       <c r="H14" t="n">
         <v>0</v>
@@ -923,17 +929,17 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>0.4993</v>
+        <v>0.5024</v>
       </c>
       <c r="F15" t="n">
-        <v>0.0007</v>
+        <v>0.0031</v>
       </c>
       <c r="G15" t="n">
-        <v>0.14</v>
+        <v>0.62</v>
       </c>
       <c r="H15" t="n">
         <v>0</v>
@@ -957,17 +963,17 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>0.5305</v>
+        <v>0.532</v>
       </c>
       <c r="F16" t="n">
-        <v>0.0004</v>
+        <v>0.0015</v>
       </c>
       <c r="G16" t="n">
-        <v>0.08</v>
+        <v>0.28</v>
       </c>
       <c r="H16" t="n">
         <v>0</v>
@@ -991,17 +997,17 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>0.404</v>
+        <v>0.4028</v>
       </c>
       <c r="F17" t="n">
-        <v>0.0015</v>
+        <v>-0.0012</v>
       </c>
       <c r="G17" t="n">
-        <v>0.37</v>
+        <v>-0.3</v>
       </c>
       <c r="H17" t="n">
         <v>0</v>
@@ -1025,14 +1031,20 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>81.295</v>
+      </c>
+      <c r="F18" t="n">
+        <v>-0.335</v>
+      </c>
+      <c r="G18" t="n">
+        <v>-0.41</v>
+      </c>
       <c r="H18" t="n">
-        <v>19529180</v>
+        <v>5234941</v>
       </c>
     </row>
     <row r="19">
@@ -1053,14 +1065,20 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>77.62</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0.03</v>
+      </c>
       <c r="H19" t="n">
-        <v>54988363</v>
+        <v>18163774</v>
       </c>
     </row>
     <row r="20">
@@ -1081,20 +1099,20 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>4075.2</v>
+        <v>4055.7</v>
       </c>
       <c r="F20" t="n">
-        <v>36.8</v>
+        <v>-18.9001</v>
       </c>
       <c r="G20" t="n">
-        <v>0.91</v>
+        <v>-0.46</v>
       </c>
       <c r="H20" t="n">
-        <v>6054</v>
+        <v>68517</v>
       </c>
     </row>
     <row r="21">
@@ -1115,20 +1133,20 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>100.5</v>
+        <v>102.6</v>
       </c>
       <c r="F21" t="n">
-        <v>-1.26</v>
+        <v>2.7</v>
       </c>
       <c r="G21" t="n">
-        <v>-1.24</v>
+        <v>2.7</v>
       </c>
       <c r="H21" t="n">
-        <v>5845</v>
+        <v>131244</v>
       </c>
     </row>
     <row r="22">
@@ -1149,20 +1167,20 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="E22" t="n">
-        <v>109.87</v>
+        <v>112.02</v>
       </c>
       <c r="F22" t="n">
-        <v>-5.94</v>
+        <v>-1.86</v>
       </c>
       <c r="G22" t="n">
-        <v>-5.13</v>
+        <v>-1.63</v>
       </c>
       <c r="H22" t="n">
-        <v>480</v>
+        <v>22762</v>
       </c>
     </row>
     <row r="23">
@@ -1183,20 +1201,20 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="E23" t="n">
         <v>6.6585</v>
       </c>
       <c r="F23" t="n">
-        <v>0.1505</v>
+        <v>0.0365</v>
       </c>
       <c r="G23" t="n">
-        <v>2.31</v>
+        <v>0.55</v>
       </c>
       <c r="H23" t="n">
-        <v>507</v>
+        <v>19153</v>
       </c>
     </row>
     <row r="24">
@@ -1217,14 +1235,20 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr"/>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr"/>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>63.085</v>
+      </c>
+      <c r="F24" t="n">
+        <v>0.5649999999999999</v>
+      </c>
+      <c r="G24" t="n">
+        <v>0.9</v>
+      </c>
       <c r="H24" t="n">
-        <v>23450109</v>
+        <v>4409947</v>
       </c>
     </row>
     <row r="25">
@@ -1245,17 +1269,17 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="E25" t="n">
-        <v>17.52</v>
+        <v>17.35</v>
       </c>
       <c r="F25" t="n">
-        <v>-0.87</v>
+        <v>-0.17</v>
       </c>
       <c r="G25" t="n">
-        <v>-4.73</v>
+        <v>-0.97</v>
       </c>
       <c r="H25" t="n">
         <v>0</v>
@@ -1283,16 +1307,16 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>80659.99219999999</v>
+        <v>80448.4375</v>
       </c>
       <c r="F26" t="n">
-        <v>653.3359</v>
+        <v>-356.6406</v>
       </c>
       <c r="G26" t="n">
-        <v>0.82</v>
+        <v>-0.44</v>
       </c>
       <c r="H26" t="n">
-        <v>22768437248</v>
+        <v>22507993088</v>
       </c>
     </row>
     <row r="27">
@@ -1313,20 +1337,20 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="E27" t="n">
-        <v>1325</v>
+        <v>1235</v>
       </c>
       <c r="F27" t="n">
-        <v>-95</v>
+        <v>-90</v>
       </c>
       <c r="G27" t="n">
-        <v>-6.69</v>
+        <v>-6.79</v>
       </c>
       <c r="H27" t="n">
-        <v>94747900</v>
+        <v>142341100</v>
       </c>
     </row>
     <row r="28">
@@ -1347,20 +1371,20 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="E28" t="n">
-        <v>1360</v>
+        <v>1335</v>
       </c>
       <c r="F28" t="n">
-        <v>-85</v>
+        <v>-25</v>
       </c>
       <c r="G28" t="n">
-        <v>-5.88</v>
+        <v>-1.84</v>
       </c>
       <c r="H28" t="n">
-        <v>552502700</v>
+        <v>277508900</v>
       </c>
     </row>
     <row r="29">
@@ -1381,20 +1405,20 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="E29" t="n">
-        <v>456</v>
+        <v>432</v>
       </c>
       <c r="F29" t="n">
-        <v>-26</v>
+        <v>-24</v>
       </c>
       <c r="G29" t="n">
-        <v>-5.39</v>
+        <v>-5.26</v>
       </c>
       <c r="H29" t="n">
-        <v>771278300</v>
+        <v>444377000</v>
       </c>
     </row>
     <row r="30">
@@ -1415,20 +1439,20 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="E30" t="n">
-        <v>2160</v>
+        <v>2070</v>
       </c>
       <c r="F30" t="n">
-        <v>-160</v>
+        <v>-90</v>
       </c>
       <c r="G30" t="n">
-        <v>-6.9</v>
+        <v>-4.17</v>
       </c>
       <c r="H30" t="n">
-        <v>9145800</v>
+        <v>24971000</v>
       </c>
     </row>
     <row r="31">
@@ -1449,20 +1473,20 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="E31" t="n">
-        <v>2870</v>
+        <v>2670</v>
       </c>
       <c r="F31" t="n">
-        <v>-180</v>
+        <v>-200</v>
       </c>
       <c r="G31" t="n">
-        <v>-5.9</v>
+        <v>-6.97</v>
       </c>
       <c r="H31" t="n">
-        <v>45857600</v>
+        <v>67510700</v>
       </c>
     </row>
     <row r="32">
@@ -1483,20 +1507,20 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="E32" t="n">
-        <v>398</v>
+        <v>386</v>
       </c>
       <c r="F32" t="n">
-        <v>-28</v>
+        <v>-12</v>
       </c>
       <c r="G32" t="n">
-        <v>-6.57</v>
+        <v>-3.02</v>
       </c>
       <c r="H32" t="n">
-        <v>46521100</v>
+        <v>46693200</v>
       </c>
     </row>
     <row r="33">
@@ -1517,20 +1541,20 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="E33" t="n">
-        <v>452</v>
+        <v>448</v>
       </c>
       <c r="F33" t="n">
-        <v>-20</v>
+        <v>-4</v>
       </c>
       <c r="G33" t="n">
-        <v>-4.24</v>
+        <v>-0.88</v>
       </c>
       <c r="H33" t="n">
-        <v>85657700</v>
+        <v>61693200</v>
       </c>
     </row>
     <row r="34">
@@ -1551,20 +1575,20 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="E34" t="n">
-        <v>2320</v>
+        <v>2230</v>
       </c>
       <c r="F34" t="n">
-        <v>-170</v>
+        <v>-90</v>
       </c>
       <c r="G34" t="n">
-        <v>-6.83</v>
+        <v>-3.88</v>
       </c>
       <c r="H34" t="n">
-        <v>9559800</v>
+        <v>9435100</v>
       </c>
     </row>
     <row r="35">
@@ -1585,20 +1609,20 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="E35" t="n">
-        <v>352</v>
+        <v>360</v>
       </c>
       <c r="F35" t="n">
-        <v>-24</v>
+        <v>8</v>
       </c>
       <c r="G35" t="n">
-        <v>-6.38</v>
+        <v>2.27</v>
       </c>
       <c r="H35" t="n">
-        <v>479646600</v>
+        <v>295184800</v>
       </c>
     </row>
     <row r="36">
@@ -1619,20 +1643,20 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="E36" t="n">
-        <v>156</v>
+        <v>149</v>
       </c>
       <c r="F36" t="n">
-        <v>-11</v>
+        <v>-7</v>
       </c>
       <c r="G36" t="n">
-        <v>-6.59</v>
+        <v>-4.49</v>
       </c>
       <c r="H36" t="n">
-        <v>47375000</v>
+        <v>42924100</v>
       </c>
     </row>
     <row r="37">
@@ -1653,20 +1677,20 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="E37" t="n">
-        <v>10275</v>
+        <v>10175</v>
       </c>
       <c r="F37" t="n">
-        <v>75</v>
+        <v>-100</v>
       </c>
       <c r="G37" t="n">
-        <v>0.74</v>
+        <v>-0.97</v>
       </c>
       <c r="H37" t="n">
-        <v>20401200</v>
+        <v>26793100</v>
       </c>
     </row>
   </sheetData>
@@ -1725,22 +1749,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Bocoran Insentif Mobil Hybrid dari Menperin</t>
+          <t>Pemda Bakal Lebih Sering Pelototi Pelaksanaan MBG</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Wed, 28 Oct 2026 07:30:18 +0700</t>
+          <t>Wed, 28 Oct 2026 21:30:00 +0700</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/02/sertijab-menteri-perindustrian-sarmuji-gantikan-agus-gumiwang-1790919880231_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Perindustrian Sarmuji buka-bukaan bocoran insentif mobil hybrid.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/20/penerima-manfaat-mbg-dalam-dua-tahun-pemerintahan-prabowo-1792479756724_169.jpeg?w=360&amp;amp;q=90" /&gt; Pengawasan pelaksanaan Makan Bergizi Gratis (MBG) bakal lebih banyak melibatkan pemerintah daerah.</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8726958/bocoran-insentif-mobil-hybrid-dari-menperin</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8728569/pemda-bakal-lebih-sering-pelototi-pelaksanaan-mbg</t>
         </is>
       </c>
     </row>
@@ -1752,22 +1776,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Sanksi Pajak Bisa Dihapus atau Dikurangi, Ini Rinciannya</t>
+          <t>Berdayakan Masyarakat, MIND ID Raih Penghargaan Mandaya Awards 2026</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Wed, 28 Oct 2026 07:00:01 +0700</t>
+          <t>Wed, 28 Oct 2026 21:26:17 +0700</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2024/11/22/ilustrasi-pajak-2026_169.jpeg?w=360&amp;amp;q=90" /&gt; Direktorat Jenderal Pajak (DJP) Kementerian Keuangan memberikan fasilitas pengurangan atau penghapusan sanksi administratif pajak.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/28/berdayakan-masyarakat-grup-mind-id-raih-penghargaan-mandaya-awards-2026-1793197151033_169.jpeg?w=360&amp;amp;q=90" /&gt; MIND ID meraih Anugerah Mandaya Award 2026 atas pemberdayaan masyarakat. Programnya fokus pada penguatan ekonomi da</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8726977/sanksi-pajak-bisa-dihapus-atau-dikurangi-ini-rinciannya</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8728601/berdayakan-masyarakat-mind-id-raih-penghargaan-mandaya-awards-2026</t>
         </is>
       </c>
     </row>
@@ -1779,22 +1803,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Siap-siap, Akhir Tahun Bakal Ada WFH</t>
+          <t>8 Bos Sawit RI Menghadap Menteri Singapura, Ini Daftarnya</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Wed, 28 Oct 2026 06:30:59 +0700</t>
+          <t>Wed, 28 Oct 2026 21:05:16 +0700</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/10/28/ilustrasi-wfh-1761645496439_169.jpeg?w=360&amp;amp;q=90" /&gt; Kementerian Perhubungan (Kemenhub) mengusulkan work from home (WFH) selama jelang dan sesudah libur Natal 2026 dan Tahun Baru 2027 (Nataru).</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/12/situasi-kabut-asap-di-singapura-pada-senin-1210-waktu-setempat-1791794641533_169.jpeg?w=360&amp;amp;q=90" /&gt; Delapan Petinggi perusahaan kelapa sawit besar di Indonesia memenuhi panggilan pejabat tinggi Singapura.</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8726954/siap-siap-akhir-tahun-bakal-ada-wfh</t>
+          <t>https://finance.detik.com/industri/d-8728582/8-bos-sawit-ri-menghadap-menteri-singapura-ini-daftarnya</t>
         </is>
       </c>
     </row>
@@ -1806,22 +1830,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Luhut Ungkap Isi Pembicaraan dengan Bahlil Usai Pangkas Gas ke Singapura</t>
+          <t>Dua Pintu Masuk Stasiun MRT Dukuh Atas Ditutup Sementara</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Wed, 28 Oct 2026 05:55:08 +0700</t>
+          <t>Wed, 28 Oct 2026 20:11:26 +0700</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/27/pertemuan-ketua-den-dengan-menko-kumham-imipas-1793090271348_169.jpeg?w=360&amp;amp;q=90" /&gt; Nggak juga (tidak menyebabkan konflik) saya kira karena Pak Bahlil, juga tadi saya bicara sama beliau, ya beliau menyampaikan ini aja concer</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/17/penumpang-mrt-jakarta-1792229479640_169.jpeg?w=360&amp;amp;q=90" /&gt; Pintu masuk E dan C Stasiun MRT Dukuh Atas BNI masih ditutup sementara.</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8726951/luhut-ungkap-isi-pembicaraan-dengan-bahlil-usai-pangkas-gas-ke-singapura</t>
+          <t>https://finance.detik.com/infrastruktur/d-8728516/dua-pintu-masuk-stasiun-mrt-dukuh-atas-ditutup-sementara</t>
         </is>
       </c>
     </row>
@@ -1833,22 +1857,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Petinggi Mubadala Sambangi RI Lapor Progres Blok Andaman</t>
+          <t>Impor BBM Lewat Lemigas Cuma buat Produk yang Dijual Pertamina</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Tue, 27 Oct 2026 22:50:03 +0700</t>
+          <t>Wed, 28 Oct 2026 19:30:05 +0700</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2024/04/07/energi-di-bulan-suci-dari-pulau-besi-10_169.jpeg?w=360&amp;amp;q=90" /&gt; Perusahaan minyak dan gas (migas) Uni Emirat Arab (UEA), Mubadala Energy, akan terlibat dalam proyek gas di Andaman, lepas pantai Aceh.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/14/bahlil-lahadalia-rolandodetikcom-1791978307056_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Bahlil menegaskan impor migas lewat Lemigas hanya untuk Pertamina, bukan swasta. Skema baru impor kini menggunakan G2G dan G2B.</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8727069/petinggi-mubadala-sambangi-ri-lapor-progres-blok-andaman</t>
+          <t>https://finance.detik.com/energi/d-8728437/impor-bbm-lewat-lemigas-cuma-buat-produk-yang-dijual-pertamina</t>
         </is>
       </c>
     </row>
@@ -1860,22 +1884,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Produksi Gas Blok Masela Paling Lambat Mulai 2030</t>
+          <t>Panen Zaitun Warga Kurdi di Tengah Krisis Ekonomi</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Tue, 27 Oct 2026 22:03:44 +0700</t>
+          <t>Wed, 28 Oct 2026 19:04:16 +0700</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/04/09/inpex-rilis-desain-pabrik-pengolahan-lng-masela-1744182721026_169.jpeg?w=360&amp;amp;q=90" /&gt; Produksi gas di Blok Masela, Maluku, ditargetkan mulai berjalan 2030. Blok Masela nantinya akan memproduksi liquefied natural gas (LNG) ata</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/28/panen-zaitun-warga-kurdi-di-tengah-krisis-ekonomi-1793170558501.jpeg?w=360&amp;amp;q=90" /&gt; Petani memanen zaitun di Afrin, Suriah, di tengah keterbatasan air, kenaikan biaya produksi, dan rendahnya harga jual.</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8727029/produksi-gas-blok-masela-paling-lambat-mulai-2030</t>
+          <t>https://finance.detik.com/foto-bisnis/d-8727752/panen-zaitun-warga-kurdi-di-tengah-krisis-ekonomi</t>
         </is>
       </c>
     </row>
@@ -1887,22 +1911,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Perusahaan AS Bawa Rp 9 Triliun ke Batam, Garap Proyek Silika hingga AI</t>
+          <t>Mentan Jamin Harga Beras Turun Usai Mafia Oplosan Dibongkar!</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Tue, 27 Oct 2026 21:19:43 +0700</t>
+          <t>Wed, 28 Oct 2026 19:02:09 +0700</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/04/04/ilustrasi-produksi-dan-kawasan-industri-di-batam-foto-dok-bp-batam-1743782355897_169.jpeg?w=360&amp;amp;q=90" /&gt; Proyek Strategis Nasional (PSN) WIRARAJA GESEIP resmi menggandeng investor asal Amerika Serikat, Tynergy Technology Grou</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/28/mentan-ungkap-praktik-beras-oplosan-1793173274624_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Pertanian Andi Amran Sulaiman jamin penindakan pengoplosan beras SPHP dapat turunkan harga beras.</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/industri/d-8726987/perusahaan-as-bawa-rp-9-triliun-ke-batam-garap-proyek-silika-hingga-ai</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8728410/mentan-jamin-harga-beras-turun-usai-mafia-oplosan-dibongkar</t>
         </is>
       </c>
     </row>
@@ -1914,22 +1938,22 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Daerah Kesulitan Bayar Gaji Pegawai, Dua Menteri Prabowo Buka Suara</t>
+          <t>RI Dapat Pasokan Minyak 30 Juta Barel dari UEA? Bahlil: Masih Penjajakan</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Tue, 27 Oct 2026 20:31:18 +0700</t>
+          <t>Wed, 28 Oct 2026 18:40:06 +0700</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/10/10/potret-asn-aparatur-sipil-negara-1760067743474_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Dalam Negeri Tito Karnavian dan Menteri Keuangan Suahasil Nazara buka suara soal daerah sulit bayar gaji pegawai.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/03/10/menteri-esdm-bahlil-lahadalia-1773134823836_169.jpeg?w=360&amp;amp;q=90" /&gt; Menko Hilirisasi dan Transisi Energi Bahlil Lahadalia buka suara soal potensi pasokan minyak mentah 30 juta dari Uni Emirat Arab (UEA).</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8726936/daerah-kesulitan-bayar-gaji-pegawai-dua-menteri-prabowo-buka-suara</t>
+          <t>https://finance.detik.com/energi/d-8728371/ri-dapat-pasokan-minyak-30-juta-barel-dari-uea-bahlil-masih-penjajakan</t>
         </is>
       </c>
     </row>
@@ -1941,22 +1965,22 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Produk Lokal Mendunia, Ekspor UMKM Tembus Rp6,6 Triliun Lewat Marketplace</t>
+          <t>Mentan Minta Bulog Serap Jagung Petani Sesuai Aturan</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Tue, 27 Oct 2026 20:30:50 +0700</t>
+          <t>Wed, 28 Oct 2026 18:34:32 +0700</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/27/produk-lokal-mendunia-ekspor-umkm-tembus-rp66-triliun-lewat-marketplace-1793104069684_169.jpeg?w=360&amp;amp;q=90" /&gt; UMKM Indonesia kian menembus pasar global lewat marketplace. Perdagangan digital membuka peluang ekspor produk loka</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/07/28/wawancara-khusus-menteri-pertanian-ri-andi-amran-sulaiman-1753687994517_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Pertanian (Mentan) sekaligus Kepala Badan Pangan Nasional (Bapanas) Andi Amran Sulaiman meminta Perum Bulog tidak menolak</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/foto-bisnis/d-8726838/produk-lokal-mendunia-ekspor-umkm-tembus-rp6-6-triliun-lewat-marketplace</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8728357/mentan-minta-bulog-serap-jagung-petani-sesuai-aturan</t>
         </is>
       </c>
     </row>
@@ -1968,22 +1992,22 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Siap Jadi Penyangga Jagung, BULOG Perkuat Kemitraan Petani-Peternak</t>
+          <t>Menperin Ungkap Keresahan Pengusaha soal Isu Pencabutan Bea Keluar Emas</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Tue, 27 Oct 2026 20:18:55 +0700</t>
+          <t>Wed, 28 Oct 2026 18:30:12 +0700</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/27/siap-jadi-penyangga-pasokan-jagung-bulog-perkuat-kemitraan-petani-peternak-1793106864647_169.jpeg?w=360&amp;amp;q=90" /&gt; Perum BULOG siap menjadi penyangga pasokan jagung nasional, memperkuat kemitraan antara petani dan peternak untu</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/28/menteri-perindustrian-menperin-muhammad-sarmuji-1793178348200_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Perindustrian (Menperin) Muhammad Sarmuji mengungkapkan keresahan pengusaha perhiasan terkait rumor pencabutan bea keluar bahan bak</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8726924/siap-jadi-penyangga-jagung-bulog-perkuat-kemitraan-petani-peternak</t>
+          <t>https://finance.detik.com/industri/d-8728353/menperin-ungkap-keresahan-pengusaha-soal-isu-pencabutan-bea-keluar-emas</t>
         </is>
       </c>
     </row>
@@ -1995,22 +2019,22 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Kinerja Semester I 2026 Positif, JAPFA Perkuat Inovasi dan Efisiensi</t>
+          <t>KKP Dampingi Pemda Jamin Pembangunan KNMP Sesuai Rencana Tata Ruang</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Tue, 27 Oct 2026 20:01:48 +0700</t>
+          <t>Wed, 28 Oct 2026 18:27:07 +0700</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/27/kinerja-semester-i-2026-positif-japfa-perkuat-inovasi-dan-efisiensi-1793105772143_169.jpeg?w=360&amp;amp;q=90" /&gt; PT Japfa Comfeed Indonesia Tbk mencatat laba Rp 2,68 triliun di Semester I-2026, didukung penjualan bersih Rp 35,36 tri</t>
+          <t xml:space="preserve">&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/28/kkp-dukung-pemda-jamin-pembangunan-knmp-sesuai-rencana-tata-ruang-1793186771621.jpeg?w=360&amp;amp;q=90" /&gt; Kementerian Kelautan dan Perikanan RI memastikan pembangunan Kampung Nelayan Merah Putih sesuai tata ruang. KKP dukung pemda </t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8726903/kinerja-semester-i-2026-positif-japfa-perkuat-inovasi-dan-efisiensi</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8728351/kkp-dampingi-pemda-jamin-pembangunan-knmp-sesuai-rencana-tata-ruang</t>
         </is>
       </c>
     </row>
@@ -2022,22 +2046,22 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Suntikan Dana Pusat ke Daerah Tembus Rp 720 Triliun</t>
+          <t>Shopee Buka Rute Ekspor Baru ke 4 Negara Lewat Program FLEXI</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Tue, 27 Oct 2026 19:58:37 +0700</t>
+          <t>Wed, 28 Oct 2026 18:22:53 +0700</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2015/12/17/00d5a8dc-da3d-483a-bd2e-e78ce08f1d66_169.jpg?w=360&amp;amp;q=90" /&gt; Menteri Keuangan Suahasil Nazara mengungkapkan pemerintah telah menggelontorkan dana Transfer ke Daerah (TKD) hingga Rp 720 triliun.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/28/shopee-buka-rute-ekspor-baru-ke-4-negara-lewat-program-flexi-1793186505123_169.jpeg?w=360&amp;amp;q=90" /&gt; Shopee luncurkan Program Jalan Global Kreasi Lokal, memperluas ekspor ke Singapura, Thailand, Filipina, dan Brunei. Penjual da</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8726899/suntikan-dana-pusat-ke-daerah-tembus-rp-720-triliun</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8728345/shopee-buka-rute-ekspor-baru-ke-4-negara-lewat-program-flexi</t>
         </is>
       </c>
     </row>
@@ -2049,22 +2073,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Nikmati Akhir Pekan di WKND Market PIK2, Bisa Belanja hingga Ikut Workshop</t>
+          <t>Bahlil Singgung Ada Ketegangan di ASEAN Gegara Harga Minyak Mahal</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Tue, 27 Oct 2026 19:39:02 +0700</t>
+          <t>Wed, 28 Oct 2026 18:18:22 +0700</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/27/wknd-market-vol-6-hadir-di-lands-end-pik2-cek-jadwal-aksesnya-1793104614080_169.jpeg?w=360&amp;amp;q=90" /&gt; WKND Market Vol. 6 di Pantai Indah Kapuk 2 hadir 6-8 November 2026. Nikmati belanja produk lokal, workshop kreatif, olahraga,</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/03/09/harga-minyak-mentah-hampir-us110-dunia-dilanda-kepanikan-1773053712369_169.jpeg?w=360&amp;amp;q=90" /&gt; Menko Hilirisasi dan Transisi Energi Bahlil Lahadalia menyinggung adanya ketagangan antar negara yang terjadi di ASEAN karena harg</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8726851/nikmati-akhir-pekan-di-wknd-market-pik2-bisa-belanja-hingga-ikut-workshop</t>
+          <t>https://finance.detik.com/energi/d-8728338/bahlil-singgung-ada-ketegangan-di-asean-gegara-harga-minyak-mahal</t>
         </is>
       </c>
     </row>
@@ -2076,22 +2100,22 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Proyek LNG Abadi Masela Ditargetkan Operasi 2029, Begini Progresnya</t>
+          <t>Rayakan Sumpah Pemuda, Ini Deretan Promo Spesial BRI di Merchant Favorit</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Tue, 27 Oct 2026 18:10:02 +0700</t>
+          <t>Wed, 28 Oct 2026 18:00:22 +0700</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/02/14/kepala-skk-migas-djoko-siswanto-1_169.jpeg?w=360&amp;amp;q=90" /&gt; INPEX Masela Ltd. selesaikan tahap FEED proyek LNG Abadi lebih cepat, proyek gas raksasa itu ditargetkan beroperasi paling cepat 2029.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/28/rayakan-sumpah-pemuda-ini-deretan-promo-spesial-bri-di-merchant-favorit-1793184016452_169.jpeg?w=360&amp;amp;q=90" /&gt; Rayakan Hari Sumpah Pemuda dengan Promo Spesial BRI! Nikmati cashback dan diskon menarik untuk kuliner, belanja, da</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8726688/proyek-lng-abadi-masela-ditargetkan-operasi-2029-begini-progresnya</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8728263/rayakan-sumpah-pemuda-ini-deretan-promo-spesial-bri-di-merchant-favorit</t>
         </is>
       </c>
     </row>
@@ -2103,22 +2127,22 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Bansos Digital Meluncur 10 November, 100 Juta Warga Bakal Terdaftar</t>
+          <t>Pertemuan ASCOPE ke-51 Sepakati Penguatan Kerja Sama Energi Regional</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Tue, 27 Oct 2026 17:50:31 +0700</t>
+          <t>Wed, 28 Oct 2026 17:58:16 +0700</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/27/pertemuan-ketua-den-dengan-menko-kumham-imipas-1793090271348_169.jpeg?w=360&amp;amp;q=90" /&gt; Dan kita harap nanti waktu roll out oleh Presiden tanggal 10 November itu sudah lebih 100 juta orang, kata Luhut.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/28/pertemuan-ascope-ke-51-sepakati-penguatan-kerja-sama-energi-regional-1793185034571_169.jpeg?w=360&amp;amp;q=90" /&gt; Pertamina menggelar pertemuan ASCOPE ke-51 untuk memperkuat kolaborasi energi regional. Fokus pada ketahanan energi da</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8726657/bansos-digital-meluncur-10-november-100-juta-warga-bakal-terdaftar</t>
+          <t>https://finance.detik.com/energi/d-8728300/pertemuan-ascope-ke-51-sepakati-penguatan-kerja-sama-energi-regional</t>
         </is>
       </c>
     </row>
@@ -2130,22 +2154,22 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>SMPN 2 Depok Berulang Kali Banjir, Disdik Siapkan Langkah Ini</t>
+          <t>KPK Periksa 4 Saksi soal Dugaan Imbalan Swasta di Kasus BNPB</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Wed, 28 Oct 2026 07:36:53 +0700</t>
+          <t>Wed, 28 Oct 2026 21:14:09 +0700</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Disdik Depok menyiapkan langkah jangka pendek dan menengah untuk mencegah banjir kembali merendam SMPN 2 Depok.</t>
+          <t>Penyidik KPK mendalami dugaan suap dan benturan kepentingan dalam proyek penanggulangan bencana di BNPB.</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8322781/smpn-2-depok-berulang-kali-banjir-disdik-siapkan-langkah-ini</t>
+          <t>https://www.liputan6.com/news/read/8323603/kpk-periksa-4-saksi-soal-dugaan-imbalan-swasta-di-kasus-bnpb</t>
         </is>
       </c>
     </row>
@@ -2157,22 +2181,22 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Frugal Living dan Melambatnya Daya Beli Kelas Menengah</t>
+          <t>Situasi Terkini Bundaran HI Usai Massa Demo Bubar</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Wed, 28 Oct 2026 07:06:02 +0700</t>
+          <t>Wed, 28 Oct 2026 21:01:25 +0700</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Data Mandiri Spending Index (MSI) terbaru September 2026, menangkap gejala adanya pelambatan tren belanja di masyarakat.</t>
+          <t>Pembukaan jalan dilakukan bertahap, memastikan kelancaran kendaraan.</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8322236/frugal-living-dan-melambatnya-daya-beli-kelas-menengah</t>
+          <t>https://www.liputan6.com/news/read/8323593/situasi-terkini-bundaran-hi-usai-massa-demo-bubar</t>
         </is>
       </c>
     </row>
@@ -2184,22 +2208,22 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Mengapa Orang Ber-IQ Tinggi Seperti Dwi Martono Bisa Bertindak Keji?</t>
+          <t>Kericuhan Pecah di DPRD DIY, Massa Berpakaian Hitam Bentrok dengan Polisi</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Wed, 28 Oct 2026 07:04:15 +0700</t>
+          <t>Wed, 28 Oct 2026 21:24:34 +0700</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Dwi menjadi sorotan publik setelah diduga membunuh istri sirinya, Dini Hardiyanti (30) dan anaknya di Madiun, Jawa Timur.</t>
+          <t>Massa terlibat bentrokan dengan polisi dan masyarakat sekitar yang membantu penjagaan.</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8322733/mengapa-orang-ber-iq-tinggi-seperti-dwi-martono-bisa-bertindak-keji</t>
+          <t>https://www.liputan6.com/news/read/8323607/kericuhan-pecah-di-dprd-diy-massa-berpakaian-hitam-bentrok-dengan-polisi</t>
         </is>
       </c>
     </row>
@@ -2211,22 +2235,22 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Demo BEM UI, Ini Tuntutan yang Dibawa</t>
+          <t>Momen Massa Demo Dibubarkan Berujung Ricuh di Imam Bonjol</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Wed, 28 Oct 2026 06:01:59 +0700</t>
+          <t>Wed, 28 Oct 2026 20:28:16 +0700</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Mahasiswa telah menghimpun berbagai keresahan masyarakat yang dinilai belum mendapat respons memadai dari pemerintah.</t>
+          <t>Polisi menembakkan gas air mata dan mengerahkan water cannon di Jalan Imam Bonjol, Jakarta Pusat. Massa aksi sebelumnya menyuarakan lima tuntutan, termasuk penetapan karhutla sebagai bencana nasional.</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8322753/demo-bem-ui-ini-tuntutan-yang-dibawa</t>
+          <t>https://www.liputan6.com/news/read/8323570/momen-massa-demo-dibubarkan-berujung-ricuh-di-imam-bonjol</t>
         </is>
       </c>
     </row>
@@ -2238,22 +2262,22 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Membidik Penyawer Ratusan Juta ke PCNU</t>
+          <t>KPK Geledah Bea Cukai Kudus dan PT Djarum, Sita Dokumen Elektronik</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Wed, 28 Oct 2026 06:00:56 +0700</t>
+          <t>Wed, 28 Oct 2026 20:00:34 +0700</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Dugaan praktik risywah dalam Muktamar ke-35 NU di Jombang menjadi sorotan.</t>
+          <t>Penggeledahan KPK ini menjadi bagian dari pengembangan penyidikan dugaan suap importasi barang.</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8322738/membidik-penyawer-ratusan-juta-ke-pcnu</t>
+          <t>https://www.liputan6.com/news/read/8323558/kpk-geledah-bea-cukai-kudus-dan-pt-djarum-sita-dokumen-elektronik</t>
         </is>
       </c>
     </row>
@@ -2265,22 +2289,22 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Lokasi Demo BEM UI, Hindari Jalan Ini</t>
+          <t>Bakom Sebut Aspirasi Mahasiswa Jadi Masukan Pemerintah</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Wed, 28 Oct 2026 05:51:22 +0700</t>
+          <t>Wed, 28 Oct 2026 20:44:26 +0700</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Aksi demo mahasiswa UI di Bundaran HI hari ini. Polisi siapkan rekayasa lalu lintas di sejumlah titik Jakarta.</t>
+          <t>Berbagai isu seperti lingkungan, ekonomi, dan pendidikan menjadi masukan penting bagi kebijakan pemerintah.</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8322759/lokasi-demo-bem-ui-hindari-jalan-ini</t>
+          <t>https://www.liputan6.com/news/read/8323550/bakom-sebut-aspirasi-mahasiswa-jadi-masukan-pemerintah</t>
         </is>
       </c>
     </row>
@@ -2292,22 +2316,22 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Ketika Cinta Dini Dibalas Pembunuhan Keji Dwi Martono</t>
+          <t>KPK Geledah Kantor Dinas PUPR Klaten, Sita Dokumen hingga Uang Tunai</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Wed, 28 Oct 2026 05:06:09 +0700</t>
+          <t>Wed, 28 Oct 2026 19:51:37 +0700</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Teka teki pembunuhan sadis Dini Hardiyanti (30) dan anak kandungnya, AGF (4) akhirnya terbongkar.</t>
+          <t>Penggeledahan kantor Dinas Pekerjaan Umum Dan Penataan Ruang (DPUPR) Kabupaten Klaten merupakan lanjutan</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8322710/ketika-cinta-dini-dibalas-pembunuhan-keji-dwi-martono</t>
+          <t>https://www.liputan6.com/news/read/8323549/kpk-geledah-kantor-dinas-pupr-klaten-sita-dokumen-hingga-uang-tunai</t>
         </is>
       </c>
     </row>
@@ -2319,22 +2343,22 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Demo 28 Oktober, Presiden KSPN Ajak Massa Jaga Persatuan Sesuai Sumpah Pemuda</t>
+          <t>KAI Minta Maaf Usai KRL Bablas Tak Berhenti di Stasiun Sudirman</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Wed, 28 Oct 2026 03:06:57 +0700</t>
+          <t>Wed, 28 Oct 2026 20:56:12 +0700</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Ristadi mengingatkan, aksi yang bertepatan dengan peringatan Hari Sumpah Pemuda itu perlu mengedepankan semangat persatuan</t>
+          <t>KAI Commuter Minta Maaf Usai KRL Bablas Tak Berhenti di Stasiun Sudirman</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8322689/demo-28-oktober-presiden-kspn-ajak-massa-jaga-persatuan-sesuai-sumpah-pemuda</t>
+          <t>https://www.liputan6.com/news/read/8323591/kai-minta-maaf-usai-krl-bablas-tak-berhenti-di-stasiun-sudirman</t>
         </is>
       </c>
     </row>
@@ -2346,22 +2370,22 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Ada Demo Hari Sumpah Pemuda di Jakarta, Hindari 4 Lokasi Ini</t>
+          <t>Momen Menlu Singapura Temui Prabowo di Hambalang</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Wed, 28 Oct 2026 00:57:38 +0700</t>
+          <t>Wed, 28 Oct 2026 19:34:47 +0700</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Polda Metro Jaya menyiapkan rekayasa lalu lintas secara situasional di sejumlah lokasi aksi.</t>
+          <t>Pertemuan tersebut berlangsung tertutup.</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8322734/ada-demo-hari-sumpah-pemuda-di-jakarta-hindari-4-lokasi-ini</t>
+          <t>https://www.liputan6.com/news/read/8323516/momen-menlu-singapura-temui-prabowo-di-hambalang</t>
         </is>
       </c>
     </row>
@@ -2373,22 +2397,22 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Alokasi Transfer Daerah Ditambah Jadi Rp 720 T</t>
+          <t>Daftar 20 Rute Transjakarta Terdampak Demonstrasi</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Wed, 28 Oct 2026 00:08:51 +0700</t>
+          <t>Wed, 28 Oct 2026 19:17:52 +0700</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Menkeu Suahasil Tambah Alokasi Transfer Daerah Rp 720 T</t>
+          <t>. Transjakarta menyesuaikan operasional sejumlah rute akibat demonstrasi di Jakarta pada Rabu malam.</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8322727/alokasi-transfer-daerah-ditambah-jadi-rp-720-t</t>
+          <t>https://www.liputan6.com/news/read/8323505/daftar-20-rute-transjakarta-terdampak-demonstrasi</t>
         </is>
       </c>
     </row>
@@ -2400,22 +2424,22 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Menkeu dan Mendagri Bahas Anggaran Bencana hingga Insentif Daerah</t>
+          <t>KRL Bablas Tak Berhenti di Stasiun Sudirman, Masinis Diperiksa</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Tue, 27 Oct 2026 23:54:57 +0700</t>
+          <t>Wed, 28 Oct 2026 19:19:07 +0700</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Kemenkeu dan Kemendagri menyelaraskan APBN dan APBD agar program penanganan bencana.</t>
+          <t>Akibat kejadian ini, penumpang KRL yang hendak turun di Stasiun Sudirman melanjutkan perjalanan hingga Stasiun Manggarai.</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8322721/menkeu-dan-mendagri-bahas-anggaran-bencana-hingga-insentif-daerah</t>
+          <t>https://www.liputan6.com/news/read/8323509/krl-bablas-tak-berhenti-di-stasiun-sudirman-masinis-diperiksa</t>
         </is>
       </c>
     </row>
@@ -2427,22 +2451,22 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Rumput JIS Dikritik Shin Tae-yong dan Rizky Ridho, Pramono Buka Suara</t>
+          <t>19 Orang Terlibat Tawuran Maut di Kebon Jeruk Ditangkap</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Tue, 27 Oct 2026 23:37:17 +0700</t>
+          <t>Wed, 28 Oct 2026 19:00:02 +0700</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Gubernur DKI Jakarta Pramono Anung mengakui kondisi rumput JIS masih belum sempurna</t>
+          <t>Polisi mengidentifikasi empat orang yang diduga menjadi pelaku utama dalam tawuran maut di Kebon Jeruk.</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8322714/rumput-jis-dikritik-shin-tae-yong-dan-rizky-ridho-pramono-buka-suara</t>
+          <t>https://www.liputan6.com/news/read/8323484/19-orang-terlibat-tawuran-maut-di-kebon-jeruk-ditangkap</t>
         </is>
       </c>
     </row>
@@ -2454,22 +2478,22 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>265 Sekolah Rakyat Berdiri, Seskab Teddy: 45 Ribu Anak Jalanan Kembali Bersekolah</t>
+          <t>Fakta Sopir BYD Lindas Ojol di Jaksel: Kelelahan Sampai Ketiduran Kejar Setoran</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Tue, 27 Oct 2026 23:00:36 +0700</t>
+          <t>Wed, 28 Oct 2026 20:44:12 +0700</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Sekolah Rakyat tidak hanya menyediakan ruang belajar, tetapi juga menghadirkan lingkungan yang mendukung tumbuh kembang.</t>
+          <t>Dari hasil penyelidikan, terungkap bahwa sopir BYD yang lindas ojol ternyata juga driver Gojek yang ketiduran karena kelelahan.</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8322700/265-sekolah-rakyat-berdiri-seskab-teddy-45-ribu-anak-jalanan-kembali-bersekolah</t>
+          <t>https://www.liputan6.com/news/read/8323583/fakta-sopir-byd-lindas-ojol-di-jaksel-kelelahan-sampai-ketiduran-kejar-setoran</t>
         </is>
       </c>
     </row>
@@ -2481,22 +2505,22 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Tersangka Penyerang Bobotoh di Bogor Bukan Anggota Kelompok Suporter</t>
+          <t>Pemulihan Pascabencana Sumatera: Jalan Nasional Pulih, Huntap Terus Dibangun</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Tue, 27 Oct 2026 22:54:43 +0700</t>
+          <t>Wed, 28 Oct 2026 18:51:07 +0700</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Polisi telah mengamankan tersangka yang diduga melakukan penyerangan hingga menyebabkan suporter meninggal.</t>
+          <t>Selain penyediaan hunian sementara, pemerintah melanjutkan pembangunan hunian tetap bagi warga yang rumahnya rusak berat atau hilang akibat bencana.</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8322698/tersangka-penyerang-bobotoh-di-bogor-bukan-anggota-kelompok-suporter</t>
+          <t>https://www.liputan6.com/news/read/8323478/pemulihan-pascabencana-sumatera-jalan-nasional-pulih-huntap-terus-dibangun</t>
         </is>
       </c>
     </row>
@@ -2508,22 +2532,22 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Nasib Obligasi Jakarta Usai Pramono Bertemu Menkeu</t>
+          <t>Puan Minta Generasi Muda Diberi Ruang Ikut Tentukan Kebijakan dan Arah Bangsa</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Tue, 27 Oct 2026 22:21:46 +0700</t>
+          <t>Wed, 28 Oct 2026 18:09:36 +0700</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Pemprov DKI Jakarta akan mengikuti keputusan pemerintah pusat.</t>
+          <t>Pengalaman anak muda harus menjadi bahan pertimbangan dalam pengambilan keputusan negara.</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8322673/nasib-obligasi-jakarta-usai-pramono-bertemu-menkeu</t>
+          <t>https://www.liputan6.com/news/read/8323443/puan-minta-generasi-muda-diberi-ruang-ikut-tentukan-kebijakan-dan-arah-bangsa</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data pasar & berita - 2026-10-29 01:19 UTC
</commit_message>
<xml_diff>
--- a/data/market_news_latest.xlsx
+++ b/data/market_news_latest.xlsx
@@ -487,20 +487,20 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>5282.312</v>
+        <v>5266.1299</v>
       </c>
       <c r="F2" t="n">
-        <v>16.1821</v>
+        <v>-106.9644</v>
       </c>
       <c r="G2" t="n">
-        <v>0.31</v>
+        <v>-1.99</v>
       </c>
       <c r="H2" t="n">
-        <v>0</v>
+        <v>331730400</v>
       </c>
     </row>
     <row r="3">
@@ -525,16 +525,16 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>7728.4302</v>
+        <v>7743.98</v>
       </c>
       <c r="F3" t="n">
-        <v>5.8301</v>
+        <v>21.3799</v>
       </c>
       <c r="G3" t="n">
-        <v>0.08</v>
+        <v>0.28</v>
       </c>
       <c r="H3" t="n">
-        <v>653802820</v>
+        <v>3085116000</v>
       </c>
     </row>
     <row r="4">
@@ -559,16 +559,16 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>52471.5781</v>
+        <v>52475.1016</v>
       </c>
       <c r="F4" t="n">
-        <v>94.0078</v>
+        <v>97.5312</v>
       </c>
       <c r="G4" t="n">
-        <v>0.18</v>
+        <v>0.19</v>
       </c>
       <c r="H4" t="n">
-        <v>84875450</v>
+        <v>405081041</v>
       </c>
     </row>
     <row r="5">
@@ -593,16 +593,16 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>26437.6289</v>
+        <v>26549.8516</v>
       </c>
       <c r="F5" t="n">
-        <v>-40.1816</v>
+        <v>72.041</v>
       </c>
       <c r="G5" t="n">
-        <v>-0.15</v>
+        <v>0.27</v>
       </c>
       <c r="H5" t="n">
-        <v>2518702000</v>
+        <v>7142936000</v>
       </c>
     </row>
     <row r="6">
@@ -623,17 +623,17 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>63954.1914</v>
+        <v>64738.4297</v>
       </c>
       <c r="F6" t="n">
-        <v>685.8203</v>
+        <v>1470.0586</v>
       </c>
       <c r="G6" t="n">
-        <v>1.08</v>
+        <v>2.32</v>
       </c>
       <c r="H6" t="n">
         <v>0</v>
@@ -657,20 +657,20 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>23094.8301</v>
+        <v>23041.3203</v>
       </c>
       <c r="F7" t="n">
-        <v>53.5098</v>
+        <v>-170.4902</v>
       </c>
       <c r="G7" t="n">
-        <v>0.23</v>
+        <v>-0.73</v>
       </c>
       <c r="H7" t="n">
-        <v>0</v>
+        <v>2842500000</v>
       </c>
     </row>
     <row r="8">
@@ -694,15 +694,9 @@
           <t>2026-10-28</t>
         </is>
       </c>
-      <c r="E8" t="n">
-        <v>3681.469</v>
-      </c>
-      <c r="F8" t="n">
-        <v>33.168</v>
-      </c>
-      <c r="G8" t="n">
-        <v>0.91</v>
-      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
       <c r="H8" t="n">
         <v>412609940</v>
       </c>
@@ -725,20 +719,20 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>10698.0801</v>
+        <v>10686.5</v>
       </c>
       <c r="F9" t="n">
-        <v>11.5801</v>
+        <v>-80.7998</v>
       </c>
       <c r="G9" t="n">
-        <v>0.11</v>
+        <v>-0.75</v>
       </c>
       <c r="H9" t="n">
-        <v>0</v>
+        <v>529948000</v>
       </c>
     </row>
     <row r="10">
@@ -759,20 +753,20 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>25684.5195</v>
+        <v>25590.7695</v>
       </c>
       <c r="F10" t="n">
-        <v>93.75</v>
+        <v>179.9297</v>
       </c>
       <c r="G10" t="n">
-        <v>0.37</v>
+        <v>0.71</v>
       </c>
       <c r="H10" t="n">
-        <v>0</v>
+        <v>47576700</v>
       </c>
     </row>
     <row r="11">
@@ -793,17 +787,17 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>5397.9102</v>
+        <v>5412.8101</v>
       </c>
       <c r="F11" t="n">
-        <v>0.8804</v>
+        <v>15.7803</v>
       </c>
       <c r="G11" t="n">
-        <v>0.02</v>
+        <v>0.29</v>
       </c>
       <c r="H11" t="n">
         <v>0</v>
@@ -827,17 +821,17 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="E12" t="n">
         <v>18183</v>
       </c>
       <c r="F12" t="n">
-        <v>39</v>
+        <v>43.5</v>
       </c>
       <c r="G12" t="n">
-        <v>0.21</v>
+        <v>0.24</v>
       </c>
       <c r="H12" t="n">
         <v>0</v>
@@ -865,13 +859,13 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>102.376</v>
+        <v>102.257</v>
       </c>
       <c r="F13" t="n">
-        <v>0.056</v>
+        <v>-0.063</v>
       </c>
       <c r="G13" t="n">
-        <v>0.05</v>
+        <v>-0.06</v>
       </c>
       <c r="H13" t="n">
         <v>0</v>
@@ -895,17 +889,17 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>158.147</v>
+        <v>157.867</v>
       </c>
       <c r="F14" t="n">
-        <v>0.619</v>
+        <v>-0.126</v>
       </c>
       <c r="G14" t="n">
-        <v>0.39</v>
+        <v>-0.08</v>
       </c>
       <c r="H14" t="n">
         <v>0</v>
@@ -933,13 +927,13 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>0.5024</v>
+        <v>0.5044999999999999</v>
       </c>
       <c r="F15" t="n">
-        <v>0.0031</v>
+        <v>0.0052</v>
       </c>
       <c r="G15" t="n">
-        <v>0.62</v>
+        <v>1.04</v>
       </c>
       <c r="H15" t="n">
         <v>0</v>
@@ -967,13 +961,13 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>0.532</v>
+        <v>0.5361</v>
       </c>
       <c r="F16" t="n">
-        <v>0.0015</v>
+        <v>0.0056</v>
       </c>
       <c r="G16" t="n">
-        <v>0.28</v>
+        <v>1.06</v>
       </c>
       <c r="H16" t="n">
         <v>0</v>
@@ -1001,13 +995,13 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>0.4028</v>
+        <v>0.3995</v>
       </c>
       <c r="F17" t="n">
-        <v>-0.0012</v>
+        <v>-0.0045</v>
       </c>
       <c r="G17" t="n">
-        <v>-0.3</v>
+        <v>-1.11</v>
       </c>
       <c r="H17" t="n">
         <v>0</v>
@@ -1034,17 +1028,11 @@
           <t>2026-10-28</t>
         </is>
       </c>
-      <c r="E18" t="n">
-        <v>81.295</v>
-      </c>
-      <c r="F18" t="n">
-        <v>-0.335</v>
-      </c>
-      <c r="G18" t="n">
-        <v>-0.41</v>
-      </c>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
       <c r="H18" t="n">
-        <v>5234941</v>
+        <v>35072467</v>
       </c>
     </row>
     <row r="19">
@@ -1068,17 +1056,11 @@
           <t>2026-10-28</t>
         </is>
       </c>
-      <c r="E19" t="n">
-        <v>77.62</v>
-      </c>
-      <c r="F19" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="G19" t="n">
-        <v>0.03</v>
-      </c>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr"/>
       <c r="H19" t="n">
-        <v>18163774</v>
+        <v>65283700</v>
       </c>
     </row>
     <row r="20">
@@ -1103,16 +1085,16 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>4055.7</v>
+        <v>4058.1001</v>
       </c>
       <c r="F20" t="n">
-        <v>-18.9001</v>
+        <v>-16.5</v>
       </c>
       <c r="G20" t="n">
-        <v>-0.46</v>
+        <v>-0.4</v>
       </c>
       <c r="H20" t="n">
-        <v>68517</v>
+        <v>10619</v>
       </c>
     </row>
     <row r="21">
@@ -1137,16 +1119,16 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>102.6</v>
+        <v>101.99</v>
       </c>
       <c r="F21" t="n">
-        <v>2.7</v>
+        <v>2.09</v>
       </c>
       <c r="G21" t="n">
-        <v>2.7</v>
+        <v>2.09</v>
       </c>
       <c r="H21" t="n">
-        <v>131244</v>
+        <v>7344</v>
       </c>
     </row>
     <row r="22">
@@ -1171,16 +1153,16 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>112.02</v>
+        <v>110.69</v>
       </c>
       <c r="F22" t="n">
-        <v>-1.86</v>
+        <v>-3.19</v>
       </c>
       <c r="G22" t="n">
-        <v>-1.63</v>
+        <v>-2.8</v>
       </c>
       <c r="H22" t="n">
-        <v>22762</v>
+        <v>964</v>
       </c>
     </row>
     <row r="23">
@@ -1205,16 +1187,16 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>6.6585</v>
+        <v>6.6705</v>
       </c>
       <c r="F23" t="n">
-        <v>0.0365</v>
+        <v>0.0485</v>
       </c>
       <c r="G23" t="n">
-        <v>0.55</v>
+        <v>0.73</v>
       </c>
       <c r="H23" t="n">
-        <v>19153</v>
+        <v>1234</v>
       </c>
     </row>
     <row r="24">
@@ -1238,17 +1220,11 @@
           <t>2026-10-28</t>
         </is>
       </c>
-      <c r="E24" t="n">
-        <v>63.085</v>
-      </c>
-      <c r="F24" t="n">
-        <v>0.5649999999999999</v>
-      </c>
-      <c r="G24" t="n">
-        <v>0.9</v>
-      </c>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr"/>
       <c r="H24" t="n">
-        <v>4409947</v>
+        <v>23690945</v>
       </c>
     </row>
     <row r="25">
@@ -1273,13 +1249,13 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>17.35</v>
+        <v>16.91</v>
       </c>
       <c r="F25" t="n">
-        <v>-0.17</v>
+        <v>-0.61</v>
       </c>
       <c r="G25" t="n">
-        <v>-0.97</v>
+        <v>-3.48</v>
       </c>
       <c r="H25" t="n">
         <v>0</v>
@@ -1303,20 +1279,20 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="E26" t="n">
-        <v>80448.4375</v>
+        <v>80828.8906</v>
       </c>
       <c r="F26" t="n">
-        <v>-356.6406</v>
+        <v>23.8125</v>
       </c>
       <c r="G26" t="n">
-        <v>-0.44</v>
+        <v>0.03</v>
       </c>
       <c r="H26" t="n">
-        <v>22507993088</v>
+        <v>24155543552</v>
       </c>
     </row>
     <row r="27">
@@ -1749,22 +1725,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Pemda Bakal Lebih Sering Pelototi Pelaksanaan MBG</t>
+          <t>Forum ASCOPE Ke-51 Sepakat Perkuat Arsitektur Energi Masa Depan ASEAN</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Wed, 28 Oct 2026 21:30:00 +0700</t>
+          <t>Thu, 29 Oct 2026 08:07:51 +0700</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/20/penerima-manfaat-mbg-dalam-dua-tahun-pemerintahan-prabowo-1792479756724_169.jpeg?w=360&amp;amp;q=90" /&gt; Pengawasan pelaksanaan Makan Bergizi Gratis (MBG) bakal lebih banyak melibatkan pemerintah daerah.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/29/pertamina-1793236035812_169.jpeg?w=360&amp;amp;q=90" /&gt; Rangkaian 51st ASCOPE di Bali ditutup dengan kesepakatan strategis untuk ketahanan energi regional. Negara anggota berkomitmen menghadapi tantangan energi.</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8728569/pemda-bakal-lebih-sering-pelototi-pelaksanaan-mbg</t>
+          <t>https://finance.detik.com/energi/d-8728821/forum-ascope-ke-51-sepakat-perkuat-arsitektur-energi-masa-depan-asean</t>
         </is>
       </c>
     </row>
@@ -1776,22 +1752,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Berdayakan Masyarakat, MIND ID Raih Penghargaan Mandaya Awards 2026</t>
+          <t>Sederet Manfaat QRIS, Bikin Transaksi Usaha Jadi Praktis</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Wed, 28 Oct 2026 21:26:17 +0700</t>
+          <t>Thu, 29 Oct 2026 08:01:20 +0700</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/28/berdayakan-masyarakat-grup-mind-id-raih-penghargaan-mandaya-awards-2026-1793197151033_169.jpeg?w=360&amp;amp;q=90" /&gt; MIND ID meraih Anugerah Mandaya Award 2026 atas pemberdayaan masyarakat. Programnya fokus pada penguatan ekonomi da</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/28/qris-pakai-dana-1793170176586.png?w=360&amp;amp;q=90" /&gt; QRIS memudahkan transaksi digital di Indonesia dengan satu kode QR. Pengguna dan merchant dapat menikmati kemudahan, keamanan, dan kecepatan dalam pembayaran.</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8728601/berdayakan-masyarakat-mind-id-raih-penghargaan-mandaya-awards-2026</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8727735/sederet-manfaat-qris-bikin-transaksi-usaha-jadi-praktis</t>
         </is>
       </c>
     </row>
@@ -1803,22 +1779,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>8 Bos Sawit RI Menghadap Menteri Singapura, Ini Daftarnya</t>
+          <t>Pasar Modal Dibersihkan, Kepercayaan Investor Dipulihkan</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Wed, 28 Oct 2026 21:05:16 +0700</t>
+          <t>Thu, 29 Oct 2026 08:00:42 +0700</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/12/situasi-kabut-asap-di-singapura-pada-senin-1210-waktu-setempat-1791794641533_169.jpeg?w=360&amp;amp;q=90" /&gt; Delapan Petinggi perusahaan kelapa sawit besar di Indonesia memenuhi panggilan pejabat tinggi Singapura.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/16/ihsg-ambruk-1157-ditutup-di-level-5185-1792144638939_169.jpeg?w=360&amp;amp;q=90" /&gt; IHSG anjlok 6% setelah pengumuman MSCI, memicu panic selling di pasar. OJK dan BEI siapkan reformasi untuk meningkatkan transparansi dan likuiditas.</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/industri/d-8728582/8-bos-sawit-ri-menghadap-menteri-singapura-ini-daftarnya</t>
+          <t>https://finance.detik.com/bursa-dan-valas/d-8728651/pasar-modal-dibersihkan-kepercayaan-investor-dipulihkan</t>
         </is>
       </c>
     </row>
@@ -1830,22 +1806,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Dua Pintu Masuk Stasiun MRT Dukuh Atas Ditutup Sementara</t>
+          <t>The Fed Putuskan Tahan Suku Bunga</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Wed, 28 Oct 2026 20:11:26 +0700</t>
+          <t>Thu, 29 Oct 2026 07:39:08 +0700</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/17/penumpang-mrt-jakarta-1792229479640_169.jpeg?w=360&amp;amp;q=90" /&gt; Pintu masuk E dan C Stasiun MRT Dukuh Atas BNI masih ditutup sementara.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2023/02/02/bank-sentral-as-the-fed-naikkan-suku-bunga-sebesar-025-3_169.jpeg?w=360&amp;amp;q=90" /&gt; The Fed memilih untuk tidak terburu-buru mengubah suku bunga, meskipun tekanan inflasi masih sulit dikendalikan.</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/infrastruktur/d-8728516/dua-pintu-masuk-stasiun-mrt-dukuh-atas-ditutup-sementara</t>
+          <t>https://finance.detik.com/moneter/d-8728784/the-fed-putuskan-tahan-suku-bunga</t>
         </is>
       </c>
     </row>
@@ -1857,22 +1833,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Impor BBM Lewat Lemigas Cuma buat Produk yang Dijual Pertamina</t>
+          <t>Bos BRIN Lapor Prabowo Limbah Sawit Bisa Diolah Jadi Listrik</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Wed, 28 Oct 2026 19:30:05 +0700</t>
+          <t>Thu, 29 Oct 2026 07:30:00 +0700</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/14/bahlil-lahadalia-rolandodetikcom-1791978307056_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Bahlil menegaskan impor migas lewat Lemigas hanya untuk Pertamina, bukan swasta. Skema baru impor kini menggunakan G2G dan G2B.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/28/kepala-badan-riset-dan-inovasi-nasional-brin-arif-satria-1793120446935_169.jpeg?w=360&amp;amp;q=90" /&gt; Kepala Badan Riset dan Inovasi Nasional (BRIN) Arif Satria memberikan laporan kepada Presiden Prabowo Subianto soal limbah sawit m</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8728437/impor-bbm-lewat-lemigas-cuma-buat-produk-yang-dijual-pertamina</t>
+          <t>https://finance.detik.com/energi/d-8728654/bos-brin-lapor-prabowo-limbah-sawit-bisa-diolah-jadi-listrik</t>
         </is>
       </c>
     </row>
@@ -1884,22 +1860,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Panen Zaitun Warga Kurdi di Tengah Krisis Ekonomi</t>
+          <t>Terbang Makin Hemat, Tarif Penumpang Pesawat di Bandara Samrat Turun 50 Persen</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Wed, 28 Oct 2026 19:04:16 +0700</t>
+          <t>Thu, 29 Oct 2026 07:15:43 +0700</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/28/panen-zaitun-warga-kurdi-di-tengah-krisis-ekonomi-1793170558501.jpeg?w=360&amp;amp;q=90" /&gt; Petani memanen zaitun di Afrin, Suriah, di tengah keterbatasan air, kenaikan biaya produksi, dan rendahnya harga jual.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/28/terbang-makin-hemat-tarif-penumpang-pesawat-di-bandara-samrat-turun-50-persen-1793188717765_169.jpeg?w=360&amp;amp;q=90" /&gt; Kabar baik, Bandara Sam Ratulangi Manado memangkas tarif jasa penumpang pesawat 50 persen hingga 10 Januari 2</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/foto-bisnis/d-8727752/panen-zaitun-warga-kurdi-di-tengah-krisis-ekonomi</t>
+          <t>https://finance.detik.com/foto-bisnis/d-8728409/terbang-makin-hemat-tarif-penumpang-pesawat-di-bandara-samrat-turun-50-persen</t>
         </is>
       </c>
     </row>
@@ -1911,22 +1887,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Mentan Jamin Harga Beras Turun Usai Mafia Oplosan Dibongkar!</t>
+          <t>Pertama dalam Sejarah Pasar Modal RI, BEI Bagi-bagi Dividen</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Wed, 28 Oct 2026 19:02:09 +0700</t>
+          <t>Thu, 29 Oct 2026 07:00:00 +0700</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/28/mentan-ungkap-praktik-beras-oplosan-1793173274624_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Pertanian Andi Amran Sulaiman jamin penindakan pengoplosan beras SPHP dapat turunkan harga beras.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2016/05/03/1fb20055-d8fe-4f7f-bf42-445d369dc61a_169.jpg?w=360&amp;amp;q=90" /&gt; Bursa Efek Indonesia (BEI) akan bagi-bagi dividen tunai pertamanya dalam sejarah, totalnya Rp 1,56 triliun.</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8728410/mentan-jamin-harga-beras-turun-usai-mafia-oplosan-dibongkar</t>
+          <t>https://finance.detik.com/bursa-dan-valas/d-8728605/pertama-dalam-sejarah-pasar-modal-ri-bei-bagi-bagi-dividen</t>
         </is>
       </c>
     </row>
@@ -1938,22 +1914,22 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>RI Dapat Pasokan Minyak 30 Juta Barel dari UEA? Bahlil: Masih Penjajakan</t>
+          <t>Kenapa Harga Tiket Pesawat Saat Nataru Bisa Turun 12%?</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Wed, 28 Oct 2026 18:40:06 +0700</t>
+          <t>Thu, 29 Oct 2026 06:30:57 +0700</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/03/10/menteri-esdm-bahlil-lahadalia-1773134823836_169.jpeg?w=360&amp;amp;q=90" /&gt; Menko Hilirisasi dan Transisi Energi Bahlil Lahadalia buka suara soal potensi pasokan minyak mentah 30 juta dari Uni Emirat Arab (UEA).</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/05/15/maskapai-diberikan-keleluasaan-tentukan-tarif-tiket-1778834393575_169.jpeg?w=360&amp;amp;q=90" /&gt; Harga tiket pesawat kelas ekonomi domestik berpotensi turun hingga 12% selama periode libur Natal 2026 dan Tahun Baru 2027 (Nataru).</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8728371/ri-dapat-pasokan-minyak-30-juta-barel-dari-uea-bahlil-masih-penjajakan</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8728369/kenapa-harga-tiket-pesawat-saat-nataru-bisa-turun-12</t>
         </is>
       </c>
     </row>
@@ -1965,22 +1941,22 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Mentan Minta Bulog Serap Jagung Petani Sesuai Aturan</t>
+          <t>Simak! Begini Cara Ajukan Bebas Denda Pajak</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Wed, 28 Oct 2026 18:34:32 +0700</t>
+          <t>Thu, 29 Oct 2026 05:55:41 +0700</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/07/28/wawancara-khusus-menteri-pertanian-ri-andi-amran-sulaiman-1753687994517_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Pertanian (Mentan) sekaligus Kepala Badan Pangan Nasional (Bapanas) Andi Amran Sulaiman meminta Perum Bulog tidak menolak</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2014/10/01/aba994a2-34ed-467e-b236-0838b109f70c_169.jpg?w=360&amp;amp;q=90" /&gt; Wajib pajak dapat ajukan pengurangan atau penghapusan denda pajak hingga 1 Oktober 2028. Ikuti langkah-langkah di Coretax untuk permohonan.</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8728357/mentan-minta-bulog-serap-jagung-petani-sesuai-aturan</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8728372/simak-begini-cara-ajukan-bebas-denda-pajak</t>
         </is>
       </c>
     </row>
@@ -1992,22 +1968,22 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Menperin Ungkap Keresahan Pengusaha soal Isu Pencabutan Bea Keluar Emas</t>
+          <t>Sempat Mangkrak, Proyek Pengembangan Pasar Senen Blok VI Jalan Lagi</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Wed, 28 Oct 2026 18:30:12 +0700</t>
+          <t>Wed, 28 Oct 2026 22:48:45 +0700</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/28/menteri-perindustrian-menperin-muhammad-sarmuji-1793178348200_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Perindustrian (Menperin) Muhammad Sarmuji mengungkapkan keresahan pengusaha perhiasan terkait rumor pencabutan bea keluar bahan bak</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/28/gambar-rencana-pengembangan-pasar-senen-blok-vi-1793202449109_169.jpeg?w=360&amp;amp;q=90" /&gt; Proyek pengembangan Pasar Senen Blok VI, Jakarta Pusat kembali berjalan, setelah sempat mangkrak.</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/industri/d-8728353/menperin-ungkap-keresahan-pengusaha-soal-isu-pencabutan-bea-keluar-emas</t>
+          <t>https://finance.detik.com/infrastruktur/d-8728665/sempat-mangkrak-proyek-pengembangan-pasar-senen-blok-vi-jalan-lagi</t>
         </is>
       </c>
     </row>
@@ -2019,22 +1995,22 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>KKP Dampingi Pemda Jamin Pembangunan KNMP Sesuai Rencana Tata Ruang</t>
+          <t>Pemda Bakal Lebih Sering Pelototi Pelaksanaan MBG</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Wed, 28 Oct 2026 18:27:07 +0700</t>
+          <t>Wed, 28 Oct 2026 21:30:00 +0700</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/28/kkp-dukung-pemda-jamin-pembangunan-knmp-sesuai-rencana-tata-ruang-1793186771621.jpeg?w=360&amp;amp;q=90" /&gt; Kementerian Kelautan dan Perikanan RI memastikan pembangunan Kampung Nelayan Merah Putih sesuai tata ruang. KKP dukung pemda </t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/20/penerima-manfaat-mbg-dalam-dua-tahun-pemerintahan-prabowo-1792479756724_169.jpeg?w=360&amp;amp;q=90" /&gt; Pengawasan pelaksanaan Makan Bergizi Gratis (MBG) bakal lebih banyak melibatkan pemerintah daerah.</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8728351/kkp-dampingi-pemda-jamin-pembangunan-knmp-sesuai-rencana-tata-ruang</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8728569/pemda-bakal-lebih-sering-pelototi-pelaksanaan-mbg</t>
         </is>
       </c>
     </row>
@@ -2046,22 +2022,22 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Shopee Buka Rute Ekspor Baru ke 4 Negara Lewat Program FLEXI</t>
+          <t>Berdayakan Masyarakat, MIND ID Raih Penghargaan Mandaya Awards 2026</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Wed, 28 Oct 2026 18:22:53 +0700</t>
+          <t>Wed, 28 Oct 2026 21:26:17 +0700</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/28/shopee-buka-rute-ekspor-baru-ke-4-negara-lewat-program-flexi-1793186505123_169.jpeg?w=360&amp;amp;q=90" /&gt; Shopee luncurkan Program Jalan Global Kreasi Lokal, memperluas ekspor ke Singapura, Thailand, Filipina, dan Brunei. Penjual da</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/28/berdayakan-masyarakat-grup-mind-id-raih-penghargaan-mandaya-awards-2026-1793197151033_169.jpeg?w=360&amp;amp;q=90" /&gt; MIND ID meraih Anugerah Mandaya Award 2026 atas pemberdayaan masyarakat. Programnya fokus pada penguatan ekonomi da</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8728345/shopee-buka-rute-ekspor-baru-ke-4-negara-lewat-program-flexi</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8728601/berdayakan-masyarakat-mind-id-raih-penghargaan-mandaya-awards-2026</t>
         </is>
       </c>
     </row>
@@ -2073,22 +2049,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Bahlil Singgung Ada Ketegangan di ASEAN Gegara Harga Minyak Mahal</t>
+          <t>8 Bos Sawit RI Menghadap Menteri Singapura, Ini Daftarnya</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Wed, 28 Oct 2026 18:18:22 +0700</t>
+          <t>Wed, 28 Oct 2026 21:05:16 +0700</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/03/09/harga-minyak-mentah-hampir-us110-dunia-dilanda-kepanikan-1773053712369_169.jpeg?w=360&amp;amp;q=90" /&gt; Menko Hilirisasi dan Transisi Energi Bahlil Lahadalia menyinggung adanya ketagangan antar negara yang terjadi di ASEAN karena harg</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/12/situasi-kabut-asap-di-singapura-pada-senin-1210-waktu-setempat-1791794641533_169.jpeg?w=360&amp;amp;q=90" /&gt; Delapan Petinggi perusahaan kelapa sawit besar di Indonesia memenuhi panggilan pejabat tinggi Singapura.</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8728338/bahlil-singgung-ada-ketegangan-di-asean-gegara-harga-minyak-mahal</t>
+          <t>https://finance.detik.com/industri/d-8728582/8-bos-sawit-ri-menghadap-menteri-singapura-ini-daftarnya</t>
         </is>
       </c>
     </row>
@@ -2100,22 +2076,22 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Rayakan Sumpah Pemuda, Ini Deretan Promo Spesial BRI di Merchant Favorit</t>
+          <t>Dua Pintu Masuk Stasiun MRT Dukuh Atas Ditutup Sementara</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Wed, 28 Oct 2026 18:00:22 +0700</t>
+          <t>Wed, 28 Oct 2026 20:11:26 +0700</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/28/rayakan-sumpah-pemuda-ini-deretan-promo-spesial-bri-di-merchant-favorit-1793184016452_169.jpeg?w=360&amp;amp;q=90" /&gt; Rayakan Hari Sumpah Pemuda dengan Promo Spesial BRI! Nikmati cashback dan diskon menarik untuk kuliner, belanja, da</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/17/penumpang-mrt-jakarta-1792229479640_169.jpeg?w=360&amp;amp;q=90" /&gt; Pintu masuk E dan C Stasiun MRT Dukuh Atas BNI masih ditutup sementara.</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8728263/rayakan-sumpah-pemuda-ini-deretan-promo-spesial-bri-di-merchant-favorit</t>
+          <t>https://finance.detik.com/infrastruktur/d-8728516/dua-pintu-masuk-stasiun-mrt-dukuh-atas-ditutup-sementara</t>
         </is>
       </c>
     </row>
@@ -2127,22 +2103,22 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Pertemuan ASCOPE ke-51 Sepakati Penguatan Kerja Sama Energi Regional</t>
+          <t>Impor BBM Lewat Lemigas Cuma buat Produk yang Dijual Pertamina</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Wed, 28 Oct 2026 17:58:16 +0700</t>
+          <t>Wed, 28 Oct 2026 19:30:05 +0700</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/28/pertemuan-ascope-ke-51-sepakati-penguatan-kerja-sama-energi-regional-1793185034571_169.jpeg?w=360&amp;amp;q=90" /&gt; Pertamina menggelar pertemuan ASCOPE ke-51 untuk memperkuat kolaborasi energi regional. Fokus pada ketahanan energi da</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/14/bahlil-lahadalia-rolandodetikcom-1791978307056_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Bahlil menegaskan impor migas lewat Lemigas hanya untuk Pertamina, bukan swasta. Skema baru impor kini menggunakan G2G dan G2B.</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8728300/pertemuan-ascope-ke-51-sepakati-penguatan-kerja-sama-energi-regional</t>
+          <t>https://finance.detik.com/energi/d-8728437/impor-bbm-lewat-lemigas-cuma-buat-produk-yang-dijual-pertamina</t>
         </is>
       </c>
     </row>
@@ -2154,22 +2130,22 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>KPK Periksa 4 Saksi soal Dugaan Imbalan Swasta di Kasus BNPB</t>
+          <t>Eks Wamen Imipas Silmy Karim Jalani Sidang Perdana Hari Ini</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Wed, 28 Oct 2026 21:14:09 +0700</t>
+          <t>Thu, 29 Oct 2026 07:57:27 +0700</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Penyidik KPK mendalami dugaan suap dan benturan kepentingan dalam proyek penanggulangan bencana di BNPB.</t>
+          <t>Mantan Wamen Imipas Silmy Karim menjalani sidang perdana kasus dugaan pemerasan dan gratifikasi izin tinggal WNA.</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8323603/kpk-periksa-4-saksi-soal-dugaan-imbalan-swasta-di-kasus-bnpb</t>
+          <t>https://www.liputan6.com/news/read/8323752/eks-wamen-imipas-silmy-karim-jalani-sidang-perdana-hari-ini</t>
         </is>
       </c>
     </row>
@@ -2181,22 +2157,22 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Situasi Terkini Bundaran HI Usai Massa Demo Bubar</t>
+          <t>Siasat Dwi Martono Hilangkan Jejak Pembunuhan Istri dan Balita</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Wed, 28 Oct 2026 21:01:25 +0700</t>
+          <t>Thu, 29 Oct 2026 06:03:42 +0700</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Pembukaan jalan dilakukan bertahap, memastikan kelancaran kendaraan.</t>
+          <t>Dwi menyiapkan berbagai cara dan peralatan untuk menghilangkan jejak pembunuhan terhadap kedua korban.</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8323593/situasi-terkini-bundaran-hi-usai-massa-demo-bubar</t>
+          <t>https://www.liputan6.com/news/read/8323679/siasat-dwi-martono-hilangkan-jejak-pembunuhan-istri-dan-balita</t>
         </is>
       </c>
     </row>
@@ -2208,22 +2184,22 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Kericuhan Pecah di DPRD DIY, Massa Berpakaian Hitam Bentrok dengan Polisi</t>
+          <t>Gempa Magnitudo 6,4 Guncang Tanimbar Maluku</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Wed, 28 Oct 2026 21:24:34 +0700</t>
+          <t>Thu, 29 Oct 2026 05:33:07 +0700</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Massa terlibat bentrokan dengan polisi dan masyarakat sekitar yang membantu penjagaan.</t>
+          <t>Gempa bumi berkekuatan Magnitudo 6,4 terjadi di 201 km BaratLaut Tanimbar, tidak berpotensi tsunami.</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8323607/kericuhan-pecah-di-dprd-diy-massa-berpakaian-hitam-bentrok-dengan-polisi</t>
+          <t>https://www.liputan6.com/news/read/8323703/gempa-magnitudo-64-guncang-tanimbar-maluku</t>
         </is>
       </c>
     </row>
@@ -2235,22 +2211,22 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Momen Massa Demo Dibubarkan Berujung Ricuh di Imam Bonjol</t>
+          <t>100 Hari MBG di Tangan Sudaryono</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Wed, 28 Oct 2026 20:28:16 +0700</t>
+          <t>Thu, 29 Oct 2026 05:00:10 +0700</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Polisi menembakkan gas air mata dan mengerahkan water cannon di Jalan Imam Bonjol, Jakarta Pusat. Massa aksi sebelumnya menyuarakan lima tuntutan, termasuk penetapan karhutla sebagai bencana nasional.</t>
+          <t>Selama 100 hari memimpin BGN, Sudaryono mengeluarkan sejumlah kebijakan pembenahan program MBG.</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8323570/momen-massa-demo-dibubarkan-berujung-ricuh-di-imam-bonjol</t>
+          <t>https://www.liputan6.com/news/read/8323694/100-hari-mbg-di-tangan-sudaryono</t>
         </is>
       </c>
     </row>
@@ -2262,22 +2238,22 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>KPK Geledah Bea Cukai Kudus dan PT Djarum, Sita Dokumen Elektronik</t>
+          <t>Update Kericuhan Demo DIY, Massa Bentrok Lagi dengan Polisi di Tugu Yogyakarta</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Wed, 28 Oct 2026 20:00:34 +0700</t>
+          <t>Thu, 29 Oct 2026 01:26:40 +0700</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Penggeledahan KPK ini menjadi bagian dari pengembangan penyidikan dugaan suap importasi barang.</t>
+          <t>Massa ricuh masih melakukan aksi pelemparan batu dan menembakkan kembang api.</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8323558/kpk-geledah-bea-cukai-kudus-dan-pt-djarum-sita-dokumen-elektronik</t>
+          <t>https://www.liputan6.com/news/read/8323690/update-kericuhan-demo-diy-massa-bentrok-lagi-dengan-polisi-di-tugu-yogyakarta</t>
         </is>
       </c>
     </row>
@@ -2289,22 +2265,22 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Bakom Sebut Aspirasi Mahasiswa Jadi Masukan Pemerintah</t>
+          <t>Kronologi Demo Sumpah Pemuda di Yogyakarta Berujung Ricuh</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Wed, 28 Oct 2026 20:44:26 +0700</t>
+          <t>Thu, 29 Oct 2026 01:21:18 +0700</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Berbagai isu seperti lingkungan, ekonomi, dan pendidikan menjadi masukan penting bagi kebijakan pemerintah.</t>
+          <t>Konsentrasi massa terbagi di sisi selatan dan utara gedung DPRD.</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8323550/bakom-sebut-aspirasi-mahasiswa-jadi-masukan-pemerintah</t>
+          <t>https://www.liputan6.com/news/read/8323689/kronologi-demo-sumpah-pemuda-di-yogyakarta-berujung-ricuh</t>
         </is>
       </c>
     </row>
@@ -2316,22 +2292,22 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>KPK Geledah Kantor Dinas PUPR Klaten, Sita Dokumen hingga Uang Tunai</t>
+          <t>Sektor Kelistrikan Bidik Hidrogen dan Amonia untuk Tekan Emisi</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Wed, 28 Oct 2026 19:51:37 +0700</t>
+          <t>Thu, 29 Oct 2026 01:02:20 +0700</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Penggeledahan kantor Dinas Pekerjaan Umum Dan Penataan Ruang (DPUPR) Kabupaten Klaten merupakan lanjutan</t>
+          <t>Pengujian hidrogen dan amonia di Bali dan Banten menunjukkan potensi pengurangan emisi sekaligus penghematan bahan bakar fosil.</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8323549/kpk-geledah-kantor-dinas-pupr-klaten-sita-dokumen-hingga-uang-tunai</t>
+          <t>https://www.liputan6.com/news/read/8323684/sektor-kelistrikan-bidik-hidrogen-dan-amonia-untuk-tekan-emisi</t>
         </is>
       </c>
     </row>
@@ -2343,22 +2319,22 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>KAI Minta Maaf Usai KRL Bablas Tak Berhenti di Stasiun Sudirman</t>
+          <t>Mabes Polri: Terima Kasih Massa Aksi, Demo Sumpah Pemuda Tertib dan Damai</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Wed, 28 Oct 2026 20:56:12 +0700</t>
+          <t>Wed, 28 Oct 2026 23:48:02 +0700</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>KAI Commuter Minta Maaf Usai KRL Bablas Tak Berhenti di Stasiun Sudirman</t>
+          <t>Polri mengatakan, situasi yang aman dan kondusif terwujud berkat kerja sama masyarakat dan kepolisian.</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8323591/kai-minta-maaf-usai-krl-bablas-tak-berhenti-di-stasiun-sudirman</t>
+          <t>https://www.liputan6.com/news/read/8323668/mabes-polri-terima-kasih-massa-aksi-demo-sumpah-pemuda-tertib-dan-damai</t>
         </is>
       </c>
     </row>
@@ -2370,22 +2346,22 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Momen Menlu Singapura Temui Prabowo di Hambalang</t>
+          <t>Respons PT Djarum soal Penggeledahan KPK</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Wed, 28 Oct 2026 19:34:47 +0700</t>
+          <t>Wed, 28 Oct 2026 22:50:39 +0700</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Pertemuan tersebut berlangsung tertutup.</t>
+          <t>PT Djarum akan bersikap kooperatif membantu mengusut dugaan korupsi yang sedang didalami KPK.</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8323516/momen-menlu-singapura-temui-prabowo-di-hambalang</t>
+          <t>https://www.liputan6.com/news/read/8323644/respons-pt-djarum-soal-penggeledahan-kpk</t>
         </is>
       </c>
     </row>
@@ -2397,22 +2373,22 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Daftar 20 Rute Transjakarta Terdampak Demonstrasi</t>
+          <t>Infografis: 10 Negara Termiskin di Asia</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Wed, 28 Oct 2026 19:17:52 +0700</t>
+          <t>Wed, 28 Oct 2026 22:33:49 +0700</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>. Transjakarta menyesuaikan operasional sejumlah rute akibat demonstrasi di Jakarta pada Rabu malam.</t>
+          <t>Dari Afghanistan hingga Bangladesh, berikut 10 negara Asia dengan PDB per kapita terendah.</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8323505/daftar-20-rute-transjakarta-terdampak-demonstrasi</t>
+          <t>https://www.liputan6.com/news/read/8323635/infografis-10-negara-termiskin-di-asia</t>
         </is>
       </c>
     </row>
@@ -2424,22 +2400,22 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>KRL Bablas Tak Berhenti di Stasiun Sudirman, Masinis Diperiksa</t>
+          <t>Kepala BGN Usul Pelajaran Gizi di Sekolah Lewat MBG</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Wed, 28 Oct 2026 19:19:07 +0700</t>
+          <t>Wed, 28 Oct 2026 21:57:08 +0700</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Akibat kejadian ini, penumpang KRL yang hendak turun di Stasiun Sudirman melanjutkan perjalanan hingga Stasiun Manggarai.</t>
+          <t>Kepala BGN Sudaryono mendorong edukasi gizi masuk kurikulum sekolah melalui program MBG.</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8323509/krl-bablas-tak-berhenti-di-stasiun-sudirman-masinis-diperiksa</t>
+          <t>https://www.liputan6.com/news/read/8323620/kepala-bgn-usul-pelajaran-gizi-di-sekolah-lewat-mbg</t>
         </is>
       </c>
     </row>
@@ -2451,22 +2427,22 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>19 Orang Terlibat Tawuran Maut di Kebon Jeruk Ditangkap</t>
+          <t>Suasana Ricuh Demo Sumpah Pemuda di Kawasan Dukuh Atas</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Wed, 28 Oct 2026 19:00:02 +0700</t>
+          <t>Wed, 28 Oct 2026 21:56:34 +0700</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Polisi mengidentifikasi empat orang yang diduga menjadi pelaku utama dalam tawuran maut di Kebon Jeruk.</t>
+          <t>Aksi demonstrasi memperingati Hari Sumpah Pemuda yang digelar Badan Eksekutif Mahasiswa Universitas Indonesia (BEM UI) bersama Komite Selamatkan Daulat Rakyat (SADAR) di kawasan Dukuh Atas Jalan Jenderal Sudirman, Jakarta Pusat, Rabu (28/10/2026), berujung ricuh menjelang malam hari. Situasi memanas</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8323484/19-orang-terlibat-tawuran-maut-di-kebon-jeruk-ditangkap</t>
+          <t>https://www.liputan6.com/photo/read/8323619/suasana-ricuh-demo-sumpah-pemuda-di-kawasan-dukuh-atas</t>
         </is>
       </c>
     </row>
@@ -2478,22 +2454,22 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Fakta Sopir BYD Lindas Ojol di Jaksel: Kelelahan Sampai Ketiduran Kejar Setoran</t>
+          <t>KPK Periksa 4 Saksi soal Dugaan Imbalan Swasta di Kasus BNPB</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Wed, 28 Oct 2026 20:44:12 +0700</t>
+          <t>Wed, 28 Oct 2026 21:14:09 +0700</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Dari hasil penyelidikan, terungkap bahwa sopir BYD yang lindas ojol ternyata juga driver Gojek yang ketiduran karena kelelahan.</t>
+          <t>Penyidik KPK mendalami dugaan suap dan benturan kepentingan dalam proyek penanggulangan bencana di BNPB.</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8323583/fakta-sopir-byd-lindas-ojol-di-jaksel-kelelahan-sampai-ketiduran-kejar-setoran</t>
+          <t>https://www.liputan6.com/news/read/8323603/kpk-periksa-4-saksi-soal-dugaan-imbalan-swasta-di-kasus-bnpb</t>
         </is>
       </c>
     </row>
@@ -2505,22 +2481,22 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Pemulihan Pascabencana Sumatera: Jalan Nasional Pulih, Huntap Terus Dibangun</t>
+          <t>Situasi Terkini Bundaran HI Usai Massa Demo Bubar</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Wed, 28 Oct 2026 18:51:07 +0700</t>
+          <t>Wed, 28 Oct 2026 21:01:25 +0700</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Selain penyediaan hunian sementara, pemerintah melanjutkan pembangunan hunian tetap bagi warga yang rumahnya rusak berat atau hilang akibat bencana.</t>
+          <t>Pembukaan jalan dilakukan bertahap, memastikan kelancaran kendaraan.</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8323478/pemulihan-pascabencana-sumatera-jalan-nasional-pulih-huntap-terus-dibangun</t>
+          <t>https://www.liputan6.com/news/read/8323593/situasi-terkini-bundaran-hi-usai-massa-demo-bubar</t>
         </is>
       </c>
     </row>
@@ -2532,22 +2508,22 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Puan Minta Generasi Muda Diberi Ruang Ikut Tentukan Kebijakan dan Arah Bangsa</t>
+          <t>Kericuhan Pecah di DPRD DIY, Massa Berpakaian Hitam Bentrok dengan Polisi</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Wed, 28 Oct 2026 18:09:36 +0700</t>
+          <t>Wed, 28 Oct 2026 21:24:34 +0700</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Pengalaman anak muda harus menjadi bahan pertimbangan dalam pengambilan keputusan negara.</t>
+          <t>Massa terlibat bentrokan dengan polisi dan masyarakat sekitar yang membantu penjagaan.</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8323443/puan-minta-generasi-muda-diberi-ruang-ikut-tentukan-kebijakan-dan-arah-bangsa</t>
+          <t>https://www.liputan6.com/news/read/8323607/kericuhan-pecah-di-dprd-diy-massa-berpakaian-hitam-bentrok-dengan-polisi</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data pasar & berita - 2026-10-29 15:05 UTC
</commit_message>
<xml_diff>
--- a/data/market_news_latest.xlsx
+++ b/data/market_news_latest.xlsx
@@ -487,20 +487,20 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>5266.1299</v>
+        <v>5098.0571</v>
       </c>
       <c r="F2" t="n">
-        <v>-106.9644</v>
+        <v>-184.2549</v>
       </c>
       <c r="G2" t="n">
-        <v>-1.99</v>
+        <v>-3.49</v>
       </c>
       <c r="H2" t="n">
-        <v>331730400</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -521,20 +521,20 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>7743.98</v>
+        <v>7718.0498</v>
       </c>
       <c r="F3" t="n">
-        <v>21.3799</v>
+        <v>-25.9302</v>
       </c>
       <c r="G3" t="n">
-        <v>0.28</v>
+        <v>-0.33</v>
       </c>
       <c r="H3" t="n">
-        <v>3085116000</v>
+        <v>924439246</v>
       </c>
     </row>
     <row r="4">
@@ -555,20 +555,20 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>52475.1016</v>
+        <v>52361.3398</v>
       </c>
       <c r="F4" t="n">
-        <v>97.5312</v>
+        <v>-113.7617</v>
       </c>
       <c r="G4" t="n">
-        <v>0.19</v>
+        <v>-0.22</v>
       </c>
       <c r="H4" t="n">
-        <v>405081041</v>
+        <v>188869776</v>
       </c>
     </row>
     <row r="5">
@@ -589,20 +589,20 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>26549.8516</v>
+        <v>26205.1895</v>
       </c>
       <c r="F5" t="n">
-        <v>72.041</v>
+        <v>-344.6602</v>
       </c>
       <c r="G5" t="n">
-        <v>0.27</v>
+        <v>-1.3</v>
       </c>
       <c r="H5" t="n">
-        <v>7142936000</v>
+        <v>2158787000</v>
       </c>
     </row>
     <row r="6">
@@ -623,20 +623,20 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>64738.4297</v>
+        <v>63954.1914</v>
       </c>
       <c r="F6" t="n">
-        <v>1470.0586</v>
+        <v>685.8203</v>
       </c>
       <c r="G6" t="n">
-        <v>2.32</v>
+        <v>1.08</v>
       </c>
       <c r="H6" t="n">
-        <v>0</v>
+        <v>165400000</v>
       </c>
     </row>
     <row r="7">
@@ -657,20 +657,20 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>23041.3203</v>
+        <v>22958.6504</v>
       </c>
       <c r="F7" t="n">
-        <v>-170.4902</v>
+        <v>-136.1797</v>
       </c>
       <c r="G7" t="n">
-        <v>-0.73</v>
+        <v>-0.59</v>
       </c>
       <c r="H7" t="n">
-        <v>2842500000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -691,14 +691,20 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>3651.4336</v>
+      </c>
+      <c r="F8" t="n">
+        <v>-30.0354</v>
+      </c>
+      <c r="G8" t="n">
+        <v>-0.82</v>
+      </c>
       <c r="H8" t="n">
-        <v>412609940</v>
+        <v>1406741440</v>
       </c>
     </row>
     <row r="9">
@@ -719,20 +725,20 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>10686.5</v>
+        <v>10749.9004</v>
       </c>
       <c r="F9" t="n">
-        <v>-80.7998</v>
+        <v>55.4004</v>
       </c>
       <c r="G9" t="n">
-        <v>-0.75</v>
+        <v>0.52</v>
       </c>
       <c r="H9" t="n">
-        <v>529948000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -753,20 +759,20 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>25590.7695</v>
+        <v>26061.7793</v>
       </c>
       <c r="F10" t="n">
-        <v>179.9297</v>
+        <v>357.7598</v>
       </c>
       <c r="G10" t="n">
-        <v>0.71</v>
+        <v>1.39</v>
       </c>
       <c r="H10" t="n">
-        <v>47576700</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -791,13 +797,13 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>5412.8101</v>
+        <v>5396.0298</v>
       </c>
       <c r="F11" t="n">
-        <v>15.7803</v>
+        <v>-1.8804</v>
       </c>
       <c r="G11" t="n">
-        <v>0.29</v>
+        <v>-0.03</v>
       </c>
       <c r="H11" t="n">
         <v>0</v>
@@ -825,13 +831,13 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>18183</v>
+        <v>18128</v>
       </c>
       <c r="F12" t="n">
-        <v>43.5</v>
+        <v>-11.5</v>
       </c>
       <c r="G12" t="n">
-        <v>0.24</v>
+        <v>-0.06</v>
       </c>
       <c r="H12" t="n">
         <v>0</v>
@@ -855,17 +861,17 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>102.257</v>
+        <v>102.017</v>
       </c>
       <c r="F13" t="n">
-        <v>-0.063</v>
+        <v>-0.173</v>
       </c>
       <c r="G13" t="n">
-        <v>-0.06</v>
+        <v>-0.17</v>
       </c>
       <c r="H13" t="n">
         <v>0</v>
@@ -893,13 +899,13 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>157.867</v>
+        <v>157.851</v>
       </c>
       <c r="F14" t="n">
-        <v>-0.126</v>
+        <v>-0.142</v>
       </c>
       <c r="G14" t="n">
-        <v>-0.08</v>
+        <v>-0.09</v>
       </c>
       <c r="H14" t="n">
         <v>0</v>
@@ -923,17 +929,17 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>0.5044999999999999</v>
+        <v>0.4966</v>
       </c>
       <c r="F15" t="n">
-        <v>0.0052</v>
+        <v>-0.007900000000000001</v>
       </c>
       <c r="G15" t="n">
-        <v>1.04</v>
+        <v>-1.57</v>
       </c>
       <c r="H15" t="n">
         <v>0</v>
@@ -957,17 +963,17 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>0.5361</v>
+        <v>0.531</v>
       </c>
       <c r="F16" t="n">
-        <v>0.0056</v>
+        <v>-0.0051</v>
       </c>
       <c r="G16" t="n">
-        <v>1.06</v>
+        <v>-0.95</v>
       </c>
       <c r="H16" t="n">
         <v>0</v>
@@ -991,17 +997,17 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>0.3995</v>
+        <v>0.3982</v>
       </c>
       <c r="F17" t="n">
-        <v>-0.0045</v>
+        <v>-0.0013</v>
       </c>
       <c r="G17" t="n">
-        <v>-1.11</v>
+        <v>-0.33</v>
       </c>
       <c r="H17" t="n">
         <v>0</v>
@@ -1025,14 +1031,20 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>81.55500000000001</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0.5649999999999999</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0.7</v>
+      </c>
       <c r="H18" t="n">
-        <v>35072467</v>
+        <v>9208615</v>
       </c>
     </row>
     <row r="19">
@@ -1053,14 +1065,20 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>77.5976</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0.0076</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0.01</v>
+      </c>
       <c r="H19" t="n">
-        <v>65283700</v>
+        <v>18334013</v>
       </c>
     </row>
     <row r="20">
@@ -1081,20 +1099,20 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>4058.1001</v>
+        <v>4042.2</v>
       </c>
       <c r="F20" t="n">
-        <v>-16.5</v>
+        <v>-9.4001</v>
       </c>
       <c r="G20" t="n">
-        <v>-0.4</v>
+        <v>-0.23</v>
       </c>
       <c r="H20" t="n">
-        <v>10619</v>
+        <v>98721</v>
       </c>
     </row>
     <row r="21">
@@ -1115,20 +1133,20 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>101.99</v>
+        <v>100.27</v>
       </c>
       <c r="F21" t="n">
-        <v>2.09</v>
+        <v>-2.51</v>
       </c>
       <c r="G21" t="n">
-        <v>2.09</v>
+        <v>-2.44</v>
       </c>
       <c r="H21" t="n">
-        <v>7344</v>
+        <v>136117</v>
       </c>
     </row>
     <row r="22">
@@ -1149,20 +1167,20 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="E22" t="n">
-        <v>110.69</v>
+        <v>109.56</v>
       </c>
       <c r="F22" t="n">
-        <v>-3.19</v>
+        <v>-5.76</v>
       </c>
       <c r="G22" t="n">
-        <v>-2.8</v>
+        <v>-4.99</v>
       </c>
       <c r="H22" t="n">
-        <v>964</v>
+        <v>21059</v>
       </c>
     </row>
     <row r="23">
@@ -1183,20 +1201,20 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="E23" t="n">
-        <v>6.6705</v>
+        <v>6.58</v>
       </c>
       <c r="F23" t="n">
-        <v>0.0485</v>
+        <v>-0.0615</v>
       </c>
       <c r="G23" t="n">
-        <v>0.73</v>
+        <v>-0.93</v>
       </c>
       <c r="H23" t="n">
-        <v>1234</v>
+        <v>24204</v>
       </c>
     </row>
     <row r="24">
@@ -1217,14 +1235,20 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr"/>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr"/>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>62.68</v>
+      </c>
+      <c r="F24" t="n">
+        <v>-0.84</v>
+      </c>
+      <c r="G24" t="n">
+        <v>-1.32</v>
+      </c>
       <c r="H24" t="n">
-        <v>23690945</v>
+        <v>4896291</v>
       </c>
     </row>
     <row r="25">
@@ -1245,17 +1269,17 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="E25" t="n">
-        <v>16.91</v>
+        <v>16.81</v>
       </c>
       <c r="F25" t="n">
-        <v>-0.61</v>
+        <v>-0.1</v>
       </c>
       <c r="G25" t="n">
-        <v>-3.48</v>
+        <v>-0.59</v>
       </c>
       <c r="H25" t="n">
         <v>0</v>
@@ -1283,16 +1307,16 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>80828.8906</v>
+        <v>81201.7812</v>
       </c>
       <c r="F26" t="n">
-        <v>23.8125</v>
+        <v>-65.8047</v>
       </c>
       <c r="G26" t="n">
-        <v>0.03</v>
+        <v>-0.08</v>
       </c>
       <c r="H26" t="n">
-        <v>24155543552</v>
+        <v>27420071936</v>
       </c>
     </row>
     <row r="27">
@@ -1313,20 +1337,20 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="E27" t="n">
-        <v>1235</v>
+        <v>1150</v>
       </c>
       <c r="F27" t="n">
-        <v>-90</v>
+        <v>-85</v>
       </c>
       <c r="G27" t="n">
-        <v>-6.79</v>
+        <v>-6.88</v>
       </c>
       <c r="H27" t="n">
-        <v>142341100</v>
+        <v>100005900</v>
       </c>
     </row>
     <row r="28">
@@ -1347,20 +1371,20 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="E28" t="n">
-        <v>1335</v>
+        <v>1350</v>
       </c>
       <c r="F28" t="n">
-        <v>-25</v>
+        <v>15</v>
       </c>
       <c r="G28" t="n">
-        <v>-1.84</v>
+        <v>1.12</v>
       </c>
       <c r="H28" t="n">
-        <v>277508900</v>
+        <v>360528200</v>
       </c>
     </row>
     <row r="29">
@@ -1381,20 +1405,20 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="E29" t="n">
-        <v>432</v>
+        <v>410</v>
       </c>
       <c r="F29" t="n">
-        <v>-24</v>
+        <v>-22</v>
       </c>
       <c r="G29" t="n">
-        <v>-5.26</v>
+        <v>-5.09</v>
       </c>
       <c r="H29" t="n">
-        <v>444377000</v>
+        <v>517058000</v>
       </c>
     </row>
     <row r="30">
@@ -1415,20 +1439,20 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="E30" t="n">
-        <v>2070</v>
+        <v>1930</v>
       </c>
       <c r="F30" t="n">
-        <v>-90</v>
+        <v>-140</v>
       </c>
       <c r="G30" t="n">
-        <v>-4.17</v>
+        <v>-6.76</v>
       </c>
       <c r="H30" t="n">
-        <v>24971000</v>
+        <v>6505000</v>
       </c>
     </row>
     <row r="31">
@@ -1449,20 +1473,20 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="E31" t="n">
-        <v>2670</v>
+        <v>2490</v>
       </c>
       <c r="F31" t="n">
-        <v>-200</v>
+        <v>-180</v>
       </c>
       <c r="G31" t="n">
-        <v>-6.97</v>
+        <v>-6.74</v>
       </c>
       <c r="H31" t="n">
-        <v>67510700</v>
+        <v>32711600</v>
       </c>
     </row>
     <row r="32">
@@ -1483,20 +1507,20 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="E32" t="n">
-        <v>386</v>
+        <v>362</v>
       </c>
       <c r="F32" t="n">
-        <v>-12</v>
+        <v>-24</v>
       </c>
       <c r="G32" t="n">
-        <v>-3.02</v>
+        <v>-6.22</v>
       </c>
       <c r="H32" t="n">
-        <v>46693200</v>
+        <v>31775900</v>
       </c>
     </row>
     <row r="33">
@@ -1517,20 +1541,20 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="E33" t="n">
-        <v>448</v>
+        <v>418</v>
       </c>
       <c r="F33" t="n">
-        <v>-4</v>
+        <v>-30</v>
       </c>
       <c r="G33" t="n">
-        <v>-0.88</v>
+        <v>-6.7</v>
       </c>
       <c r="H33" t="n">
-        <v>61693200</v>
+        <v>40857300</v>
       </c>
     </row>
     <row r="34">
@@ -1551,20 +1575,20 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="E34" t="n">
-        <v>2230</v>
+        <v>2080</v>
       </c>
       <c r="F34" t="n">
-        <v>-90</v>
+        <v>-150</v>
       </c>
       <c r="G34" t="n">
-        <v>-3.88</v>
+        <v>-6.73</v>
       </c>
       <c r="H34" t="n">
-        <v>9435100</v>
+        <v>4890600</v>
       </c>
     </row>
     <row r="35">
@@ -1585,20 +1609,20 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="E35" t="n">
-        <v>360</v>
+        <v>336</v>
       </c>
       <c r="F35" t="n">
-        <v>8</v>
+        <v>-24</v>
       </c>
       <c r="G35" t="n">
-        <v>2.27</v>
+        <v>-6.67</v>
       </c>
       <c r="H35" t="n">
-        <v>295184800</v>
+        <v>183254800</v>
       </c>
     </row>
     <row r="36">
@@ -1619,20 +1643,20 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="E36" t="n">
-        <v>149</v>
+        <v>139</v>
       </c>
       <c r="F36" t="n">
-        <v>-7</v>
+        <v>-10</v>
       </c>
       <c r="G36" t="n">
-        <v>-4.49</v>
+        <v>-6.71</v>
       </c>
       <c r="H36" t="n">
-        <v>42924100</v>
+        <v>24239300</v>
       </c>
     </row>
     <row r="37">
@@ -1653,20 +1677,20 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="E37" t="n">
-        <v>10175</v>
+        <v>9475</v>
       </c>
       <c r="F37" t="n">
-        <v>-100</v>
+        <v>-700</v>
       </c>
       <c r="G37" t="n">
-        <v>-0.97</v>
+        <v>-6.88</v>
       </c>
       <c r="H37" t="n">
-        <v>26793100</v>
+        <v>10634000</v>
       </c>
     </row>
   </sheetData>
@@ -1725,22 +1749,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Forum ASCOPE Ke-51 Sepakat Perkuat Arsitektur Energi Masa Depan ASEAN</t>
+          <t>GOTO Cetak Laba Rp 441 Miliar</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Thu, 29 Oct 2026 08:07:51 +0700</t>
+          <t>Thu, 29 Oct 2026 21:41:04 +0700</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/29/pertamina-1793236035812_169.jpeg?w=360&amp;amp;q=90" /&gt; Rangkaian 51st ASCOPE di Bali ditutup dengan kesepakatan strategis untuk ketahanan energi regional. Negara anggota berkomitmen menghadapi tantangan energi.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/20/goto-rilis-model-llm-27b-paham-bahasa-indonesia-hingga-daerah-1792493682697_169.jpeg?w=360&amp;amp;q=90" /&gt; PT GoTo Gojek Tokopedia Tbk (GOTO) mencatat laba bersih Rp 441 miliar pada kuartal III-2026.</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8728821/forum-ascope-ke-51-sepakat-perkuat-arsitektur-energi-masa-depan-asean</t>
+          <t>https://finance.detik.com/bursa-dan-valas/d-8730220/goto-cetak-laba-rp-441-miliar</t>
         </is>
       </c>
     </row>
@@ -1752,22 +1776,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Sederet Manfaat QRIS, Bikin Transaksi Usaha Jadi Praktis</t>
+          <t>Laba PTBA Melonjak, Capai Rp 4,41 Triliun hingga Triwulan III 2026</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Thu, 29 Oct 2026 08:01:20 +0700</t>
+          <t>Thu, 29 Oct 2026 21:34:47 +0700</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/28/qris-pakai-dana-1793170176586.png?w=360&amp;amp;q=90" /&gt; QRIS memudahkan transaksi digital di Indonesia dengan satu kode QR. Pengguna dan merchant dapat menikmati kemudahan, keamanan, dan kecepatan dalam pembayaran.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/29/ptba-1793284413718_169.jpeg?w=360&amp;amp;q=90" /&gt; PT Bukit Asam (PTBA) laporkan laba bersih Rp 4,41 triliun hingga September 2026. Kinerja operasional pulih dengan produksi dan penjualan meningkat.</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8727735/sederet-manfaat-qris-bikin-transaksi-usaha-jadi-praktis</t>
+          <t>https://finance.detik.com/bursa-dan-valas/d-8730215/laba-ptba-melonjak-capai-rp-4-41-triliun-hingga-triwulan-iii-2026</t>
         </is>
       </c>
     </row>
@@ -1779,22 +1803,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Pasar Modal Dibersihkan, Kepercayaan Investor Dipulihkan</t>
+          <t>Prabowo Bakal Resmikan Pabrik Baterai Mobil Listrik di Karawang</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Thu, 29 Oct 2026 08:00:42 +0700</t>
+          <t>Thu, 29 Oct 2026 20:58:34 +0700</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/16/ihsg-ambruk-1157-ditutup-di-level-5185-1792144638939_169.jpeg?w=360&amp;amp;q=90" /&gt; IHSG anjlok 6% setelah pengumuman MSCI, memicu panic selling di pasar. OJK dan BEI siapkan reformasi untuk meningkatkan transparansi dan likuiditas.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/08/27/baterai-mobil-listrik-1787794586277_169.jpeg?w=360&amp;amp;q=90" /&gt; Presiden Prabowo Subianto bakal meresmikan pabrik baterai mobil listrik di Karawang, kerja sama CATL dan Antam.</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/bursa-dan-valas/d-8728651/pasar-modal-dibersihkan-kepercayaan-investor-dipulihkan</t>
+          <t>https://finance.detik.com/industri/d-8730191/prabowo-bakal-resmikan-pabrik-baterai-mobil-listrik-di-karawang</t>
         </is>
       </c>
     </row>
@@ -1806,22 +1830,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>The Fed Putuskan Tahan Suku Bunga</t>
+          <t>Investor AS Pede MSCI Tak Turunkan Kasta Bursa RI, Ini Alasannya</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Thu, 29 Oct 2026 07:39:08 +0700</t>
+          <t>Thu, 29 Oct 2026 20:30:03 +0700</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2023/02/02/bank-sentral-as-the-fed-naikkan-suku-bunga-sebesar-025-3_169.jpeg?w=360&amp;amp;q=90" /&gt; The Fed memilih untuk tidak terburu-buru mengubah suku bunga, meskipun tekanan inflasi masih sulit dikendalikan.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/16/ihsg-ambruk-1157-ditutup-di-level-5185-1792144638880_169.jpeg?w=360&amp;amp;q=90" /&gt; Investor Amerika Serikat (AS) sekaligus Anggota Komite High Shareholding Concentration (HSC), Chapman Taylor, meyakini pasar modal Indonesia tidak t</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/moneter/d-8728784/the-fed-putuskan-tahan-suku-bunga</t>
+          <t>https://finance.detik.com/bursa-dan-valas/d-8730091/investor-as-pede-msci-tak-turunkan-kasta-bursa-ri-ini-alasannya</t>
         </is>
       </c>
     </row>
@@ -1833,22 +1857,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Bos BRIN Lapor Prabowo Limbah Sawit Bisa Diolah Jadi Listrik</t>
+          <t>Minerba Convex 2026 Digelar 2-3 November, Ada Klinik RKAB hingga Zona Anak</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Thu, 29 Oct 2026 07:30:00 +0700</t>
+          <t>Thu, 29 Oct 2026 20:23:05 +0700</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/28/kepala-badan-riset-dan-inovasi-nasional-brin-arif-satria-1793120446935_169.jpeg?w=360&amp;amp;q=90" /&gt; Kepala Badan Riset dan Inovasi Nasional (BRIN) Arif Satria memberikan laporan kepada Presiden Prabowo Subianto soal limbah sawit m</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/29/kementerian-esdm-1793280061440_169.jpeg?w=360&amp;amp;q=90" /&gt; Minerba Convex 2026 di Jakarta mengajak masyarakat mengenal sektor pertambangan. Acara ini menawarkan edukasi, penghargaan, dan konsultasi untuk pelaku usaha.</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8728654/bos-brin-lapor-prabowo-limbah-sawit-bisa-diolah-jadi-listrik</t>
+          <t>https://finance.detik.com/energi/d-8730161/minerba-convex-2026-digelar-2-3-november-ada-klinik-rkab-hingga-zona-anak</t>
         </is>
       </c>
     </row>
@@ -1860,22 +1884,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Terbang Makin Hemat, Tarif Penumpang Pesawat di Bandara Samrat Turun 50 Persen</t>
+          <t>Impor BBM-LPG Kini Lewat Lemigas, Bakal Lebih Murah?</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Thu, 29 Oct 2026 07:15:43 +0700</t>
+          <t>Thu, 29 Oct 2026 20:00:00 +0700</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/28/terbang-makin-hemat-tarif-penumpang-pesawat-di-bandara-samrat-turun-50-persen-1793188717765_169.jpeg?w=360&amp;amp;q=90" /&gt; Kabar baik, Bandara Sam Ratulangi Manado memangkas tarif jasa penumpang pesawat 50 persen hingga 10 Januari 2</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/03/09/harga-minyak-mentah-hampir-us110-dunia-dilanda-kepanikan-1773053712369_169.jpeg?w=360&amp;amp;q=90" /&gt; Pemerintah ubah mekanisme impor minyak dan gas lewat BLU Lemigas, skema ini disebut membuat pengadaan jadi mudah dan cepat.</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/foto-bisnis/d-8728409/terbang-makin-hemat-tarif-penumpang-pesawat-di-bandara-samrat-turun-50-persen</t>
+          <t>https://finance.detik.com/energi/d-8730095/impor-bbm-lpg-kini-lewat-lemigas-bakal-lebih-murah</t>
         </is>
       </c>
     </row>
@@ -1887,22 +1911,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Pertama dalam Sejarah Pasar Modal RI, BEI Bagi-bagi Dividen</t>
+          <t>Denda Rp 2,1 Triliun di Kasus DSSA, BREN, dan CUAN Sudah Dibayar</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Thu, 29 Oct 2026 07:00:00 +0700</t>
+          <t>Thu, 29 Oct 2026 19:30:47 +0700</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2016/05/03/1fb20055-d8fe-4f7f-bf42-445d369dc61a_169.jpg?w=360&amp;amp;q=90" /&gt; Bursa Efek Indonesia (BEI) akan bagi-bagi dividen tunai pertamanya dalam sejarah, totalnya Rp 1,56 triliun.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/27/ketua-dewan-komisioner-ojk-friderica-widyasari-dewi-1793077340311_169.jpeg?w=360&amp;amp;q=90" /&gt; Ketua Dewan Komisioner OJK Friderica Widyasari Dewi, mengaku pihaknya telah menerima pembayaran denda dari pelanggaran pasar modal sebe</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/bursa-dan-valas/d-8728605/pertama-dalam-sejarah-pasar-modal-ri-bei-bagi-bagi-dividen</t>
+          <t>https://finance.detik.com/bursa-dan-valas/d-8730078/denda-rp-2-1-triliun-di-kasus-dssa-bren-dan-cuan-sudah-dibayar</t>
         </is>
       </c>
     </row>
@@ -1914,22 +1938,22 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Kenapa Harga Tiket Pesawat Saat Nataru Bisa Turun 12%?</t>
+          <t>Panen Marigold di Meksiko, Bunga untuk Menyambut Arwah Leluhur</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Thu, 29 Oct 2026 06:30:57 +0700</t>
+          <t>Thu, 29 Oct 2026 19:02:44 +0700</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/05/15/maskapai-diberikan-keleluasaan-tentukan-tarif-tiket-1778834393575_169.jpeg?w=360&amp;amp;q=90" /&gt; Harga tiket pesawat kelas ekonomi domestik berpotensi turun hingga 12% selama periode libur Natal 2026 dan Tahun Baru 2027 (Nataru).</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/29/panen-marigold-di-meksiko-bunga-untuk-menyambut-arwah-leluhur-1793251008236.jpeg?w=360&amp;amp;q=90" /&gt; Petani memanen bunga marigold di Atlixco, Meksiko, menjelang perayaan Hari Orang Mati pada awal November.</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8728369/kenapa-harga-tiket-pesawat-saat-nataru-bisa-turun-12</t>
+          <t>https://finance.detik.com/foto-bisnis/d-8729219/panen-marigold-di-meksiko-bunga-untuk-menyambut-arwah-leluhur</t>
         </is>
       </c>
     </row>
@@ -1941,22 +1965,22 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Simak! Begini Cara Ajukan Bebas Denda Pajak</t>
+          <t>Hashim Sebut Dolar AS bisa Tembus Rp 22.000 Gegara MSCI, Bos BI Buka Suara</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Thu, 29 Oct 2026 05:55:41 +0700</t>
+          <t>Thu, 29 Oct 2026 19:00:39 +0700</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2014/10/01/aba994a2-34ed-467e-b236-0838b109f70c_169.jpg?w=360&amp;amp;q=90" /&gt; Wajib pajak dapat ajukan pengurangan atau penghapusan denda pajak hingga 1 Oktober 2028. Ikuti langkah-langkah di Coretax untuk permohonan.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/21/bank-indonesia-bi-memutuskan-menaikkan-suku-bunga-deposit-facility-sebesar-25-basis-poin-bps-menjadi-5-keputusan-tersebut-diam-1792576096896_169.jpeg?w=360&amp;amp;q=90" /&gt; Gubernur Bank Indonesia (BI), Destry Damayanti, buka suara s</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8728372/simak-begini-cara-ajukan-bebas-denda-pajak</t>
+          <t>https://finance.detik.com/bursa-dan-valas/d-8730007/hashim-sebut-dolar-as-bisa-tembus-rp-22-000-gegara-msci-bos-bi-buka-suara</t>
         </is>
       </c>
     </row>
@@ -1968,22 +1992,22 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Sempat Mangkrak, Proyek Pengembangan Pasar Senen Blok VI Jalan Lagi</t>
+          <t>Bahlil Tuding Singapura Jual Lagi Pasokan Gas dari RI</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Wed, 28 Oct 2026 22:48:45 +0700</t>
+          <t>Thu, 29 Oct 2026 18:55:53 +0700</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/28/gambar-rencana-pengembangan-pasar-senen-blok-vi-1793202449109_169.jpeg?w=360&amp;amp;q=90" /&gt; Proyek pengembangan Pasar Senen Blok VI, Jakarta Pusat kembali berjalan, setelah sempat mangkrak.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/14/bahlil-lahadalia-rolandodetikcom-1791978307056_169.jpeg?w=360&amp;amp;q=90" /&gt; Menko Hilirisasi dan Transisi Energi Bahlil Lahadalia menduga sebagian LNG yang diekspor dari Indonesia dijual lagi oleh Singapura ke negara lain.</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/infrastruktur/d-8728665/sempat-mangkrak-proyek-pengembangan-pasar-senen-blok-vi-jalan-lagi</t>
+          <t>https://finance.detik.com/energi/d-8730027/bahlil-tuding-singapura-jual-lagi-pasokan-gas-dari-ri</t>
         </is>
       </c>
     </row>
@@ -1995,22 +2019,22 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Pemda Bakal Lebih Sering Pelototi Pelaksanaan MBG</t>
+          <t>Bos BI Buka-bukaan soal MSCI Bikin Investor Asing Bingung</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Wed, 28 Oct 2026 21:30:00 +0700</t>
+          <t>Thu, 29 Oct 2026 18:30:37 +0700</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/20/penerima-manfaat-mbg-dalam-dua-tahun-pemerintahan-prabowo-1792479756724_169.jpeg?w=360&amp;amp;q=90" /&gt; Pengawasan pelaksanaan Makan Bergizi Gratis (MBG) bakal lebih banyak melibatkan pemerintah daerah.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/29/gubernur-bank-indonesia-bi-destry-damayanti-1793272001596_169.jpeg?w=360&amp;amp;q=90" /&gt; Gubernur Bank Indonesia (BI), Destry Damayanti, mengaku menerima sejumlah keluhan dari raksasa investor asing terkait dengan persoalan MSCI.</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8728569/pemda-bakal-lebih-sering-pelototi-pelaksanaan-mbg</t>
+          <t>https://finance.detik.com/bursa-dan-valas/d-8729933/bos-bi-buka-bukaan-soal-msci-bikin-investor-asing-bingung</t>
         </is>
       </c>
     </row>
@@ -2022,22 +2046,22 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Berdayakan Masyarakat, MIND ID Raih Penghargaan Mandaya Awards 2026</t>
+          <t>Bocoran Hashim: Shopee-GoTo Pungut Pajak Digital Mulai 9 November 2026</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Wed, 28 Oct 2026 21:26:17 +0700</t>
+          <t>Thu, 29 Oct 2026 18:08:52 +0700</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/28/berdayakan-masyarakat-grup-mind-id-raih-penghargaan-mandaya-awards-2026-1793197151033_169.jpeg?w=360&amp;amp;q=90" /&gt; MIND ID meraih Anugerah Mandaya Award 2026 atas pemberdayaan masyarakat. Programnya fokus pada penguatan ekonomi da</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2024/11/14/hashim-djojohadikusumo-1_169.jpeg?w=360&amp;amp;q=90" /&gt; Ketua Dewan Penasihat Kadin Hashim Djojohadikusumo menyebut GoTo hingga Shopee bakal pungut pajak digital mulai bulan depan.</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8728601/berdayakan-masyarakat-mind-id-raih-penghargaan-mandaya-awards-2026</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8729936/bocoran-hashim-shopee-goto-pungut-pajak-digital-mulai-9-november-2026</t>
         </is>
       </c>
     </row>
@@ -2049,22 +2073,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>8 Bos Sawit RI Menghadap Menteri Singapura, Ini Daftarnya</t>
+          <t>MSCI Soroti Pasar Modal RI, Rosan Beri Bukti Investor Masih Percaya</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Wed, 28 Oct 2026 21:05:16 +0700</t>
+          <t>Thu, 29 Oct 2026 17:45:00 +0700</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/12/situasi-kabut-asap-di-singapura-pada-senin-1210-waktu-setempat-1791794641533_169.jpeg?w=360&amp;amp;q=90" /&gt; Delapan Petinggi perusahaan kelapa sawit besar di Indonesia memenuhi panggilan pejabat tinggi Singapura.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/11/20/menteri-investasi-dan-hilirisasikepala-bkpm-rosan-roeslani-1763634019135_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Investasi Rosan Roeslani menyatakan kepercayaan investor terhadap Indonesia tetap tinggi, dengan realisasi investasi men</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/industri/d-8728582/8-bos-sawit-ri-menghadap-menteri-singapura-ini-daftarnya</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8729905/msci-soroti-pasar-modal-ri-rosan-beri-bukti-investor-masih-percaya</t>
         </is>
       </c>
     </row>
@@ -2076,22 +2100,22 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Dua Pintu Masuk Stasiun MRT Dukuh Atas Ditutup Sementara</t>
+          <t>Revisi RKAB Rampung: Nikel 300 Juta Ton-Batu Bara 700 Juta Ton</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Wed, 28 Oct 2026 20:11:26 +0700</t>
+          <t>Thu, 29 Oct 2026 17:36:21 +0700</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/17/penumpang-mrt-jakarta-1792229479640_169.jpeg?w=360&amp;amp;q=90" /&gt; Pintu masuk E dan C Stasiun MRT Dukuh Atas BNI masih ditutup sementara.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2021/09/10/ada-di-sumsel-tambang-batu-bara-ini-punya-cadangan-3-miliar-ton-6_169.jpeg?w=360&amp;amp;q=90" /&gt; Kementerian ESDM menerbitkan revisi RKAB 2026, dengan produksi nikel sekitar 300 juta ton dan batu bara 700 juta ton.</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/infrastruktur/d-8728516/dua-pintu-masuk-stasiun-mrt-dukuh-atas-ditutup-sementara</t>
+          <t>https://finance.detik.com/energi/d-8729888/revisi-rkab-rampung-nikel-300-juta-ton-batu-bara-700-juta-ton</t>
         </is>
       </c>
     </row>
@@ -2103,22 +2127,22 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Impor BBM Lewat Lemigas Cuma buat Produk yang Dijual Pertamina</t>
+          <t>RI Rawan Bencana, OJK Dorong Sektor PPDP Jaga Ekonomi Warga</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Wed, 28 Oct 2026 19:30:05 +0700</t>
+          <t>Thu, 29 Oct 2026 17:23:00 +0700</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/14/bahlil-lahadalia-rolandodetikcom-1791978307056_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Bahlil menegaskan impor migas lewat Lemigas hanya untuk Pertamina, bukan swasta. Skema baru impor kini menggunakan G2G dan G2B.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/29/ojk-1793269261385_169.jpeg?w=360&amp;amp;q=90" /&gt; OJK luncurkan peta jalan keuangan berkelanjutan untuk sektor PPDP 2026-2030. Fokus pada mitigasi risiko bencana dan iklim demi stabilitas ekonomi Indonesia.</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8728437/impor-bbm-lewat-lemigas-cuma-buat-produk-yang-dijual-pertamina</t>
+          <t>https://finance.detik.com/moneter/d-8729850/ri-rawan-bencana-ojk-dorong-sektor-ppdp-jaga-ekonomi-warga</t>
         </is>
       </c>
     </row>
@@ -2130,22 +2154,22 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Eks Wamen Imipas Silmy Karim Jalani Sidang Perdana Hari Ini</t>
+          <t>Infografis: 100 Hari MBG di Tangan Sudaryono</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Thu, 29 Oct 2026 07:57:27 +0700</t>
+          <t>Thu, 29 Oct 2026 21:58:48 +0700</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Mantan Wamen Imipas Silmy Karim menjalani sidang perdana kasus dugaan pemerasan dan gratifikasi izin tinggal WNA.</t>
+          <t>Sudaryono menerapkan sejumlah aturan untuk memperkuat keamanan pangan, kedisiplinan, dan transparansi program MBG.</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8323752/eks-wamen-imipas-silmy-karim-jalani-sidang-perdana-hari-ini</t>
+          <t>https://www.liputan6.com/news/read/8324499/infografis-100-hari-mbg-di-tangan-sudaryono</t>
         </is>
       </c>
     </row>
@@ -2157,22 +2181,22 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Siasat Dwi Martono Hilangkan Jejak Pembunuhan Istri dan Balita</t>
+          <t>Rincian Bonus Atlet Asian Games dan Asian Para Games dari Prabowo</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Thu, 29 Oct 2026 06:03:42 +0700</t>
+          <t>Thu, 29 Oct 2026 21:48:55 +0700</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Dwi menyiapkan berbagai cara dan peralatan untuk menghilangkan jejak pembunuhan terhadap kedua korban.</t>
+          <t>Pemerintah memberikan bonus dengan besaran berbeda sesuai medali dan nomor pertandingan.</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8323679/siasat-dwi-martono-hilangkan-jejak-pembunuhan-istri-dan-balita</t>
+          <t>https://www.liputan6.com/news/read/8324491/rincian-bonus-atlet-asian-games-dan-asian-para-games-dari-prabowo</t>
         </is>
       </c>
     </row>
@@ -2184,22 +2208,22 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Gempa Magnitudo 6,4 Guncang Tanimbar Maluku</t>
+          <t>Kuasa Hukum Bantah Silmy Karim Terjaring OTT KPK</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Thu, 29 Oct 2026 05:33:07 +0700</t>
+          <t>Thu, 29 Oct 2026 21:47:30 +0700</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Gempa bumi berkekuatan Magnitudo 6,4 terjadi di 201 km BaratLaut Tanimbar, tidak berpotensi tsunami.</t>
+          <t>Silmy Karim didakwa melakukan pemerasan terkait dokumen keimigrasian senilai Rp 168,9 miliar dan menerima gratifikasi Rp 33,8 miliar.</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8323703/gempa-magnitudo-64-guncang-tanimbar-maluku</t>
+          <t>https://www.liputan6.com/news/read/8324487/kuasa-hukum-bantah-silmy-karim-terjaring-ott-kpk</t>
         </is>
       </c>
     </row>
@@ -2211,22 +2235,22 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>100 Hari MBG di Tangan Sudaryono</t>
+          <t>Seskab Teddy Beberkan Capaian Dua Tahun Pemerintahan Prabowo</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Thu, 29 Oct 2026 05:00:10 +0700</t>
+          <t>Thu, 29 Oct 2026 21:35:47 +0700</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Selama 100 hari memimpin BGN, Sudaryono mengeluarkan sejumlah kebijakan pembenahan program MBG.</t>
+          <t>Seskab melaporkan sejumlah capaian program prioritas dan pembangunan selama dua tahun pemerintahan Presiden Prabowo Subianto.</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8323694/100-hari-mbg-di-tangan-sudaryono</t>
+          <t>https://www.liputan6.com/news/read/8324485/seskab-teddy-beberkan-capaian-dua-tahun-pemerintahan-prabowo</t>
         </is>
       </c>
     </row>
@@ -2238,22 +2262,22 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Update Kericuhan Demo DIY, Massa Bentrok Lagi dengan Polisi di Tugu Yogyakarta</t>
+          <t>DPR: TNI Amankan Demo Hal Lumrah</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Thu, 29 Oct 2026 01:26:40 +0700</t>
+          <t>Thu, 29 Oct 2026 21:07:45 +0700</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Massa ricuh masih melakukan aksi pelemparan batu dan menembakkan kembang api.</t>
+          <t>Menurut Dave, aparat tetap harus memastikan aksi berlangsung aman dan tertib tanpa mengabaikan hak masyarakat</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8323690/update-kericuhan-demo-diy-massa-bentrok-lagi-dengan-polisi-di-tugu-yogyakarta</t>
+          <t>https://www.liputan6.com/news/read/8324473/dpr-tni-amankan-demo-hal-lumrah</t>
         </is>
       </c>
     </row>
@@ -2265,22 +2289,22 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Kronologi Demo Sumpah Pemuda di Yogyakarta Berujung Ricuh</t>
+          <t>Di Sidang Yaqut, Anwar Abbas Singgung Integritas dan Motif Finansial</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Thu, 29 Oct 2026 01:21:18 +0700</t>
+          <t>Thu, 29 Oct 2026 21:31:54 +0700</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Konsentrasi massa terbagi di sisi selatan dan utara gedung DPRD.</t>
+          <t>Dalam sidang dugaan korupsi kuota haji, Anwar Abbas menyebut Yaqut bukan orang miskin.</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8323689/kronologi-demo-sumpah-pemuda-di-yogyakarta-berujung-ricuh</t>
+          <t>https://www.liputan6.com/news/read/8324464/di-sidang-yaqut-anwar-abbas-singgung-integritas-dan-motif-finansial</t>
         </is>
       </c>
     </row>
@@ -2292,22 +2316,22 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Sektor Kelistrikan Bidik Hidrogen dan Amonia untuk Tekan Emisi</t>
+          <t>Perintah Prabowo ke Erick Thohir soal Pembinaan Atlet</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Thu, 29 Oct 2026 01:02:20 +0700</t>
+          <t>Thu, 29 Oct 2026 20:56:39 +0700</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Pengujian hidrogen dan amonia di Bali dan Banten menunjukkan potensi pengurangan emisi sekaligus penghematan bahan bakar fosil.</t>
+          <t>Prabowo menilai Indonesia masih harus bekerja dan berjuang lebih keras untuk meningkatkan prestasi di ajang olahraga internasional.</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8323684/sektor-kelistrikan-bidik-hidrogen-dan-amonia-untuk-tekan-emisi</t>
+          <t>https://www.liputan6.com/news/read/8324463/perintah-prabowo-ke-erick-thohir-soal-pembinaan-atlet</t>
         </is>
       </c>
     </row>
@@ -2319,22 +2343,22 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Mabes Polri: Terima Kasih Massa Aksi, Demo Sumpah Pemuda Tertib dan Damai</t>
+          <t>Kondisi Terkini Medan Merdeka Selatan Usai Demo Mahasiswa Trisakti</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Wed, 28 Oct 2026 23:48:02 +0700</t>
+          <t>Thu, 29 Oct 2026 20:25:30 +0700</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Polri mengatakan, situasi yang aman dan kondusif terwujud berkat kerja sama masyarakat dan kepolisian.</t>
+          <t>Kondisi Jalan Medan Merdeka Selatan normal kembali usai demo mahasiswa Trisakti.</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8323668/mabes-polri-terima-kasih-massa-aksi-demo-sumpah-pemuda-tertib-dan-damai</t>
+          <t>https://www.liputan6.com/news/read/8324449/kondisi-terkini-medan-merdeka-selatan-usai-demo-mahasiswa-trisakti</t>
         </is>
       </c>
     </row>
@@ -2346,22 +2370,22 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Respons PT Djarum soal Penggeledahan KPK</t>
+          <t>Kubu Gibran Tunjukkan Riwayat Pendidikan, Penggugat Soroti Bukti Penyetaraan</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Wed, 28 Oct 2026 22:50:39 +0700</t>
+          <t>Thu, 29 Oct 2026 20:24:04 +0700</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>PT Djarum akan bersikap kooperatif membantu mengusut dugaan korupsi yang sedang didalami KPK.</t>
+          <t>Rullyandi mengatakan dokumen riwayat pendidikan Gibran telah dilampirkan dalam jawaban pihak intervensi.</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8323644/respons-pt-djarum-soal-penggeledahan-kpk</t>
+          <t>https://www.liputan6.com/news/read/8324447/kubu-gibran-tunjukkan-riwayat-pendidikan-penggugat-soroti-bukti-penyetaraan</t>
         </is>
       </c>
     </row>
@@ -2373,22 +2397,22 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Infografis: 10 Negara Termiskin di Asia</t>
+          <t>Bibit Siklon Tropis 91B Picu Potensi Hujan Lebat di Sumatra Bagian Utara</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Wed, 28 Oct 2026 22:33:49 +0700</t>
+          <t>Thu, 29 Oct 2026 20:19:04 +0700</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Dari Afghanistan hingga Bangladesh, berikut 10 negara Asia dengan PDB per kapita terendah.</t>
+          <t>BNPB memperingatkan potensi hujan sedang hingga lebat di Aceh dan Sumatera Utara akibat bibit siklon tropis 91B di Teluk Andaman</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8323635/infografis-10-negara-termiskin-di-asia</t>
+          <t>https://www.liputan6.com/news/read/8324444/bibit-siklon-tropis-91b-picu-potensi-hujan-lebat-di-sumatra-bagian-utara</t>
         </is>
       </c>
     </row>
@@ -2400,22 +2424,22 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Kepala BGN Usul Pelajaran Gizi di Sekolah Lewat MBG</t>
+          <t>Prabowo Sebut Olahraga Jadi Simbol Kehormatan Bangsa</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Wed, 28 Oct 2026 21:57:08 +0700</t>
+          <t>Thu, 29 Oct 2026 19:55:00 +0700</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Kepala BGN Sudaryono mendorong edukasi gizi masuk kurikulum sekolah melalui program MBG.</t>
+          <t>Prabowo Subianto menyerahkan bonus kepada atlet berprestasi Asian Games dan Para Games.</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8323620/kepala-bgn-usul-pelajaran-gizi-di-sekolah-lewat-mbg</t>
+          <t>https://www.liputan6.com/news/read/8324424/prabowo-sebut-olahraga-jadi-simbol-kehormatan-bangsa</t>
         </is>
       </c>
     </row>
@@ -2427,22 +2451,22 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Suasana Ricuh Demo Sumpah Pemuda di Kawasan Dukuh Atas</t>
+          <t>Momen Massa Trisakti Bakar Flare Sebelum Bubarkan Diri</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Wed, 28 Oct 2026 21:56:34 +0700</t>
+          <t>Thu, 29 Oct 2026 20:32:54 +0700</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Aksi demonstrasi memperingati Hari Sumpah Pemuda yang digelar Badan Eksekutif Mahasiswa Universitas Indonesia (BEM UI) bersama Komite Selamatkan Daulat Rakyat (SADAR) di kawasan Dukuh Atas Jalan Jenderal Sudirman, Jakarta Pusat, Rabu (28/10/2026), berujung ricuh menjelang malam hari. Situasi memanas</t>
+          <t>Massa mahasiswa Universitas Trisakti menggelar demonstrasi di kawasan Patung Kuda, Jalan Medan Merdeka Selatan, Jakpus.</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/photo/read/8323619/suasana-ricuh-demo-sumpah-pemuda-di-kawasan-dukuh-atas</t>
+          <t>https://www.liputan6.com/news/read/8324416/momen-massa-trisakti-bakar-flare-sebelum-bubarkan-diri</t>
         </is>
       </c>
     </row>
@@ -2454,22 +2478,22 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>KPK Periksa 4 Saksi soal Dugaan Imbalan Swasta di Kasus BNPB</t>
+          <t>Silmy Karim Melawan Usai Didakwa Terlibat Pemerasan WNA Rp 168 M</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Wed, 28 Oct 2026 21:14:09 +0700</t>
+          <t>Thu, 29 Oct 2026 19:38:38 +0700</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Penyidik KPK mendalami dugaan suap dan benturan kepentingan dalam proyek penanggulangan bencana di BNPB.</t>
+          <t>Kubu Silmy Karim membutuhkan waktu sekitar satu pekan untuk mempersiapkan nota perlawanan.</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8323603/kpk-periksa-4-saksi-soal-dugaan-imbalan-swasta-di-kasus-bnpb</t>
+          <t>https://www.liputan6.com/news/read/8324415/silmy-karim-melawan-usai-didakwa-terlibat-pemerasan-wna-rp-168-m</t>
         </is>
       </c>
     </row>
@@ -2481,22 +2505,22 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Situasi Terkini Bundaran HI Usai Massa Demo Bubar</t>
+          <t>Jadi Saksi Sidang Kuota Haji, Anwar Abbas Sebut Yaqut Bijaksana</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Wed, 28 Oct 2026 21:01:25 +0700</t>
+          <t>Thu, 29 Oct 2026 19:17:26 +0700</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Pembukaan jalan dilakukan bertahap, memastikan kelancaran kendaraan.</t>
+          <t>Ketua PP Muhammadiyah Anwar Abbas menyoroti kebijakan haji saat Yaqut Cholil Qoumas menjabat Menteri Agama.</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8323593/situasi-terkini-bundaran-hi-usai-massa-demo-bubar</t>
+          <t>https://www.liputan6.com/news/read/8324404/jadi-saksi-sidang-kuota-haji-anwar-abbas-sebut-yaqut-bijaksana</t>
         </is>
       </c>
     </row>
@@ -2508,22 +2532,22 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Kericuhan Pecah di DPRD DIY, Massa Berpakaian Hitam Bentrok dengan Polisi</t>
+          <t>Silmy Karim Perintahkan Bawahan Bayar Kuliah S3 Rp 50 Juta</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Wed, 28 Oct 2026 21:24:34 +0700</t>
+          <t>Thu, 29 Oct 2026 19:15:00 +0700</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Massa terlibat bentrokan dengan polisi dan masyarakat sekitar yang membantu penjagaan.</t>
+          <t>Silmy Karim disebut perintahkan bawahan bayar Rp 50 juta untuk kuliah S3 dari uang kas, diduga hasil pungli.</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8323607/kericuhan-pecah-di-dprd-diy-massa-berpakaian-hitam-bentrok-dengan-polisi</t>
+          <t>https://www.liputan6.com/news/read/8324397/silmy-karim-perintahkan-bawahan-bayar-kuliah-s3-rp-50-juta</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data pasar & berita - 2026-10-30 01:23 UTC
</commit_message>
<xml_diff>
--- a/data/market_news_latest.xlsx
+++ b/data/market_news_latest.xlsx
@@ -422,7 +422,7 @@
     <col width="26" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
   </cols>
@@ -487,20 +487,20 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>5098.0571</v>
+        <v>5282.312</v>
       </c>
       <c r="F2" t="n">
-        <v>-184.2549</v>
+        <v>16.1821</v>
       </c>
       <c r="G2" t="n">
-        <v>-3.49</v>
+        <v>0.31</v>
       </c>
       <c r="H2" t="n">
-        <v>0</v>
+        <v>301071800</v>
       </c>
     </row>
     <row r="3">
@@ -525,16 +525,16 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>7718.0498</v>
+        <v>7720.3901</v>
       </c>
       <c r="F3" t="n">
-        <v>-25.9302</v>
+        <v>-23.5898</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.33</v>
+        <v>-0.3</v>
       </c>
       <c r="H3" t="n">
-        <v>924439246</v>
+        <v>3300311000</v>
       </c>
     </row>
     <row r="4">
@@ -559,16 +559,16 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>52361.3398</v>
+        <v>52342.5586</v>
       </c>
       <c r="F4" t="n">
-        <v>-113.7617</v>
+        <v>-132.543</v>
       </c>
       <c r="G4" t="n">
-        <v>-0.22</v>
+        <v>-0.25</v>
       </c>
       <c r="H4" t="n">
-        <v>188869776</v>
+        <v>549807356</v>
       </c>
     </row>
     <row r="5">
@@ -593,16 +593,16 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>26205.1895</v>
+        <v>26184.7246</v>
       </c>
       <c r="F5" t="n">
-        <v>-344.6602</v>
+        <v>-365.125</v>
       </c>
       <c r="G5" t="n">
-        <v>-1.3</v>
+        <v>-1.38</v>
       </c>
       <c r="H5" t="n">
-        <v>2158787000</v>
+        <v>6506000000</v>
       </c>
     </row>
     <row r="6">
@@ -623,20 +623,20 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>63954.1914</v>
+        <v>63036.3008</v>
       </c>
       <c r="F6" t="n">
-        <v>685.8203</v>
+        <v>-917.8905999999999</v>
       </c>
       <c r="G6" t="n">
-        <v>1.08</v>
+        <v>-1.44</v>
       </c>
       <c r="H6" t="n">
-        <v>165400000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -657,20 +657,20 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>22958.6504</v>
+        <v>23094.8301</v>
       </c>
       <c r="F7" t="n">
-        <v>-136.1797</v>
+        <v>53.5098</v>
       </c>
       <c r="G7" t="n">
-        <v>-0.59</v>
+        <v>0.23</v>
       </c>
       <c r="H7" t="n">
-        <v>0</v>
+        <v>2397000000</v>
       </c>
     </row>
     <row r="8">
@@ -694,15 +694,9 @@
           <t>2026-10-29</t>
         </is>
       </c>
-      <c r="E8" t="n">
-        <v>3651.4336</v>
-      </c>
-      <c r="F8" t="n">
-        <v>-30.0354</v>
-      </c>
-      <c r="G8" t="n">
-        <v>-0.82</v>
-      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
       <c r="H8" t="n">
         <v>1406741440</v>
       </c>
@@ -725,20 +719,20 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>10749.9004</v>
+        <v>10694.5</v>
       </c>
       <c r="F9" t="n">
-        <v>55.4004</v>
+        <v>8</v>
       </c>
       <c r="G9" t="n">
-        <v>0.52</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="H9" t="n">
-        <v>0</v>
+        <v>694027600</v>
       </c>
     </row>
     <row r="10">
@@ -759,20 +753,20 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>26061.7793</v>
+        <v>25704.0195</v>
       </c>
       <c r="F10" t="n">
-        <v>357.7598</v>
+        <v>113.25</v>
       </c>
       <c r="G10" t="n">
-        <v>1.39</v>
+        <v>0.44</v>
       </c>
       <c r="H10" t="n">
-        <v>0</v>
+        <v>49500500</v>
       </c>
     </row>
     <row r="11">
@@ -793,17 +787,17 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>5396.0298</v>
+        <v>5395.1401</v>
       </c>
       <c r="F11" t="n">
-        <v>-1.8804</v>
+        <v>-2.77</v>
       </c>
       <c r="G11" t="n">
-        <v>-0.03</v>
+        <v>-0.05</v>
       </c>
       <c r="H11" t="n">
         <v>0</v>
@@ -827,17 +821,17 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="E12" t="n">
         <v>18128</v>
       </c>
       <c r="F12" t="n">
-        <v>-11.5</v>
+        <v>62.5996</v>
       </c>
       <c r="G12" t="n">
-        <v>-0.06</v>
+        <v>0.35</v>
       </c>
       <c r="H12" t="n">
         <v>0</v>
@@ -865,13 +859,13 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>102.017</v>
+        <v>101.634</v>
       </c>
       <c r="F13" t="n">
-        <v>-0.173</v>
+        <v>-0.556</v>
       </c>
       <c r="G13" t="n">
-        <v>-0.17</v>
+        <v>-0.54</v>
       </c>
       <c r="H13" t="n">
         <v>0</v>
@@ -895,17 +889,17 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>157.851</v>
+        <v>157.369</v>
       </c>
       <c r="F14" t="n">
-        <v>-0.142</v>
+        <v>-0.464</v>
       </c>
       <c r="G14" t="n">
-        <v>-0.09</v>
+        <v>-0.29</v>
       </c>
       <c r="H14" t="n">
         <v>0</v>
@@ -933,13 +927,13 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>0.4966</v>
+        <v>0.4989</v>
       </c>
       <c r="F15" t="n">
-        <v>-0.007900000000000001</v>
+        <v>-0.0056</v>
       </c>
       <c r="G15" t="n">
-        <v>-1.57</v>
+        <v>-1.11</v>
       </c>
       <c r="H15" t="n">
         <v>0</v>
@@ -967,13 +961,13 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>0.531</v>
+        <v>0.5329</v>
       </c>
       <c r="F16" t="n">
-        <v>-0.0051</v>
+        <v>-0.0032</v>
       </c>
       <c r="G16" t="n">
-        <v>-0.95</v>
+        <v>-0.6</v>
       </c>
       <c r="H16" t="n">
         <v>0</v>
@@ -1001,13 +995,13 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>0.3982</v>
+        <v>0.3998</v>
       </c>
       <c r="F17" t="n">
-        <v>-0.0013</v>
+        <v>0.0003</v>
       </c>
       <c r="G17" t="n">
-        <v>-0.33</v>
+        <v>0.08</v>
       </c>
       <c r="H17" t="n">
         <v>0</v>
@@ -1034,17 +1028,11 @@
           <t>2026-10-29</t>
         </is>
       </c>
-      <c r="E18" t="n">
-        <v>81.55500000000001</v>
-      </c>
-      <c r="F18" t="n">
-        <v>0.5649999999999999</v>
-      </c>
-      <c r="G18" t="n">
-        <v>0.7</v>
-      </c>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
       <c r="H18" t="n">
-        <v>9208615</v>
+        <v>25798836</v>
       </c>
     </row>
     <row r="19">
@@ -1068,17 +1056,11 @@
           <t>2026-10-29</t>
         </is>
       </c>
-      <c r="E19" t="n">
-        <v>77.5976</v>
-      </c>
-      <c r="F19" t="n">
-        <v>0.0076</v>
-      </c>
-      <c r="G19" t="n">
-        <v>0.01</v>
-      </c>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr"/>
       <c r="H19" t="n">
-        <v>18334013</v>
+        <v>51350114</v>
       </c>
     </row>
     <row r="20">
@@ -1103,16 +1085,16 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>4042.2</v>
+        <v>4010</v>
       </c>
       <c r="F20" t="n">
-        <v>-9.4001</v>
+        <v>-41.6001</v>
       </c>
       <c r="G20" t="n">
-        <v>-0.23</v>
+        <v>-1.03</v>
       </c>
       <c r="H20" t="n">
-        <v>98721</v>
+        <v>12321</v>
       </c>
     </row>
     <row r="21">
@@ -1137,16 +1119,16 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>100.27</v>
+        <v>102.83</v>
       </c>
       <c r="F21" t="n">
-        <v>-2.51</v>
+        <v>0.05</v>
       </c>
       <c r="G21" t="n">
-        <v>-2.44</v>
+        <v>0.05</v>
       </c>
       <c r="H21" t="n">
-        <v>136117</v>
+        <v>8239</v>
       </c>
     </row>
     <row r="22">
@@ -1171,16 +1153,16 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>109.56</v>
+        <v>111.57</v>
       </c>
       <c r="F22" t="n">
-        <v>-5.76</v>
+        <v>-3.75</v>
       </c>
       <c r="G22" t="n">
-        <v>-4.99</v>
+        <v>-3.25</v>
       </c>
       <c r="H22" t="n">
-        <v>21059</v>
+        <v>1397</v>
       </c>
     </row>
     <row r="23">
@@ -1205,16 +1187,16 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>6.58</v>
+        <v>6.542</v>
       </c>
       <c r="F23" t="n">
-        <v>-0.0615</v>
+        <v>-0.09950000000000001</v>
       </c>
       <c r="G23" t="n">
-        <v>-0.93</v>
+        <v>-1.5</v>
       </c>
       <c r="H23" t="n">
-        <v>24204</v>
+        <v>2474</v>
       </c>
     </row>
     <row r="24">
@@ -1238,17 +1220,11 @@
           <t>2026-10-29</t>
         </is>
       </c>
-      <c r="E24" t="n">
-        <v>62.68</v>
-      </c>
-      <c r="F24" t="n">
-        <v>-0.84</v>
-      </c>
-      <c r="G24" t="n">
-        <v>-1.32</v>
-      </c>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr"/>
       <c r="H24" t="n">
-        <v>4896291</v>
+        <v>22053571</v>
       </c>
     </row>
     <row r="25">
@@ -1273,13 +1249,13 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>16.81</v>
+        <v>17.2</v>
       </c>
       <c r="F25" t="n">
-        <v>-0.1</v>
+        <v>0.29</v>
       </c>
       <c r="G25" t="n">
-        <v>-0.59</v>
+        <v>1.71</v>
       </c>
       <c r="H25" t="n">
         <v>0</v>
@@ -1303,20 +1279,20 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="E26" t="n">
-        <v>81201.7812</v>
+        <v>76806.5938</v>
       </c>
       <c r="F26" t="n">
-        <v>-65.8047</v>
+        <v>-4460.9922</v>
       </c>
       <c r="G26" t="n">
-        <v>-0.08</v>
+        <v>-5.49</v>
       </c>
       <c r="H26" t="n">
-        <v>27420071936</v>
+        <v>48511234048</v>
       </c>
     </row>
     <row r="27">
@@ -1749,22 +1725,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>GOTO Cetak Laba Rp 441 Miliar</t>
+          <t>Bank Sentral Eropa Tahan Suku Bunga, Ada Sinyal Kenaikan di Akhir Tahun</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Thu, 29 Oct 2026 21:41:04 +0700</t>
+          <t>Fri, 30 Oct 2026 08:11:38 +0700</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/20/goto-rilis-model-llm-27b-paham-bahasa-indonesia-hingga-daerah-1792493682697_169.jpeg?w=360&amp;amp;q=90" /&gt; PT GoTo Gojek Tokopedia Tbk (GOTO) mencatat laba bersih Rp 441 miliar pada kuartal III-2026.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2017/04/06/2945e8b1-4fe5-47aa-833f-748663cb4abe_169.jpeg?w=360&amp;amp;q=90" /&gt; Bank Sentral Eropa (ECB) menahan suku bunga acuannya di level 2,5% pada Kamis (29/10).</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/bursa-dan-valas/d-8730220/goto-cetak-laba-rp-441-miliar</t>
+          <t>https://finance.detik.com/moneter/d-8730465/bank-sentral-eropa-tahan-suku-bunga-ada-sinyal-kenaikan-di-akhir-tahun</t>
         </is>
       </c>
     </row>
@@ -1776,22 +1752,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Laba PTBA Melonjak, Capai Rp 4,41 Triliun hingga Triwulan III 2026</t>
+          <t>Dari Dapur ke Pesawat, Minyak Jelantah Dibeli hingga Rp6.000 per Liter</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Thu, 29 Oct 2026 21:34:47 +0700</t>
+          <t>Fri, 30 Oct 2026 08:00:32 +0700</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/29/ptba-1793284413718_169.jpeg?w=360&amp;amp;q=90" /&gt; PT Bukit Asam (PTBA) laporkan laba bersih Rp 4,41 triliun hingga September 2026. Kinerja operasional pulih dengan produksi dan penjualan meningkat.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/29/dari-dapur-ke-pesawat-minyak-jelantah-dibeli-hingga-rp6000-per-liter-1793265451125_169.jpeg?w=360&amp;amp;q=90" /&gt; Warga Banyumas mengumpulkan minyak jelantah dengan harga Rp5.000-Rp6.000 per liter untuk diolah menjadi bahan bakar pe</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/bursa-dan-valas/d-8730215/laba-ptba-melonjak-capai-rp-4-41-triliun-hingga-triwulan-iii-2026</t>
+          <t>https://finance.detik.com/foto-bisnis/d-8729719/dari-dapur-ke-pesawat-minyak-jelantah-dibeli-hingga-rp6-000-per-liter</t>
         </is>
       </c>
     </row>
@@ -1803,22 +1779,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Prabowo Bakal Resmikan Pabrik Baterai Mobil Listrik di Karawang</t>
+          <t>BI Buka Suara soal Potensi Dolar AS Tembus Rp 22.000 Imbas MSCI</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Thu, 29 Oct 2026 20:58:34 +0700</t>
+          <t>Fri, 30 Oct 2026 07:58:00 +0700</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/08/27/baterai-mobil-listrik-1787794586277_169.jpeg?w=360&amp;amp;q=90" /&gt; Presiden Prabowo Subianto bakal meresmikan pabrik baterai mobil listrik di Karawang, kerja sama CATL dan Antam.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/29/detik-pagi-bi-buka-suara-soal-potensi-dolar-as-tembus-rp-22000-imbas-msci-1793285659063_169.jpeg?w=360&amp;amp;q=90" /&gt; Rupiah disebut bisa semakin terpuruk imbas keputusan MSCI. Hal ini diungkap oleh Ketua Dewan Penasihat Kadin Indo</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/industri/d-8730191/prabowo-bakal-resmikan-pabrik-baterai-mobil-listrik-di-karawang</t>
+          <t>https://finance.detik.com/bursa-dan-valas/d-8730205/bi-buka-suara-soal-potensi-dolar-as-tembus-rp-22-000-imbas-msci</t>
         </is>
       </c>
     </row>
@@ -1830,22 +1806,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Investor AS Pede MSCI Tak Turunkan Kasta Bursa RI, Ini Alasannya</t>
+          <t>Oplos Beras Rugikan Negara Rp 3,3 Miliar, 8 Pejabat Dicopot</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Thu, 29 Oct 2026 20:30:03 +0700</t>
+          <t>Fri, 30 Oct 2026 07:55:00 +0700</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/16/ihsg-ambruk-1157-ditutup-di-level-5185-1792144638880_169.jpeg?w=360&amp;amp;q=90" /&gt; Investor Amerika Serikat (AS) sekaligus Anggota Komite High Shareholding Concentration (HSC), Chapman Taylor, meyakini pasar modal Indonesia tidak t</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/17/harga-beras-di-pasar-serpong-tangerang-selatan-pada-kamis-17092026-rata-rata-cenderung-stabil-di-bawah-angka-rp-14000-per-lite-1789644359234_169.jpeg?w=360&amp;amp;q=90" /&gt; Oplos beras SPHP menjadi premium di Jakarta Timur terkuak. P</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/bursa-dan-valas/d-8730091/investor-as-pede-msci-tak-turunkan-kasta-bursa-ri-ini-alasannya</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8730179/oplos-beras-rugikan-negara-rp-3-3-miliar-8-pejabat-dicopot</t>
         </is>
       </c>
     </row>
@@ -1857,22 +1833,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Minerba Convex 2026 Digelar 2-3 November, Ada Klinik RKAB hingga Zona Anak</t>
+          <t>QRIS Cross-Border Bikin Transaksi di Luar Negeri Lebih Mudah &amp;amp; Praktis</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Thu, 29 Oct 2026 20:23:05 +0700</t>
+          <t>Fri, 30 Oct 2026 07:45:21 +0700</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/29/kementerian-esdm-1793280061440_169.jpeg?w=360&amp;amp;q=90" /&gt; Minerba Convex 2026 di Jakarta mengajak masyarakat mengenal sektor pertambangan. Acara ini menawarkan edukasi, penghargaan, dan konsultasi untuk pelaku usaha.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2020/10/04/solo-traveling.jpeg?w=360&amp;amp;q=90" /&gt; QRIS Cross-Border memudahkan pembayaran di luar negeri tanpa uang tunai. Cukup scan QR dengan aplikasi yang mendukung, transaksi jadi cepat dan aman.</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8730161/minerba-convex-2026-digelar-2-3-november-ada-klinik-rkab-hingga-zona-anak</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8727732/qris-cross-border-bikin-transaksi-di-luar-negeri-lebih-mudah-praktis</t>
         </is>
       </c>
     </row>
@@ -1884,22 +1860,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Impor BBM-LPG Kini Lewat Lemigas, Bakal Lebih Murah?</t>
+          <t>Hashim Sebut di Medsos Banyak yang Bohong soal Utang Indonesia</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Thu, 29 Oct 2026 20:00:00 +0700</t>
+          <t>Fri, 30 Oct 2026 07:25:00 +0700</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/03/09/harga-minyak-mentah-hampir-us110-dunia-dilanda-kepanikan-1773053712369_169.jpeg?w=360&amp;amp;q=90" /&gt; Pemerintah ubah mekanisme impor minyak dan gas lewat BLU Lemigas, skema ini disebut membuat pengadaan jadi mudah dan cepat.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2024/10/31/hashim-djojohadikusumo-bertemu-ahy_169.jpeg?w=360&amp;amp;q=90" /&gt; Ketua Dewan Penasihat Kadin Hashim Djojohadikusumo menepis isu krisis utang Indonesia yang muncul di media sosial.</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8730095/impor-bbm-lpg-kini-lewat-lemigas-bakal-lebih-murah</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8730168/hashim-sebut-di-medsos-banyak-yang-bohong-soal-utang-indonesia</t>
         </is>
       </c>
     </row>
@@ -1911,22 +1887,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Denda Rp 2,1 Triliun di Kasus DSSA, BREN, dan CUAN Sudah Dibayar</t>
+          <t>Jawaban Bos Kadin soal Tudingan RI di Ambang Krisis</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Thu, 29 Oct 2026 19:30:47 +0700</t>
+          <t>Fri, 30 Oct 2026 06:55:00 +0700</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/27/ketua-dewan-komisioner-ojk-friderica-widyasari-dewi-1793077340311_169.jpeg?w=360&amp;amp;q=90" /&gt; Ketua Dewan Komisioner OJK Friderica Widyasari Dewi, mengaku pihaknya telah menerima pembayaran denda dari pelanggaran pasar modal sebe</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/29/ketua-umum-kadin-indonesia-anindya-novyan-bakrie-1793261193891_169.jpeg?w=360&amp;amp;q=90" /&gt; Ketua Umum Kadin Indonesia, Anindya Novyan Bakrie, menegaskan ekonomi Indonesia saat ini masih jauh lebih baik dibandingkan saat krisis 19</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/bursa-dan-valas/d-8730078/denda-rp-2-1-triliun-di-kasus-dssa-bren-dan-cuan-sudah-dibayar</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8730172/jawaban-bos-kadin-soal-tudingan-ri-di-ambang-krisis</t>
         </is>
       </c>
     </row>
@@ -1938,22 +1914,22 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Panen Marigold di Meksiko, Bunga untuk Menyambut Arwah Leluhur</t>
+          <t>Pembalut Masih Dikenai Pajak, Ini Alasannya</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Thu, 29 Oct 2026 19:02:44 +0700</t>
+          <t>Fri, 30 Oct 2026 06:25:00 +0700</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/29/panen-marigold-di-meksiko-bunga-untuk-menyambut-arwah-leluhur-1793251008236.jpeg?w=360&amp;amp;q=90" /&gt; Petani memanen bunga marigold di Atlixco, Meksiko, menjelang perayaan Hari Orang Mati pada awal November.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2022/10/18/pembalut-nifas_169.jpeg?w=360&amp;amp;q=90" /&gt; Ramai di media sosial (medsos) pembalut dikenakan pajak. Netizen mempertanyakan alasan pembalut masih kena pajak, padahal merupakan kebutuhan dasar perempuan.</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/foto-bisnis/d-8729219/panen-marigold-di-meksiko-bunga-untuk-menyambut-arwah-leluhur</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8730154/pembalut-masih-dikenai-pajak-ini-alasannya</t>
         </is>
       </c>
     </row>
@@ -1965,22 +1941,22 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Hashim Sebut Dolar AS bisa Tembus Rp 22.000 Gegara MSCI, Bos BI Buka Suara</t>
+          <t>Hashim Ungkap Dampak Ngeri Pengumuman MSCI</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Thu, 29 Oct 2026 19:00:39 +0700</t>
+          <t>Fri, 30 Oct 2026 05:55:00 +0700</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/21/bank-indonesia-bi-memutuskan-menaikkan-suku-bunga-deposit-facility-sebesar-25-basis-poin-bps-menjadi-5-keputusan-tersebut-diam-1792576096896_169.jpeg?w=360&amp;amp;q=90" /&gt; Gubernur Bank Indonesia (BI), Destry Damayanti, buka suara s</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2024/11/12/hashim-dalam-cop-29_169.png?w=360&amp;amp;q=90" /&gt; Ketua Dewan Penasihat Kadin Hashim Djojohadikusumo mengungkap dampak buruk jika MSCI jadi menurunkan kasta pasar modal Indonesia ke Standalone Market.</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/bursa-dan-valas/d-8730007/hashim-sebut-dolar-as-bisa-tembus-rp-22-000-gegara-msci-bos-bi-buka-suara</t>
+          <t>https://finance.detik.com/bursa-dan-valas/d-8730131/hashim-ungkap-dampak-ngeri-pengumuman-msci</t>
         </is>
       </c>
     </row>
@@ -1992,22 +1968,22 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Bahlil Tuding Singapura Jual Lagi Pasokan Gas dari RI</t>
+          <t>Integrasi Tarif Tol Jabodetabek Bisakah Dilakukan? Ini Jawabannya</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Thu, 29 Oct 2026 18:55:53 +0700</t>
+          <t>Thu, 29 Oct 2026 22:37:00 +0700</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/14/bahlil-lahadalia-rolandodetikcom-1791978307056_169.jpeg?w=360&amp;amp;q=90" /&gt; Menko Hilirisasi dan Transisi Energi Bahlil Lahadalia menduga sebagian LNG yang diekspor dari Indonesia dijual lagi oleh Singapura ke negara lain.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2020/11/05/rencana-kenikan-tarif-tol-lingkar-luar-jakarta-3_169.jpeg?w=360&amp;amp;q=90" /&gt; Integrasi tarif tol Jabodetabek dinilai bisa membuat perjalanan lebih lancar, biaya terjangkau, dan akses ke kawasan industri dan pelabuhan yang efisien</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8730027/bahlil-tuding-singapura-jual-lagi-pasokan-gas-dari-ri</t>
+          <t>https://finance.detik.com/infrastruktur/d-8730303/integrasi-tarif-tol-jabodetabek-bisakah-dilakukan-ini-jawabannya</t>
         </is>
       </c>
     </row>
@@ -2019,22 +1995,22 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Bos BI Buka-bukaan soal MSCI Bikin Investor Asing Bingung</t>
+          <t>Kopdes Jadi Titik Kumpul Minyak Jelantah Sebelum 'Disulap' Jadi Bioavtur</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Thu, 29 Oct 2026 18:30:37 +0700</t>
+          <t>Thu, 29 Oct 2026 22:30:00 +0700</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/29/gubernur-bank-indonesia-bi-destry-damayanti-1793272001596_169.jpeg?w=360&amp;amp;q=90" /&gt; Gubernur Bank Indonesia (BI), Destry Damayanti, mengaku menerima sejumlah keluhan dari raksasa investor asing terkait dengan persoalan MSCI.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/21/kopdes-merah-putih-bersiap-operasional-23-ribu-bangunan-telah-rampung-1789986171319_169.jpeg?w=360&amp;amp;q=90" /&gt; PT Pertamina Patra Niaga bersama Kementerian Koperasi memulai program percontohan pengumpulan minyak jelantah berbasi</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/bursa-dan-valas/d-8729933/bos-bi-buka-bukaan-soal-msci-bikin-investor-asing-bingung</t>
+          <t>https://finance.detik.com/energi/d-8730274/kopdes-jadi-titik-kumpul-minyak-jelantah-sebelum-disulap-jadi-bioavtur</t>
         </is>
       </c>
     </row>
@@ -2046,22 +2022,22 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Bocoran Hashim: Shopee-GoTo Pungut Pajak Digital Mulai 9 November 2026</t>
+          <t>Garuda Cetak Pendapatan Rp 49,24 Triliun di Tengah Tekanan Harga Avtur</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Thu, 29 Oct 2026 18:08:52 +0700</t>
+          <t>Thu, 29 Oct 2026 22:02:21 +0700</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2024/11/14/hashim-djojohadikusumo-1_169.jpeg?w=360&amp;amp;q=90" /&gt; Ketua Dewan Penasihat Kadin Hashim Djojohadikusumo menyebut GoTo hingga Shopee bakal pungut pajak digital mulai bulan depan.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/07/19/pesawat-garuda-indonesia-1752916632356_169.jpeg?w=360&amp;amp;q=90" /&gt; PT Garuda Indonesia (Persero) Tbk (GIAA) membukukan pertumbuhan pendapatan konsolidasi sebesar 13,2% menjadi US$ 2,71 miliar atau sekitar Rp 49,24 triliun.</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8729936/bocoran-hashim-shopee-goto-pungut-pajak-digital-mulai-9-november-2026</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8730237/garuda-cetak-pendapatan-rp-49-24-triliun-di-tengah-tekanan-harga-avtur</t>
         </is>
       </c>
     </row>
@@ -2073,22 +2049,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>MSCI Soroti Pasar Modal RI, Rosan Beri Bukti Investor Masih Percaya</t>
+          <t>GOTO Cetak Laba Rp 441 Miliar</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Thu, 29 Oct 2026 17:45:00 +0700</t>
+          <t>Thu, 29 Oct 2026 21:41:04 +0700</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/11/20/menteri-investasi-dan-hilirisasikepala-bkpm-rosan-roeslani-1763634019135_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Investasi Rosan Roeslani menyatakan kepercayaan investor terhadap Indonesia tetap tinggi, dengan realisasi investasi men</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/20/goto-rilis-model-llm-27b-paham-bahasa-indonesia-hingga-daerah-1792493682697_169.jpeg?w=360&amp;amp;q=90" /&gt; PT GoTo Gojek Tokopedia Tbk (GOTO) mencatat laba bersih Rp 441 miliar pada kuartal III-2026.</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8729905/msci-soroti-pasar-modal-ri-rosan-beri-bukti-investor-masih-percaya</t>
+          <t>https://finance.detik.com/bursa-dan-valas/d-8730220/goto-cetak-laba-rp-441-miliar</t>
         </is>
       </c>
     </row>
@@ -2100,22 +2076,22 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Revisi RKAB Rampung: Nikel 300 Juta Ton-Batu Bara 700 Juta Ton</t>
+          <t>Laba PTBA Melonjak, Capai Rp 4,41 Triliun hingga Triwulan III 2026</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Thu, 29 Oct 2026 17:36:21 +0700</t>
+          <t>Thu, 29 Oct 2026 21:34:47 +0700</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2021/09/10/ada-di-sumsel-tambang-batu-bara-ini-punya-cadangan-3-miliar-ton-6_169.jpeg?w=360&amp;amp;q=90" /&gt; Kementerian ESDM menerbitkan revisi RKAB 2026, dengan produksi nikel sekitar 300 juta ton dan batu bara 700 juta ton.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/29/ptba-1793284413718_169.jpeg?w=360&amp;amp;q=90" /&gt; PT Bukit Asam (PTBA) laporkan laba bersih Rp 4,41 triliun hingga September 2026. Kinerja operasional pulih dengan produksi dan penjualan meningkat.</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8729888/revisi-rkab-rampung-nikel-300-juta-ton-batu-bara-700-juta-ton</t>
+          <t>https://finance.detik.com/bursa-dan-valas/d-8730215/laba-ptba-melonjak-capai-rp-4-41-triliun-hingga-triwulan-iii-2026</t>
         </is>
       </c>
     </row>
@@ -2127,22 +2103,22 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>RI Rawan Bencana, OJK Dorong Sektor PPDP Jaga Ekonomi Warga</t>
+          <t>Prabowo Bakal Resmikan Pabrik Baterai Mobil Listrik di Karawang</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Thu, 29 Oct 2026 17:23:00 +0700</t>
+          <t>Thu, 29 Oct 2026 20:58:34 +0700</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/29/ojk-1793269261385_169.jpeg?w=360&amp;amp;q=90" /&gt; OJK luncurkan peta jalan keuangan berkelanjutan untuk sektor PPDP 2026-2030. Fokus pada mitigasi risiko bencana dan iklim demi stabilitas ekonomi Indonesia.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/08/27/baterai-mobil-listrik-1787794586277_169.jpeg?w=360&amp;amp;q=90" /&gt; Presiden Prabowo Subianto bakal meresmikan pabrik baterai mobil listrik di Karawang, kerja sama CATL dan Antam.</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/moneter/d-8729850/ri-rawan-bencana-ojk-dorong-sektor-ppdp-jaga-ekonomi-warga</t>
+          <t>https://finance.detik.com/industri/d-8730191/prabowo-bakal-resmikan-pabrik-baterai-mobil-listrik-di-karawang</t>
         </is>
       </c>
     </row>
@@ -2154,22 +2130,22 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Infografis: 100 Hari MBG di Tangan Sudaryono</t>
+          <t>Akal Bulus Silmy Karim Terbongkar di Persidangan</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Thu, 29 Oct 2026 21:58:48 +0700</t>
+          <t>Fri, 30 Oct 2026 07:30:56 +0700</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Sudaryono menerapkan sejumlah aturan untuk memperkuat keamanan pangan, kedisiplinan, dan transparansi program MBG.</t>
+          <t>Silmy Karim melawan atas dakwaan yang disampaikan dengan mengajukan eksepsi.</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8324499/infografis-100-hari-mbg-di-tangan-sudaryono</t>
+          <t>https://www.liputan6.com/news/read/8324597/akal-bulus-silmy-karim-terbongkar-di-persidangan</t>
         </is>
       </c>
     </row>
@@ -2181,22 +2157,22 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Rincian Bonus Atlet Asian Games dan Asian Para Games dari Prabowo</t>
+          <t>1,5 Tahun Berlalu, Induk Harimau Sumatera Kembali Terekam Bareng 3 Anaknya</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Thu, 29 Oct 2026 21:48:55 +0700</t>
+          <t>Fri, 30 Oct 2026 07:19:09 +0700</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Pemerintah memberikan bonus dengan besaran berbeda sesuai medali dan nomor pertandingan.</t>
+          <t>Mereka berkumpul di dekat bak penampungan air minum disediakan petugas.</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8324491/rincian-bonus-atlet-asian-games-dan-asian-para-games-dari-prabowo</t>
+          <t>https://www.liputan6.com/news/read/8324599/15-tahun-berlalu-induk-harimau-sumatera-kembali-terekam-bareng-3-anaknya</t>
         </is>
       </c>
     </row>
@@ -2208,22 +2184,22 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Kuasa Hukum Bantah Silmy Karim Terjaring OTT KPK</t>
+          <t>Kisah 'Pilot Darat' Antar Mahasiswa UI Terobos Barikade Polisi</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Thu, 29 Oct 2026 21:47:30 +0700</t>
+          <t>Thu, 29 Oct 2026 21:03:09 +0700</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Silmy Karim didakwa melakukan pemerasan terkait dokumen keimigrasian senilai Rp 168,9 miliar dan menerima gratifikasi Rp 33,8 miliar.</t>
+          <t>Marsudi punya keyakinan soal niat baik mahasiswa memperjuangkan nasib rakyat dan menyuarakan kondisi negara.</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8324487/kuasa-hukum-bantah-silmy-karim-terjaring-ott-kpk</t>
+          <t>https://www.liputan6.com/news/read/8324469/kisah-pilot-darat-antar-mahasiswa-ui-terobos-barikade-polisi</t>
         </is>
       </c>
     </row>
@@ -2235,22 +2211,22 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Seskab Teddy Beberkan Capaian Dua Tahun Pemerintahan Prabowo</t>
+          <t>Taktik Sudaryono Tutup Celah Rasuah BGN hingga MBG</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Thu, 29 Oct 2026 21:35:47 +0700</t>
+          <t>Fri, 30 Oct 2026 06:30:00 +0700</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Seskab melaporkan sejumlah capaian program prioritas dan pembangunan selama dua tahun pemerintahan Presiden Prabowo Subianto.</t>
+          <t>Sudaryono mengaku tidak melayani permintaan pengurusan dapur MBG melalui jalur pribadi.</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8324485/seskab-teddy-beberkan-capaian-dua-tahun-pemerintahan-prabowo</t>
+          <t>https://www.liputan6.com/news/read/8324582/taktik-sudaryono-tutup-celah-rasuah-bgn-hingga-mbg</t>
         </is>
       </c>
     </row>
@@ -2262,22 +2238,22 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>DPR: TNI Amankan Demo Hal Lumrah</t>
+          <t>12 Perusuh Saat Demo di Alun-Alun Tugu Malang Ditangkap, Bom Molotov Disita</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Thu, 29 Oct 2026 21:07:45 +0700</t>
+          <t>Fri, 30 Oct 2026 05:54:28 +0700</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Menurut Dave, aparat tetap harus memastikan aksi berlangsung aman dan tertib tanpa mengabaikan hak masyarakat</t>
+          <t>Hasil tes urine, mereka positif sabu.</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8324473/dpr-tni-amankan-demo-hal-lumrah</t>
+          <t>https://www.liputan6.com/news/read/8324580/12-perusuh-saat-demo-di-alun-alun-tugu-malang-ditangkap-bom-molotov-disita</t>
         </is>
       </c>
     </row>
@@ -2289,22 +2265,22 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Di Sidang Yaqut, Anwar Abbas Singgung Integritas dan Motif Finansial</t>
+          <t>Cerita Kepala BGN  Tiap Hari Didemo soal Program MBG</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Thu, 29 Oct 2026 21:31:54 +0700</t>
+          <t>Fri, 30 Oct 2026 01:00:13 +0700</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Dalam sidang dugaan korupsi kuota haji, Anwar Abbas menyebut Yaqut bukan orang miskin.</t>
+          <t>Sudaryono menyatakan terbuka terhadap kritik soal MBG, tetapi menegaskan pihaknya selektif dalam menanggapi demonstrasi yang dinilai hanya ikut-ikutan.</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8324464/di-sidang-yaqut-anwar-abbas-singgung-integritas-dan-motif-finansial</t>
+          <t>https://www.liputan6.com/news/read/8324563/cerita-kepala-bgn-tiap-hari-didemo-soal-program-mbg</t>
         </is>
       </c>
     </row>
@@ -2316,22 +2292,22 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Perintah Prabowo ke Erick Thohir soal Pembinaan Atlet</t>
+          <t>Kuasa Hukum: Uang Rp 186 M Bukan Milik Silmy Karim</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Thu, 29 Oct 2026 20:56:39 +0700</t>
+          <t>Fri, 30 Oct 2026 00:18:32 +0700</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Prabowo menilai Indonesia masih harus bekerja dan berjuang lebih keras untuk meningkatkan prestasi di ajang olahraga internasional.</t>
+          <t>Silmy didakwa melakukan pemerasan terhadap pemohon dokumen keimigrasian terkait izin tinggal WNA senilai Rp 168,9 miliar.</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8324463/perintah-prabowo-ke-erick-thohir-soal-pembinaan-atlet</t>
+          <t>https://www.liputan6.com/news/read/8324556/kuasa-hukum-uang-rp-186-m-bukan-milik-silmy-karim</t>
         </is>
       </c>
     </row>
@@ -2343,22 +2319,22 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Kondisi Terkini Medan Merdeka Selatan Usai Demo Mahasiswa Trisakti</t>
+          <t>RPTRA Kebon Sirih, Oase Hijau di Tengah Padatnya Jakarta</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Thu, 29 Oct 2026 20:25:30 +0700</t>
+          <t>Thu, 29 Oct 2026 22:46:04 +0700</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Kondisi Jalan Medan Merdeka Selatan normal kembali usai demo mahasiswa Trisakti.</t>
+          <t>Kebun sayur, kolam ikan, dan pengolahan sampah menjadi bagian dari upaya merawat lingkungan sekaligus kehidupan warga.</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8324449/kondisi-terkini-medan-merdeka-selatan-usai-demo-mahasiswa-trisakti</t>
+          <t>https://www.liputan6.com/news/read/8324517/rptra-kebon-sirih-oase-hijau-di-tengah-padatnya-jakarta</t>
         </is>
       </c>
     </row>
@@ -2370,22 +2346,22 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Kubu Gibran Tunjukkan Riwayat Pendidikan, Penggugat Soroti Bukti Penyetaraan</t>
+          <t>Waspada Banjir dan Longsor, Catat Sederet Imbauan BNPB</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Thu, 29 Oct 2026 20:24:04 +0700</t>
+          <t>Thu, 29 Oct 2026 22:43:06 +0700</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Rullyandi mengatakan dokumen riwayat pendidikan Gibran telah dilampirkan dalam jawaban pihak intervensi.</t>
+          <t>Imbauan bencana hidrometeorologi ini ditujukan kepada pemerintah, relawan hingga masyarakat</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8324447/kubu-gibran-tunjukkan-riwayat-pendidikan-penggugat-soroti-bukti-penyetaraan</t>
+          <t>https://www.liputan6.com/news/read/8324514/waspada-banjir-dan-longsor-catat-sederet-imbauan-bnpb</t>
         </is>
       </c>
     </row>
@@ -2397,22 +2373,22 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Bibit Siklon Tropis 91B Picu Potensi Hujan Lebat di Sumatra Bagian Utara</t>
+          <t>Residivis Jambret Lukai Korban di Depok Ditangkap</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Thu, 29 Oct 2026 20:19:04 +0700</t>
+          <t>Thu, 29 Oct 2026 22:33:17 +0700</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>BNPB memperingatkan potensi hujan sedang hingga lebat di Aceh dan Sumatera Utara akibat bibit siklon tropis 91B di Teluk Andaman</t>
+          <t>Korban mengalami luka dan dibawa ke rumah sakit oleh warga yang mengetahui kejadian tersebut.</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8324444/bibit-siklon-tropis-91b-picu-potensi-hujan-lebat-di-sumatra-bagian-utara</t>
+          <t>https://www.liputan6.com/news/read/8324509/residivis-jambret-lukai-korban-di-depok-ditangkap</t>
         </is>
       </c>
     </row>
@@ -2424,22 +2400,22 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Prabowo Sebut Olahraga Jadi Simbol Kehormatan Bangsa</t>
+          <t>Infografis: 100 Hari MBG di Tangan Sudaryono</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Thu, 29 Oct 2026 19:55:00 +0700</t>
+          <t>Thu, 29 Oct 2026 21:58:48 +0700</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Prabowo Subianto menyerahkan bonus kepada atlet berprestasi Asian Games dan Para Games.</t>
+          <t>Sudaryono menerapkan sejumlah aturan untuk memperkuat keamanan pangan, kedisiplinan, dan transparansi program MBG.</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8324424/prabowo-sebut-olahraga-jadi-simbol-kehormatan-bangsa</t>
+          <t>https://www.liputan6.com/news/read/8324499/infografis-100-hari-mbg-di-tangan-sudaryono</t>
         </is>
       </c>
     </row>
@@ -2451,22 +2427,22 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Momen Massa Trisakti Bakar Flare Sebelum Bubarkan Diri</t>
+          <t>Rincian Bonus Atlet Asian Games dan Asian Para Games dari Prabowo</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Thu, 29 Oct 2026 20:32:54 +0700</t>
+          <t>Thu, 29 Oct 2026 21:48:55 +0700</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Massa mahasiswa Universitas Trisakti menggelar demonstrasi di kawasan Patung Kuda, Jalan Medan Merdeka Selatan, Jakpus.</t>
+          <t>Pemerintah memberikan bonus dengan besaran berbeda sesuai medali dan nomor pertandingan.</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8324416/momen-massa-trisakti-bakar-flare-sebelum-bubarkan-diri</t>
+          <t>https://www.liputan6.com/news/read/8324491/rincian-bonus-atlet-asian-games-dan-asian-para-games-dari-prabowo</t>
         </is>
       </c>
     </row>
@@ -2478,22 +2454,22 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Silmy Karim Melawan Usai Didakwa Terlibat Pemerasan WNA Rp 168 M</t>
+          <t>Kuasa Hukum Bantah Silmy Karim Terjaring OTT KPK</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Thu, 29 Oct 2026 19:38:38 +0700</t>
+          <t>Thu, 29 Oct 2026 21:47:30 +0700</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Kubu Silmy Karim membutuhkan waktu sekitar satu pekan untuk mempersiapkan nota perlawanan.</t>
+          <t>Silmy Karim didakwa melakukan pemerasan terkait dokumen keimigrasian senilai Rp 168,9 miliar dan menerima gratifikasi Rp 33,8 miliar.</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8324415/silmy-karim-melawan-usai-didakwa-terlibat-pemerasan-wna-rp-168-m</t>
+          <t>https://www.liputan6.com/news/read/8324487/kuasa-hukum-bantah-silmy-karim-terjaring-ott-kpk</t>
         </is>
       </c>
     </row>
@@ -2505,22 +2481,22 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Jadi Saksi Sidang Kuota Haji, Anwar Abbas Sebut Yaqut Bijaksana</t>
+          <t>Seskab Teddy Beberkan Capaian Dua Tahun Pemerintahan Prabowo</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Thu, 29 Oct 2026 19:17:26 +0700</t>
+          <t>Thu, 29 Oct 2026 21:35:47 +0700</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Ketua PP Muhammadiyah Anwar Abbas menyoroti kebijakan haji saat Yaqut Cholil Qoumas menjabat Menteri Agama.</t>
+          <t>Seskab melaporkan sejumlah capaian program prioritas dan pembangunan selama dua tahun pemerintahan Presiden Prabowo Subianto.</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8324404/jadi-saksi-sidang-kuota-haji-anwar-abbas-sebut-yaqut-bijaksana</t>
+          <t>https://www.liputan6.com/news/read/8324485/seskab-teddy-beberkan-capaian-dua-tahun-pemerintahan-prabowo</t>
         </is>
       </c>
     </row>
@@ -2532,22 +2508,22 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Silmy Karim Perintahkan Bawahan Bayar Kuliah S3 Rp 50 Juta</t>
+          <t>DPR: TNI Amankan Demo Hal Lumrah</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Thu, 29 Oct 2026 19:15:00 +0700</t>
+          <t>Thu, 29 Oct 2026 21:07:45 +0700</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Silmy Karim disebut perintahkan bawahan bayar Rp 50 juta untuk kuliah S3 dari uang kas, diduga hasil pungli.</t>
+          <t>Menurut Dave, aparat tetap harus memastikan aksi berlangsung aman dan tertib tanpa mengabaikan hak masyarakat</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8324397/silmy-karim-perintahkan-bawahan-bayar-kuliah-s3-rp-50-juta</t>
+          <t>https://www.liputan6.com/news/read/8324473/dpr-tni-amankan-demo-hal-lumrah</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data pasar & berita - 2026-10-30 14:57 UTC
</commit_message>
<xml_diff>
--- a/data/market_news_latest.xlsx
+++ b/data/market_news_latest.xlsx
@@ -487,20 +487,20 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>5282.312</v>
+        <v>5057.0498</v>
       </c>
       <c r="F2" t="n">
-        <v>16.1821</v>
+        <v>-41.0073</v>
       </c>
       <c r="G2" t="n">
-        <v>0.31</v>
+        <v>-0.8</v>
       </c>
       <c r="H2" t="n">
-        <v>301071800</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -521,20 +521,20 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>7720.3901</v>
+        <v>7617.9102</v>
       </c>
       <c r="F3" t="n">
-        <v>-23.5898</v>
+        <v>-102.48</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.3</v>
+        <v>-1.33</v>
       </c>
       <c r="H3" t="n">
-        <v>3300311000</v>
+        <v>1055669000</v>
       </c>
     </row>
     <row r="4">
@@ -555,20 +555,20 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>52342.5586</v>
+        <v>52093.0195</v>
       </c>
       <c r="F4" t="n">
-        <v>-132.543</v>
+        <v>-249.5391</v>
       </c>
       <c r="G4" t="n">
-        <v>-0.25</v>
+        <v>-0.48</v>
       </c>
       <c r="H4" t="n">
-        <v>549807356</v>
+        <v>180560123</v>
       </c>
     </row>
     <row r="5">
@@ -589,20 +589,20 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>26184.7246</v>
+        <v>25611.877</v>
       </c>
       <c r="F5" t="n">
-        <v>-365.125</v>
+        <v>-572.8438</v>
       </c>
       <c r="G5" t="n">
-        <v>-1.38</v>
+        <v>-2.19</v>
       </c>
       <c r="H5" t="n">
-        <v>6506000000</v>
+        <v>2383002000</v>
       </c>
     </row>
     <row r="6">
@@ -627,13 +627,13 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>63036.3008</v>
+        <v>63290.1094</v>
       </c>
       <c r="F6" t="n">
-        <v>-917.8905999999999</v>
+        <v>-1369.3594</v>
       </c>
       <c r="G6" t="n">
-        <v>-1.44</v>
+        <v>-2.12</v>
       </c>
       <c r="H6" t="n">
         <v>0</v>
@@ -657,20 +657,20 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>23094.8301</v>
+        <v>23294.4199</v>
       </c>
       <c r="F7" t="n">
-        <v>53.5098</v>
+        <v>335.7695</v>
       </c>
       <c r="G7" t="n">
-        <v>0.23</v>
+        <v>1.46</v>
       </c>
       <c r="H7" t="n">
-        <v>2397000000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -691,14 +691,20 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>3599.0166</v>
+      </c>
+      <c r="F8" t="n">
+        <v>-52.4175</v>
+      </c>
+      <c r="G8" t="n">
+        <v>-1.44</v>
+      </c>
       <c r="H8" t="n">
-        <v>1406741440</v>
+        <v>2552753744</v>
       </c>
     </row>
     <row r="9">
@@ -719,20 +725,20 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>10694.5</v>
+        <v>10725.8496</v>
       </c>
       <c r="F9" t="n">
-        <v>8</v>
+        <v>3.75</v>
       </c>
       <c r="G9" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.03</v>
       </c>
       <c r="H9" t="n">
-        <v>694027600</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -753,20 +759,20 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>25704.0195</v>
+        <v>25870.7305</v>
       </c>
       <c r="F10" t="n">
-        <v>113.25</v>
+        <v>-168.9492</v>
       </c>
       <c r="G10" t="n">
-        <v>0.44</v>
+        <v>-0.65</v>
       </c>
       <c r="H10" t="n">
-        <v>49500500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -791,13 +797,13 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>5395.1401</v>
+        <v>5376.7402</v>
       </c>
       <c r="F11" t="n">
-        <v>-2.77</v>
+        <v>-19.2896</v>
       </c>
       <c r="G11" t="n">
-        <v>-0.05</v>
+        <v>-0.36</v>
       </c>
       <c r="H11" t="n">
         <v>0</v>
@@ -825,13 +831,13 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>18128</v>
+        <v>18138</v>
       </c>
       <c r="F12" t="n">
-        <v>62.5996</v>
+        <v>72.5996</v>
       </c>
       <c r="G12" t="n">
-        <v>0.35</v>
+        <v>0.4</v>
       </c>
       <c r="H12" t="n">
         <v>0</v>
@@ -855,17 +861,17 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>101.634</v>
+        <v>101.982</v>
       </c>
       <c r="F13" t="n">
-        <v>-0.556</v>
+        <v>-0.058</v>
       </c>
       <c r="G13" t="n">
-        <v>-0.54</v>
+        <v>-0.06</v>
       </c>
       <c r="H13" t="n">
         <v>0</v>
@@ -893,13 +899,13 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>157.369</v>
+        <v>157.294</v>
       </c>
       <c r="F14" t="n">
-        <v>-0.464</v>
+        <v>-0.539</v>
       </c>
       <c r="G14" t="n">
-        <v>-0.29</v>
+        <v>-0.34</v>
       </c>
       <c r="H14" t="n">
         <v>0</v>
@@ -923,17 +929,17 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>0.4989</v>
+        <v>0.4952</v>
       </c>
       <c r="F15" t="n">
-        <v>-0.0056</v>
+        <v>-0.0037</v>
       </c>
       <c r="G15" t="n">
-        <v>-1.11</v>
+        <v>-0.74</v>
       </c>
       <c r="H15" t="n">
         <v>0</v>
@@ -957,17 +963,17 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>0.5329</v>
+        <v>0.5316</v>
       </c>
       <c r="F16" t="n">
-        <v>-0.0032</v>
+        <v>-0.0013</v>
       </c>
       <c r="G16" t="n">
-        <v>-0.6</v>
+        <v>-0.24</v>
       </c>
       <c r="H16" t="n">
         <v>0</v>
@@ -991,17 +997,17 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>0.3998</v>
+        <v>0.3978</v>
       </c>
       <c r="F17" t="n">
-        <v>0.0003</v>
+        <v>-0.002</v>
       </c>
       <c r="G17" t="n">
-        <v>0.08</v>
+        <v>-0.5</v>
       </c>
       <c r="H17" t="n">
         <v>0</v>
@@ -1025,14 +1031,20 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>81.545</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0.055</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0.07000000000000001</v>
+      </c>
       <c r="H18" t="n">
-        <v>25798836</v>
+        <v>8008532</v>
       </c>
     </row>
     <row r="19">
@@ -1053,14 +1065,20 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>77.39</v>
+      </c>
+      <c r="F19" t="n">
+        <v>-0.19</v>
+      </c>
+      <c r="G19" t="n">
+        <v>-0.24</v>
+      </c>
       <c r="H19" t="n">
-        <v>51350114</v>
+        <v>14948187</v>
       </c>
     </row>
     <row r="20">
@@ -1081,20 +1099,20 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>4010</v>
+        <v>3920.2</v>
       </c>
       <c r="F20" t="n">
-        <v>-41.6001</v>
+        <v>-111.2</v>
       </c>
       <c r="G20" t="n">
-        <v>-1.03</v>
+        <v>-2.76</v>
       </c>
       <c r="H20" t="n">
-        <v>12321</v>
+        <v>159747</v>
       </c>
     </row>
     <row r="21">
@@ -1115,20 +1133,20 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>102.83</v>
+        <v>104.22</v>
       </c>
       <c r="F21" t="n">
-        <v>0.05</v>
+        <v>2.22</v>
       </c>
       <c r="G21" t="n">
-        <v>0.05</v>
+        <v>2.18</v>
       </c>
       <c r="H21" t="n">
-        <v>8239</v>
+        <v>134199</v>
       </c>
     </row>
     <row r="22">
@@ -1149,20 +1167,20 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="E22" t="n">
-        <v>111.57</v>
+        <v>113.47</v>
       </c>
       <c r="F22" t="n">
-        <v>-3.75</v>
+        <v>-1.41</v>
       </c>
       <c r="G22" t="n">
-        <v>-3.25</v>
+        <v>-1.23</v>
       </c>
       <c r="H22" t="n">
-        <v>1397</v>
+        <v>24546</v>
       </c>
     </row>
     <row r="23">
@@ -1183,20 +1201,20 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="E23" t="n">
-        <v>6.542</v>
+        <v>6.5165</v>
       </c>
       <c r="F23" t="n">
-        <v>-0.09950000000000001</v>
+        <v>-0.0645</v>
       </c>
       <c r="G23" t="n">
-        <v>-1.5</v>
+        <v>-0.98</v>
       </c>
       <c r="H23" t="n">
-        <v>2474</v>
+        <v>26923</v>
       </c>
     </row>
     <row r="24">
@@ -1217,14 +1235,20 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr"/>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr"/>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>61.35</v>
+      </c>
+      <c r="F24" t="n">
+        <v>-1.37</v>
+      </c>
+      <c r="G24" t="n">
+        <v>-2.18</v>
+      </c>
       <c r="H24" t="n">
-        <v>22053571</v>
+        <v>8254911</v>
       </c>
     </row>
     <row r="25">
@@ -1245,17 +1269,17 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="E25" t="n">
-        <v>17.2</v>
+        <v>19.13</v>
       </c>
       <c r="F25" t="n">
-        <v>0.29</v>
+        <v>1.93</v>
       </c>
       <c r="G25" t="n">
-        <v>1.71</v>
+        <v>11.22</v>
       </c>
       <c r="H25" t="n">
         <v>0</v>
@@ -1283,16 +1307,16 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>76806.5938</v>
+        <v>76972.9062</v>
       </c>
       <c r="F26" t="n">
-        <v>-4460.9922</v>
+        <v>-802.2030999999999</v>
       </c>
       <c r="G26" t="n">
-        <v>-5.49</v>
+        <v>-1.03</v>
       </c>
       <c r="H26" t="n">
-        <v>48511234048</v>
+        <v>59101728768</v>
       </c>
     </row>
     <row r="27">
@@ -1313,20 +1337,20 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="E27" t="n">
-        <v>1150</v>
+        <v>1070</v>
       </c>
       <c r="F27" t="n">
-        <v>-85</v>
+        <v>-80</v>
       </c>
       <c r="G27" t="n">
-        <v>-6.88</v>
+        <v>-6.96</v>
       </c>
       <c r="H27" t="n">
-        <v>100005900</v>
+        <v>86605000</v>
       </c>
     </row>
     <row r="28">
@@ -1347,20 +1371,20 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="E28" t="n">
-        <v>1350</v>
+        <v>1280</v>
       </c>
       <c r="F28" t="n">
-        <v>15</v>
+        <v>-70</v>
       </c>
       <c r="G28" t="n">
-        <v>1.12</v>
+        <v>-5.19</v>
       </c>
       <c r="H28" t="n">
-        <v>360528200</v>
+        <v>234540600</v>
       </c>
     </row>
     <row r="29">
@@ -1381,20 +1405,20 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="E29" t="n">
-        <v>410</v>
+        <v>382</v>
       </c>
       <c r="F29" t="n">
-        <v>-22</v>
+        <v>-28</v>
       </c>
       <c r="G29" t="n">
-        <v>-5.09</v>
+        <v>-6.83</v>
       </c>
       <c r="H29" t="n">
-        <v>517058000</v>
+        <v>294307300</v>
       </c>
     </row>
     <row r="30">
@@ -1415,20 +1439,20 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="E30" t="n">
-        <v>1930</v>
+        <v>1795</v>
       </c>
       <c r="F30" t="n">
-        <v>-140</v>
+        <v>-135</v>
       </c>
       <c r="G30" t="n">
-        <v>-6.76</v>
+        <v>-6.99</v>
       </c>
       <c r="H30" t="n">
-        <v>6505000</v>
+        <v>7711900</v>
       </c>
     </row>
     <row r="31">
@@ -1449,20 +1473,20 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="E31" t="n">
-        <v>2490</v>
+        <v>2320</v>
       </c>
       <c r="F31" t="n">
-        <v>-180</v>
+        <v>-170</v>
       </c>
       <c r="G31" t="n">
-        <v>-6.74</v>
+        <v>-6.83</v>
       </c>
       <c r="H31" t="n">
-        <v>32711600</v>
+        <v>18952500</v>
       </c>
     </row>
     <row r="32">
@@ -1483,20 +1507,20 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="E32" t="n">
-        <v>362</v>
+        <v>338</v>
       </c>
       <c r="F32" t="n">
         <v>-24</v>
       </c>
       <c r="G32" t="n">
-        <v>-6.22</v>
+        <v>-6.63</v>
       </c>
       <c r="H32" t="n">
-        <v>31775900</v>
+        <v>38873200</v>
       </c>
     </row>
     <row r="33">
@@ -1517,20 +1541,20 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="E33" t="n">
-        <v>418</v>
+        <v>394</v>
       </c>
       <c r="F33" t="n">
-        <v>-30</v>
+        <v>-24</v>
       </c>
       <c r="G33" t="n">
-        <v>-6.7</v>
+        <v>-5.74</v>
       </c>
       <c r="H33" t="n">
-        <v>40857300</v>
+        <v>72248200</v>
       </c>
     </row>
     <row r="34">
@@ -1551,20 +1575,20 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="E34" t="n">
-        <v>2080</v>
+        <v>1935</v>
       </c>
       <c r="F34" t="n">
-        <v>-150</v>
+        <v>-145</v>
       </c>
       <c r="G34" t="n">
-        <v>-6.73</v>
+        <v>-6.97</v>
       </c>
       <c r="H34" t="n">
-        <v>4890600</v>
+        <v>8850100</v>
       </c>
     </row>
     <row r="35">
@@ -1585,20 +1609,20 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="E35" t="n">
-        <v>336</v>
+        <v>314</v>
       </c>
       <c r="F35" t="n">
-        <v>-24</v>
+        <v>-22</v>
       </c>
       <c r="G35" t="n">
-        <v>-6.67</v>
+        <v>-6.55</v>
       </c>
       <c r="H35" t="n">
-        <v>183254800</v>
+        <v>77499900</v>
       </c>
     </row>
     <row r="36">
@@ -1619,20 +1643,20 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="E36" t="n">
-        <v>139</v>
+        <v>130</v>
       </c>
       <c r="F36" t="n">
-        <v>-10</v>
+        <v>-9</v>
       </c>
       <c r="G36" t="n">
-        <v>-6.71</v>
+        <v>-6.47</v>
       </c>
       <c r="H36" t="n">
-        <v>24239300</v>
+        <v>23229900</v>
       </c>
     </row>
     <row r="37">
@@ -1653,20 +1677,20 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="E37" t="n">
-        <v>9475</v>
+        <v>8825</v>
       </c>
       <c r="F37" t="n">
-        <v>-700</v>
+        <v>-650</v>
       </c>
       <c r="G37" t="n">
-        <v>-6.88</v>
+        <v>-6.86</v>
       </c>
       <c r="H37" t="n">
-        <v>10634000</v>
+        <v>4987200</v>
       </c>
     </row>
   </sheetData>
@@ -1725,22 +1749,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Bank Sentral Eropa Tahan Suku Bunga, Ada Sinyal Kenaikan di Akhir Tahun</t>
+          <t>SETC Dorong Tepa Selira Kembangkan Usaha dan Berdayakan Warga</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Fri, 30 Oct 2026 08:11:38 +0700</t>
+          <t>Fri, 30 Oct 2026 21:43:09 +0700</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2017/04/06/2945e8b1-4fe5-47aa-833f-748663cb4abe_169.jpeg?w=360&amp;amp;q=90" /&gt; Bank Sentral Eropa (ECB) menahan suku bunga acuannya di level 2,5% pada Kamis (29/10).</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/30/youtube-inside-sampoerna-1793371074799_169.jpeg?w=360&amp;amp;q=90" /&gt; Sampoerna Entrepreneurship Training Center mendukung UMKM Tepa Selira untuk berkembang berkelanjutan, fokus pada kearifan lokal dan dampak sosial positif.</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/moneter/d-8730465/bank-sentral-eropa-tahan-suku-bunga-ada-sinyal-kenaikan-di-akhir-tahun</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8731841/setc-dorong-tepa-selira-kembangkan-usaha-dan-berdayakan-warga</t>
         </is>
       </c>
     </row>
@@ -1752,22 +1776,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Dari Dapur ke Pesawat, Minyak Jelantah Dibeli hingga Rp6.000 per Liter</t>
+          <t>Dukung UMKM, SETC Dorong Tepa Selira Jaga Kearifan Lokal</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Fri, 30 Oct 2026 08:00:32 +0700</t>
+          <t>Fri, 30 Oct 2026 21:38:35 +0700</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/29/dari-dapur-ke-pesawat-minyak-jelantah-dibeli-hingga-rp6000-per-liter-1793265451125_169.jpeg?w=360&amp;amp;q=90" /&gt; Warga Banyumas mengumpulkan minyak jelantah dengan harga Rp5.000-Rp6.000 per liter untuk diolah menjadi bahan bakar pe</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/30/youtube-inside-sampoerna-1793371074799_169.jpeg?w=360&amp;amp;q=90" /&gt; Sampoerna Entrepreneurship Training Center mendukung UMKM Tepa Selira untuk berkembang berkelanjutan, fokus pada kearifan lokal dan dampak sosial positif.</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/foto-bisnis/d-8729719/dari-dapur-ke-pesawat-minyak-jelantah-dibeli-hingga-rp6-000-per-liter</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8731834/dukung-umkm-setc-dorong-tepa-selira-jaga-kearifan-lokal</t>
         </is>
       </c>
     </row>
@@ -1779,22 +1803,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>BI Buka Suara soal Potensi Dolar AS Tembus Rp 22.000 Imbas MSCI</t>
+          <t>250 Proyek Strategis Nasional Rampung, Total Investasi Rp 2.396 Triliun</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Fri, 30 Oct 2026 07:58:00 +0700</t>
+          <t>Fri, 30 Oct 2026 21:30:40 +0700</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/29/detik-pagi-bi-buka-suara-soal-potensi-dolar-as-tembus-rp-22000-imbas-msci-1793285659063_169.jpeg?w=360&amp;amp;q=90" /&gt; Rupiah disebut bisa semakin terpuruk imbas keputusan MSCI. Hal ini diungkap oleh Ketua Dewan Penasihat Kadin Indo</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2020/11/08/siap-siap-tol-cimanggis-cibitung-bakal-segera-dibuka-1_169.jpeg?w=360&amp;amp;q=90" /&gt; Pemerintah mencatat 250 Proyek Strategis Nasional (PSN) rampung sejak 2016 hingga 29 Oktober 2026. Total nilai investasi Rp 2.396 triliun.</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/bursa-dan-valas/d-8730205/bi-buka-suara-soal-potensi-dolar-as-tembus-rp-22-000-imbas-msci</t>
+          <t>https://finance.detik.com/infrastruktur/d-8731826/250-proyek-strategis-nasional-rampung-total-investasi-rp-2-396-triliun</t>
         </is>
       </c>
     </row>
@@ -1806,22 +1830,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Oplos Beras Rugikan Negara Rp 3,3 Miliar, 8 Pejabat Dicopot</t>
+          <t>Menteri PU Bongkar Masalah Kali Angke, Ada Bendung Peninggalan Belanda</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Fri, 30 Oct 2026 07:55:00 +0700</t>
+          <t>Fri, 30 Oct 2026 21:00:39 +0700</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/17/harga-beras-di-pasar-serpong-tangerang-selatan-pada-kamis-17092026-rata-rata-cenderung-stabil-di-bawah-angka-rp-14000-per-lite-1789644359234_169.jpeg?w=360&amp;amp;q=90" /&gt; Oplos beras SPHP menjadi premium di Jakarta Timur terkuak. P</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/30/menteri-pekerjaan-umum-pu-dody-hanggodo-1793356949850_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri PU Dody Hanggodo meninjau Kali Angke untuk antisipasi banjir. Ia temukan masalah pendangkalan dan penyempitan sungai akibat sampah dan pemu</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8730179/oplos-beras-rugikan-negara-rp-3-3-miliar-8-pejabat-dicopot</t>
+          <t>https://finance.detik.com/infrastruktur/d-8731647/menteri-pu-bongkar-masalah-kali-angke-ada-bendung-peninggalan-belanda</t>
         </is>
       </c>
     </row>
@@ -1833,22 +1857,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>QRIS Cross-Border Bikin Transaksi di Luar Negeri Lebih Mudah &amp;amp; Praktis</t>
+          <t>Tim Kemenperin Usut Insiden Gas Pindo Deli Ganggu Warga di Karawang</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Fri, 30 Oct 2026 07:45:21 +0700</t>
+          <t>Fri, 30 Oct 2026 20:45:15 +0700</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2020/10/04/solo-traveling.jpeg?w=360&amp;amp;q=90" /&gt; QRIS Cross-Border memudahkan pembayaran di luar negeri tanpa uang tunai. Cukup scan QR dengan aplikasi yang mendukung, transaksi jadi cepat dan aman.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/06/24/ipal-milik-pt-pindo-deli-pulp-and-paper-mills-1-saat-proses-produksi-dan-membuang-limbah-ke-sungai-citarum-kecamatan-telukjamb-1750750993653_169.jpeg?w=360&amp;amp;q=90" /&gt; Kementerian Perindustrian (Kemenperin) bergerak cepat meresp</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8727732/qris-cross-border-bikin-transaksi-di-luar-negeri-lebih-mudah-praktis</t>
+          <t>https://finance.detik.com/industri/d-8731786/tim-kemenperin-usut-insiden-gas-pindo-deli-ganggu-warga-di-karawang</t>
         </is>
       </c>
     </row>
@@ -1860,22 +1884,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Hashim Sebut di Medsos Banyak yang Bohong soal Utang Indonesia</t>
+          <t>OJK Serahkan Laporan Penelusuran Dana PT DSI ke Bareskrim</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Fri, 30 Oct 2026 07:25:00 +0700</t>
+          <t>Fri, 30 Oct 2026 20:30:55 +0700</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2024/10/31/hashim-djojohadikusumo-bertemu-ahy_169.jpeg?w=360&amp;amp;q=90" /&gt; Ketua Dewan Penasihat Kadin Hashim Djojohadikusumo menepis isu krisis utang Indonesia yang muncul di media sosial.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2016/12/30/ed5ec33a-5357-40f8-8f66-6713c06687ea_169.jpg?w=360&amp;amp;q=90" /&gt; OJK menyerahkan hasil penelusuran aliran dana dan identifikasi aset PT Dana Syariah Indonesia (DSI) kepada Bareskrim Polri pada Oktober 2026.</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8730168/hashim-sebut-di-medsos-banyak-yang-bohong-soal-utang-indonesia</t>
+          <t>https://finance.detik.com/moneter/d-8731630/ojk-serahkan-laporan-penelusuran-dana-pt-dsi-ke-bareskrim</t>
         </is>
       </c>
     </row>
@@ -1887,22 +1911,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Jawaban Bos Kadin soal Tudingan RI di Ambang Krisis</t>
+          <t>Perkuat Kawasan Industri, Danareksa Target Model Bisnis Jalan 2027</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Fri, 30 Oct 2026 06:55:00 +0700</t>
+          <t>Fri, 30 Oct 2026 20:24:14 +0700</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/29/ketua-umum-kadin-indonesia-anindya-novyan-bakrie-1793261193891_169.jpeg?w=360&amp;amp;q=90" /&gt; Ketua Umum Kadin Indonesia, Anindya Novyan Bakrie, menegaskan ekonomi Indonesia saat ini masih jauh lebih baik dibandingkan saat krisis 19</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/30/danareksa-1793366374308_169.jpeg?w=360&amp;amp;q=90" /&gt; PT Danareksa berkomitmen perkuat nilai tambah dan kinerja bisnis sebagai Holding Kawasan Industri Indonesia, mendukung transformasi ekonomi yang berkelanjutan.</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8730172/jawaban-bos-kadin-soal-tudingan-ri-di-ambang-krisis</t>
+          <t>https://finance.detik.com/industri/d-8731775/perkuat-kawasan-industri-danareksa-target-model-bisnis-jalan-2027</t>
         </is>
       </c>
     </row>
@@ -1914,22 +1938,22 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Pembalut Masih Dikenai Pajak, Ini Alasannya</t>
+          <t>Danareksa dan Danantara Siapkan Model Bisnis Baru Kawasan Industri</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Fri, 30 Oct 2026 06:25:00 +0700</t>
+          <t>Fri, 30 Oct 2026 20:20:42 +0700</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2022/10/18/pembalut-nifas_169.jpeg?w=360&amp;amp;q=90" /&gt; Ramai di media sosial (medsos) pembalut dikenakan pajak. Netizen mempertanyakan alasan pembalut masih kena pajak, padahal merupakan kebutuhan dasar perempuan.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/30/danareksa-1793366374308_169.jpeg?w=360&amp;amp;q=90" /&gt; PT Danareksa berkomitmen perkuat nilai tambah dan kinerja bisnis sebagai Holding Kawasan Industri Indonesia, mendukung transformasi ekonomi yang berkelanjutan.</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8730154/pembalut-masih-dikenai-pajak-ini-alasannya</t>
+          <t>https://finance.detik.com/industri/d-8731771/danareksa-dan-danantara-siapkan-model-bisnis-baru-kawasan-industri</t>
         </is>
       </c>
     </row>
@@ -1941,22 +1965,22 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Hashim Ungkap Dampak Ngeri Pengumuman MSCI</t>
+          <t>ASDP Gratiskan Tarif Jasa Kepelabuhan Libur Nataru</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Fri, 30 Oct 2026 05:55:00 +0700</t>
+          <t>Fri, 30 Oct 2026 20:13:37 +0700</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2024/11/12/hashim-dalam-cop-29_169.png?w=360&amp;amp;q=90" /&gt; Ketua Dewan Penasihat Kadin Hashim Djojohadikusumo mengungkap dampak buruk jika MSCI jadi menurunkan kasta pasar modal Indonesia ke Standalone Market.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/30/km-legundi-asdp-1790751914690_169.jpeg?w=360&amp;amp;q=90" /&gt; PT ASDP Indonesia Ferry (Persero) membebaskan 100% tarif jasa kepelabuhanan bagi pengguna jasa penyeberangan pada periode Natal dan Tahun Baru (Nataru)</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/bursa-dan-valas/d-8730131/hashim-ungkap-dampak-ngeri-pengumuman-msci</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8731760/asdp-gratiskan-tarif-jasa-kepelabuhan-libur-nataru</t>
         </is>
       </c>
     </row>
@@ -1968,22 +1992,22 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Integrasi Tarif Tol Jabodetabek Bisakah Dilakukan? Ini Jawabannya</t>
+          <t>Pengusaha Respons soal Pembalut Kena Pajak</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Thu, 29 Oct 2026 22:37:00 +0700</t>
+          <t>Fri, 30 Oct 2026 19:50:08 +0700</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2020/11/05/rencana-kenikan-tarif-tol-lingkar-luar-jakarta-3_169.jpeg?w=360&amp;amp;q=90" /&gt; Integrasi tarif tol Jabodetabek dinilai bisa membuat perjalanan lebih lancar, biaya terjangkau, dan akses ke kawasan industri dan pelabuhan yang efisien</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/12/25/626173166-1766621550931_169.jpeg?w=360&amp;amp;q=90" /&gt; Wacana pajak pembalut ramai diperbincangkan, para pengusaha dari Kadin Indonesia buka suara soal hal ini.</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/infrastruktur/d-8730303/integrasi-tarif-tol-jabodetabek-bisakah-dilakukan-ini-jawabannya</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8731731/pengusaha-respons-soal-pembalut-kena-pajak</t>
         </is>
       </c>
     </row>
@@ -1995,22 +2019,22 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Kopdes Jadi Titik Kumpul Minyak Jelantah Sebelum 'Disulap' Jadi Bioavtur</t>
+          <t>Maluku Dibidik Jadi Kawasan Ekonomi Khusus</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Thu, 29 Oct 2026 22:30:00 +0700</t>
+          <t>Fri, 30 Oct 2026 19:30:00 +0700</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/09/21/kopdes-merah-putih-bersiap-operasional-23-ribu-bangunan-telah-rampung-1789986171319_169.jpeg?w=360&amp;amp;q=90" /&gt; PT Pertamina Patra Niaga bersama Kementerian Koperasi memulai program percontohan pengumpulan minyak jelantah berbasi</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/23/menperin-sarmuji-sebut-danantara-siapkan-rp-100-t-buat-industri-tekstil-1792748495902_169.jpeg?w=360&amp;amp;q=90" /&gt; Menteri Perindustrian Muhammad Sarmuji menyampaikan bahwa pemerintah tengah membidik salah satu dulau di Maluku unt</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/energi/d-8730274/kopdes-jadi-titik-kumpul-minyak-jelantah-sebelum-disulap-jadi-bioavtur</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8731625/maluku-dibidik-jadi-kawasan-ekonomi-khusus</t>
         </is>
       </c>
     </row>
@@ -2022,22 +2046,22 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Garuda Cetak Pendapatan Rp 49,24 Triliun di Tengah Tekanan Harga Avtur</t>
+          <t>Ramai-ramai Petinggi Mandom Indonesia Mundur, Ada Apa?</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Thu, 29 Oct 2026 22:02:21 +0700</t>
+          <t>Fri, 30 Oct 2026 19:00:47 +0700</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2025/07/19/pesawat-garuda-indonesia-1752916632356_169.jpeg?w=360&amp;amp;q=90" /&gt; PT Garuda Indonesia (Persero) Tbk (GIAA) membukukan pertumbuhan pendapatan konsolidasi sebesar 13,2% menjadi US$ 2,71 miliar atau sekitar Rp 49,24 triliun.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/16/ihsg-ambruk-1157-ditutup-di-level-5185-1792144638880_169.jpeg?w=360&amp;amp;q=90" /&gt; PT Mandom Indonesia Tbk (TCID) mengumumkan pengunduran diri anggota direksi dan komisaris secara serentak.</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8730237/garuda-cetak-pendapatan-rp-49-24-triliun-di-tengah-tekanan-harga-avtur</t>
+          <t>https://finance.detik.com/bursa-dan-valas/d-8731611/ramai-ramai-petinggi-mandom-indonesia-mundur-ada-apa</t>
         </is>
       </c>
     </row>
@@ -2049,22 +2073,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>GOTO Cetak Laba Rp 441 Miliar</t>
+          <t>Dikejar Waktu, Jastiper Berburu Barang Diskon di Imperfect Sale 2026</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Thu, 29 Oct 2026 21:41:04 +0700</t>
+          <t>Fri, 30 Oct 2026 19:00:10 +0700</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/20/goto-rilis-model-llm-27b-paham-bahasa-indonesia-hingga-daerah-1792493682697_169.jpeg?w=360&amp;amp;q=90" /&gt; PT GoTo Gojek Tokopedia Tbk (GOTO) mencatat laba bersih Rp 441 miliar pada kuartal III-2026.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/30/dikejar-waktu-jastiper-berburu-barang-diskon-di-imperfect-sale-2026-1793346505988.jpeg?w=360&amp;amp;q=90" /&gt; Berbekal waktu satu jam, para jastiper berburu produk diskon di Imperfect Sale 2026, Blok M Square, Jakarta.</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/bursa-dan-valas/d-8730220/goto-cetak-laba-rp-441-miliar</t>
+          <t>https://finance.detik.com/foto-bisnis/d-8731108/dikejar-waktu-jastiper-berburu-barang-diskon-di-imperfect-sale-2026</t>
         </is>
       </c>
     </row>
@@ -2076,22 +2100,22 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Laba PTBA Melonjak, Capai Rp 4,41 Triliun hingga Triwulan III 2026</t>
+          <t>Bulog Serap 4,25 Juta Ton Beras, Begini Perjalanan Gabah dari Petani</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Thu, 29 Oct 2026 21:34:47 +0700</t>
+          <t>Fri, 30 Oct 2026 18:38:32 +0700</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/29/ptba-1793284413718_169.jpeg?w=360&amp;amp;q=90" /&gt; PT Bukit Asam (PTBA) laporkan laba bersih Rp 4,41 triliun hingga September 2026. Kinerja operasional pulih dengan produksi dan penjualan meningkat.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/10/30/gudang-perum-bulog-kancab-semarang-tambakaji-kecamatan-ngaliyan-kota-semarang-1793360294855_169.jpeg?w=360&amp;amp;q=90" /&gt; Perum Bulog berhasil menyerap 4,25 juta ton gabah hingga 28 Oktober 2026. Proses panjang melibatkan petani hi</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/bursa-dan-valas/d-8730215/laba-ptba-melonjak-capai-rp-4-41-triliun-hingga-triwulan-iii-2026</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8731624/bulog-serap-4-25-juta-ton-beras-begini-perjalanan-gabah-dari-petani</t>
         </is>
       </c>
     </row>
@@ -2103,22 +2127,22 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Prabowo Bakal Resmikan Pabrik Baterai Mobil Listrik di Karawang</t>
+          <t>Dirut Indofarma Diganti!</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Thu, 29 Oct 2026 20:58:34 +0700</t>
+          <t>Fri, 30 Oct 2026 18:32:56 +0700</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2026/08/27/baterai-mobil-listrik-1787794586277_169.jpeg?w=360&amp;amp;q=90" /&gt; Presiden Prabowo Subianto bakal meresmikan pabrik baterai mobil listrik di Karawang, kerja sama CATL dan Antam.</t>
+          <t>&lt;img src="https://akcdn.detik.net.id/community/media/visual/2024/10/15/ilustrasi-serah-terima-kunci-pembelian-properti-rumah-pertama_169.jpeg?w=360&amp;amp;q=90" /&gt; PT Indofarma (Persero) Tbk memiliki Direktur Utama (Dirut) baru yakni Dicky Henria Nugraha. Dicky mengantikan Sahat Sihombing.</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://finance.detik.com/industri/d-8730191/prabowo-bakal-resmikan-pabrik-baterai-mobil-listrik-di-karawang</t>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8731610/dirut-indofarma-diganti</t>
         </is>
       </c>
     </row>
@@ -2130,22 +2154,22 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Akal Bulus Silmy Karim Terbongkar di Persidangan</t>
+          <t>Menteri Wihaji: Perbaiki Negara Dimulai dari Keluarga</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Fri, 30 Oct 2026 07:30:56 +0700</t>
+          <t>Fri, 30 Oct 2026 21:48:50 +0700</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Silmy Karim melawan atas dakwaan yang disampaikan dengan mengajukan eksepsi.</t>
+          <t>Wihaji menegaskan, kesehatan keluarga menjadi kunci untuk meningkatkan kualitas bangsa.</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8324597/akal-bulus-silmy-karim-terbongkar-di-persidangan</t>
+          <t>https://www.liputan6.com/news/read/8325303/menteri-wihaji-perbaiki-negara-dimulai-dari-keluarga</t>
         </is>
       </c>
     </row>
@@ -2157,22 +2181,22 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>1,5 Tahun Berlalu, Induk Harimau Sumatera Kembali Terekam Bareng 3 Anaknya</t>
+          <t>TNI AD: Letda AG Jadi Tersangka Kasus Tewasnya Letda Jihad</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Fri, 30 Oct 2026 07:19:09 +0700</t>
+          <t>Fri, 30 Oct 2026 21:39:12 +0700</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Mereka berkumpul di dekat bak penampungan air minum disediakan petugas.</t>
+          <t>Letda Inf. AG dijerat Pasal 474 ayat (3) KUHP tentang kelalaian yang mengakibatkan kematian</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8324599/15-tahun-berlalu-induk-harimau-sumatera-kembali-terekam-bareng-3-anaknya</t>
+          <t>https://www.liputan6.com/news/read/8325298/tni-ad-letda-ag-jadi-tersangka-kasus-tewasnya-letda-jihad</t>
         </is>
       </c>
     </row>
@@ -2184,22 +2208,22 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Kisah 'Pilot Darat' Antar Mahasiswa UI Terobos Barikade Polisi</t>
+          <t>Geledah PT IPPS, Kejagung Temukan Ruangan Tersembunyi di Balik Lemari</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Thu, 29 Oct 2026 21:03:09 +0700</t>
+          <t>Fri, 30 Oct 2026 21:39:22 +0700</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Marsudi punya keyakinan soal niat baik mahasiswa memperjuangkan nasib rakyat dan menyuarakan kondisi negara.</t>
+          <t>Kejagung menggeledah kantor PT IPPS selama sekitar 17 jam dalam penyidikan dugaan korupsi transfer pricing PT Toba Pulp Lestari.</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8324469/kisah-pilot-darat-antar-mahasiswa-ui-terobos-barikade-polisi</t>
+          <t>https://www.liputan6.com/news/read/8325293/geledah-pt-ipps-kejagung-temukan-ruangan-tersembunyi-di-balik-lemari</t>
         </is>
       </c>
     </row>
@@ -2211,22 +2235,22 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Taktik Sudaryono Tutup Celah Rasuah BGN hingga MBG</t>
+          <t>JIS Dilirik 15 Konser Besar</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Fri, 30 Oct 2026 06:30:00 +0700</t>
+          <t>Fri, 30 Oct 2026 21:06:30 +0700</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Sudaryono mengaku tidak melayani permintaan pengurusan dapur MBG melalui jalur pribadi.</t>
+          <t>Pramono menilai, salah satu faktor yang membuat JIS semakin menarik penyelenggara acara adalah akses transportasi.</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8324582/taktik-sudaryono-tutup-celah-rasuah-bgn-hingga-mbg</t>
+          <t>https://www.liputan6.com/news/read/8325274/jis-dilirik-15-konser-besar</t>
         </is>
       </c>
     </row>
@@ -2238,22 +2262,22 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>12 Perusuh Saat Demo di Alun-Alun Tugu Malang Ditangkap, Bom Molotov Disita</t>
+          <t>SMA Taruna Nusantara Kini Gratis, Prabowo Perluas Jadi 6 Kampus</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Fri, 30 Oct 2026 05:54:28 +0700</t>
+          <t>Fri, 30 Oct 2026 20:48:53 +0700</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Hasil tes urine, mereka positif sabu.</t>
+          <t>Peresmian kampus di Cimahi menandai perluasan jaringan SMA Taruna Nusantara sekaligus penerapan kebijakan pendidikan gratis.</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8324580/12-perusuh-saat-demo-di-alun-alun-tugu-malang-ditangkap-bom-molotov-disita</t>
+          <t>https://www.liputan6.com/news/read/8325269/sma-taruna-nusantara-kini-gratis-prabowo-perluas-jadi-6-kampus</t>
         </is>
       </c>
     </row>
@@ -2265,22 +2289,22 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Cerita Kepala BGN  Tiap Hari Didemo soal Program MBG</t>
+          <t>Pramono Matangkan Usulan 76 Taman Jakarta Buka 24 Jam</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Fri, 30 Oct 2026 01:00:13 +0700</t>
+          <t>Fri, 30 Oct 2026 20:26:34 +0700</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Sudaryono menyatakan terbuka terhadap kritik soal MBG, tetapi menegaskan pihaknya selektif dalam menanggapi demonstrasi yang dinilai hanya ikut-ikutan.</t>
+          <t>Pramono meminta jajarannya mematangkan rencana tersebut.</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8324563/cerita-kepala-bgn-tiap-hari-didemo-soal-program-mbg</t>
+          <t>https://www.liputan6.com/news/read/8325259/pramono-matangkan-usulan-76-taman-jakarta-buka-24-jam</t>
         </is>
       </c>
     </row>
@@ -2292,22 +2316,22 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Kuasa Hukum: Uang Rp 186 M Bukan Milik Silmy Karim</t>
+          <t>5,9 Juta Orang Terdampak Bencana Sepanjang 2026</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Fri, 30 Oct 2026 00:18:32 +0700</t>
+          <t>Fri, 30 Oct 2026 20:07:54 +0700</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Silmy didakwa melakukan pemerasan terhadap pemohon dokumen keimigrasian terkait izin tinggal WNA senilai Rp 168,9 miliar.</t>
+          <t>BNPB mencatat 2.247 kejadian bencana di Indonesia hingga 30 Oktober 2026.</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8324556/kuasa-hukum-uang-rp-186-m-bukan-milik-silmy-karim</t>
+          <t>https://www.liputan6.com/news/read/8325249/59-juta-orang-terdampak-bencana-sepanjang-2026</t>
         </is>
       </c>
     </row>
@@ -2319,22 +2343,22 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>RPTRA Kebon Sirih, Oase Hijau di Tengah Padatnya Jakarta</t>
+          <t>Wamendagri: Bonus Demografi Modal Lahirkan Pemimpin Muda Indonesia Emas</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Thu, 29 Oct 2026 22:46:04 +0700</t>
+          <t>Fri, 30 Oct 2026 20:12:05 +0700</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Kebun sayur, kolam ikan, dan pengolahan sampah menjadi bagian dari upaya merawat lingkungan sekaligus kehidupan warga.</t>
+          <t>Wiyagus menilai generasi milenial dan generasi Z memiliki peran penting dalam menentukan arah bangsa.</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8324517/rptra-kebon-sirih-oase-hijau-di-tengah-padatnya-jakarta</t>
+          <t>https://www.liputan6.com/news/read/8325251/wamendagri-bonus-demografi-modal-lahirkan-pemimpin-muda-indonesia-emas</t>
         </is>
       </c>
     </row>
@@ -2346,22 +2370,22 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Waspada Banjir dan Longsor, Catat Sederet Imbauan BNPB</t>
+          <t>Di Hadapan Ulama Suriah, Asrorun Ni’am Bicara Peran Agama dan Negara</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Thu, 29 Oct 2026 22:43:06 +0700</t>
+          <t>Fri, 30 Oct 2026 19:52:30 +0700</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Imbauan bencana hidrometeorologi ini ditujukan kepada pemerintah, relawan hingga masyarakat</t>
+          <t>Di hadapan ratusan ulama dan akademisi Suriah, Asrorun Ni’am menegaskan pentingnya hubungan simbiotik antara agama dan negara.</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8324514/waspada-banjir-dan-longsor-catat-sederet-imbauan-bnpb</t>
+          <t>https://www.liputan6.com/news/read/8325234/di-hadapan-ulama-suriah-asrorun-niam-bicara-peran-agama-dan-negara</t>
         </is>
       </c>
     </row>
@@ -2373,22 +2397,22 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Residivis Jambret Lukai Korban di Depok Ditangkap</t>
+          <t>KPK Geledah Bea Cukai Semarang, Sita Dokumen dan Uang</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Thu, 29 Oct 2026 22:33:17 +0700</t>
+          <t>Fri, 30 Oct 2026 19:50:11 +0700</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Korban mengalami luka dan dibawa ke rumah sakit oleh warga yang mengetahui kejadian tersebut.</t>
+          <t>Dua kantor bea cukai di Semarang disasar KPK.</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8324509/residivis-jambret-lukai-korban-di-depok-ditangkap</t>
+          <t>https://www.liputan6.com/news/read/8325232/kpk-geledah-bea-cukai-semarang-sita-dokumen-dan-uang</t>
         </is>
       </c>
     </row>
@@ -2400,22 +2424,22 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Infografis: 100 Hari MBG di Tangan Sudaryono</t>
+          <t>Tiga Gunung Api Berstatus Siaga, Ini Imbauan BNPB</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Thu, 29 Oct 2026 21:58:48 +0700</t>
+          <t>Fri, 30 Oct 2026 19:37:03 +0700</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Sudaryono menerapkan sejumlah aturan untuk memperkuat keamanan pangan, kedisiplinan, dan transparansi program MBG.</t>
+          <t>pemutakhiran data aktivitas gunung api di Indonesia tercatat per Jumat (30/10/2026) pukul 06.00 WIB.</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8324499/infografis-100-hari-mbg-di-tangan-sudaryono</t>
+          <t>https://www.liputan6.com/news/read/8325224/tiga-gunung-api-berstatus-siaga-ini-imbauan-bnpb</t>
         </is>
       </c>
     </row>
@@ -2427,22 +2451,22 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Rincian Bonus Atlet Asian Games dan Asian Para Games dari Prabowo</t>
+          <t>Mensos Dampingi Siswa Sekolah Rakyat Diduga Korban Perundungan</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Thu, 29 Oct 2026 21:48:55 +0700</t>
+          <t>Fri, 30 Oct 2026 18:50:50 +0700</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Pemerintah memberikan bonus dengan besaran berbeda sesuai medali dan nomor pertandingan.</t>
+          <t>Kementerian Sosial (Kemensos) juga terus mendampingi siswa tersebut beserta orang tuanya.</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8324491/rincian-bonus-atlet-asian-games-dan-asian-para-games-dari-prabowo</t>
+          <t>https://www.liputan6.com/news/read/8325196/mensos-dampingi-siswa-sekolah-rakyat-diduga-korban-perundungan</t>
         </is>
       </c>
     </row>
@@ -2454,22 +2478,22 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Kuasa Hukum Bantah Silmy Karim Terjaring OTT KPK</t>
+          <t>MA Kabulkan Gugatan soal Suket Penyetaraan Ijazah SMA Gibran</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Thu, 29 Oct 2026 21:47:30 +0700</t>
+          <t>Fri, 30 Oct 2026 19:05:35 +0700</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Silmy Karim didakwa melakukan pemerasan terkait dokumen keimigrasian senilai Rp 168,9 miliar dan menerima gratifikasi Rp 33,8 miliar.</t>
+          <t>Putusan ini membatalkan keputusan PTUN Jakarta sebelumnya.</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8324487/kuasa-hukum-bantah-silmy-karim-terjaring-ott-kpk</t>
+          <t>https://www.liputan6.com/news/read/8325179/ma-kabulkan-gugatan-soal-suket-penyetaraan-ijazah-sma-gibran</t>
         </is>
       </c>
     </row>
@@ -2481,22 +2505,22 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Seskab Teddy Beberkan Capaian Dua Tahun Pemerintahan Prabowo</t>
+          <t>Triple 80, Strategi Menkes Tekan Kematian Akibat Stroke dan Penyakit Ginjal</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Thu, 29 Oct 2026 21:35:47 +0700</t>
+          <t>Fri, 30 Oct 2026 18:20:33 +0700</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Seskab melaporkan sejumlah capaian program prioritas dan pembangunan selama dua tahun pemerintahan Presiden Prabowo Subianto.</t>
+          <t>Menkes mendorong perubahan strategi dari mengobati orang sakit menjadi menjaga masyarakat tetap sehat.</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8324485/seskab-teddy-beberkan-capaian-dua-tahun-pemerintahan-prabowo</t>
+          <t>https://www.liputan6.com/news/read/8325184/triple-80-strategi-menkes-tekan-kematian-akibat-stroke-dan-penyakit-ginjal</t>
         </is>
       </c>
     </row>
@@ -2508,22 +2532,22 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>DPR: TNI Amankan Demo Hal Lumrah</t>
+          <t>Data Bansos Dibenahi, 4 Juta Keluarga Baru Dapat Bantuan</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Thu, 29 Oct 2026 21:07:45 +0700</t>
+          <t>Fri, 30 Oct 2026 18:19:15 +0700</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Menurut Dave, aparat tetap harus memastikan aksi berlangsung aman dan tertib tanpa mengabaikan hak masyarakat</t>
+          <t>Kemensos memperbarui data penerima PKH, bantuan sembako, dan PBI JKN agar bantuan pemerintah lebih tepat sasaran.</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>https://www.liputan6.com/news/read/8324473/dpr-tni-amankan-demo-hal-lumrah</t>
+          <t>https://www.liputan6.com/news/read/8325175/data-bansos-dibenahi-4-juta-keluarga-baru-dapat-bantuan</t>
         </is>
       </c>
     </row>

</xml_diff>